<commit_message>
update template DDG extracteur
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmy/Desktop/Betagouv/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8F139D2-E493-5F48-919C-8D1671F02DF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F81F938F-CD76-C846-8210-14F4E0829026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24580" windowHeight="14560" activeTab="5" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -626,9 +626,6 @@
     <t>#! DUMP_COLS x.actions</t>
   </si>
   <si>
-    <t xml:space="preserve">         Extracteur De Données D'Effectifs</t>
-  </si>
-  <si>
     <t>#` ${arrondissement}</t>
   </si>
   <si>
@@ -672,6 +669,9 @@
   </si>
   <si>
     <t xml:space="preserve">         Extracteur de données d'effectifs - Format DDG (avec réintégration de l'absentéisme)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         Extracteur de données d'effectifs</t>
   </si>
 </sst>
 </file>
@@ -1548,7 +1548,7 @@
   <sheetData>
     <row r="1" spans="1:118" s="4" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -1858,7 +1858,7 @@
   <sheetData>
     <row r="1" spans="1:8" s="4" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -1927,10 +1927,10 @@
   <sheetData>
     <row r="1" spans="1:13" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="52" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B1" s="45" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -1938,7 +1938,7 @@
     </row>
     <row r="2" spans="1:13" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A2" s="56" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B2" s="46" t="e">
         <f>VLOOKUP(A2,'codage tribunal'!A:B,2,FALSE)</f>
@@ -1959,37 +1959,37 @@
       <c r="C4" s="39"/>
       <c r="D4" s="40"/>
       <c r="E4" s="41" t="s">
+        <v>73</v>
+      </c>
+      <c r="F4" s="42" t="s">
         <v>74</v>
       </c>
-      <c r="F4" s="42" t="s">
+      <c r="G4" s="42" t="s">
         <v>75</v>
       </c>
-      <c r="G4" s="42" t="s">
+      <c r="H4" s="42" t="s">
         <v>76</v>
       </c>
-      <c r="H4" s="42" t="s">
+      <c r="I4" s="42" t="s">
         <v>77</v>
       </c>
-      <c r="I4" s="42" t="s">
+      <c r="J4" s="42" t="s">
         <v>78</v>
       </c>
-      <c r="J4" s="42" t="s">
+      <c r="K4" s="43" t="s">
         <v>79</v>
       </c>
-      <c r="K4" s="43" t="s">
-        <v>80</v>
-      </c>
       <c r="L4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="44"/>
       <c r="C5" s="48" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D5" s="47" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E5" s="51" t="e">
         <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-TIT",'ETPT Format DDG'!$C:$C,$A$2)</f>
@@ -2020,7 +2020,7 @@
         <v>#N/A</v>
       </c>
       <c r="L5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
update template excel données d'effectif
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10409"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10611"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmy/Desktop/Betagouv/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E054AD9C-5FEE-444C-AC9A-C915ED0C461A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AFA25C5-CCD6-A14E-8507-17C853FC29DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24580" windowHeight="14560" activeTab="5" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -784,7 +784,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -868,36 +868,37 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="3" builtinId="3"/>
@@ -1615,7 +1616,7 @@
       <c r="E4"/>
     </row>
     <row r="5" spans="1:118" x14ac:dyDescent="0.2">
-      <c r="B5" t="s">
+      <c r="B5" s="39" t="s">
         <v>15</v>
       </c>
       <c r="C5"/>
@@ -1693,7 +1694,7 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B5" t="s">
+      <c r="B5" s="39" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1706,7 +1707,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E893F90-1EC7-764C-B747-7920FCEC73CB}">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.33203125" customWidth="1"/>
@@ -1721,7 +1722,7 @@
     <col min="11" max="11" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
         <v>35</v>
       </c>
@@ -1732,7 +1733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A2" s="27" t="s">
         <v>22</v>
       </c>
@@ -1744,13 +1745,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="9"/>
     </row>
-    <row r="4" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="10"/>
       <c r="C4" s="10"/>
       <c r="D4" s="11"/>
@@ -1779,7 +1780,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="15"/>
       <c r="C5" s="19" t="s">
         <v>34</v>
@@ -1819,8 +1820,8 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="M6" t="s">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="L6" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1857,258 +1858,268 @@
   <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.1640625" style="36" customWidth="1"/>
-    <col min="2" max="2" width="7.33203125" style="36" customWidth="1"/>
-    <col min="3" max="9" width="10.83203125" style="36"/>
-    <col min="10" max="10" width="71.1640625" style="36" customWidth="1"/>
-    <col min="11" max="16384" width="10.83203125" style="36"/>
+    <col min="1" max="1" width="8.1640625" style="24" customWidth="1"/>
+    <col min="2" max="2" width="7.33203125" style="24" customWidth="1"/>
+    <col min="3" max="9" width="10.83203125" style="24"/>
+    <col min="10" max="10" width="71.1640625" style="24" customWidth="1"/>
+    <col min="11" max="16384" width="10.83203125" style="24"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="29" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
-    </row>
-    <row r="2" spans="1:10" s="32" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+    </row>
+    <row r="2" spans="1:10" s="10" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-    </row>
-    <row r="3" spans="1:10" s="32" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
+    </row>
+    <row r="3" spans="1:10" s="10" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="30"/>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="34" t="s">
+      <c r="C3" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="34"/>
-      <c r="J3" s="34"/>
-    </row>
-    <row r="4" spans="1:10" s="32" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
+      <c r="G3" s="37"/>
+      <c r="H3" s="37"/>
+      <c r="I3" s="37"/>
+      <c r="J3" s="37"/>
+    </row>
+    <row r="4" spans="1:10" s="10" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="30"/>
-      <c r="B4" s="33" t="s">
+      <c r="B4" s="31" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="34" t="s">
+      <c r="C4" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
-    </row>
-    <row r="5" spans="1:10" s="32" customFormat="1" ht="43" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D4" s="37"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="37"/>
+      <c r="H4" s="37"/>
+      <c r="I4" s="37"/>
+      <c r="J4" s="37"/>
+    </row>
+    <row r="5" spans="1:10" s="10" customFormat="1" ht="43" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="30"/>
-      <c r="B5" s="33" t="s">
+      <c r="B5" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="C5" s="34" t="s">
+      <c r="C5" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="34"/>
-      <c r="H5" s="34"/>
-      <c r="I5" s="34"/>
-      <c r="J5" s="34"/>
-    </row>
-    <row r="6" spans="1:10" s="32" customFormat="1" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="33" t="s">
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="37"/>
+      <c r="I5" s="37"/>
+      <c r="J5" s="37"/>
+    </row>
+    <row r="6" spans="1:10" s="10" customFormat="1" ht="37" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="34"/>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
-      <c r="J6" s="34"/>
-    </row>
-    <row r="7" spans="1:10" s="32" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C6" s="37"/>
+      <c r="D6" s="37"/>
+      <c r="E6" s="37"/>
+      <c r="F6" s="37"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="37"/>
+      <c r="J6" s="37"/>
+    </row>
+    <row r="7" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="30"/>
-      <c r="B7" s="31" t="s">
+      <c r="B7" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="31"/>
-      <c r="D7" s="31"/>
-      <c r="E7" s="31"/>
-      <c r="F7" s="31"/>
-      <c r="G7" s="31"/>
-      <c r="H7" s="31"/>
-      <c r="I7" s="31"/>
-      <c r="J7" s="31"/>
-    </row>
-    <row r="8" spans="1:10" s="32" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="35" t="s">
+      <c r="C7" s="34"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="34"/>
+      <c r="J7" s="34"/>
+    </row>
+    <row r="8" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="35"/>
-      <c r="I8" s="35"/>
-      <c r="J8" s="35"/>
-    </row>
-    <row r="9" spans="1:10" s="32" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="35" t="s">
+      <c r="C8" s="38"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="38"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="38"/>
+      <c r="I8" s="38"/>
+      <c r="J8" s="38"/>
+    </row>
+    <row r="9" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="35"/>
-      <c r="G9" s="35"/>
-      <c r="H9" s="35"/>
-      <c r="I9" s="35"/>
-      <c r="J9" s="35"/>
-    </row>
-    <row r="10" spans="1:10" s="32" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="35" t="s">
+      <c r="C9" s="38"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="38"/>
+      <c r="F9" s="38"/>
+      <c r="G9" s="38"/>
+      <c r="H9" s="38"/>
+      <c r="I9" s="38"/>
+      <c r="J9" s="38"/>
+    </row>
+    <row r="10" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="C10" s="35"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="35"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="35"/>
-      <c r="I10" s="35"/>
-      <c r="J10" s="35"/>
-    </row>
-    <row r="11" spans="1:10" s="32" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="35" t="s">
+      <c r="C10" s="38"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="38"/>
+      <c r="F10" s="38"/>
+      <c r="G10" s="38"/>
+      <c r="H10" s="38"/>
+      <c r="I10" s="38"/>
+      <c r="J10" s="38"/>
+    </row>
+    <row r="11" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="38" t="s">
         <v>50</v>
       </c>
-      <c r="C11" s="35"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="35"/>
-      <c r="G11" s="35"/>
-      <c r="H11" s="35"/>
-      <c r="I11" s="35"/>
-      <c r="J11" s="35"/>
-    </row>
-    <row r="12" spans="1:10" s="32" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C11" s="38"/>
+      <c r="D11" s="38"/>
+      <c r="E11" s="38"/>
+      <c r="F11" s="38"/>
+      <c r="G11" s="38"/>
+      <c r="H11" s="38"/>
+      <c r="I11" s="38"/>
+      <c r="J11" s="38"/>
+    </row>
+    <row r="12" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="30" t="s">
         <v>10</v>
       </c>
       <c r="B12" s="32" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" s="32" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="33" t="s">
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="33"/>
+      <c r="F12" s="33"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="33"/>
+      <c r="I12" s="33"/>
+      <c r="J12" s="33"/>
+    </row>
+    <row r="13" spans="1:10" s="10" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="34" t="s">
+      <c r="C13" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="34"/>
-      <c r="I13" s="34"/>
-      <c r="J13" s="34"/>
-    </row>
-    <row r="14" spans="1:10" s="32" customFormat="1" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="33" t="s">
+      <c r="D13" s="37"/>
+      <c r="E13" s="37"/>
+      <c r="F13" s="37"/>
+      <c r="G13" s="37"/>
+      <c r="H13" s="37"/>
+      <c r="I13" s="37"/>
+      <c r="J13" s="37"/>
+    </row>
+    <row r="14" spans="1:10" s="10" customFormat="1" ht="56" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="34" t="s">
+      <c r="C14" s="37" t="s">
         <v>53</v>
       </c>
-      <c r="D14" s="34"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="34"/>
-      <c r="G14" s="34"/>
-      <c r="H14" s="34"/>
-      <c r="I14" s="34"/>
-      <c r="J14" s="34"/>
-    </row>
-    <row r="15" spans="1:10" s="32" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="33" t="s">
+      <c r="D14" s="37"/>
+      <c r="E14" s="37"/>
+      <c r="F14" s="37"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="37"/>
+      <c r="I14" s="37"/>
+      <c r="J14" s="37"/>
+    </row>
+    <row r="15" spans="1:10" s="10" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="34" t="s">
+      <c r="C15" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="D15" s="34"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="34"/>
-      <c r="G15" s="34"/>
-      <c r="H15" s="34"/>
-      <c r="I15" s="34"/>
-      <c r="J15" s="34"/>
-    </row>
-    <row r="16" spans="1:10" s="32" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="33" t="s">
+      <c r="D15" s="37"/>
+      <c r="E15" s="37"/>
+      <c r="F15" s="37"/>
+      <c r="G15" s="37"/>
+      <c r="H15" s="37"/>
+      <c r="I15" s="37"/>
+      <c r="J15" s="37"/>
+    </row>
+    <row r="16" spans="1:10" s="10" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="34" t="s">
+      <c r="B16" s="37" t="s">
         <v>55</v>
       </c>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="34"/>
-      <c r="G16" s="34"/>
-      <c r="H16" s="34"/>
-      <c r="I16" s="34"/>
-      <c r="J16" s="34"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="37"/>
+      <c r="E16" s="37"/>
+      <c r="F16" s="37"/>
+      <c r="G16" s="37"/>
+      <c r="H16" s="37"/>
+      <c r="I16" s="37"/>
+      <c r="J16" s="37"/>
     </row>
     <row r="18" spans="1:10" s="29" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="37" t="s">
+      <c r="A18" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="38"/>
-      <c r="G18" s="38"/>
-      <c r="H18" s="38"/>
-      <c r="I18" s="38"/>
-      <c r="J18" s="38"/>
+      <c r="B18" s="36"/>
+      <c r="C18" s="36"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="36"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="36"/>
+      <c r="H18" s="36"/>
+      <c r="I18" s="36"/>
+      <c r="J18" s="36"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="17">
+    <mergeCell ref="C14:J14"/>
+    <mergeCell ref="B12:J12"/>
     <mergeCell ref="B7:J7"/>
     <mergeCell ref="A18:J18"/>
     <mergeCell ref="A1:J1"/>
@@ -2124,7 +2135,6 @@
     <mergeCell ref="B10:J10"/>
     <mergeCell ref="B11:J11"/>
     <mergeCell ref="C13:J13"/>
-    <mergeCell ref="C14:J14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
update extraction template ddg
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmy/Desktop/Betagouv/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AFA25C5-CCD6-A14E-8507-17C853FC29DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85F89413-D477-E346-84BF-35A1BA14109B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24580" windowHeight="14560" activeTab="5" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24580" windowHeight="14560" activeTab="2" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ETPT A-JUST" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="62">
   <si>
     <t>#! END_ROW</t>
   </si>
@@ -134,9 +134,6 @@
     <t>Fonctionnaires placés de substitution</t>
   </si>
   <si>
-    <t>Contractuels</t>
-  </si>
-  <si>
     <t>Code</t>
   </si>
   <si>
@@ -570,6 +567,24 @@
   </si>
   <si>
     <t>Pour toute question, n'hésitez pas à contacter l'équipe A-JUST : support-utilisateurs@a-just.fr</t>
+  </si>
+  <si>
+    <t>SIEGE</t>
+  </si>
+  <si>
+    <t>GREFFE</t>
+  </si>
+  <si>
+    <t>EQUIPE AUTOUR DU MAGISTRAT</t>
+  </si>
+  <si>
+    <t>Contractuels et vacataires</t>
+  </si>
+  <si>
+    <t>TOTAL SIEGE</t>
+  </si>
+  <si>
+    <t>TOTAL GREFFE</t>
   </si>
 </sst>
 </file>
@@ -583,7 +598,7 @@
     <numFmt numFmtId="166" formatCode="General;General;\-"/>
     <numFmt numFmtId="167" formatCode="0.###;0.###;\-"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -660,6 +675,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -705,7 +728,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -777,6 +800,82 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -784,7 +883,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -825,9 +924,6 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -877,6 +973,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -892,13 +992,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="12" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="3" builtinId="3"/>
@@ -906,7 +1026,22 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1345,7 +1480,7 @@
   <sheetData>
     <row r="1" spans="1:118" s="4" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -1360,131 +1495,131 @@
       </c>
     </row>
     <row r="2" spans="1:118" ht="66" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
-      <c r="M2" s="24"/>
-      <c r="N2" s="24"/>
-      <c r="O2" s="24"/>
-      <c r="P2" s="24"/>
-      <c r="Q2" s="24"/>
-      <c r="R2" s="24"/>
-      <c r="S2" s="24"/>
-      <c r="T2" s="24"/>
-      <c r="U2" s="24"/>
-      <c r="V2" s="24"/>
-      <c r="W2" s="24"/>
-      <c r="X2" s="24"/>
-      <c r="Y2" s="24"/>
-      <c r="Z2" s="24"/>
-      <c r="AA2" s="24"/>
-      <c r="AB2" s="24"/>
-      <c r="AC2" s="24"/>
-      <c r="AD2" s="24"/>
-      <c r="AE2" s="24"/>
-      <c r="AF2" s="24"/>
-      <c r="AG2" s="24"/>
-      <c r="AH2" s="24"/>
-      <c r="AI2" s="24"/>
-      <c r="AJ2" s="24"/>
-      <c r="AK2" s="24"/>
-      <c r="AL2" s="24"/>
-      <c r="AM2" s="24"/>
-      <c r="AN2" s="24"/>
-      <c r="AO2" s="24"/>
-      <c r="AP2" s="24"/>
-      <c r="AQ2" s="24"/>
-      <c r="AR2" s="24"/>
-      <c r="AS2" s="24"/>
-      <c r="AT2" s="24"/>
-      <c r="AU2" s="24"/>
-      <c r="AV2" s="24"/>
-      <c r="AW2" s="24"/>
-      <c r="AX2" s="24"/>
-      <c r="AY2" s="24"/>
-      <c r="AZ2" s="24"/>
-      <c r="BA2" s="24"/>
-      <c r="BB2" s="24"/>
-      <c r="BC2" s="24"/>
-      <c r="BD2" s="24"/>
-      <c r="BE2" s="24"/>
-      <c r="BF2" s="24"/>
-      <c r="BG2" s="24"/>
-      <c r="BH2" s="24"/>
-      <c r="BI2" s="24"/>
-      <c r="BJ2" s="24"/>
-      <c r="BK2" s="24"/>
-      <c r="BL2" s="24"/>
-      <c r="BM2" s="24"/>
-      <c r="BN2" s="24"/>
-      <c r="BO2" s="24"/>
-      <c r="BP2" s="24"/>
-      <c r="BQ2" s="24"/>
-      <c r="BR2" s="24"/>
-      <c r="BS2" s="24"/>
-      <c r="BT2" s="24"/>
-      <c r="BU2" s="24"/>
-      <c r="BV2" s="24"/>
-      <c r="BW2" s="24"/>
-      <c r="BX2" s="24"/>
-      <c r="BY2" s="24"/>
-      <c r="BZ2" s="24"/>
-      <c r="CA2" s="24"/>
-      <c r="CB2" s="24"/>
-      <c r="CC2" s="24"/>
-      <c r="CD2" s="24"/>
-      <c r="CE2" s="24"/>
-      <c r="CF2" s="24"/>
-      <c r="CG2" s="24"/>
-      <c r="CH2" s="24"/>
-      <c r="CI2" s="24"/>
-      <c r="CJ2" s="24"/>
-      <c r="CK2" s="24"/>
-      <c r="CL2" s="24"/>
-      <c r="CM2" s="24"/>
-      <c r="CN2" s="24"/>
-      <c r="CO2" s="24"/>
-      <c r="CP2" s="24"/>
-      <c r="CQ2" s="24"/>
-      <c r="CR2" s="24"/>
-      <c r="CS2" s="24"/>
-      <c r="CT2" s="24"/>
-      <c r="CU2" s="24"/>
-      <c r="CV2" s="24"/>
-      <c r="CW2" s="24"/>
-      <c r="CX2" s="24"/>
-      <c r="CY2" s="24"/>
-      <c r="CZ2" s="24"/>
-      <c r="DA2" s="24"/>
-      <c r="DB2" s="24"/>
-      <c r="DC2" s="24"/>
-      <c r="DD2" s="24"/>
-      <c r="DE2" s="24"/>
-      <c r="DF2" s="24"/>
-      <c r="DG2" s="24"/>
-      <c r="DH2" s="24"/>
-      <c r="DI2" s="24"/>
-      <c r="DJ2" s="24"/>
-      <c r="DK2" s="24"/>
-      <c r="DL2" s="24"/>
-      <c r="DM2" s="24"/>
-      <c r="DN2" s="24"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+      <c r="L2" s="23"/>
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+      <c r="O2" s="23"/>
+      <c r="P2" s="23"/>
+      <c r="Q2" s="23"/>
+      <c r="R2" s="23"/>
+      <c r="S2" s="23"/>
+      <c r="T2" s="23"/>
+      <c r="U2" s="23"/>
+      <c r="V2" s="23"/>
+      <c r="W2" s="23"/>
+      <c r="X2" s="23"/>
+      <c r="Y2" s="23"/>
+      <c r="Z2" s="23"/>
+      <c r="AA2" s="23"/>
+      <c r="AB2" s="23"/>
+      <c r="AC2" s="23"/>
+      <c r="AD2" s="23"/>
+      <c r="AE2" s="23"/>
+      <c r="AF2" s="23"/>
+      <c r="AG2" s="23"/>
+      <c r="AH2" s="23"/>
+      <c r="AI2" s="23"/>
+      <c r="AJ2" s="23"/>
+      <c r="AK2" s="23"/>
+      <c r="AL2" s="23"/>
+      <c r="AM2" s="23"/>
+      <c r="AN2" s="23"/>
+      <c r="AO2" s="23"/>
+      <c r="AP2" s="23"/>
+      <c r="AQ2" s="23"/>
+      <c r="AR2" s="23"/>
+      <c r="AS2" s="23"/>
+      <c r="AT2" s="23"/>
+      <c r="AU2" s="23"/>
+      <c r="AV2" s="23"/>
+      <c r="AW2" s="23"/>
+      <c r="AX2" s="23"/>
+      <c r="AY2" s="23"/>
+      <c r="AZ2" s="23"/>
+      <c r="BA2" s="23"/>
+      <c r="BB2" s="23"/>
+      <c r="BC2" s="23"/>
+      <c r="BD2" s="23"/>
+      <c r="BE2" s="23"/>
+      <c r="BF2" s="23"/>
+      <c r="BG2" s="23"/>
+      <c r="BH2" s="23"/>
+      <c r="BI2" s="23"/>
+      <c r="BJ2" s="23"/>
+      <c r="BK2" s="23"/>
+      <c r="BL2" s="23"/>
+      <c r="BM2" s="23"/>
+      <c r="BN2" s="23"/>
+      <c r="BO2" s="23"/>
+      <c r="BP2" s="23"/>
+      <c r="BQ2" s="23"/>
+      <c r="BR2" s="23"/>
+      <c r="BS2" s="23"/>
+      <c r="BT2" s="23"/>
+      <c r="BU2" s="23"/>
+      <c r="BV2" s="23"/>
+      <c r="BW2" s="23"/>
+      <c r="BX2" s="23"/>
+      <c r="BY2" s="23"/>
+      <c r="BZ2" s="23"/>
+      <c r="CA2" s="23"/>
+      <c r="CB2" s="23"/>
+      <c r="CC2" s="23"/>
+      <c r="CD2" s="23"/>
+      <c r="CE2" s="23"/>
+      <c r="CF2" s="23"/>
+      <c r="CG2" s="23"/>
+      <c r="CH2" s="23"/>
+      <c r="CI2" s="23"/>
+      <c r="CJ2" s="23"/>
+      <c r="CK2" s="23"/>
+      <c r="CL2" s="23"/>
+      <c r="CM2" s="23"/>
+      <c r="CN2" s="23"/>
+      <c r="CO2" s="23"/>
+      <c r="CP2" s="23"/>
+      <c r="CQ2" s="23"/>
+      <c r="CR2" s="23"/>
+      <c r="CS2" s="23"/>
+      <c r="CT2" s="23"/>
+      <c r="CU2" s="23"/>
+      <c r="CV2" s="23"/>
+      <c r="CW2" s="23"/>
+      <c r="CX2" s="23"/>
+      <c r="CY2" s="23"/>
+      <c r="CZ2" s="23"/>
+      <c r="DA2" s="23"/>
+      <c r="DB2" s="23"/>
+      <c r="DC2" s="23"/>
+      <c r="DD2" s="23"/>
+      <c r="DE2" s="23"/>
+      <c r="DF2" s="23"/>
+      <c r="DG2" s="23"/>
+      <c r="DH2" s="23"/>
+      <c r="DI2" s="23"/>
+      <c r="DJ2" s="23"/>
+      <c r="DK2" s="23"/>
+      <c r="DL2" s="23"/>
+      <c r="DM2" s="23"/>
+      <c r="DN2" s="23"/>
     </row>
     <row r="3" spans="1:118" x14ac:dyDescent="0.2">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="27" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
@@ -1493,119 +1628,119 @@
       <c r="C3"/>
       <c r="D3"/>
       <c r="E3"/>
-      <c r="I3" s="26"/>
-      <c r="J3" s="26"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="26"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="26"/>
-      <c r="O3" s="26"/>
-      <c r="P3" s="26"/>
-      <c r="Q3" s="26"/>
-      <c r="R3" s="26"/>
-      <c r="S3" s="26"/>
-      <c r="T3" s="26"/>
-      <c r="U3" s="26"/>
-      <c r="V3" s="26"/>
-      <c r="W3" s="26"/>
-      <c r="X3" s="26"/>
-      <c r="Y3" s="26"/>
-      <c r="Z3" s="26"/>
-      <c r="AA3" s="26"/>
-      <c r="AB3" s="26"/>
-      <c r="AC3" s="26"/>
-      <c r="AD3" s="26"/>
-      <c r="AE3" s="26"/>
-      <c r="AF3" s="26"/>
-      <c r="AG3" s="26"/>
-      <c r="AH3" s="26"/>
-      <c r="AI3" s="26"/>
-      <c r="AJ3" s="26"/>
-      <c r="AK3" s="26"/>
-      <c r="AL3" s="26"/>
-      <c r="AM3" s="26"/>
-      <c r="AN3" s="26"/>
-      <c r="AO3" s="26"/>
-      <c r="AP3" s="26"/>
-      <c r="AQ3" s="26"/>
-      <c r="AR3" s="26"/>
-      <c r="AS3" s="26"/>
-      <c r="AT3" s="26"/>
-      <c r="AU3" s="26"/>
-      <c r="AV3" s="26"/>
-      <c r="AW3" s="26"/>
-      <c r="AX3" s="26"/>
-      <c r="AY3" s="26"/>
-      <c r="AZ3" s="26"/>
-      <c r="BA3" s="26"/>
-      <c r="BB3" s="26"/>
-      <c r="BC3" s="26"/>
-      <c r="BD3" s="26"/>
-      <c r="BE3" s="26"/>
-      <c r="BF3" s="26"/>
-      <c r="BG3" s="26"/>
-      <c r="BH3" s="26"/>
-      <c r="BI3" s="26"/>
-      <c r="BJ3" s="26"/>
-      <c r="BK3" s="26"/>
-      <c r="BL3" s="26"/>
-      <c r="BM3" s="26"/>
-      <c r="BN3" s="26"/>
-      <c r="BO3" s="26"/>
-      <c r="BP3" s="26"/>
-      <c r="BQ3" s="26"/>
-      <c r="BR3" s="26"/>
-      <c r="BS3" s="26"/>
-      <c r="BT3" s="26"/>
-      <c r="BU3" s="26"/>
-      <c r="BV3" s="26"/>
-      <c r="BW3" s="26"/>
-      <c r="BX3" s="26"/>
-      <c r="BY3" s="26"/>
-      <c r="BZ3" s="26"/>
-      <c r="CA3" s="26"/>
-      <c r="CB3" s="26"/>
-      <c r="CC3" s="26"/>
-      <c r="CD3" s="26"/>
-      <c r="CE3" s="26"/>
-      <c r="CF3" s="26"/>
-      <c r="CG3" s="26"/>
-      <c r="CH3" s="26"/>
-      <c r="CI3" s="26"/>
-      <c r="CJ3" s="26"/>
-      <c r="CK3" s="26"/>
-      <c r="CL3" s="26"/>
-      <c r="CM3" s="26"/>
-      <c r="CN3" s="26"/>
-      <c r="CO3" s="26"/>
-      <c r="CP3" s="26"/>
-      <c r="CQ3" s="26"/>
-      <c r="CR3" s="26"/>
-      <c r="CS3" s="26"/>
-      <c r="CT3" s="26"/>
-      <c r="CU3" s="26"/>
-      <c r="CV3" s="26"/>
-      <c r="CW3" s="26"/>
-      <c r="CX3" s="26"/>
-      <c r="CY3" s="26"/>
-      <c r="CZ3" s="26"/>
-      <c r="DA3" s="26"/>
-      <c r="DB3" s="26"/>
-      <c r="DC3" s="26"/>
-      <c r="DD3" s="26"/>
-      <c r="DE3" s="26"/>
-      <c r="DF3" s="26"/>
-      <c r="DG3" s="26"/>
-      <c r="DH3" s="26"/>
-      <c r="DI3" s="26"/>
-      <c r="DJ3" s="26"/>
-      <c r="DK3" s="26"/>
-      <c r="DL3" s="26"/>
-      <c r="DM3" s="26"/>
-      <c r="DN3" s="26"/>
+      <c r="I3" s="25"/>
+      <c r="J3" s="25"/>
+      <c r="K3" s="25"/>
+      <c r="L3" s="25"/>
+      <c r="M3" s="25"/>
+      <c r="N3" s="25"/>
+      <c r="O3" s="25"/>
+      <c r="P3" s="25"/>
+      <c r="Q3" s="25"/>
+      <c r="R3" s="25"/>
+      <c r="S3" s="25"/>
+      <c r="T3" s="25"/>
+      <c r="U3" s="25"/>
+      <c r="V3" s="25"/>
+      <c r="W3" s="25"/>
+      <c r="X3" s="25"/>
+      <c r="Y3" s="25"/>
+      <c r="Z3" s="25"/>
+      <c r="AA3" s="25"/>
+      <c r="AB3" s="25"/>
+      <c r="AC3" s="25"/>
+      <c r="AD3" s="25"/>
+      <c r="AE3" s="25"/>
+      <c r="AF3" s="25"/>
+      <c r="AG3" s="25"/>
+      <c r="AH3" s="25"/>
+      <c r="AI3" s="25"/>
+      <c r="AJ3" s="25"/>
+      <c r="AK3" s="25"/>
+      <c r="AL3" s="25"/>
+      <c r="AM3" s="25"/>
+      <c r="AN3" s="25"/>
+      <c r="AO3" s="25"/>
+      <c r="AP3" s="25"/>
+      <c r="AQ3" s="25"/>
+      <c r="AR3" s="25"/>
+      <c r="AS3" s="25"/>
+      <c r="AT3" s="25"/>
+      <c r="AU3" s="25"/>
+      <c r="AV3" s="25"/>
+      <c r="AW3" s="25"/>
+      <c r="AX3" s="25"/>
+      <c r="AY3" s="25"/>
+      <c r="AZ3" s="25"/>
+      <c r="BA3" s="25"/>
+      <c r="BB3" s="25"/>
+      <c r="BC3" s="25"/>
+      <c r="BD3" s="25"/>
+      <c r="BE3" s="25"/>
+      <c r="BF3" s="25"/>
+      <c r="BG3" s="25"/>
+      <c r="BH3" s="25"/>
+      <c r="BI3" s="25"/>
+      <c r="BJ3" s="25"/>
+      <c r="BK3" s="25"/>
+      <c r="BL3" s="25"/>
+      <c r="BM3" s="25"/>
+      <c r="BN3" s="25"/>
+      <c r="BO3" s="25"/>
+      <c r="BP3" s="25"/>
+      <c r="BQ3" s="25"/>
+      <c r="BR3" s="25"/>
+      <c r="BS3" s="25"/>
+      <c r="BT3" s="25"/>
+      <c r="BU3" s="25"/>
+      <c r="BV3" s="25"/>
+      <c r="BW3" s="25"/>
+      <c r="BX3" s="25"/>
+      <c r="BY3" s="25"/>
+      <c r="BZ3" s="25"/>
+      <c r="CA3" s="25"/>
+      <c r="CB3" s="25"/>
+      <c r="CC3" s="25"/>
+      <c r="CD3" s="25"/>
+      <c r="CE3" s="25"/>
+      <c r="CF3" s="25"/>
+      <c r="CG3" s="25"/>
+      <c r="CH3" s="25"/>
+      <c r="CI3" s="25"/>
+      <c r="CJ3" s="25"/>
+      <c r="CK3" s="25"/>
+      <c r="CL3" s="25"/>
+      <c r="CM3" s="25"/>
+      <c r="CN3" s="25"/>
+      <c r="CO3" s="25"/>
+      <c r="CP3" s="25"/>
+      <c r="CQ3" s="25"/>
+      <c r="CR3" s="25"/>
+      <c r="CS3" s="25"/>
+      <c r="CT3" s="25"/>
+      <c r="CU3" s="25"/>
+      <c r="CV3" s="25"/>
+      <c r="CW3" s="25"/>
+      <c r="CX3" s="25"/>
+      <c r="CY3" s="25"/>
+      <c r="CZ3" s="25"/>
+      <c r="DA3" s="25"/>
+      <c r="DB3" s="25"/>
+      <c r="DC3" s="25"/>
+      <c r="DD3" s="25"/>
+      <c r="DE3" s="25"/>
+      <c r="DF3" s="25"/>
+      <c r="DG3" s="25"/>
+      <c r="DH3" s="25"/>
+      <c r="DI3" s="25"/>
+      <c r="DJ3" s="25"/>
+      <c r="DK3" s="25"/>
+      <c r="DL3" s="25"/>
+      <c r="DM3" s="25"/>
+      <c r="DN3" s="25"/>
     </row>
     <row r="4" spans="1:118" x14ac:dyDescent="0.2">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="27" t="s">
         <v>3</v>
       </c>
       <c r="B4" t="s">
@@ -1616,7 +1751,7 @@
       <c r="E4"/>
     </row>
     <row r="5" spans="1:118" x14ac:dyDescent="0.2">
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="31" t="s">
         <v>15</v>
       </c>
       <c r="C5"/>
@@ -1655,7 +1790,7 @@
   <sheetData>
     <row r="1" spans="1:8" s="4" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -1670,7 +1805,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="66" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="24" t="s">
         <v>16</v>
       </c>
       <c r="B2" t="s">
@@ -1678,7 +1813,7 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="27" t="s">
         <v>21</v>
       </c>
       <c r="B3" t="s">
@@ -1686,7 +1821,7 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="27" t="s">
         <v>21</v>
       </c>
       <c r="B4" t="s">
@@ -1694,7 +1829,7 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="31" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1707,7 +1842,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E893F90-1EC7-764C-B747-7920FCEC73CB}">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.33203125" customWidth="1"/>
@@ -1720,24 +1855,25 @@
     <col min="9" max="9" width="18.33203125" customWidth="1"/>
     <col min="10" max="10" width="20.5" customWidth="1"/>
     <col min="11" max="11" width="16.6640625" customWidth="1"/>
+    <col min="15" max="15" width="18.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="B1" s="16" t="s">
-        <v>30</v>
+    <row r="1" spans="1:16" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>29</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="27" t="s">
+    <row r="2" spans="1:16" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="17" t="e">
+      <c r="B2" s="16" t="e">
         <f>VLOOKUP(A2,'codage tribunal'!A:B,2,FALSE)</f>
         <v>#N/A</v>
       </c>
@@ -1745,13 +1881,30 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row r="3" spans="1:16" ht="40" x14ac:dyDescent="0.2">
+      <c r="C3" s="9"/>
+      <c r="E3" s="39" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="41"/>
+      <c r="J3" s="39" t="s">
+        <v>57</v>
+      </c>
+      <c r="K3" s="40"/>
+      <c r="L3" s="40"/>
+      <c r="M3" s="40"/>
+      <c r="N3" s="41"/>
+      <c r="O3" s="42" t="s">
+        <v>58</v>
+      </c>
+      <c r="P3" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="9"/>
-    </row>
-    <row r="4" spans="1:12" ht="32" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:16" ht="80" x14ac:dyDescent="0.2">
       <c r="A4" s="10"/>
       <c r="C4" s="10"/>
       <c r="D4" s="11"/>
@@ -1764,70 +1917,126 @@
       <c r="G4" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="13" t="s">
+      <c r="H4" s="43" t="s">
+        <v>59</v>
+      </c>
+      <c r="I4" s="44" t="s">
+        <v>60</v>
+      </c>
+      <c r="J4" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="K4" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="J4" s="13" t="s">
+      <c r="L4" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="K4" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="L4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5" s="15"/>
-      <c r="C5" s="19" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" s="18" t="s">
+      <c r="M4" s="43" t="s">
+        <v>59</v>
+      </c>
+      <c r="N4" s="44" t="s">
+        <v>61</v>
+      </c>
+      <c r="O4" s="45" t="s">
+        <v>59</v>
+      </c>
+      <c r="P4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A5" s="14"/>
+      <c r="C5" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="22" t="e">
+      <c r="D5" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="21" t="e">
         <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-TIT",'ETPT Format DDG'!$C:$C,$A$2)</f>
         <v>#N/A</v>
       </c>
-      <c r="F5" s="20" t="e">
+      <c r="F5" s="19" t="e">
         <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$2)</f>
         <v>#N/A</v>
       </c>
-      <c r="G5" s="20" t="e">
+      <c r="G5" s="19" t="e">
         <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$2)</f>
         <v>#N/A</v>
       </c>
-      <c r="H5" s="20" t="e">
+      <c r="H5" s="19" t="e">
+        <f>SUMIFS(
+INDEX('ETPT Format DDG'!$A:$DU,
+,
+IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))
+),'ETPT Format DDG'!$I:$I,"C",
+'ETPT Format DDG'!$C:$C,$A$2,
+'ETPT Format DDG'!$G:$G,"Magistrat")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I5" s="46" t="e">
+        <f>SUMIFS(
+INDEX('ETPT Format DDG'!$A:$DU,
+,
+IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))
+),
+'ETPT Format DDG'!$C:$C,$A$2,
+'ETPT Format DDG'!$G:$G,"Magistrat")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J5" s="19" t="e">
         <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"F-TIT",'ETPT Format DDG'!$C:$C,$A$2)</f>
         <v>#N/A</v>
       </c>
-      <c r="I5" s="20" t="e">
+      <c r="K5" s="19" t="e">
         <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"F-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$2)</f>
         <v>#N/A</v>
       </c>
-      <c r="J5" s="20" t="e">
+      <c r="L5" s="19" t="e">
         <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"F-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$2)</f>
         <v>#N/A</v>
       </c>
-      <c r="K5" s="21" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"C",'ETPT Format DDG'!$C:$C,$A$2)</f>
+      <c r="M5" s="20" t="e">
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"C",'ETPT Format DDG'!$C:$C,$A$2,'ETPT Format DDG'!$G:$G,"Greffe")</f>
         <v>#N/A</v>
       </c>
-      <c r="L5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="L6" t="s">
+      <c r="N5" s="46" t="e">
+        <f>SUMIFS(
+INDEX('ETPT Format DDG'!$A:$DU,
+,
+IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))
+),
+'ETPT Format DDG'!$C:$C,$A$2,
+'ETPT Format DDG'!$G:$G,"Greffe")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="O5" s="20" t="e">
+        <f>SUMIFS(
+INDEX('ETPT Format DDG'!$A:$DU,
+,
+IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))
+),'ETPT Format DDG'!$I:$I,"C",
+'ETPT Format DDG'!$C:$C,$A$2,
+'ETPT Format DDG'!$G:$G,"Autour du magistrat")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="P5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="P6" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:K150">
-    <cfRule type="expression" dxfId="0" priority="1">
+  <mergeCells count="2">
+    <mergeCell ref="E3:I3"/>
+    <mergeCell ref="J3:N3"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C5:O150">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>AND(ISBLANK($C5)=FALSE,ISBLANK($D5)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1858,124 +2067,124 @@
   <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.1640625" style="24" customWidth="1"/>
-    <col min="2" max="2" width="7.33203125" style="24" customWidth="1"/>
-    <col min="3" max="9" width="10.83203125" style="24"/>
-    <col min="10" max="10" width="71.1640625" style="24" customWidth="1"/>
-    <col min="11" max="16384" width="10.83203125" style="24"/>
+    <col min="1" max="1" width="8.1640625" style="23" customWidth="1"/>
+    <col min="2" max="2" width="7.33203125" style="23" customWidth="1"/>
+    <col min="3" max="9" width="10.83203125" style="23"/>
+    <col min="10" max="10" width="71.1640625" style="23" customWidth="1"/>
+    <col min="11" max="16384" width="10.83203125" style="23"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="29" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="35" t="s">
+    <row r="1" spans="1:10" s="28" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+    </row>
+    <row r="2" spans="1:10" s="10" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-    </row>
-    <row r="2" spans="1:10" s="10" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="30" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="34" t="s">
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+    </row>
+    <row r="3" spans="1:10" s="10" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="29"/>
+      <c r="B3" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
-    </row>
-    <row r="3" spans="1:10" s="10" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="30"/>
-      <c r="B3" s="31" t="s">
+      <c r="C3" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
+      <c r="J3" s="32"/>
+    </row>
+    <row r="4" spans="1:10" s="10" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="29"/>
+      <c r="B4" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="37"/>
-      <c r="H3" s="37"/>
-      <c r="I3" s="37"/>
-      <c r="J3" s="37"/>
-    </row>
-    <row r="4" spans="1:10" s="10" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="30"/>
-      <c r="B4" s="31" t="s">
+      <c r="C4" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="37" t="s">
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="32"/>
+      <c r="J4" s="32"/>
+    </row>
+    <row r="5" spans="1:10" s="10" customFormat="1" ht="43" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="29"/>
+      <c r="B5" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="D4" s="37"/>
-      <c r="E4" s="37"/>
-      <c r="F4" s="37"/>
-      <c r="G4" s="37"/>
-      <c r="H4" s="37"/>
-      <c r="I4" s="37"/>
-      <c r="J4" s="37"/>
-    </row>
-    <row r="5" spans="1:10" s="10" customFormat="1" ht="43" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="30"/>
-      <c r="B5" s="31" t="s">
+      <c r="C5" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="C5" s="37" t="s">
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+    </row>
+    <row r="6" spans="1:10" s="10" customFormat="1" ht="37" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="37"/>
-      <c r="I5" s="37"/>
-      <c r="J5" s="37"/>
-    </row>
-    <row r="6" spans="1:10" s="10" customFormat="1" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="31" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="37" t="s">
+      <c r="C6" s="32"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
+    </row>
+    <row r="7" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="29"/>
+      <c r="B7" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="37"/>
-      <c r="I6" s="37"/>
-      <c r="J6" s="37"/>
-    </row>
-    <row r="7" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="30"/>
-      <c r="B7" s="34" t="s">
-        <v>47</v>
-      </c>
-      <c r="C7" s="34"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="34"/>
-      <c r="F7" s="34"/>
-      <c r="G7" s="34"/>
-      <c r="H7" s="34"/>
-      <c r="I7" s="34"/>
-      <c r="J7" s="34"/>
+      <c r="C7" s="35"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="35"/>
+      <c r="F7" s="35"/>
+      <c r="G7" s="35"/>
+      <c r="H7" s="35"/>
+      <c r="I7" s="35"/>
+      <c r="J7" s="35"/>
     </row>
     <row r="8" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="38" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C8" s="38"/>
       <c r="D8" s="38"/>
@@ -2001,7 +2210,7 @@
     </row>
     <row r="10" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="38" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C10" s="38"/>
       <c r="D10" s="38"/>
@@ -2014,7 +2223,7 @@
     </row>
     <row r="11" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="38" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C11" s="38"/>
       <c r="D11" s="38"/>
@@ -2026,98 +2235,99 @@
       <c r="J11" s="38"/>
     </row>
     <row r="12" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="30" t="s">
+      <c r="A12" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="33" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="34"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
+      <c r="G12" s="34"/>
+      <c r="H12" s="34"/>
+      <c r="I12" s="34"/>
+      <c r="J12" s="34"/>
+    </row>
+    <row r="13" spans="1:10" s="10" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="32" t="s">
         <v>51</v>
       </c>
-      <c r="C12" s="33"/>
-      <c r="D12" s="33"/>
-      <c r="E12" s="33"/>
-      <c r="F12" s="33"/>
-      <c r="G12" s="33"/>
-      <c r="H12" s="33"/>
-      <c r="I12" s="33"/>
-      <c r="J12" s="33"/>
-    </row>
-    <row r="13" spans="1:10" s="10" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="31" t="s">
-        <v>11</v>
-      </c>
-      <c r="C13" s="37" t="s">
+      <c r="D13" s="32"/>
+      <c r="E13" s="32"/>
+      <c r="F13" s="32"/>
+      <c r="G13" s="32"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="32"/>
+    </row>
+    <row r="14" spans="1:10" s="10" customFormat="1" ht="56" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="32" t="s">
         <v>52</v>
       </c>
-      <c r="D13" s="37"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="37"/>
-      <c r="G13" s="37"/>
-      <c r="H13" s="37"/>
-      <c r="I13" s="37"/>
-      <c r="J13" s="37"/>
-    </row>
-    <row r="14" spans="1:10" s="10" customFormat="1" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="31" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" s="37" t="s">
+      <c r="D14" s="32"/>
+      <c r="E14" s="32"/>
+      <c r="F14" s="32"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="32"/>
+      <c r="I14" s="32"/>
+      <c r="J14" s="32"/>
+    </row>
+    <row r="15" spans="1:10" s="10" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="30" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="32" t="s">
         <v>53</v>
       </c>
-      <c r="D14" s="37"/>
-      <c r="E14" s="37"/>
-      <c r="F14" s="37"/>
-      <c r="G14" s="37"/>
-      <c r="H14" s="37"/>
-      <c r="I14" s="37"/>
-      <c r="J14" s="37"/>
-    </row>
-    <row r="15" spans="1:10" s="10" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="31" t="s">
-        <v>13</v>
-      </c>
-      <c r="C15" s="37" t="s">
+      <c r="D15" s="32"/>
+      <c r="E15" s="32"/>
+      <c r="F15" s="32"/>
+      <c r="G15" s="32"/>
+      <c r="H15" s="32"/>
+      <c r="I15" s="32"/>
+      <c r="J15" s="32"/>
+    </row>
+    <row r="16" spans="1:10" s="10" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="32" t="s">
         <v>54</v>
       </c>
-      <c r="D15" s="37"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="37"/>
-      <c r="G15" s="37"/>
-      <c r="H15" s="37"/>
-      <c r="I15" s="37"/>
-      <c r="J15" s="37"/>
-    </row>
-    <row r="16" spans="1:10" s="10" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="B16" s="37" t="s">
+      <c r="C16" s="32"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
+    </row>
+    <row r="18" spans="1:10" s="28" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="C16" s="37"/>
-      <c r="D16" s="37"/>
-      <c r="E16" s="37"/>
-      <c r="F16" s="37"/>
-      <c r="G16" s="37"/>
-      <c r="H16" s="37"/>
-      <c r="I16" s="37"/>
-      <c r="J16" s="37"/>
-    </row>
-    <row r="18" spans="1:10" s="29" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="35" t="s">
-        <v>56</v>
-      </c>
-      <c r="B18" s="36"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="36"/>
-      <c r="F18" s="36"/>
-      <c r="G18" s="36"/>
-      <c r="H18" s="36"/>
-      <c r="I18" s="36"/>
-      <c r="J18" s="36"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="37"/>
+      <c r="I18" s="37"/>
+      <c r="J18" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="C13:J13"/>
     <mergeCell ref="C14:J14"/>
     <mergeCell ref="B12:J12"/>
     <mergeCell ref="B7:J7"/>
@@ -2134,7 +2344,6 @@
     <mergeCell ref="B9:J9"/>
     <mergeCell ref="B10:J10"/>
     <mergeCell ref="B11:J11"/>
-    <mergeCell ref="C13:J13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
update DDG template 2
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmy/Desktop/Betagouv/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85F89413-D477-E346-84BF-35A1BA14109B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24816E1E-27A1-9147-92A5-D82FD9079116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24580" windowHeight="14560" activeTab="2" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24580" windowHeight="14560" activeTab="5" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ETPT A-JUST" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
update popin extracteur & formatage fichier ETPT
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10611"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10709"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmy/Desktop/Betagouv/a-just/front/src/assets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24816E1E-27A1-9147-92A5-D82FD9079116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47C34238-0F47-A349-9585-09C806FD1DFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24580" windowHeight="14560" activeTab="5" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="22480" windowHeight="17620" activeTab="5" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ETPT A-JUST" sheetId="1" r:id="rId1"/>
@@ -592,11 +592,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="5">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0.000_-;\-* #,##0.000_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="General;General;\-"/>
-    <numFmt numFmtId="167" formatCode="0.###;0.###;\-"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0.000_-;\-* #,##0.000_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="General;General;\-"/>
+    <numFmt numFmtId="168" formatCode="0.###;0.###;\-"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -880,8 +880,8 @@
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -918,10 +918,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -933,19 +933,13 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -957,11 +951,11 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -974,6 +968,30 @@
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="12" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -995,53 +1013,20 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="12" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="4" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
-    <cellStyle name="Comma" xfId="3" builtinId="3"/>
     <cellStyle name="Comma 2" xfId="2" xr:uid="{C877C5E8-FCBF-114F-9ECB-F75EF7C9C0EB}"/>
+    <cellStyle name="Milliers" xfId="3" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <fill>
         <patternFill>
@@ -1169,7 +1154,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1495,131 +1480,131 @@
       </c>
     </row>
     <row r="2" spans="1:118" ht="66" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="23"/>
-      <c r="O2" s="23"/>
-      <c r="P2" s="23"/>
-      <c r="Q2" s="23"/>
-      <c r="R2" s="23"/>
-      <c r="S2" s="23"/>
-      <c r="T2" s="23"/>
-      <c r="U2" s="23"/>
-      <c r="V2" s="23"/>
-      <c r="W2" s="23"/>
-      <c r="X2" s="23"/>
-      <c r="Y2" s="23"/>
-      <c r="Z2" s="23"/>
-      <c r="AA2" s="23"/>
-      <c r="AB2" s="23"/>
-      <c r="AC2" s="23"/>
-      <c r="AD2" s="23"/>
-      <c r="AE2" s="23"/>
-      <c r="AF2" s="23"/>
-      <c r="AG2" s="23"/>
-      <c r="AH2" s="23"/>
-      <c r="AI2" s="23"/>
-      <c r="AJ2" s="23"/>
-      <c r="AK2" s="23"/>
-      <c r="AL2" s="23"/>
-      <c r="AM2" s="23"/>
-      <c r="AN2" s="23"/>
-      <c r="AO2" s="23"/>
-      <c r="AP2" s="23"/>
-      <c r="AQ2" s="23"/>
-      <c r="AR2" s="23"/>
-      <c r="AS2" s="23"/>
-      <c r="AT2" s="23"/>
-      <c r="AU2" s="23"/>
-      <c r="AV2" s="23"/>
-      <c r="AW2" s="23"/>
-      <c r="AX2" s="23"/>
-      <c r="AY2" s="23"/>
-      <c r="AZ2" s="23"/>
-      <c r="BA2" s="23"/>
-      <c r="BB2" s="23"/>
-      <c r="BC2" s="23"/>
-      <c r="BD2" s="23"/>
-      <c r="BE2" s="23"/>
-      <c r="BF2" s="23"/>
-      <c r="BG2" s="23"/>
-      <c r="BH2" s="23"/>
-      <c r="BI2" s="23"/>
-      <c r="BJ2" s="23"/>
-      <c r="BK2" s="23"/>
-      <c r="BL2" s="23"/>
-      <c r="BM2" s="23"/>
-      <c r="BN2" s="23"/>
-      <c r="BO2" s="23"/>
-      <c r="BP2" s="23"/>
-      <c r="BQ2" s="23"/>
-      <c r="BR2" s="23"/>
-      <c r="BS2" s="23"/>
-      <c r="BT2" s="23"/>
-      <c r="BU2" s="23"/>
-      <c r="BV2" s="23"/>
-      <c r="BW2" s="23"/>
-      <c r="BX2" s="23"/>
-      <c r="BY2" s="23"/>
-      <c r="BZ2" s="23"/>
-      <c r="CA2" s="23"/>
-      <c r="CB2" s="23"/>
-      <c r="CC2" s="23"/>
-      <c r="CD2" s="23"/>
-      <c r="CE2" s="23"/>
-      <c r="CF2" s="23"/>
-      <c r="CG2" s="23"/>
-      <c r="CH2" s="23"/>
-      <c r="CI2" s="23"/>
-      <c r="CJ2" s="23"/>
-      <c r="CK2" s="23"/>
-      <c r="CL2" s="23"/>
-      <c r="CM2" s="23"/>
-      <c r="CN2" s="23"/>
-      <c r="CO2" s="23"/>
-      <c r="CP2" s="23"/>
-      <c r="CQ2" s="23"/>
-      <c r="CR2" s="23"/>
-      <c r="CS2" s="23"/>
-      <c r="CT2" s="23"/>
-      <c r="CU2" s="23"/>
-      <c r="CV2" s="23"/>
-      <c r="CW2" s="23"/>
-      <c r="CX2" s="23"/>
-      <c r="CY2" s="23"/>
-      <c r="CZ2" s="23"/>
-      <c r="DA2" s="23"/>
-      <c r="DB2" s="23"/>
-      <c r="DC2" s="23"/>
-      <c r="DD2" s="23"/>
-      <c r="DE2" s="23"/>
-      <c r="DF2" s="23"/>
-      <c r="DG2" s="23"/>
-      <c r="DH2" s="23"/>
-      <c r="DI2" s="23"/>
-      <c r="DJ2" s="23"/>
-      <c r="DK2" s="23"/>
-      <c r="DL2" s="23"/>
-      <c r="DM2" s="23"/>
-      <c r="DN2" s="23"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="21"/>
+      <c r="L2" s="21"/>
+      <c r="M2" s="21"/>
+      <c r="N2" s="21"/>
+      <c r="O2" s="21"/>
+      <c r="P2" s="21"/>
+      <c r="Q2" s="21"/>
+      <c r="R2" s="21"/>
+      <c r="S2" s="21"/>
+      <c r="T2" s="21"/>
+      <c r="U2" s="21"/>
+      <c r="V2" s="21"/>
+      <c r="W2" s="21"/>
+      <c r="X2" s="21"/>
+      <c r="Y2" s="21"/>
+      <c r="Z2" s="21"/>
+      <c r="AA2" s="21"/>
+      <c r="AB2" s="21"/>
+      <c r="AC2" s="21"/>
+      <c r="AD2" s="21"/>
+      <c r="AE2" s="21"/>
+      <c r="AF2" s="21"/>
+      <c r="AG2" s="21"/>
+      <c r="AH2" s="21"/>
+      <c r="AI2" s="21"/>
+      <c r="AJ2" s="21"/>
+      <c r="AK2" s="21"/>
+      <c r="AL2" s="21"/>
+      <c r="AM2" s="21"/>
+      <c r="AN2" s="21"/>
+      <c r="AO2" s="21"/>
+      <c r="AP2" s="21"/>
+      <c r="AQ2" s="21"/>
+      <c r="AR2" s="21"/>
+      <c r="AS2" s="21"/>
+      <c r="AT2" s="21"/>
+      <c r="AU2" s="21"/>
+      <c r="AV2" s="21"/>
+      <c r="AW2" s="21"/>
+      <c r="AX2" s="21"/>
+      <c r="AY2" s="21"/>
+      <c r="AZ2" s="21"/>
+      <c r="BA2" s="21"/>
+      <c r="BB2" s="21"/>
+      <c r="BC2" s="21"/>
+      <c r="BD2" s="21"/>
+      <c r="BE2" s="21"/>
+      <c r="BF2" s="21"/>
+      <c r="BG2" s="21"/>
+      <c r="BH2" s="21"/>
+      <c r="BI2" s="21"/>
+      <c r="BJ2" s="21"/>
+      <c r="BK2" s="21"/>
+      <c r="BL2" s="21"/>
+      <c r="BM2" s="21"/>
+      <c r="BN2" s="21"/>
+      <c r="BO2" s="21"/>
+      <c r="BP2" s="21"/>
+      <c r="BQ2" s="21"/>
+      <c r="BR2" s="21"/>
+      <c r="BS2" s="21"/>
+      <c r="BT2" s="21"/>
+      <c r="BU2" s="21"/>
+      <c r="BV2" s="21"/>
+      <c r="BW2" s="21"/>
+      <c r="BX2" s="21"/>
+      <c r="BY2" s="21"/>
+      <c r="BZ2" s="21"/>
+      <c r="CA2" s="21"/>
+      <c r="CB2" s="21"/>
+      <c r="CC2" s="21"/>
+      <c r="CD2" s="21"/>
+      <c r="CE2" s="21"/>
+      <c r="CF2" s="21"/>
+      <c r="CG2" s="21"/>
+      <c r="CH2" s="21"/>
+      <c r="CI2" s="21"/>
+      <c r="CJ2" s="21"/>
+      <c r="CK2" s="21"/>
+      <c r="CL2" s="21"/>
+      <c r="CM2" s="21"/>
+      <c r="CN2" s="21"/>
+      <c r="CO2" s="21"/>
+      <c r="CP2" s="21"/>
+      <c r="CQ2" s="21"/>
+      <c r="CR2" s="21"/>
+      <c r="CS2" s="21"/>
+      <c r="CT2" s="21"/>
+      <c r="CU2" s="21"/>
+      <c r="CV2" s="21"/>
+      <c r="CW2" s="21"/>
+      <c r="CX2" s="21"/>
+      <c r="CY2" s="21"/>
+      <c r="CZ2" s="21"/>
+      <c r="DA2" s="21"/>
+      <c r="DB2" s="21"/>
+      <c r="DC2" s="21"/>
+      <c r="DD2" s="21"/>
+      <c r="DE2" s="21"/>
+      <c r="DF2" s="21"/>
+      <c r="DG2" s="21"/>
+      <c r="DH2" s="21"/>
+      <c r="DI2" s="21"/>
+      <c r="DJ2" s="21"/>
+      <c r="DK2" s="21"/>
+      <c r="DL2" s="21"/>
+      <c r="DM2" s="21"/>
+      <c r="DN2" s="21"/>
     </row>
     <row r="3" spans="1:118" x14ac:dyDescent="0.2">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="25" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
@@ -1628,119 +1613,119 @@
       <c r="C3"/>
       <c r="D3"/>
       <c r="E3"/>
-      <c r="I3" s="25"/>
-      <c r="J3" s="25"/>
-      <c r="K3" s="25"/>
-      <c r="L3" s="25"/>
-      <c r="M3" s="25"/>
-      <c r="N3" s="25"/>
-      <c r="O3" s="25"/>
-      <c r="P3" s="25"/>
-      <c r="Q3" s="25"/>
-      <c r="R3" s="25"/>
-      <c r="S3" s="25"/>
-      <c r="T3" s="25"/>
-      <c r="U3" s="25"/>
-      <c r="V3" s="25"/>
-      <c r="W3" s="25"/>
-      <c r="X3" s="25"/>
-      <c r="Y3" s="25"/>
-      <c r="Z3" s="25"/>
-      <c r="AA3" s="25"/>
-      <c r="AB3" s="25"/>
-      <c r="AC3" s="25"/>
-      <c r="AD3" s="25"/>
-      <c r="AE3" s="25"/>
-      <c r="AF3" s="25"/>
-      <c r="AG3" s="25"/>
-      <c r="AH3" s="25"/>
-      <c r="AI3" s="25"/>
-      <c r="AJ3" s="25"/>
-      <c r="AK3" s="25"/>
-      <c r="AL3" s="25"/>
-      <c r="AM3" s="25"/>
-      <c r="AN3" s="25"/>
-      <c r="AO3" s="25"/>
-      <c r="AP3" s="25"/>
-      <c r="AQ3" s="25"/>
-      <c r="AR3" s="25"/>
-      <c r="AS3" s="25"/>
-      <c r="AT3" s="25"/>
-      <c r="AU3" s="25"/>
-      <c r="AV3" s="25"/>
-      <c r="AW3" s="25"/>
-      <c r="AX3" s="25"/>
-      <c r="AY3" s="25"/>
-      <c r="AZ3" s="25"/>
-      <c r="BA3" s="25"/>
-      <c r="BB3" s="25"/>
-      <c r="BC3" s="25"/>
-      <c r="BD3" s="25"/>
-      <c r="BE3" s="25"/>
-      <c r="BF3" s="25"/>
-      <c r="BG3" s="25"/>
-      <c r="BH3" s="25"/>
-      <c r="BI3" s="25"/>
-      <c r="BJ3" s="25"/>
-      <c r="BK3" s="25"/>
-      <c r="BL3" s="25"/>
-      <c r="BM3" s="25"/>
-      <c r="BN3" s="25"/>
-      <c r="BO3" s="25"/>
-      <c r="BP3" s="25"/>
-      <c r="BQ3" s="25"/>
-      <c r="BR3" s="25"/>
-      <c r="BS3" s="25"/>
-      <c r="BT3" s="25"/>
-      <c r="BU3" s="25"/>
-      <c r="BV3" s="25"/>
-      <c r="BW3" s="25"/>
-      <c r="BX3" s="25"/>
-      <c r="BY3" s="25"/>
-      <c r="BZ3" s="25"/>
-      <c r="CA3" s="25"/>
-      <c r="CB3" s="25"/>
-      <c r="CC3" s="25"/>
-      <c r="CD3" s="25"/>
-      <c r="CE3" s="25"/>
-      <c r="CF3" s="25"/>
-      <c r="CG3" s="25"/>
-      <c r="CH3" s="25"/>
-      <c r="CI3" s="25"/>
-      <c r="CJ3" s="25"/>
-      <c r="CK3" s="25"/>
-      <c r="CL3" s="25"/>
-      <c r="CM3" s="25"/>
-      <c r="CN3" s="25"/>
-      <c r="CO3" s="25"/>
-      <c r="CP3" s="25"/>
-      <c r="CQ3" s="25"/>
-      <c r="CR3" s="25"/>
-      <c r="CS3" s="25"/>
-      <c r="CT3" s="25"/>
-      <c r="CU3" s="25"/>
-      <c r="CV3" s="25"/>
-      <c r="CW3" s="25"/>
-      <c r="CX3" s="25"/>
-      <c r="CY3" s="25"/>
-      <c r="CZ3" s="25"/>
-      <c r="DA3" s="25"/>
-      <c r="DB3" s="25"/>
-      <c r="DC3" s="25"/>
-      <c r="DD3" s="25"/>
-      <c r="DE3" s="25"/>
-      <c r="DF3" s="25"/>
-      <c r="DG3" s="25"/>
-      <c r="DH3" s="25"/>
-      <c r="DI3" s="25"/>
-      <c r="DJ3" s="25"/>
-      <c r="DK3" s="25"/>
-      <c r="DL3" s="25"/>
-      <c r="DM3" s="25"/>
-      <c r="DN3" s="25"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="23"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="23"/>
+      <c r="Q3" s="23"/>
+      <c r="R3" s="23"/>
+      <c r="S3" s="23"/>
+      <c r="T3" s="23"/>
+      <c r="U3" s="23"/>
+      <c r="V3" s="23"/>
+      <c r="W3" s="23"/>
+      <c r="X3" s="23"/>
+      <c r="Y3" s="23"/>
+      <c r="Z3" s="23"/>
+      <c r="AA3" s="23"/>
+      <c r="AB3" s="23"/>
+      <c r="AC3" s="23"/>
+      <c r="AD3" s="23"/>
+      <c r="AE3" s="23"/>
+      <c r="AF3" s="23"/>
+      <c r="AG3" s="23"/>
+      <c r="AH3" s="23"/>
+      <c r="AI3" s="23"/>
+      <c r="AJ3" s="23"/>
+      <c r="AK3" s="23"/>
+      <c r="AL3" s="23"/>
+      <c r="AM3" s="23"/>
+      <c r="AN3" s="23"/>
+      <c r="AO3" s="23"/>
+      <c r="AP3" s="23"/>
+      <c r="AQ3" s="23"/>
+      <c r="AR3" s="23"/>
+      <c r="AS3" s="23"/>
+      <c r="AT3" s="23"/>
+      <c r="AU3" s="23"/>
+      <c r="AV3" s="23"/>
+      <c r="AW3" s="23"/>
+      <c r="AX3" s="23"/>
+      <c r="AY3" s="23"/>
+      <c r="AZ3" s="23"/>
+      <c r="BA3" s="23"/>
+      <c r="BB3" s="23"/>
+      <c r="BC3" s="23"/>
+      <c r="BD3" s="23"/>
+      <c r="BE3" s="23"/>
+      <c r="BF3" s="23"/>
+      <c r="BG3" s="23"/>
+      <c r="BH3" s="23"/>
+      <c r="BI3" s="23"/>
+      <c r="BJ3" s="23"/>
+      <c r="BK3" s="23"/>
+      <c r="BL3" s="23"/>
+      <c r="BM3" s="23"/>
+      <c r="BN3" s="23"/>
+      <c r="BO3" s="23"/>
+      <c r="BP3" s="23"/>
+      <c r="BQ3" s="23"/>
+      <c r="BR3" s="23"/>
+      <c r="BS3" s="23"/>
+      <c r="BT3" s="23"/>
+      <c r="BU3" s="23"/>
+      <c r="BV3" s="23"/>
+      <c r="BW3" s="23"/>
+      <c r="BX3" s="23"/>
+      <c r="BY3" s="23"/>
+      <c r="BZ3" s="23"/>
+      <c r="CA3" s="23"/>
+      <c r="CB3" s="23"/>
+      <c r="CC3" s="23"/>
+      <c r="CD3" s="23"/>
+      <c r="CE3" s="23"/>
+      <c r="CF3" s="23"/>
+      <c r="CG3" s="23"/>
+      <c r="CH3" s="23"/>
+      <c r="CI3" s="23"/>
+      <c r="CJ3" s="23"/>
+      <c r="CK3" s="23"/>
+      <c r="CL3" s="23"/>
+      <c r="CM3" s="23"/>
+      <c r="CN3" s="23"/>
+      <c r="CO3" s="23"/>
+      <c r="CP3" s="23"/>
+      <c r="CQ3" s="23"/>
+      <c r="CR3" s="23"/>
+      <c r="CS3" s="23"/>
+      <c r="CT3" s="23"/>
+      <c r="CU3" s="23"/>
+      <c r="CV3" s="23"/>
+      <c r="CW3" s="23"/>
+      <c r="CX3" s="23"/>
+      <c r="CY3" s="23"/>
+      <c r="CZ3" s="23"/>
+      <c r="DA3" s="23"/>
+      <c r="DB3" s="23"/>
+      <c r="DC3" s="23"/>
+      <c r="DD3" s="23"/>
+      <c r="DE3" s="23"/>
+      <c r="DF3" s="23"/>
+      <c r="DG3" s="23"/>
+      <c r="DH3" s="23"/>
+      <c r="DI3" s="23"/>
+      <c r="DJ3" s="23"/>
+      <c r="DK3" s="23"/>
+      <c r="DL3" s="23"/>
+      <c r="DM3" s="23"/>
+      <c r="DN3" s="23"/>
     </row>
     <row r="4" spans="1:118" x14ac:dyDescent="0.2">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="25" t="s">
         <v>3</v>
       </c>
       <c r="B4" t="s">
@@ -1751,7 +1736,7 @@
       <c r="E4"/>
     </row>
     <row r="5" spans="1:118" x14ac:dyDescent="0.2">
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="29" t="s">
         <v>15</v>
       </c>
       <c r="C5"/>
@@ -1805,7 +1790,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="66" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="22" t="s">
         <v>16</v>
       </c>
       <c r="B2" t="s">
@@ -1813,7 +1798,7 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="25" t="s">
         <v>21</v>
       </c>
       <c r="B3" t="s">
@@ -1821,7 +1806,7 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="25" t="s">
         <v>21</v>
       </c>
       <c r="B4" t="s">
@@ -1829,7 +1814,7 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="29" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1848,18 +1833,19 @@
     <col min="1" max="1" width="21.33203125" customWidth="1"/>
     <col min="2" max="2" width="21.33203125" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="38.33203125" customWidth="1"/>
-    <col min="4" max="4" width="34.6640625" customWidth="1"/>
+    <col min="4" max="4" width="42.83203125" customWidth="1"/>
     <col min="5" max="5" width="19" customWidth="1"/>
     <col min="6" max="6" width="17.6640625" customWidth="1"/>
     <col min="7" max="8" width="16.83203125" customWidth="1"/>
     <col min="9" max="9" width="18.33203125" customWidth="1"/>
     <col min="10" max="10" width="20.5" customWidth="1"/>
     <col min="11" max="11" width="16.6640625" customWidth="1"/>
-    <col min="15" max="15" width="18.1640625" customWidth="1"/>
+    <col min="12" max="13" width="16.83203125" customWidth="1"/>
+    <col min="15" max="15" width="20.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B1" s="15" t="s">
@@ -1870,7 +1856,7 @@
       </c>
     </row>
     <row r="2" spans="1:16" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="24" t="s">
         <v>22</v>
       </c>
       <c r="B2" s="16" t="e">
@@ -1883,28 +1869,28 @@
     </row>
     <row r="3" spans="1:16" ht="40" x14ac:dyDescent="0.2">
       <c r="C3" s="9"/>
-      <c r="E3" s="39" t="s">
+      <c r="E3" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="40"/>
-      <c r="I3" s="41"/>
-      <c r="J3" s="39" t="s">
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="37"/>
+      <c r="J3" s="35" t="s">
         <v>57</v>
       </c>
-      <c r="K3" s="40"/>
-      <c r="L3" s="40"/>
-      <c r="M3" s="40"/>
-      <c r="N3" s="41"/>
-      <c r="O3" s="42" t="s">
+      <c r="K3" s="36"/>
+      <c r="L3" s="36"/>
+      <c r="M3" s="36"/>
+      <c r="N3" s="37"/>
+      <c r="O3" s="30" t="s">
         <v>58</v>
       </c>
       <c r="P3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="80" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A4" s="10"/>
       <c r="C4" s="10"/>
       <c r="D4" s="11"/>
@@ -1917,10 +1903,10 @@
       <c r="G4" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="43" t="s">
+      <c r="H4" s="31" t="s">
         <v>59</v>
       </c>
-      <c r="I4" s="44" t="s">
+      <c r="I4" s="32" t="s">
         <v>60</v>
       </c>
       <c r="J4" s="13" t="s">
@@ -1932,40 +1918,40 @@
       <c r="L4" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="M4" s="43" t="s">
+      <c r="M4" s="31" t="s">
         <v>59</v>
       </c>
-      <c r="N4" s="44" t="s">
+      <c r="N4" s="32" t="s">
         <v>61</v>
       </c>
-      <c r="O4" s="45" t="s">
+      <c r="O4" s="33" t="s">
         <v>59</v>
       </c>
       <c r="P4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="14"/>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="D5" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="21" t="e">
+      <c r="E5" s="19" t="e">
         <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-TIT",'ETPT Format DDG'!$C:$C,$A$2)</f>
         <v>#N/A</v>
       </c>
-      <c r="F5" s="19" t="e">
+      <c r="F5" s="17" t="e">
         <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$2)</f>
         <v>#N/A</v>
       </c>
-      <c r="G5" s="19" t="e">
+      <c r="G5" s="17" t="e">
         <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$2)</f>
         <v>#N/A</v>
       </c>
-      <c r="H5" s="19" t="e">
+      <c r="H5" s="17" t="e">
         <f>SUMIFS(
 INDEX('ETPT Format DDG'!$A:$DU,
 ,
@@ -1975,7 +1961,7 @@
 'ETPT Format DDG'!$G:$G,"Magistrat")</f>
         <v>#N/A</v>
       </c>
-      <c r="I5" s="46" t="e">
+      <c r="I5" s="34" t="e">
         <f>SUMIFS(
 INDEX('ETPT Format DDG'!$A:$DU,
 ,
@@ -1985,23 +1971,23 @@
 'ETPT Format DDG'!$G:$G,"Magistrat")</f>
         <v>#N/A</v>
       </c>
-      <c r="J5" s="19" t="e">
+      <c r="J5" s="17" t="e">
         <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"F-TIT",'ETPT Format DDG'!$C:$C,$A$2)</f>
         <v>#N/A</v>
       </c>
-      <c r="K5" s="19" t="e">
+      <c r="K5" s="17" t="e">
         <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"F-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$2)</f>
         <v>#N/A</v>
       </c>
-      <c r="L5" s="19" t="e">
+      <c r="L5" s="17" t="e">
         <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"F-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$2)</f>
         <v>#N/A</v>
       </c>
-      <c r="M5" s="20" t="e">
+      <c r="M5" s="18" t="e">
         <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"C",'ETPT Format DDG'!$C:$C,$A$2,'ETPT Format DDG'!$G:$G,"Greffe")</f>
         <v>#N/A</v>
       </c>
-      <c r="N5" s="46" t="e">
+      <c r="N5" s="34" t="e">
         <f>SUMIFS(
 INDEX('ETPT Format DDG'!$A:$DU,
 ,
@@ -2011,7 +1997,7 @@
 'ETPT Format DDG'!$G:$G,"Greffe")</f>
         <v>#N/A</v>
       </c>
-      <c r="O5" s="20" t="e">
+      <c r="O5" s="18" t="e">
         <f>SUMIFS(
 INDEX('ETPT Format DDG'!$A:$DU,
 ,
@@ -2036,7 +2022,7 @@
     <mergeCell ref="J3:N3"/>
   </mergeCells>
   <conditionalFormatting sqref="C5:O150">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>AND(ISBLANK($C5)=FALSE,ISBLANK($D5)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2067,276 +2053,266 @@
   <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.1640625" style="23" customWidth="1"/>
-    <col min="2" max="2" width="7.33203125" style="23" customWidth="1"/>
-    <col min="3" max="9" width="10.83203125" style="23"/>
-    <col min="10" max="10" width="71.1640625" style="23" customWidth="1"/>
-    <col min="11" max="16384" width="10.83203125" style="23"/>
+    <col min="1" max="1" width="8.1640625" style="21" customWidth="1"/>
+    <col min="2" max="2" width="7.33203125" style="21" customWidth="1"/>
+    <col min="3" max="9" width="10.83203125" style="21"/>
+    <col min="10" max="10" width="71.1640625" style="21" customWidth="1"/>
+    <col min="11" max="16384" width="10.83203125" style="21"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="28" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="36" t="s">
+    <row r="1" spans="1:10" s="26" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="42" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
     </row>
     <row r="2" spans="1:10" s="10" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="35" t="s">
+      <c r="B2" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="35"/>
-      <c r="J2" s="35"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
     </row>
     <row r="3" spans="1:10" s="10" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="29"/>
-      <c r="B3" s="30" t="s">
+      <c r="A3" s="27"/>
+      <c r="B3" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="32" t="s">
+      <c r="C3" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
-      <c r="J3" s="32"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="38"/>
+      <c r="H3" s="38"/>
+      <c r="I3" s="38"/>
+      <c r="J3" s="38"/>
     </row>
     <row r="4" spans="1:10" s="10" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="29"/>
-      <c r="B4" s="30" t="s">
+      <c r="A4" s="27"/>
+      <c r="B4" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="C4" s="32" t="s">
+      <c r="C4" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32"/>
-      <c r="H4" s="32"/>
-      <c r="I4" s="32"/>
-      <c r="J4" s="32"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="38"/>
+      <c r="H4" s="38"/>
+      <c r="I4" s="38"/>
+      <c r="J4" s="38"/>
     </row>
     <row r="5" spans="1:10" s="10" customFormat="1" ht="43" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="29"/>
-      <c r="B5" s="30" t="s">
+      <c r="A5" s="27"/>
+      <c r="B5" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="C5" s="32" t="s">
+      <c r="C5" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="32"/>
-      <c r="I5" s="32"/>
-      <c r="J5" s="32"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="38"/>
+      <c r="H5" s="38"/>
+      <c r="I5" s="38"/>
+      <c r="J5" s="38"/>
     </row>
     <row r="6" spans="1:10" s="10" customFormat="1" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="30" t="s">
+      <c r="A6" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="C6" s="32"/>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32"/>
-      <c r="F6" s="32"/>
-      <c r="G6" s="32"/>
-      <c r="H6" s="32"/>
-      <c r="I6" s="32"/>
-      <c r="J6" s="32"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="38"/>
+      <c r="G6" s="38"/>
+      <c r="H6" s="38"/>
+      <c r="I6" s="38"/>
+      <c r="J6" s="38"/>
     </row>
     <row r="7" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="29"/>
-      <c r="B7" s="35" t="s">
+      <c r="A7" s="27"/>
+      <c r="B7" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="35"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="35"/>
-      <c r="G7" s="35"/>
-      <c r="H7" s="35"/>
-      <c r="I7" s="35"/>
-      <c r="J7" s="35"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
+      <c r="G7" s="41"/>
+      <c r="H7" s="41"/>
+      <c r="I7" s="41"/>
+      <c r="J7" s="41"/>
     </row>
     <row r="8" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="38" t="s">
+      <c r="B8" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="38"/>
-      <c r="D8" s="38"/>
-      <c r="E8" s="38"/>
-      <c r="F8" s="38"/>
-      <c r="G8" s="38"/>
-      <c r="H8" s="38"/>
-      <c r="I8" s="38"/>
-      <c r="J8" s="38"/>
+      <c r="C8" s="44"/>
+      <c r="D8" s="44"/>
+      <c r="E8" s="44"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="44"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="44"/>
+      <c r="J8" s="44"/>
     </row>
     <row r="9" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="38"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="38"/>
-      <c r="F9" s="38"/>
-      <c r="G9" s="38"/>
-      <c r="H9" s="38"/>
-      <c r="I9" s="38"/>
-      <c r="J9" s="38"/>
+      <c r="C9" s="44"/>
+      <c r="D9" s="44"/>
+      <c r="E9" s="44"/>
+      <c r="F9" s="44"/>
+      <c r="G9" s="44"/>
+      <c r="H9" s="44"/>
+      <c r="I9" s="44"/>
+      <c r="J9" s="44"/>
     </row>
     <row r="10" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="38" t="s">
+      <c r="B10" s="44" t="s">
         <v>48</v>
       </c>
-      <c r="C10" s="38"/>
-      <c r="D10" s="38"/>
-      <c r="E10" s="38"/>
-      <c r="F10" s="38"/>
-      <c r="G10" s="38"/>
-      <c r="H10" s="38"/>
-      <c r="I10" s="38"/>
-      <c r="J10" s="38"/>
+      <c r="C10" s="44"/>
+      <c r="D10" s="44"/>
+      <c r="E10" s="44"/>
+      <c r="F10" s="44"/>
+      <c r="G10" s="44"/>
+      <c r="H10" s="44"/>
+      <c r="I10" s="44"/>
+      <c r="J10" s="44"/>
     </row>
     <row r="11" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="38" t="s">
+      <c r="B11" s="44" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="38"/>
-      <c r="D11" s="38"/>
-      <c r="E11" s="38"/>
-      <c r="F11" s="38"/>
-      <c r="G11" s="38"/>
-      <c r="H11" s="38"/>
-      <c r="I11" s="38"/>
-      <c r="J11" s="38"/>
+      <c r="C11" s="44"/>
+      <c r="D11" s="44"/>
+      <c r="E11" s="44"/>
+      <c r="F11" s="44"/>
+      <c r="G11" s="44"/>
+      <c r="H11" s="44"/>
+      <c r="I11" s="44"/>
+      <c r="J11" s="44"/>
     </row>
     <row r="12" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="29" t="s">
+      <c r="A12" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="33" t="s">
+      <c r="B12" s="39" t="s">
         <v>50</v>
       </c>
-      <c r="C12" s="34"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="34"/>
-      <c r="F12" s="34"/>
-      <c r="G12" s="34"/>
-      <c r="H12" s="34"/>
-      <c r="I12" s="34"/>
-      <c r="J12" s="34"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="40"/>
+      <c r="F12" s="40"/>
+      <c r="G12" s="40"/>
+      <c r="H12" s="40"/>
+      <c r="I12" s="40"/>
+      <c r="J12" s="40"/>
     </row>
     <row r="13" spans="1:10" s="10" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="30" t="s">
+      <c r="B13" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="32" t="s">
+      <c r="C13" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="32"/>
-      <c r="E13" s="32"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="32"/>
-      <c r="H13" s="32"/>
-      <c r="I13" s="32"/>
-      <c r="J13" s="32"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="38"/>
+      <c r="G13" s="38"/>
+      <c r="H13" s="38"/>
+      <c r="I13" s="38"/>
+      <c r="J13" s="38"/>
     </row>
     <row r="14" spans="1:10" s="10" customFormat="1" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="30" t="s">
+      <c r="B14" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="32" t="s">
+      <c r="C14" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="D14" s="32"/>
-      <c r="E14" s="32"/>
-      <c r="F14" s="32"/>
-      <c r="G14" s="32"/>
-      <c r="H14" s="32"/>
-      <c r="I14" s="32"/>
-      <c r="J14" s="32"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="38"/>
+      <c r="G14" s="38"/>
+      <c r="H14" s="38"/>
+      <c r="I14" s="38"/>
+      <c r="J14" s="38"/>
     </row>
     <row r="15" spans="1:10" s="10" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="30" t="s">
+      <c r="B15" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="32" t="s">
+      <c r="C15" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="D15" s="32"/>
-      <c r="E15" s="32"/>
-      <c r="F15" s="32"/>
-      <c r="G15" s="32"/>
-      <c r="H15" s="32"/>
-      <c r="I15" s="32"/>
-      <c r="J15" s="32"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="38"/>
+      <c r="G15" s="38"/>
+      <c r="H15" s="38"/>
+      <c r="I15" s="38"/>
+      <c r="J15" s="38"/>
     </row>
     <row r="16" spans="1:10" s="10" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="30" t="s">
+      <c r="A16" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="32" t="s">
+      <c r="B16" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="C16" s="32"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="32"/>
-      <c r="F16" s="32"/>
-      <c r="G16" s="32"/>
-      <c r="H16" s="32"/>
-      <c r="I16" s="32"/>
-      <c r="J16" s="32"/>
-    </row>
-    <row r="18" spans="1:10" s="28" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="36" t="s">
+      <c r="C16" s="38"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="38"/>
+      <c r="G16" s="38"/>
+      <c r="H16" s="38"/>
+      <c r="I16" s="38"/>
+      <c r="J16" s="38"/>
+    </row>
+    <row r="18" spans="1:10" s="26" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="42" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="37"/>
-      <c r="C18" s="37"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="37"/>
-      <c r="G18" s="37"/>
-      <c r="H18" s="37"/>
-      <c r="I18" s="37"/>
-      <c r="J18" s="37"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="43"/>
+      <c r="E18" s="43"/>
+      <c r="F18" s="43"/>
+      <c r="G18" s="43"/>
+      <c r="H18" s="43"/>
+      <c r="I18" s="43"/>
+      <c r="J18" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="C13:J13"/>
-    <mergeCell ref="C14:J14"/>
-    <mergeCell ref="B12:J12"/>
-    <mergeCell ref="B7:J7"/>
-    <mergeCell ref="A18:J18"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B2:J2"/>
-    <mergeCell ref="C3:J3"/>
-    <mergeCell ref="C4:J4"/>
-    <mergeCell ref="C5:J5"/>
     <mergeCell ref="B6:J6"/>
     <mergeCell ref="C15:J15"/>
     <mergeCell ref="B16:J16"/>
@@ -2344,6 +2320,16 @@
     <mergeCell ref="B9:J9"/>
     <mergeCell ref="B10:J10"/>
     <mergeCell ref="B11:J11"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="C3:J3"/>
+    <mergeCell ref="C4:J4"/>
+    <mergeCell ref="C5:J5"/>
+    <mergeCell ref="C13:J13"/>
+    <mergeCell ref="C14:J14"/>
+    <mergeCell ref="B12:J12"/>
+    <mergeCell ref="B7:J7"/>
+    <mergeCell ref="A18:J18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
update extractor Mme DE JONG
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42B14F26-027E-9F4C-A957-F1AF0E6DE8ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA203BC9-F64E-6A46-951B-47BBC64CF6DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="22480" windowHeight="17620" activeTab="5" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17760" activeTab="5" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ETPT A-JUST" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ETPT A-JUST'!$A$2:$DN$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ETPT Format DDG'!$A$2:$DT$2</definedName>
+    <definedName name="J">#REF!</definedName>
+    <definedName name="JA">#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="63">
   <si>
     <t>#! END_ROW</t>
   </si>
@@ -152,12 +154,6 @@
     <t>Selectionner une juridiction</t>
   </si>
   <si>
-    <t xml:space="preserve">         Extracteur de données d'effectifs - Format DDG (avec réintégration de l'absentéisme)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">         Extracteur de données d'effectifs</t>
-  </si>
-  <si>
     <t xml:space="preserve">        EXPLICATIONS ET CONTROLES A EFFECTUER</t>
   </si>
   <si>
@@ -301,6 +297,211 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Précisions nécessaires aux DDG</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (dans l'onglet "ETPT Format DDG"):</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">La colonne "JURIDICTION" permet de préciser le </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>tribunal d'affectation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (TJ / TPRX) -&gt; les données ont été prérenseignées à partir des éléments présents dans A-JUST. LEs magistrats sont, par défaut, affectés au TJ. Il convient de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>contrôler ces renseignements et de réaffecter, au besoin, les agents dans l'un des TPRX proposés dans le menu déroulant.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Les éventuels </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>CET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ont été répartis entre les CET de</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> moins d'un mois</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (colonne DS), qui sont considérés, lors des DDG, comme de l'absentéisme et ceux de</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> plus d'un mois</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (colonne DR) qui déduisent de l'ETPT (action 99).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Dans l'onglet </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"Agrégats DDG"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, il convient de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">sélectionner le tribunal voulu dans le menu déroulant </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(case en bleu) pour que s'affiche une synthèse montrant, pour le tribunal sélectionné (TJ ou TPRX), les ETPT affectés à chaque activité ou contentieux, ainsi que les indisponibilités déduisant de l'ETPT (action 99) et celles qui ont été réintégrées (absentéisme).</t>
+    </r>
+  </si>
+  <si>
+    <t>Pour toute question, n'hésitez pas à contacter l'équipe A-JUST : support-utilisateurs@a-just.fr</t>
+  </si>
+  <si>
+    <t>SIEGE</t>
+  </si>
+  <si>
+    <t>GREFFE</t>
+  </si>
+  <si>
+    <t>EQUIPE AUTOUR DU MAGISTRAT</t>
+  </si>
+  <si>
+    <t>Contractuels et vacataires</t>
+  </si>
+  <si>
+    <t>TOTAL SIEGE</t>
+  </si>
+  <si>
+    <t>TOTAL GREFFE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                Extracteur de données d'effectifs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                Extracteur de données d'effectifs - Format DDG (avec réintégration de l'absentéisme)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                Agrégats DDG</t>
+  </si>
+  <si>
+    <r>
       <t xml:space="preserve">Un </t>
     </r>
     <r>
@@ -324,114 +525,64 @@
       </rPr>
       <t>appelle une vérification. Soit l'agent était effectivement absent pendant toute la période (en CLM par ex.), soit il n'a pas été ventilé.</t>
     </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Il est nécessaire de ventiler durant les temps d'indisponibilité.</t>
+    </r>
   </si>
   <si>
     <r>
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Précisions nécessaires aux DDG</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> (dans l'onglet "ETPT Format DDG"):</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">La colonne "JURIDICTION" permet de préciser le </t>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>La colonne "Fonction"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> est remplie automatiquement mais </t>
     </r>
     <r>
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>tribunal d'affectation</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> (TJ / TPRX) -&gt; les données ont été prérenseignées à partir des éléments présents dans A-JUST. LEs magistrats sont, par défaut, affectés au TJ. Il convient de </t>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>doit être contrôlée et, au besoin, corrigée pour les agents placés</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> car elle permet de distinguer</t>
     </r>
     <r>
       <rPr>
         <b/>
         <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>contrôler ces renseignements et de réaffecter, au besoin, les agents dans l'un des TPRX proposés dans le menu déroulant.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>La colonne "Code fonction"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> est remplie automatiquement mais </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>doit être contrôlée et, au besoin, corrigée pour les agents placés</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> car elle permet de distinguer</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
@@ -447,144 +598,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>. Par défaut, tous les placés ont été codés en "M-PLAC-ADD" (Magistrat placé additionnel) ou "F-PLAC-ADD" (Fonctionnaire placé additionnel). Si des Placés étaient des effectifs de substitution, les recoder "M-PLAC-SUB" pour les magistrats ou "F-PLAC-SUB" pour les fonctionnaires, à l'aide du menu déroulant.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Les éventuels </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>CET</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> ont été répartis entre les CET de</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> moins d'un mois</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> (colonne DS), qui sont considérés, lors des DDG, comme de l'absentéisme et ceux de</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> plus d'un mois</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> (colonne DR) qui déduisent de l'ETPT (action 99).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Dans l'onglet </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>"Agrégats DDG"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, il convient de </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">sélectionner le tribunal voulu dans le menu déroulant </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(case en bleu) pour que s'affiche une synthèse montrant, pour le tribunal sélectionné (TJ ou TPRX), les ETPT affectés à chaque activité ou contentieux, ainsi que les indisponibilités déduisant de l'ETPT (action 99) et celles qui ont été réintégrées (absentéisme).</t>
-    </r>
-  </si>
-  <si>
-    <t>Pour toute question, n'hésitez pas à contacter l'équipe A-JUST : support-utilisateurs@a-just.fr</t>
-  </si>
-  <si>
-    <t>SIEGE</t>
-  </si>
-  <si>
-    <t>GREFFE</t>
-  </si>
-  <si>
-    <t>EQUIPE AUTOUR DU MAGISTRAT</t>
-  </si>
-  <si>
-    <t>Contractuels et vacataires</t>
-  </si>
-  <si>
-    <t>TOTAL SIEGE</t>
-  </si>
-  <si>
-    <t>TOTAL GREFFE</t>
+      <t>. Par défaut, tous les placés sont "* PLACÉ ADDITIONNEL". Si des Placés étaient des effectifs de substitution, il faut les renseigner en "* PLACÉ SUBSTITUTION", à l'aide du menu déroulant.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -598,7 +613,7 @@
     <numFmt numFmtId="167" formatCode="General;General;\-"/>
     <numFmt numFmtId="168" formatCode="0.###;0.###;\-"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -683,6 +698,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="22"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -883,7 +913,7 @@
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1001,23 +1031,35 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1060,15 +1102,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>46180</xdr:colOff>
+      <xdr:colOff>103906</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>23090</xdr:rowOff>
+      <xdr:rowOff>57725</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>542634</xdr:colOff>
+      <xdr:colOff>923635</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>476535</xdr:rowOff>
+      <xdr:rowOff>806439</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1091,8 +1133,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="46180" y="23090"/>
-          <a:ext cx="496454" cy="453445"/>
+          <a:off x="103906" y="57725"/>
+          <a:ext cx="819729" cy="748714"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1109,22 +1151,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>46180</xdr:colOff>
+      <xdr:colOff>103905</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>23090</xdr:rowOff>
+      <xdr:rowOff>57725</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>542634</xdr:colOff>
+      <xdr:colOff>923634</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>476535</xdr:rowOff>
+      <xdr:rowOff>806439</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 5">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6CD8D5B3-C3E9-E94E-BD8C-2EF269EA8931}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0D7A5D8C-BE33-ED45-A77A-8F455267161F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1140,8 +1182,106 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="46180" y="23090"/>
-          <a:ext cx="496454" cy="453445"/>
+          <a:off x="103905" y="57725"/>
+          <a:ext cx="819729" cy="748714"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>98777</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>84665</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1114778</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>1012648</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FD1D57F9-87BD-BD45-83E9-42F2487B9728}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="98777" y="84665"/>
+          <a:ext cx="1016001" cy="927983"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>103910</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>69271</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>300184</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>817985</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3DC1CFF2-AC52-DD4F-9E83-87135FE34159}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="103910" y="69271"/>
+          <a:ext cx="819729" cy="748714"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1453,7 +1593,7 @@
   <dimension ref="A1:DN8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="26.1640625" customWidth="1"/>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.1640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="7.6640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="12" style="2" customWidth="1"/>
@@ -1463,9 +1603,9 @@
     <col min="8" max="8" width="9.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:118" s="4" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:118" s="4" customFormat="1" ht="67" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -1773,9 +1913,9 @@
     <col min="2" max="2" width="71.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="4" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="4" customFormat="1" ht="67" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -1827,7 +1967,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E893F90-1EC7-764C-B747-7920FCEC73CB}">
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.33203125" customWidth="1"/>
@@ -1844,189 +1984,215 @@
     <col min="15" max="15" width="20.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+    <row r="1" spans="1:16" s="4" customFormat="1" ht="84" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+    </row>
+    <row r="2" spans="1:16" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B2" s="15" t="s">
         <v>29</v>
-      </c>
-      <c r="C1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="16" t="e">
-        <f>VLOOKUP(A2,'codage tribunal'!A:B,2,FALSE)</f>
-        <v>#N/A</v>
       </c>
       <c r="C2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="40" x14ac:dyDescent="0.2">
-      <c r="C3" s="9"/>
-      <c r="E3" s="37" t="s">
+    <row r="3" spans="1:16" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="16" t="e">
+        <f>VLOOKUP(A3,'codage tribunal'!A:B,2,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="40" x14ac:dyDescent="0.2">
+      <c r="C4" s="9"/>
+      <c r="E4" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="38"/>
+      <c r="G4" s="38"/>
+      <c r="H4" s="38"/>
+      <c r="I4" s="39"/>
+      <c r="J4" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="K4" s="38"/>
+      <c r="L4" s="38"/>
+      <c r="M4" s="38"/>
+      <c r="N4" s="39"/>
+      <c r="O4" s="30" t="s">
+        <v>54</v>
+      </c>
+      <c r="P4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+      <c r="A5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="31" t="s">
+        <v>55</v>
+      </c>
+      <c r="I5" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="F3" s="38"/>
-      <c r="G3" s="38"/>
-      <c r="H3" s="38"/>
-      <c r="I3" s="39"/>
-      <c r="J3" s="37" t="s">
+      <c r="J5" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="K5" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="L5" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="M5" s="31" t="s">
+        <v>55</v>
+      </c>
+      <c r="N5" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="K3" s="38"/>
-      <c r="L3" s="38"/>
-      <c r="M3" s="38"/>
-      <c r="N3" s="39"/>
-      <c r="O3" s="30" t="s">
-        <v>58</v>
-      </c>
-      <c r="P3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" ht="48" x14ac:dyDescent="0.2">
-      <c r="A4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="G4" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="H4" s="31" t="s">
-        <v>59</v>
-      </c>
-      <c r="I4" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="J4" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="K4" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="L4" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="M4" s="31" t="s">
-        <v>59</v>
-      </c>
-      <c r="N4" s="32" t="s">
-        <v>61</v>
-      </c>
-      <c r="O4" s="33" t="s">
-        <v>59</v>
-      </c>
-      <c r="P4" t="s">
+      <c r="O5" s="33" t="s">
+        <v>55</v>
+      </c>
+      <c r="P5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="14"/>
-      <c r="C5" s="35" t="s">
+    <row r="6" spans="1:16" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="14"/>
+      <c r="C6" s="35" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="36" t="s">
+      <c r="D6" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="19" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-TIT",'ETPT Format DDG'!$C:$C,$A$2)</f>
+      <c r="E6" s="19" t="e">
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
-      <c r="F5" s="17" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$2)</f>
+      <c r="F6" s="17" t="e">
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3,'ETPT Format DDG'!$H:$H,"*ADDITIONNEL*")</f>
         <v>#N/A</v>
       </c>
-      <c r="G5" s="17" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$2)</f>
+      <c r="G6" s="17" t="e">
+        <f>SUMIFS(
+INDEX('ETPT Format DDG'!$A:$DU,
+,IFERROR(MATCH(D6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3,'ETPT Format DDG'!$H:$H,"*SUBSTITUTION*")</f>
         <v>#N/A</v>
       </c>
-      <c r="H5" s="17" t="e">
+      <c r="H6" s="17" t="e">
         <f>SUMIFS(
 INDEX('ETPT Format DDG'!$A:$DU,
 ,
-IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))
+IFERROR(MATCH(D6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
 ),'ETPT Format DDG'!$I:$I,"C",
-'ETPT Format DDG'!$C:$C,$A$2,
+'ETPT Format DDG'!$C:$C,$A$3,
 'ETPT Format DDG'!$G:$G,"Magistrat")</f>
         <v>#N/A</v>
       </c>
-      <c r="I5" s="34" t="e">
+      <c r="I6" s="34" t="e">
         <f>SUMIFS(
 INDEX('ETPT Format DDG'!$A:$DU,
 ,
-IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))
+IFERROR(MATCH(D6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
 ),
-'ETPT Format DDG'!$C:$C,$A$2,
+'ETPT Format DDG'!$C:$C,$A$3,
 'ETPT Format DDG'!$G:$G,"Magistrat")</f>
         <v>#N/A</v>
       </c>
-      <c r="J5" s="17" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"F-TIT",'ETPT Format DDG'!$C:$C,$A$2)</f>
+      <c r="J6" s="17" t="e">
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"F-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
-      <c r="K5" s="17" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"F-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$2)</f>
+      <c r="K6" s="17" t="e">
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"F-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3,'ETPT Format DDG'!$H:$H,"*ADDITIONNEL*")</f>
         <v>#N/A</v>
       </c>
-      <c r="L5" s="17" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"F-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$2)</f>
+      <c r="L6" s="17" t="e">
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"F-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3,'ETPT Format DDG'!$H:$H,"*SUBSTITUTION*")</f>
         <v>#N/A</v>
       </c>
-      <c r="M5" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"C",'ETPT Format DDG'!$C:$C,$A$2,'ETPT Format DDG'!$G:$G,"Greffe")</f>
+      <c r="M6" s="18" t="e">
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(D6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"C",'ETPT Format DDG'!$C:$C,$A$3,'ETPT Format DDG'!$G:$G,"Greffe")</f>
         <v>#N/A</v>
       </c>
-      <c r="N5" s="34" t="e">
+      <c r="N6" s="34" t="e">
         <f>SUMIFS(
 INDEX('ETPT Format DDG'!$A:$DU,
 ,
-IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))
+IFERROR(MATCH(D6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
 ),
-'ETPT Format DDG'!$C:$C,$A$2,
+'ETPT Format DDG'!$C:$C,$A$3,
 'ETPT Format DDG'!$G:$G,"Greffe")</f>
         <v>#N/A</v>
       </c>
-      <c r="O5" s="18" t="e">
+      <c r="O6" s="18" t="e">
         <f>SUMIFS(
 INDEX('ETPT Format DDG'!$A:$DU,
 ,
-IFERROR(MATCH(D5,'ETPT Format DDG'!$2:$2,0),MATCH(C5,'ETPT Format DDG'!$2:$2,0))
+IFERROR(MATCH(D6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
 ),'ETPT Format DDG'!$I:$I,"C",
-'ETPT Format DDG'!$C:$C,$A$2,
+'ETPT Format DDG'!$C:$C,$A$3,
 'ETPT Format DDG'!$G:$G,"Autour du magistrat")</f>
         <v>#N/A</v>
       </c>
-      <c r="P5" t="s">
+      <c r="P6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="P6" t="s">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="P7" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="E3:I3"/>
-    <mergeCell ref="J3:N3"/>
+    <mergeCell ref="E4:I4"/>
+    <mergeCell ref="J4:N4"/>
   </mergeCells>
-  <conditionalFormatting sqref="C5:O150">
+  <conditionalFormatting sqref="C6:O151">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>AND(ISBLANK($C5)=FALSE,ISBLANK($D5)=TRUE)</formula>
+      <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($D6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2060,43 +2226,43 @@
     <col min="11" max="16384" width="10.83203125" style="21"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="26" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="42" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
+    <row r="1" spans="1:10" s="26" customFormat="1" ht="67" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="46" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
     </row>
     <row r="2" spans="1:10" s="10" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="44" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
-      <c r="I2" s="44"/>
-      <c r="J2" s="44"/>
+      <c r="B2" s="43" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="43"/>
     </row>
     <row r="3" spans="1:10" s="10" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="27"/>
       <c r="B3" s="28" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C3" s="40" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D3" s="40"/>
       <c r="E3" s="40"/>
@@ -2109,10 +2275,10 @@
     <row r="4" spans="1:10" s="10" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="27"/>
       <c r="B4" s="28" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C4" s="40" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D4" s="40"/>
       <c r="E4" s="40"/>
@@ -2125,10 +2291,10 @@
     <row r="5" spans="1:10" s="10" customFormat="1" ht="43" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="27"/>
       <c r="B5" s="28" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C5" s="40" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D5" s="40"/>
       <c r="E5" s="40"/>
@@ -2143,7 +2309,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="40" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C6" s="40"/>
       <c r="D6" s="40"/>
@@ -2156,92 +2322,92 @@
     </row>
     <row r="7" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="27"/>
-      <c r="B7" s="44" t="s">
+      <c r="B7" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="43"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="43"/>
+      <c r="I7" s="43"/>
+      <c r="J7" s="43"/>
+    </row>
+    <row r="8" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="48" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="48"/>
+      <c r="D8" s="48"/>
+      <c r="E8" s="48"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="48"/>
+      <c r="H8" s="48"/>
+      <c r="I8" s="48"/>
+      <c r="J8" s="48"/>
+    </row>
+    <row r="9" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="48" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="48"/>
+      <c r="D9" s="48"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="48"/>
+      <c r="H9" s="48"/>
+      <c r="I9" s="48"/>
+      <c r="J9" s="48"/>
+    </row>
+    <row r="10" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="48" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="44"/>
-      <c r="D7" s="44"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="44"/>
-      <c r="G7" s="44"/>
-      <c r="H7" s="44"/>
-      <c r="I7" s="44"/>
-      <c r="J7" s="44"/>
-    </row>
-    <row r="8" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="41" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" s="41"/>
-      <c r="D8" s="41"/>
-      <c r="E8" s="41"/>
-      <c r="F8" s="41"/>
-      <c r="G8" s="41"/>
-      <c r="H8" s="41"/>
-      <c r="I8" s="41"/>
-      <c r="J8" s="41"/>
-    </row>
-    <row r="9" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="41" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="41"/>
-      <c r="D9" s="41"/>
-      <c r="E9" s="41"/>
-      <c r="F9" s="41"/>
-      <c r="G9" s="41"/>
-      <c r="H9" s="41"/>
-      <c r="I9" s="41"/>
-      <c r="J9" s="41"/>
-    </row>
-    <row r="10" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="41" t="s">
-        <v>48</v>
-      </c>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
-      <c r="G10" s="41"/>
-      <c r="H10" s="41"/>
-      <c r="I10" s="41"/>
-      <c r="J10" s="41"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48"/>
+      <c r="G10" s="48"/>
+      <c r="H10" s="48"/>
+      <c r="I10" s="48"/>
+      <c r="J10" s="48"/>
     </row>
     <row r="11" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="41" t="s">
-        <v>49</v>
-      </c>
-      <c r="C11" s="41"/>
-      <c r="D11" s="41"/>
-      <c r="E11" s="41"/>
-      <c r="F11" s="41"/>
-      <c r="G11" s="41"/>
-      <c r="H11" s="41"/>
-      <c r="I11" s="41"/>
-      <c r="J11" s="41"/>
+      <c r="B11" s="49" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="48"/>
+      <c r="D11" s="48"/>
+      <c r="E11" s="48"/>
+      <c r="F11" s="48"/>
+      <c r="G11" s="48"/>
+      <c r="H11" s="48"/>
+      <c r="I11" s="48"/>
+      <c r="J11" s="48"/>
     </row>
     <row r="12" spans="1:10" s="10" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="45" t="s">
-        <v>50</v>
-      </c>
-      <c r="C12" s="46"/>
-      <c r="D12" s="46"/>
-      <c r="E12" s="46"/>
-      <c r="F12" s="46"/>
-      <c r="G12" s="46"/>
-      <c r="H12" s="46"/>
-      <c r="I12" s="46"/>
-      <c r="J12" s="46"/>
+      <c r="B12" s="41" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" s="42"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="42"/>
+      <c r="F12" s="42"/>
+      <c r="G12" s="42"/>
+      <c r="H12" s="42"/>
+      <c r="I12" s="42"/>
+      <c r="J12" s="42"/>
     </row>
     <row r="13" spans="1:10" s="10" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="28" t="s">
         <v>11</v>
       </c>
       <c r="C13" s="40" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D13" s="40"/>
       <c r="E13" s="40"/>
@@ -2255,8 +2421,8 @@
       <c r="B14" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="40" t="s">
-        <v>52</v>
+      <c r="C14" s="50" t="s">
+        <v>62</v>
       </c>
       <c r="D14" s="40"/>
       <c r="E14" s="40"/>
@@ -2271,7 +2437,7 @@
         <v>13</v>
       </c>
       <c r="C15" s="40" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D15" s="40"/>
       <c r="E15" s="40"/>
@@ -2286,7 +2452,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="40" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C16" s="40"/>
       <c r="D16" s="40"/>
@@ -2298,21 +2464,25 @@
       <c r="J16" s="40"/>
     </row>
     <row r="18" spans="1:10" s="26" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="42" t="s">
-        <v>55</v>
-      </c>
-      <c r="B18" s="43"/>
-      <c r="C18" s="43"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="43"/>
-      <c r="F18" s="43"/>
-      <c r="G18" s="43"/>
-      <c r="H18" s="43"/>
-      <c r="I18" s="43"/>
-      <c r="J18" s="43"/>
+      <c r="A18" s="44" t="s">
+        <v>51</v>
+      </c>
+      <c r="B18" s="45"/>
+      <c r="C18" s="45"/>
+      <c r="D18" s="45"/>
+      <c r="E18" s="45"/>
+      <c r="F18" s="45"/>
+      <c r="G18" s="45"/>
+      <c r="H18" s="45"/>
+      <c r="I18" s="45"/>
+      <c r="J18" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="C13:J13"/>
+    <mergeCell ref="C14:J14"/>
+    <mergeCell ref="B12:J12"/>
+    <mergeCell ref="B7:J7"/>
     <mergeCell ref="A18:J18"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="B2:J2"/>
@@ -2326,12 +2496,9 @@
     <mergeCell ref="B9:J9"/>
     <mergeCell ref="B10:J10"/>
     <mergeCell ref="B11:J11"/>
-    <mergeCell ref="C13:J13"/>
-    <mergeCell ref="C14:J14"/>
-    <mergeCell ref="B12:J12"/>
-    <mergeCell ref="B7:J7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
extractor final display DDG
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F327840D-70B6-7B48-B14F-7A0BA89B1209}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1867FA-6BD2-604C-AC39-EE3945E7A4B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="22940" windowHeight="13240" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -3210,7 +3210,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="42">
+  <borders count="46">
     <border>
       <left/>
       <right/>
@@ -3553,19 +3553,6 @@
     </border>
     <border>
       <left/>
-      <right style="medium">
-        <color rgb="FF333F4F"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF333F4F"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF333F4F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right/>
       <top style="thick">
         <color rgb="FFFF0000"/>
@@ -3685,6 +3672,57 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF333F4F"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF333F4F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF333F4F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF333F4F"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF333F4F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -3695,7 +3733,7 @@
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="258">
+  <cellXfs count="260">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -4367,19 +4405,10 @@
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="4" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="4" applyBorder="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="40" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -4393,13 +4422,58 @@
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="25" xfId="6" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="27" xfId="6" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="29" xfId="6" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="40" xfId="6" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="22" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4408,11 +4482,35 @@
     <xf numFmtId="0" fontId="9" fillId="22" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4444,14 +4542,14 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="32" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="31" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -4461,60 +4559,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="25" xfId="6" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="27" xfId="6" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="29" xfId="6" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="41" xfId="6" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -4654,9 +4698,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>13121</xdr:colOff>
+      <xdr:colOff>227016</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>81478</xdr:rowOff>
+      <xdr:rowOff>14635</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="960661" cy="902640"/>
     <xdr:pic>
@@ -4680,7 +4724,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="838621" y="81478"/>
+          <a:off x="320595" y="14635"/>
           <a:ext cx="960661" cy="902640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5305,11 +5349,11 @@
       <c r="B1" s="197" t="s">
         <v>494</v>
       </c>
-      <c r="C1" s="222" t="s">
+      <c r="C1" s="225" t="s">
         <v>495</v>
       </c>
-      <c r="D1" s="222"/>
-      <c r="E1" s="222"/>
+      <c r="D1" s="225"/>
+      <c r="E1" s="225"/>
       <c r="F1" s="198"/>
       <c r="H1" s="28" t="s">
         <v>0</v>
@@ -5318,11 +5362,11 @@
     <row r="2" spans="1:8" s="202" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="199"/>
       <c r="B2" s="200"/>
-      <c r="C2" s="223" t="s">
+      <c r="C2" s="226" t="s">
         <v>496</v>
       </c>
-      <c r="D2" s="223"/>
-      <c r="E2" s="223"/>
+      <c r="D2" s="226"/>
+      <c r="E2" s="226"/>
       <c r="F2" s="201"/>
       <c r="H2" s="28" t="s">
         <v>0</v>
@@ -5346,156 +5390,163 @@
       <c r="D4" s="207" t="s">
         <v>499</v>
       </c>
-      <c r="E4" s="220" t="s">
+      <c r="E4" s="232" t="s">
         <v>500</v>
       </c>
-      <c r="F4" s="221"/>
+      <c r="F4" s="233"/>
+      <c r="G4" s="221"/>
       <c r="H4" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="28" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="203"/>
-      <c r="B5" s="240" t="s">
+      <c r="B5" s="214" t="s">
         <v>501</v>
       </c>
-      <c r="C5" s="241" t="s">
+      <c r="C5" s="215" t="s">
         <v>502</v>
       </c>
-      <c r="D5" s="241" t="s">
+      <c r="D5" s="215" t="s">
         <v>503</v>
       </c>
-      <c r="E5" s="242" t="s">
+      <c r="E5" s="234" t="s">
         <v>518</v>
       </c>
-      <c r="F5" s="243"/>
+      <c r="F5" s="235"/>
+      <c r="G5" s="220"/>
       <c r="H5" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="28" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="203"/>
-      <c r="B6" s="244" t="s">
+      <c r="B6" s="216" t="s">
         <v>504</v>
       </c>
-      <c r="C6" s="245" t="s">
+      <c r="C6" s="217" t="s">
         <v>505</v>
       </c>
-      <c r="D6" s="245" t="s">
+      <c r="D6" s="217" t="s">
         <v>506</v>
       </c>
-      <c r="E6" s="246" t="s">
+      <c r="E6" s="236" t="s">
         <v>519</v>
       </c>
-      <c r="F6" s="247"/>
+      <c r="F6" s="237"/>
+      <c r="G6" s="220"/>
       <c r="H6" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="28" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="203"/>
-      <c r="B7" s="244" t="s">
+      <c r="B7" s="216" t="s">
         <v>507</v>
       </c>
-      <c r="C7" s="245" t="s">
+      <c r="C7" s="217" t="s">
         <v>508</v>
       </c>
-      <c r="D7" s="245" t="s">
+      <c r="D7" s="217" t="s">
         <v>509</v>
       </c>
-      <c r="E7" s="246" t="s">
+      <c r="E7" s="236" t="s">
         <v>518</v>
       </c>
-      <c r="F7" s="247"/>
+      <c r="F7" s="237"/>
+      <c r="G7" s="220"/>
       <c r="H7" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="28" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="203"/>
-      <c r="B8" s="248" t="s">
+      <c r="B8" s="218" t="s">
         <v>510</v>
       </c>
-      <c r="C8" s="249" t="s">
+      <c r="C8" s="227" t="s">
         <v>511</v>
       </c>
-      <c r="D8" s="249" t="s">
+      <c r="D8" s="227" t="s">
         <v>512</v>
       </c>
-      <c r="E8" s="250" t="s">
+      <c r="E8" s="238" t="s">
         <v>520</v>
       </c>
-      <c r="F8" s="251"/>
+      <c r="F8" s="239"/>
+      <c r="G8" s="220"/>
       <c r="H8" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:8" s="28" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="203"/>
-      <c r="B9" s="248" t="s">
+      <c r="B9" s="218" t="s">
         <v>513</v>
       </c>
-      <c r="C9" s="249"/>
-      <c r="D9" s="249"/>
-      <c r="E9" s="252"/>
-      <c r="F9" s="253"/>
+      <c r="C9" s="227"/>
+      <c r="D9" s="227"/>
+      <c r="E9" s="240"/>
+      <c r="F9" s="241"/>
+      <c r="G9" s="220"/>
       <c r="H9" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:8" s="28" customFormat="1" ht="23" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="203"/>
-      <c r="B10" s="254" t="s">
+      <c r="B10" s="219" t="s">
         <v>514</v>
       </c>
-      <c r="C10" s="255"/>
-      <c r="D10" s="255"/>
-      <c r="E10" s="256"/>
-      <c r="F10" s="257"/>
+      <c r="C10" s="228"/>
+      <c r="D10" s="228"/>
+      <c r="E10" s="242"/>
+      <c r="F10" s="243"/>
+      <c r="G10" s="220"/>
       <c r="H10" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:8" s="28" customFormat="1" ht="5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="203"/>
-      <c r="B11" s="209"/>
-      <c r="C11" s="209"/>
-      <c r="D11" s="209"/>
-      <c r="E11" s="209"/>
-      <c r="F11" s="209"/>
+      <c r="B11" s="224"/>
+      <c r="C11" s="224"/>
+      <c r="D11" s="224"/>
+      <c r="E11" s="224"/>
+      <c r="F11" s="224"/>
       <c r="H11" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="28" customFormat="1" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="203"/>
-      <c r="B12" s="210"/>
-      <c r="C12" s="219" t="s">
+      <c r="B12" s="222"/>
+      <c r="C12" s="231" t="s">
         <v>515</v>
       </c>
-      <c r="D12" s="219"/>
-      <c r="E12" s="219"/>
-      <c r="F12" s="211"/>
+      <c r="D12" s="231"/>
+      <c r="E12" s="231"/>
+      <c r="F12" s="223"/>
       <c r="H12" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:8" s="28" customFormat="1" ht="6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="212"/>
+      <c r="A13" s="209"/>
       <c r="F13" s="204"/>
       <c r="H13" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:8" s="28" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="217" t="s">
+      <c r="A14" s="229" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="217"/>
-      <c r="C14" s="217"/>
-      <c r="D14" s="217"/>
-      <c r="E14" s="217"/>
-      <c r="F14" s="218"/>
+      <c r="B14" s="229"/>
+      <c r="C14" s="229"/>
+      <c r="D14" s="229"/>
+      <c r="E14" s="229"/>
+      <c r="F14" s="230"/>
       <c r="H14" s="28" t="s">
         <v>0</v>
       </c>
@@ -5548,16 +5599,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A1" s="232" t="s">
+      <c r="A1" s="252" t="s">
         <v>483</v>
       </c>
-      <c r="B1" s="232"/>
-      <c r="C1" s="232"/>
-      <c r="D1" s="232"/>
-      <c r="E1" s="232"/>
-      <c r="F1" s="232"/>
-      <c r="G1" s="232"/>
-      <c r="H1" s="232"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
+      <c r="H1" s="252"/>
       <c r="I1" s="112"/>
       <c r="J1" s="112"/>
       <c r="K1" s="112"/>
@@ -5596,7 +5647,7 @@
       <c r="G2" s="155" t="s">
         <v>438</v>
       </c>
-      <c r="H2" s="230" t="s">
+      <c r="H2" s="250" t="s">
         <v>437</v>
       </c>
       <c r="I2" s="155" t="s">
@@ -5629,13 +5680,13 @@
       <c r="R2" s="155" t="s">
         <v>436</v>
       </c>
-      <c r="S2" s="230" t="s">
+      <c r="S2" s="250" t="s">
         <v>435</v>
       </c>
       <c r="T2" s="155" t="s">
         <v>152</v>
       </c>
-      <c r="U2" s="230" t="s">
+      <c r="U2" s="250" t="s">
         <v>434</v>
       </c>
       <c r="V2" s="155" t="s">
@@ -5665,7 +5716,7 @@
       <c r="AD2" s="155" t="s">
         <v>433</v>
       </c>
-      <c r="AE2" s="230" t="s">
+      <c r="AE2" s="250" t="s">
         <v>482</v>
       </c>
       <c r="AF2" s="155" t="s">
@@ -5677,7 +5728,7 @@
       <c r="AH2" s="155" t="s">
         <v>481</v>
       </c>
-      <c r="AI2" s="230" t="s">
+      <c r="AI2" s="250" t="s">
         <v>480</v>
       </c>
     </row>
@@ -5691,7 +5742,7 @@
       <c r="G3" s="155" t="s">
         <v>427</v>
       </c>
-      <c r="H3" s="230"/>
+      <c r="H3" s="250"/>
       <c r="I3" s="155" t="s">
         <v>479</v>
       </c>
@@ -5722,11 +5773,11 @@
       <c r="R3" s="155" t="s">
         <v>414</v>
       </c>
-      <c r="S3" s="230"/>
+      <c r="S3" s="250"/>
       <c r="T3" s="155" t="s">
         <v>411</v>
       </c>
-      <c r="U3" s="230"/>
+      <c r="U3" s="250"/>
       <c r="V3" s="155" t="s">
         <v>470</v>
       </c>
@@ -5754,7 +5805,7 @@
       <c r="AD3" s="155" t="s">
         <v>462</v>
       </c>
-      <c r="AE3" s="230"/>
+      <c r="AE3" s="250"/>
       <c r="AF3" s="155" t="s">
         <v>461</v>
       </c>
@@ -5764,7 +5815,7 @@
       <c r="AH3" s="155" t="s">
         <v>391</v>
       </c>
-      <c r="AI3" s="230"/>
+      <c r="AI3" s="250"/>
     </row>
     <row r="4" spans="1:35" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="158"/>
@@ -5786,7 +5837,7 @@
       <c r="G4" s="155" t="s">
         <v>377</v>
       </c>
-      <c r="H4" s="230"/>
+      <c r="H4" s="250"/>
       <c r="I4" s="155" t="s">
         <v>460</v>
       </c>
@@ -5817,11 +5868,11 @@
       <c r="R4" s="155" t="s">
         <v>363</v>
       </c>
-      <c r="S4" s="230"/>
+      <c r="S4" s="250"/>
       <c r="T4" s="155" t="s">
         <v>359</v>
       </c>
-      <c r="U4" s="230"/>
+      <c r="U4" s="250"/>
       <c r="V4" s="155" t="s">
         <v>451</v>
       </c>
@@ -5849,7 +5900,7 @@
       <c r="AD4" s="155" t="s">
         <v>443</v>
       </c>
-      <c r="AE4" s="230"/>
+      <c r="AE4" s="250"/>
       <c r="AF4" s="155" t="s">
         <v>442</v>
       </c>
@@ -5859,7 +5910,7 @@
       <c r="AH4" s="155" t="s">
         <v>338</v>
       </c>
-      <c r="AI4" s="230"/>
+      <c r="AI4" s="250"/>
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A5" s="161" t="s">
@@ -6963,13 +7014,13 @@
       <c r="G2" s="155" t="s">
         <v>436</v>
       </c>
-      <c r="H2" s="230" t="s">
+      <c r="H2" s="250" t="s">
         <v>435</v>
       </c>
       <c r="I2" s="155" t="s">
         <v>152</v>
       </c>
-      <c r="J2" s="230" t="s">
+      <c r="J2" s="250" t="s">
         <v>434</v>
       </c>
     </row>
@@ -6983,11 +7034,11 @@
       <c r="G3" s="155" t="s">
         <v>414</v>
       </c>
-      <c r="H3" s="230"/>
+      <c r="H3" s="250"/>
       <c r="I3" s="155" t="s">
         <v>411</v>
       </c>
-      <c r="J3" s="230"/>
+      <c r="J3" s="250"/>
     </row>
     <row r="4" spans="1:10" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="177"/>
@@ -7009,11 +7060,11 @@
       <c r="G4" s="155" t="s">
         <v>363</v>
       </c>
-      <c r="H4" s="230"/>
+      <c r="H4" s="250"/>
       <c r="I4" s="155" t="s">
         <v>359</v>
       </c>
-      <c r="J4" s="230"/>
+      <c r="J4" s="250"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="171" t="s">
@@ -7412,7 +7463,7 @@
       <c r="G2" s="155" t="s">
         <v>438</v>
       </c>
-      <c r="H2" s="230" t="s">
+      <c r="H2" s="250" t="s">
         <v>437</v>
       </c>
       <c r="I2" s="154" t="s">
@@ -7457,7 +7508,7 @@
       <c r="V2" s="154" t="s">
         <v>436</v>
       </c>
-      <c r="W2" s="230" t="s">
+      <c r="W2" s="250" t="s">
         <v>435</v>
       </c>
       <c r="X2" s="155" t="s">
@@ -7472,7 +7523,7 @@
       <c r="AA2" s="155" t="s">
         <v>152</v>
       </c>
-      <c r="AB2" s="230" t="s">
+      <c r="AB2" s="250" t="s">
         <v>434</v>
       </c>
       <c r="AC2" s="152" t="s">
@@ -7502,7 +7553,7 @@
       <c r="AK2" s="152" t="s">
         <v>433</v>
       </c>
-      <c r="AL2" s="230" t="s">
+      <c r="AL2" s="250" t="s">
         <v>432</v>
       </c>
       <c r="AM2" s="152" t="s">
@@ -7544,7 +7595,7 @@
       <c r="AY2" s="152" t="s">
         <v>431</v>
       </c>
-      <c r="AZ2" s="230" t="s">
+      <c r="AZ2" s="250" t="s">
         <v>430</v>
       </c>
       <c r="BA2" s="151" t="s">
@@ -7574,7 +7625,7 @@
       <c r="BI2" s="151" t="s">
         <v>429</v>
       </c>
-      <c r="BJ2" s="230" t="s">
+      <c r="BJ2" s="250" t="s">
         <v>428</v>
       </c>
       <c r="BK2"/>
@@ -7589,7 +7640,7 @@
       <c r="G3" s="155" t="s">
         <v>427</v>
       </c>
-      <c r="H3" s="230"/>
+      <c r="H3" s="250"/>
       <c r="I3" s="154" t="s">
         <v>426</v>
       </c>
@@ -7630,7 +7681,7 @@
       <c r="V3" s="154" t="s">
         <v>414</v>
       </c>
-      <c r="W3" s="230"/>
+      <c r="W3" s="250"/>
       <c r="X3" s="150"/>
       <c r="Y3" s="155" t="s">
         <v>413</v>
@@ -7641,7 +7692,7 @@
       <c r="AA3" s="155" t="s">
         <v>411</v>
       </c>
-      <c r="AB3" s="230"/>
+      <c r="AB3" s="250"/>
       <c r="AC3" s="152" t="s">
         <v>410</v>
       </c>
@@ -7669,7 +7720,7 @@
       <c r="AK3" s="152" t="s">
         <v>404</v>
       </c>
-      <c r="AL3" s="230"/>
+      <c r="AL3" s="250"/>
       <c r="AM3" s="152" t="s">
         <v>403</v>
       </c>
@@ -7709,7 +7760,7 @@
       <c r="AY3" s="152" t="s">
         <v>391</v>
       </c>
-      <c r="AZ3" s="230"/>
+      <c r="AZ3" s="250"/>
       <c r="BA3" s="151" t="s">
         <v>390</v>
       </c>
@@ -7737,7 +7788,7 @@
       <c r="BI3" s="151" t="s">
         <v>382</v>
       </c>
-      <c r="BJ3" s="230"/>
+      <c r="BJ3" s="250"/>
     </row>
     <row r="4" spans="1:63" s="112" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="157"/>
@@ -7759,7 +7810,7 @@
       <c r="G4" s="155" t="s">
         <v>377</v>
       </c>
-      <c r="H4" s="230"/>
+      <c r="H4" s="250"/>
       <c r="I4" s="154" t="s">
         <v>376</v>
       </c>
@@ -7802,7 +7853,7 @@
       <c r="V4" s="154" t="s">
         <v>363</v>
       </c>
-      <c r="W4" s="230"/>
+      <c r="W4" s="250"/>
       <c r="X4" s="153" t="s">
         <v>362</v>
       </c>
@@ -7815,7 +7866,7 @@
       <c r="AA4" s="153" t="s">
         <v>359</v>
       </c>
-      <c r="AB4" s="230"/>
+      <c r="AB4" s="250"/>
       <c r="AC4" s="152" t="s">
         <v>358</v>
       </c>
@@ -7843,7 +7894,7 @@
       <c r="AK4" s="152" t="s">
         <v>351</v>
       </c>
-      <c r="AL4" s="230"/>
+      <c r="AL4" s="250"/>
       <c r="AM4" s="152" t="s">
         <v>350</v>
       </c>
@@ -7883,7 +7934,7 @@
       <c r="AY4" s="152" t="s">
         <v>338</v>
       </c>
-      <c r="AZ4" s="230"/>
+      <c r="AZ4" s="250"/>
       <c r="BA4" s="151" t="s">
         <v>337</v>
       </c>
@@ -7911,7 +7962,7 @@
       <c r="BI4" s="151" t="s">
         <v>329</v>
       </c>
-      <c r="BJ4" s="230"/>
+      <c r="BJ4" s="250"/>
       <c r="BK4"/>
     </row>
     <row r="5" spans="1:63" s="112" customFormat="1" ht="15" x14ac:dyDescent="0.2">
@@ -7920,7 +7971,7 @@
       </c>
       <c r="B5" s="132"/>
       <c r="C5" s="132"/>
-      <c r="D5" s="215"/>
+      <c r="D5" s="212"/>
       <c r="E5" s="132" t="s">
         <v>328</v>
       </c>
@@ -8132,7 +8183,7 @@
       </c>
       <c r="B6" s="132"/>
       <c r="C6" s="132"/>
-      <c r="D6" s="216" t="str">
+      <c r="D6" s="213" t="str">
         <f t="shared" ref="D6:D15" si="6">IF(ISBLANK($D$5),"",$D$5)</f>
         <v/>
       </c>
@@ -8346,7 +8397,7 @@
       </c>
       <c r="B7" s="132"/>
       <c r="C7" s="132"/>
-      <c r="D7" s="216" t="str">
+      <c r="D7" s="213" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -8560,7 +8611,7 @@
       </c>
       <c r="B8" s="132"/>
       <c r="C8" s="132"/>
-      <c r="D8" s="216" t="str">
+      <c r="D8" s="213" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -8774,7 +8825,7 @@
       </c>
       <c r="B9" s="132"/>
       <c r="C9" s="132"/>
-      <c r="D9" s="216" t="str">
+      <c r="D9" s="213" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -8988,7 +9039,7 @@
       </c>
       <c r="B10" s="132"/>
       <c r="C10" s="132"/>
-      <c r="D10" s="216" t="str">
+      <c r="D10" s="213" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -9202,7 +9253,7 @@
       </c>
       <c r="B11" s="132"/>
       <c r="C11" s="132"/>
-      <c r="D11" s="216" t="str">
+      <c r="D11" s="213" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -9416,7 +9467,7 @@
       </c>
       <c r="B12" s="132"/>
       <c r="C12" s="132"/>
-      <c r="D12" s="216" t="str">
+      <c r="D12" s="213" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -9630,7 +9681,7 @@
       </c>
       <c r="B13" s="132"/>
       <c r="C13" s="132"/>
-      <c r="D13" s="216" t="str">
+      <c r="D13" s="213" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -9844,7 +9895,7 @@
       </c>
       <c r="B14" s="132"/>
       <c r="C14" s="132"/>
-      <c r="D14" s="216" t="str">
+      <c r="D14" s="213" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -10058,7 +10109,7 @@
       </c>
       <c r="B15" s="132"/>
       <c r="C15" s="132"/>
-      <c r="D15" s="216" t="str">
+      <c r="D15" s="213" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -10569,17 +10620,17 @@
       <c r="AZ18" s="111"/>
     </row>
     <row r="19" spans="1:62" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E19" s="233" t="s">
+      <c r="E19" s="253" t="s">
         <v>440</v>
       </c>
-      <c r="F19" s="234"/>
-      <c r="G19" s="234"/>
-      <c r="H19" s="234"/>
-      <c r="I19" s="234"/>
-      <c r="J19" s="234"/>
-      <c r="K19" s="234"/>
-      <c r="L19" s="234"/>
-      <c r="M19" s="235"/>
+      <c r="F19" s="254"/>
+      <c r="G19" s="254"/>
+      <c r="H19" s="254"/>
+      <c r="I19" s="254"/>
+      <c r="J19" s="254"/>
+      <c r="K19" s="254"/>
+      <c r="L19" s="254"/>
+      <c r="M19" s="255"/>
     </row>
     <row r="20" spans="1:62" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
     <row r="22" spans="1:62" x14ac:dyDescent="0.2">
@@ -10695,7 +10746,7 @@
       <c r="G2" s="155" t="s">
         <v>438</v>
       </c>
-      <c r="H2" s="230" t="s">
+      <c r="H2" s="250" t="s">
         <v>437</v>
       </c>
       <c r="I2" s="155" t="s">
@@ -10728,13 +10779,13 @@
       <c r="R2" s="155" t="s">
         <v>436</v>
       </c>
-      <c r="S2" s="230" t="s">
+      <c r="S2" s="250" t="s">
         <v>435</v>
       </c>
       <c r="T2" s="155" t="s">
         <v>152</v>
       </c>
-      <c r="U2" s="230" t="s">
+      <c r="U2" s="250" t="s">
         <v>434</v>
       </c>
       <c r="V2" s="155" t="s">
@@ -10764,7 +10815,7 @@
       <c r="AD2" s="155" t="s">
         <v>433</v>
       </c>
-      <c r="AE2" s="230" t="s">
+      <c r="AE2" s="250" t="s">
         <v>482</v>
       </c>
       <c r="AF2" s="155" t="s">
@@ -10776,7 +10827,7 @@
       <c r="AH2" s="155" t="s">
         <v>481</v>
       </c>
-      <c r="AI2" s="230" t="s">
+      <c r="AI2" s="250" t="s">
         <v>480</v>
       </c>
     </row>
@@ -10790,7 +10841,7 @@
       <c r="G3" s="155" t="s">
         <v>427</v>
       </c>
-      <c r="H3" s="230"/>
+      <c r="H3" s="250"/>
       <c r="I3" s="155" t="s">
         <v>479</v>
       </c>
@@ -10821,11 +10872,11 @@
       <c r="R3" s="155" t="s">
         <v>414</v>
       </c>
-      <c r="S3" s="230"/>
+      <c r="S3" s="250"/>
       <c r="T3" s="155" t="s">
         <v>411</v>
       </c>
-      <c r="U3" s="230"/>
+      <c r="U3" s="250"/>
       <c r="V3" s="155" t="s">
         <v>470</v>
       </c>
@@ -10853,7 +10904,7 @@
       <c r="AD3" s="155" t="s">
         <v>462</v>
       </c>
-      <c r="AE3" s="230"/>
+      <c r="AE3" s="250"/>
       <c r="AF3" s="155" t="s">
         <v>461</v>
       </c>
@@ -10863,7 +10914,7 @@
       <c r="AH3" s="155" t="s">
         <v>391</v>
       </c>
-      <c r="AI3" s="230"/>
+      <c r="AI3" s="250"/>
     </row>
     <row r="4" spans="1:62" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="158"/>
@@ -10885,7 +10936,7 @@
       <c r="G4" s="155" t="s">
         <v>377</v>
       </c>
-      <c r="H4" s="230"/>
+      <c r="H4" s="250"/>
       <c r="I4" s="155" t="s">
         <v>460</v>
       </c>
@@ -10916,11 +10967,11 @@
       <c r="R4" s="155" t="s">
         <v>363</v>
       </c>
-      <c r="S4" s="230"/>
+      <c r="S4" s="250"/>
       <c r="T4" s="155" t="s">
         <v>359</v>
       </c>
-      <c r="U4" s="230"/>
+      <c r="U4" s="250"/>
       <c r="V4" s="155" t="s">
         <v>451</v>
       </c>
@@ -10948,7 +10999,7 @@
       <c r="AD4" s="155" t="s">
         <v>443</v>
       </c>
-      <c r="AE4" s="230"/>
+      <c r="AE4" s="250"/>
       <c r="AF4" s="155" t="s">
         <v>442</v>
       </c>
@@ -10958,7 +11009,7 @@
       <c r="AH4" s="155" t="s">
         <v>338</v>
       </c>
-      <c r="AI4" s="230"/>
+      <c r="AI4" s="250"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="161" t="s">
@@ -12550,32 +12601,32 @@
       <c r="S17" s="111"/>
     </row>
     <row r="18" spans="5:19" ht="21" x14ac:dyDescent="0.25">
-      <c r="E18" s="236" t="s">
+      <c r="E18" s="256" t="s">
         <v>517</v>
       </c>
-      <c r="F18" s="237"/>
-      <c r="G18" s="237"/>
-      <c r="H18" s="237"/>
-      <c r="I18" s="237"/>
-      <c r="J18" s="237"/>
-      <c r="K18" s="237"/>
-      <c r="L18" s="237"/>
-      <c r="M18" s="237"/>
+      <c r="F18" s="257"/>
+      <c r="G18" s="257"/>
+      <c r="H18" s="257"/>
+      <c r="I18" s="257"/>
+      <c r="J18" s="257"/>
+      <c r="K18" s="257"/>
+      <c r="L18" s="257"/>
+      <c r="M18" s="257"/>
     </row>
     <row r="19" spans="5:19" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="20" spans="5:19" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E20" s="233" t="s">
+      <c r="E20" s="253" t="s">
         <v>440</v>
       </c>
-      <c r="F20" s="234"/>
-      <c r="G20" s="234"/>
-      <c r="H20" s="234"/>
-      <c r="I20" s="234"/>
-      <c r="J20" s="234"/>
-      <c r="K20" s="234"/>
-      <c r="L20" s="234"/>
-      <c r="M20" s="234"/>
-      <c r="N20" s="213"/>
+      <c r="F20" s="254"/>
+      <c r="G20" s="254"/>
+      <c r="H20" s="254"/>
+      <c r="I20" s="254"/>
+      <c r="J20" s="254"/>
+      <c r="K20" s="254"/>
+      <c r="L20" s="254"/>
+      <c r="M20" s="254"/>
+      <c r="N20" s="210"/>
     </row>
     <row r="21" spans="5:19" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
     <row r="23" spans="5:19" x14ac:dyDescent="0.2">
@@ -12689,13 +12740,13 @@
       <c r="G2" s="155" t="s">
         <v>436</v>
       </c>
-      <c r="H2" s="230" t="s">
+      <c r="H2" s="250" t="s">
         <v>435</v>
       </c>
       <c r="I2" s="155" t="s">
         <v>152</v>
       </c>
-      <c r="J2" s="230" t="s">
+      <c r="J2" s="250" t="s">
         <v>434</v>
       </c>
     </row>
@@ -12709,11 +12760,11 @@
       <c r="G3" s="155" t="s">
         <v>414</v>
       </c>
-      <c r="H3" s="230"/>
+      <c r="H3" s="250"/>
       <c r="I3" s="155" t="s">
         <v>411</v>
       </c>
-      <c r="J3" s="230"/>
+      <c r="J3" s="250"/>
     </row>
     <row r="4" spans="1:62" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="177"/>
@@ -12735,11 +12786,11 @@
       <c r="G4" s="155" t="s">
         <v>363</v>
       </c>
-      <c r="H4" s="230"/>
+      <c r="H4" s="250"/>
       <c r="I4" s="155" t="s">
         <v>359</v>
       </c>
-      <c r="J4" s="230"/>
+      <c r="J4" s="250"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="171" t="s">
@@ -13062,23 +13113,23 @@
       </c>
     </row>
     <row r="16" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="E16" s="238" t="s">
+      <c r="E16" s="258" t="s">
         <v>516</v>
       </c>
-      <c r="F16" s="239"/>
-      <c r="G16" s="239"/>
-      <c r="H16" s="239"/>
-      <c r="I16" s="239"/>
-      <c r="J16" s="239"/>
+      <c r="F16" s="259"/>
+      <c r="G16" s="259"/>
+      <c r="H16" s="259"/>
+      <c r="I16" s="259"/>
+      <c r="J16" s="259"/>
     </row>
     <row r="17" spans="4:10" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D17" s="110"/>
-      <c r="E17" s="239"/>
-      <c r="F17" s="239"/>
-      <c r="G17" s="239"/>
-      <c r="H17" s="239"/>
-      <c r="I17" s="239"/>
-      <c r="J17" s="239"/>
+      <c r="E17" s="259"/>
+      <c r="F17" s="259"/>
+      <c r="G17" s="259"/>
+      <c r="H17" s="259"/>
+      <c r="I17" s="259"/>
+      <c r="J17" s="259"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -13447,14 +13498,14 @@
       <c r="H1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="EA1" s="224" t="s">
+      <c r="EA1" s="244" t="s">
         <v>492</v>
       </c>
-      <c r="EB1" s="224"/>
-      <c r="EC1" s="224"/>
-      <c r="ED1" s="224"/>
-      <c r="EE1" s="224"/>
-      <c r="EF1" s="224"/>
+      <c r="EB1" s="244"/>
+      <c r="EC1" s="244"/>
+      <c r="ED1" s="244"/>
+      <c r="EE1" s="244"/>
+      <c r="EF1" s="244"/>
     </row>
     <row r="2" spans="1:136" ht="66" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="24" t="s">
@@ -13531,7 +13582,7 @@
     <row r="1" spans="1:16" s="4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3"/>
       <c r="B1" s="5"/>
-      <c r="C1" s="214" t="s">
+      <c r="C1" s="211" t="s">
         <v>507</v>
       </c>
       <c r="D1" s="7"/>
@@ -13576,20 +13627,20 @@
     </row>
     <row r="4" spans="1:16" ht="40" x14ac:dyDescent="0.2">
       <c r="C4" s="9"/>
-      <c r="E4" s="225" t="s">
+      <c r="E4" s="245" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="226"/>
-      <c r="G4" s="226"/>
-      <c r="H4" s="226"/>
-      <c r="I4" s="227"/>
-      <c r="J4" s="225" t="s">
+      <c r="F4" s="246"/>
+      <c r="G4" s="246"/>
+      <c r="H4" s="246"/>
+      <c r="I4" s="247"/>
+      <c r="J4" s="245" t="s">
         <v>28</v>
       </c>
-      <c r="K4" s="226"/>
-      <c r="L4" s="226"/>
-      <c r="M4" s="226"/>
-      <c r="N4" s="227"/>
+      <c r="K4" s="246"/>
+      <c r="L4" s="246"/>
+      <c r="M4" s="246"/>
+      <c r="N4" s="247"/>
       <c r="O4" s="30" t="s">
         <v>29</v>
       </c>
@@ -15188,16 +15239,16 @@
   <sheetData>
     <row r="1" spans="1:62" s="64" customFormat="1" ht="12" x14ac:dyDescent="0.15">
       <c r="A1" s="107"/>
-      <c r="B1" s="229" t="s">
+      <c r="B1" s="249" t="s">
         <v>439</v>
       </c>
-      <c r="C1" s="229"/>
-      <c r="D1" s="229"/>
-      <c r="E1" s="229"/>
-      <c r="F1" s="229"/>
-      <c r="G1" s="229"/>
-      <c r="H1" s="229"/>
-      <c r="I1" s="229"/>
+      <c r="C1" s="249"/>
+      <c r="D1" s="249"/>
+      <c r="E1" s="249"/>
+      <c r="F1" s="249"/>
+      <c r="G1" s="249"/>
+      <c r="H1" s="249"/>
+      <c r="I1" s="249"/>
       <c r="AC1" s="106"/>
       <c r="AD1" s="106"/>
       <c r="AE1" s="106"/>
@@ -15218,7 +15269,7 @@
       <c r="G2" s="102" t="s">
         <v>438</v>
       </c>
-      <c r="H2" s="228" t="s">
+      <c r="H2" s="248" t="s">
         <v>437</v>
       </c>
       <c r="I2" s="101" t="s">
@@ -15263,7 +15314,7 @@
       <c r="V2" s="101" t="s">
         <v>436</v>
       </c>
-      <c r="W2" s="228" t="s">
+      <c r="W2" s="248" t="s">
         <v>435</v>
       </c>
       <c r="X2" s="102" t="s">
@@ -15278,7 +15329,7 @@
       <c r="AA2" s="102" t="s">
         <v>152</v>
       </c>
-      <c r="AB2" s="228" t="s">
+      <c r="AB2" s="248" t="s">
         <v>434</v>
       </c>
       <c r="AC2" s="98" t="s">
@@ -15308,7 +15359,7 @@
       <c r="AK2" s="98" t="s">
         <v>433</v>
       </c>
-      <c r="AL2" s="228" t="s">
+      <c r="AL2" s="248" t="s">
         <v>432</v>
       </c>
       <c r="AM2" s="98" t="s">
@@ -15350,7 +15401,7 @@
       <c r="AY2" s="98" t="s">
         <v>431</v>
       </c>
-      <c r="AZ2" s="228" t="s">
+      <c r="AZ2" s="248" t="s">
         <v>430</v>
       </c>
       <c r="BA2" s="97" t="s">
@@ -15380,7 +15431,7 @@
       <c r="BI2" s="97" t="s">
         <v>429</v>
       </c>
-      <c r="BJ2" s="228" t="s">
+      <c r="BJ2" s="248" t="s">
         <v>428</v>
       </c>
     </row>
@@ -15394,7 +15445,7 @@
       <c r="G3" s="102" t="s">
         <v>427</v>
       </c>
-      <c r="H3" s="228"/>
+      <c r="H3" s="248"/>
       <c r="I3" s="101" t="s">
         <v>426</v>
       </c>
@@ -15435,7 +15486,7 @@
       <c r="V3" s="101" t="s">
         <v>414</v>
       </c>
-      <c r="W3" s="228"/>
+      <c r="W3" s="248"/>
       <c r="X3" s="96"/>
       <c r="Y3" s="102" t="s">
         <v>413</v>
@@ -15446,7 +15497,7 @@
       <c r="AA3" s="102" t="s">
         <v>411</v>
       </c>
-      <c r="AB3" s="228"/>
+      <c r="AB3" s="248"/>
       <c r="AC3" s="98" t="s">
         <v>410</v>
       </c>
@@ -15474,7 +15525,7 @@
       <c r="AK3" s="98" t="s">
         <v>404</v>
       </c>
-      <c r="AL3" s="228"/>
+      <c r="AL3" s="248"/>
       <c r="AM3" s="98" t="s">
         <v>403</v>
       </c>
@@ -15514,7 +15565,7 @@
       <c r="AY3" s="98" t="s">
         <v>391</v>
       </c>
-      <c r="AZ3" s="228"/>
+      <c r="AZ3" s="248"/>
       <c r="BA3" s="97" t="s">
         <v>390</v>
       </c>
@@ -15542,7 +15593,7 @@
       <c r="BI3" s="97" t="s">
         <v>382</v>
       </c>
-      <c r="BJ3" s="228"/>
+      <c r="BJ3" s="248"/>
     </row>
     <row r="4" spans="1:62" s="64" customFormat="1" ht="60" x14ac:dyDescent="0.15">
       <c r="A4" s="104"/>
@@ -15564,7 +15615,7 @@
       <c r="G4" s="102" t="s">
         <v>377</v>
       </c>
-      <c r="H4" s="228"/>
+      <c r="H4" s="248"/>
       <c r="I4" s="101" t="s">
         <v>376</v>
       </c>
@@ -15607,7 +15658,7 @@
       <c r="V4" s="100" t="s">
         <v>363</v>
       </c>
-      <c r="W4" s="228"/>
+      <c r="W4" s="248"/>
       <c r="X4" s="99" t="s">
         <v>362</v>
       </c>
@@ -15620,7 +15671,7 @@
       <c r="AA4" s="99" t="s">
         <v>359</v>
       </c>
-      <c r="AB4" s="228"/>
+      <c r="AB4" s="248"/>
       <c r="AC4" s="98" t="s">
         <v>358</v>
       </c>
@@ -15648,7 +15699,7 @@
       <c r="AK4" s="98" t="s">
         <v>351</v>
       </c>
-      <c r="AL4" s="228"/>
+      <c r="AL4" s="248"/>
       <c r="AM4" s="98" t="s">
         <v>350</v>
       </c>
@@ -15688,7 +15739,7 @@
       <c r="AY4" s="98" t="s">
         <v>338</v>
       </c>
-      <c r="AZ4" s="228"/>
+      <c r="AZ4" s="248"/>
       <c r="BA4" s="97" t="s">
         <v>337</v>
       </c>
@@ -15716,7 +15767,7 @@
       <c r="BI4" s="97" t="s">
         <v>329</v>
       </c>
-      <c r="BJ4" s="228"/>
+      <c r="BJ4" s="248"/>
     </row>
     <row r="5" spans="1:62" s="64" customFormat="1" ht="144" x14ac:dyDescent="0.15">
       <c r="A5" s="72" t="s">
@@ -16694,7 +16745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:62" s="64" customFormat="1" ht="36" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:62" s="64" customFormat="1" ht="48" x14ac:dyDescent="0.15">
       <c r="A13" s="72" t="s">
         <v>233</v>
       </c>
@@ -17406,16 +17457,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:62" s="112" customFormat="1" ht="23.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B1" s="231" t="s">
+      <c r="B1" s="251" t="s">
         <v>439</v>
       </c>
-      <c r="C1" s="231"/>
-      <c r="D1" s="231"/>
-      <c r="E1" s="231"/>
-      <c r="F1" s="231"/>
-      <c r="G1" s="231"/>
-      <c r="H1" s="231"/>
-      <c r="I1" s="231"/>
+      <c r="C1" s="251"/>
+      <c r="D1" s="251"/>
+      <c r="E1" s="251"/>
+      <c r="F1" s="251"/>
+      <c r="G1" s="251"/>
+      <c r="H1" s="251"/>
+      <c r="I1" s="251"/>
     </row>
     <row r="2" spans="1:62" s="112" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="158"/>
@@ -17427,7 +17478,7 @@
       <c r="G2" s="155" t="s">
         <v>438</v>
       </c>
-      <c r="H2" s="230" t="s">
+      <c r="H2" s="250" t="s">
         <v>437</v>
       </c>
       <c r="I2" s="154" t="s">
@@ -17472,7 +17523,7 @@
       <c r="V2" s="154" t="s">
         <v>436</v>
       </c>
-      <c r="W2" s="230" t="s">
+      <c r="W2" s="250" t="s">
         <v>435</v>
       </c>
       <c r="X2" s="155" t="s">
@@ -17487,7 +17538,7 @@
       <c r="AA2" s="155" t="s">
         <v>152</v>
       </c>
-      <c r="AB2" s="230" t="s">
+      <c r="AB2" s="250" t="s">
         <v>434</v>
       </c>
       <c r="AC2" s="152" t="s">
@@ -17517,7 +17568,7 @@
       <c r="AK2" s="152" t="s">
         <v>433</v>
       </c>
-      <c r="AL2" s="230" t="s">
+      <c r="AL2" s="250" t="s">
         <v>432</v>
       </c>
       <c r="AM2" s="152" t="s">
@@ -17559,7 +17610,7 @@
       <c r="AY2" s="152" t="s">
         <v>431</v>
       </c>
-      <c r="AZ2" s="230" t="s">
+      <c r="AZ2" s="250" t="s">
         <v>430</v>
       </c>
       <c r="BA2" s="151" t="s">
@@ -17589,7 +17640,7 @@
       <c r="BI2" s="151" t="s">
         <v>429</v>
       </c>
-      <c r="BJ2" s="230" t="s">
+      <c r="BJ2" s="250" t="s">
         <v>428</v>
       </c>
     </row>
@@ -17603,7 +17654,7 @@
       <c r="G3" s="155" t="s">
         <v>427</v>
       </c>
-      <c r="H3" s="230"/>
+      <c r="H3" s="250"/>
       <c r="I3" s="154" t="s">
         <v>426</v>
       </c>
@@ -17644,7 +17695,7 @@
       <c r="V3" s="154" t="s">
         <v>414</v>
       </c>
-      <c r="W3" s="230"/>
+      <c r="W3" s="250"/>
       <c r="X3" s="150"/>
       <c r="Y3" s="155" t="s">
         <v>413</v>
@@ -17655,7 +17706,7 @@
       <c r="AA3" s="155" t="s">
         <v>411</v>
       </c>
-      <c r="AB3" s="230"/>
+      <c r="AB3" s="250"/>
       <c r="AC3" s="152" t="s">
         <v>410</v>
       </c>
@@ -17683,7 +17734,7 @@
       <c r="AK3" s="152" t="s">
         <v>404</v>
       </c>
-      <c r="AL3" s="230"/>
+      <c r="AL3" s="250"/>
       <c r="AM3" s="152" t="s">
         <v>403</v>
       </c>
@@ -17723,7 +17774,7 @@
       <c r="AY3" s="152" t="s">
         <v>391</v>
       </c>
-      <c r="AZ3" s="230"/>
+      <c r="AZ3" s="250"/>
       <c r="BA3" s="151" t="s">
         <v>390</v>
       </c>
@@ -17751,7 +17802,7 @@
       <c r="BI3" s="151" t="s">
         <v>382</v>
       </c>
-      <c r="BJ3" s="230"/>
+      <c r="BJ3" s="250"/>
     </row>
     <row r="4" spans="1:62" s="112" customFormat="1" ht="60" x14ac:dyDescent="0.15">
       <c r="A4" s="157"/>
@@ -17773,7 +17824,7 @@
       <c r="G4" s="155" t="s">
         <v>377</v>
       </c>
-      <c r="H4" s="230"/>
+      <c r="H4" s="250"/>
       <c r="I4" s="154" t="s">
         <v>376</v>
       </c>
@@ -17816,7 +17867,7 @@
       <c r="V4" s="154" t="s">
         <v>363</v>
       </c>
-      <c r="W4" s="230"/>
+      <c r="W4" s="250"/>
       <c r="X4" s="153" t="s">
         <v>362</v>
       </c>
@@ -17829,7 +17880,7 @@
       <c r="AA4" s="153" t="s">
         <v>359</v>
       </c>
-      <c r="AB4" s="230"/>
+      <c r="AB4" s="250"/>
       <c r="AC4" s="152" t="s">
         <v>358</v>
       </c>
@@ -17857,7 +17908,7 @@
       <c r="AK4" s="152" t="s">
         <v>351</v>
       </c>
-      <c r="AL4" s="230"/>
+      <c r="AL4" s="250"/>
       <c r="AM4" s="152" t="s">
         <v>350</v>
       </c>
@@ -17897,7 +17948,7 @@
       <c r="AY4" s="152" t="s">
         <v>338</v>
       </c>
-      <c r="AZ4" s="230"/>
+      <c r="AZ4" s="250"/>
       <c r="BA4" s="151" t="s">
         <v>337</v>
       </c>
@@ -17925,7 +17976,7 @@
       <c r="BI4" s="151" t="s">
         <v>329</v>
       </c>
-      <c r="BJ4" s="230"/>
+      <c r="BJ4" s="250"/>
     </row>
     <row r="5" spans="1:62" s="112" customFormat="1" ht="11" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="122" t="s">

</xml_diff>

<commit_message>
changes extractor format notice
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1867FA-6BD2-604C-AC39-EE3945E7A4B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66E1AFE1-6CA2-E94C-AACA-7E3E27C0DD10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="22940" windowHeight="13240" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -2688,16 +2688,76 @@
     </r>
   </si>
   <si>
-    <t>→ Sélectionner la juridiction souhaitée à partir du menu déroulant qui se trouve dans la cellule D5 identifiée en orange.</t>
+    <t>#! HYPERLINK firstLink.label firstLink.url</t>
+  </si>
+  <si>
+    <t>#! HYPERLINK secondLink.label secondLink.url</t>
+  </si>
+  <si>
+    <t>#! HYPERLINK thirdLink.label thirdLink.url</t>
   </si>
   <si>
     <r>
-      <t xml:space="preserve">→ Sélectionner la juridiction souhaitée à partir du menu déroulant qui se trouve dans la cellule D5 identifiée en </t>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF2D46E0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>→ Sélectionner la juridiction souhaitée à partir du menu déroulant qui se trouve dans la cellule D5 identifiée en</t>
     </r>
     <r>
       <rPr>
         <b/>
-        <sz val="16"/>
+        <sz val="12"/>
+        <color rgb="FF860000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>orange.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF2D46E0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>→ Sélectionner la juridiction souhaitée à partir du menu déroulant qui se trouve dans la cellule D5 identifiée en</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF860000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
         <color theme="5"/>
         <rFont val="Calibri (Corps)"/>
       </rPr>
@@ -2706,7 +2766,7 @@
     <r>
       <rPr>
         <b/>
-        <sz val="16"/>
+        <sz val="12"/>
         <color rgb="FF860000"/>
         <rFont val="Calibri"/>
         <family val="2"/>
@@ -2714,15 +2774,6 @@
       </rPr>
       <t>.</t>
     </r>
-  </si>
-  <si>
-    <t>#! HYPERLINK firstLink.label firstLink.url</t>
-  </si>
-  <si>
-    <t>#! HYPERLINK secondLink.label secondLink.url</t>
-  </si>
-  <si>
-    <t>#! HYPERLINK thirdLink.label thirdLink.url</t>
   </si>
 </sst>
 </file>
@@ -2737,9 +2788,16 @@
     <numFmt numFmtId="168" formatCode="0.###;0.###;\-"/>
     <numFmt numFmtId="169" formatCode="#,##0.00_ ;[Red]\-#,##0.00\ "/>
   </numFmts>
-  <fonts count="48" x14ac:knownFonts="1">
+  <fonts count="52" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -3009,14 +3067,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="22"/>
       <color theme="0"/>
@@ -3037,20 +3087,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="16"/>
-      <color rgb="FF860000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="16"/>
-      <color theme="5"/>
-      <name val="Calibri (Corps)"/>
     </font>
     <font>
       <b/>
@@ -3075,8 +3111,53 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF860000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF2D46E0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="5"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="5"/>
+      <name val="Calibri (Corps)"/>
+    </font>
   </fonts>
-  <fills count="23">
+  <fills count="29">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3209,8 +3290,44 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE64B85"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2D46E0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0B0B97"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7F02D"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B252"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="46">
+  <borders count="45">
     <border>
       <left/>
       <right/>
@@ -3576,15 +3693,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thick">
-        <color rgb="FFFF0000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thick">
         <color rgb="FFFF0000"/>
@@ -3724,16 +3832,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="7">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="260">
+  <cellXfs count="262">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -3741,7 +3848,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3750,61 +3857,61 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -3817,287 +3924,520 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="12" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="12" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="4" applyFont="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="4" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="14" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="4"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="169" fontId="21" fillId="10" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="21" fillId="11" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="21" fillId="10" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="21" fillId="11" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="9" borderId="16" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="23" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="24" fillId="13" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="25" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="169" fontId="25" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="25" fillId="9" borderId="17" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="23" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="21" fillId="10" borderId="18" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="25" fillId="0" borderId="10" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="21" fillId="10" borderId="19" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="25" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="25" fillId="9" borderId="20" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="13" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="23" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="25" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="23" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="25" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="25" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="29" fillId="9" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="4" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyProtection="1">
+      <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="4" applyFont="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="4" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="169" fontId="13" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="169" fontId="21" fillId="9" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="17" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="4"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="10" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="20" fillId="11" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="20" fillId="10" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="11" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="9" borderId="16" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="22" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="23" fillId="13" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="23" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="9" borderId="17" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="22" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="10" borderId="18" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="10" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="10" borderId="19" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="9" borderId="20" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="23" fillId="13" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="22" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="22" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="23" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="23" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="28" fillId="9" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="4" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="4" applyFont="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="12" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="9" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="169" fontId="21" fillId="10" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="21" fillId="11" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="26" fillId="11" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="20" fillId="10" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="11" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="25" fillId="11" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="23" fillId="9" borderId="16" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="9" borderId="16" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="169" fontId="23" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="13" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="25" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="13" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="23" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="25" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="8" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="26" fillId="10" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="13" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="22" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="23" fillId="13" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="169" fontId="25" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="13" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="8" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="8" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="23" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="8" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="25" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="25" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="13" borderId="15" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="23" fillId="8" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="23" fillId="8" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="29" fillId="9" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="16" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="21" fillId="10" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="23" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="29" fillId="10" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="11" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="34" fillId="8" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="9" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="34" fillId="19" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="34" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="34" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="18" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="29" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="35" fillId="9" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="31" fillId="9" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="8" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="16" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="15" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="23" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection hidden="1"/>
     </xf>
@@ -4105,269 +4445,36 @@
       <alignment horizontal="right"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="23" fillId="13" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="22" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="169" fontId="25" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="23" fillId="8" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="25" fillId="10" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="23" fillId="13" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="15" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="20" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="23" fillId="13" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="23" fillId="8" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="23" fillId="8" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="23" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="23" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="23" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="22" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="23" fillId="8" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="23" fillId="13" borderId="15" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="23" fillId="12" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="22" fillId="8" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="22" fillId="8" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="37" fillId="20" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="28" fillId="9" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="16" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="10" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="22" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="28" fillId="10" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="11" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="33" fillId="8" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="9" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="33" fillId="19" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="33" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="33" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="18" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="28" fillId="9" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="9" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="30" fillId="9" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="23" fillId="8" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="16" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="15" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="22" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="23" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="23" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="20" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="36" fillId="20" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="40" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -4393,66 +4500,51 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="22" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="22" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="22" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="22" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="4" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
     <xf numFmtId="0" fontId="40" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="15" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="15" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="43" fillId="9" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="25" xfId="6" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="27" xfId="6" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="29" xfId="6" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="40" xfId="6" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="40" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -4464,106 +4556,132 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="22" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="22" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="22" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="22" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="31" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="31" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="31" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="46" fillId="23" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="24" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="25" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="26" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="27" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="28" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="6">
     <cellStyle name="Comma 2" xfId="2" xr:uid="{C877C5E8-FCBF-114F-9ECB-F75EF7C9C0EB}"/>
-    <cellStyle name="Lien hypertexte" xfId="6" builtinId="8"/>
     <cellStyle name="Milliers" xfId="3" builtinId="3"/>
     <cellStyle name="Milliers 2" xfId="5" xr:uid="{C98A9282-6AC5-784B-80AA-54BB74A59302}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4588,6 +4706,16 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF01A94F"/>
+      <color rgb="FFF7EF2D"/>
+      <color rgb="FFFE0000"/>
+      <color rgb="FF0B0B97"/>
+      <color rgb="FF2C45E0"/>
+      <color rgb="FFCE4275"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -5349,11 +5477,11 @@
       <c r="B1" s="197" t="s">
         <v>494</v>
       </c>
-      <c r="C1" s="225" t="s">
+      <c r="C1" s="220" t="s">
         <v>495</v>
       </c>
-      <c r="D1" s="225"/>
-      <c r="E1" s="225"/>
+      <c r="D1" s="220"/>
+      <c r="E1" s="220"/>
       <c r="F1" s="198"/>
       <c r="H1" s="28" t="s">
         <v>0</v>
@@ -5362,11 +5490,11 @@
     <row r="2" spans="1:8" s="202" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="199"/>
       <c r="B2" s="200"/>
-      <c r="C2" s="226" t="s">
+      <c r="C2" s="221" t="s">
         <v>496</v>
       </c>
-      <c r="D2" s="226"/>
-      <c r="E2" s="226"/>
+      <c r="D2" s="221"/>
+      <c r="E2" s="221"/>
       <c r="F2" s="201"/>
       <c r="H2" s="28" t="s">
         <v>0</v>
@@ -5390,143 +5518,143 @@
       <c r="D4" s="207" t="s">
         <v>499</v>
       </c>
-      <c r="E4" s="232" t="s">
+      <c r="E4" s="227" t="s">
         <v>500</v>
       </c>
-      <c r="F4" s="233"/>
-      <c r="G4" s="221"/>
+      <c r="F4" s="228"/>
+      <c r="G4" s="216"/>
       <c r="H4" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="28" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="203"/>
-      <c r="B5" s="214" t="s">
+      <c r="B5" s="248" t="s">
         <v>501</v>
       </c>
-      <c r="C5" s="215" t="s">
+      <c r="C5" s="213" t="s">
         <v>502</v>
       </c>
-      <c r="D5" s="215" t="s">
+      <c r="D5" s="213" t="s">
         <v>503</v>
       </c>
-      <c r="E5" s="234" t="s">
-        <v>518</v>
-      </c>
-      <c r="F5" s="235"/>
-      <c r="G5" s="220"/>
+      <c r="E5" s="229" t="s">
+        <v>516</v>
+      </c>
+      <c r="F5" s="230"/>
+      <c r="G5" s="215"/>
       <c r="H5" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="28" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="203"/>
-      <c r="B6" s="216" t="s">
+      <c r="B6" s="249" t="s">
         <v>504</v>
       </c>
-      <c r="C6" s="217" t="s">
+      <c r="C6" s="214" t="s">
         <v>505</v>
       </c>
-      <c r="D6" s="217" t="s">
+      <c r="D6" s="214" t="s">
         <v>506</v>
       </c>
-      <c r="E6" s="236" t="s">
-        <v>519</v>
-      </c>
-      <c r="F6" s="237"/>
-      <c r="G6" s="220"/>
+      <c r="E6" s="231" t="s">
+        <v>517</v>
+      </c>
+      <c r="F6" s="232"/>
+      <c r="G6" s="215"/>
       <c r="H6" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="28" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="203"/>
-      <c r="B7" s="216" t="s">
+      <c r="B7" s="250" t="s">
         <v>507</v>
       </c>
-      <c r="C7" s="217" t="s">
+      <c r="C7" s="214" t="s">
         <v>508</v>
       </c>
-      <c r="D7" s="217" t="s">
+      <c r="D7" s="214" t="s">
         <v>509</v>
       </c>
-      <c r="E7" s="236" t="s">
-        <v>518</v>
-      </c>
-      <c r="F7" s="237"/>
-      <c r="G7" s="220"/>
+      <c r="E7" s="231" t="s">
+        <v>516</v>
+      </c>
+      <c r="F7" s="232"/>
+      <c r="G7" s="215"/>
       <c r="H7" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="28" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="203"/>
-      <c r="B8" s="218" t="s">
+      <c r="B8" s="251" t="s">
         <v>510</v>
       </c>
-      <c r="C8" s="227" t="s">
+      <c r="C8" s="222" t="s">
         <v>511</v>
       </c>
-      <c r="D8" s="227" t="s">
+      <c r="D8" s="222" t="s">
         <v>512</v>
       </c>
-      <c r="E8" s="238" t="s">
-        <v>520</v>
-      </c>
-      <c r="F8" s="239"/>
-      <c r="G8" s="220"/>
+      <c r="E8" s="233" t="s">
+        <v>518</v>
+      </c>
+      <c r="F8" s="234"/>
+      <c r="G8" s="215"/>
       <c r="H8" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:8" s="28" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="203"/>
-      <c r="B9" s="218" t="s">
+      <c r="B9" s="252" t="s">
         <v>513</v>
       </c>
-      <c r="C9" s="227"/>
-      <c r="D9" s="227"/>
-      <c r="E9" s="240"/>
-      <c r="F9" s="241"/>
-      <c r="G9" s="220"/>
+      <c r="C9" s="222"/>
+      <c r="D9" s="222"/>
+      <c r="E9" s="235"/>
+      <c r="F9" s="236"/>
+      <c r="G9" s="215"/>
       <c r="H9" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:8" s="28" customFormat="1" ht="23" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="203"/>
-      <c r="B10" s="219" t="s">
+      <c r="B10" s="253" t="s">
         <v>514</v>
       </c>
-      <c r="C10" s="228"/>
-      <c r="D10" s="228"/>
-      <c r="E10" s="242"/>
-      <c r="F10" s="243"/>
-      <c r="G10" s="220"/>
+      <c r="C10" s="223"/>
+      <c r="D10" s="223"/>
+      <c r="E10" s="237"/>
+      <c r="F10" s="238"/>
+      <c r="G10" s="215"/>
       <c r="H10" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:8" s="28" customFormat="1" ht="5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="203"/>
-      <c r="B11" s="224"/>
-      <c r="C11" s="224"/>
-      <c r="D11" s="224"/>
-      <c r="E11" s="224"/>
-      <c r="F11" s="224"/>
+      <c r="B11" s="219"/>
+      <c r="C11" s="219"/>
+      <c r="D11" s="219"/>
+      <c r="E11" s="219"/>
+      <c r="F11" s="219"/>
       <c r="H11" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="28" customFormat="1" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="203"/>
-      <c r="B12" s="222"/>
-      <c r="C12" s="231" t="s">
+      <c r="B12" s="217"/>
+      <c r="C12" s="226" t="s">
         <v>515</v>
       </c>
-      <c r="D12" s="231"/>
-      <c r="E12" s="231"/>
-      <c r="F12" s="223"/>
+      <c r="D12" s="226"/>
+      <c r="E12" s="226"/>
+      <c r="F12" s="218"/>
       <c r="H12" s="28" t="s">
         <v>0</v>
       </c>
@@ -5539,14 +5667,14 @@
       </c>
     </row>
     <row r="14" spans="1:8" s="28" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="229" t="s">
+      <c r="A14" s="224" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="229"/>
-      <c r="C14" s="229"/>
-      <c r="D14" s="229"/>
-      <c r="E14" s="229"/>
-      <c r="F14" s="230"/>
+      <c r="B14" s="224"/>
+      <c r="C14" s="224"/>
+      <c r="D14" s="224"/>
+      <c r="E14" s="224"/>
+      <c r="F14" s="225"/>
       <c r="H14" s="28" t="s">
         <v>0</v>
       </c>
@@ -5570,14 +5698,6 @@
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="E8:F10"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="B5" location="'ETPT A-JUST'!A1" display="ETPT A-JUST" xr:uid="{A4B55920-38FE-8C44-A223-5786C8919747}"/>
-    <hyperlink ref="B6" location="'ETPT Format DDG'!A1" display="ETPT Format DDG" xr:uid="{79FC5922-FC41-BA4A-995C-9841D25952FF}"/>
-    <hyperlink ref="B7" location="'Agrégats DDG'!A1" display="Agrégats DDG" xr:uid="{81D3F220-88AB-F743-B1AC-13451DEA3C28}"/>
-    <hyperlink ref="B8" location="ETPT_TJ_DDG!A1" display="ETPT_TJ_DDG" xr:uid="{43523AD2-5123-C849-8EFA-27E13C4C136A}"/>
-    <hyperlink ref="B9" location="ETPT_TPRX_DDG!A1" display="ETPT_TPRX-DDG" xr:uid="{97476A23-C1B3-284C-B5B5-53A729579959}"/>
-    <hyperlink ref="B10" location="ETPT_CPH_DDG!A1" display="ETPT_CPH_DDG" xr:uid="{1F598F93-AFA2-E243-9BD5-6F6F6C8A32A5}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
   <drawing r:id="rId1"/>
@@ -5599,16 +5719,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A1" s="252" t="s">
+      <c r="A1" s="247" t="s">
         <v>483</v>
       </c>
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
-      <c r="H1" s="252"/>
+      <c r="B1" s="247"/>
+      <c r="C1" s="247"/>
+      <c r="D1" s="247"/>
+      <c r="E1" s="247"/>
+      <c r="F1" s="247"/>
+      <c r="G1" s="247"/>
+      <c r="H1" s="247"/>
       <c r="I1" s="112"/>
       <c r="J1" s="112"/>
       <c r="K1" s="112"/>
@@ -5647,7 +5767,7 @@
       <c r="G2" s="155" t="s">
         <v>438</v>
       </c>
-      <c r="H2" s="250" t="s">
+      <c r="H2" s="245" t="s">
         <v>437</v>
       </c>
       <c r="I2" s="155" t="s">
@@ -5680,13 +5800,13 @@
       <c r="R2" s="155" t="s">
         <v>436</v>
       </c>
-      <c r="S2" s="250" t="s">
+      <c r="S2" s="245" t="s">
         <v>435</v>
       </c>
       <c r="T2" s="155" t="s">
         <v>152</v>
       </c>
-      <c r="U2" s="250" t="s">
+      <c r="U2" s="245" t="s">
         <v>434</v>
       </c>
       <c r="V2" s="155" t="s">
@@ -5716,7 +5836,7 @@
       <c r="AD2" s="155" t="s">
         <v>433</v>
       </c>
-      <c r="AE2" s="250" t="s">
+      <c r="AE2" s="245" t="s">
         <v>482</v>
       </c>
       <c r="AF2" s="155" t="s">
@@ -5728,7 +5848,7 @@
       <c r="AH2" s="155" t="s">
         <v>481</v>
       </c>
-      <c r="AI2" s="250" t="s">
+      <c r="AI2" s="245" t="s">
         <v>480</v>
       </c>
     </row>
@@ -5742,7 +5862,7 @@
       <c r="G3" s="155" t="s">
         <v>427</v>
       </c>
-      <c r="H3" s="250"/>
+      <c r="H3" s="245"/>
       <c r="I3" s="155" t="s">
         <v>479</v>
       </c>
@@ -5773,11 +5893,11 @@
       <c r="R3" s="155" t="s">
         <v>414</v>
       </c>
-      <c r="S3" s="250"/>
+      <c r="S3" s="245"/>
       <c r="T3" s="155" t="s">
         <v>411</v>
       </c>
-      <c r="U3" s="250"/>
+      <c r="U3" s="245"/>
       <c r="V3" s="155" t="s">
         <v>470</v>
       </c>
@@ -5805,7 +5925,7 @@
       <c r="AD3" s="155" t="s">
         <v>462</v>
       </c>
-      <c r="AE3" s="250"/>
+      <c r="AE3" s="245"/>
       <c r="AF3" s="155" t="s">
         <v>461</v>
       </c>
@@ -5815,7 +5935,7 @@
       <c r="AH3" s="155" t="s">
         <v>391</v>
       </c>
-      <c r="AI3" s="250"/>
+      <c r="AI3" s="245"/>
     </row>
     <row r="4" spans="1:35" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="158"/>
@@ -5837,7 +5957,7 @@
       <c r="G4" s="155" t="s">
         <v>377</v>
       </c>
-      <c r="H4" s="250"/>
+      <c r="H4" s="245"/>
       <c r="I4" s="155" t="s">
         <v>460</v>
       </c>
@@ -5868,11 +5988,11 @@
       <c r="R4" s="155" t="s">
         <v>363</v>
       </c>
-      <c r="S4" s="250"/>
+      <c r="S4" s="245"/>
       <c r="T4" s="155" t="s">
         <v>359</v>
       </c>
-      <c r="U4" s="250"/>
+      <c r="U4" s="245"/>
       <c r="V4" s="155" t="s">
         <v>451</v>
       </c>
@@ -5900,7 +6020,7 @@
       <c r="AD4" s="155" t="s">
         <v>443</v>
       </c>
-      <c r="AE4" s="250"/>
+      <c r="AE4" s="245"/>
       <c r="AF4" s="155" t="s">
         <v>442</v>
       </c>
@@ -5910,7 +6030,7 @@
       <c r="AH4" s="155" t="s">
         <v>338</v>
       </c>
-      <c r="AI4" s="250"/>
+      <c r="AI4" s="245"/>
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A5" s="161" t="s">
@@ -7014,13 +7134,13 @@
       <c r="G2" s="155" t="s">
         <v>436</v>
       </c>
-      <c r="H2" s="250" t="s">
+      <c r="H2" s="245" t="s">
         <v>435</v>
       </c>
       <c r="I2" s="155" t="s">
         <v>152</v>
       </c>
-      <c r="J2" s="250" t="s">
+      <c r="J2" s="245" t="s">
         <v>434</v>
       </c>
     </row>
@@ -7034,11 +7154,11 @@
       <c r="G3" s="155" t="s">
         <v>414</v>
       </c>
-      <c r="H3" s="250"/>
+      <c r="H3" s="245"/>
       <c r="I3" s="155" t="s">
         <v>411</v>
       </c>
-      <c r="J3" s="250"/>
+      <c r="J3" s="245"/>
     </row>
     <row r="4" spans="1:10" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="177"/>
@@ -7060,11 +7180,11 @@
       <c r="G4" s="155" t="s">
         <v>363</v>
       </c>
-      <c r="H4" s="250"/>
+      <c r="H4" s="245"/>
       <c r="I4" s="155" t="s">
         <v>359</v>
       </c>
-      <c r="J4" s="250"/>
+      <c r="J4" s="245"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="171" t="s">
@@ -7363,9 +7483,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C2925AE-B1C3-2143-BED8-865F5DD872E0}">
   <sheetPr codeName="Feuil9">
-    <tabColor rgb="FFC00000"/>
+    <tabColor rgb="FFFE0000"/>
   </sheetPr>
-  <dimension ref="A1:BK23"/>
+  <dimension ref="A1:BK21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" style="108" hidden="1" customWidth="1"/>
@@ -7463,7 +7583,7 @@
       <c r="G2" s="155" t="s">
         <v>438</v>
       </c>
-      <c r="H2" s="250" t="s">
+      <c r="H2" s="245" t="s">
         <v>437</v>
       </c>
       <c r="I2" s="154" t="s">
@@ -7508,7 +7628,7 @@
       <c r="V2" s="154" t="s">
         <v>436</v>
       </c>
-      <c r="W2" s="250" t="s">
+      <c r="W2" s="245" t="s">
         <v>435</v>
       </c>
       <c r="X2" s="155" t="s">
@@ -7523,7 +7643,7 @@
       <c r="AA2" s="155" t="s">
         <v>152</v>
       </c>
-      <c r="AB2" s="250" t="s">
+      <c r="AB2" s="245" t="s">
         <v>434</v>
       </c>
       <c r="AC2" s="152" t="s">
@@ -7553,7 +7673,7 @@
       <c r="AK2" s="152" t="s">
         <v>433</v>
       </c>
-      <c r="AL2" s="250" t="s">
+      <c r="AL2" s="245" t="s">
         <v>432</v>
       </c>
       <c r="AM2" s="152" t="s">
@@ -7595,7 +7715,7 @@
       <c r="AY2" s="152" t="s">
         <v>431</v>
       </c>
-      <c r="AZ2" s="250" t="s">
+      <c r="AZ2" s="245" t="s">
         <v>430</v>
       </c>
       <c r="BA2" s="151" t="s">
@@ -7625,7 +7745,7 @@
       <c r="BI2" s="151" t="s">
         <v>429</v>
       </c>
-      <c r="BJ2" s="250" t="s">
+      <c r="BJ2" s="245" t="s">
         <v>428</v>
       </c>
       <c r="BK2"/>
@@ -7640,7 +7760,7 @@
       <c r="G3" s="155" t="s">
         <v>427</v>
       </c>
-      <c r="H3" s="250"/>
+      <c r="H3" s="245"/>
       <c r="I3" s="154" t="s">
         <v>426</v>
       </c>
@@ -7681,7 +7801,7 @@
       <c r="V3" s="154" t="s">
         <v>414</v>
       </c>
-      <c r="W3" s="250"/>
+      <c r="W3" s="245"/>
       <c r="X3" s="150"/>
       <c r="Y3" s="155" t="s">
         <v>413</v>
@@ -7692,7 +7812,7 @@
       <c r="AA3" s="155" t="s">
         <v>411</v>
       </c>
-      <c r="AB3" s="250"/>
+      <c r="AB3" s="245"/>
       <c r="AC3" s="152" t="s">
         <v>410</v>
       </c>
@@ -7720,7 +7840,7 @@
       <c r="AK3" s="152" t="s">
         <v>404</v>
       </c>
-      <c r="AL3" s="250"/>
+      <c r="AL3" s="245"/>
       <c r="AM3" s="152" t="s">
         <v>403</v>
       </c>
@@ -7760,7 +7880,7 @@
       <c r="AY3" s="152" t="s">
         <v>391</v>
       </c>
-      <c r="AZ3" s="250"/>
+      <c r="AZ3" s="245"/>
       <c r="BA3" s="151" t="s">
         <v>390</v>
       </c>
@@ -7788,7 +7908,7 @@
       <c r="BI3" s="151" t="s">
         <v>382</v>
       </c>
-      <c r="BJ3" s="250"/>
+      <c r="BJ3" s="245"/>
     </row>
     <row r="4" spans="1:63" s="112" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="157"/>
@@ -7810,7 +7930,7 @@
       <c r="G4" s="155" t="s">
         <v>377</v>
       </c>
-      <c r="H4" s="250"/>
+      <c r="H4" s="245"/>
       <c r="I4" s="154" t="s">
         <v>376</v>
       </c>
@@ -7853,7 +7973,7 @@
       <c r="V4" s="154" t="s">
         <v>363</v>
       </c>
-      <c r="W4" s="250"/>
+      <c r="W4" s="245"/>
       <c r="X4" s="153" t="s">
         <v>362</v>
       </c>
@@ -7866,7 +7986,7 @@
       <c r="AA4" s="153" t="s">
         <v>359</v>
       </c>
-      <c r="AB4" s="250"/>
+      <c r="AB4" s="245"/>
       <c r="AC4" s="152" t="s">
         <v>358</v>
       </c>
@@ -7894,7 +8014,7 @@
       <c r="AK4" s="152" t="s">
         <v>351</v>
       </c>
-      <c r="AL4" s="250"/>
+      <c r="AL4" s="245"/>
       <c r="AM4" s="152" t="s">
         <v>350</v>
       </c>
@@ -7934,7 +8054,7 @@
       <c r="AY4" s="152" t="s">
         <v>338</v>
       </c>
-      <c r="AZ4" s="250"/>
+      <c r="AZ4" s="245"/>
       <c r="BA4" s="151" t="s">
         <v>337</v>
       </c>
@@ -7962,7 +8082,7 @@
       <c r="BI4" s="151" t="s">
         <v>329</v>
       </c>
-      <c r="BJ4" s="250"/>
+      <c r="BJ4" s="245"/>
       <c r="BK4"/>
     </row>
     <row r="5" spans="1:63" s="112" customFormat="1" ht="15" x14ac:dyDescent="0.2">
@@ -7971,7 +8091,7 @@
       </c>
       <c r="B5" s="132"/>
       <c r="C5" s="132"/>
-      <c r="D5" s="212"/>
+      <c r="D5" s="211"/>
       <c r="E5" s="132" t="s">
         <v>328</v>
       </c>
@@ -8183,7 +8303,7 @@
       </c>
       <c r="B6" s="132"/>
       <c r="C6" s="132"/>
-      <c r="D6" s="213" t="str">
+      <c r="D6" s="212" t="str">
         <f t="shared" ref="D6:D15" si="6">IF(ISBLANK($D$5),"",$D$5)</f>
         <v/>
       </c>
@@ -8397,7 +8517,7 @@
       </c>
       <c r="B7" s="132"/>
       <c r="C7" s="132"/>
-      <c r="D7" s="213" t="str">
+      <c r="D7" s="212" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -8611,7 +8731,7 @@
       </c>
       <c r="B8" s="132"/>
       <c r="C8" s="132"/>
-      <c r="D8" s="213" t="str">
+      <c r="D8" s="212" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -8825,7 +8945,7 @@
       </c>
       <c r="B9" s="132"/>
       <c r="C9" s="132"/>
-      <c r="D9" s="213" t="str">
+      <c r="D9" s="212" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -9039,7 +9159,7 @@
       </c>
       <c r="B10" s="132"/>
       <c r="C10" s="132"/>
-      <c r="D10" s="213" t="str">
+      <c r="D10" s="212" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -9253,7 +9373,7 @@
       </c>
       <c r="B11" s="132"/>
       <c r="C11" s="132"/>
-      <c r="D11" s="213" t="str">
+      <c r="D11" s="212" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -9467,7 +9587,7 @@
       </c>
       <c r="B12" s="132"/>
       <c r="C12" s="132"/>
-      <c r="D12" s="213" t="str">
+      <c r="D12" s="212" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -9681,7 +9801,7 @@
       </c>
       <c r="B13" s="132"/>
       <c r="C13" s="132"/>
-      <c r="D13" s="213" t="str">
+      <c r="D13" s="212" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -9895,7 +10015,7 @@
       </c>
       <c r="B14" s="132"/>
       <c r="C14" s="132"/>
-      <c r="D14" s="213" t="str">
+      <c r="D14" s="212" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -10109,7 +10229,7 @@
       </c>
       <c r="B15" s="132"/>
       <c r="C15" s="132"/>
-      <c r="D15" s="213" t="str">
+      <c r="D15" s="212" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
@@ -10551,97 +10671,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:62" s="112" customFormat="1" ht="9" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="116"/>
-      <c r="B17" s="115"/>
-      <c r="C17" s="115"/>
-      <c r="D17" s="115"/>
-      <c r="E17" s="115"/>
-      <c r="F17" s="114"/>
-      <c r="G17" s="113"/>
-      <c r="H17" s="113"/>
-      <c r="I17" s="113"/>
-      <c r="J17" s="113"/>
-      <c r="K17" s="113"/>
-      <c r="L17" s="113"/>
-      <c r="M17" s="113"/>
-      <c r="N17" s="113"/>
-      <c r="O17" s="113"/>
-      <c r="P17" s="113"/>
-      <c r="Q17" s="113"/>
-      <c r="R17" s="113"/>
-      <c r="S17" s="113"/>
-      <c r="T17" s="113"/>
-      <c r="U17" s="113"/>
-      <c r="V17" s="113"/>
-      <c r="W17" s="113"/>
-      <c r="X17" s="113"/>
-      <c r="Y17" s="113"/>
-      <c r="Z17" s="113"/>
-      <c r="AA17" s="113"/>
-      <c r="AB17" s="113"/>
-      <c r="AC17" s="113"/>
-      <c r="AD17" s="113"/>
-      <c r="AE17" s="113"/>
-      <c r="AF17" s="113"/>
-      <c r="AG17" s="113"/>
-      <c r="AH17" s="113"/>
-      <c r="AI17" s="113"/>
-      <c r="AJ17" s="113"/>
-      <c r="AK17" s="113"/>
-      <c r="AL17" s="113"/>
-      <c r="AM17" s="113"/>
-      <c r="AN17" s="113"/>
-      <c r="AO17" s="113"/>
-      <c r="AP17" s="113"/>
-      <c r="AQ17" s="113"/>
-      <c r="AR17" s="113"/>
-      <c r="AS17" s="113"/>
-      <c r="AT17" s="113"/>
-      <c r="AU17" s="113"/>
-      <c r="AV17" s="113"/>
-      <c r="AW17" s="113"/>
-      <c r="AX17" s="113"/>
-      <c r="AY17" s="113"/>
-      <c r="AZ17" s="113"/>
-      <c r="BA17" s="113"/>
-      <c r="BB17" s="113"/>
-      <c r="BC17" s="113"/>
-      <c r="BD17" s="113"/>
-      <c r="BE17" s="113"/>
-      <c r="BF17" s="113"/>
-      <c r="BG17" s="113"/>
-      <c r="BH17" s="113"/>
-      <c r="BI17" s="113"/>
-      <c r="BJ17" s="113"/>
-    </row>
-    <row r="18" spans="1:62" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="W18" s="111"/>
-      <c r="AZ18" s="111"/>
-    </row>
-    <row r="19" spans="1:62" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E19" s="253" t="s">
+    <row r="17" spans="4:52" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="W17" s="111"/>
+      <c r="AZ17" s="111"/>
+    </row>
+    <row r="18" spans="4:52" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="D18" s="258" t="s">
         <v>440</v>
       </c>
-      <c r="F19" s="254"/>
-      <c r="G19" s="254"/>
-      <c r="H19" s="254"/>
-      <c r="I19" s="254"/>
-      <c r="J19" s="254"/>
-      <c r="K19" s="254"/>
-      <c r="L19" s="254"/>
-      <c r="M19" s="255"/>
-    </row>
-    <row r="20" spans="1:62" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="22" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="AH22" s="109"/>
-    </row>
-    <row r="23" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="E23" s="110"/>
+      <c r="E18" s="260"/>
+      <c r="F18" s="260"/>
+      <c r="G18" s="260"/>
+      <c r="H18" s="260"/>
+      <c r="I18" s="261"/>
+    </row>
+    <row r="19" spans="4:52" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="20" spans="4:52" x14ac:dyDescent="0.2">
+      <c r="AH20" s="109"/>
+    </row>
+    <row r="21" spans="4:52" x14ac:dyDescent="0.2">
+      <c r="E21" s="110"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="E19:M19"/>
+  <mergeCells count="6">
     <mergeCell ref="BJ2:BJ4"/>
     <mergeCell ref="H2:H4"/>
     <mergeCell ref="W2:W4"/>
@@ -10657,9 +10709,9 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B695F461-4586-D34F-8E14-1071CB20CB72}">
   <sheetPr codeName="Feuil15">
-    <tabColor rgb="FFFFC000"/>
+    <tabColor rgb="FFF7EF2D"/>
   </sheetPr>
-  <dimension ref="A1:BJ23"/>
+  <dimension ref="A1:BJ21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="3" width="11" style="108" hidden="1" customWidth="1"/>
@@ -10746,7 +10798,7 @@
       <c r="G2" s="155" t="s">
         <v>438</v>
       </c>
-      <c r="H2" s="250" t="s">
+      <c r="H2" s="245" t="s">
         <v>437</v>
       </c>
       <c r="I2" s="155" t="s">
@@ -10779,13 +10831,13 @@
       <c r="R2" s="155" t="s">
         <v>436</v>
       </c>
-      <c r="S2" s="250" t="s">
+      <c r="S2" s="245" t="s">
         <v>435</v>
       </c>
       <c r="T2" s="155" t="s">
         <v>152</v>
       </c>
-      <c r="U2" s="250" t="s">
+      <c r="U2" s="245" t="s">
         <v>434</v>
       </c>
       <c r="V2" s="155" t="s">
@@ -10815,7 +10867,7 @@
       <c r="AD2" s="155" t="s">
         <v>433</v>
       </c>
-      <c r="AE2" s="250" t="s">
+      <c r="AE2" s="245" t="s">
         <v>482</v>
       </c>
       <c r="AF2" s="155" t="s">
@@ -10827,7 +10879,7 @@
       <c r="AH2" s="155" t="s">
         <v>481</v>
       </c>
-      <c r="AI2" s="250" t="s">
+      <c r="AI2" s="245" t="s">
         <v>480</v>
       </c>
     </row>
@@ -10841,7 +10893,7 @@
       <c r="G3" s="155" t="s">
         <v>427</v>
       </c>
-      <c r="H3" s="250"/>
+      <c r="H3" s="245"/>
       <c r="I3" s="155" t="s">
         <v>479</v>
       </c>
@@ -10872,11 +10924,11 @@
       <c r="R3" s="155" t="s">
         <v>414</v>
       </c>
-      <c r="S3" s="250"/>
+      <c r="S3" s="245"/>
       <c r="T3" s="155" t="s">
         <v>411</v>
       </c>
-      <c r="U3" s="250"/>
+      <c r="U3" s="245"/>
       <c r="V3" s="155" t="s">
         <v>470</v>
       </c>
@@ -10904,7 +10956,7 @@
       <c r="AD3" s="155" t="s">
         <v>462</v>
       </c>
-      <c r="AE3" s="250"/>
+      <c r="AE3" s="245"/>
       <c r="AF3" s="155" t="s">
         <v>461</v>
       </c>
@@ -10914,7 +10966,7 @@
       <c r="AH3" s="155" t="s">
         <v>391</v>
       </c>
-      <c r="AI3" s="250"/>
+      <c r="AI3" s="245"/>
     </row>
     <row r="4" spans="1:62" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="158"/>
@@ -10936,7 +10988,7 @@
       <c r="G4" s="155" t="s">
         <v>377</v>
       </c>
-      <c r="H4" s="250"/>
+      <c r="H4" s="245"/>
       <c r="I4" s="155" t="s">
         <v>460</v>
       </c>
@@ -10967,11 +11019,11 @@
       <c r="R4" s="155" t="s">
         <v>363</v>
       </c>
-      <c r="S4" s="250"/>
+      <c r="S4" s="245"/>
       <c r="T4" s="155" t="s">
         <v>359</v>
       </c>
-      <c r="U4" s="250"/>
+      <c r="U4" s="245"/>
       <c r="V4" s="155" t="s">
         <v>451</v>
       </c>
@@ -10999,7 +11051,7 @@
       <c r="AD4" s="155" t="s">
         <v>443</v>
       </c>
-      <c r="AE4" s="250"/>
+      <c r="AE4" s="245"/>
       <c r="AF4" s="155" t="s">
         <v>442</v>
       </c>
@@ -11009,7 +11061,7 @@
       <c r="AH4" s="155" t="s">
         <v>338</v>
       </c>
-      <c r="AI4" s="250"/>
+      <c r="AI4" s="245"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="161" t="s">
@@ -12597,45 +12649,46 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="5:19" x14ac:dyDescent="0.2">
+    <row r="17" spans="4:19" x14ac:dyDescent="0.2">
       <c r="S17" s="111"/>
     </row>
-    <row r="18" spans="5:19" ht="21" x14ac:dyDescent="0.25">
-      <c r="E18" s="256" t="s">
-        <v>517</v>
-      </c>
-      <c r="F18" s="257"/>
-      <c r="G18" s="257"/>
-      <c r="H18" s="257"/>
-      <c r="I18" s="257"/>
-      <c r="J18" s="257"/>
-      <c r="K18" s="257"/>
-      <c r="L18" s="257"/>
-      <c r="M18" s="257"/>
-    </row>
-    <row r="19" spans="5:19" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="5:19" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E20" s="253" t="s">
+    <row r="18" spans="4:19" x14ac:dyDescent="0.2">
+      <c r="D18" s="255" t="s">
+        <v>520</v>
+      </c>
+      <c r="E18" s="256"/>
+      <c r="F18"/>
+      <c r="G18"/>
+      <c r="H18"/>
+      <c r="I18"/>
+      <c r="J18"/>
+      <c r="K18"/>
+    </row>
+    <row r="19" spans="4:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="D19" s="257"/>
+      <c r="E19" s="256"/>
+      <c r="F19" s="256"/>
+      <c r="G19" s="256"/>
+      <c r="H19" s="256"/>
+      <c r="I19" s="256"/>
+      <c r="J19" s="256"/>
+      <c r="K19" s="256"/>
+    </row>
+    <row r="20" spans="4:19" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="D20" s="258" t="s">
         <v>440</v>
       </c>
-      <c r="F20" s="254"/>
-      <c r="G20" s="254"/>
-      <c r="H20" s="254"/>
-      <c r="I20" s="254"/>
-      <c r="J20" s="254"/>
-      <c r="K20" s="254"/>
-      <c r="L20" s="254"/>
-      <c r="M20" s="254"/>
-      <c r="N20" s="210"/>
-    </row>
-    <row r="21" spans="5:19" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="23" spans="5:19" x14ac:dyDescent="0.2">
-      <c r="F23" s="110"/>
-    </row>
+      <c r="E20" s="259"/>
+      <c r="F20" s="260"/>
+      <c r="G20" s="260"/>
+      <c r="H20" s="260"/>
+      <c r="I20" s="260"/>
+      <c r="J20" s="261"/>
+      <c r="K20" s="4"/>
+    </row>
+    <row r="21" spans="4:19" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="E18:M18"/>
-    <mergeCell ref="E20:M20"/>
+  <mergeCells count="5">
     <mergeCell ref="AI2:AI4"/>
     <mergeCell ref="H2:H4"/>
     <mergeCell ref="S2:S4"/>
@@ -12650,7 +12703,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70C2B6A9-5FC7-3A43-BF37-0B81E3F33F51}">
   <sheetPr codeName="Feuil16">
-    <tabColor rgb="FF92D050"/>
+    <tabColor rgb="FF01A94F"/>
   </sheetPr>
   <dimension ref="A1:BJ17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -12740,13 +12793,13 @@
       <c r="G2" s="155" t="s">
         <v>436</v>
       </c>
-      <c r="H2" s="250" t="s">
+      <c r="H2" s="245" t="s">
         <v>435</v>
       </c>
       <c r="I2" s="155" t="s">
         <v>152</v>
       </c>
-      <c r="J2" s="250" t="s">
+      <c r="J2" s="245" t="s">
         <v>434</v>
       </c>
     </row>
@@ -12760,11 +12813,11 @@
       <c r="G3" s="155" t="s">
         <v>414</v>
       </c>
-      <c r="H3" s="250"/>
+      <c r="H3" s="245"/>
       <c r="I3" s="155" t="s">
         <v>411</v>
       </c>
-      <c r="J3" s="250"/>
+      <c r="J3" s="245"/>
     </row>
     <row r="4" spans="1:62" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="177"/>
@@ -12786,11 +12839,11 @@
       <c r="G4" s="155" t="s">
         <v>363</v>
       </c>
-      <c r="H4" s="250"/>
+      <c r="H4" s="245"/>
       <c r="I4" s="155" t="s">
         <v>359</v>
       </c>
-      <c r="J4" s="250"/>
+      <c r="J4" s="245"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="171" t="s">
@@ -13113,29 +13166,29 @@
       </c>
     </row>
     <row r="16" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="E16" s="258" t="s">
-        <v>516</v>
-      </c>
-      <c r="F16" s="259"/>
-      <c r="G16" s="259"/>
-      <c r="H16" s="259"/>
-      <c r="I16" s="259"/>
-      <c r="J16" s="259"/>
+      <c r="D16" s="255" t="s">
+        <v>519</v>
+      </c>
+      <c r="E16" s="256"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="23"/>
     </row>
     <row r="17" spans="4:10" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D17" s="110"/>
-      <c r="E17" s="259"/>
-      <c r="F17" s="259"/>
-      <c r="G17" s="259"/>
-      <c r="H17" s="259"/>
-      <c r="I17" s="259"/>
-      <c r="J17" s="259"/>
+      <c r="D17" s="254"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="23"/>
+      <c r="I17" s="23"/>
+      <c r="J17" s="23"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="H2:H4"/>
     <mergeCell ref="J2:J4"/>
-    <mergeCell ref="E16:J17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13145,7 +13198,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3674A8A-13E9-4EDB-B294-D1FF8F18362C}">
   <sheetPr codeName="Feuil4">
-    <tabColor theme="0"/>
+    <tabColor rgb="FFCE4275"/>
   </sheetPr>
   <dimension ref="A1:DN8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -13464,7 +13517,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B89445B-6ECC-4440-B85C-E593AE209933}">
   <sheetPr codeName="Feuil13">
-    <tabColor theme="0"/>
+    <tabColor rgb="FF2C45E0"/>
   </sheetPr>
   <dimension ref="A1:EF4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -13498,14 +13551,14 @@
       <c r="H1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="EA1" s="244" t="s">
+      <c r="EA1" s="239" t="s">
         <v>492</v>
       </c>
-      <c r="EB1" s="244"/>
-      <c r="EC1" s="244"/>
-      <c r="ED1" s="244"/>
-      <c r="EE1" s="244"/>
-      <c r="EF1" s="244"/>
+      <c r="EB1" s="239"/>
+      <c r="EC1" s="239"/>
+      <c r="ED1" s="239"/>
+      <c r="EE1" s="239"/>
+      <c r="EF1" s="239"/>
     </row>
     <row r="2" spans="1:136" ht="66" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="24" t="s">
@@ -13561,7 +13614,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E893F90-1EC7-764C-B747-7920FCEC73CB}">
   <sheetPr codeName="Feuil18">
-    <tabColor theme="2" tint="-9.9978637043366805E-2"/>
+    <tabColor rgb="FF0B0B97"/>
   </sheetPr>
   <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -13582,7 +13635,7 @@
     <row r="1" spans="1:16" s="4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3"/>
       <c r="B1" s="5"/>
-      <c r="C1" s="211" t="s">
+      <c r="C1" s="210" t="s">
         <v>507</v>
       </c>
       <c r="D1" s="7"/>
@@ -13627,20 +13680,20 @@
     </row>
     <row r="4" spans="1:16" ht="40" x14ac:dyDescent="0.2">
       <c r="C4" s="9"/>
-      <c r="E4" s="245" t="s">
+      <c r="E4" s="240" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="246"/>
-      <c r="G4" s="246"/>
-      <c r="H4" s="246"/>
-      <c r="I4" s="247"/>
-      <c r="J4" s="245" t="s">
+      <c r="F4" s="241"/>
+      <c r="G4" s="241"/>
+      <c r="H4" s="241"/>
+      <c r="I4" s="242"/>
+      <c r="J4" s="240" t="s">
         <v>28</v>
       </c>
-      <c r="K4" s="246"/>
-      <c r="L4" s="246"/>
-      <c r="M4" s="246"/>
-      <c r="N4" s="247"/>
+      <c r="K4" s="241"/>
+      <c r="L4" s="241"/>
+      <c r="M4" s="241"/>
+      <c r="N4" s="242"/>
       <c r="O4" s="30" t="s">
         <v>29</v>
       </c>
@@ -15239,16 +15292,16 @@
   <sheetData>
     <row r="1" spans="1:62" s="64" customFormat="1" ht="12" x14ac:dyDescent="0.15">
       <c r="A1" s="107"/>
-      <c r="B1" s="249" t="s">
+      <c r="B1" s="244" t="s">
         <v>439</v>
       </c>
-      <c r="C1" s="249"/>
-      <c r="D1" s="249"/>
-      <c r="E1" s="249"/>
-      <c r="F1" s="249"/>
-      <c r="G1" s="249"/>
-      <c r="H1" s="249"/>
-      <c r="I1" s="249"/>
+      <c r="C1" s="244"/>
+      <c r="D1" s="244"/>
+      <c r="E1" s="244"/>
+      <c r="F1" s="244"/>
+      <c r="G1" s="244"/>
+      <c r="H1" s="244"/>
+      <c r="I1" s="244"/>
       <c r="AC1" s="106"/>
       <c r="AD1" s="106"/>
       <c r="AE1" s="106"/>
@@ -15269,7 +15322,7 @@
       <c r="G2" s="102" t="s">
         <v>438</v>
       </c>
-      <c r="H2" s="248" t="s">
+      <c r="H2" s="243" t="s">
         <v>437</v>
       </c>
       <c r="I2" s="101" t="s">
@@ -15314,7 +15367,7 @@
       <c r="V2" s="101" t="s">
         <v>436</v>
       </c>
-      <c r="W2" s="248" t="s">
+      <c r="W2" s="243" t="s">
         <v>435</v>
       </c>
       <c r="X2" s="102" t="s">
@@ -15329,7 +15382,7 @@
       <c r="AA2" s="102" t="s">
         <v>152</v>
       </c>
-      <c r="AB2" s="248" t="s">
+      <c r="AB2" s="243" t="s">
         <v>434</v>
       </c>
       <c r="AC2" s="98" t="s">
@@ -15359,7 +15412,7 @@
       <c r="AK2" s="98" t="s">
         <v>433</v>
       </c>
-      <c r="AL2" s="248" t="s">
+      <c r="AL2" s="243" t="s">
         <v>432</v>
       </c>
       <c r="AM2" s="98" t="s">
@@ -15401,7 +15454,7 @@
       <c r="AY2" s="98" t="s">
         <v>431</v>
       </c>
-      <c r="AZ2" s="248" t="s">
+      <c r="AZ2" s="243" t="s">
         <v>430</v>
       </c>
       <c r="BA2" s="97" t="s">
@@ -15431,7 +15484,7 @@
       <c r="BI2" s="97" t="s">
         <v>429</v>
       </c>
-      <c r="BJ2" s="248" t="s">
+      <c r="BJ2" s="243" t="s">
         <v>428</v>
       </c>
     </row>
@@ -15445,7 +15498,7 @@
       <c r="G3" s="102" t="s">
         <v>427</v>
       </c>
-      <c r="H3" s="248"/>
+      <c r="H3" s="243"/>
       <c r="I3" s="101" t="s">
         <v>426</v>
       </c>
@@ -15486,7 +15539,7 @@
       <c r="V3" s="101" t="s">
         <v>414</v>
       </c>
-      <c r="W3" s="248"/>
+      <c r="W3" s="243"/>
       <c r="X3" s="96"/>
       <c r="Y3" s="102" t="s">
         <v>413</v>
@@ -15497,7 +15550,7 @@
       <c r="AA3" s="102" t="s">
         <v>411</v>
       </c>
-      <c r="AB3" s="248"/>
+      <c r="AB3" s="243"/>
       <c r="AC3" s="98" t="s">
         <v>410</v>
       </c>
@@ -15525,7 +15578,7 @@
       <c r="AK3" s="98" t="s">
         <v>404</v>
       </c>
-      <c r="AL3" s="248"/>
+      <c r="AL3" s="243"/>
       <c r="AM3" s="98" t="s">
         <v>403</v>
       </c>
@@ -15565,7 +15618,7 @@
       <c r="AY3" s="98" t="s">
         <v>391</v>
       </c>
-      <c r="AZ3" s="248"/>
+      <c r="AZ3" s="243"/>
       <c r="BA3" s="97" t="s">
         <v>390</v>
       </c>
@@ -15593,7 +15646,7 @@
       <c r="BI3" s="97" t="s">
         <v>382</v>
       </c>
-      <c r="BJ3" s="248"/>
+      <c r="BJ3" s="243"/>
     </row>
     <row r="4" spans="1:62" s="64" customFormat="1" ht="60" x14ac:dyDescent="0.15">
       <c r="A4" s="104"/>
@@ -15615,7 +15668,7 @@
       <c r="G4" s="102" t="s">
         <v>377</v>
       </c>
-      <c r="H4" s="248"/>
+      <c r="H4" s="243"/>
       <c r="I4" s="101" t="s">
         <v>376</v>
       </c>
@@ -15658,7 +15711,7 @@
       <c r="V4" s="100" t="s">
         <v>363</v>
       </c>
-      <c r="W4" s="248"/>
+      <c r="W4" s="243"/>
       <c r="X4" s="99" t="s">
         <v>362</v>
       </c>
@@ -15671,7 +15724,7 @@
       <c r="AA4" s="99" t="s">
         <v>359</v>
       </c>
-      <c r="AB4" s="248"/>
+      <c r="AB4" s="243"/>
       <c r="AC4" s="98" t="s">
         <v>358</v>
       </c>
@@ -15699,7 +15752,7 @@
       <c r="AK4" s="98" t="s">
         <v>351</v>
       </c>
-      <c r="AL4" s="248"/>
+      <c r="AL4" s="243"/>
       <c r="AM4" s="98" t="s">
         <v>350</v>
       </c>
@@ -15739,7 +15792,7 @@
       <c r="AY4" s="98" t="s">
         <v>338</v>
       </c>
-      <c r="AZ4" s="248"/>
+      <c r="AZ4" s="243"/>
       <c r="BA4" s="97" t="s">
         <v>337</v>
       </c>
@@ -15767,7 +15820,7 @@
       <c r="BI4" s="97" t="s">
         <v>329</v>
       </c>
-      <c r="BJ4" s="248"/>
+      <c r="BJ4" s="243"/>
     </row>
     <row r="5" spans="1:62" s="64" customFormat="1" ht="144" x14ac:dyDescent="0.15">
       <c r="A5" s="72" t="s">
@@ -17457,16 +17510,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:62" s="112" customFormat="1" ht="23.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B1" s="251" t="s">
+      <c r="B1" s="246" t="s">
         <v>439</v>
       </c>
-      <c r="C1" s="251"/>
-      <c r="D1" s="251"/>
-      <c r="E1" s="251"/>
-      <c r="F1" s="251"/>
-      <c r="G1" s="251"/>
-      <c r="H1" s="251"/>
-      <c r="I1" s="251"/>
+      <c r="C1" s="246"/>
+      <c r="D1" s="246"/>
+      <c r="E1" s="246"/>
+      <c r="F1" s="246"/>
+      <c r="G1" s="246"/>
+      <c r="H1" s="246"/>
+      <c r="I1" s="246"/>
     </row>
     <row r="2" spans="1:62" s="112" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="158"/>
@@ -17478,7 +17531,7 @@
       <c r="G2" s="155" t="s">
         <v>438</v>
       </c>
-      <c r="H2" s="250" t="s">
+      <c r="H2" s="245" t="s">
         <v>437</v>
       </c>
       <c r="I2" s="154" t="s">
@@ -17523,7 +17576,7 @@
       <c r="V2" s="154" t="s">
         <v>436</v>
       </c>
-      <c r="W2" s="250" t="s">
+      <c r="W2" s="245" t="s">
         <v>435</v>
       </c>
       <c r="X2" s="155" t="s">
@@ -17538,7 +17591,7 @@
       <c r="AA2" s="155" t="s">
         <v>152</v>
       </c>
-      <c r="AB2" s="250" t="s">
+      <c r="AB2" s="245" t="s">
         <v>434</v>
       </c>
       <c r="AC2" s="152" t="s">
@@ -17568,7 +17621,7 @@
       <c r="AK2" s="152" t="s">
         <v>433</v>
       </c>
-      <c r="AL2" s="250" t="s">
+      <c r="AL2" s="245" t="s">
         <v>432</v>
       </c>
       <c r="AM2" s="152" t="s">
@@ -17610,7 +17663,7 @@
       <c r="AY2" s="152" t="s">
         <v>431</v>
       </c>
-      <c r="AZ2" s="250" t="s">
+      <c r="AZ2" s="245" t="s">
         <v>430</v>
       </c>
       <c r="BA2" s="151" t="s">
@@ -17640,7 +17693,7 @@
       <c r="BI2" s="151" t="s">
         <v>429</v>
       </c>
-      <c r="BJ2" s="250" t="s">
+      <c r="BJ2" s="245" t="s">
         <v>428</v>
       </c>
     </row>
@@ -17654,7 +17707,7 @@
       <c r="G3" s="155" t="s">
         <v>427</v>
       </c>
-      <c r="H3" s="250"/>
+      <c r="H3" s="245"/>
       <c r="I3" s="154" t="s">
         <v>426</v>
       </c>
@@ -17695,7 +17748,7 @@
       <c r="V3" s="154" t="s">
         <v>414</v>
       </c>
-      <c r="W3" s="250"/>
+      <c r="W3" s="245"/>
       <c r="X3" s="150"/>
       <c r="Y3" s="155" t="s">
         <v>413</v>
@@ -17706,7 +17759,7 @@
       <c r="AA3" s="155" t="s">
         <v>411</v>
       </c>
-      <c r="AB3" s="250"/>
+      <c r="AB3" s="245"/>
       <c r="AC3" s="152" t="s">
         <v>410</v>
       </c>
@@ -17734,7 +17787,7 @@
       <c r="AK3" s="152" t="s">
         <v>404</v>
       </c>
-      <c r="AL3" s="250"/>
+      <c r="AL3" s="245"/>
       <c r="AM3" s="152" t="s">
         <v>403</v>
       </c>
@@ -17774,7 +17827,7 @@
       <c r="AY3" s="152" t="s">
         <v>391</v>
       </c>
-      <c r="AZ3" s="250"/>
+      <c r="AZ3" s="245"/>
       <c r="BA3" s="151" t="s">
         <v>390</v>
       </c>
@@ -17802,7 +17855,7 @@
       <c r="BI3" s="151" t="s">
         <v>382</v>
       </c>
-      <c r="BJ3" s="250"/>
+      <c r="BJ3" s="245"/>
     </row>
     <row r="4" spans="1:62" s="112" customFormat="1" ht="60" x14ac:dyDescent="0.15">
       <c r="A4" s="157"/>
@@ -17824,7 +17877,7 @@
       <c r="G4" s="155" t="s">
         <v>377</v>
       </c>
-      <c r="H4" s="250"/>
+      <c r="H4" s="245"/>
       <c r="I4" s="154" t="s">
         <v>376</v>
       </c>
@@ -17867,7 +17920,7 @@
       <c r="V4" s="154" t="s">
         <v>363</v>
       </c>
-      <c r="W4" s="250"/>
+      <c r="W4" s="245"/>
       <c r="X4" s="153" t="s">
         <v>362</v>
       </c>
@@ -17880,7 +17933,7 @@
       <c r="AA4" s="153" t="s">
         <v>359</v>
       </c>
-      <c r="AB4" s="250"/>
+      <c r="AB4" s="245"/>
       <c r="AC4" s="152" t="s">
         <v>358</v>
       </c>
@@ -17908,7 +17961,7 @@
       <c r="AK4" s="152" t="s">
         <v>351</v>
       </c>
-      <c r="AL4" s="250"/>
+      <c r="AL4" s="245"/>
       <c r="AM4" s="152" t="s">
         <v>350</v>
       </c>
@@ -17948,7 +18001,7 @@
       <c r="AY4" s="152" t="s">
         <v>338</v>
       </c>
-      <c r="AZ4" s="250"/>
+      <c r="AZ4" s="245"/>
       <c r="BA4" s="151" t="s">
         <v>337</v>
       </c>
@@ -17976,7 +18029,7 @@
       <c r="BI4" s="151" t="s">
         <v>329</v>
       </c>
-      <c r="BJ4" s="250"/>
+      <c r="BJ4" s="245"/>
     </row>
     <row r="5" spans="1:62" s="112" customFormat="1" ht="11" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="122" t="s">

</xml_diff>

<commit_message>
add JA VIF extractor
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10114"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A96EFCC9-952B-9C47-8418-74278CEBA416}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{747CEEAA-2D6B-7D4C-8FEC-C5ACAC0255E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="22940" windowHeight="13240" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -31,7 +31,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ETPT A-JUST'!$A$2:$DN$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ETPT Format DDG'!$A$2:$DT$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Table_Fonctions!$A$1:$F$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Table_Fonctions!$A$1:$F$66</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1623" uniqueCount="520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1629" uniqueCount="521">
   <si>
     <t>#! END_ROW</t>
   </si>
@@ -2771,6 +2771,9 @@
   </si>
   <si>
     <t>JA JP</t>
+  </si>
+  <si>
+    <t>JA VIF</t>
   </si>
 </sst>
 </file>
@@ -13924,7 +13927,7 @@
   <sheetPr codeName="Feuil14">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.83203125" style="41" bestFit="1" customWidth="1"/>
@@ -15191,7 +15194,7 @@
         <v>143</v>
       </c>
       <c r="C63" s="48" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="D63" s="48" t="s">
         <v>137</v>
@@ -15202,51 +15205,72 @@
       <c r="F63" s="48" t="s">
         <v>132</v>
       </c>
+      <c r="G63" s="42"/>
     </row>
     <row r="64" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="47" t="s">
+      <c r="A64" s="49" t="s">
         <v>140</v>
       </c>
-      <c r="B64" s="42" t="s">
+      <c r="B64" s="48" t="s">
+        <v>143</v>
+      </c>
+      <c r="C64" s="48" t="s">
+        <v>519</v>
+      </c>
+      <c r="D64" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="E64" s="48" t="s">
+        <v>109</v>
+      </c>
+      <c r="F64" s="48" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="47" t="s">
+        <v>140</v>
+      </c>
+      <c r="B65" s="42" t="s">
         <v>142</v>
       </c>
-      <c r="C64" s="42" t="s">
+      <c r="C65" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="D64" s="42" t="s">
+      <c r="D65" s="42" t="s">
         <v>137</v>
       </c>
-      <c r="E64" s="42" t="s">
+      <c r="E65" s="42" t="s">
         <v>109</v>
       </c>
-      <c r="F64" s="46"/>
-      <c r="G64" s="42" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="45" t="s">
-        <v>140</v>
-      </c>
-      <c r="B65" s="44" t="s">
-        <v>139</v>
-      </c>
-      <c r="C65" s="44" t="s">
-        <v>138</v>
-      </c>
-      <c r="D65" s="44" t="s">
-        <v>137</v>
-      </c>
-      <c r="E65" s="44" t="s">
-        <v>109</v>
-      </c>
-      <c r="F65" s="43"/>
+      <c r="F65" s="46"/>
       <c r="G65" s="42" t="s">
         <v>136</v>
       </c>
     </row>
+    <row r="66" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="45" t="s">
+        <v>140</v>
+      </c>
+      <c r="B66" s="44" t="s">
+        <v>139</v>
+      </c>
+      <c r="C66" s="44" t="s">
+        <v>138</v>
+      </c>
+      <c r="D66" s="44" t="s">
+        <v>137</v>
+      </c>
+      <c r="E66" s="44" t="s">
+        <v>109</v>
+      </c>
+      <c r="F66" s="43"/>
+      <c r="G66" s="42" t="s">
+        <v>136</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F65" xr:uid="{00000000-0001-0000-0300-000000000000}"/>
+  <autoFilter ref="A1:F66" xr:uid="{00000000-0001-0000-0300-000000000000}"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="8" scale="74" orientation="landscape" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
DDG ajout cont a jp autour du juge
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7161F2AA-EFD1-F948-B7A2-01F41596DC86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31930DC9-534D-2849-8A1A-BC0A9312649C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="22940" windowHeight="13240" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -31,7 +31,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ETPT A-JUST'!$A$2:$DN$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ETPT Format DDG'!$A$2:$DT$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Table_Fonctions!$A$1:$F$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Table_Fonctions!$A$1:$F$67</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1629" uniqueCount="520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1635" uniqueCount="521">
   <si>
     <t>#! END_ROW</t>
   </si>
@@ -2771,6 +2771,9 @@
   </si>
   <si>
     <t>CONT C JP Greffe</t>
+  </si>
+  <si>
+    <t>CONT A JP Autour du magistrat</t>
   </si>
 </sst>
 </file>
@@ -13924,7 +13927,7 @@
   <sheetPr codeName="Feuil14">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.83203125" style="41" bestFit="1" customWidth="1"/>
@@ -15225,49 +15228,69 @@
       </c>
     </row>
     <row r="65" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="47" t="s">
+      <c r="A65" s="49" t="s">
         <v>137</v>
       </c>
-      <c r="B65" s="42" t="s">
+      <c r="B65" s="48" t="s">
+        <v>140</v>
+      </c>
+      <c r="C65" s="48" t="s">
+        <v>520</v>
+      </c>
+      <c r="D65" s="48" t="s">
+        <v>134</v>
+      </c>
+      <c r="E65" s="48" t="s">
+        <v>109</v>
+      </c>
+      <c r="F65" s="48" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="47" t="s">
+        <v>137</v>
+      </c>
+      <c r="B66" s="42" t="s">
         <v>139</v>
       </c>
-      <c r="C65" s="42" t="s">
+      <c r="C66" s="42" t="s">
         <v>138</v>
       </c>
-      <c r="D65" s="42" t="s">
+      <c r="D66" s="42" t="s">
         <v>134</v>
       </c>
-      <c r="E65" s="42" t="s">
+      <c r="E66" s="42" t="s">
         <v>109</v>
       </c>
-      <c r="F65" s="46"/>
-      <c r="G65" s="42" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="45" t="s">
-        <v>137</v>
-      </c>
-      <c r="B66" s="44" t="s">
-        <v>136</v>
-      </c>
-      <c r="C66" s="44" t="s">
-        <v>135</v>
-      </c>
-      <c r="D66" s="44" t="s">
-        <v>134</v>
-      </c>
-      <c r="E66" s="44" t="s">
-        <v>109</v>
-      </c>
-      <c r="F66" s="43"/>
+      <c r="F66" s="46"/>
       <c r="G66" s="42" t="s">
         <v>133</v>
       </c>
     </row>
+    <row r="67" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A67" s="45" t="s">
+        <v>137</v>
+      </c>
+      <c r="B67" s="44" t="s">
+        <v>136</v>
+      </c>
+      <c r="C67" s="44" t="s">
+        <v>135</v>
+      </c>
+      <c r="D67" s="44" t="s">
+        <v>134</v>
+      </c>
+      <c r="E67" s="44" t="s">
+        <v>109</v>
+      </c>
+      <c r="F67" s="43"/>
+      <c r="G67" s="42" t="s">
+        <v>133</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F66" xr:uid="{00000000-0001-0000-0300-000000000000}"/>
+  <autoFilter ref="A1:F67" xr:uid="{00000000-0001-0000-0300-000000000000}"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="8" scale="74" orientation="landscape" r:id="rId1"/>
 </worksheet>
@@ -16813,7 +16836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:62" s="64" customFormat="1" ht="36" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:62" s="64" customFormat="1" ht="48" x14ac:dyDescent="0.15">
       <c r="A13" s="72" t="s">
         <v>228</v>
       </c>

</xml_diff>

<commit_message>
DDG add cont a jp autour du magistrat
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10311"/>
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C175DC4F-D524-694E-A1E8-046EB5A40464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FFF230F-D554-BF4B-801A-5BCCA5A7E477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="22940" windowHeight="13240" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -31,7 +31,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ETPT A-JUST'!$A$2:$DN$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ETPT Format DDG'!$A$2:$DT$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Table_Fonctions!$A$1:$F$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Table_Fonctions!$A$1:$F$67</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1629" uniqueCount="522">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1635" uniqueCount="523">
   <si>
     <t>#! END_ROW</t>
   </si>
@@ -2777,6 +2777,9 @@
   </si>
   <si>
     <t>JA VIF</t>
+  </si>
+  <si>
+    <t>CONT A JP Autour du magistrat</t>
   </si>
 </sst>
 </file>
@@ -4592,6 +4595,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="40" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -4678,12 +4687,6 @@
     <xf numFmtId="0" fontId="31" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -5166,9 +5169,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office 2013 – 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -5206,7 +5209,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -5312,7 +5315,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -5454,7 +5457,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -5483,11 +5486,11 @@
       <c r="B1" s="197" t="s">
         <v>492</v>
       </c>
-      <c r="C1" s="233" t="s">
+      <c r="C1" s="235" t="s">
         <v>493</v>
       </c>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
+      <c r="D1" s="235"/>
+      <c r="E1" s="235"/>
       <c r="F1" s="198"/>
       <c r="H1" s="28" t="s">
         <v>0</v>
@@ -5496,11 +5499,11 @@
     <row r="2" spans="1:8" s="202" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="199"/>
       <c r="B2" s="200"/>
-      <c r="C2" s="234" t="s">
+      <c r="C2" s="236" t="s">
         <v>494</v>
       </c>
-      <c r="D2" s="234"/>
-      <c r="E2" s="234"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
       <c r="F2" s="201"/>
       <c r="H2" s="28" t="s">
         <v>0</v>
@@ -5524,10 +5527,10 @@
       <c r="D4" s="207" t="s">
         <v>497</v>
       </c>
-      <c r="E4" s="240" t="s">
+      <c r="E4" s="242" t="s">
         <v>498</v>
       </c>
-      <c r="F4" s="241"/>
+      <c r="F4" s="243"/>
       <c r="G4" s="216"/>
       <c r="H4" s="28" t="s">
         <v>0</v>
@@ -5544,10 +5547,10 @@
       <c r="D5" s="213" t="s">
         <v>501</v>
       </c>
-      <c r="E5" s="242" t="s">
+      <c r="E5" s="244" t="s">
         <v>514</v>
       </c>
-      <c r="F5" s="243"/>
+      <c r="F5" s="245"/>
       <c r="G5" s="215"/>
       <c r="H5" s="28" t="s">
         <v>0</v>
@@ -5564,10 +5567,10 @@
       <c r="D6" s="214" t="s">
         <v>504</v>
       </c>
-      <c r="E6" s="244" t="s">
+      <c r="E6" s="246" t="s">
         <v>515</v>
       </c>
-      <c r="F6" s="245"/>
+      <c r="F6" s="247"/>
       <c r="G6" s="215"/>
       <c r="H6" s="28" t="s">
         <v>0</v>
@@ -5584,10 +5587,10 @@
       <c r="D7" s="214" t="s">
         <v>507</v>
       </c>
-      <c r="E7" s="244" t="s">
+      <c r="E7" s="246" t="s">
         <v>514</v>
       </c>
-      <c r="F7" s="245"/>
+      <c r="F7" s="247"/>
       <c r="G7" s="215"/>
       <c r="H7" s="28" t="s">
         <v>0</v>
@@ -5598,16 +5601,16 @@
       <c r="B8" s="223" t="s">
         <v>508</v>
       </c>
-      <c r="C8" s="235" t="s">
+      <c r="C8" s="237" t="s">
         <v>509</v>
       </c>
-      <c r="D8" s="235" t="s">
+      <c r="D8" s="237" t="s">
         <v>510</v>
       </c>
-      <c r="E8" s="246" t="s">
+      <c r="E8" s="248" t="s">
         <v>516</v>
       </c>
-      <c r="F8" s="247"/>
+      <c r="F8" s="249"/>
       <c r="G8" s="215"/>
       <c r="H8" s="28" t="s">
         <v>0</v>
@@ -5618,10 +5621,10 @@
       <c r="B9" s="224" t="s">
         <v>511</v>
       </c>
-      <c r="C9" s="235"/>
-      <c r="D9" s="235"/>
-      <c r="E9" s="248"/>
-      <c r="F9" s="249"/>
+      <c r="C9" s="237"/>
+      <c r="D9" s="237"/>
+      <c r="E9" s="250"/>
+      <c r="F9" s="251"/>
       <c r="G9" s="215"/>
       <c r="H9" s="28" t="s">
         <v>0</v>
@@ -5632,10 +5635,10 @@
       <c r="B10" s="225" t="s">
         <v>512</v>
       </c>
-      <c r="C10" s="236"/>
-      <c r="D10" s="236"/>
-      <c r="E10" s="250"/>
-      <c r="F10" s="251"/>
+      <c r="C10" s="238"/>
+      <c r="D10" s="238"/>
+      <c r="E10" s="252"/>
+      <c r="F10" s="253"/>
       <c r="G10" s="215"/>
       <c r="H10" s="28" t="s">
         <v>0</v>
@@ -5655,11 +5658,11 @@
     <row r="12" spans="1:8" s="28" customFormat="1" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="203"/>
       <c r="B12" s="217"/>
-      <c r="C12" s="239" t="s">
+      <c r="C12" s="241" t="s">
         <v>513</v>
       </c>
-      <c r="D12" s="239"/>
-      <c r="E12" s="239"/>
+      <c r="D12" s="241"/>
+      <c r="E12" s="241"/>
       <c r="F12" s="218"/>
       <c r="H12" s="28" t="s">
         <v>0</v>
@@ -5673,14 +5676,14 @@
       </c>
     </row>
     <row r="14" spans="1:8" s="28" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="237" t="s">
+      <c r="A14" s="239" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="237"/>
-      <c r="C14" s="237"/>
-      <c r="D14" s="237"/>
-      <c r="E14" s="237"/>
-      <c r="F14" s="238"/>
+      <c r="B14" s="239"/>
+      <c r="C14" s="239"/>
+      <c r="D14" s="239"/>
+      <c r="E14" s="239"/>
+      <c r="F14" s="240"/>
       <c r="H14" s="28" t="s">
         <v>0</v>
       </c>
@@ -5725,16 +5728,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A1" s="260" t="s">
+      <c r="A1" s="262" t="s">
         <v>481</v>
       </c>
-      <c r="B1" s="260"/>
-      <c r="C1" s="260"/>
-      <c r="D1" s="260"/>
-      <c r="E1" s="260"/>
-      <c r="F1" s="260"/>
-      <c r="G1" s="260"/>
-      <c r="H1" s="260"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
+      <c r="H1" s="262"/>
       <c r="I1" s="112"/>
       <c r="J1" s="112"/>
       <c r="K1" s="112"/>
@@ -5773,7 +5776,7 @@
       <c r="G2" s="155" t="s">
         <v>436</v>
       </c>
-      <c r="H2" s="258" t="s">
+      <c r="H2" s="260" t="s">
         <v>435</v>
       </c>
       <c r="I2" s="155" t="s">
@@ -5806,13 +5809,13 @@
       <c r="R2" s="155" t="s">
         <v>434</v>
       </c>
-      <c r="S2" s="258" t="s">
+      <c r="S2" s="260" t="s">
         <v>433</v>
       </c>
       <c r="T2" s="155" t="s">
         <v>150</v>
       </c>
-      <c r="U2" s="258" t="s">
+      <c r="U2" s="260" t="s">
         <v>432</v>
       </c>
       <c r="V2" s="155" t="s">
@@ -5842,7 +5845,7 @@
       <c r="AD2" s="155" t="s">
         <v>431</v>
       </c>
-      <c r="AE2" s="258" t="s">
+      <c r="AE2" s="260" t="s">
         <v>480</v>
       </c>
       <c r="AF2" s="155" t="s">
@@ -5854,7 +5857,7 @@
       <c r="AH2" s="155" t="s">
         <v>479</v>
       </c>
-      <c r="AI2" s="258" t="s">
+      <c r="AI2" s="260" t="s">
         <v>478</v>
       </c>
     </row>
@@ -5868,7 +5871,7 @@
       <c r="G3" s="155" t="s">
         <v>425</v>
       </c>
-      <c r="H3" s="258"/>
+      <c r="H3" s="260"/>
       <c r="I3" s="155" t="s">
         <v>477</v>
       </c>
@@ -5899,11 +5902,11 @@
       <c r="R3" s="155" t="s">
         <v>412</v>
       </c>
-      <c r="S3" s="258"/>
+      <c r="S3" s="260"/>
       <c r="T3" s="155" t="s">
         <v>409</v>
       </c>
-      <c r="U3" s="258"/>
+      <c r="U3" s="260"/>
       <c r="V3" s="155" t="s">
         <v>468</v>
       </c>
@@ -5931,7 +5934,7 @@
       <c r="AD3" s="155" t="s">
         <v>460</v>
       </c>
-      <c r="AE3" s="258"/>
+      <c r="AE3" s="260"/>
       <c r="AF3" s="155" t="s">
         <v>459</v>
       </c>
@@ -5941,7 +5944,7 @@
       <c r="AH3" s="155" t="s">
         <v>389</v>
       </c>
-      <c r="AI3" s="258"/>
+      <c r="AI3" s="260"/>
     </row>
     <row r="4" spans="1:35" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="158"/>
@@ -5963,7 +5966,7 @@
       <c r="G4" s="155" t="s">
         <v>375</v>
       </c>
-      <c r="H4" s="258"/>
+      <c r="H4" s="260"/>
       <c r="I4" s="155" t="s">
         <v>458</v>
       </c>
@@ -5994,11 +5997,11 @@
       <c r="R4" s="155" t="s">
         <v>361</v>
       </c>
-      <c r="S4" s="258"/>
+      <c r="S4" s="260"/>
       <c r="T4" s="155" t="s">
         <v>357</v>
       </c>
-      <c r="U4" s="258"/>
+      <c r="U4" s="260"/>
       <c r="V4" s="155" t="s">
         <v>449</v>
       </c>
@@ -6026,7 +6029,7 @@
       <c r="AD4" s="155" t="s">
         <v>441</v>
       </c>
-      <c r="AE4" s="258"/>
+      <c r="AE4" s="260"/>
       <c r="AF4" s="155" t="s">
         <v>440</v>
       </c>
@@ -6036,7 +6039,7 @@
       <c r="AH4" s="155" t="s">
         <v>336</v>
       </c>
-      <c r="AI4" s="258"/>
+      <c r="AI4" s="260"/>
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A5" s="161" t="s">
@@ -7140,13 +7143,13 @@
       <c r="G2" s="155" t="s">
         <v>434</v>
       </c>
-      <c r="H2" s="258" t="s">
+      <c r="H2" s="260" t="s">
         <v>433</v>
       </c>
       <c r="I2" s="155" t="s">
         <v>150</v>
       </c>
-      <c r="J2" s="258" t="s">
+      <c r="J2" s="260" t="s">
         <v>432</v>
       </c>
     </row>
@@ -7160,11 +7163,11 @@
       <c r="G3" s="155" t="s">
         <v>412</v>
       </c>
-      <c r="H3" s="258"/>
+      <c r="H3" s="260"/>
       <c r="I3" s="155" t="s">
         <v>409</v>
       </c>
-      <c r="J3" s="258"/>
+      <c r="J3" s="260"/>
     </row>
     <row r="4" spans="1:10" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="177"/>
@@ -7186,11 +7189,11 @@
       <c r="G4" s="155" t="s">
         <v>361</v>
       </c>
-      <c r="H4" s="258"/>
+      <c r="H4" s="260"/>
       <c r="I4" s="155" t="s">
         <v>357</v>
       </c>
-      <c r="J4" s="258"/>
+      <c r="J4" s="260"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="171" t="s">
@@ -7589,7 +7592,7 @@
       <c r="G2" s="155" t="s">
         <v>436</v>
       </c>
-      <c r="H2" s="258" t="s">
+      <c r="H2" s="260" t="s">
         <v>435</v>
       </c>
       <c r="I2" s="154" t="s">
@@ -7634,7 +7637,7 @@
       <c r="V2" s="154" t="s">
         <v>434</v>
       </c>
-      <c r="W2" s="258" t="s">
+      <c r="W2" s="260" t="s">
         <v>433</v>
       </c>
       <c r="X2" s="155" t="s">
@@ -7649,7 +7652,7 @@
       <c r="AA2" s="155" t="s">
         <v>150</v>
       </c>
-      <c r="AB2" s="258" t="s">
+      <c r="AB2" s="260" t="s">
         <v>432</v>
       </c>
       <c r="AC2" s="152" t="s">
@@ -7679,7 +7682,7 @@
       <c r="AK2" s="152" t="s">
         <v>431</v>
       </c>
-      <c r="AL2" s="258" t="s">
+      <c r="AL2" s="260" t="s">
         <v>430</v>
       </c>
       <c r="AM2" s="152" t="s">
@@ -7721,7 +7724,7 @@
       <c r="AY2" s="152" t="s">
         <v>429</v>
       </c>
-      <c r="AZ2" s="258" t="s">
+      <c r="AZ2" s="260" t="s">
         <v>428</v>
       </c>
       <c r="BA2" s="151" t="s">
@@ -7751,7 +7754,7 @@
       <c r="BI2" s="151" t="s">
         <v>427</v>
       </c>
-      <c r="BJ2" s="258" t="s">
+      <c r="BJ2" s="260" t="s">
         <v>426</v>
       </c>
       <c r="BK2"/>
@@ -7766,7 +7769,7 @@
       <c r="G3" s="155" t="s">
         <v>425</v>
       </c>
-      <c r="H3" s="258"/>
+      <c r="H3" s="260"/>
       <c r="I3" s="154" t="s">
         <v>424</v>
       </c>
@@ -7807,7 +7810,7 @@
       <c r="V3" s="154" t="s">
         <v>412</v>
       </c>
-      <c r="W3" s="258"/>
+      <c r="W3" s="260"/>
       <c r="X3" s="150"/>
       <c r="Y3" s="155" t="s">
         <v>411</v>
@@ -7818,7 +7821,7 @@
       <c r="AA3" s="155" t="s">
         <v>409</v>
       </c>
-      <c r="AB3" s="258"/>
+      <c r="AB3" s="260"/>
       <c r="AC3" s="152" t="s">
         <v>408</v>
       </c>
@@ -7846,7 +7849,7 @@
       <c r="AK3" s="152" t="s">
         <v>402</v>
       </c>
-      <c r="AL3" s="258"/>
+      <c r="AL3" s="260"/>
       <c r="AM3" s="152" t="s">
         <v>401</v>
       </c>
@@ -7886,7 +7889,7 @@
       <c r="AY3" s="152" t="s">
         <v>389</v>
       </c>
-      <c r="AZ3" s="258"/>
+      <c r="AZ3" s="260"/>
       <c r="BA3" s="151" t="s">
         <v>388</v>
       </c>
@@ -7914,7 +7917,7 @@
       <c r="BI3" s="151" t="s">
         <v>380</v>
       </c>
-      <c r="BJ3" s="258"/>
+      <c r="BJ3" s="260"/>
     </row>
     <row r="4" spans="1:63" s="112" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="157"/>
@@ -7936,7 +7939,7 @@
       <c r="G4" s="155" t="s">
         <v>375</v>
       </c>
-      <c r="H4" s="258"/>
+      <c r="H4" s="260"/>
       <c r="I4" s="154" t="s">
         <v>374</v>
       </c>
@@ -7979,7 +7982,7 @@
       <c r="V4" s="154" t="s">
         <v>361</v>
       </c>
-      <c r="W4" s="258"/>
+      <c r="W4" s="260"/>
       <c r="X4" s="153" t="s">
         <v>360</v>
       </c>
@@ -7992,7 +7995,7 @@
       <c r="AA4" s="153" t="s">
         <v>357</v>
       </c>
-      <c r="AB4" s="258"/>
+      <c r="AB4" s="260"/>
       <c r="AC4" s="152" t="s">
         <v>356</v>
       </c>
@@ -8020,7 +8023,7 @@
       <c r="AK4" s="152" t="s">
         <v>349</v>
       </c>
-      <c r="AL4" s="258"/>
+      <c r="AL4" s="260"/>
       <c r="AM4" s="152" t="s">
         <v>348</v>
       </c>
@@ -8060,7 +8063,7 @@
       <c r="AY4" s="152" t="s">
         <v>336</v>
       </c>
-      <c r="AZ4" s="258"/>
+      <c r="AZ4" s="260"/>
       <c r="BA4" s="151" t="s">
         <v>335</v>
       </c>
@@ -8088,7 +8091,7 @@
       <c r="BI4" s="151" t="s">
         <v>327</v>
       </c>
-      <c r="BJ4" s="258"/>
+      <c r="BJ4" s="260"/>
       <c r="BK4"/>
     </row>
     <row r="5" spans="1:63" s="112" customFormat="1" ht="15" x14ac:dyDescent="0.2">
@@ -10804,7 +10807,7 @@
       <c r="G2" s="155" t="s">
         <v>436</v>
       </c>
-      <c r="H2" s="258" t="s">
+      <c r="H2" s="260" t="s">
         <v>435</v>
       </c>
       <c r="I2" s="155" t="s">
@@ -10837,13 +10840,13 @@
       <c r="R2" s="155" t="s">
         <v>434</v>
       </c>
-      <c r="S2" s="258" t="s">
+      <c r="S2" s="260" t="s">
         <v>433</v>
       </c>
       <c r="T2" s="155" t="s">
         <v>150</v>
       </c>
-      <c r="U2" s="258" t="s">
+      <c r="U2" s="260" t="s">
         <v>432</v>
       </c>
       <c r="V2" s="155" t="s">
@@ -10873,7 +10876,7 @@
       <c r="AD2" s="155" t="s">
         <v>431</v>
       </c>
-      <c r="AE2" s="258" t="s">
+      <c r="AE2" s="260" t="s">
         <v>480</v>
       </c>
       <c r="AF2" s="155" t="s">
@@ -10885,7 +10888,7 @@
       <c r="AH2" s="155" t="s">
         <v>479</v>
       </c>
-      <c r="AI2" s="258" t="s">
+      <c r="AI2" s="260" t="s">
         <v>478</v>
       </c>
     </row>
@@ -10899,7 +10902,7 @@
       <c r="G3" s="155" t="s">
         <v>425</v>
       </c>
-      <c r="H3" s="258"/>
+      <c r="H3" s="260"/>
       <c r="I3" s="155" t="s">
         <v>477</v>
       </c>
@@ -10930,11 +10933,11 @@
       <c r="R3" s="155" t="s">
         <v>412</v>
       </c>
-      <c r="S3" s="258"/>
+      <c r="S3" s="260"/>
       <c r="T3" s="155" t="s">
         <v>409</v>
       </c>
-      <c r="U3" s="258"/>
+      <c r="U3" s="260"/>
       <c r="V3" s="155" t="s">
         <v>468</v>
       </c>
@@ -10962,7 +10965,7 @@
       <c r="AD3" s="155" t="s">
         <v>460</v>
       </c>
-      <c r="AE3" s="258"/>
+      <c r="AE3" s="260"/>
       <c r="AF3" s="155" t="s">
         <v>459</v>
       </c>
@@ -10972,7 +10975,7 @@
       <c r="AH3" s="155" t="s">
         <v>389</v>
       </c>
-      <c r="AI3" s="258"/>
+      <c r="AI3" s="260"/>
     </row>
     <row r="4" spans="1:62" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="158"/>
@@ -10994,7 +10997,7 @@
       <c r="G4" s="155" t="s">
         <v>375</v>
       </c>
-      <c r="H4" s="258"/>
+      <c r="H4" s="260"/>
       <c r="I4" s="155" t="s">
         <v>458</v>
       </c>
@@ -11025,11 +11028,11 @@
       <c r="R4" s="155" t="s">
         <v>361</v>
       </c>
-      <c r="S4" s="258"/>
+      <c r="S4" s="260"/>
       <c r="T4" s="155" t="s">
         <v>357</v>
       </c>
-      <c r="U4" s="258"/>
+      <c r="U4" s="260"/>
       <c r="V4" s="155" t="s">
         <v>449</v>
       </c>
@@ -11057,7 +11060,7 @@
       <c r="AD4" s="155" t="s">
         <v>441</v>
       </c>
-      <c r="AE4" s="258"/>
+      <c r="AE4" s="260"/>
       <c r="AF4" s="155" t="s">
         <v>440</v>
       </c>
@@ -11067,7 +11070,7 @@
       <c r="AH4" s="155" t="s">
         <v>336</v>
       </c>
-      <c r="AI4" s="258"/>
+      <c r="AI4" s="260"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="161" t="s">
@@ -12799,13 +12802,13 @@
       <c r="G2" s="155" t="s">
         <v>434</v>
       </c>
-      <c r="H2" s="258" t="s">
+      <c r="H2" s="260" t="s">
         <v>433</v>
       </c>
       <c r="I2" s="155" t="s">
         <v>150</v>
       </c>
-      <c r="J2" s="258" t="s">
+      <c r="J2" s="260" t="s">
         <v>432</v>
       </c>
     </row>
@@ -12819,11 +12822,11 @@
       <c r="G3" s="155" t="s">
         <v>412</v>
       </c>
-      <c r="H3" s="258"/>
+      <c r="H3" s="260"/>
       <c r="I3" s="155" t="s">
         <v>409</v>
       </c>
-      <c r="J3" s="258"/>
+      <c r="J3" s="260"/>
     </row>
     <row r="4" spans="1:62" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="177"/>
@@ -12845,11 +12848,11 @@
       <c r="G4" s="155" t="s">
         <v>361</v>
       </c>
-      <c r="H4" s="258"/>
+      <c r="H4" s="260"/>
       <c r="I4" s="155" t="s">
         <v>357</v>
       </c>
-      <c r="J4" s="258"/>
+      <c r="J4" s="260"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="171" t="s">
@@ -13554,14 +13557,14 @@
       <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="EA1" s="252" t="s">
+      <c r="EA1" s="254" t="s">
         <v>490</v>
       </c>
-      <c r="EB1" s="252"/>
-      <c r="EC1" s="252"/>
-      <c r="ED1" s="252"/>
-      <c r="EE1" s="252"/>
-      <c r="EF1" s="252"/>
+      <c r="EB1" s="254"/>
+      <c r="EC1" s="254"/>
+      <c r="ED1" s="254"/>
+      <c r="EE1" s="254"/>
+      <c r="EF1" s="254"/>
       <c r="EG1" s="8" t="s">
         <v>0</v>
       </c>
@@ -13686,20 +13689,20 @@
     </row>
     <row r="4" spans="1:16" ht="40" x14ac:dyDescent="0.2">
       <c r="C4" s="9"/>
-      <c r="E4" s="253" t="s">
+      <c r="E4" s="255" t="s">
         <v>26</v>
       </c>
-      <c r="F4" s="254"/>
-      <c r="G4" s="254"/>
-      <c r="H4" s="254"/>
-      <c r="I4" s="255"/>
-      <c r="J4" s="253" t="s">
+      <c r="F4" s="256"/>
+      <c r="G4" s="256"/>
+      <c r="H4" s="256"/>
+      <c r="I4" s="257"/>
+      <c r="J4" s="255" t="s">
         <v>27</v>
       </c>
-      <c r="K4" s="254"/>
-      <c r="L4" s="254"/>
-      <c r="M4" s="254"/>
-      <c r="N4" s="255"/>
+      <c r="K4" s="256"/>
+      <c r="L4" s="256"/>
+      <c r="M4" s="256"/>
+      <c r="N4" s="257"/>
       <c r="O4" s="30" t="s">
         <v>28</v>
       </c>
@@ -13936,7 +13939,7 @@
   <sheetPr codeName="Feuil14">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.83203125" style="41" bestFit="1" customWidth="1"/>
@@ -15176,19 +15179,19 @@
       </c>
     </row>
     <row r="62" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="261" t="s">
+      <c r="A62" s="233" t="s">
         <v>140</v>
       </c>
-      <c r="B62" s="262" t="s">
+      <c r="B62" s="234" t="s">
         <v>520</v>
       </c>
-      <c r="C62" s="262" t="s">
+      <c r="C62" s="234" t="s">
         <v>521</v>
       </c>
-      <c r="D62" s="262" t="s">
+      <c r="D62" s="234" t="s">
         <v>137</v>
       </c>
-      <c r="E62" s="262" t="s">
+      <c r="E62" s="234" t="s">
         <v>109</v>
       </c>
       <c r="F62" s="48" t="s">
@@ -15237,49 +15240,69 @@
       </c>
     </row>
     <row r="65" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="47" t="s">
+      <c r="A65" s="49" t="s">
         <v>140</v>
       </c>
-      <c r="B65" s="42" t="s">
+      <c r="B65" s="48" t="s">
+        <v>143</v>
+      </c>
+      <c r="C65" s="48" t="s">
+        <v>522</v>
+      </c>
+      <c r="D65" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="E65" s="48" t="s">
+        <v>109</v>
+      </c>
+      <c r="F65" s="48" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="47" t="s">
+        <v>140</v>
+      </c>
+      <c r="B66" s="42" t="s">
         <v>142</v>
       </c>
-      <c r="C65" s="42" t="s">
+      <c r="C66" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="D65" s="42" t="s">
+      <c r="D66" s="42" t="s">
         <v>137</v>
       </c>
-      <c r="E65" s="42" t="s">
+      <c r="E66" s="42" t="s">
         <v>109</v>
       </c>
-      <c r="F65" s="46"/>
-      <c r="G65" s="42" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="45" t="s">
-        <v>140</v>
-      </c>
-      <c r="B66" s="44" t="s">
-        <v>139</v>
-      </c>
-      <c r="C66" s="44" t="s">
-        <v>138</v>
-      </c>
-      <c r="D66" s="44" t="s">
-        <v>137</v>
-      </c>
-      <c r="E66" s="44" t="s">
-        <v>109</v>
-      </c>
-      <c r="F66" s="43"/>
+      <c r="F66" s="46"/>
       <c r="G66" s="42" t="s">
         <v>136</v>
       </c>
     </row>
+    <row r="67" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A67" s="45" t="s">
+        <v>140</v>
+      </c>
+      <c r="B67" s="44" t="s">
+        <v>139</v>
+      </c>
+      <c r="C67" s="44" t="s">
+        <v>138</v>
+      </c>
+      <c r="D67" s="44" t="s">
+        <v>137</v>
+      </c>
+      <c r="E67" s="44" t="s">
+        <v>109</v>
+      </c>
+      <c r="F67" s="43"/>
+      <c r="G67" s="42" t="s">
+        <v>136</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F66" xr:uid="{00000000-0001-0000-0300-000000000000}"/>
+  <autoFilter ref="A1:F67" xr:uid="{00000000-0001-0000-0300-000000000000}"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="8" scale="74" orientation="landscape" r:id="rId1"/>
 </worksheet>
@@ -15319,16 +15342,16 @@
   <sheetData>
     <row r="1" spans="1:62" s="64" customFormat="1" ht="12" x14ac:dyDescent="0.15">
       <c r="A1" s="107"/>
-      <c r="B1" s="257" t="s">
+      <c r="B1" s="259" t="s">
         <v>437</v>
       </c>
-      <c r="C1" s="257"/>
-      <c r="D1" s="257"/>
-      <c r="E1" s="257"/>
-      <c r="F1" s="257"/>
-      <c r="G1" s="257"/>
-      <c r="H1" s="257"/>
-      <c r="I1" s="257"/>
+      <c r="C1" s="259"/>
+      <c r="D1" s="259"/>
+      <c r="E1" s="259"/>
+      <c r="F1" s="259"/>
+      <c r="G1" s="259"/>
+      <c r="H1" s="259"/>
+      <c r="I1" s="259"/>
       <c r="AC1" s="106"/>
       <c r="AD1" s="106"/>
       <c r="AE1" s="106"/>
@@ -15349,7 +15372,7 @@
       <c r="G2" s="102" t="s">
         <v>436</v>
       </c>
-      <c r="H2" s="256" t="s">
+      <c r="H2" s="258" t="s">
         <v>435</v>
       </c>
       <c r="I2" s="101" t="s">
@@ -15394,7 +15417,7 @@
       <c r="V2" s="101" t="s">
         <v>434</v>
       </c>
-      <c r="W2" s="256" t="s">
+      <c r="W2" s="258" t="s">
         <v>433</v>
       </c>
       <c r="X2" s="102" t="s">
@@ -15409,7 +15432,7 @@
       <c r="AA2" s="102" t="s">
         <v>150</v>
       </c>
-      <c r="AB2" s="256" t="s">
+      <c r="AB2" s="258" t="s">
         <v>432</v>
       </c>
       <c r="AC2" s="98" t="s">
@@ -15439,7 +15462,7 @@
       <c r="AK2" s="98" t="s">
         <v>431</v>
       </c>
-      <c r="AL2" s="256" t="s">
+      <c r="AL2" s="258" t="s">
         <v>430</v>
       </c>
       <c r="AM2" s="98" t="s">
@@ -15481,7 +15504,7 @@
       <c r="AY2" s="98" t="s">
         <v>429</v>
       </c>
-      <c r="AZ2" s="256" t="s">
+      <c r="AZ2" s="258" t="s">
         <v>428</v>
       </c>
       <c r="BA2" s="97" t="s">
@@ -15511,7 +15534,7 @@
       <c r="BI2" s="97" t="s">
         <v>427</v>
       </c>
-      <c r="BJ2" s="256" t="s">
+      <c r="BJ2" s="258" t="s">
         <v>426</v>
       </c>
     </row>
@@ -15525,7 +15548,7 @@
       <c r="G3" s="102" t="s">
         <v>425</v>
       </c>
-      <c r="H3" s="256"/>
+      <c r="H3" s="258"/>
       <c r="I3" s="101" t="s">
         <v>424</v>
       </c>
@@ -15566,7 +15589,7 @@
       <c r="V3" s="101" t="s">
         <v>412</v>
       </c>
-      <c r="W3" s="256"/>
+      <c r="W3" s="258"/>
       <c r="X3" s="96"/>
       <c r="Y3" s="102" t="s">
         <v>411</v>
@@ -15577,7 +15600,7 @@
       <c r="AA3" s="102" t="s">
         <v>409</v>
       </c>
-      <c r="AB3" s="256"/>
+      <c r="AB3" s="258"/>
       <c r="AC3" s="98" t="s">
         <v>408</v>
       </c>
@@ -15605,7 +15628,7 @@
       <c r="AK3" s="98" t="s">
         <v>402</v>
       </c>
-      <c r="AL3" s="256"/>
+      <c r="AL3" s="258"/>
       <c r="AM3" s="98" t="s">
         <v>401</v>
       </c>
@@ -15645,7 +15668,7 @@
       <c r="AY3" s="98" t="s">
         <v>389</v>
       </c>
-      <c r="AZ3" s="256"/>
+      <c r="AZ3" s="258"/>
       <c r="BA3" s="97" t="s">
         <v>388</v>
       </c>
@@ -15673,7 +15696,7 @@
       <c r="BI3" s="97" t="s">
         <v>380</v>
       </c>
-      <c r="BJ3" s="256"/>
+      <c r="BJ3" s="258"/>
     </row>
     <row r="4" spans="1:62" s="64" customFormat="1" ht="60" x14ac:dyDescent="0.15">
       <c r="A4" s="104"/>
@@ -15695,7 +15718,7 @@
       <c r="G4" s="102" t="s">
         <v>375</v>
       </c>
-      <c r="H4" s="256"/>
+      <c r="H4" s="258"/>
       <c r="I4" s="101" t="s">
         <v>374</v>
       </c>
@@ -15738,7 +15761,7 @@
       <c r="V4" s="100" t="s">
         <v>361</v>
       </c>
-      <c r="W4" s="256"/>
+      <c r="W4" s="258"/>
       <c r="X4" s="99" t="s">
         <v>360</v>
       </c>
@@ -15751,7 +15774,7 @@
       <c r="AA4" s="99" t="s">
         <v>357</v>
       </c>
-      <c r="AB4" s="256"/>
+      <c r="AB4" s="258"/>
       <c r="AC4" s="98" t="s">
         <v>356</v>
       </c>
@@ -15779,7 +15802,7 @@
       <c r="AK4" s="98" t="s">
         <v>349</v>
       </c>
-      <c r="AL4" s="256"/>
+      <c r="AL4" s="258"/>
       <c r="AM4" s="98" t="s">
         <v>348</v>
       </c>
@@ -15819,7 +15842,7 @@
       <c r="AY4" s="98" t="s">
         <v>336</v>
       </c>
-      <c r="AZ4" s="256"/>
+      <c r="AZ4" s="258"/>
       <c r="BA4" s="97" t="s">
         <v>335</v>
       </c>
@@ -15847,7 +15870,7 @@
       <c r="BI4" s="97" t="s">
         <v>327</v>
       </c>
-      <c r="BJ4" s="256"/>
+      <c r="BJ4" s="258"/>
     </row>
     <row r="5" spans="1:62" s="64" customFormat="1" ht="144" x14ac:dyDescent="0.15">
       <c r="A5" s="72" t="s">
@@ -16825,7 +16848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:62" s="64" customFormat="1" ht="48" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:62" s="64" customFormat="1" ht="36" x14ac:dyDescent="0.15">
       <c r="A13" s="72" t="s">
         <v>231</v>
       </c>
@@ -17537,16 +17560,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:62" s="112" customFormat="1" ht="23.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B1" s="259" t="s">
+      <c r="B1" s="261" t="s">
         <v>437</v>
       </c>
-      <c r="C1" s="259"/>
-      <c r="D1" s="259"/>
-      <c r="E1" s="259"/>
-      <c r="F1" s="259"/>
-      <c r="G1" s="259"/>
-      <c r="H1" s="259"/>
-      <c r="I1" s="259"/>
+      <c r="C1" s="261"/>
+      <c r="D1" s="261"/>
+      <c r="E1" s="261"/>
+      <c r="F1" s="261"/>
+      <c r="G1" s="261"/>
+      <c r="H1" s="261"/>
+      <c r="I1" s="261"/>
     </row>
     <row r="2" spans="1:62" s="112" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="158"/>
@@ -17558,7 +17581,7 @@
       <c r="G2" s="155" t="s">
         <v>436</v>
       </c>
-      <c r="H2" s="258" t="s">
+      <c r="H2" s="260" t="s">
         <v>435</v>
       </c>
       <c r="I2" s="154" t="s">
@@ -17603,7 +17626,7 @@
       <c r="V2" s="154" t="s">
         <v>434</v>
       </c>
-      <c r="W2" s="258" t="s">
+      <c r="W2" s="260" t="s">
         <v>433</v>
       </c>
       <c r="X2" s="155" t="s">
@@ -17618,7 +17641,7 @@
       <c r="AA2" s="155" t="s">
         <v>150</v>
       </c>
-      <c r="AB2" s="258" t="s">
+      <c r="AB2" s="260" t="s">
         <v>432</v>
       </c>
       <c r="AC2" s="152" t="s">
@@ -17648,7 +17671,7 @@
       <c r="AK2" s="152" t="s">
         <v>431</v>
       </c>
-      <c r="AL2" s="258" t="s">
+      <c r="AL2" s="260" t="s">
         <v>430</v>
       </c>
       <c r="AM2" s="152" t="s">
@@ -17690,7 +17713,7 @@
       <c r="AY2" s="152" t="s">
         <v>429</v>
       </c>
-      <c r="AZ2" s="258" t="s">
+      <c r="AZ2" s="260" t="s">
         <v>428</v>
       </c>
       <c r="BA2" s="151" t="s">
@@ -17720,7 +17743,7 @@
       <c r="BI2" s="151" t="s">
         <v>427</v>
       </c>
-      <c r="BJ2" s="258" t="s">
+      <c r="BJ2" s="260" t="s">
         <v>426</v>
       </c>
     </row>
@@ -17734,7 +17757,7 @@
       <c r="G3" s="155" t="s">
         <v>425</v>
       </c>
-      <c r="H3" s="258"/>
+      <c r="H3" s="260"/>
       <c r="I3" s="154" t="s">
         <v>424</v>
       </c>
@@ -17775,7 +17798,7 @@
       <c r="V3" s="154" t="s">
         <v>412</v>
       </c>
-      <c r="W3" s="258"/>
+      <c r="W3" s="260"/>
       <c r="X3" s="150"/>
       <c r="Y3" s="155" t="s">
         <v>411</v>
@@ -17786,7 +17809,7 @@
       <c r="AA3" s="155" t="s">
         <v>409</v>
       </c>
-      <c r="AB3" s="258"/>
+      <c r="AB3" s="260"/>
       <c r="AC3" s="152" t="s">
         <v>408</v>
       </c>
@@ -17814,7 +17837,7 @@
       <c r="AK3" s="152" t="s">
         <v>402</v>
       </c>
-      <c r="AL3" s="258"/>
+      <c r="AL3" s="260"/>
       <c r="AM3" s="152" t="s">
         <v>401</v>
       </c>
@@ -17854,7 +17877,7 @@
       <c r="AY3" s="152" t="s">
         <v>389</v>
       </c>
-      <c r="AZ3" s="258"/>
+      <c r="AZ3" s="260"/>
       <c r="BA3" s="151" t="s">
         <v>388</v>
       </c>
@@ -17882,7 +17905,7 @@
       <c r="BI3" s="151" t="s">
         <v>380</v>
       </c>
-      <c r="BJ3" s="258"/>
+      <c r="BJ3" s="260"/>
     </row>
     <row r="4" spans="1:62" s="112" customFormat="1" ht="60" x14ac:dyDescent="0.15">
       <c r="A4" s="157"/>
@@ -17904,7 +17927,7 @@
       <c r="G4" s="155" t="s">
         <v>375</v>
       </c>
-      <c r="H4" s="258"/>
+      <c r="H4" s="260"/>
       <c r="I4" s="154" t="s">
         <v>374</v>
       </c>
@@ -17947,7 +17970,7 @@
       <c r="V4" s="154" t="s">
         <v>361</v>
       </c>
-      <c r="W4" s="258"/>
+      <c r="W4" s="260"/>
       <c r="X4" s="153" t="s">
         <v>360</v>
       </c>
@@ -17960,7 +17983,7 @@
       <c r="AA4" s="153" t="s">
         <v>357</v>
       </c>
-      <c r="AB4" s="258"/>
+      <c r="AB4" s="260"/>
       <c r="AC4" s="152" t="s">
         <v>356</v>
       </c>
@@ -17988,7 +18011,7 @@
       <c r="AK4" s="152" t="s">
         <v>349</v>
       </c>
-      <c r="AL4" s="258"/>
+      <c r="AL4" s="260"/>
       <c r="AM4" s="152" t="s">
         <v>348</v>
       </c>
@@ -18028,7 +18051,7 @@
       <c r="AY4" s="152" t="s">
         <v>336</v>
       </c>
-      <c r="AZ4" s="258"/>
+      <c r="AZ4" s="260"/>
       <c r="BA4" s="151" t="s">
         <v>335</v>
       </c>
@@ -18056,7 +18079,7 @@
       <c r="BI4" s="151" t="s">
         <v>327</v>
       </c>
-      <c r="BJ4" s="258"/>
+      <c r="BJ4" s="260"/>
     </row>
     <row r="5" spans="1:62" s="112" customFormat="1" ht="11" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="122" t="s">

</xml_diff>

<commit_message>
update extractor and error etp simulator
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2236A0B-2A89-994D-BFA7-9C2642E3F64E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7C9A653-5F3B-1848-BAAE-D5C33538B0BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" activeTab="3" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -2795,13 +2795,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="_-* #,##0.000_-;\-* #,##0.000_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="167" formatCode="General;General;\-"/>
     <numFmt numFmtId="168" formatCode="0.###;0.###;\-"/>
     <numFmt numFmtId="169" formatCode="#,##0.00_ ;[Red]\-#,##0.00\ "/>
+    <numFmt numFmtId="170" formatCode="0.0%"/>
   </numFmts>
   <fonts count="53" x14ac:knownFonts="1">
     <font>
@@ -4579,6 +4580,22 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="52" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="52" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="40" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -4643,6 +4660,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="10" borderId="13" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4663,36 +4689,11 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="52" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="52" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="52" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="52" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="52" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="52" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -4703,67 +4704,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
     <cellStyle name="Normal 3" xfId="4" xr:uid="{6BD57324-3FD5-D341-A299-730D14794802}"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -5567,11 +5508,11 @@
       <c r="B1" s="192" t="s">
         <v>492</v>
       </c>
-      <c r="C1" s="230" t="s">
+      <c r="C1" s="236" t="s">
         <v>493</v>
       </c>
-      <c r="D1" s="230"/>
-      <c r="E1" s="230"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
       <c r="F1" s="193"/>
       <c r="H1" s="27" t="s">
         <v>0</v>
@@ -5580,11 +5521,11 @@
     <row r="2" spans="1:8" s="197" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="194"/>
       <c r="B2" s="195"/>
-      <c r="C2" s="231" t="s">
+      <c r="C2" s="237" t="s">
         <v>494</v>
       </c>
-      <c r="D2" s="231"/>
-      <c r="E2" s="231"/>
+      <c r="D2" s="237"/>
+      <c r="E2" s="237"/>
       <c r="F2" s="196"/>
       <c r="H2" s="27" t="s">
         <v>0</v>
@@ -5608,10 +5549,10 @@
       <c r="D4" s="202" t="s">
         <v>497</v>
       </c>
-      <c r="E4" s="237" t="s">
+      <c r="E4" s="243" t="s">
         <v>498</v>
       </c>
-      <c r="F4" s="238"/>
+      <c r="F4" s="244"/>
       <c r="G4" s="211"/>
       <c r="H4" s="27" t="s">
         <v>0</v>
@@ -5628,10 +5569,10 @@
       <c r="D5" s="208" t="s">
         <v>501</v>
       </c>
-      <c r="E5" s="239" t="s">
+      <c r="E5" s="245" t="s">
         <v>514</v>
       </c>
-      <c r="F5" s="240"/>
+      <c r="F5" s="246"/>
       <c r="G5" s="210"/>
       <c r="H5" s="27" t="s">
         <v>0</v>
@@ -5648,10 +5589,10 @@
       <c r="D6" s="209" t="s">
         <v>504</v>
       </c>
-      <c r="E6" s="241" t="s">
+      <c r="E6" s="247" t="s">
         <v>515</v>
       </c>
-      <c r="F6" s="242"/>
+      <c r="F6" s="248"/>
       <c r="G6" s="210"/>
       <c r="H6" s="27" t="s">
         <v>0</v>
@@ -5668,10 +5609,10 @@
       <c r="D7" s="209" t="s">
         <v>507</v>
       </c>
-      <c r="E7" s="241" t="s">
+      <c r="E7" s="247" t="s">
         <v>514</v>
       </c>
-      <c r="F7" s="242"/>
+      <c r="F7" s="248"/>
       <c r="G7" s="210"/>
       <c r="H7" s="27" t="s">
         <v>0</v>
@@ -5682,16 +5623,16 @@
       <c r="B8" s="218" t="s">
         <v>508</v>
       </c>
-      <c r="C8" s="232" t="s">
+      <c r="C8" s="238" t="s">
         <v>509</v>
       </c>
-      <c r="D8" s="232" t="s">
+      <c r="D8" s="238" t="s">
         <v>510</v>
       </c>
-      <c r="E8" s="243" t="s">
+      <c r="E8" s="249" t="s">
         <v>516</v>
       </c>
-      <c r="F8" s="244"/>
+      <c r="F8" s="250"/>
       <c r="G8" s="210"/>
       <c r="H8" s="27" t="s">
         <v>0</v>
@@ -5702,10 +5643,10 @@
       <c r="B9" s="219" t="s">
         <v>511</v>
       </c>
-      <c r="C9" s="232"/>
-      <c r="D9" s="232"/>
-      <c r="E9" s="245"/>
-      <c r="F9" s="246"/>
+      <c r="C9" s="238"/>
+      <c r="D9" s="238"/>
+      <c r="E9" s="251"/>
+      <c r="F9" s="252"/>
       <c r="G9" s="210"/>
       <c r="H9" s="27" t="s">
         <v>0</v>
@@ -5716,10 +5657,10 @@
       <c r="B10" s="220" t="s">
         <v>512</v>
       </c>
-      <c r="C10" s="233"/>
-      <c r="D10" s="233"/>
-      <c r="E10" s="247"/>
-      <c r="F10" s="248"/>
+      <c r="C10" s="239"/>
+      <c r="D10" s="239"/>
+      <c r="E10" s="253"/>
+      <c r="F10" s="254"/>
       <c r="G10" s="210"/>
       <c r="H10" s="27" t="s">
         <v>0</v>
@@ -5739,11 +5680,11 @@
     <row r="12" spans="1:8" s="27" customFormat="1" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="198"/>
       <c r="B12" s="212"/>
-      <c r="C12" s="236" t="s">
+      <c r="C12" s="242" t="s">
         <v>513</v>
       </c>
-      <c r="D12" s="236"/>
-      <c r="E12" s="236"/>
+      <c r="D12" s="242"/>
+      <c r="E12" s="242"/>
       <c r="F12" s="213"/>
       <c r="H12" s="27" t="s">
         <v>0</v>
@@ -5757,14 +5698,14 @@
       </c>
     </row>
     <row r="14" spans="1:8" s="27" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="234" t="s">
+      <c r="A14" s="240" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="234"/>
-      <c r="C14" s="234"/>
-      <c r="D14" s="234"/>
-      <c r="E14" s="234"/>
-      <c r="F14" s="235"/>
+      <c r="B14" s="240"/>
+      <c r="C14" s="240"/>
+      <c r="D14" s="240"/>
+      <c r="E14" s="240"/>
+      <c r="F14" s="241"/>
       <c r="H14" s="27" t="s">
         <v>0</v>
       </c>
@@ -5809,16 +5750,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A1" s="256" t="s">
+      <c r="A1" s="265" t="s">
         <v>481</v>
       </c>
-      <c r="B1" s="256"/>
-      <c r="C1" s="256"/>
-      <c r="D1" s="256"/>
-      <c r="E1" s="256"/>
-      <c r="F1" s="256"/>
-      <c r="G1" s="256"/>
-      <c r="H1" s="256"/>
+      <c r="B1" s="265"/>
+      <c r="C1" s="265"/>
+      <c r="D1" s="265"/>
+      <c r="E1" s="265"/>
+      <c r="F1" s="265"/>
+      <c r="G1" s="265"/>
+      <c r="H1" s="265"/>
       <c r="I1" s="107"/>
       <c r="J1" s="107"/>
       <c r="K1" s="107"/>
@@ -5857,7 +5798,7 @@
       <c r="G2" s="150" t="s">
         <v>436</v>
       </c>
-      <c r="H2" s="254" t="s">
+      <c r="H2" s="263" t="s">
         <v>435</v>
       </c>
       <c r="I2" s="150" t="s">
@@ -5890,13 +5831,13 @@
       <c r="R2" s="150" t="s">
         <v>434</v>
       </c>
-      <c r="S2" s="254" t="s">
+      <c r="S2" s="263" t="s">
         <v>433</v>
       </c>
       <c r="T2" s="150" t="s">
         <v>150</v>
       </c>
-      <c r="U2" s="254" t="s">
+      <c r="U2" s="263" t="s">
         <v>432</v>
       </c>
       <c r="V2" s="150" t="s">
@@ -5926,7 +5867,7 @@
       <c r="AD2" s="150" t="s">
         <v>431</v>
       </c>
-      <c r="AE2" s="254" t="s">
+      <c r="AE2" s="263" t="s">
         <v>480</v>
       </c>
       <c r="AF2" s="150" t="s">
@@ -5938,7 +5879,7 @@
       <c r="AH2" s="150" t="s">
         <v>479</v>
       </c>
-      <c r="AI2" s="254" t="s">
+      <c r="AI2" s="263" t="s">
         <v>478</v>
       </c>
     </row>
@@ -5952,7 +5893,7 @@
       <c r="G3" s="150" t="s">
         <v>425</v>
       </c>
-      <c r="H3" s="254"/>
+      <c r="H3" s="263"/>
       <c r="I3" s="150" t="s">
         <v>477</v>
       </c>
@@ -5983,11 +5924,11 @@
       <c r="R3" s="150" t="s">
         <v>412</v>
       </c>
-      <c r="S3" s="254"/>
+      <c r="S3" s="263"/>
       <c r="T3" s="150" t="s">
         <v>409</v>
       </c>
-      <c r="U3" s="254"/>
+      <c r="U3" s="263"/>
       <c r="V3" s="150" t="s">
         <v>468</v>
       </c>
@@ -6015,7 +5956,7 @@
       <c r="AD3" s="150" t="s">
         <v>460</v>
       </c>
-      <c r="AE3" s="254"/>
+      <c r="AE3" s="263"/>
       <c r="AF3" s="150" t="s">
         <v>459</v>
       </c>
@@ -6025,7 +5966,7 @@
       <c r="AH3" s="150" t="s">
         <v>389</v>
       </c>
-      <c r="AI3" s="254"/>
+      <c r="AI3" s="263"/>
     </row>
     <row r="4" spans="1:35" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="153"/>
@@ -6047,7 +5988,7 @@
       <c r="G4" s="150" t="s">
         <v>375</v>
       </c>
-      <c r="H4" s="254"/>
+      <c r="H4" s="263"/>
       <c r="I4" s="150" t="s">
         <v>458</v>
       </c>
@@ -6078,11 +6019,11 @@
       <c r="R4" s="150" t="s">
         <v>361</v>
       </c>
-      <c r="S4" s="254"/>
+      <c r="S4" s="263"/>
       <c r="T4" s="150" t="s">
         <v>357</v>
       </c>
-      <c r="U4" s="254"/>
+      <c r="U4" s="263"/>
       <c r="V4" s="150" t="s">
         <v>449</v>
       </c>
@@ -6110,7 +6051,7 @@
       <c r="AD4" s="150" t="s">
         <v>441</v>
       </c>
-      <c r="AE4" s="254"/>
+      <c r="AE4" s="263"/>
       <c r="AF4" s="150" t="s">
         <v>440</v>
       </c>
@@ -6120,7 +6061,7 @@
       <c r="AH4" s="150" t="s">
         <v>336</v>
       </c>
-      <c r="AI4" s="254"/>
+      <c r="AI4" s="263"/>
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A5" s="156" t="s">
@@ -7224,13 +7165,13 @@
       <c r="G2" s="150" t="s">
         <v>434</v>
       </c>
-      <c r="H2" s="254" t="s">
+      <c r="H2" s="263" t="s">
         <v>433</v>
       </c>
       <c r="I2" s="150" t="s">
         <v>150</v>
       </c>
-      <c r="J2" s="254" t="s">
+      <c r="J2" s="263" t="s">
         <v>432</v>
       </c>
     </row>
@@ -7244,11 +7185,11 @@
       <c r="G3" s="150" t="s">
         <v>412</v>
       </c>
-      <c r="H3" s="254"/>
+      <c r="H3" s="263"/>
       <c r="I3" s="150" t="s">
         <v>409</v>
       </c>
-      <c r="J3" s="254"/>
+      <c r="J3" s="263"/>
     </row>
     <row r="4" spans="1:10" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="172"/>
@@ -7270,11 +7211,11 @@
       <c r="G4" s="150" t="s">
         <v>361</v>
       </c>
-      <c r="H4" s="254"/>
+      <c r="H4" s="263"/>
       <c r="I4" s="150" t="s">
         <v>357</v>
       </c>
-      <c r="J4" s="254"/>
+      <c r="J4" s="263"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="166" t="s">
@@ -7673,7 +7614,7 @@
       <c r="G2" s="150" t="s">
         <v>436</v>
       </c>
-      <c r="H2" s="254" t="s">
+      <c r="H2" s="263" t="s">
         <v>435</v>
       </c>
       <c r="I2" s="149" t="s">
@@ -7718,7 +7659,7 @@
       <c r="V2" s="149" t="s">
         <v>434</v>
       </c>
-      <c r="W2" s="254" t="s">
+      <c r="W2" s="263" t="s">
         <v>433</v>
       </c>
       <c r="X2" s="150" t="s">
@@ -7733,7 +7674,7 @@
       <c r="AA2" s="150" t="s">
         <v>150</v>
       </c>
-      <c r="AB2" s="254" t="s">
+      <c r="AB2" s="263" t="s">
         <v>432</v>
       </c>
       <c r="AC2" s="147" t="s">
@@ -7763,7 +7704,7 @@
       <c r="AK2" s="147" t="s">
         <v>431</v>
       </c>
-      <c r="AL2" s="254" t="s">
+      <c r="AL2" s="263" t="s">
         <v>430</v>
       </c>
       <c r="AM2" s="147" t="s">
@@ -7805,7 +7746,7 @@
       <c r="AY2" s="147" t="s">
         <v>429</v>
       </c>
-      <c r="AZ2" s="254" t="s">
+      <c r="AZ2" s="263" t="s">
         <v>428</v>
       </c>
       <c r="BA2" s="146" t="s">
@@ -7835,7 +7776,7 @@
       <c r="BI2" s="146" t="s">
         <v>427</v>
       </c>
-      <c r="BJ2" s="254" t="s">
+      <c r="BJ2" s="263" t="s">
         <v>426</v>
       </c>
       <c r="BK2"/>
@@ -7850,7 +7791,7 @@
       <c r="G3" s="150" t="s">
         <v>425</v>
       </c>
-      <c r="H3" s="254"/>
+      <c r="H3" s="263"/>
       <c r="I3" s="149" t="s">
         <v>424</v>
       </c>
@@ -7891,7 +7832,7 @@
       <c r="V3" s="149" t="s">
         <v>412</v>
       </c>
-      <c r="W3" s="254"/>
+      <c r="W3" s="263"/>
       <c r="X3" s="145"/>
       <c r="Y3" s="150" t="s">
         <v>411</v>
@@ -7902,7 +7843,7 @@
       <c r="AA3" s="150" t="s">
         <v>409</v>
       </c>
-      <c r="AB3" s="254"/>
+      <c r="AB3" s="263"/>
       <c r="AC3" s="147" t="s">
         <v>408</v>
       </c>
@@ -7930,7 +7871,7 @@
       <c r="AK3" s="147" t="s">
         <v>402</v>
       </c>
-      <c r="AL3" s="254"/>
+      <c r="AL3" s="263"/>
       <c r="AM3" s="147" t="s">
         <v>401</v>
       </c>
@@ -7970,7 +7911,7 @@
       <c r="AY3" s="147" t="s">
         <v>389</v>
       </c>
-      <c r="AZ3" s="254"/>
+      <c r="AZ3" s="263"/>
       <c r="BA3" s="146" t="s">
         <v>388</v>
       </c>
@@ -7998,7 +7939,7 @@
       <c r="BI3" s="146" t="s">
         <v>380</v>
       </c>
-      <c r="BJ3" s="254"/>
+      <c r="BJ3" s="263"/>
     </row>
     <row r="4" spans="1:63" s="107" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="152"/>
@@ -8020,7 +7961,7 @@
       <c r="G4" s="150" t="s">
         <v>375</v>
       </c>
-      <c r="H4" s="254"/>
+      <c r="H4" s="263"/>
       <c r="I4" s="149" t="s">
         <v>374</v>
       </c>
@@ -8063,7 +8004,7 @@
       <c r="V4" s="149" t="s">
         <v>361</v>
       </c>
-      <c r="W4" s="254"/>
+      <c r="W4" s="263"/>
       <c r="X4" s="148" t="s">
         <v>360</v>
       </c>
@@ -8076,7 +8017,7 @@
       <c r="AA4" s="148" t="s">
         <v>357</v>
       </c>
-      <c r="AB4" s="254"/>
+      <c r="AB4" s="263"/>
       <c r="AC4" s="147" t="s">
         <v>356</v>
       </c>
@@ -8104,7 +8045,7 @@
       <c r="AK4" s="147" t="s">
         <v>349</v>
       </c>
-      <c r="AL4" s="254"/>
+      <c r="AL4" s="263"/>
       <c r="AM4" s="147" t="s">
         <v>348</v>
       </c>
@@ -8144,7 +8085,7 @@
       <c r="AY4" s="147" t="s">
         <v>336</v>
       </c>
-      <c r="AZ4" s="254"/>
+      <c r="AZ4" s="263"/>
       <c r="BA4" s="146" t="s">
         <v>335</v>
       </c>
@@ -8172,7 +8113,7 @@
       <c r="BI4" s="146" t="s">
         <v>327</v>
       </c>
-      <c r="BJ4" s="254"/>
+      <c r="BJ4" s="263"/>
       <c r="BK4"/>
     </row>
     <row r="5" spans="1:63" s="107" customFormat="1" ht="15" x14ac:dyDescent="0.2">
@@ -10888,7 +10829,7 @@
       <c r="G2" s="150" t="s">
         <v>436</v>
       </c>
-      <c r="H2" s="254" t="s">
+      <c r="H2" s="263" t="s">
         <v>435</v>
       </c>
       <c r="I2" s="150" t="s">
@@ -10921,13 +10862,13 @@
       <c r="R2" s="150" t="s">
         <v>434</v>
       </c>
-      <c r="S2" s="254" t="s">
+      <c r="S2" s="263" t="s">
         <v>433</v>
       </c>
       <c r="T2" s="150" t="s">
         <v>150</v>
       </c>
-      <c r="U2" s="254" t="s">
+      <c r="U2" s="263" t="s">
         <v>432</v>
       </c>
       <c r="V2" s="150" t="s">
@@ -10957,7 +10898,7 @@
       <c r="AD2" s="150" t="s">
         <v>431</v>
       </c>
-      <c r="AE2" s="254" t="s">
+      <c r="AE2" s="263" t="s">
         <v>480</v>
       </c>
       <c r="AF2" s="150" t="s">
@@ -10969,7 +10910,7 @@
       <c r="AH2" s="150" t="s">
         <v>479</v>
       </c>
-      <c r="AI2" s="254" t="s">
+      <c r="AI2" s="263" t="s">
         <v>478</v>
       </c>
     </row>
@@ -10983,7 +10924,7 @@
       <c r="G3" s="150" t="s">
         <v>425</v>
       </c>
-      <c r="H3" s="254"/>
+      <c r="H3" s="263"/>
       <c r="I3" s="150" t="s">
         <v>477</v>
       </c>
@@ -11014,11 +10955,11 @@
       <c r="R3" s="150" t="s">
         <v>412</v>
       </c>
-      <c r="S3" s="254"/>
+      <c r="S3" s="263"/>
       <c r="T3" s="150" t="s">
         <v>409</v>
       </c>
-      <c r="U3" s="254"/>
+      <c r="U3" s="263"/>
       <c r="V3" s="150" t="s">
         <v>468</v>
       </c>
@@ -11046,7 +10987,7 @@
       <c r="AD3" s="150" t="s">
         <v>460</v>
       </c>
-      <c r="AE3" s="254"/>
+      <c r="AE3" s="263"/>
       <c r="AF3" s="150" t="s">
         <v>459</v>
       </c>
@@ -11056,7 +10997,7 @@
       <c r="AH3" s="150" t="s">
         <v>389</v>
       </c>
-      <c r="AI3" s="254"/>
+      <c r="AI3" s="263"/>
     </row>
     <row r="4" spans="1:62" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="153"/>
@@ -11078,7 +11019,7 @@
       <c r="G4" s="150" t="s">
         <v>375</v>
       </c>
-      <c r="H4" s="254"/>
+      <c r="H4" s="263"/>
       <c r="I4" s="150" t="s">
         <v>458</v>
       </c>
@@ -11109,11 +11050,11 @@
       <c r="R4" s="150" t="s">
         <v>361</v>
       </c>
-      <c r="S4" s="254"/>
+      <c r="S4" s="263"/>
       <c r="T4" s="150" t="s">
         <v>357</v>
       </c>
-      <c r="U4" s="254"/>
+      <c r="U4" s="263"/>
       <c r="V4" s="150" t="s">
         <v>449</v>
       </c>
@@ -11141,7 +11082,7 @@
       <c r="AD4" s="150" t="s">
         <v>441</v>
       </c>
-      <c r="AE4" s="254"/>
+      <c r="AE4" s="263"/>
       <c r="AF4" s="150" t="s">
         <v>440</v>
       </c>
@@ -11151,7 +11092,7 @@
       <c r="AH4" s="150" t="s">
         <v>336</v>
       </c>
-      <c r="AI4" s="254"/>
+      <c r="AI4" s="263"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="156" t="s">
@@ -12883,13 +12824,13 @@
       <c r="G2" s="150" t="s">
         <v>434</v>
       </c>
-      <c r="H2" s="254" t="s">
+      <c r="H2" s="263" t="s">
         <v>433</v>
       </c>
       <c r="I2" s="150" t="s">
         <v>150</v>
       </c>
-      <c r="J2" s="254" t="s">
+      <c r="J2" s="263" t="s">
         <v>432</v>
       </c>
     </row>
@@ -12903,11 +12844,11 @@
       <c r="G3" s="150" t="s">
         <v>412</v>
       </c>
-      <c r="H3" s="254"/>
+      <c r="H3" s="263"/>
       <c r="I3" s="150" t="s">
         <v>409</v>
       </c>
-      <c r="J3" s="254"/>
+      <c r="J3" s="263"/>
     </row>
     <row r="4" spans="1:62" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="172"/>
@@ -12929,11 +12870,11 @@
       <c r="G4" s="150" t="s">
         <v>361</v>
       </c>
-      <c r="H4" s="254"/>
+      <c r="H4" s="263"/>
       <c r="I4" s="150" t="s">
         <v>357</v>
       </c>
-      <c r="J4" s="254"/>
+      <c r="J4" s="263"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="166" t="s">
@@ -13638,14 +13579,14 @@
       <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="EA1" s="249" t="s">
+      <c r="EA1" s="255" t="s">
         <v>490</v>
       </c>
-      <c r="EB1" s="249"/>
-      <c r="EC1" s="249"/>
-      <c r="ED1" s="249"/>
-      <c r="EE1" s="249"/>
-      <c r="EF1" s="249"/>
+      <c r="EB1" s="255"/>
+      <c r="EC1" s="255"/>
+      <c r="ED1" s="255"/>
+      <c r="EE1" s="255"/>
+      <c r="EF1" s="255"/>
       <c r="EG1" s="8" t="s">
         <v>0</v>
       </c>
@@ -13782,30 +13723,30 @@
     </row>
     <row r="4" spans="1:24" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D4" s="9"/>
-      <c r="E4" s="264"/>
-      <c r="G4" s="250" t="s">
+      <c r="E4" s="234"/>
+      <c r="G4" s="256" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="251"/>
-      <c r="I4" s="251"/>
-      <c r="J4" s="251"/>
-      <c r="K4" s="251"/>
-      <c r="L4" s="251"/>
-      <c r="M4" s="260"/>
-      <c r="N4" s="250" t="s">
+      <c r="H4" s="257"/>
+      <c r="I4" s="257"/>
+      <c r="J4" s="257"/>
+      <c r="K4" s="257"/>
+      <c r="L4" s="257"/>
+      <c r="M4" s="258"/>
+      <c r="N4" s="256" t="s">
         <v>27</v>
       </c>
-      <c r="O4" s="251"/>
-      <c r="P4" s="251"/>
-      <c r="Q4" s="251"/>
-      <c r="R4" s="251"/>
-      <c r="S4" s="261"/>
-      <c r="T4" s="260"/>
-      <c r="U4" s="250" t="s">
+      <c r="O4" s="257"/>
+      <c r="P4" s="257"/>
+      <c r="Q4" s="257"/>
+      <c r="R4" s="257"/>
+      <c r="S4" s="260"/>
+      <c r="T4" s="258"/>
+      <c r="U4" s="256" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="258"/>
-      <c r="W4" s="267"/>
+      <c r="V4" s="259"/>
+      <c r="W4" s="235"/>
       <c r="X4" t="s">
         <v>0</v>
       </c>
@@ -13818,7 +13759,7 @@
       <c r="G5" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="262" t="s">
+      <c r="H5" s="232" t="s">
         <v>525</v>
       </c>
       <c r="I5" s="13" t="s">
@@ -13830,16 +13771,16 @@
       <c r="K5" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="L5" s="259" t="s">
+      <c r="L5" s="231" t="s">
         <v>30</v>
       </c>
-      <c r="M5" s="263" t="s">
+      <c r="M5" s="233" t="s">
         <v>525</v>
       </c>
       <c r="N5" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="O5" s="262" t="s">
+      <c r="O5" s="232" t="s">
         <v>525</v>
       </c>
       <c r="P5" s="13" t="s">
@@ -13851,16 +13792,16 @@
       <c r="R5" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="S5" s="259" t="s">
+      <c r="S5" s="231" t="s">
         <v>31</v>
       </c>
-      <c r="T5" s="263" t="s">
+      <c r="T5" s="233" t="s">
         <v>525</v>
       </c>
       <c r="U5" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="V5" s="263" t="s">
+      <c r="V5" s="233" t="s">
         <v>525</v>
       </c>
       <c r="W5" t="s">
@@ -13917,7 +13858,7 @@
 'ETPT Format DDG'!$G:$G,"Magistrat")</f>
         <v>#N/A</v>
       </c>
-      <c r="M6" s="265" t="str">
+      <c r="M6" s="267" t="str">
         <f>IF(OR(LEFT(C6,3)="12.",LEFT(E6,3)="12.",LEFT(E6,5)="CET &gt;", IFERROR(L6/$L$6,"")=0),"", IFERROR(L6/$L$6,""))</f>
         <v/>
       </c>
@@ -13951,7 +13892,7 @@
 'ETPT Format DDG'!$G:$G,"Greffe")</f>
         <v>#N/A</v>
       </c>
-      <c r="T6" s="265" t="str">
+      <c r="T6" s="267" t="str">
         <f>IF(OR(LEFT(C6,3)="12.",LEFT(E6,3)="12.",LEFT(E6,5)="CET &gt;",IFERROR(S6/$S$6,"")=0),"", IFERROR(S6/$S$6,""))</f>
         <v/>
       </c>
@@ -13965,7 +13906,7 @@
 'ETPT Format DDG'!$G:$G,"Autour du magistrat")</f>
         <v>#N/A</v>
       </c>
-      <c r="V6" s="265" t="str">
+      <c r="V6" s="267" t="str">
         <f>IF(OR(LEFT(C6,3)="12.",LEFT(E6,3)="12.",LEFT(E6,5)="CET &gt;",IFERROR(U6/$U$6,"")=0),"", IFERROR(U6/$U$6,""))</f>
         <v/>
       </c>
@@ -13974,589 +13915,589 @@
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="I7" s="257"/>
+      <c r="I7" s="230"/>
       <c r="W7" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="I8" s="257"/>
+      <c r="I8" s="230"/>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="I9" s="257"/>
+      <c r="I9" s="230"/>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="I10" s="257"/>
+      <c r="I10" s="230"/>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="I11" s="257"/>
+      <c r="I11" s="230"/>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="I12" s="257"/>
+      <c r="I12" s="230"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="I13" s="257"/>
+      <c r="I13" s="230"/>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="I14" s="257"/>
+      <c r="I14" s="230"/>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="I15" s="257"/>
+      <c r="I15" s="230"/>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="I16" s="257"/>
+      <c r="I16" s="230"/>
     </row>
     <row r="17" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I17" s="257"/>
+      <c r="I17" s="230"/>
     </row>
     <row r="18" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I18" s="257"/>
+      <c r="I18" s="230"/>
     </row>
     <row r="19" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I19" s="257"/>
+      <c r="I19" s="230"/>
     </row>
     <row r="20" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I20" s="257"/>
+      <c r="I20" s="230"/>
     </row>
     <row r="21" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I21" s="257"/>
+      <c r="I21" s="230"/>
     </row>
     <row r="22" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I22" s="257"/>
+      <c r="I22" s="230"/>
     </row>
     <row r="23" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I23" s="257"/>
+      <c r="I23" s="230"/>
     </row>
     <row r="24" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I24" s="257"/>
+      <c r="I24" s="230"/>
     </row>
     <row r="25" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I25" s="257"/>
+      <c r="I25" s="230"/>
     </row>
     <row r="26" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I26" s="257"/>
+      <c r="I26" s="230"/>
     </row>
     <row r="27" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I27" s="257"/>
+      <c r="I27" s="230"/>
     </row>
     <row r="28" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I28" s="257"/>
+      <c r="I28" s="230"/>
     </row>
     <row r="29" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I29" s="257"/>
+      <c r="I29" s="230"/>
     </row>
     <row r="30" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I30" s="257"/>
+      <c r="I30" s="230"/>
     </row>
     <row r="31" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I31" s="257"/>
+      <c r="I31" s="230"/>
     </row>
     <row r="32" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I32" s="257"/>
+      <c r="I32" s="230"/>
     </row>
     <row r="33" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I33" s="257"/>
+      <c r="I33" s="230"/>
     </row>
     <row r="34" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I34" s="257"/>
+      <c r="I34" s="230"/>
     </row>
     <row r="35" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I35" s="257"/>
+      <c r="I35" s="230"/>
     </row>
     <row r="36" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I36" s="257"/>
+      <c r="I36" s="230"/>
     </row>
     <row r="37" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I37" s="257"/>
+      <c r="I37" s="230"/>
     </row>
     <row r="38" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I38" s="257"/>
+      <c r="I38" s="230"/>
     </row>
     <row r="39" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I39" s="257"/>
+      <c r="I39" s="230"/>
     </row>
     <row r="40" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I40" s="257"/>
+      <c r="I40" s="230"/>
     </row>
     <row r="41" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I41" s="257"/>
+      <c r="I41" s="230"/>
     </row>
     <row r="42" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I42" s="257"/>
+      <c r="I42" s="230"/>
     </row>
     <row r="43" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I43" s="257"/>
+      <c r="I43" s="230"/>
     </row>
     <row r="44" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I44" s="257"/>
+      <c r="I44" s="230"/>
     </row>
     <row r="45" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I45" s="257"/>
+      <c r="I45" s="230"/>
     </row>
     <row r="46" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I46" s="257"/>
+      <c r="I46" s="230"/>
     </row>
     <row r="47" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I47" s="257"/>
+      <c r="I47" s="230"/>
     </row>
     <row r="48" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I48" s="257"/>
+      <c r="I48" s="230"/>
     </row>
     <row r="49" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I49" s="257"/>
+      <c r="I49" s="230"/>
     </row>
     <row r="50" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I50" s="257"/>
+      <c r="I50" s="230"/>
     </row>
     <row r="51" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I51" s="257"/>
+      <c r="I51" s="230"/>
     </row>
     <row r="52" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I52" s="257"/>
+      <c r="I52" s="230"/>
     </row>
     <row r="53" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I53" s="257"/>
+      <c r="I53" s="230"/>
     </row>
     <row r="54" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I54" s="257"/>
+      <c r="I54" s="230"/>
     </row>
     <row r="55" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I55" s="257"/>
+      <c r="I55" s="230"/>
     </row>
     <row r="56" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I56" s="257"/>
+      <c r="I56" s="230"/>
     </row>
     <row r="57" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I57" s="257"/>
+      <c r="I57" s="230"/>
     </row>
     <row r="58" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I58" s="257"/>
+      <c r="I58" s="230"/>
     </row>
     <row r="59" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I59" s="257"/>
+      <c r="I59" s="230"/>
     </row>
     <row r="60" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I60" s="257"/>
+      <c r="I60" s="230"/>
     </row>
     <row r="61" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I61" s="257"/>
+      <c r="I61" s="230"/>
     </row>
     <row r="62" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I62" s="257"/>
+      <c r="I62" s="230"/>
     </row>
     <row r="63" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I63" s="257"/>
+      <c r="I63" s="230"/>
     </row>
     <row r="64" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I64" s="257"/>
+      <c r="I64" s="230"/>
     </row>
     <row r="65" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I65" s="257"/>
+      <c r="I65" s="230"/>
     </row>
     <row r="66" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I66" s="257"/>
+      <c r="I66" s="230"/>
     </row>
     <row r="67" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I67" s="257"/>
+      <c r="I67" s="230"/>
     </row>
     <row r="68" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I68" s="257"/>
+      <c r="I68" s="230"/>
     </row>
     <row r="69" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I69" s="257"/>
+      <c r="I69" s="230"/>
     </row>
     <row r="70" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I70" s="257"/>
+      <c r="I70" s="230"/>
     </row>
     <row r="71" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I71" s="257"/>
+      <c r="I71" s="230"/>
     </row>
     <row r="72" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I72" s="257"/>
+      <c r="I72" s="230"/>
     </row>
     <row r="73" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I73" s="257"/>
+      <c r="I73" s="230"/>
     </row>
     <row r="74" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I74" s="257"/>
+      <c r="I74" s="230"/>
     </row>
     <row r="75" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I75" s="257"/>
+      <c r="I75" s="230"/>
     </row>
     <row r="76" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I76" s="257"/>
+      <c r="I76" s="230"/>
     </row>
     <row r="77" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I77" s="257"/>
+      <c r="I77" s="230"/>
     </row>
     <row r="78" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I78" s="257"/>
+      <c r="I78" s="230"/>
     </row>
     <row r="79" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I79" s="257"/>
+      <c r="I79" s="230"/>
     </row>
     <row r="80" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I80" s="257"/>
+      <c r="I80" s="230"/>
     </row>
     <row r="81" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I81" s="257"/>
+      <c r="I81" s="230"/>
     </row>
     <row r="82" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I82" s="257"/>
+      <c r="I82" s="230"/>
     </row>
     <row r="83" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I83" s="257"/>
+      <c r="I83" s="230"/>
     </row>
     <row r="84" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I84" s="257"/>
+      <c r="I84" s="230"/>
     </row>
     <row r="85" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I85" s="257"/>
+      <c r="I85" s="230"/>
     </row>
     <row r="86" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I86" s="257"/>
+      <c r="I86" s="230"/>
     </row>
     <row r="87" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I87" s="257"/>
+      <c r="I87" s="230"/>
     </row>
     <row r="88" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I88" s="257"/>
+      <c r="I88" s="230"/>
     </row>
     <row r="89" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I89" s="257"/>
+      <c r="I89" s="230"/>
     </row>
     <row r="90" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I90" s="257"/>
+      <c r="I90" s="230"/>
     </row>
     <row r="91" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I91" s="257"/>
+      <c r="I91" s="230"/>
     </row>
     <row r="92" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I92" s="257"/>
+      <c r="I92" s="230"/>
     </row>
     <row r="93" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I93" s="257"/>
+      <c r="I93" s="230"/>
     </row>
     <row r="94" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I94" s="257"/>
+      <c r="I94" s="230"/>
     </row>
     <row r="95" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I95" s="257"/>
+      <c r="I95" s="230"/>
     </row>
     <row r="96" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I96" s="257"/>
+      <c r="I96" s="230"/>
     </row>
     <row r="97" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I97" s="257"/>
+      <c r="I97" s="230"/>
     </row>
     <row r="98" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I98" s="257"/>
+      <c r="I98" s="230"/>
     </row>
     <row r="99" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I99" s="257"/>
+      <c r="I99" s="230"/>
     </row>
     <row r="100" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I100" s="257"/>
+      <c r="I100" s="230"/>
     </row>
     <row r="101" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I101" s="257"/>
+      <c r="I101" s="230"/>
     </row>
     <row r="102" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I102" s="257"/>
+      <c r="I102" s="230"/>
     </row>
     <row r="103" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I103" s="257"/>
+      <c r="I103" s="230"/>
     </row>
     <row r="104" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I104" s="257"/>
+      <c r="I104" s="230"/>
     </row>
     <row r="105" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I105" s="257"/>
+      <c r="I105" s="230"/>
     </row>
     <row r="106" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I106" s="257"/>
+      <c r="I106" s="230"/>
     </row>
     <row r="107" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I107" s="257"/>
+      <c r="I107" s="230"/>
     </row>
     <row r="108" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I108" s="257"/>
+      <c r="I108" s="230"/>
     </row>
     <row r="109" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I109" s="257"/>
+      <c r="I109" s="230"/>
     </row>
     <row r="110" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I110" s="257"/>
+      <c r="I110" s="230"/>
     </row>
     <row r="111" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I111" s="257"/>
+      <c r="I111" s="230"/>
     </row>
     <row r="112" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I112" s="257"/>
+      <c r="I112" s="230"/>
     </row>
     <row r="113" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I113" s="257"/>
+      <c r="I113" s="230"/>
     </row>
     <row r="114" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I114" s="257"/>
+      <c r="I114" s="230"/>
     </row>
     <row r="115" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I115" s="257"/>
+      <c r="I115" s="230"/>
     </row>
     <row r="116" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I116" s="257"/>
+      <c r="I116" s="230"/>
     </row>
     <row r="117" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I117" s="257"/>
+      <c r="I117" s="230"/>
     </row>
     <row r="118" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I118" s="257"/>
+      <c r="I118" s="230"/>
     </row>
     <row r="119" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I119" s="257"/>
+      <c r="I119" s="230"/>
     </row>
     <row r="120" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I120" s="257"/>
+      <c r="I120" s="230"/>
     </row>
     <row r="121" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I121" s="257"/>
+      <c r="I121" s="230"/>
     </row>
     <row r="122" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I122" s="257"/>
+      <c r="I122" s="230"/>
     </row>
     <row r="123" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I123" s="257"/>
+      <c r="I123" s="230"/>
     </row>
     <row r="124" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I124" s="257"/>
+      <c r="I124" s="230"/>
     </row>
     <row r="125" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I125" s="257"/>
+      <c r="I125" s="230"/>
     </row>
     <row r="126" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I126" s="257"/>
+      <c r="I126" s="230"/>
     </row>
     <row r="127" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I127" s="257"/>
+      <c r="I127" s="230"/>
     </row>
     <row r="128" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I128" s="257"/>
+      <c r="I128" s="230"/>
     </row>
     <row r="129" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I129" s="257"/>
+      <c r="I129" s="230"/>
     </row>
     <row r="130" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I130" s="257"/>
+      <c r="I130" s="230"/>
     </row>
     <row r="131" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I131" s="257"/>
+      <c r="I131" s="230"/>
     </row>
     <row r="132" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I132" s="257"/>
+      <c r="I132" s="230"/>
     </row>
     <row r="133" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I133" s="257"/>
+      <c r="I133" s="230"/>
     </row>
     <row r="134" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I134" s="257"/>
+      <c r="I134" s="230"/>
     </row>
     <row r="135" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I135" s="257"/>
+      <c r="I135" s="230"/>
     </row>
     <row r="136" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I136" s="257"/>
+      <c r="I136" s="230"/>
     </row>
     <row r="137" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I137" s="257"/>
+      <c r="I137" s="230"/>
     </row>
     <row r="138" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I138" s="257"/>
+      <c r="I138" s="230"/>
     </row>
     <row r="139" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I139" s="257"/>
+      <c r="I139" s="230"/>
     </row>
     <row r="140" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I140" s="257"/>
+      <c r="I140" s="230"/>
     </row>
     <row r="141" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I141" s="257"/>
+      <c r="I141" s="230"/>
     </row>
     <row r="142" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I142" s="257"/>
+      <c r="I142" s="230"/>
     </row>
     <row r="143" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I143" s="257"/>
+      <c r="I143" s="230"/>
     </row>
     <row r="144" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I144" s="257"/>
+      <c r="I144" s="230"/>
     </row>
     <row r="145" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I145" s="257"/>
+      <c r="I145" s="230"/>
     </row>
     <row r="146" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I146" s="257"/>
+      <c r="I146" s="230"/>
     </row>
     <row r="147" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I147" s="257"/>
+      <c r="I147" s="230"/>
     </row>
     <row r="148" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I148" s="257"/>
+      <c r="I148" s="230"/>
     </row>
     <row r="149" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I149" s="257"/>
+      <c r="I149" s="230"/>
     </row>
     <row r="150" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I150" s="257"/>
+      <c r="I150" s="230"/>
     </row>
     <row r="151" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I151" s="257"/>
+      <c r="I151" s="230"/>
     </row>
     <row r="152" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I152" s="257"/>
+      <c r="I152" s="230"/>
     </row>
     <row r="153" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I153" s="257"/>
+      <c r="I153" s="230"/>
     </row>
     <row r="154" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I154" s="257"/>
+      <c r="I154" s="230"/>
     </row>
     <row r="155" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I155" s="257"/>
+      <c r="I155" s="230"/>
     </row>
     <row r="156" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I156" s="257"/>
+      <c r="I156" s="230"/>
     </row>
     <row r="157" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I157" s="257"/>
+      <c r="I157" s="230"/>
     </row>
     <row r="158" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I158" s="257"/>
+      <c r="I158" s="230"/>
     </row>
     <row r="159" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I159" s="257"/>
+      <c r="I159" s="230"/>
     </row>
     <row r="160" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I160" s="257"/>
+      <c r="I160" s="230"/>
     </row>
     <row r="161" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I161" s="257"/>
+      <c r="I161" s="230"/>
     </row>
     <row r="162" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I162" s="257"/>
+      <c r="I162" s="230"/>
     </row>
     <row r="163" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I163" s="257"/>
+      <c r="I163" s="230"/>
     </row>
     <row r="164" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I164" s="257"/>
+      <c r="I164" s="230"/>
     </row>
     <row r="165" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I165" s="257"/>
+      <c r="I165" s="230"/>
     </row>
     <row r="166" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I166" s="257"/>
+      <c r="I166" s="230"/>
     </row>
     <row r="167" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I167" s="257"/>
+      <c r="I167" s="230"/>
     </row>
     <row r="168" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I168" s="257"/>
+      <c r="I168" s="230"/>
     </row>
     <row r="169" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I169" s="257"/>
+      <c r="I169" s="230"/>
     </row>
     <row r="170" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I170" s="257"/>
+      <c r="I170" s="230"/>
     </row>
     <row r="171" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I171" s="257"/>
+      <c r="I171" s="230"/>
     </row>
     <row r="172" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I172" s="257"/>
+      <c r="I172" s="230"/>
     </row>
     <row r="173" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I173" s="257"/>
+      <c r="I173" s="230"/>
     </row>
     <row r="174" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I174" s="257"/>
+      <c r="I174" s="230"/>
     </row>
     <row r="175" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I175" s="257"/>
+      <c r="I175" s="230"/>
     </row>
     <row r="176" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I176" s="257"/>
+      <c r="I176" s="230"/>
     </row>
     <row r="177" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I177" s="257"/>
+      <c r="I177" s="230"/>
     </row>
     <row r="178" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I178" s="257"/>
+      <c r="I178" s="230"/>
     </row>
     <row r="179" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I179" s="257"/>
+      <c r="I179" s="230"/>
     </row>
     <row r="180" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I180" s="257"/>
+      <c r="I180" s="230"/>
     </row>
     <row r="181" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I181" s="257"/>
+      <c r="I181" s="230"/>
     </row>
     <row r="182" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I182" s="257"/>
+      <c r="I182" s="230"/>
     </row>
     <row r="183" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I183" s="257"/>
+      <c r="I183" s="230"/>
     </row>
     <row r="184" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I184" s="257"/>
+      <c r="I184" s="230"/>
     </row>
     <row r="185" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I185" s="257"/>
+      <c r="I185" s="230"/>
     </row>
     <row r="186" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I186" s="257"/>
+      <c r="I186" s="230"/>
     </row>
     <row r="187" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I187" s="257"/>
+      <c r="I187" s="230"/>
     </row>
     <row r="188" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I188" s="257"/>
+      <c r="I188" s="230"/>
     </row>
     <row r="189" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I189" s="257"/>
+      <c r="I189" s="230"/>
     </row>
     <row r="190" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I190" s="257"/>
+      <c r="I190" s="230"/>
     </row>
     <row r="191" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I191" s="257"/>
+      <c r="I191" s="230"/>
     </row>
     <row r="192" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I192" s="257"/>
+      <c r="I192" s="230"/>
     </row>
     <row r="193" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I193" s="257"/>
+      <c r="I193" s="230"/>
     </row>
     <row r="194" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I194" s="257"/>
+      <c r="I194" s="230"/>
     </row>
     <row r="195" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I195" s="257"/>
+      <c r="I195" s="230"/>
     </row>
     <row r="196" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I196" s="257"/>
+      <c r="I196" s="230"/>
     </row>
     <row r="197" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I197" s="257"/>
+      <c r="I197" s="230"/>
     </row>
     <row r="198" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I198" s="257"/>
+      <c r="I198" s="230"/>
     </row>
     <row r="199" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I199" s="257"/>
+      <c r="I199" s="230"/>
     </row>
     <row r="200" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I200" s="257"/>
+      <c r="I200" s="230"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -14564,13 +14505,13 @@
     <mergeCell ref="U4:V4"/>
     <mergeCell ref="N4:T4"/>
   </mergeCells>
-  <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="1" priority="2">
+  <conditionalFormatting sqref="C6">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>AND(ISBLANK($D6)=FALSE,ISBLANK($F6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C6">
-    <cfRule type="expression" dxfId="0" priority="1">
+  <conditionalFormatting sqref="C6:V151">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>AND(ISBLANK($D6)=FALSE,ISBLANK($F6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16070,16 +16011,16 @@
   <sheetData>
     <row r="1" spans="1:62" s="59" customFormat="1" ht="12" x14ac:dyDescent="0.15">
       <c r="A1" s="102"/>
-      <c r="B1" s="253" t="s">
+      <c r="B1" s="262" t="s">
         <v>437</v>
       </c>
-      <c r="C1" s="253"/>
-      <c r="D1" s="253"/>
-      <c r="E1" s="253"/>
-      <c r="F1" s="253"/>
-      <c r="G1" s="253"/>
-      <c r="H1" s="253"/>
-      <c r="I1" s="253"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
+      <c r="H1" s="262"/>
+      <c r="I1" s="262"/>
       <c r="AC1" s="101"/>
       <c r="AD1" s="101"/>
       <c r="AE1" s="101"/>
@@ -16100,7 +16041,7 @@
       <c r="G2" s="97" t="s">
         <v>436</v>
       </c>
-      <c r="H2" s="252" t="s">
+      <c r="H2" s="261" t="s">
         <v>435</v>
       </c>
       <c r="I2" s="96" t="s">
@@ -16145,7 +16086,7 @@
       <c r="V2" s="96" t="s">
         <v>434</v>
       </c>
-      <c r="W2" s="252" t="s">
+      <c r="W2" s="261" t="s">
         <v>433</v>
       </c>
       <c r="X2" s="97" t="s">
@@ -16160,7 +16101,7 @@
       <c r="AA2" s="97" t="s">
         <v>150</v>
       </c>
-      <c r="AB2" s="252" t="s">
+      <c r="AB2" s="261" t="s">
         <v>432</v>
       </c>
       <c r="AC2" s="93" t="s">
@@ -16190,7 +16131,7 @@
       <c r="AK2" s="93" t="s">
         <v>431</v>
       </c>
-      <c r="AL2" s="252" t="s">
+      <c r="AL2" s="261" t="s">
         <v>430</v>
       </c>
       <c r="AM2" s="93" t="s">
@@ -16232,7 +16173,7 @@
       <c r="AY2" s="93" t="s">
         <v>429</v>
       </c>
-      <c r="AZ2" s="252" t="s">
+      <c r="AZ2" s="261" t="s">
         <v>428</v>
       </c>
       <c r="BA2" s="92" t="s">
@@ -16262,7 +16203,7 @@
       <c r="BI2" s="92" t="s">
         <v>427</v>
       </c>
-      <c r="BJ2" s="252" t="s">
+      <c r="BJ2" s="261" t="s">
         <v>426</v>
       </c>
     </row>
@@ -16276,7 +16217,7 @@
       <c r="G3" s="97" t="s">
         <v>425</v>
       </c>
-      <c r="H3" s="252"/>
+      <c r="H3" s="261"/>
       <c r="I3" s="96" t="s">
         <v>424</v>
       </c>
@@ -16317,7 +16258,7 @@
       <c r="V3" s="96" t="s">
         <v>412</v>
       </c>
-      <c r="W3" s="252"/>
+      <c r="W3" s="261"/>
       <c r="X3" s="91"/>
       <c r="Y3" s="97" t="s">
         <v>411</v>
@@ -16328,7 +16269,7 @@
       <c r="AA3" s="97" t="s">
         <v>409</v>
       </c>
-      <c r="AB3" s="252"/>
+      <c r="AB3" s="261"/>
       <c r="AC3" s="93" t="s">
         <v>408</v>
       </c>
@@ -16356,7 +16297,7 @@
       <c r="AK3" s="93" t="s">
         <v>402</v>
       </c>
-      <c r="AL3" s="252"/>
+      <c r="AL3" s="261"/>
       <c r="AM3" s="93" t="s">
         <v>401</v>
       </c>
@@ -16396,7 +16337,7 @@
       <c r="AY3" s="93" t="s">
         <v>389</v>
       </c>
-      <c r="AZ3" s="252"/>
+      <c r="AZ3" s="261"/>
       <c r="BA3" s="92" t="s">
         <v>388</v>
       </c>
@@ -16424,7 +16365,7 @@
       <c r="BI3" s="92" t="s">
         <v>380</v>
       </c>
-      <c r="BJ3" s="252"/>
+      <c r="BJ3" s="261"/>
     </row>
     <row r="4" spans="1:62" s="59" customFormat="1" ht="60" x14ac:dyDescent="0.15">
       <c r="A4" s="99"/>
@@ -16446,7 +16387,7 @@
       <c r="G4" s="97" t="s">
         <v>375</v>
       </c>
-      <c r="H4" s="252"/>
+      <c r="H4" s="261"/>
       <c r="I4" s="96" t="s">
         <v>374</v>
       </c>
@@ -16489,7 +16430,7 @@
       <c r="V4" s="95" t="s">
         <v>361</v>
       </c>
-      <c r="W4" s="252"/>
+      <c r="W4" s="261"/>
       <c r="X4" s="94" t="s">
         <v>360</v>
       </c>
@@ -16502,7 +16443,7 @@
       <c r="AA4" s="94" t="s">
         <v>357</v>
       </c>
-      <c r="AB4" s="252"/>
+      <c r="AB4" s="261"/>
       <c r="AC4" s="93" t="s">
         <v>356</v>
       </c>
@@ -16530,7 +16471,7 @@
       <c r="AK4" s="93" t="s">
         <v>349</v>
       </c>
-      <c r="AL4" s="252"/>
+      <c r="AL4" s="261"/>
       <c r="AM4" s="93" t="s">
         <v>348</v>
       </c>
@@ -16570,7 +16511,7 @@
       <c r="AY4" s="93" t="s">
         <v>336</v>
       </c>
-      <c r="AZ4" s="252"/>
+      <c r="AZ4" s="261"/>
       <c r="BA4" s="92" t="s">
         <v>335</v>
       </c>
@@ -16598,7 +16539,7 @@
       <c r="BI4" s="92" t="s">
         <v>327</v>
       </c>
-      <c r="BJ4" s="252"/>
+      <c r="BJ4" s="261"/>
     </row>
     <row r="5" spans="1:62" s="59" customFormat="1" ht="144" x14ac:dyDescent="0.15">
       <c r="A5" s="67" t="s">
@@ -17576,7 +17517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:62" s="59" customFormat="1" ht="48" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:62" s="59" customFormat="1" ht="36" x14ac:dyDescent="0.15">
       <c r="A13" s="67" t="s">
         <v>231</v>
       </c>
@@ -18288,16 +18229,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:62" s="107" customFormat="1" ht="23.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B1" s="255" t="s">
+      <c r="B1" s="264" t="s">
         <v>437</v>
       </c>
-      <c r="C1" s="255"/>
-      <c r="D1" s="255"/>
-      <c r="E1" s="255"/>
-      <c r="F1" s="255"/>
-      <c r="G1" s="255"/>
-      <c r="H1" s="255"/>
-      <c r="I1" s="255"/>
+      <c r="C1" s="264"/>
+      <c r="D1" s="264"/>
+      <c r="E1" s="264"/>
+      <c r="F1" s="264"/>
+      <c r="G1" s="264"/>
+      <c r="H1" s="264"/>
+      <c r="I1" s="264"/>
     </row>
     <row r="2" spans="1:62" s="107" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="153"/>
@@ -18309,7 +18250,7 @@
       <c r="G2" s="150" t="s">
         <v>436</v>
       </c>
-      <c r="H2" s="254" t="s">
+      <c r="H2" s="263" t="s">
         <v>435</v>
       </c>
       <c r="I2" s="149" t="s">
@@ -18354,7 +18295,7 @@
       <c r="V2" s="149" t="s">
         <v>434</v>
       </c>
-      <c r="W2" s="254" t="s">
+      <c r="W2" s="263" t="s">
         <v>433</v>
       </c>
       <c r="X2" s="150" t="s">
@@ -18369,7 +18310,7 @@
       <c r="AA2" s="150" t="s">
         <v>150</v>
       </c>
-      <c r="AB2" s="254" t="s">
+      <c r="AB2" s="263" t="s">
         <v>432</v>
       </c>
       <c r="AC2" s="147" t="s">
@@ -18399,7 +18340,7 @@
       <c r="AK2" s="147" t="s">
         <v>431</v>
       </c>
-      <c r="AL2" s="254" t="s">
+      <c r="AL2" s="263" t="s">
         <v>430</v>
       </c>
       <c r="AM2" s="147" t="s">
@@ -18441,7 +18382,7 @@
       <c r="AY2" s="147" t="s">
         <v>429</v>
       </c>
-      <c r="AZ2" s="254" t="s">
+      <c r="AZ2" s="263" t="s">
         <v>428</v>
       </c>
       <c r="BA2" s="146" t="s">
@@ -18471,7 +18412,7 @@
       <c r="BI2" s="146" t="s">
         <v>427</v>
       </c>
-      <c r="BJ2" s="254" t="s">
+      <c r="BJ2" s="263" t="s">
         <v>426</v>
       </c>
     </row>
@@ -18485,7 +18426,7 @@
       <c r="G3" s="150" t="s">
         <v>425</v>
       </c>
-      <c r="H3" s="254"/>
+      <c r="H3" s="263"/>
       <c r="I3" s="149" t="s">
         <v>424</v>
       </c>
@@ -18526,7 +18467,7 @@
       <c r="V3" s="149" t="s">
         <v>412</v>
       </c>
-      <c r="W3" s="254"/>
+      <c r="W3" s="263"/>
       <c r="X3" s="145"/>
       <c r="Y3" s="150" t="s">
         <v>411</v>
@@ -18537,7 +18478,7 @@
       <c r="AA3" s="150" t="s">
         <v>409</v>
       </c>
-      <c r="AB3" s="254"/>
+      <c r="AB3" s="263"/>
       <c r="AC3" s="147" t="s">
         <v>408</v>
       </c>
@@ -18565,7 +18506,7 @@
       <c r="AK3" s="147" t="s">
         <v>402</v>
       </c>
-      <c r="AL3" s="254"/>
+      <c r="AL3" s="263"/>
       <c r="AM3" s="147" t="s">
         <v>401</v>
       </c>
@@ -18605,7 +18546,7 @@
       <c r="AY3" s="147" t="s">
         <v>389</v>
       </c>
-      <c r="AZ3" s="254"/>
+      <c r="AZ3" s="263"/>
       <c r="BA3" s="146" t="s">
         <v>388</v>
       </c>
@@ -18633,7 +18574,7 @@
       <c r="BI3" s="146" t="s">
         <v>380</v>
       </c>
-      <c r="BJ3" s="254"/>
+      <c r="BJ3" s="263"/>
     </row>
     <row r="4" spans="1:62" s="107" customFormat="1" ht="60" x14ac:dyDescent="0.15">
       <c r="A4" s="152"/>
@@ -18655,7 +18596,7 @@
       <c r="G4" s="150" t="s">
         <v>375</v>
       </c>
-      <c r="H4" s="254"/>
+      <c r="H4" s="263"/>
       <c r="I4" s="149" t="s">
         <v>374</v>
       </c>
@@ -18698,7 +18639,7 @@
       <c r="V4" s="149" t="s">
         <v>361</v>
       </c>
-      <c r="W4" s="254"/>
+      <c r="W4" s="263"/>
       <c r="X4" s="148" t="s">
         <v>360</v>
       </c>
@@ -18711,7 +18652,7 @@
       <c r="AA4" s="148" t="s">
         <v>357</v>
       </c>
-      <c r="AB4" s="254"/>
+      <c r="AB4" s="263"/>
       <c r="AC4" s="147" t="s">
         <v>356</v>
       </c>
@@ -18739,7 +18680,7 @@
       <c r="AK4" s="147" t="s">
         <v>349</v>
       </c>
-      <c r="AL4" s="254"/>
+      <c r="AL4" s="263"/>
       <c r="AM4" s="147" t="s">
         <v>348</v>
       </c>
@@ -18779,7 +18720,7 @@
       <c r="AY4" s="147" t="s">
         <v>336</v>
       </c>
-      <c r="AZ4" s="254"/>
+      <c r="AZ4" s="263"/>
       <c r="BA4" s="146" t="s">
         <v>335</v>
       </c>
@@ -18807,7 +18748,7 @@
       <c r="BI4" s="146" t="s">
         <v>327</v>
       </c>
-      <c r="BJ4" s="254"/>
+      <c r="BJ4" s="263"/>
     </row>
     <row r="5" spans="1:62" s="107" customFormat="1" ht="11" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="117" t="s">

</xml_diff>

<commit_message>
attaché de justice extracteur CA et TJ
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54D69408-9140-1F4F-916F-2356CC71142F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{956251AA-BB3D-9C4F-A9C1-8FA0D21741F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1947" uniqueCount="578">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1948" uniqueCount="580">
   <si>
     <t>#! END_ROW</t>
   </si>
@@ -5203,6 +5203,12 @@
       </rPr>
       <t>Critère sur le TPRX</t>
     </r>
+  </si>
+  <si>
+    <t>Att J</t>
+  </si>
+  <si>
+    <t>Pas encore appelé dans la matrice DDG, à voir en fonction de la circulaire 2025/2026</t>
   </si>
 </sst>
 </file>
@@ -6398,7 +6404,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="374">
+  <cellXfs count="373">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -7471,6 +7477,55 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="169" fontId="67" fillId="16" borderId="13" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="71" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="42" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="41" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -7587,56 +7642,6 @@
     </xf>
     <xf numFmtId="0" fontId="55" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="67" fillId="16" borderId="13" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="68" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="71" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="42" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="62" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
   </cellXfs>
@@ -8442,11 +8447,11 @@
       <c r="B1" s="145" t="s">
         <v>384</v>
       </c>
-      <c r="C1" s="321" t="s">
+      <c r="C1" s="336" t="s">
         <v>385</v>
       </c>
-      <c r="D1" s="321"/>
-      <c r="E1" s="321"/>
+      <c r="D1" s="336"/>
+      <c r="E1" s="336"/>
       <c r="F1" s="146"/>
       <c r="H1" s="26" t="s">
         <v>0</v>
@@ -8455,11 +8460,11 @@
     <row r="2" spans="1:8" s="150" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="147"/>
       <c r="B2" s="148"/>
-      <c r="C2" s="322" t="s">
+      <c r="C2" s="337" t="s">
         <v>386</v>
       </c>
-      <c r="D2" s="322"/>
-      <c r="E2" s="322"/>
+      <c r="D2" s="337"/>
+      <c r="E2" s="337"/>
       <c r="F2" s="149"/>
       <c r="H2" s="26" t="s">
         <v>0</v>
@@ -8483,10 +8488,10 @@
       <c r="D4" s="155" t="s">
         <v>389</v>
       </c>
-      <c r="E4" s="328" t="s">
+      <c r="E4" s="343" t="s">
         <v>390</v>
       </c>
-      <c r="F4" s="329"/>
+      <c r="F4" s="344"/>
       <c r="G4" s="164"/>
       <c r="H4" s="26" t="s">
         <v>0</v>
@@ -8503,10 +8508,10 @@
       <c r="D5" s="161" t="s">
         <v>393</v>
       </c>
-      <c r="E5" s="330" t="s">
+      <c r="E5" s="345" t="s">
         <v>406</v>
       </c>
-      <c r="F5" s="331"/>
+      <c r="F5" s="346"/>
       <c r="G5" s="163"/>
       <c r="H5" s="26" t="s">
         <v>0</v>
@@ -8523,10 +8528,10 @@
       <c r="D6" s="162" t="s">
         <v>396</v>
       </c>
-      <c r="E6" s="332" t="s">
+      <c r="E6" s="347" t="s">
         <v>407</v>
       </c>
-      <c r="F6" s="333"/>
+      <c r="F6" s="348"/>
       <c r="G6" s="163"/>
       <c r="H6" s="26" t="s">
         <v>0</v>
@@ -8543,10 +8548,10 @@
       <c r="D7" s="162" t="s">
         <v>399</v>
       </c>
-      <c r="E7" s="332" t="s">
+      <c r="E7" s="347" t="s">
         <v>406</v>
       </c>
-      <c r="F7" s="333"/>
+      <c r="F7" s="348"/>
       <c r="G7" s="163"/>
       <c r="H7" s="26" t="s">
         <v>0</v>
@@ -8557,16 +8562,16 @@
       <c r="B8" s="171" t="s">
         <v>400</v>
       </c>
-      <c r="C8" s="323" t="s">
+      <c r="C8" s="338" t="s">
         <v>401</v>
       </c>
-      <c r="D8" s="323" t="s">
+      <c r="D8" s="338" t="s">
         <v>402</v>
       </c>
-      <c r="E8" s="334" t="s">
+      <c r="E8" s="349" t="s">
         <v>408</v>
       </c>
-      <c r="F8" s="335"/>
+      <c r="F8" s="350"/>
       <c r="G8" s="163"/>
       <c r="H8" s="26" t="s">
         <v>0</v>
@@ -8577,10 +8582,10 @@
       <c r="B9" s="172" t="s">
         <v>403</v>
       </c>
-      <c r="C9" s="323"/>
-      <c r="D9" s="323"/>
-      <c r="E9" s="336"/>
-      <c r="F9" s="337"/>
+      <c r="C9" s="338"/>
+      <c r="D9" s="338"/>
+      <c r="E9" s="351"/>
+      <c r="F9" s="352"/>
       <c r="G9" s="163"/>
       <c r="H9" s="26" t="s">
         <v>0</v>
@@ -8591,10 +8596,10 @@
       <c r="B10" s="173" t="s">
         <v>404</v>
       </c>
-      <c r="C10" s="324"/>
-      <c r="D10" s="324"/>
-      <c r="E10" s="338"/>
-      <c r="F10" s="339"/>
+      <c r="C10" s="339"/>
+      <c r="D10" s="339"/>
+      <c r="E10" s="353"/>
+      <c r="F10" s="354"/>
       <c r="G10" s="163"/>
       <c r="H10" s="26" t="s">
         <v>0</v>
@@ -8614,11 +8619,11 @@
     <row r="12" spans="1:8" s="26" customFormat="1" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="151"/>
       <c r="B12" s="165"/>
-      <c r="C12" s="327" t="s">
+      <c r="C12" s="342" t="s">
         <v>405</v>
       </c>
-      <c r="D12" s="327"/>
-      <c r="E12" s="327"/>
+      <c r="D12" s="342"/>
+      <c r="E12" s="342"/>
       <c r="F12" s="166"/>
       <c r="H12" s="26" t="s">
         <v>0</v>
@@ -8632,14 +8637,14 @@
       </c>
     </row>
     <row r="14" spans="1:8" s="26" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="325" t="s">
+      <c r="A14" s="340" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="325"/>
-      <c r="C14" s="325"/>
-      <c r="D14" s="325"/>
-      <c r="E14" s="325"/>
-      <c r="F14" s="326"/>
+      <c r="B14" s="340"/>
+      <c r="C14" s="340"/>
+      <c r="D14" s="340"/>
+      <c r="E14" s="340"/>
+      <c r="F14" s="341"/>
       <c r="H14" s="26" t="s">
         <v>0</v>
       </c>
@@ -8707,13 +8712,13 @@
       <c r="G2" s="103" t="s">
         <v>326</v>
       </c>
-      <c r="H2" s="347" t="s">
+      <c r="H2" s="362" t="s">
         <v>325</v>
       </c>
       <c r="I2" s="103" t="s">
         <v>144</v>
       </c>
-      <c r="J2" s="347" t="s">
+      <c r="J2" s="362" t="s">
         <v>324</v>
       </c>
     </row>
@@ -8727,11 +8732,11 @@
       <c r="G3" s="103" t="s">
         <v>304</v>
       </c>
-      <c r="H3" s="347"/>
+      <c r="H3" s="362"/>
       <c r="I3" s="103" t="s">
         <v>301</v>
       </c>
-      <c r="J3" s="347"/>
+      <c r="J3" s="362"/>
     </row>
     <row r="4" spans="1:10" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="125"/>
@@ -8753,11 +8758,11 @@
       <c r="G4" s="103" t="s">
         <v>253</v>
       </c>
-      <c r="H4" s="347"/>
+      <c r="H4" s="362"/>
       <c r="I4" s="103" t="s">
         <v>249</v>
       </c>
-      <c r="J4" s="347"/>
+      <c r="J4" s="362"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="119" t="s">
@@ -9156,7 +9161,7 @@
       <c r="G2" s="103" t="s">
         <v>328</v>
       </c>
-      <c r="H2" s="347" t="s">
+      <c r="H2" s="362" t="s">
         <v>327</v>
       </c>
       <c r="I2" s="102" t="s">
@@ -9201,7 +9206,7 @@
       <c r="V2" s="102" t="s">
         <v>326</v>
       </c>
-      <c r="W2" s="347" t="s">
+      <c r="W2" s="362" t="s">
         <v>325</v>
       </c>
       <c r="X2" s="103" t="s">
@@ -9216,7 +9221,7 @@
       <c r="AA2" s="103" t="s">
         <v>144</v>
       </c>
-      <c r="AB2" s="347" t="s">
+      <c r="AB2" s="362" t="s">
         <v>324</v>
       </c>
       <c r="AC2" s="100" t="s">
@@ -9246,7 +9251,7 @@
       <c r="AK2" s="100" t="s">
         <v>323</v>
       </c>
-      <c r="AL2" s="347" t="s">
+      <c r="AL2" s="362" t="s">
         <v>322</v>
       </c>
       <c r="AM2" s="100" t="s">
@@ -9288,7 +9293,7 @@
       <c r="AY2" s="100" t="s">
         <v>321</v>
       </c>
-      <c r="AZ2" s="347" t="s">
+      <c r="AZ2" s="362" t="s">
         <v>320</v>
       </c>
       <c r="BA2" s="99" t="s">
@@ -9318,7 +9323,7 @@
       <c r="BI2" s="99" t="s">
         <v>319</v>
       </c>
-      <c r="BJ2" s="347" t="s">
+      <c r="BJ2" s="362" t="s">
         <v>318</v>
       </c>
       <c r="BK2"/>
@@ -9333,7 +9338,7 @@
       <c r="G3" s="103" t="s">
         <v>317</v>
       </c>
-      <c r="H3" s="347"/>
+      <c r="H3" s="362"/>
       <c r="I3" s="102" t="s">
         <v>316</v>
       </c>
@@ -9374,7 +9379,7 @@
       <c r="V3" s="102" t="s">
         <v>304</v>
       </c>
-      <c r="W3" s="347"/>
+      <c r="W3" s="362"/>
       <c r="X3" s="98"/>
       <c r="Y3" s="103" t="s">
         <v>303</v>
@@ -9385,7 +9390,7 @@
       <c r="AA3" s="103" t="s">
         <v>301</v>
       </c>
-      <c r="AB3" s="347"/>
+      <c r="AB3" s="362"/>
       <c r="AC3" s="100" t="s">
         <v>300</v>
       </c>
@@ -9413,7 +9418,7 @@
       <c r="AK3" s="100" t="s">
         <v>294</v>
       </c>
-      <c r="AL3" s="347"/>
+      <c r="AL3" s="362"/>
       <c r="AM3" s="100" t="s">
         <v>293</v>
       </c>
@@ -9453,7 +9458,7 @@
       <c r="AY3" s="100" t="s">
         <v>281</v>
       </c>
-      <c r="AZ3" s="347"/>
+      <c r="AZ3" s="362"/>
       <c r="BA3" s="99" t="s">
         <v>280</v>
       </c>
@@ -9481,7 +9486,7 @@
       <c r="BI3" s="99" t="s">
         <v>272</v>
       </c>
-      <c r="BJ3" s="347"/>
+      <c r="BJ3" s="362"/>
     </row>
     <row r="4" spans="1:63" s="60" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="105"/>
@@ -9503,7 +9508,7 @@
       <c r="G4" s="103" t="s">
         <v>267</v>
       </c>
-      <c r="H4" s="347"/>
+      <c r="H4" s="362"/>
       <c r="I4" s="102" t="s">
         <v>266</v>
       </c>
@@ -9546,7 +9551,7 @@
       <c r="V4" s="102" t="s">
         <v>253</v>
       </c>
-      <c r="W4" s="347"/>
+      <c r="W4" s="362"/>
       <c r="X4" s="101" t="s">
         <v>252</v>
       </c>
@@ -9559,7 +9564,7 @@
       <c r="AA4" s="101" t="s">
         <v>249</v>
       </c>
-      <c r="AB4" s="347"/>
+      <c r="AB4" s="362"/>
       <c r="AC4" s="100" t="s">
         <v>248</v>
       </c>
@@ -9587,7 +9592,7 @@
       <c r="AK4" s="100" t="s">
         <v>241</v>
       </c>
-      <c r="AL4" s="347"/>
+      <c r="AL4" s="362"/>
       <c r="AM4" s="100" t="s">
         <v>240</v>
       </c>
@@ -9627,7 +9632,7 @@
       <c r="AY4" s="100" t="s">
         <v>228</v>
       </c>
-      <c r="AZ4" s="347"/>
+      <c r="AZ4" s="362"/>
       <c r="BA4" s="99" t="s">
         <v>227</v>
       </c>
@@ -9655,7 +9660,7 @@
       <c r="BI4" s="99" t="s">
         <v>219</v>
       </c>
-      <c r="BJ4" s="347"/>
+      <c r="BJ4" s="362"/>
       <c r="BK4"/>
     </row>
     <row r="5" spans="1:63" s="60" customFormat="1" ht="15" x14ac:dyDescent="0.2">
@@ -12267,15 +12272,15 @@
       </c>
     </row>
     <row r="19" spans="4:52" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="20" spans="4:52" ht="280" x14ac:dyDescent="0.2">
-      <c r="F20" s="360" t="s">
+    <row r="20" spans="4:52" ht="28" x14ac:dyDescent="0.2">
+      <c r="F20" s="323" t="s">
         <v>553</v>
       </c>
       <c r="G20" s="254" t="str">
         <f>IF(ISBLANK(ETPT_TJ_DDG!$D$5),"",IF(ISERROR(ETPT_TJ!G20),"",IF(ETPT_TJ!G20=0,"",ETPT_TJ!G20)))</f>
         <v/>
       </c>
-      <c r="U20" s="361" t="s">
+      <c r="U20" s="324" t="s">
         <v>555</v>
       </c>
       <c r="V20" s="254" t="str">
@@ -12283,7 +12288,7 @@
         <v/>
       </c>
       <c r="AH20" s="57"/>
-      <c r="AX20" s="359" t="s">
+      <c r="AX20" s="322" t="s">
         <v>551</v>
       </c>
       <c r="AY20" s="196" t="str">
@@ -12400,7 +12405,7 @@
       <c r="G2" s="103" t="s">
         <v>328</v>
       </c>
-      <c r="H2" s="347" t="s">
+      <c r="H2" s="362" t="s">
         <v>327</v>
       </c>
       <c r="I2" s="103" t="s">
@@ -12433,13 +12438,13 @@
       <c r="R2" s="103" t="s">
         <v>326</v>
       </c>
-      <c r="S2" s="347" t="s">
+      <c r="S2" s="362" t="s">
         <v>325</v>
       </c>
       <c r="T2" s="103" t="s">
         <v>144</v>
       </c>
-      <c r="U2" s="347" t="s">
+      <c r="U2" s="362" t="s">
         <v>324</v>
       </c>
       <c r="V2" s="103" t="s">
@@ -12469,7 +12474,7 @@
       <c r="AD2" s="103" t="s">
         <v>323</v>
       </c>
-      <c r="AE2" s="347" t="s">
+      <c r="AE2" s="362" t="s">
         <v>372</v>
       </c>
       <c r="AF2" s="103" t="s">
@@ -12481,7 +12486,7 @@
       <c r="AH2" s="103" t="s">
         <v>371</v>
       </c>
-      <c r="AI2" s="347" t="s">
+      <c r="AI2" s="362" t="s">
         <v>370</v>
       </c>
     </row>
@@ -12495,7 +12500,7 @@
       <c r="G3" s="103" t="s">
         <v>317</v>
       </c>
-      <c r="H3" s="347"/>
+      <c r="H3" s="362"/>
       <c r="I3" s="103" t="s">
         <v>369</v>
       </c>
@@ -12526,11 +12531,11 @@
       <c r="R3" s="103" t="s">
         <v>304</v>
       </c>
-      <c r="S3" s="347"/>
+      <c r="S3" s="362"/>
       <c r="T3" s="103" t="s">
         <v>301</v>
       </c>
-      <c r="U3" s="347"/>
+      <c r="U3" s="362"/>
       <c r="V3" s="103" t="s">
         <v>360</v>
       </c>
@@ -12558,7 +12563,7 @@
       <c r="AD3" s="103" t="s">
         <v>352</v>
       </c>
-      <c r="AE3" s="347"/>
+      <c r="AE3" s="362"/>
       <c r="AF3" s="103" t="s">
         <v>351</v>
       </c>
@@ -12568,7 +12573,7 @@
       <c r="AH3" s="103" t="s">
         <v>281</v>
       </c>
-      <c r="AI3" s="347"/>
+      <c r="AI3" s="362"/>
     </row>
     <row r="4" spans="1:62" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="106"/>
@@ -12590,7 +12595,7 @@
       <c r="G4" s="103" t="s">
         <v>267</v>
       </c>
-      <c r="H4" s="347"/>
+      <c r="H4" s="362"/>
       <c r="I4" s="103" t="s">
         <v>350</v>
       </c>
@@ -12621,11 +12626,11 @@
       <c r="R4" s="103" t="s">
         <v>253</v>
       </c>
-      <c r="S4" s="347"/>
+      <c r="S4" s="362"/>
       <c r="T4" s="103" t="s">
         <v>249</v>
       </c>
-      <c r="U4" s="347"/>
+      <c r="U4" s="362"/>
       <c r="V4" s="103" t="s">
         <v>341</v>
       </c>
@@ -12653,7 +12658,7 @@
       <c r="AD4" s="103" t="s">
         <v>333</v>
       </c>
-      <c r="AE4" s="347"/>
+      <c r="AE4" s="362"/>
       <c r="AF4" s="103" t="s">
         <v>332</v>
       </c>
@@ -12663,7 +12668,7 @@
       <c r="AH4" s="103" t="s">
         <v>228</v>
       </c>
-      <c r="AI4" s="347"/>
+      <c r="AI4" s="362"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="109" t="s">
@@ -14255,9 +14260,9 @@
       <c r="S17" s="59"/>
     </row>
     <row r="18" spans="4:34" ht="93" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D18" s="363"/>
-      <c r="E18" s="364"/>
-      <c r="F18" s="360" t="s">
+      <c r="D18" s="326"/>
+      <c r="E18"/>
+      <c r="F18" s="323" t="s">
         <v>553</v>
       </c>
       <c r="G18" s="254" t="str">
@@ -14268,15 +14273,15 @@
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
-      <c r="Q18" s="361" t="s">
+      <c r="Q18" s="324" t="s">
         <v>555</v>
       </c>
       <c r="R18" s="254" t="str">
         <f>IF(ISBLANK(ETPT_TPRX_DDG!$D$5),"",IF(ISERROR(ETPT_TPRX!R18),"",IF(ETPT_TPRX!R18=0,"",ETPT_TPRX!R18)))</f>
         <v/>
       </c>
-      <c r="AF18" s="362"/>
-      <c r="AG18" s="359" t="s">
+      <c r="AF18" s="325"/>
+      <c r="AG18" s="322" t="s">
         <v>551</v>
       </c>
       <c r="AH18" s="254" t="str">
@@ -14415,13 +14420,13 @@
       <c r="G2" s="103" t="s">
         <v>326</v>
       </c>
-      <c r="H2" s="347" t="s">
+      <c r="H2" s="362" t="s">
         <v>325</v>
       </c>
       <c r="I2" s="103" t="s">
         <v>144</v>
       </c>
-      <c r="J2" s="347" t="s">
+      <c r="J2" s="362" t="s">
         <v>324</v>
       </c>
     </row>
@@ -14435,11 +14440,11 @@
       <c r="G3" s="103" t="s">
         <v>304</v>
       </c>
-      <c r="H3" s="347"/>
+      <c r="H3" s="362"/>
       <c r="I3" s="103" t="s">
         <v>301</v>
       </c>
-      <c r="J3" s="347"/>
+      <c r="J3" s="362"/>
     </row>
     <row r="4" spans="1:62" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="125"/>
@@ -14461,11 +14466,11 @@
       <c r="G4" s="103" t="s">
         <v>253</v>
       </c>
-      <c r="H4" s="347"/>
+      <c r="H4" s="362"/>
       <c r="I4" s="103" t="s">
         <v>249</v>
       </c>
-      <c r="J4" s="347"/>
+      <c r="J4" s="362"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="119" t="s">
@@ -14852,13 +14857,13 @@
   <sheetData>
     <row r="1" spans="1:61" s="186" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="185"/>
-      <c r="B1" s="351" t="s">
+      <c r="B1" s="366" t="s">
         <v>329</v>
       </c>
-      <c r="C1" s="351"/>
-      <c r="D1" s="351"/>
-      <c r="E1" s="351"/>
-      <c r="F1" s="351"/>
+      <c r="C1" s="366"/>
+      <c r="D1" s="366"/>
+      <c r="E1" s="366"/>
+      <c r="F1" s="366"/>
       <c r="G1" s="187"/>
       <c r="H1" s="187"/>
       <c r="I1" s="187"/>
@@ -14903,7 +14908,7 @@
       <c r="O2" s="189" t="s">
         <v>323</v>
       </c>
-      <c r="P2" s="350" t="s">
+      <c r="P2" s="365" t="s">
         <v>322</v>
       </c>
       <c r="Q2" s="189" t="s">
@@ -14945,7 +14950,7 @@
       <c r="AC2" s="189" t="s">
         <v>321</v>
       </c>
-      <c r="AD2" s="350" t="s">
+      <c r="AD2" s="365" t="s">
         <v>320</v>
       </c>
       <c r="AE2" s="190" t="s">
@@ -14975,7 +14980,7 @@
       <c r="AM2" s="190" t="s">
         <v>319</v>
       </c>
-      <c r="AN2" s="350" t="s">
+      <c r="AN2" s="365" t="s">
         <v>318</v>
       </c>
       <c r="AQ2" s="189"/>
@@ -14986,7 +14991,7 @@
       <c r="AV2" s="189"/>
       <c r="AW2" s="189"/>
       <c r="AX2" s="189"/>
-      <c r="AY2" s="350"/>
+      <c r="AY2" s="365"/>
       <c r="AZ2" s="190"/>
       <c r="BA2" s="190"/>
       <c r="BB2" s="190"/>
@@ -14996,7 +15001,7 @@
       <c r="BF2" s="190"/>
       <c r="BG2" s="190"/>
       <c r="BH2" s="190"/>
-      <c r="BI2" s="350"/>
+      <c r="BI2" s="365"/>
     </row>
     <row r="3" spans="1:61" s="186" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="188"/>
@@ -15032,7 +15037,7 @@
       <c r="O3" s="189" t="s">
         <v>294</v>
       </c>
-      <c r="P3" s="350"/>
+      <c r="P3" s="365"/>
       <c r="Q3" s="189" t="s">
         <v>293</v>
       </c>
@@ -15072,7 +15077,7 @@
       <c r="AC3" s="189" t="s">
         <v>281</v>
       </c>
-      <c r="AD3" s="350"/>
+      <c r="AD3" s="365"/>
       <c r="AE3" s="190" t="s">
         <v>280</v>
       </c>
@@ -15100,7 +15105,7 @@
       <c r="AM3" s="190" t="s">
         <v>272</v>
       </c>
-      <c r="AN3" s="350"/>
+      <c r="AN3" s="365"/>
       <c r="AQ3" s="189"/>
       <c r="AR3" s="189"/>
       <c r="AS3" s="189"/>
@@ -15109,7 +15114,7 @@
       <c r="AV3" s="189"/>
       <c r="AW3" s="189"/>
       <c r="AX3" s="189"/>
-      <c r="AY3" s="350"/>
+      <c r="AY3" s="365"/>
       <c r="AZ3" s="190"/>
       <c r="BA3" s="190"/>
       <c r="BB3" s="190"/>
@@ -15119,7 +15124,7 @@
       <c r="BF3" s="190"/>
       <c r="BG3" s="190"/>
       <c r="BH3" s="190"/>
-      <c r="BI3" s="350"/>
+      <c r="BI3" s="365"/>
     </row>
     <row r="4" spans="1:61" s="186" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="191"/>
@@ -15165,7 +15170,7 @@
       <c r="O4" s="189" t="s">
         <v>241</v>
       </c>
-      <c r="P4" s="350"/>
+      <c r="P4" s="365"/>
       <c r="Q4" s="189" t="s">
         <v>240</v>
       </c>
@@ -15205,7 +15210,7 @@
       <c r="AC4" s="189" t="s">
         <v>228</v>
       </c>
-      <c r="AD4" s="350"/>
+      <c r="AD4" s="365"/>
       <c r="AE4" s="190" t="s">
         <v>227</v>
       </c>
@@ -15233,7 +15238,7 @@
       <c r="AM4" s="190" t="s">
         <v>219</v>
       </c>
-      <c r="AN4" s="350"/>
+      <c r="AN4" s="365"/>
       <c r="AQ4" s="189"/>
       <c r="AR4" s="189"/>
       <c r="AS4" s="189"/>
@@ -15242,7 +15247,7 @@
       <c r="AV4" s="189"/>
       <c r="AW4" s="189"/>
       <c r="AX4" s="189"/>
-      <c r="AY4" s="350"/>
+      <c r="AY4" s="365"/>
       <c r="AZ4" s="190"/>
       <c r="BA4" s="190"/>
       <c r="BB4" s="190"/>
@@ -15252,7 +15257,7 @@
       <c r="BF4" s="190"/>
       <c r="BG4" s="190"/>
       <c r="BH4" s="190"/>
-      <c r="BI4" s="350"/>
+      <c r="BI4" s="365"/>
     </row>
     <row r="5" spans="1:61" s="186" customFormat="1" ht="144" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="193" t="s">
@@ -16464,492 +16469,492 @@
       <c r="BI16" s="197"/>
     </row>
     <row r="17" spans="1:42" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="365"/>
-      <c r="B17" s="362"/>
-      <c r="C17" s="362"/>
-      <c r="D17" s="365"/>
-      <c r="E17" s="365"/>
-      <c r="F17" s="365"/>
-      <c r="G17" s="362"/>
-      <c r="H17" s="362"/>
-      <c r="I17" s="362"/>
-      <c r="J17" s="362"/>
-      <c r="K17" s="362"/>
-      <c r="L17" s="362"/>
-      <c r="M17" s="362"/>
-      <c r="N17" s="362"/>
-      <c r="O17" s="362"/>
-      <c r="P17" s="362"/>
-      <c r="Q17" s="362"/>
-      <c r="R17" s="362"/>
-      <c r="S17" s="362"/>
-      <c r="T17" s="362"/>
-      <c r="U17" s="362"/>
-      <c r="V17" s="362"/>
-      <c r="W17" s="362"/>
-      <c r="X17" s="362"/>
-      <c r="Y17" s="362"/>
-      <c r="Z17" s="362"/>
-      <c r="AA17" s="362"/>
-      <c r="AB17" s="362"/>
-      <c r="AC17" s="362"/>
-      <c r="AD17" s="362"/>
-      <c r="AE17" s="362"/>
-      <c r="AF17" s="362"/>
-      <c r="AG17" s="362"/>
-      <c r="AH17" s="362"/>
-      <c r="AI17" s="362"/>
-      <c r="AJ17" s="362"/>
-      <c r="AK17" s="362"/>
-      <c r="AL17" s="362"/>
-      <c r="AM17" s="362"/>
-      <c r="AN17" s="362"/>
-      <c r="AO17" s="362"/>
-      <c r="AP17" s="362"/>
+      <c r="A17" s="327"/>
+      <c r="B17" s="325"/>
+      <c r="C17" s="325"/>
+      <c r="D17" s="327"/>
+      <c r="E17" s="327"/>
+      <c r="F17" s="327"/>
+      <c r="G17" s="325"/>
+      <c r="H17" s="325"/>
+      <c r="I17" s="325"/>
+      <c r="J17" s="325"/>
+      <c r="K17" s="325"/>
+      <c r="L17" s="325"/>
+      <c r="M17" s="325"/>
+      <c r="N17" s="325"/>
+      <c r="O17" s="325"/>
+      <c r="P17" s="325"/>
+      <c r="Q17" s="325"/>
+      <c r="R17" s="325"/>
+      <c r="S17" s="325"/>
+      <c r="T17" s="325"/>
+      <c r="U17" s="325"/>
+      <c r="V17" s="325"/>
+      <c r="W17" s="325"/>
+      <c r="X17" s="325"/>
+      <c r="Y17" s="325"/>
+      <c r="Z17" s="325"/>
+      <c r="AA17" s="325"/>
+      <c r="AB17" s="325"/>
+      <c r="AC17" s="325"/>
+      <c r="AD17" s="325"/>
+      <c r="AE17" s="325"/>
+      <c r="AF17" s="325"/>
+      <c r="AG17" s="325"/>
+      <c r="AH17" s="325"/>
+      <c r="AI17" s="325"/>
+      <c r="AJ17" s="325"/>
+      <c r="AK17" s="325"/>
+      <c r="AL17" s="325"/>
+      <c r="AM17" s="325"/>
+      <c r="AN17" s="325"/>
+      <c r="AO17" s="325"/>
+      <c r="AP17" s="325"/>
     </row>
     <row r="18" spans="1:42" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="365"/>
-      <c r="B18" s="362"/>
-      <c r="C18" s="362"/>
-      <c r="D18" s="365"/>
-      <c r="E18" s="365"/>
-      <c r="F18" s="365"/>
-      <c r="G18" s="362"/>
-      <c r="H18" s="362"/>
-      <c r="I18" s="362"/>
-      <c r="J18" s="362"/>
-      <c r="K18" s="362"/>
-      <c r="L18" s="362"/>
-      <c r="M18" s="362"/>
-      <c r="N18" s="362"/>
-      <c r="O18" s="362"/>
-      <c r="P18" s="362"/>
-      <c r="Q18" s="362"/>
-      <c r="R18" s="362"/>
-      <c r="S18" s="362"/>
-      <c r="T18" s="362"/>
-      <c r="U18" s="362"/>
-      <c r="V18" s="362"/>
-      <c r="W18" s="362"/>
-      <c r="X18" s="362"/>
-      <c r="Y18" s="362"/>
-      <c r="Z18" s="362"/>
-      <c r="AA18" s="362"/>
-      <c r="AB18" s="362"/>
-      <c r="AC18" s="362"/>
-      <c r="AD18" s="362"/>
-      <c r="AE18" s="362"/>
-      <c r="AF18" s="362"/>
-      <c r="AG18" s="362"/>
-      <c r="AH18" s="362"/>
-      <c r="AI18" s="362"/>
-      <c r="AJ18" s="362"/>
-      <c r="AK18" s="362"/>
-      <c r="AL18" s="362"/>
-      <c r="AM18" s="362"/>
-      <c r="AN18" s="362"/>
-      <c r="AO18" s="362"/>
-      <c r="AP18" s="362"/>
+      <c r="A18" s="327"/>
+      <c r="B18" s="325"/>
+      <c r="C18" s="325"/>
+      <c r="D18" s="327"/>
+      <c r="E18" s="327"/>
+      <c r="F18" s="327"/>
+      <c r="G18" s="325"/>
+      <c r="H18" s="325"/>
+      <c r="I18" s="325"/>
+      <c r="J18" s="325"/>
+      <c r="K18" s="325"/>
+      <c r="L18" s="325"/>
+      <c r="M18" s="325"/>
+      <c r="N18" s="325"/>
+      <c r="O18" s="325"/>
+      <c r="P18" s="325"/>
+      <c r="Q18" s="325"/>
+      <c r="R18" s="325"/>
+      <c r="S18" s="325"/>
+      <c r="T18" s="325"/>
+      <c r="U18" s="325"/>
+      <c r="V18" s="325"/>
+      <c r="W18" s="325"/>
+      <c r="X18" s="325"/>
+      <c r="Y18" s="325"/>
+      <c r="Z18" s="325"/>
+      <c r="AA18" s="325"/>
+      <c r="AB18" s="325"/>
+      <c r="AC18" s="325"/>
+      <c r="AD18" s="325"/>
+      <c r="AE18" s="325"/>
+      <c r="AF18" s="325"/>
+      <c r="AG18" s="325"/>
+      <c r="AH18" s="325"/>
+      <c r="AI18" s="325"/>
+      <c r="AJ18" s="325"/>
+      <c r="AK18" s="325"/>
+      <c r="AL18" s="325"/>
+      <c r="AM18" s="325"/>
+      <c r="AN18" s="325"/>
+      <c r="AO18" s="325"/>
+      <c r="AP18" s="325"/>
     </row>
     <row r="19" spans="1:42" ht="84" x14ac:dyDescent="0.2">
-      <c r="A19" s="365"/>
-      <c r="B19" s="362"/>
-      <c r="C19" s="362"/>
-      <c r="D19" s="365"/>
-      <c r="E19" s="365"/>
-      <c r="F19" s="365"/>
-      <c r="G19" s="362"/>
-      <c r="H19" s="362"/>
-      <c r="I19" s="362"/>
-      <c r="J19" s="362"/>
-      <c r="K19" s="362"/>
-      <c r="L19" s="362"/>
-      <c r="M19" s="362"/>
-      <c r="N19" s="362"/>
-      <c r="O19" s="362"/>
-      <c r="P19" s="362"/>
-      <c r="Q19" s="362"/>
-      <c r="R19" s="362"/>
-      <c r="S19" s="362"/>
-      <c r="T19" s="362"/>
-      <c r="U19" s="362"/>
-      <c r="V19" s="362"/>
-      <c r="W19" s="362"/>
-      <c r="X19" s="362"/>
-      <c r="Y19" s="362"/>
-      <c r="Z19" s="362"/>
-      <c r="AA19" s="362"/>
-      <c r="AB19" s="359" t="s">
+      <c r="A19" s="327"/>
+      <c r="B19" s="325"/>
+      <c r="C19" s="325"/>
+      <c r="D19" s="327"/>
+      <c r="E19" s="327"/>
+      <c r="F19" s="327"/>
+      <c r="G19" s="325"/>
+      <c r="H19" s="325"/>
+      <c r="I19" s="325"/>
+      <c r="J19" s="325"/>
+      <c r="K19" s="325"/>
+      <c r="L19" s="325"/>
+      <c r="M19" s="325"/>
+      <c r="N19" s="325"/>
+      <c r="O19" s="325"/>
+      <c r="P19" s="325"/>
+      <c r="Q19" s="325"/>
+      <c r="R19" s="325"/>
+      <c r="S19" s="325"/>
+      <c r="T19" s="325"/>
+      <c r="U19" s="325"/>
+      <c r="V19" s="325"/>
+      <c r="W19" s="325"/>
+      <c r="X19" s="325"/>
+      <c r="Y19" s="325"/>
+      <c r="Z19" s="325"/>
+      <c r="AA19" s="325"/>
+      <c r="AB19" s="322" t="s">
         <v>551</v>
       </c>
       <c r="AC19" s="196" t="s">
         <v>552</v>
       </c>
-      <c r="AD19" s="362"/>
-      <c r="AE19" s="362"/>
-      <c r="AF19" s="362"/>
-      <c r="AG19" s="362"/>
-      <c r="AH19" s="362"/>
-      <c r="AI19" s="362"/>
-      <c r="AJ19" s="362"/>
-      <c r="AK19" s="362"/>
-      <c r="AL19" s="362"/>
-      <c r="AM19" s="362"/>
-      <c r="AN19" s="362"/>
-      <c r="AO19" s="362"/>
-      <c r="AP19" s="362"/>
+      <c r="AD19" s="325"/>
+      <c r="AE19" s="325"/>
+      <c r="AF19" s="325"/>
+      <c r="AG19" s="325"/>
+      <c r="AH19" s="325"/>
+      <c r="AI19" s="325"/>
+      <c r="AJ19" s="325"/>
+      <c r="AK19" s="325"/>
+      <c r="AL19" s="325"/>
+      <c r="AM19" s="325"/>
+      <c r="AN19" s="325"/>
+      <c r="AO19" s="325"/>
+      <c r="AP19" s="325"/>
     </row>
     <row r="20" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A20" s="365"/>
-      <c r="B20" s="362"/>
-      <c r="C20" s="362"/>
-      <c r="D20" s="365"/>
-      <c r="E20" s="365"/>
-      <c r="F20" s="365"/>
-      <c r="G20" s="362"/>
-      <c r="H20" s="362"/>
-      <c r="I20" s="362"/>
-      <c r="J20" s="362"/>
-      <c r="K20" s="362"/>
-      <c r="L20" s="362"/>
-      <c r="M20" s="362"/>
-      <c r="N20" s="362"/>
-      <c r="O20" s="362"/>
-      <c r="P20" s="362"/>
-      <c r="Q20" s="362"/>
-      <c r="R20" s="362"/>
-      <c r="S20" s="362"/>
-      <c r="T20" s="362"/>
-      <c r="U20" s="362"/>
-      <c r="V20" s="362"/>
-      <c r="W20" s="362"/>
-      <c r="X20" s="362"/>
-      <c r="Y20" s="362"/>
-      <c r="Z20" s="362"/>
-      <c r="AA20" s="362"/>
-      <c r="AB20" s="362"/>
-      <c r="AC20" s="362"/>
-      <c r="AD20" s="362"/>
-      <c r="AE20" s="362"/>
-      <c r="AF20" s="362"/>
-      <c r="AG20" s="362"/>
-      <c r="AH20" s="362"/>
-      <c r="AI20" s="362"/>
-      <c r="AJ20" s="362"/>
-      <c r="AK20" s="362"/>
-      <c r="AL20" s="362"/>
-      <c r="AM20" s="362"/>
-      <c r="AN20" s="362"/>
-      <c r="AO20" s="362"/>
-      <c r="AP20" s="362"/>
+      <c r="A20" s="327"/>
+      <c r="B20" s="325"/>
+      <c r="C20" s="325"/>
+      <c r="D20" s="327"/>
+      <c r="E20" s="327"/>
+      <c r="F20" s="327"/>
+      <c r="G20" s="325"/>
+      <c r="H20" s="325"/>
+      <c r="I20" s="325"/>
+      <c r="J20" s="325"/>
+      <c r="K20" s="325"/>
+      <c r="L20" s="325"/>
+      <c r="M20" s="325"/>
+      <c r="N20" s="325"/>
+      <c r="O20" s="325"/>
+      <c r="P20" s="325"/>
+      <c r="Q20" s="325"/>
+      <c r="R20" s="325"/>
+      <c r="S20" s="325"/>
+      <c r="T20" s="325"/>
+      <c r="U20" s="325"/>
+      <c r="V20" s="325"/>
+      <c r="W20" s="325"/>
+      <c r="X20" s="325"/>
+      <c r="Y20" s="325"/>
+      <c r="Z20" s="325"/>
+      <c r="AA20" s="325"/>
+      <c r="AB20" s="325"/>
+      <c r="AC20" s="325"/>
+      <c r="AD20" s="325"/>
+      <c r="AE20" s="325"/>
+      <c r="AF20" s="325"/>
+      <c r="AG20" s="325"/>
+      <c r="AH20" s="325"/>
+      <c r="AI20" s="325"/>
+      <c r="AJ20" s="325"/>
+      <c r="AK20" s="325"/>
+      <c r="AL20" s="325"/>
+      <c r="AM20" s="325"/>
+      <c r="AN20" s="325"/>
+      <c r="AO20" s="325"/>
+      <c r="AP20" s="325"/>
     </row>
     <row r="21" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A21" s="365"/>
-      <c r="B21" s="362"/>
-      <c r="C21" s="362"/>
-      <c r="D21" s="365"/>
-      <c r="E21" s="365"/>
-      <c r="F21" s="365"/>
-      <c r="G21" s="362"/>
-      <c r="H21" s="362"/>
-      <c r="I21" s="362"/>
-      <c r="J21" s="362"/>
-      <c r="K21" s="362"/>
-      <c r="L21" s="362"/>
-      <c r="M21" s="362"/>
-      <c r="N21" s="362"/>
-      <c r="O21" s="362"/>
-      <c r="P21" s="362"/>
-      <c r="Q21" s="362"/>
-      <c r="R21" s="362"/>
-      <c r="S21" s="362"/>
-      <c r="T21" s="362"/>
-      <c r="U21" s="362"/>
-      <c r="V21" s="362"/>
-      <c r="W21" s="362"/>
-      <c r="X21" s="362"/>
-      <c r="Y21" s="362"/>
-      <c r="Z21" s="362"/>
-      <c r="AA21" s="362"/>
-      <c r="AB21" s="362"/>
-      <c r="AC21" s="362"/>
-      <c r="AD21" s="362"/>
-      <c r="AE21" s="362"/>
-      <c r="AF21" s="362"/>
-      <c r="AG21" s="362"/>
-      <c r="AH21" s="362"/>
-      <c r="AI21" s="362"/>
-      <c r="AJ21" s="362"/>
-      <c r="AK21" s="362"/>
-      <c r="AL21" s="362"/>
-      <c r="AM21" s="362"/>
-      <c r="AN21" s="362"/>
-      <c r="AO21" s="362"/>
-      <c r="AP21" s="362"/>
+      <c r="A21" s="327"/>
+      <c r="B21" s="325"/>
+      <c r="C21" s="325"/>
+      <c r="D21" s="327"/>
+      <c r="E21" s="327"/>
+      <c r="F21" s="327"/>
+      <c r="G21" s="325"/>
+      <c r="H21" s="325"/>
+      <c r="I21" s="325"/>
+      <c r="J21" s="325"/>
+      <c r="K21" s="325"/>
+      <c r="L21" s="325"/>
+      <c r="M21" s="325"/>
+      <c r="N21" s="325"/>
+      <c r="O21" s="325"/>
+      <c r="P21" s="325"/>
+      <c r="Q21" s="325"/>
+      <c r="R21" s="325"/>
+      <c r="S21" s="325"/>
+      <c r="T21" s="325"/>
+      <c r="U21" s="325"/>
+      <c r="V21" s="325"/>
+      <c r="W21" s="325"/>
+      <c r="X21" s="325"/>
+      <c r="Y21" s="325"/>
+      <c r="Z21" s="325"/>
+      <c r="AA21" s="325"/>
+      <c r="AB21" s="325"/>
+      <c r="AC21" s="325"/>
+      <c r="AD21" s="325"/>
+      <c r="AE21" s="325"/>
+      <c r="AF21" s="325"/>
+      <c r="AG21" s="325"/>
+      <c r="AH21" s="325"/>
+      <c r="AI21" s="325"/>
+      <c r="AJ21" s="325"/>
+      <c r="AK21" s="325"/>
+      <c r="AL21" s="325"/>
+      <c r="AM21" s="325"/>
+      <c r="AN21" s="325"/>
+      <c r="AO21" s="325"/>
+      <c r="AP21" s="325"/>
     </row>
     <row r="22" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A22" s="365"/>
-      <c r="B22" s="362"/>
-      <c r="C22" s="362"/>
-      <c r="D22" s="365"/>
-      <c r="E22" s="365"/>
-      <c r="F22" s="365"/>
-      <c r="G22" s="362"/>
-      <c r="H22" s="362"/>
-      <c r="I22" s="362"/>
-      <c r="J22" s="362"/>
-      <c r="K22" s="362"/>
-      <c r="L22" s="362"/>
-      <c r="M22" s="362"/>
-      <c r="N22" s="362"/>
-      <c r="O22" s="362"/>
-      <c r="P22" s="362"/>
-      <c r="Q22" s="362"/>
-      <c r="R22" s="362"/>
-      <c r="S22" s="362"/>
-      <c r="T22" s="362"/>
-      <c r="U22" s="362"/>
-      <c r="V22" s="362"/>
-      <c r="W22" s="362"/>
-      <c r="X22" s="362"/>
-      <c r="Y22" s="362"/>
-      <c r="Z22" s="362"/>
-      <c r="AA22" s="362"/>
-      <c r="AB22" s="362"/>
-      <c r="AC22" s="362"/>
-      <c r="AD22" s="362"/>
-      <c r="AE22" s="362"/>
-      <c r="AF22" s="362"/>
-      <c r="AG22" s="362"/>
-      <c r="AH22" s="362"/>
-      <c r="AI22" s="362"/>
-      <c r="AJ22" s="362"/>
-      <c r="AK22" s="362"/>
-      <c r="AL22" s="362"/>
-      <c r="AM22" s="362"/>
-      <c r="AN22" s="362"/>
-      <c r="AO22" s="362"/>
-      <c r="AP22" s="362"/>
+      <c r="A22" s="327"/>
+      <c r="B22" s="325"/>
+      <c r="C22" s="325"/>
+      <c r="D22" s="327"/>
+      <c r="E22" s="327"/>
+      <c r="F22" s="327"/>
+      <c r="G22" s="325"/>
+      <c r="H22" s="325"/>
+      <c r="I22" s="325"/>
+      <c r="J22" s="325"/>
+      <c r="K22" s="325"/>
+      <c r="L22" s="325"/>
+      <c r="M22" s="325"/>
+      <c r="N22" s="325"/>
+      <c r="O22" s="325"/>
+      <c r="P22" s="325"/>
+      <c r="Q22" s="325"/>
+      <c r="R22" s="325"/>
+      <c r="S22" s="325"/>
+      <c r="T22" s="325"/>
+      <c r="U22" s="325"/>
+      <c r="V22" s="325"/>
+      <c r="W22" s="325"/>
+      <c r="X22" s="325"/>
+      <c r="Y22" s="325"/>
+      <c r="Z22" s="325"/>
+      <c r="AA22" s="325"/>
+      <c r="AB22" s="325"/>
+      <c r="AC22" s="325"/>
+      <c r="AD22" s="325"/>
+      <c r="AE22" s="325"/>
+      <c r="AF22" s="325"/>
+      <c r="AG22" s="325"/>
+      <c r="AH22" s="325"/>
+      <c r="AI22" s="325"/>
+      <c r="AJ22" s="325"/>
+      <c r="AK22" s="325"/>
+      <c r="AL22" s="325"/>
+      <c r="AM22" s="325"/>
+      <c r="AN22" s="325"/>
+      <c r="AO22" s="325"/>
+      <c r="AP22" s="325"/>
     </row>
     <row r="23" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A23" s="365"/>
-      <c r="B23" s="362"/>
-      <c r="C23" s="362"/>
-      <c r="D23" s="365"/>
-      <c r="E23" s="365"/>
-      <c r="F23" s="365"/>
-      <c r="G23" s="362"/>
-      <c r="H23" s="362"/>
-      <c r="I23" s="362"/>
-      <c r="J23" s="362"/>
-      <c r="K23" s="362"/>
-      <c r="L23" s="362"/>
-      <c r="M23" s="362"/>
-      <c r="N23" s="362"/>
-      <c r="O23" s="362"/>
-      <c r="P23" s="362"/>
-      <c r="Q23" s="362"/>
-      <c r="R23" s="362"/>
-      <c r="S23" s="362"/>
-      <c r="T23" s="362"/>
-      <c r="U23" s="362"/>
-      <c r="V23" s="362"/>
-      <c r="W23" s="362"/>
-      <c r="X23" s="362"/>
-      <c r="Y23" s="362"/>
-      <c r="Z23" s="362"/>
-      <c r="AA23" s="362"/>
-      <c r="AB23" s="362"/>
-      <c r="AC23" s="362"/>
-      <c r="AD23" s="362"/>
-      <c r="AE23" s="362"/>
-      <c r="AF23" s="362"/>
-      <c r="AG23" s="362"/>
-      <c r="AH23" s="362"/>
-      <c r="AI23" s="362"/>
-      <c r="AJ23" s="362"/>
-      <c r="AK23" s="362"/>
-      <c r="AL23" s="362"/>
-      <c r="AM23" s="362"/>
-      <c r="AN23" s="362"/>
-      <c r="AO23" s="362"/>
-      <c r="AP23" s="362"/>
+      <c r="A23" s="327"/>
+      <c r="B23" s="325"/>
+      <c r="C23" s="325"/>
+      <c r="D23" s="327"/>
+      <c r="E23" s="327"/>
+      <c r="F23" s="327"/>
+      <c r="G23" s="325"/>
+      <c r="H23" s="325"/>
+      <c r="I23" s="325"/>
+      <c r="J23" s="325"/>
+      <c r="K23" s="325"/>
+      <c r="L23" s="325"/>
+      <c r="M23" s="325"/>
+      <c r="N23" s="325"/>
+      <c r="O23" s="325"/>
+      <c r="P23" s="325"/>
+      <c r="Q23" s="325"/>
+      <c r="R23" s="325"/>
+      <c r="S23" s="325"/>
+      <c r="T23" s="325"/>
+      <c r="U23" s="325"/>
+      <c r="V23" s="325"/>
+      <c r="W23" s="325"/>
+      <c r="X23" s="325"/>
+      <c r="Y23" s="325"/>
+      <c r="Z23" s="325"/>
+      <c r="AA23" s="325"/>
+      <c r="AB23" s="325"/>
+      <c r="AC23" s="325"/>
+      <c r="AD23" s="325"/>
+      <c r="AE23" s="325"/>
+      <c r="AF23" s="325"/>
+      <c r="AG23" s="325"/>
+      <c r="AH23" s="325"/>
+      <c r="AI23" s="325"/>
+      <c r="AJ23" s="325"/>
+      <c r="AK23" s="325"/>
+      <c r="AL23" s="325"/>
+      <c r="AM23" s="325"/>
+      <c r="AN23" s="325"/>
+      <c r="AO23" s="325"/>
+      <c r="AP23" s="325"/>
     </row>
     <row r="24" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A24" s="365"/>
-      <c r="B24" s="362"/>
-      <c r="C24" s="362"/>
-      <c r="D24" s="365"/>
-      <c r="E24" s="365"/>
-      <c r="F24" s="365"/>
-      <c r="G24" s="362"/>
-      <c r="H24" s="362"/>
-      <c r="I24" s="362"/>
-      <c r="J24" s="362"/>
-      <c r="K24" s="362"/>
-      <c r="L24" s="362"/>
-      <c r="M24" s="362"/>
-      <c r="N24" s="362"/>
-      <c r="O24" s="362"/>
-      <c r="P24" s="362"/>
-      <c r="Q24" s="362"/>
-      <c r="R24" s="362"/>
-      <c r="S24" s="362"/>
-      <c r="T24" s="362"/>
-      <c r="U24" s="362"/>
-      <c r="V24" s="362"/>
-      <c r="W24" s="362"/>
-      <c r="X24" s="362"/>
-      <c r="Y24" s="362"/>
-      <c r="Z24" s="362"/>
-      <c r="AA24" s="362"/>
-      <c r="AB24" s="362"/>
-      <c r="AC24" s="362"/>
-      <c r="AD24" s="362"/>
-      <c r="AE24" s="362"/>
-      <c r="AF24" s="362"/>
-      <c r="AG24" s="362"/>
-      <c r="AH24" s="362"/>
-      <c r="AI24" s="362"/>
-      <c r="AJ24" s="362"/>
-      <c r="AK24" s="362"/>
-      <c r="AL24" s="362"/>
-      <c r="AM24" s="362"/>
-      <c r="AN24" s="362"/>
-      <c r="AO24" s="362"/>
-      <c r="AP24" s="362"/>
+      <c r="A24" s="327"/>
+      <c r="B24" s="325"/>
+      <c r="C24" s="325"/>
+      <c r="D24" s="327"/>
+      <c r="E24" s="327"/>
+      <c r="F24" s="327"/>
+      <c r="G24" s="325"/>
+      <c r="H24" s="325"/>
+      <c r="I24" s="325"/>
+      <c r="J24" s="325"/>
+      <c r="K24" s="325"/>
+      <c r="L24" s="325"/>
+      <c r="M24" s="325"/>
+      <c r="N24" s="325"/>
+      <c r="O24" s="325"/>
+      <c r="P24" s="325"/>
+      <c r="Q24" s="325"/>
+      <c r="R24" s="325"/>
+      <c r="S24" s="325"/>
+      <c r="T24" s="325"/>
+      <c r="U24" s="325"/>
+      <c r="V24" s="325"/>
+      <c r="W24" s="325"/>
+      <c r="X24" s="325"/>
+      <c r="Y24" s="325"/>
+      <c r="Z24" s="325"/>
+      <c r="AA24" s="325"/>
+      <c r="AB24" s="325"/>
+      <c r="AC24" s="325"/>
+      <c r="AD24" s="325"/>
+      <c r="AE24" s="325"/>
+      <c r="AF24" s="325"/>
+      <c r="AG24" s="325"/>
+      <c r="AH24" s="325"/>
+      <c r="AI24" s="325"/>
+      <c r="AJ24" s="325"/>
+      <c r="AK24" s="325"/>
+      <c r="AL24" s="325"/>
+      <c r="AM24" s="325"/>
+      <c r="AN24" s="325"/>
+      <c r="AO24" s="325"/>
+      <c r="AP24" s="325"/>
     </row>
     <row r="25" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A25" s="365"/>
-      <c r="B25" s="362"/>
-      <c r="C25" s="362"/>
-      <c r="D25" s="365"/>
-      <c r="E25" s="365"/>
-      <c r="F25" s="365"/>
-      <c r="G25" s="362"/>
-      <c r="H25" s="362"/>
-      <c r="I25" s="362"/>
-      <c r="J25" s="362"/>
-      <c r="K25" s="362"/>
-      <c r="L25" s="362"/>
-      <c r="M25" s="362"/>
-      <c r="N25" s="362"/>
-      <c r="O25" s="362"/>
-      <c r="P25" s="362"/>
-      <c r="Q25" s="362"/>
-      <c r="R25" s="362"/>
-      <c r="S25" s="362"/>
-      <c r="T25" s="362"/>
-      <c r="U25" s="362"/>
-      <c r="V25" s="362"/>
-      <c r="W25" s="362"/>
-      <c r="X25" s="362"/>
-      <c r="Y25" s="362"/>
-      <c r="Z25" s="362"/>
-      <c r="AA25" s="362"/>
-      <c r="AB25" s="362"/>
-      <c r="AC25" s="362"/>
-      <c r="AD25" s="362"/>
-      <c r="AE25" s="362"/>
-      <c r="AF25" s="362"/>
-      <c r="AG25" s="362"/>
-      <c r="AH25" s="362"/>
-      <c r="AI25" s="362"/>
-      <c r="AJ25" s="362"/>
-      <c r="AK25" s="362"/>
-      <c r="AL25" s="362"/>
-      <c r="AM25" s="362"/>
-      <c r="AN25" s="362"/>
-      <c r="AO25" s="362"/>
-      <c r="AP25" s="362"/>
+      <c r="A25" s="327"/>
+      <c r="B25" s="325"/>
+      <c r="C25" s="325"/>
+      <c r="D25" s="327"/>
+      <c r="E25" s="327"/>
+      <c r="F25" s="327"/>
+      <c r="G25" s="325"/>
+      <c r="H25" s="325"/>
+      <c r="I25" s="325"/>
+      <c r="J25" s="325"/>
+      <c r="K25" s="325"/>
+      <c r="L25" s="325"/>
+      <c r="M25" s="325"/>
+      <c r="N25" s="325"/>
+      <c r="O25" s="325"/>
+      <c r="P25" s="325"/>
+      <c r="Q25" s="325"/>
+      <c r="R25" s="325"/>
+      <c r="S25" s="325"/>
+      <c r="T25" s="325"/>
+      <c r="U25" s="325"/>
+      <c r="V25" s="325"/>
+      <c r="W25" s="325"/>
+      <c r="X25" s="325"/>
+      <c r="Y25" s="325"/>
+      <c r="Z25" s="325"/>
+      <c r="AA25" s="325"/>
+      <c r="AB25" s="325"/>
+      <c r="AC25" s="325"/>
+      <c r="AD25" s="325"/>
+      <c r="AE25" s="325"/>
+      <c r="AF25" s="325"/>
+      <c r="AG25" s="325"/>
+      <c r="AH25" s="325"/>
+      <c r="AI25" s="325"/>
+      <c r="AJ25" s="325"/>
+      <c r="AK25" s="325"/>
+      <c r="AL25" s="325"/>
+      <c r="AM25" s="325"/>
+      <c r="AN25" s="325"/>
+      <c r="AO25" s="325"/>
+      <c r="AP25" s="325"/>
     </row>
     <row r="26" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A26" s="365"/>
-      <c r="B26" s="362"/>
-      <c r="C26" s="362"/>
-      <c r="D26" s="365"/>
-      <c r="E26" s="365"/>
-      <c r="F26" s="365"/>
-      <c r="G26" s="362"/>
-      <c r="H26" s="362"/>
-      <c r="I26" s="362"/>
-      <c r="J26" s="362"/>
-      <c r="K26" s="362"/>
-      <c r="L26" s="362"/>
-      <c r="M26" s="362"/>
-      <c r="N26" s="362"/>
-      <c r="O26" s="362"/>
-      <c r="P26" s="362"/>
-      <c r="Q26" s="362"/>
-      <c r="R26" s="362"/>
-      <c r="S26" s="362"/>
-      <c r="T26" s="362"/>
-      <c r="U26" s="362"/>
-      <c r="V26" s="362"/>
-      <c r="W26" s="362"/>
-      <c r="X26" s="362"/>
-      <c r="Y26" s="362"/>
-      <c r="Z26" s="362"/>
-      <c r="AA26" s="362"/>
-      <c r="AB26" s="362"/>
-      <c r="AC26" s="362"/>
-      <c r="AD26" s="362"/>
-      <c r="AE26" s="362"/>
-      <c r="AF26" s="362"/>
-      <c r="AG26" s="362"/>
-      <c r="AH26" s="362"/>
-      <c r="AI26" s="362"/>
-      <c r="AJ26" s="362"/>
-      <c r="AK26" s="362"/>
-      <c r="AL26" s="362"/>
-      <c r="AM26" s="362"/>
-      <c r="AN26" s="362"/>
-      <c r="AO26" s="362"/>
-      <c r="AP26" s="362"/>
+      <c r="A26" s="327"/>
+      <c r="B26" s="325"/>
+      <c r="C26" s="325"/>
+      <c r="D26" s="327"/>
+      <c r="E26" s="327"/>
+      <c r="F26" s="327"/>
+      <c r="G26" s="325"/>
+      <c r="H26" s="325"/>
+      <c r="I26" s="325"/>
+      <c r="J26" s="325"/>
+      <c r="K26" s="325"/>
+      <c r="L26" s="325"/>
+      <c r="M26" s="325"/>
+      <c r="N26" s="325"/>
+      <c r="O26" s="325"/>
+      <c r="P26" s="325"/>
+      <c r="Q26" s="325"/>
+      <c r="R26" s="325"/>
+      <c r="S26" s="325"/>
+      <c r="T26" s="325"/>
+      <c r="U26" s="325"/>
+      <c r="V26" s="325"/>
+      <c r="W26" s="325"/>
+      <c r="X26" s="325"/>
+      <c r="Y26" s="325"/>
+      <c r="Z26" s="325"/>
+      <c r="AA26" s="325"/>
+      <c r="AB26" s="325"/>
+      <c r="AC26" s="325"/>
+      <c r="AD26" s="325"/>
+      <c r="AE26" s="325"/>
+      <c r="AF26" s="325"/>
+      <c r="AG26" s="325"/>
+      <c r="AH26" s="325"/>
+      <c r="AI26" s="325"/>
+      <c r="AJ26" s="325"/>
+      <c r="AK26" s="325"/>
+      <c r="AL26" s="325"/>
+      <c r="AM26" s="325"/>
+      <c r="AN26" s="325"/>
+      <c r="AO26" s="325"/>
+      <c r="AP26" s="325"/>
     </row>
     <row r="27" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A27" s="365"/>
-      <c r="B27" s="362"/>
-      <c r="C27" s="362"/>
-      <c r="D27" s="365"/>
-      <c r="E27" s="365"/>
-      <c r="F27" s="365"/>
-      <c r="G27" s="362"/>
-      <c r="H27" s="362"/>
-      <c r="I27" s="362"/>
-      <c r="J27" s="362"/>
-      <c r="K27" s="362"/>
-      <c r="L27" s="362"/>
-      <c r="M27" s="362"/>
-      <c r="N27" s="362"/>
-      <c r="O27" s="362"/>
-      <c r="P27" s="362"/>
-      <c r="Q27" s="362"/>
-      <c r="R27" s="362"/>
-      <c r="S27" s="362"/>
-      <c r="T27" s="362"/>
-      <c r="U27" s="362"/>
-      <c r="V27" s="362"/>
-      <c r="W27" s="362"/>
-      <c r="X27" s="362"/>
-      <c r="Y27" s="362"/>
-      <c r="Z27" s="362"/>
-      <c r="AA27" s="362"/>
-      <c r="AB27" s="362"/>
-      <c r="AC27" s="362"/>
-      <c r="AD27" s="362"/>
-      <c r="AE27" s="362"/>
-      <c r="AF27" s="362"/>
-      <c r="AG27" s="362"/>
-      <c r="AH27" s="362"/>
-      <c r="AI27" s="362"/>
-      <c r="AJ27" s="362"/>
-      <c r="AK27" s="362"/>
-      <c r="AL27" s="362"/>
-      <c r="AM27" s="362"/>
-      <c r="AN27" s="362"/>
-      <c r="AO27" s="362"/>
-      <c r="AP27" s="362"/>
+      <c r="A27" s="327"/>
+      <c r="B27" s="325"/>
+      <c r="C27" s="325"/>
+      <c r="D27" s="327"/>
+      <c r="E27" s="327"/>
+      <c r="F27" s="327"/>
+      <c r="G27" s="325"/>
+      <c r="H27" s="325"/>
+      <c r="I27" s="325"/>
+      <c r="J27" s="325"/>
+      <c r="K27" s="325"/>
+      <c r="L27" s="325"/>
+      <c r="M27" s="325"/>
+      <c r="N27" s="325"/>
+      <c r="O27" s="325"/>
+      <c r="P27" s="325"/>
+      <c r="Q27" s="325"/>
+      <c r="R27" s="325"/>
+      <c r="S27" s="325"/>
+      <c r="T27" s="325"/>
+      <c r="U27" s="325"/>
+      <c r="V27" s="325"/>
+      <c r="W27" s="325"/>
+      <c r="X27" s="325"/>
+      <c r="Y27" s="325"/>
+      <c r="Z27" s="325"/>
+      <c r="AA27" s="325"/>
+      <c r="AB27" s="325"/>
+      <c r="AC27" s="325"/>
+      <c r="AD27" s="325"/>
+      <c r="AE27" s="325"/>
+      <c r="AF27" s="325"/>
+      <c r="AG27" s="325"/>
+      <c r="AH27" s="325"/>
+      <c r="AI27" s="325"/>
+      <c r="AJ27" s="325"/>
+      <c r="AK27" s="325"/>
+      <c r="AL27" s="325"/>
+      <c r="AM27" s="325"/>
+      <c r="AN27" s="325"/>
+      <c r="AO27" s="325"/>
+      <c r="AP27" s="325"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -16974,14 +16979,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="352" t="s">
+      <c r="A1" s="367" t="s">
         <v>373</v>
       </c>
-      <c r="B1" s="352"/>
-      <c r="C1" s="352"/>
-      <c r="D1" s="352"/>
-      <c r="E1" s="352"/>
-      <c r="F1" s="352"/>
+      <c r="B1" s="367"/>
+      <c r="C1" s="367"/>
+      <c r="D1" s="367"/>
+      <c r="E1" s="367"/>
+      <c r="F1" s="367"/>
       <c r="G1" s="218"/>
       <c r="H1" s="218"/>
       <c r="I1" s="218"/>
@@ -17031,7 +17036,7 @@
       <c r="O2" s="221" t="s">
         <v>323</v>
       </c>
-      <c r="P2" s="353" t="s">
+      <c r="P2" s="368" t="s">
         <v>372</v>
       </c>
       <c r="Q2" s="221" t="s">
@@ -17043,7 +17048,7 @@
       <c r="S2" s="221" t="s">
         <v>371</v>
       </c>
-      <c r="T2" s="353" t="s">
+      <c r="T2" s="368" t="s">
         <v>370</v>
       </c>
     </row>
@@ -17081,7 +17086,7 @@
       <c r="O3" s="221" t="s">
         <v>352</v>
       </c>
-      <c r="P3" s="353"/>
+      <c r="P3" s="368"/>
       <c r="Q3" s="221" t="s">
         <v>351</v>
       </c>
@@ -17091,7 +17096,7 @@
       <c r="S3" s="221" t="s">
         <v>281</v>
       </c>
-      <c r="T3" s="353"/>
+      <c r="T3" s="368"/>
     </row>
     <row r="4" spans="1:20" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="220"/>
@@ -17137,7 +17142,7 @@
       <c r="O4" s="221" t="s">
         <v>333</v>
       </c>
-      <c r="P4" s="353"/>
+      <c r="P4" s="368"/>
       <c r="Q4" s="221" t="s">
         <v>332</v>
       </c>
@@ -17147,7 +17152,7 @@
       <c r="S4" s="221" t="s">
         <v>228</v>
       </c>
-      <c r="T4" s="353"/>
+      <c r="T4" s="368"/>
     </row>
     <row r="5" spans="1:20" ht="317" x14ac:dyDescent="0.2">
       <c r="A5" s="224" t="s">
@@ -17704,8 +17709,8 @@
       <c r="N19" s="4"/>
       <c r="O19" s="4"/>
       <c r="P19" s="4"/>
-      <c r="Q19" s="362"/>
-      <c r="R19" s="359" t="s">
+      <c r="Q19" s="325"/>
+      <c r="R19" s="322" t="s">
         <v>551</v>
       </c>
       <c r="S19" s="196" t="s">
@@ -17733,16 +17738,16 @@
   <sheetData>
     <row r="1" spans="1:28" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="244"/>
-      <c r="B1" s="355" t="s">
+      <c r="B1" s="370" t="s">
         <v>329</v>
       </c>
-      <c r="C1" s="355"/>
-      <c r="D1" s="355"/>
-      <c r="E1" s="355"/>
-      <c r="F1" s="355"/>
-      <c r="G1" s="355"/>
-      <c r="H1" s="355"/>
-      <c r="I1" s="355"/>
+      <c r="C1" s="370"/>
+      <c r="D1" s="370"/>
+      <c r="E1" s="370"/>
+      <c r="F1" s="370"/>
+      <c r="G1" s="370"/>
+      <c r="H1" s="370"/>
+      <c r="I1" s="370"/>
       <c r="J1" s="241"/>
       <c r="K1" s="241"/>
       <c r="L1" s="241"/>
@@ -17773,7 +17778,7 @@
       <c r="G2" s="243" t="s">
         <v>328</v>
       </c>
-      <c r="H2" s="354" t="s">
+      <c r="H2" s="369" t="s">
         <v>327</v>
       </c>
       <c r="I2" s="246" t="s">
@@ -17818,7 +17823,7 @@
       <c r="V2" s="246" t="s">
         <v>326</v>
       </c>
-      <c r="W2" s="354" t="s">
+      <c r="W2" s="369" t="s">
         <v>325</v>
       </c>
       <c r="X2" s="243" t="s">
@@ -17833,7 +17838,7 @@
       <c r="AA2" s="243" t="s">
         <v>144</v>
       </c>
-      <c r="AB2" s="354" t="s">
+      <c r="AB2" s="369" t="s">
         <v>324</v>
       </c>
     </row>
@@ -17847,7 +17852,7 @@
       <c r="G3" s="243" t="s">
         <v>317</v>
       </c>
-      <c r="H3" s="354"/>
+      <c r="H3" s="369"/>
       <c r="I3" s="246" t="s">
         <v>316</v>
       </c>
@@ -17888,7 +17893,7 @@
       <c r="V3" s="246" t="s">
         <v>304</v>
       </c>
-      <c r="W3" s="354"/>
+      <c r="W3" s="369"/>
       <c r="X3" s="245"/>
       <c r="Y3" s="243" t="s">
         <v>303</v>
@@ -17899,7 +17904,7 @@
       <c r="AA3" s="243" t="s">
         <v>301</v>
       </c>
-      <c r="AB3" s="354"/>
+      <c r="AB3" s="369"/>
     </row>
     <row r="4" spans="1:28" ht="98" x14ac:dyDescent="0.2">
       <c r="A4" s="247"/>
@@ -17921,7 +17926,7 @@
       <c r="G4" s="243" t="s">
         <v>267</v>
       </c>
-      <c r="H4" s="354"/>
+      <c r="H4" s="369"/>
       <c r="I4" s="246" t="s">
         <v>266</v>
       </c>
@@ -17964,7 +17969,7 @@
       <c r="V4" s="249" t="s">
         <v>253</v>
       </c>
-      <c r="W4" s="354"/>
+      <c r="W4" s="369"/>
       <c r="X4" s="250" t="s">
         <v>252</v>
       </c>
@@ -17977,7 +17982,7 @@
       <c r="AA4" s="250" t="s">
         <v>249</v>
       </c>
-      <c r="AB4" s="354"/>
+      <c r="AB4" s="369"/>
     </row>
     <row r="5" spans="1:28" ht="196" x14ac:dyDescent="0.2">
       <c r="A5" s="251" t="s">
@@ -18754,102 +18759,102 @@
       </c>
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A17" s="366"/>
-      <c r="B17" s="366"/>
-      <c r="C17" s="366"/>
-      <c r="D17" s="366"/>
-      <c r="E17" s="366"/>
-      <c r="F17" s="366"/>
-      <c r="G17" s="367"/>
-      <c r="H17" s="367"/>
-      <c r="I17" s="367"/>
-      <c r="J17" s="367"/>
-      <c r="K17" s="367"/>
-      <c r="L17" s="367"/>
-      <c r="M17" s="367"/>
-      <c r="N17" s="367"/>
-      <c r="O17" s="367"/>
-      <c r="P17" s="367"/>
-      <c r="Q17" s="367"/>
-      <c r="R17" s="367"/>
-      <c r="S17" s="367"/>
-      <c r="T17" s="367"/>
-      <c r="U17" s="367"/>
-      <c r="V17" s="367"/>
-      <c r="W17" s="367"/>
-      <c r="X17" s="367"/>
-      <c r="Y17" s="367"/>
-      <c r="Z17" s="367"/>
-      <c r="AA17" s="367"/>
-      <c r="AB17" s="367"/>
+      <c r="A17" s="328"/>
+      <c r="B17" s="328"/>
+      <c r="C17" s="328"/>
+      <c r="D17" s="328"/>
+      <c r="E17" s="328"/>
+      <c r="F17" s="328"/>
+      <c r="G17" s="329"/>
+      <c r="H17" s="329"/>
+      <c r="I17" s="329"/>
+      <c r="J17" s="329"/>
+      <c r="K17" s="329"/>
+      <c r="L17" s="329"/>
+      <c r="M17" s="329"/>
+      <c r="N17" s="329"/>
+      <c r="O17" s="329"/>
+      <c r="P17" s="329"/>
+      <c r="Q17" s="329"/>
+      <c r="R17" s="329"/>
+      <c r="S17" s="329"/>
+      <c r="T17" s="329"/>
+      <c r="U17" s="329"/>
+      <c r="V17" s="329"/>
+      <c r="W17" s="329"/>
+      <c r="X17" s="329"/>
+      <c r="Y17" s="329"/>
+      <c r="Z17" s="329"/>
+      <c r="AA17" s="329"/>
+      <c r="AB17" s="329"/>
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A18" s="366"/>
-      <c r="B18" s="366"/>
-      <c r="C18" s="366"/>
-      <c r="D18" s="366"/>
-      <c r="E18" s="366"/>
-      <c r="F18" s="366"/>
-      <c r="G18" s="367"/>
-      <c r="H18" s="367"/>
-      <c r="I18" s="367"/>
-      <c r="J18" s="367"/>
-      <c r="K18" s="367"/>
-      <c r="L18" s="367"/>
-      <c r="M18" s="367"/>
-      <c r="N18" s="367"/>
-      <c r="O18" s="367"/>
-      <c r="P18" s="367"/>
-      <c r="Q18" s="367"/>
-      <c r="R18" s="367"/>
-      <c r="S18" s="367"/>
-      <c r="T18" s="367"/>
-      <c r="U18" s="367"/>
-      <c r="V18" s="367"/>
-      <c r="W18" s="367"/>
-      <c r="X18" s="367"/>
-      <c r="Y18" s="367"/>
-      <c r="Z18" s="367"/>
-      <c r="AA18" s="367"/>
-      <c r="AB18" s="367"/>
+      <c r="A18" s="328"/>
+      <c r="B18" s="328"/>
+      <c r="C18" s="328"/>
+      <c r="D18" s="328"/>
+      <c r="E18" s="328"/>
+      <c r="F18" s="328"/>
+      <c r="G18" s="329"/>
+      <c r="H18" s="329"/>
+      <c r="I18" s="329"/>
+      <c r="J18" s="329"/>
+      <c r="K18" s="329"/>
+      <c r="L18" s="329"/>
+      <c r="M18" s="329"/>
+      <c r="N18" s="329"/>
+      <c r="O18" s="329"/>
+      <c r="P18" s="329"/>
+      <c r="Q18" s="329"/>
+      <c r="R18" s="329"/>
+      <c r="S18" s="329"/>
+      <c r="T18" s="329"/>
+      <c r="U18" s="329"/>
+      <c r="V18" s="329"/>
+      <c r="W18" s="329"/>
+      <c r="X18" s="329"/>
+      <c r="Y18" s="329"/>
+      <c r="Z18" s="329"/>
+      <c r="AA18" s="329"/>
+      <c r="AB18" s="329"/>
     </row>
     <row r="19" spans="1:28" ht="210" x14ac:dyDescent="0.2">
-      <c r="A19" s="366"/>
-      <c r="B19" s="366"/>
-      <c r="C19" s="366"/>
-      <c r="D19" s="366"/>
-      <c r="E19" s="366"/>
-      <c r="F19" s="360" t="s">
+      <c r="A19" s="328"/>
+      <c r="B19" s="328"/>
+      <c r="C19" s="328"/>
+      <c r="D19" s="328"/>
+      <c r="E19" s="328"/>
+      <c r="F19" s="323" t="s">
         <v>553</v>
       </c>
       <c r="G19" s="254" t="s">
         <v>554</v>
       </c>
-      <c r="H19" s="367"/>
-      <c r="I19" s="367"/>
-      <c r="J19" s="367"/>
-      <c r="K19" s="367"/>
-      <c r="L19" s="367"/>
-      <c r="M19" s="367"/>
-      <c r="N19" s="367"/>
-      <c r="O19" s="367"/>
-      <c r="P19" s="367"/>
-      <c r="Q19" s="367"/>
-      <c r="R19" s="367"/>
-      <c r="S19" s="367"/>
-      <c r="T19" s="367"/>
-      <c r="U19" s="361" t="s">
+      <c r="H19" s="329"/>
+      <c r="I19" s="329"/>
+      <c r="J19" s="329"/>
+      <c r="K19" s="329"/>
+      <c r="L19" s="329"/>
+      <c r="M19" s="329"/>
+      <c r="N19" s="329"/>
+      <c r="O19" s="329"/>
+      <c r="P19" s="329"/>
+      <c r="Q19" s="329"/>
+      <c r="R19" s="329"/>
+      <c r="S19" s="329"/>
+      <c r="T19" s="329"/>
+      <c r="U19" s="324" t="s">
         <v>555</v>
       </c>
       <c r="V19" s="254" t="s">
         <v>556</v>
       </c>
-      <c r="W19" s="367"/>
-      <c r="X19" s="367"/>
-      <c r="Y19" s="367"/>
-      <c r="Z19" s="367"/>
-      <c r="AA19" s="367"/>
-      <c r="AB19" s="367"/>
+      <c r="W19" s="329"/>
+      <c r="X19" s="329"/>
+      <c r="Y19" s="329"/>
+      <c r="Z19" s="329"/>
+      <c r="AA19" s="329"/>
+      <c r="AB19" s="329"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -18871,16 +18876,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="357" t="s">
+      <c r="A1" s="372" t="s">
         <v>373</v>
       </c>
-      <c r="B1" s="357"/>
-      <c r="C1" s="357"/>
-      <c r="D1" s="357"/>
-      <c r="E1" s="357"/>
-      <c r="F1" s="357"/>
-      <c r="G1" s="357"/>
-      <c r="H1" s="357"/>
+      <c r="B1" s="372"/>
+      <c r="C1" s="372"/>
+      <c r="D1" s="372"/>
+      <c r="E1" s="372"/>
+      <c r="F1" s="372"/>
+      <c r="G1" s="372"/>
+      <c r="H1" s="372"/>
       <c r="I1" s="291"/>
       <c r="J1" s="291"/>
       <c r="K1" s="291"/>
@@ -18905,7 +18910,7 @@
       <c r="G2" s="293" t="s">
         <v>328</v>
       </c>
-      <c r="H2" s="356" t="s">
+      <c r="H2" s="371" t="s">
         <v>327</v>
       </c>
       <c r="I2" s="293" t="s">
@@ -18938,13 +18943,13 @@
       <c r="R2" s="293" t="s">
         <v>326</v>
       </c>
-      <c r="S2" s="356" t="s">
+      <c r="S2" s="371" t="s">
         <v>325</v>
       </c>
       <c r="T2" s="293" t="s">
         <v>144</v>
       </c>
-      <c r="U2" s="356" t="s">
+      <c r="U2" s="371" t="s">
         <v>324</v>
       </c>
     </row>
@@ -18958,7 +18963,7 @@
       <c r="G3" s="293" t="s">
         <v>317</v>
       </c>
-      <c r="H3" s="356"/>
+      <c r="H3" s="371"/>
       <c r="I3" s="293" t="s">
         <v>369</v>
       </c>
@@ -18989,11 +18994,11 @@
       <c r="R3" s="293" t="s">
         <v>304</v>
       </c>
-      <c r="S3" s="356"/>
+      <c r="S3" s="371"/>
       <c r="T3" s="293" t="s">
         <v>301</v>
       </c>
-      <c r="U3" s="356"/>
+      <c r="U3" s="371"/>
     </row>
     <row r="4" spans="1:21" ht="112" x14ac:dyDescent="0.2">
       <c r="A4" s="290"/>
@@ -19015,7 +19020,7 @@
       <c r="G4" s="293" t="s">
         <v>267</v>
       </c>
-      <c r="H4" s="356"/>
+      <c r="H4" s="371"/>
       <c r="I4" s="293" t="s">
         <v>350</v>
       </c>
@@ -19046,11 +19051,11 @@
       <c r="R4" s="293" t="s">
         <v>253</v>
       </c>
-      <c r="S4" s="356"/>
+      <c r="S4" s="371"/>
       <c r="T4" s="293" t="s">
         <v>249</v>
       </c>
-      <c r="U4" s="356"/>
+      <c r="U4" s="371"/>
     </row>
     <row r="5" spans="1:21" ht="196" x14ac:dyDescent="0.2">
       <c r="A5" s="296" t="s">
@@ -19609,81 +19614,81 @@
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A17" s="368"/>
-      <c r="B17" s="368"/>
-      <c r="C17" s="368"/>
-      <c r="D17" s="368"/>
-      <c r="E17" s="368"/>
-      <c r="F17" s="368"/>
-      <c r="G17" s="368"/>
-      <c r="H17" s="368"/>
-      <c r="I17" s="368"/>
-      <c r="J17" s="368"/>
-      <c r="K17" s="368"/>
-      <c r="L17" s="368"/>
-      <c r="M17" s="368"/>
-      <c r="N17" s="368"/>
-      <c r="O17" s="368"/>
-      <c r="P17" s="368"/>
-      <c r="Q17" s="368"/>
-      <c r="R17" s="368"/>
-      <c r="S17" s="369"/>
-      <c r="T17" s="368"/>
-      <c r="U17" s="368"/>
+      <c r="A17" s="330"/>
+      <c r="B17" s="330"/>
+      <c r="C17" s="330"/>
+      <c r="D17" s="330"/>
+      <c r="E17" s="330"/>
+      <c r="F17" s="330"/>
+      <c r="G17" s="330"/>
+      <c r="H17" s="330"/>
+      <c r="I17" s="330"/>
+      <c r="J17" s="330"/>
+      <c r="K17" s="330"/>
+      <c r="L17" s="330"/>
+      <c r="M17" s="330"/>
+      <c r="N17" s="330"/>
+      <c r="O17" s="330"/>
+      <c r="P17" s="330"/>
+      <c r="Q17" s="330"/>
+      <c r="R17" s="330"/>
+      <c r="S17" s="331"/>
+      <c r="T17" s="330"/>
+      <c r="U17" s="330"/>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A18" s="368"/>
-      <c r="B18" s="368"/>
-      <c r="C18" s="368"/>
-      <c r="D18" s="368"/>
-      <c r="E18" s="368"/>
-      <c r="F18" s="368"/>
-      <c r="G18" s="368"/>
-      <c r="H18" s="368"/>
-      <c r="I18" s="368"/>
-      <c r="J18" s="368"/>
-      <c r="K18" s="368"/>
-      <c r="L18" s="368"/>
-      <c r="M18" s="368"/>
-      <c r="N18" s="368"/>
-      <c r="O18" s="368"/>
-      <c r="P18" s="368"/>
-      <c r="Q18" s="368"/>
-      <c r="R18" s="368"/>
-      <c r="S18" s="370"/>
-      <c r="T18" s="368"/>
-      <c r="U18" s="368"/>
+      <c r="A18" s="330"/>
+      <c r="B18" s="330"/>
+      <c r="C18" s="330"/>
+      <c r="D18" s="330"/>
+      <c r="E18" s="330"/>
+      <c r="F18" s="330"/>
+      <c r="G18" s="330"/>
+      <c r="H18" s="330"/>
+      <c r="I18" s="330"/>
+      <c r="J18" s="330"/>
+      <c r="K18" s="330"/>
+      <c r="L18" s="330"/>
+      <c r="M18" s="330"/>
+      <c r="N18" s="330"/>
+      <c r="O18" s="330"/>
+      <c r="P18" s="330"/>
+      <c r="Q18" s="330"/>
+      <c r="R18" s="330"/>
+      <c r="S18" s="332"/>
+      <c r="T18" s="330"/>
+      <c r="U18" s="330"/>
     </row>
     <row r="19" spans="1:21" ht="210" x14ac:dyDescent="0.2">
-      <c r="A19" s="371"/>
-      <c r="B19" s="371"/>
-      <c r="C19" s="371"/>
-      <c r="D19" s="372"/>
-      <c r="E19" s="371"/>
-      <c r="F19" s="360" t="s">
+      <c r="A19" s="333"/>
+      <c r="B19" s="333"/>
+      <c r="C19" s="333"/>
+      <c r="D19" s="334"/>
+      <c r="E19" s="333"/>
+      <c r="F19" s="323" t="s">
         <v>553</v>
       </c>
       <c r="G19" s="254" t="s">
         <v>554</v>
       </c>
-      <c r="H19" s="371"/>
-      <c r="I19" s="371"/>
-      <c r="J19" s="371"/>
-      <c r="K19" s="371"/>
-      <c r="L19" s="371"/>
-      <c r="M19" s="371"/>
-      <c r="N19" s="371"/>
-      <c r="O19" s="371"/>
-      <c r="P19" s="371"/>
-      <c r="Q19" s="361" t="s">
+      <c r="H19" s="333"/>
+      <c r="I19" s="333"/>
+      <c r="J19" s="333"/>
+      <c r="K19" s="333"/>
+      <c r="L19" s="333"/>
+      <c r="M19" s="333"/>
+      <c r="N19" s="333"/>
+      <c r="O19" s="333"/>
+      <c r="P19" s="333"/>
+      <c r="Q19" s="324" t="s">
         <v>555</v>
       </c>
       <c r="R19" s="254" t="s">
         <v>556</v>
       </c>
-      <c r="S19" s="371"/>
-      <c r="T19" s="371"/>
-      <c r="U19" s="371"/>
+      <c r="S19" s="333"/>
+      <c r="T19" s="333"/>
+      <c r="U19" s="333"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -19715,9 +19720,9 @@
       <c r="A1" s="269"/>
       <c r="C1" s="271"/>
       <c r="E1" s="269"/>
-      <c r="F1" s="373"/>
+      <c r="F1" s="335"/>
       <c r="G1" s="271"/>
-      <c r="H1" s="373"/>
+      <c r="H1" s="335"/>
       <c r="I1" s="271" t="s">
         <v>375</v>
       </c>
@@ -19741,13 +19746,13 @@
       <c r="K2" s="221" t="s">
         <v>326</v>
       </c>
-      <c r="L2" s="353" t="s">
+      <c r="L2" s="368" t="s">
         <v>325</v>
       </c>
       <c r="M2" s="221" t="s">
         <v>144</v>
       </c>
-      <c r="N2" s="353" t="s">
+      <c r="N2" s="368" t="s">
         <v>324</v>
       </c>
     </row>
@@ -19765,11 +19770,11 @@
       <c r="K3" s="221" t="s">
         <v>304</v>
       </c>
-      <c r="L3" s="353"/>
+      <c r="L3" s="368"/>
       <c r="M3" s="221" t="s">
         <v>301</v>
       </c>
-      <c r="N3" s="353"/>
+      <c r="N3" s="368"/>
     </row>
     <row r="4" spans="1:14" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="274"/>
@@ -19795,11 +19800,11 @@
       <c r="K4" s="221" t="s">
         <v>253</v>
       </c>
-      <c r="L4" s="353"/>
+      <c r="L4" s="368"/>
       <c r="M4" s="221" t="s">
         <v>249</v>
       </c>
-      <c r="N4" s="353"/>
+      <c r="N4" s="368"/>
     </row>
     <row r="5" spans="1:14" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="276"/>
@@ -20092,28 +20097,28 @@
       </c>
     </row>
     <row r="15" spans="1:14" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E15" s="373"/>
-      <c r="F15" s="373"/>
-      <c r="G15" s="373"/>
-      <c r="H15" s="373"/>
-      <c r="I15" s="373"/>
-      <c r="J15" s="373"/>
-      <c r="K15" s="373"/>
-      <c r="L15" s="373"/>
-      <c r="M15" s="373"/>
-      <c r="N15" s="373"/>
+      <c r="E15" s="335"/>
+      <c r="F15" s="335"/>
+      <c r="G15" s="335"/>
+      <c r="H15" s="335"/>
+      <c r="I15" s="335"/>
+      <c r="J15" s="335"/>
+      <c r="K15" s="335"/>
+      <c r="L15" s="335"/>
+      <c r="M15" s="335"/>
+      <c r="N15" s="335"/>
     </row>
     <row r="16" spans="1:14" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E16" s="373"/>
-      <c r="F16" s="373"/>
-      <c r="G16" s="373"/>
-      <c r="H16" s="373"/>
-      <c r="I16" s="373"/>
-      <c r="J16" s="373"/>
-      <c r="K16" s="373"/>
-      <c r="L16" s="373"/>
-      <c r="M16" s="373"/>
-      <c r="N16" s="373"/>
+      <c r="E16" s="335"/>
+      <c r="F16" s="335"/>
+      <c r="G16" s="335"/>
+      <c r="H16" s="335"/>
+      <c r="I16" s="335"/>
+      <c r="J16" s="335"/>
+      <c r="K16" s="335"/>
+      <c r="L16" s="335"/>
+      <c r="M16" s="335"/>
+      <c r="N16" s="335"/>
     </row>
     <row r="17" spans="4:4" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D17" s="289"/>
@@ -20480,14 +20485,14 @@
       <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="FA1" s="340" t="s">
+      <c r="FA1" s="355" t="s">
         <v>382</v>
       </c>
-      <c r="FB1" s="340"/>
-      <c r="FC1" s="340"/>
-      <c r="FD1" s="340"/>
-      <c r="FE1" s="340"/>
-      <c r="FF1" s="340"/>
+      <c r="FB1" s="355"/>
+      <c r="FC1" s="355"/>
+      <c r="FD1" s="355"/>
+      <c r="FE1" s="355"/>
+      <c r="FF1" s="355"/>
       <c r="FG1" s="8" t="s">
         <v>0</v>
       </c>
@@ -20625,28 +20630,28 @@
       <c r="D4" s="312"/>
       <c r="E4" s="312"/>
       <c r="F4" s="312"/>
-      <c r="G4" s="341" t="s">
+      <c r="G4" s="356" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="342"/>
-      <c r="I4" s="342"/>
-      <c r="J4" s="342"/>
-      <c r="K4" s="342"/>
-      <c r="L4" s="343"/>
-      <c r="M4" s="344"/>
-      <c r="N4" s="345" t="s">
+      <c r="H4" s="357"/>
+      <c r="I4" s="357"/>
+      <c r="J4" s="357"/>
+      <c r="K4" s="357"/>
+      <c r="L4" s="358"/>
+      <c r="M4" s="359"/>
+      <c r="N4" s="360" t="s">
         <v>27</v>
       </c>
-      <c r="O4" s="343"/>
-      <c r="P4" s="343"/>
-      <c r="Q4" s="343"/>
-      <c r="R4" s="343"/>
-      <c r="S4" s="343"/>
-      <c r="T4" s="346"/>
-      <c r="U4" s="341" t="s">
+      <c r="O4" s="358"/>
+      <c r="P4" s="358"/>
+      <c r="Q4" s="358"/>
+      <c r="R4" s="358"/>
+      <c r="S4" s="358"/>
+      <c r="T4" s="361"/>
+      <c r="U4" s="356" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="344"/>
+      <c r="V4" s="359"/>
       <c r="W4" s="319"/>
       <c r="X4" t="s">
         <v>0</v>
@@ -22135,9 +22140,11 @@
         <v>105</v>
       </c>
       <c r="F59" s="36" t="s">
-        <v>144</v>
-      </c>
-      <c r="G59" s="36"/>
+        <v>578</v>
+      </c>
+      <c r="G59" s="36" t="s">
+        <v>579</v>
+      </c>
     </row>
     <row r="60" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="43" t="s">
@@ -22357,16 +22364,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:62" s="60" customFormat="1" ht="23.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B1" s="348" t="s">
+      <c r="B1" s="363" t="s">
         <v>329</v>
       </c>
-      <c r="C1" s="348"/>
-      <c r="D1" s="348"/>
-      <c r="E1" s="348"/>
-      <c r="F1" s="348"/>
-      <c r="G1" s="348"/>
-      <c r="H1" s="348"/>
-      <c r="I1" s="348"/>
+      <c r="C1" s="363"/>
+      <c r="D1" s="363"/>
+      <c r="E1" s="363"/>
+      <c r="F1" s="363"/>
+      <c r="G1" s="363"/>
+      <c r="H1" s="363"/>
+      <c r="I1" s="363"/>
     </row>
     <row r="2" spans="1:62" s="60" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="106"/>
@@ -22378,7 +22385,7 @@
       <c r="G2" s="103" t="s">
         <v>328</v>
       </c>
-      <c r="H2" s="347" t="s">
+      <c r="H2" s="362" t="s">
         <v>327</v>
       </c>
       <c r="I2" s="102" t="s">
@@ -22423,7 +22430,7 @@
       <c r="V2" s="102" t="s">
         <v>326</v>
       </c>
-      <c r="W2" s="347" t="s">
+      <c r="W2" s="362" t="s">
         <v>325</v>
       </c>
       <c r="X2" s="103" t="s">
@@ -22438,7 +22445,7 @@
       <c r="AA2" s="103" t="s">
         <v>144</v>
       </c>
-      <c r="AB2" s="347" t="s">
+      <c r="AB2" s="362" t="s">
         <v>324</v>
       </c>
       <c r="AC2" s="100" t="s">
@@ -22468,7 +22475,7 @@
       <c r="AK2" s="100" t="s">
         <v>323</v>
       </c>
-      <c r="AL2" s="347" t="s">
+      <c r="AL2" s="362" t="s">
         <v>322</v>
       </c>
       <c r="AM2" s="100" t="s">
@@ -22510,7 +22517,7 @@
       <c r="AY2" s="100" t="s">
         <v>321</v>
       </c>
-      <c r="AZ2" s="347" t="s">
+      <c r="AZ2" s="362" t="s">
         <v>320</v>
       </c>
       <c r="BA2" s="99" t="s">
@@ -22540,7 +22547,7 @@
       <c r="BI2" s="99" t="s">
         <v>319</v>
       </c>
-      <c r="BJ2" s="347" t="s">
+      <c r="BJ2" s="362" t="s">
         <v>318</v>
       </c>
     </row>
@@ -22554,7 +22561,7 @@
       <c r="G3" s="103" t="s">
         <v>317</v>
       </c>
-      <c r="H3" s="347"/>
+      <c r="H3" s="362"/>
       <c r="I3" s="102" t="s">
         <v>316</v>
       </c>
@@ -22595,7 +22602,7 @@
       <c r="V3" s="102" t="s">
         <v>304</v>
       </c>
-      <c r="W3" s="347"/>
+      <c r="W3" s="362"/>
       <c r="X3" s="98"/>
       <c r="Y3" s="103" t="s">
         <v>303</v>
@@ -22606,7 +22613,7 @@
       <c r="AA3" s="103" t="s">
         <v>301</v>
       </c>
-      <c r="AB3" s="347"/>
+      <c r="AB3" s="362"/>
       <c r="AC3" s="100" t="s">
         <v>300</v>
       </c>
@@ -22634,7 +22641,7 @@
       <c r="AK3" s="100" t="s">
         <v>294</v>
       </c>
-      <c r="AL3" s="347"/>
+      <c r="AL3" s="362"/>
       <c r="AM3" s="100" t="s">
         <v>293</v>
       </c>
@@ -22674,7 +22681,7 @@
       <c r="AY3" s="100" t="s">
         <v>281</v>
       </c>
-      <c r="AZ3" s="347"/>
+      <c r="AZ3" s="362"/>
       <c r="BA3" s="99" t="s">
         <v>280</v>
       </c>
@@ -22702,7 +22709,7 @@
       <c r="BI3" s="99" t="s">
         <v>272</v>
       </c>
-      <c r="BJ3" s="347"/>
+      <c r="BJ3" s="362"/>
     </row>
     <row r="4" spans="1:62" s="60" customFormat="1" ht="60" x14ac:dyDescent="0.15">
       <c r="A4" s="105"/>
@@ -22724,7 +22731,7 @@
       <c r="G4" s="103" t="s">
         <v>267</v>
       </c>
-      <c r="H4" s="347"/>
+      <c r="H4" s="362"/>
       <c r="I4" s="102" t="s">
         <v>266</v>
       </c>
@@ -22767,7 +22774,7 @@
       <c r="V4" s="102" t="s">
         <v>253</v>
       </c>
-      <c r="W4" s="347"/>
+      <c r="W4" s="362"/>
       <c r="X4" s="101" t="s">
         <v>252</v>
       </c>
@@ -22780,7 +22787,7 @@
       <c r="AA4" s="101" t="s">
         <v>249</v>
       </c>
-      <c r="AB4" s="347"/>
+      <c r="AB4" s="362"/>
       <c r="AC4" s="100" t="s">
         <v>248</v>
       </c>
@@ -22808,7 +22815,7 @@
       <c r="AK4" s="100" t="s">
         <v>241</v>
       </c>
-      <c r="AL4" s="347"/>
+      <c r="AL4" s="362"/>
       <c r="AM4" s="100" t="s">
         <v>240</v>
       </c>
@@ -22848,7 +22855,7 @@
       <c r="AY4" s="100" t="s">
         <v>228</v>
       </c>
-      <c r="AZ4" s="347"/>
+      <c r="AZ4" s="362"/>
       <c r="BA4" s="99" t="s">
         <v>227</v>
       </c>
@@ -22876,7 +22883,7 @@
       <c r="BI4" s="99" t="s">
         <v>219</v>
       </c>
-      <c r="BJ4" s="347"/>
+      <c r="BJ4" s="362"/>
     </row>
     <row r="5" spans="1:62" s="60" customFormat="1" ht="11" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="70" t="s">
@@ -24169,13 +24176,13 @@
         <v>#N/A</v>
       </c>
       <c r="AC13" s="82"/>
-      <c r="AD13" s="358" t="e">
+      <c r="AD13" s="321" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"JCP")+
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"VPCP")+
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPCP")</f>
         <v>#N/A</v>
       </c>
-      <c r="AE13" s="358" t="e">
+      <c r="AE13" s="321" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"JI")+
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"VPI")+
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPI")</f>
@@ -24184,19 +24191,19 @@
       <c r="AF13" s="82"/>
       <c r="AG13" s="82"/>
       <c r="AH13" s="82"/>
-      <c r="AI13" s="358" t="e">
+      <c r="AI13" s="321" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"JAP")+
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"VPAP")+
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPAP")</f>
         <v>#N/A</v>
       </c>
-      <c r="AJ13" s="358" t="e">
+      <c r="AJ13" s="321" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"JE")+
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"VPE")+
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPE")</f>
         <v>#N/A</v>
       </c>
-      <c r="AK13" s="358" t="e">
+      <c r="AK13" s="321" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"VPLD")+
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPLD")</f>
         <v>#N/A</v>
@@ -24217,7 +24224,7 @@
       <c r="AV13" s="82"/>
       <c r="AW13" s="82"/>
       <c r="AX13" s="82"/>
-      <c r="AY13" s="358" t="e">
+      <c r="AY13" s="321" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"Magistrat SIEGE NS")</f>
         <v>#N/A</v>
       </c>
@@ -24997,8 +25004,8 @@
       </c>
       <c r="AZ19" s="57"/>
     </row>
-    <row r="20" spans="1:62" ht="252" x14ac:dyDescent="0.2">
-      <c r="F20" s="360" t="s">
+    <row r="20" spans="1:62" ht="28" x14ac:dyDescent="0.2">
+      <c r="F20" s="323" t="s">
         <v>553</v>
       </c>
       <c r="G20" s="254" t="e">
@@ -25006,7 +25013,7 @@
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé SUB")</f>
         <v>#N/A</v>
       </c>
-      <c r="U20" s="361" t="s">
+      <c r="U20" s="324" t="s">
         <v>555</v>
       </c>
       <c r="V20" s="254" t="e">
@@ -25015,7 +25022,7 @@
         <v>#N/A</v>
       </c>
       <c r="W20" s="57"/>
-      <c r="AX20" s="359" t="s">
+      <c r="AX20" s="322" t="s">
         <v>551</v>
       </c>
       <c r="AY20" s="196" t="e">
@@ -25065,16 +25072,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A1" s="349" t="s">
+      <c r="A1" s="364" t="s">
         <v>373</v>
       </c>
-      <c r="B1" s="349"/>
-      <c r="C1" s="349"/>
-      <c r="D1" s="349"/>
-      <c r="E1" s="349"/>
-      <c r="F1" s="349"/>
-      <c r="G1" s="349"/>
-      <c r="H1" s="349"/>
+      <c r="B1" s="364"/>
+      <c r="C1" s="364"/>
+      <c r="D1" s="364"/>
+      <c r="E1" s="364"/>
+      <c r="F1" s="364"/>
+      <c r="G1" s="364"/>
+      <c r="H1" s="364"/>
       <c r="I1" s="60"/>
       <c r="J1" s="60"/>
       <c r="K1" s="60"/>
@@ -25113,7 +25120,7 @@
       <c r="G2" s="103" t="s">
         <v>328</v>
       </c>
-      <c r="H2" s="347" t="s">
+      <c r="H2" s="362" t="s">
         <v>327</v>
       </c>
       <c r="I2" s="103" t="s">
@@ -25146,13 +25153,13 @@
       <c r="R2" s="103" t="s">
         <v>326</v>
       </c>
-      <c r="S2" s="347" t="s">
+      <c r="S2" s="362" t="s">
         <v>325</v>
       </c>
       <c r="T2" s="103" t="s">
         <v>144</v>
       </c>
-      <c r="U2" s="347" t="s">
+      <c r="U2" s="362" t="s">
         <v>324</v>
       </c>
       <c r="V2" s="103" t="s">
@@ -25182,7 +25189,7 @@
       <c r="AD2" s="103" t="s">
         <v>323</v>
       </c>
-      <c r="AE2" s="347" t="s">
+      <c r="AE2" s="362" t="s">
         <v>372</v>
       </c>
       <c r="AF2" s="103" t="s">
@@ -25194,7 +25201,7 @@
       <c r="AH2" s="103" t="s">
         <v>371</v>
       </c>
-      <c r="AI2" s="347" t="s">
+      <c r="AI2" s="362" t="s">
         <v>370</v>
       </c>
     </row>
@@ -25208,7 +25215,7 @@
       <c r="G3" s="103" t="s">
         <v>317</v>
       </c>
-      <c r="H3" s="347"/>
+      <c r="H3" s="362"/>
       <c r="I3" s="103" t="s">
         <v>369</v>
       </c>
@@ -25239,11 +25246,11 @@
       <c r="R3" s="103" t="s">
         <v>304</v>
       </c>
-      <c r="S3" s="347"/>
+      <c r="S3" s="362"/>
       <c r="T3" s="103" t="s">
         <v>301</v>
       </c>
-      <c r="U3" s="347"/>
+      <c r="U3" s="362"/>
       <c r="V3" s="103" t="s">
         <v>360</v>
       </c>
@@ -25271,7 +25278,7 @@
       <c r="AD3" s="103" t="s">
         <v>352</v>
       </c>
-      <c r="AE3" s="347"/>
+      <c r="AE3" s="362"/>
       <c r="AF3" s="103" t="s">
         <v>351</v>
       </c>
@@ -25281,7 +25288,7 @@
       <c r="AH3" s="103" t="s">
         <v>281</v>
       </c>
-      <c r="AI3" s="347"/>
+      <c r="AI3" s="362"/>
     </row>
     <row r="4" spans="1:35" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="106"/>
@@ -25303,7 +25310,7 @@
       <c r="G4" s="103" t="s">
         <v>267</v>
       </c>
-      <c r="H4" s="347"/>
+      <c r="H4" s="362"/>
       <c r="I4" s="103" t="s">
         <v>350</v>
       </c>
@@ -25334,11 +25341,11 @@
       <c r="R4" s="103" t="s">
         <v>253</v>
       </c>
-      <c r="S4" s="347"/>
+      <c r="S4" s="362"/>
       <c r="T4" s="103" t="s">
         <v>249</v>
       </c>
-      <c r="U4" s="347"/>
+      <c r="U4" s="362"/>
       <c r="V4" s="103" t="s">
         <v>341</v>
       </c>
@@ -25366,7 +25373,7 @@
       <c r="AD4" s="103" t="s">
         <v>333</v>
       </c>
-      <c r="AE4" s="347"/>
+      <c r="AE4" s="362"/>
       <c r="AF4" s="103" t="s">
         <v>332</v>
       </c>
@@ -25376,7 +25383,7 @@
       <c r="AH4" s="103" t="s">
         <v>228</v>
       </c>
-      <c r="AI4" s="347"/>
+      <c r="AI4" s="362"/>
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A5" s="109" t="s">
@@ -26043,7 +26050,7 @@
       </c>
       <c r="AF13" s="82"/>
       <c r="AG13" s="82"/>
-      <c r="AH13" s="358" t="e">
+      <c r="AH13" s="321" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
         <v>#N/A</v>
       </c>
@@ -26382,8 +26389,8 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="18" spans="4:34" ht="196" x14ac:dyDescent="0.2">
-      <c r="F18" s="360" t="s">
+    <row r="18" spans="4:34" ht="28" x14ac:dyDescent="0.2">
+      <c r="F18" s="323" t="s">
         <v>553</v>
       </c>
       <c r="G18" s="254" t="e">
@@ -26391,7 +26398,7 @@
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé SUB")</f>
         <v>#N/A</v>
       </c>
-      <c r="Q18" s="361" t="s">
+      <c r="Q18" s="324" t="s">
         <v>555</v>
       </c>
       <c r="R18" s="254" t="e">
@@ -26400,8 +26407,8 @@
         <v>#N/A</v>
       </c>
       <c r="S18" s="57"/>
-      <c r="AF18" s="362"/>
-      <c r="AG18" s="359" t="s">
+      <c r="AF18" s="325"/>
+      <c r="AG18" s="322" t="s">
         <v>551</v>
       </c>
       <c r="AH18" s="72" t="e">

</xml_diff>

<commit_message>
add column JE JI extractor
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{956251AA-BB3D-9C4F-A9C1-8FA0D21741F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{570E6720-6A4F-8F4B-BBDD-39A5917784D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1948" uniqueCount="580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1950" uniqueCount="582">
   <si>
     <t>#! END_ROW</t>
   </si>
@@ -5209,6 +5209,12 @@
   </si>
   <si>
     <t>Pas encore appelé dans la matrice DDG, à voir en fonction de la circulaire 2025/2026</t>
+  </si>
+  <si>
+    <t>Ecart JE</t>
+  </si>
+  <si>
+    <t>Ecart JI</t>
   </si>
 </sst>
 </file>
@@ -6404,7 +6410,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="373">
+  <cellXfs count="374">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -7585,6 +7591,9 @@
     </xf>
     <xf numFmtId="0" fontId="39" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -8712,13 +8721,13 @@
       <c r="G2" s="103" t="s">
         <v>326</v>
       </c>
-      <c r="H2" s="362" t="s">
+      <c r="H2" s="363" t="s">
         <v>325</v>
       </c>
       <c r="I2" s="103" t="s">
         <v>144</v>
       </c>
-      <c r="J2" s="362" t="s">
+      <c r="J2" s="363" t="s">
         <v>324</v>
       </c>
     </row>
@@ -8732,11 +8741,11 @@
       <c r="G3" s="103" t="s">
         <v>304</v>
       </c>
-      <c r="H3" s="362"/>
+      <c r="H3" s="363"/>
       <c r="I3" s="103" t="s">
         <v>301</v>
       </c>
-      <c r="J3" s="362"/>
+      <c r="J3" s="363"/>
     </row>
     <row r="4" spans="1:10" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="125"/>
@@ -8758,11 +8767,11 @@
       <c r="G4" s="103" t="s">
         <v>253</v>
       </c>
-      <c r="H4" s="362"/>
+      <c r="H4" s="363"/>
       <c r="I4" s="103" t="s">
         <v>249</v>
       </c>
-      <c r="J4" s="362"/>
+      <c r="J4" s="363"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="119" t="s">
@@ -9161,7 +9170,7 @@
       <c r="G2" s="103" t="s">
         <v>328</v>
       </c>
-      <c r="H2" s="362" t="s">
+      <c r="H2" s="363" t="s">
         <v>327</v>
       </c>
       <c r="I2" s="102" t="s">
@@ -9206,7 +9215,7 @@
       <c r="V2" s="102" t="s">
         <v>326</v>
       </c>
-      <c r="W2" s="362" t="s">
+      <c r="W2" s="363" t="s">
         <v>325</v>
       </c>
       <c r="X2" s="103" t="s">
@@ -9221,7 +9230,7 @@
       <c r="AA2" s="103" t="s">
         <v>144</v>
       </c>
-      <c r="AB2" s="362" t="s">
+      <c r="AB2" s="363" t="s">
         <v>324</v>
       </c>
       <c r="AC2" s="100" t="s">
@@ -9251,7 +9260,7 @@
       <c r="AK2" s="100" t="s">
         <v>323</v>
       </c>
-      <c r="AL2" s="362" t="s">
+      <c r="AL2" s="363" t="s">
         <v>322</v>
       </c>
       <c r="AM2" s="100" t="s">
@@ -9293,7 +9302,7 @@
       <c r="AY2" s="100" t="s">
         <v>321</v>
       </c>
-      <c r="AZ2" s="362" t="s">
+      <c r="AZ2" s="363" t="s">
         <v>320</v>
       </c>
       <c r="BA2" s="99" t="s">
@@ -9323,7 +9332,7 @@
       <c r="BI2" s="99" t="s">
         <v>319</v>
       </c>
-      <c r="BJ2" s="362" t="s">
+      <c r="BJ2" s="363" t="s">
         <v>318</v>
       </c>
       <c r="BK2"/>
@@ -9338,7 +9347,7 @@
       <c r="G3" s="103" t="s">
         <v>317</v>
       </c>
-      <c r="H3" s="362"/>
+      <c r="H3" s="363"/>
       <c r="I3" s="102" t="s">
         <v>316</v>
       </c>
@@ -9379,7 +9388,7 @@
       <c r="V3" s="102" t="s">
         <v>304</v>
       </c>
-      <c r="W3" s="362"/>
+      <c r="W3" s="363"/>
       <c r="X3" s="98"/>
       <c r="Y3" s="103" t="s">
         <v>303</v>
@@ -9390,7 +9399,7 @@
       <c r="AA3" s="103" t="s">
         <v>301</v>
       </c>
-      <c r="AB3" s="362"/>
+      <c r="AB3" s="363"/>
       <c r="AC3" s="100" t="s">
         <v>300</v>
       </c>
@@ -9418,7 +9427,7 @@
       <c r="AK3" s="100" t="s">
         <v>294</v>
       </c>
-      <c r="AL3" s="362"/>
+      <c r="AL3" s="363"/>
       <c r="AM3" s="100" t="s">
         <v>293</v>
       </c>
@@ -9458,7 +9467,7 @@
       <c r="AY3" s="100" t="s">
         <v>281</v>
       </c>
-      <c r="AZ3" s="362"/>
+      <c r="AZ3" s="363"/>
       <c r="BA3" s="99" t="s">
         <v>280</v>
       </c>
@@ -9486,7 +9495,7 @@
       <c r="BI3" s="99" t="s">
         <v>272</v>
       </c>
-      <c r="BJ3" s="362"/>
+      <c r="BJ3" s="363"/>
     </row>
     <row r="4" spans="1:63" s="60" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="105"/>
@@ -9508,7 +9517,7 @@
       <c r="G4" s="103" t="s">
         <v>267</v>
       </c>
-      <c r="H4" s="362"/>
+      <c r="H4" s="363"/>
       <c r="I4" s="102" t="s">
         <v>266</v>
       </c>
@@ -9551,7 +9560,7 @@
       <c r="V4" s="102" t="s">
         <v>253</v>
       </c>
-      <c r="W4" s="362"/>
+      <c r="W4" s="363"/>
       <c r="X4" s="101" t="s">
         <v>252</v>
       </c>
@@ -9564,7 +9573,7 @@
       <c r="AA4" s="101" t="s">
         <v>249</v>
       </c>
-      <c r="AB4" s="362"/>
+      <c r="AB4" s="363"/>
       <c r="AC4" s="100" t="s">
         <v>248</v>
       </c>
@@ -9592,7 +9601,7 @@
       <c r="AK4" s="100" t="s">
         <v>241</v>
       </c>
-      <c r="AL4" s="362"/>
+      <c r="AL4" s="363"/>
       <c r="AM4" s="100" t="s">
         <v>240</v>
       </c>
@@ -9632,7 +9641,7 @@
       <c r="AY4" s="100" t="s">
         <v>228</v>
       </c>
-      <c r="AZ4" s="362"/>
+      <c r="AZ4" s="363"/>
       <c r="BA4" s="99" t="s">
         <v>227</v>
       </c>
@@ -9660,7 +9669,7 @@
       <c r="BI4" s="99" t="s">
         <v>219</v>
       </c>
-      <c r="BJ4" s="362"/>
+      <c r="BJ4" s="363"/>
       <c r="BK4"/>
     </row>
     <row r="5" spans="1:63" s="60" customFormat="1" ht="15" x14ac:dyDescent="0.2">
@@ -12405,7 +12414,7 @@
       <c r="G2" s="103" t="s">
         <v>328</v>
       </c>
-      <c r="H2" s="362" t="s">
+      <c r="H2" s="363" t="s">
         <v>327</v>
       </c>
       <c r="I2" s="103" t="s">
@@ -12438,13 +12447,13 @@
       <c r="R2" s="103" t="s">
         <v>326</v>
       </c>
-      <c r="S2" s="362" t="s">
+      <c r="S2" s="363" t="s">
         <v>325</v>
       </c>
       <c r="T2" s="103" t="s">
         <v>144</v>
       </c>
-      <c r="U2" s="362" t="s">
+      <c r="U2" s="363" t="s">
         <v>324</v>
       </c>
       <c r="V2" s="103" t="s">
@@ -12474,7 +12483,7 @@
       <c r="AD2" s="103" t="s">
         <v>323</v>
       </c>
-      <c r="AE2" s="362" t="s">
+      <c r="AE2" s="363" t="s">
         <v>372</v>
       </c>
       <c r="AF2" s="103" t="s">
@@ -12486,7 +12495,7 @@
       <c r="AH2" s="103" t="s">
         <v>371</v>
       </c>
-      <c r="AI2" s="362" t="s">
+      <c r="AI2" s="363" t="s">
         <v>370</v>
       </c>
     </row>
@@ -12500,7 +12509,7 @@
       <c r="G3" s="103" t="s">
         <v>317</v>
       </c>
-      <c r="H3" s="362"/>
+      <c r="H3" s="363"/>
       <c r="I3" s="103" t="s">
         <v>369</v>
       </c>
@@ -12531,11 +12540,11 @@
       <c r="R3" s="103" t="s">
         <v>304</v>
       </c>
-      <c r="S3" s="362"/>
+      <c r="S3" s="363"/>
       <c r="T3" s="103" t="s">
         <v>301</v>
       </c>
-      <c r="U3" s="362"/>
+      <c r="U3" s="363"/>
       <c r="V3" s="103" t="s">
         <v>360</v>
       </c>
@@ -12563,7 +12572,7 @@
       <c r="AD3" s="103" t="s">
         <v>352</v>
       </c>
-      <c r="AE3" s="362"/>
+      <c r="AE3" s="363"/>
       <c r="AF3" s="103" t="s">
         <v>351</v>
       </c>
@@ -12573,7 +12582,7 @@
       <c r="AH3" s="103" t="s">
         <v>281</v>
       </c>
-      <c r="AI3" s="362"/>
+      <c r="AI3" s="363"/>
     </row>
     <row r="4" spans="1:62" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="106"/>
@@ -12595,7 +12604,7 @@
       <c r="G4" s="103" t="s">
         <v>267</v>
       </c>
-      <c r="H4" s="362"/>
+      <c r="H4" s="363"/>
       <c r="I4" s="103" t="s">
         <v>350</v>
       </c>
@@ -12626,11 +12635,11 @@
       <c r="R4" s="103" t="s">
         <v>253</v>
       </c>
-      <c r="S4" s="362"/>
+      <c r="S4" s="363"/>
       <c r="T4" s="103" t="s">
         <v>249</v>
       </c>
-      <c r="U4" s="362"/>
+      <c r="U4" s="363"/>
       <c r="V4" s="103" t="s">
         <v>341</v>
       </c>
@@ -12658,7 +12667,7 @@
       <c r="AD4" s="103" t="s">
         <v>333</v>
       </c>
-      <c r="AE4" s="362"/>
+      <c r="AE4" s="363"/>
       <c r="AF4" s="103" t="s">
         <v>332</v>
       </c>
@@ -12668,7 +12677,7 @@
       <c r="AH4" s="103" t="s">
         <v>228</v>
       </c>
-      <c r="AI4" s="362"/>
+      <c r="AI4" s="363"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="109" t="s">
@@ -14420,13 +14429,13 @@
       <c r="G2" s="103" t="s">
         <v>326</v>
       </c>
-      <c r="H2" s="362" t="s">
+      <c r="H2" s="363" t="s">
         <v>325</v>
       </c>
       <c r="I2" s="103" t="s">
         <v>144</v>
       </c>
-      <c r="J2" s="362" t="s">
+      <c r="J2" s="363" t="s">
         <v>324</v>
       </c>
     </row>
@@ -14440,11 +14449,11 @@
       <c r="G3" s="103" t="s">
         <v>304</v>
       </c>
-      <c r="H3" s="362"/>
+      <c r="H3" s="363"/>
       <c r="I3" s="103" t="s">
         <v>301</v>
       </c>
-      <c r="J3" s="362"/>
+      <c r="J3" s="363"/>
     </row>
     <row r="4" spans="1:62" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="125"/>
@@ -14466,11 +14475,11 @@
       <c r="G4" s="103" t="s">
         <v>253</v>
       </c>
-      <c r="H4" s="362"/>
+      <c r="H4" s="363"/>
       <c r="I4" s="103" t="s">
         <v>249</v>
       </c>
-      <c r="J4" s="362"/>
+      <c r="J4" s="363"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="119" t="s">
@@ -14857,13 +14866,13 @@
   <sheetData>
     <row r="1" spans="1:61" s="186" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="185"/>
-      <c r="B1" s="366" t="s">
+      <c r="B1" s="367" t="s">
         <v>329</v>
       </c>
-      <c r="C1" s="366"/>
-      <c r="D1" s="366"/>
-      <c r="E1" s="366"/>
-      <c r="F1" s="366"/>
+      <c r="C1" s="367"/>
+      <c r="D1" s="367"/>
+      <c r="E1" s="367"/>
+      <c r="F1" s="367"/>
       <c r="G1" s="187"/>
       <c r="H1" s="187"/>
       <c r="I1" s="187"/>
@@ -14908,7 +14917,7 @@
       <c r="O2" s="189" t="s">
         <v>323</v>
       </c>
-      <c r="P2" s="365" t="s">
+      <c r="P2" s="366" t="s">
         <v>322</v>
       </c>
       <c r="Q2" s="189" t="s">
@@ -14950,7 +14959,7 @@
       <c r="AC2" s="189" t="s">
         <v>321</v>
       </c>
-      <c r="AD2" s="365" t="s">
+      <c r="AD2" s="366" t="s">
         <v>320</v>
       </c>
       <c r="AE2" s="190" t="s">
@@ -14980,7 +14989,7 @@
       <c r="AM2" s="190" t="s">
         <v>319</v>
       </c>
-      <c r="AN2" s="365" t="s">
+      <c r="AN2" s="366" t="s">
         <v>318</v>
       </c>
       <c r="AQ2" s="189"/>
@@ -14991,7 +15000,7 @@
       <c r="AV2" s="189"/>
       <c r="AW2" s="189"/>
       <c r="AX2" s="189"/>
-      <c r="AY2" s="365"/>
+      <c r="AY2" s="366"/>
       <c r="AZ2" s="190"/>
       <c r="BA2" s="190"/>
       <c r="BB2" s="190"/>
@@ -15001,7 +15010,7 @@
       <c r="BF2" s="190"/>
       <c r="BG2" s="190"/>
       <c r="BH2" s="190"/>
-      <c r="BI2" s="365"/>
+      <c r="BI2" s="366"/>
     </row>
     <row r="3" spans="1:61" s="186" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="188"/>
@@ -15037,7 +15046,7 @@
       <c r="O3" s="189" t="s">
         <v>294</v>
       </c>
-      <c r="P3" s="365"/>
+      <c r="P3" s="366"/>
       <c r="Q3" s="189" t="s">
         <v>293</v>
       </c>
@@ -15077,7 +15086,7 @@
       <c r="AC3" s="189" t="s">
         <v>281</v>
       </c>
-      <c r="AD3" s="365"/>
+      <c r="AD3" s="366"/>
       <c r="AE3" s="190" t="s">
         <v>280</v>
       </c>
@@ -15105,7 +15114,7 @@
       <c r="AM3" s="190" t="s">
         <v>272</v>
       </c>
-      <c r="AN3" s="365"/>
+      <c r="AN3" s="366"/>
       <c r="AQ3" s="189"/>
       <c r="AR3" s="189"/>
       <c r="AS3" s="189"/>
@@ -15114,7 +15123,7 @@
       <c r="AV3" s="189"/>
       <c r="AW3" s="189"/>
       <c r="AX3" s="189"/>
-      <c r="AY3" s="365"/>
+      <c r="AY3" s="366"/>
       <c r="AZ3" s="190"/>
       <c r="BA3" s="190"/>
       <c r="BB3" s="190"/>
@@ -15124,7 +15133,7 @@
       <c r="BF3" s="190"/>
       <c r="BG3" s="190"/>
       <c r="BH3" s="190"/>
-      <c r="BI3" s="365"/>
+      <c r="BI3" s="366"/>
     </row>
     <row r="4" spans="1:61" s="186" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="191"/>
@@ -15170,7 +15179,7 @@
       <c r="O4" s="189" t="s">
         <v>241</v>
       </c>
-      <c r="P4" s="365"/>
+      <c r="P4" s="366"/>
       <c r="Q4" s="189" t="s">
         <v>240</v>
       </c>
@@ -15210,7 +15219,7 @@
       <c r="AC4" s="189" t="s">
         <v>228</v>
       </c>
-      <c r="AD4" s="365"/>
+      <c r="AD4" s="366"/>
       <c r="AE4" s="190" t="s">
         <v>227</v>
       </c>
@@ -15238,7 +15247,7 @@
       <c r="AM4" s="190" t="s">
         <v>219</v>
       </c>
-      <c r="AN4" s="365"/>
+      <c r="AN4" s="366"/>
       <c r="AQ4" s="189"/>
       <c r="AR4" s="189"/>
       <c r="AS4" s="189"/>
@@ -15247,7 +15256,7 @@
       <c r="AV4" s="189"/>
       <c r="AW4" s="189"/>
       <c r="AX4" s="189"/>
-      <c r="AY4" s="365"/>
+      <c r="AY4" s="366"/>
       <c r="AZ4" s="190"/>
       <c r="BA4" s="190"/>
       <c r="BB4" s="190"/>
@@ -15257,7 +15266,7 @@
       <c r="BF4" s="190"/>
       <c r="BG4" s="190"/>
       <c r="BH4" s="190"/>
-      <c r="BI4" s="365"/>
+      <c r="BI4" s="366"/>
     </row>
     <row r="5" spans="1:61" s="186" customFormat="1" ht="144" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="193" t="s">
@@ -16979,14 +16988,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="367" t="s">
+      <c r="A1" s="368" t="s">
         <v>373</v>
       </c>
-      <c r="B1" s="367"/>
-      <c r="C1" s="367"/>
-      <c r="D1" s="367"/>
-      <c r="E1" s="367"/>
-      <c r="F1" s="367"/>
+      <c r="B1" s="368"/>
+      <c r="C1" s="368"/>
+      <c r="D1" s="368"/>
+      <c r="E1" s="368"/>
+      <c r="F1" s="368"/>
       <c r="G1" s="218"/>
       <c r="H1" s="218"/>
       <c r="I1" s="218"/>
@@ -17036,7 +17045,7 @@
       <c r="O2" s="221" t="s">
         <v>323</v>
       </c>
-      <c r="P2" s="368" t="s">
+      <c r="P2" s="369" t="s">
         <v>372</v>
       </c>
       <c r="Q2" s="221" t="s">
@@ -17048,7 +17057,7 @@
       <c r="S2" s="221" t="s">
         <v>371</v>
       </c>
-      <c r="T2" s="368" t="s">
+      <c r="T2" s="369" t="s">
         <v>370</v>
       </c>
     </row>
@@ -17086,7 +17095,7 @@
       <c r="O3" s="221" t="s">
         <v>352</v>
       </c>
-      <c r="P3" s="368"/>
+      <c r="P3" s="369"/>
       <c r="Q3" s="221" t="s">
         <v>351</v>
       </c>
@@ -17096,7 +17105,7 @@
       <c r="S3" s="221" t="s">
         <v>281</v>
       </c>
-      <c r="T3" s="368"/>
+      <c r="T3" s="369"/>
     </row>
     <row r="4" spans="1:20" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="220"/>
@@ -17142,7 +17151,7 @@
       <c r="O4" s="221" t="s">
         <v>333</v>
       </c>
-      <c r="P4" s="368"/>
+      <c r="P4" s="369"/>
       <c r="Q4" s="221" t="s">
         <v>332</v>
       </c>
@@ -17152,7 +17161,7 @@
       <c r="S4" s="221" t="s">
         <v>228</v>
       </c>
-      <c r="T4" s="368"/>
+      <c r="T4" s="369"/>
     </row>
     <row r="5" spans="1:20" ht="317" x14ac:dyDescent="0.2">
       <c r="A5" s="224" t="s">
@@ -17738,16 +17747,16 @@
   <sheetData>
     <row r="1" spans="1:28" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="244"/>
-      <c r="B1" s="370" t="s">
+      <c r="B1" s="371" t="s">
         <v>329</v>
       </c>
-      <c r="C1" s="370"/>
-      <c r="D1" s="370"/>
-      <c r="E1" s="370"/>
-      <c r="F1" s="370"/>
-      <c r="G1" s="370"/>
-      <c r="H1" s="370"/>
-      <c r="I1" s="370"/>
+      <c r="C1" s="371"/>
+      <c r="D1" s="371"/>
+      <c r="E1" s="371"/>
+      <c r="F1" s="371"/>
+      <c r="G1" s="371"/>
+      <c r="H1" s="371"/>
+      <c r="I1" s="371"/>
       <c r="J1" s="241"/>
       <c r="K1" s="241"/>
       <c r="L1" s="241"/>
@@ -17778,7 +17787,7 @@
       <c r="G2" s="243" t="s">
         <v>328</v>
       </c>
-      <c r="H2" s="369" t="s">
+      <c r="H2" s="370" t="s">
         <v>327</v>
       </c>
       <c r="I2" s="246" t="s">
@@ -17823,7 +17832,7 @@
       <c r="V2" s="246" t="s">
         <v>326</v>
       </c>
-      <c r="W2" s="369" t="s">
+      <c r="W2" s="370" t="s">
         <v>325</v>
       </c>
       <c r="X2" s="243" t="s">
@@ -17838,7 +17847,7 @@
       <c r="AA2" s="243" t="s">
         <v>144</v>
       </c>
-      <c r="AB2" s="369" t="s">
+      <c r="AB2" s="370" t="s">
         <v>324</v>
       </c>
     </row>
@@ -17852,7 +17861,7 @@
       <c r="G3" s="243" t="s">
         <v>317</v>
       </c>
-      <c r="H3" s="369"/>
+      <c r="H3" s="370"/>
       <c r="I3" s="246" t="s">
         <v>316</v>
       </c>
@@ -17893,7 +17902,7 @@
       <c r="V3" s="246" t="s">
         <v>304</v>
       </c>
-      <c r="W3" s="369"/>
+      <c r="W3" s="370"/>
       <c r="X3" s="245"/>
       <c r="Y3" s="243" t="s">
         <v>303</v>
@@ -17904,7 +17913,7 @@
       <c r="AA3" s="243" t="s">
         <v>301</v>
       </c>
-      <c r="AB3" s="369"/>
+      <c r="AB3" s="370"/>
     </row>
     <row r="4" spans="1:28" ht="98" x14ac:dyDescent="0.2">
       <c r="A4" s="247"/>
@@ -17926,7 +17935,7 @@
       <c r="G4" s="243" t="s">
         <v>267</v>
       </c>
-      <c r="H4" s="369"/>
+      <c r="H4" s="370"/>
       <c r="I4" s="246" t="s">
         <v>266</v>
       </c>
@@ -17969,7 +17978,7 @@
       <c r="V4" s="249" t="s">
         <v>253</v>
       </c>
-      <c r="W4" s="369"/>
+      <c r="W4" s="370"/>
       <c r="X4" s="250" t="s">
         <v>252</v>
       </c>
@@ -17982,7 +17991,7 @@
       <c r="AA4" s="250" t="s">
         <v>249</v>
       </c>
-      <c r="AB4" s="369"/>
+      <c r="AB4" s="370"/>
     </row>
     <row r="5" spans="1:28" ht="196" x14ac:dyDescent="0.2">
       <c r="A5" s="251" t="s">
@@ -18876,16 +18885,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="372" t="s">
+      <c r="A1" s="373" t="s">
         <v>373</v>
       </c>
-      <c r="B1" s="372"/>
-      <c r="C1" s="372"/>
-      <c r="D1" s="372"/>
-      <c r="E1" s="372"/>
-      <c r="F1" s="372"/>
-      <c r="G1" s="372"/>
-      <c r="H1" s="372"/>
+      <c r="B1" s="373"/>
+      <c r="C1" s="373"/>
+      <c r="D1" s="373"/>
+      <c r="E1" s="373"/>
+      <c r="F1" s="373"/>
+      <c r="G1" s="373"/>
+      <c r="H1" s="373"/>
       <c r="I1" s="291"/>
       <c r="J1" s="291"/>
       <c r="K1" s="291"/>
@@ -18910,7 +18919,7 @@
       <c r="G2" s="293" t="s">
         <v>328</v>
       </c>
-      <c r="H2" s="371" t="s">
+      <c r="H2" s="372" t="s">
         <v>327</v>
       </c>
       <c r="I2" s="293" t="s">
@@ -18943,13 +18952,13 @@
       <c r="R2" s="293" t="s">
         <v>326</v>
       </c>
-      <c r="S2" s="371" t="s">
+      <c r="S2" s="372" t="s">
         <v>325</v>
       </c>
       <c r="T2" s="293" t="s">
         <v>144</v>
       </c>
-      <c r="U2" s="371" t="s">
+      <c r="U2" s="372" t="s">
         <v>324</v>
       </c>
     </row>
@@ -18963,7 +18972,7 @@
       <c r="G3" s="293" t="s">
         <v>317</v>
       </c>
-      <c r="H3" s="371"/>
+      <c r="H3" s="372"/>
       <c r="I3" s="293" t="s">
         <v>369</v>
       </c>
@@ -18994,11 +19003,11 @@
       <c r="R3" s="293" t="s">
         <v>304</v>
       </c>
-      <c r="S3" s="371"/>
+      <c r="S3" s="372"/>
       <c r="T3" s="293" t="s">
         <v>301</v>
       </c>
-      <c r="U3" s="371"/>
+      <c r="U3" s="372"/>
     </row>
     <row r="4" spans="1:21" ht="112" x14ac:dyDescent="0.2">
       <c r="A4" s="290"/>
@@ -19020,7 +19029,7 @@
       <c r="G4" s="293" t="s">
         <v>267</v>
       </c>
-      <c r="H4" s="371"/>
+      <c r="H4" s="372"/>
       <c r="I4" s="293" t="s">
         <v>350</v>
       </c>
@@ -19051,11 +19060,11 @@
       <c r="R4" s="293" t="s">
         <v>253</v>
       </c>
-      <c r="S4" s="371"/>
+      <c r="S4" s="372"/>
       <c r="T4" s="293" t="s">
         <v>249</v>
       </c>
-      <c r="U4" s="371"/>
+      <c r="U4" s="372"/>
     </row>
     <row r="5" spans="1:21" ht="196" x14ac:dyDescent="0.2">
       <c r="A5" s="296" t="s">
@@ -19746,13 +19755,13 @@
       <c r="K2" s="221" t="s">
         <v>326</v>
       </c>
-      <c r="L2" s="368" t="s">
+      <c r="L2" s="369" t="s">
         <v>325</v>
       </c>
       <c r="M2" s="221" t="s">
         <v>144</v>
       </c>
-      <c r="N2" s="368" t="s">
+      <c r="N2" s="369" t="s">
         <v>324</v>
       </c>
     </row>
@@ -19770,11 +19779,11 @@
       <c r="K3" s="221" t="s">
         <v>304</v>
       </c>
-      <c r="L3" s="368"/>
+      <c r="L3" s="369"/>
       <c r="M3" s="221" t="s">
         <v>301</v>
       </c>
-      <c r="N3" s="368"/>
+      <c r="N3" s="369"/>
     </row>
     <row r="4" spans="1:14" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="274"/>
@@ -19800,11 +19809,11 @@
       <c r="K4" s="221" t="s">
         <v>253</v>
       </c>
-      <c r="L4" s="368"/>
+      <c r="L4" s="369"/>
       <c r="M4" s="221" t="s">
         <v>249</v>
       </c>
-      <c r="N4" s="368"/>
+      <c r="N4" s="369"/>
     </row>
     <row r="5" spans="1:14" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="276"/>
@@ -20456,7 +20465,7 @@
   <sheetPr codeName="Feuil13">
     <tabColor rgb="FF2C45E0"/>
   </sheetPr>
-  <dimension ref="A1:FG4"/>
+  <dimension ref="A1:FJ4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.6640625" customWidth="1"/>
@@ -20473,7 +20482,7 @@
     <col min="170" max="170" width="15.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:163" s="4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:166" s="4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>377</v>
       </c>
@@ -20493,11 +20502,13 @@
       <c r="FD1" s="355"/>
       <c r="FE1" s="355"/>
       <c r="FF1" s="355"/>
-      <c r="FG1" s="8" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:163" ht="66" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="FG1" s="356"/>
+      <c r="FH1" s="356"/>
+      <c r="FJ1" s="26" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:166" ht="66" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="22" t="s">
         <v>8</v>
       </c>
@@ -20522,8 +20533,15 @@
       <c r="FF2" s="142" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="3" spans="1:163" x14ac:dyDescent="0.2">
+      <c r="FG2" s="142" t="s">
+        <v>580</v>
+      </c>
+      <c r="FH2" s="142" t="s">
+        <v>581</v>
+      </c>
+      <c r="FJ2" s="26"/>
+    </row>
+    <row r="3" spans="1:166" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="s">
         <v>11</v>
       </c>
@@ -20531,7 +20549,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:163" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:166" x14ac:dyDescent="0.2">
       <c r="B4" s="27" t="s">
         <v>7</v>
       </c>
@@ -20540,7 +20558,7 @@
   </sheetData>
   <autoFilter ref="A2:DT2" xr:uid="{3B89445B-6ECC-4440-B85C-E593AE209933}"/>
   <mergeCells count="1">
-    <mergeCell ref="FA1:FF1"/>
+    <mergeCell ref="FA1:FH1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -20630,28 +20648,28 @@
       <c r="D4" s="312"/>
       <c r="E4" s="312"/>
       <c r="F4" s="312"/>
-      <c r="G4" s="356" t="s">
+      <c r="G4" s="357" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="357"/>
-      <c r="I4" s="357"/>
-      <c r="J4" s="357"/>
-      <c r="K4" s="357"/>
-      <c r="L4" s="358"/>
-      <c r="M4" s="359"/>
-      <c r="N4" s="360" t="s">
+      <c r="H4" s="358"/>
+      <c r="I4" s="358"/>
+      <c r="J4" s="358"/>
+      <c r="K4" s="358"/>
+      <c r="L4" s="359"/>
+      <c r="M4" s="360"/>
+      <c r="N4" s="361" t="s">
         <v>27</v>
       </c>
-      <c r="O4" s="358"/>
-      <c r="P4" s="358"/>
-      <c r="Q4" s="358"/>
-      <c r="R4" s="358"/>
-      <c r="S4" s="358"/>
-      <c r="T4" s="361"/>
-      <c r="U4" s="356" t="s">
+      <c r="O4" s="359"/>
+      <c r="P4" s="359"/>
+      <c r="Q4" s="359"/>
+      <c r="R4" s="359"/>
+      <c r="S4" s="359"/>
+      <c r="T4" s="362"/>
+      <c r="U4" s="357" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="359"/>
+      <c r="V4" s="360"/>
       <c r="W4" s="319"/>
       <c r="X4" t="s">
         <v>0</v>
@@ -22364,16 +22382,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:62" s="60" customFormat="1" ht="23.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B1" s="363" t="s">
+      <c r="B1" s="364" t="s">
         <v>329</v>
       </c>
-      <c r="C1" s="363"/>
-      <c r="D1" s="363"/>
-      <c r="E1" s="363"/>
-      <c r="F1" s="363"/>
-      <c r="G1" s="363"/>
-      <c r="H1" s="363"/>
-      <c r="I1" s="363"/>
+      <c r="C1" s="364"/>
+      <c r="D1" s="364"/>
+      <c r="E1" s="364"/>
+      <c r="F1" s="364"/>
+      <c r="G1" s="364"/>
+      <c r="H1" s="364"/>
+      <c r="I1" s="364"/>
     </row>
     <row r="2" spans="1:62" s="60" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="106"/>
@@ -22385,7 +22403,7 @@
       <c r="G2" s="103" t="s">
         <v>328</v>
       </c>
-      <c r="H2" s="362" t="s">
+      <c r="H2" s="363" t="s">
         <v>327</v>
       </c>
       <c r="I2" s="102" t="s">
@@ -22430,7 +22448,7 @@
       <c r="V2" s="102" t="s">
         <v>326</v>
       </c>
-      <c r="W2" s="362" t="s">
+      <c r="W2" s="363" t="s">
         <v>325</v>
       </c>
       <c r="X2" s="103" t="s">
@@ -22445,7 +22463,7 @@
       <c r="AA2" s="103" t="s">
         <v>144</v>
       </c>
-      <c r="AB2" s="362" t="s">
+      <c r="AB2" s="363" t="s">
         <v>324</v>
       </c>
       <c r="AC2" s="100" t="s">
@@ -22475,7 +22493,7 @@
       <c r="AK2" s="100" t="s">
         <v>323</v>
       </c>
-      <c r="AL2" s="362" t="s">
+      <c r="AL2" s="363" t="s">
         <v>322</v>
       </c>
       <c r="AM2" s="100" t="s">
@@ -22517,7 +22535,7 @@
       <c r="AY2" s="100" t="s">
         <v>321</v>
       </c>
-      <c r="AZ2" s="362" t="s">
+      <c r="AZ2" s="363" t="s">
         <v>320</v>
       </c>
       <c r="BA2" s="99" t="s">
@@ -22547,7 +22565,7 @@
       <c r="BI2" s="99" t="s">
         <v>319</v>
       </c>
-      <c r="BJ2" s="362" t="s">
+      <c r="BJ2" s="363" t="s">
         <v>318</v>
       </c>
     </row>
@@ -22561,7 +22579,7 @@
       <c r="G3" s="103" t="s">
         <v>317</v>
       </c>
-      <c r="H3" s="362"/>
+      <c r="H3" s="363"/>
       <c r="I3" s="102" t="s">
         <v>316</v>
       </c>
@@ -22602,7 +22620,7 @@
       <c r="V3" s="102" t="s">
         <v>304</v>
       </c>
-      <c r="W3" s="362"/>
+      <c r="W3" s="363"/>
       <c r="X3" s="98"/>
       <c r="Y3" s="103" t="s">
         <v>303</v>
@@ -22613,7 +22631,7 @@
       <c r="AA3" s="103" t="s">
         <v>301</v>
       </c>
-      <c r="AB3" s="362"/>
+      <c r="AB3" s="363"/>
       <c r="AC3" s="100" t="s">
         <v>300</v>
       </c>
@@ -22641,7 +22659,7 @@
       <c r="AK3" s="100" t="s">
         <v>294</v>
       </c>
-      <c r="AL3" s="362"/>
+      <c r="AL3" s="363"/>
       <c r="AM3" s="100" t="s">
         <v>293</v>
       </c>
@@ -22681,7 +22699,7 @@
       <c r="AY3" s="100" t="s">
         <v>281</v>
       </c>
-      <c r="AZ3" s="362"/>
+      <c r="AZ3" s="363"/>
       <c r="BA3" s="99" t="s">
         <v>280</v>
       </c>
@@ -22709,7 +22727,7 @@
       <c r="BI3" s="99" t="s">
         <v>272</v>
       </c>
-      <c r="BJ3" s="362"/>
+      <c r="BJ3" s="363"/>
     </row>
     <row r="4" spans="1:62" s="60" customFormat="1" ht="60" x14ac:dyDescent="0.15">
       <c r="A4" s="105"/>
@@ -22731,7 +22749,7 @@
       <c r="G4" s="103" t="s">
         <v>267</v>
       </c>
-      <c r="H4" s="362"/>
+      <c r="H4" s="363"/>
       <c r="I4" s="102" t="s">
         <v>266</v>
       </c>
@@ -22774,7 +22792,7 @@
       <c r="V4" s="102" t="s">
         <v>253</v>
       </c>
-      <c r="W4" s="362"/>
+      <c r="W4" s="363"/>
       <c r="X4" s="101" t="s">
         <v>252</v>
       </c>
@@ -22787,7 +22805,7 @@
       <c r="AA4" s="101" t="s">
         <v>249</v>
       </c>
-      <c r="AB4" s="362"/>
+      <c r="AB4" s="363"/>
       <c r="AC4" s="100" t="s">
         <v>248</v>
       </c>
@@ -22815,7 +22833,7 @@
       <c r="AK4" s="100" t="s">
         <v>241</v>
       </c>
-      <c r="AL4" s="362"/>
+      <c r="AL4" s="363"/>
       <c r="AM4" s="100" t="s">
         <v>240</v>
       </c>
@@ -22855,7 +22873,7 @@
       <c r="AY4" s="100" t="s">
         <v>228</v>
       </c>
-      <c r="AZ4" s="362"/>
+      <c r="AZ4" s="363"/>
       <c r="BA4" s="99" t="s">
         <v>227</v>
       </c>
@@ -22883,7 +22901,7 @@
       <c r="BI4" s="99" t="s">
         <v>219</v>
       </c>
-      <c r="BJ4" s="362"/>
+      <c r="BJ4" s="363"/>
     </row>
     <row r="5" spans="1:62" s="60" customFormat="1" ht="11" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="70" t="s">
@@ -25072,16 +25090,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A1" s="364" t="s">
+      <c r="A1" s="365" t="s">
         <v>373</v>
       </c>
-      <c r="B1" s="364"/>
-      <c r="C1" s="364"/>
-      <c r="D1" s="364"/>
-      <c r="E1" s="364"/>
-      <c r="F1" s="364"/>
-      <c r="G1" s="364"/>
-      <c r="H1" s="364"/>
+      <c r="B1" s="365"/>
+      <c r="C1" s="365"/>
+      <c r="D1" s="365"/>
+      <c r="E1" s="365"/>
+      <c r="F1" s="365"/>
+      <c r="G1" s="365"/>
+      <c r="H1" s="365"/>
       <c r="I1" s="60"/>
       <c r="J1" s="60"/>
       <c r="K1" s="60"/>
@@ -25120,7 +25138,7 @@
       <c r="G2" s="103" t="s">
         <v>328</v>
       </c>
-      <c r="H2" s="362" t="s">
+      <c r="H2" s="363" t="s">
         <v>327</v>
       </c>
       <c r="I2" s="103" t="s">
@@ -25153,13 +25171,13 @@
       <c r="R2" s="103" t="s">
         <v>326</v>
       </c>
-      <c r="S2" s="362" t="s">
+      <c r="S2" s="363" t="s">
         <v>325</v>
       </c>
       <c r="T2" s="103" t="s">
         <v>144</v>
       </c>
-      <c r="U2" s="362" t="s">
+      <c r="U2" s="363" t="s">
         <v>324</v>
       </c>
       <c r="V2" s="103" t="s">
@@ -25189,7 +25207,7 @@
       <c r="AD2" s="103" t="s">
         <v>323</v>
       </c>
-      <c r="AE2" s="362" t="s">
+      <c r="AE2" s="363" t="s">
         <v>372</v>
       </c>
       <c r="AF2" s="103" t="s">
@@ -25201,7 +25219,7 @@
       <c r="AH2" s="103" t="s">
         <v>371</v>
       </c>
-      <c r="AI2" s="362" t="s">
+      <c r="AI2" s="363" t="s">
         <v>370</v>
       </c>
     </row>
@@ -25215,7 +25233,7 @@
       <c r="G3" s="103" t="s">
         <v>317</v>
       </c>
-      <c r="H3" s="362"/>
+      <c r="H3" s="363"/>
       <c r="I3" s="103" t="s">
         <v>369</v>
       </c>
@@ -25246,11 +25264,11 @@
       <c r="R3" s="103" t="s">
         <v>304</v>
       </c>
-      <c r="S3" s="362"/>
+      <c r="S3" s="363"/>
       <c r="T3" s="103" t="s">
         <v>301</v>
       </c>
-      <c r="U3" s="362"/>
+      <c r="U3" s="363"/>
       <c r="V3" s="103" t="s">
         <v>360</v>
       </c>
@@ -25278,7 +25296,7 @@
       <c r="AD3" s="103" t="s">
         <v>352</v>
       </c>
-      <c r="AE3" s="362"/>
+      <c r="AE3" s="363"/>
       <c r="AF3" s="103" t="s">
         <v>351</v>
       </c>
@@ -25288,7 +25306,7 @@
       <c r="AH3" s="103" t="s">
         <v>281</v>
       </c>
-      <c r="AI3" s="362"/>
+      <c r="AI3" s="363"/>
     </row>
     <row r="4" spans="1:35" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="106"/>
@@ -25310,7 +25328,7 @@
       <c r="G4" s="103" t="s">
         <v>267</v>
       </c>
-      <c r="H4" s="362"/>
+      <c r="H4" s="363"/>
       <c r="I4" s="103" t="s">
         <v>350</v>
       </c>
@@ -25341,11 +25359,11 @@
       <c r="R4" s="103" t="s">
         <v>253</v>
       </c>
-      <c r="S4" s="362"/>
+      <c r="S4" s="363"/>
       <c r="T4" s="103" t="s">
         <v>249</v>
       </c>
-      <c r="U4" s="362"/>
+      <c r="U4" s="363"/>
       <c r="V4" s="103" t="s">
         <v>341</v>
       </c>
@@ -25373,7 +25391,7 @@
       <c r="AD4" s="103" t="s">
         <v>333</v>
       </c>
-      <c r="AE4" s="362"/>
+      <c r="AE4" s="363"/>
       <c r="AF4" s="103" t="s">
         <v>332</v>
       </c>
@@ -25383,7 +25401,7 @@
       <c r="AH4" s="103" t="s">
         <v>228</v>
       </c>
-      <c r="AI4" s="362"/>
+      <c r="AI4" s="363"/>
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A5" s="109" t="s">

</xml_diff>

<commit_message>
update extractor JE JI
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13F5B946-2296-0149-9C85-A03EEC4EF1D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DD0B010-AF30-8243-8434-832785C3597D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1588" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1590" uniqueCount="437">
   <si>
     <t>#! END_ROW</t>
   </si>
@@ -4774,6 +4774,12 @@
   </si>
   <si>
     <t>## f.category_label</t>
+  </si>
+  <si>
+    <t>Ecart JE</t>
+  </si>
+  <si>
+    <t>Ecart JI</t>
   </si>
 </sst>
 </file>
@@ -5952,7 +5958,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="356">
+  <cellXfs count="357">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -7140,6 +7146,9 @@
     <xf numFmtId="0" fontId="53" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -19953,7 +19962,7 @@
   <sheetPr codeName="Feuil13">
     <tabColor rgb="FF2C45E0"/>
   </sheetPr>
-  <dimension ref="A1:FG4"/>
+  <dimension ref="A1:FI4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.6640625" customWidth="1"/>
@@ -19970,7 +19979,7 @@
     <col min="170" max="170" width="15.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:163" s="4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:165" s="4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>232</v>
       </c>
@@ -19990,11 +19999,13 @@
       <c r="FD1" s="338"/>
       <c r="FE1" s="338"/>
       <c r="FF1" s="338"/>
-      <c r="FG1" s="8" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:163" ht="66" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="FG1" s="356"/>
+      <c r="FH1" s="356"/>
+      <c r="FI1" s="4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:165" ht="66" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="22" t="s">
         <v>8</v>
       </c>
@@ -20019,8 +20030,14 @@
       <c r="FF2" s="126" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="3" spans="1:163" x14ac:dyDescent="0.2">
+      <c r="FG2" s="126" t="s">
+        <v>435</v>
+      </c>
+      <c r="FH2" s="126" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="3" spans="1:165" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="s">
         <v>11</v>
       </c>
@@ -20028,7 +20045,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:163" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:165" x14ac:dyDescent="0.2">
       <c r="B4" s="27" t="s">
         <v>7</v>
       </c>
@@ -20037,7 +20054,7 @@
   </sheetData>
   <autoFilter ref="A2:DT2" xr:uid="{3B89445B-6ECC-4440-B85C-E593AE209933}"/>
   <mergeCells count="1">
-    <mergeCell ref="FA1:FF1"/>
+    <mergeCell ref="FA1:FH1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
fix fct extractor round JE JI and fix agregat
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DD0B010-AF30-8243-8434-832785C3597D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E93949BE-F58E-7C44-BDD7-AD9F259563F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1590" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1591" uniqueCount="438">
   <si>
     <t>#! END_ROW</t>
   </si>
@@ -4780,6 +4780,9 @@
   </si>
   <si>
     <t>Ecart JI</t>
+  </si>
+  <si>
+    <t>Fonction agrégat</t>
   </si>
 </sst>
 </file>
@@ -7089,6 +7092,9 @@
     <xf numFmtId="0" fontId="37" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -7146,9 +7152,6 @@
     <xf numFmtId="0" fontId="53" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -8218,13 +8221,13 @@
       <c r="G2" s="87" t="s">
         <v>181</v>
       </c>
-      <c r="H2" s="345" t="s">
+      <c r="H2" s="346" t="s">
         <v>180</v>
       </c>
       <c r="I2" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="J2" s="345" t="s">
+      <c r="J2" s="346" t="s">
         <v>179</v>
       </c>
     </row>
@@ -8238,11 +8241,11 @@
       <c r="G3" s="87" t="s">
         <v>159</v>
       </c>
-      <c r="H3" s="345"/>
+      <c r="H3" s="346"/>
       <c r="I3" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="J3" s="345"/>
+      <c r="J3" s="346"/>
     </row>
     <row r="4" spans="1:10" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="109"/>
@@ -8264,11 +8267,11 @@
       <c r="G4" s="87" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="345"/>
+      <c r="H4" s="346"/>
       <c r="I4" s="87" t="s">
         <v>104</v>
       </c>
-      <c r="J4" s="345"/>
+      <c r="J4" s="346"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="103" t="s">
@@ -8667,7 +8670,7 @@
       <c r="G2" s="87" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="345" t="s">
+      <c r="H2" s="346" t="s">
         <v>182</v>
       </c>
       <c r="I2" s="86" t="s">
@@ -8712,7 +8715,7 @@
       <c r="V2" s="86" t="s">
         <v>181</v>
       </c>
-      <c r="W2" s="345" t="s">
+      <c r="W2" s="346" t="s">
         <v>180</v>
       </c>
       <c r="X2" s="87" t="s">
@@ -8727,7 +8730,7 @@
       <c r="AA2" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="AB2" s="345" t="s">
+      <c r="AB2" s="346" t="s">
         <v>179</v>
       </c>
       <c r="AC2" s="84" t="s">
@@ -8757,7 +8760,7 @@
       <c r="AK2" s="84" t="s">
         <v>178</v>
       </c>
-      <c r="AL2" s="345" t="s">
+      <c r="AL2" s="346" t="s">
         <v>177</v>
       </c>
       <c r="AM2" s="84" t="s">
@@ -8799,7 +8802,7 @@
       <c r="AY2" s="84" t="s">
         <v>176</v>
       </c>
-      <c r="AZ2" s="345" t="s">
+      <c r="AZ2" s="346" t="s">
         <v>175</v>
       </c>
       <c r="BA2" s="83" t="s">
@@ -8829,7 +8832,7 @@
       <c r="BI2" s="83" t="s">
         <v>174</v>
       </c>
-      <c r="BJ2" s="345" t="s">
+      <c r="BJ2" s="346" t="s">
         <v>173</v>
       </c>
       <c r="BK2"/>
@@ -8844,7 +8847,7 @@
       <c r="G3" s="87" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="345"/>
+      <c r="H3" s="346"/>
       <c r="I3" s="86" t="s">
         <v>171</v>
       </c>
@@ -8885,7 +8888,7 @@
       <c r="V3" s="86" t="s">
         <v>159</v>
       </c>
-      <c r="W3" s="345"/>
+      <c r="W3" s="346"/>
       <c r="X3" s="82"/>
       <c r="Y3" s="87" t="s">
         <v>158</v>
@@ -8896,7 +8899,7 @@
       <c r="AA3" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="AB3" s="345"/>
+      <c r="AB3" s="346"/>
       <c r="AC3" s="84" t="s">
         <v>155</v>
       </c>
@@ -8924,7 +8927,7 @@
       <c r="AK3" s="84" t="s">
         <v>149</v>
       </c>
-      <c r="AL3" s="345"/>
+      <c r="AL3" s="346"/>
       <c r="AM3" s="84" t="s">
         <v>148</v>
       </c>
@@ -8964,7 +8967,7 @@
       <c r="AY3" s="84" t="s">
         <v>136</v>
       </c>
-      <c r="AZ3" s="345"/>
+      <c r="AZ3" s="346"/>
       <c r="BA3" s="83" t="s">
         <v>135</v>
       </c>
@@ -8992,7 +8995,7 @@
       <c r="BI3" s="83" t="s">
         <v>127</v>
       </c>
-      <c r="BJ3" s="345"/>
+      <c r="BJ3" s="346"/>
     </row>
     <row r="4" spans="1:63" s="44" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="89"/>
@@ -9014,7 +9017,7 @@
       <c r="G4" s="87" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="345"/>
+      <c r="H4" s="346"/>
       <c r="I4" s="86" t="s">
         <v>121</v>
       </c>
@@ -9057,7 +9060,7 @@
       <c r="V4" s="86" t="s">
         <v>108</v>
       </c>
-      <c r="W4" s="345"/>
+      <c r="W4" s="346"/>
       <c r="X4" s="85" t="s">
         <v>107</v>
       </c>
@@ -9070,7 +9073,7 @@
       <c r="AA4" s="85" t="s">
         <v>104</v>
       </c>
-      <c r="AB4" s="345"/>
+      <c r="AB4" s="346"/>
       <c r="AC4" s="84" t="s">
         <v>103</v>
       </c>
@@ -9098,7 +9101,7 @@
       <c r="AK4" s="84" t="s">
         <v>96</v>
       </c>
-      <c r="AL4" s="345"/>
+      <c r="AL4" s="346"/>
       <c r="AM4" s="84" t="s">
         <v>95</v>
       </c>
@@ -9138,7 +9141,7 @@
       <c r="AY4" s="84" t="s">
         <v>83</v>
       </c>
-      <c r="AZ4" s="345"/>
+      <c r="AZ4" s="346"/>
       <c r="BA4" s="83" t="s">
         <v>82</v>
       </c>
@@ -9166,7 +9169,7 @@
       <c r="BI4" s="83" t="s">
         <v>74</v>
       </c>
-      <c r="BJ4" s="345"/>
+      <c r="BJ4" s="346"/>
       <c r="BK4"/>
     </row>
     <row r="5" spans="1:63" s="44" customFormat="1" ht="15" x14ac:dyDescent="0.2">
@@ -11911,7 +11914,7 @@
       <c r="G2" s="87" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="345" t="s">
+      <c r="H2" s="346" t="s">
         <v>182</v>
       </c>
       <c r="I2" s="87" t="s">
@@ -11944,13 +11947,13 @@
       <c r="R2" s="87" t="s">
         <v>181</v>
       </c>
-      <c r="S2" s="345" t="s">
+      <c r="S2" s="346" t="s">
         <v>180</v>
       </c>
       <c r="T2" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="U2" s="345" t="s">
+      <c r="U2" s="346" t="s">
         <v>179</v>
       </c>
       <c r="V2" s="87" t="s">
@@ -11980,7 +11983,7 @@
       <c r="AD2" s="87" t="s">
         <v>178</v>
       </c>
-      <c r="AE2" s="345" t="s">
+      <c r="AE2" s="346" t="s">
         <v>227</v>
       </c>
       <c r="AF2" s="87" t="s">
@@ -11992,7 +11995,7 @@
       <c r="AH2" s="87" t="s">
         <v>226</v>
       </c>
-      <c r="AI2" s="345" t="s">
+      <c r="AI2" s="346" t="s">
         <v>225</v>
       </c>
     </row>
@@ -12006,7 +12009,7 @@
       <c r="G3" s="87" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="345"/>
+      <c r="H3" s="346"/>
       <c r="I3" s="87" t="s">
         <v>224</v>
       </c>
@@ -12037,11 +12040,11 @@
       <c r="R3" s="87" t="s">
         <v>159</v>
       </c>
-      <c r="S3" s="345"/>
+      <c r="S3" s="346"/>
       <c r="T3" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="U3" s="345"/>
+      <c r="U3" s="346"/>
       <c r="V3" s="87" t="s">
         <v>215</v>
       </c>
@@ -12069,7 +12072,7 @@
       <c r="AD3" s="87" t="s">
         <v>207</v>
       </c>
-      <c r="AE3" s="345"/>
+      <c r="AE3" s="346"/>
       <c r="AF3" s="87" t="s">
         <v>206</v>
       </c>
@@ -12079,7 +12082,7 @@
       <c r="AH3" s="87" t="s">
         <v>136</v>
       </c>
-      <c r="AI3" s="345"/>
+      <c r="AI3" s="346"/>
     </row>
     <row r="4" spans="1:62" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="90"/>
@@ -12101,7 +12104,7 @@
       <c r="G4" s="87" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="345"/>
+      <c r="H4" s="346"/>
       <c r="I4" s="87" t="s">
         <v>205</v>
       </c>
@@ -12132,11 +12135,11 @@
       <c r="R4" s="87" t="s">
         <v>108</v>
       </c>
-      <c r="S4" s="345"/>
+      <c r="S4" s="346"/>
       <c r="T4" s="87" t="s">
         <v>104</v>
       </c>
-      <c r="U4" s="345"/>
+      <c r="U4" s="346"/>
       <c r="V4" s="87" t="s">
         <v>196</v>
       </c>
@@ -12164,7 +12167,7 @@
       <c r="AD4" s="87" t="s">
         <v>188</v>
       </c>
-      <c r="AE4" s="345"/>
+      <c r="AE4" s="346"/>
       <c r="AF4" s="87" t="s">
         <v>187</v>
       </c>
@@ -12174,7 +12177,7 @@
       <c r="AH4" s="87" t="s">
         <v>83</v>
       </c>
-      <c r="AI4" s="345"/>
+      <c r="AI4" s="346"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="93" t="s">
@@ -13926,13 +13929,13 @@
       <c r="G2" s="87" t="s">
         <v>181</v>
       </c>
-      <c r="H2" s="345" t="s">
+      <c r="H2" s="346" t="s">
         <v>180</v>
       </c>
       <c r="I2" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="J2" s="345" t="s">
+      <c r="J2" s="346" t="s">
         <v>179</v>
       </c>
     </row>
@@ -13946,11 +13949,11 @@
       <c r="G3" s="87" t="s">
         <v>159</v>
       </c>
-      <c r="H3" s="345"/>
+      <c r="H3" s="346"/>
       <c r="I3" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="J3" s="345"/>
+      <c r="J3" s="346"/>
     </row>
     <row r="4" spans="1:62" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="109"/>
@@ -13972,11 +13975,11 @@
       <c r="G4" s="87" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="345"/>
+      <c r="H4" s="346"/>
       <c r="I4" s="87" t="s">
         <v>104</v>
       </c>
-      <c r="J4" s="345"/>
+      <c r="J4" s="346"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="103" t="s">
@@ -14363,13 +14366,13 @@
   <sheetData>
     <row r="1" spans="1:61" s="168" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="167"/>
-      <c r="B1" s="349" t="s">
+      <c r="B1" s="350" t="s">
         <v>184</v>
       </c>
-      <c r="C1" s="349"/>
-      <c r="D1" s="349"/>
-      <c r="E1" s="349"/>
-      <c r="F1" s="349"/>
+      <c r="C1" s="350"/>
+      <c r="D1" s="350"/>
+      <c r="E1" s="350"/>
+      <c r="F1" s="350"/>
       <c r="G1" s="169"/>
       <c r="H1" s="169"/>
       <c r="I1" s="169"/>
@@ -14414,7 +14417,7 @@
       <c r="O2" s="171" t="s">
         <v>178</v>
       </c>
-      <c r="P2" s="348" t="s">
+      <c r="P2" s="349" t="s">
         <v>177</v>
       </c>
       <c r="Q2" s="171" t="s">
@@ -14456,7 +14459,7 @@
       <c r="AC2" s="171" t="s">
         <v>176</v>
       </c>
-      <c r="AD2" s="348" t="s">
+      <c r="AD2" s="349" t="s">
         <v>175</v>
       </c>
       <c r="AE2" s="172" t="s">
@@ -14486,7 +14489,7 @@
       <c r="AM2" s="172" t="s">
         <v>174</v>
       </c>
-      <c r="AN2" s="348" t="s">
+      <c r="AN2" s="349" t="s">
         <v>173</v>
       </c>
       <c r="AQ2" s="171"/>
@@ -14497,7 +14500,7 @@
       <c r="AV2" s="171"/>
       <c r="AW2" s="171"/>
       <c r="AX2" s="171"/>
-      <c r="AY2" s="348"/>
+      <c r="AY2" s="349"/>
       <c r="AZ2" s="172"/>
       <c r="BA2" s="172"/>
       <c r="BB2" s="172"/>
@@ -14507,7 +14510,7 @@
       <c r="BF2" s="172"/>
       <c r="BG2" s="172"/>
       <c r="BH2" s="172"/>
-      <c r="BI2" s="348"/>
+      <c r="BI2" s="349"/>
     </row>
     <row r="3" spans="1:61" s="168" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="170"/>
@@ -14543,7 +14546,7 @@
       <c r="O3" s="171" t="s">
         <v>149</v>
       </c>
-      <c r="P3" s="348"/>
+      <c r="P3" s="349"/>
       <c r="Q3" s="171" t="s">
         <v>148</v>
       </c>
@@ -14583,7 +14586,7 @@
       <c r="AC3" s="171" t="s">
         <v>136</v>
       </c>
-      <c r="AD3" s="348"/>
+      <c r="AD3" s="349"/>
       <c r="AE3" s="172" t="s">
         <v>135</v>
       </c>
@@ -14611,7 +14614,7 @@
       <c r="AM3" s="172" t="s">
         <v>127</v>
       </c>
-      <c r="AN3" s="348"/>
+      <c r="AN3" s="349"/>
       <c r="AQ3" s="171"/>
       <c r="AR3" s="171"/>
       <c r="AS3" s="171"/>
@@ -14620,7 +14623,7 @@
       <c r="AV3" s="171"/>
       <c r="AW3" s="171"/>
       <c r="AX3" s="171"/>
-      <c r="AY3" s="348"/>
+      <c r="AY3" s="349"/>
       <c r="AZ3" s="172"/>
       <c r="BA3" s="172"/>
       <c r="BB3" s="172"/>
@@ -14630,7 +14633,7 @@
       <c r="BF3" s="172"/>
       <c r="BG3" s="172"/>
       <c r="BH3" s="172"/>
-      <c r="BI3" s="348"/>
+      <c r="BI3" s="349"/>
     </row>
     <row r="4" spans="1:61" s="168" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="173"/>
@@ -14676,7 +14679,7 @@
       <c r="O4" s="171" t="s">
         <v>96</v>
       </c>
-      <c r="P4" s="348"/>
+      <c r="P4" s="349"/>
       <c r="Q4" s="171" t="s">
         <v>95</v>
       </c>
@@ -14716,7 +14719,7 @@
       <c r="AC4" s="171" t="s">
         <v>83</v>
       </c>
-      <c r="AD4" s="348"/>
+      <c r="AD4" s="349"/>
       <c r="AE4" s="172" t="s">
         <v>82</v>
       </c>
@@ -14744,7 +14747,7 @@
       <c r="AM4" s="172" t="s">
         <v>74</v>
       </c>
-      <c r="AN4" s="348"/>
+      <c r="AN4" s="349"/>
       <c r="AQ4" s="171"/>
       <c r="AR4" s="171"/>
       <c r="AS4" s="171"/>
@@ -14753,7 +14756,7 @@
       <c r="AV4" s="171"/>
       <c r="AW4" s="171"/>
       <c r="AX4" s="171"/>
-      <c r="AY4" s="348"/>
+      <c r="AY4" s="349"/>
       <c r="AZ4" s="172"/>
       <c r="BA4" s="172"/>
       <c r="BB4" s="172"/>
@@ -14763,7 +14766,7 @@
       <c r="BF4" s="172"/>
       <c r="BG4" s="172"/>
       <c r="BH4" s="172"/>
-      <c r="BI4" s="348"/>
+      <c r="BI4" s="349"/>
     </row>
     <row r="5" spans="1:61" s="168" customFormat="1" ht="144" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="175" t="s">
@@ -16485,14 +16488,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="350" t="s">
+      <c r="A1" s="351" t="s">
         <v>228</v>
       </c>
-      <c r="B1" s="350"/>
-      <c r="C1" s="350"/>
-      <c r="D1" s="350"/>
-      <c r="E1" s="350"/>
-      <c r="F1" s="350"/>
+      <c r="B1" s="351"/>
+      <c r="C1" s="351"/>
+      <c r="D1" s="351"/>
+      <c r="E1" s="351"/>
+      <c r="F1" s="351"/>
       <c r="G1" s="200"/>
       <c r="H1" s="200"/>
       <c r="I1" s="200"/>
@@ -16542,7 +16545,7 @@
       <c r="O2" s="203" t="s">
         <v>178</v>
       </c>
-      <c r="P2" s="351" t="s">
+      <c r="P2" s="352" t="s">
         <v>227</v>
       </c>
       <c r="Q2" s="203" t="s">
@@ -16554,7 +16557,7 @@
       <c r="S2" s="203" t="s">
         <v>226</v>
       </c>
-      <c r="T2" s="351" t="s">
+      <c r="T2" s="352" t="s">
         <v>225</v>
       </c>
     </row>
@@ -16592,7 +16595,7 @@
       <c r="O3" s="203" t="s">
         <v>207</v>
       </c>
-      <c r="P3" s="351"/>
+      <c r="P3" s="352"/>
       <c r="Q3" s="203" t="s">
         <v>206</v>
       </c>
@@ -16602,7 +16605,7 @@
       <c r="S3" s="203" t="s">
         <v>136</v>
       </c>
-      <c r="T3" s="351"/>
+      <c r="T3" s="352"/>
     </row>
     <row r="4" spans="1:20" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="202"/>
@@ -16648,7 +16651,7 @@
       <c r="O4" s="203" t="s">
         <v>188</v>
       </c>
-      <c r="P4" s="351"/>
+      <c r="P4" s="352"/>
       <c r="Q4" s="203" t="s">
         <v>187</v>
       </c>
@@ -16658,7 +16661,7 @@
       <c r="S4" s="203" t="s">
         <v>83</v>
       </c>
-      <c r="T4" s="351"/>
+      <c r="T4" s="352"/>
     </row>
     <row r="5" spans="1:20" ht="317" x14ac:dyDescent="0.2">
       <c r="A5" s="206" t="s">
@@ -17244,16 +17247,16 @@
   <sheetData>
     <row r="1" spans="1:28" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="226"/>
-      <c r="B1" s="353" t="s">
+      <c r="B1" s="354" t="s">
         <v>184</v>
       </c>
-      <c r="C1" s="353"/>
-      <c r="D1" s="353"/>
-      <c r="E1" s="353"/>
-      <c r="F1" s="353"/>
-      <c r="G1" s="353"/>
-      <c r="H1" s="353"/>
-      <c r="I1" s="353"/>
+      <c r="C1" s="354"/>
+      <c r="D1" s="354"/>
+      <c r="E1" s="354"/>
+      <c r="F1" s="354"/>
+      <c r="G1" s="354"/>
+      <c r="H1" s="354"/>
+      <c r="I1" s="354"/>
       <c r="J1" s="223"/>
       <c r="K1" s="223"/>
       <c r="L1" s="223"/>
@@ -17284,7 +17287,7 @@
       <c r="G2" s="225" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="352" t="s">
+      <c r="H2" s="353" t="s">
         <v>182</v>
       </c>
       <c r="I2" s="228" t="s">
@@ -17329,7 +17332,7 @@
       <c r="V2" s="228" t="s">
         <v>181</v>
       </c>
-      <c r="W2" s="352" t="s">
+      <c r="W2" s="353" t="s">
         <v>180</v>
       </c>
       <c r="X2" s="225" t="s">
@@ -17344,7 +17347,7 @@
       <c r="AA2" s="225" t="s">
         <v>45</v>
       </c>
-      <c r="AB2" s="352" t="s">
+      <c r="AB2" s="353" t="s">
         <v>179</v>
       </c>
     </row>
@@ -17358,7 +17361,7 @@
       <c r="G3" s="225" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="352"/>
+      <c r="H3" s="353"/>
       <c r="I3" s="228" t="s">
         <v>171</v>
       </c>
@@ -17399,7 +17402,7 @@
       <c r="V3" s="228" t="s">
         <v>159</v>
       </c>
-      <c r="W3" s="352"/>
+      <c r="W3" s="353"/>
       <c r="X3" s="227"/>
       <c r="Y3" s="225" t="s">
         <v>158</v>
@@ -17410,7 +17413,7 @@
       <c r="AA3" s="225" t="s">
         <v>156</v>
       </c>
-      <c r="AB3" s="352"/>
+      <c r="AB3" s="353"/>
     </row>
     <row r="4" spans="1:28" ht="98" x14ac:dyDescent="0.2">
       <c r="A4" s="229"/>
@@ -17432,7 +17435,7 @@
       <c r="G4" s="225" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="352"/>
+      <c r="H4" s="353"/>
       <c r="I4" s="228" t="s">
         <v>121</v>
       </c>
@@ -17475,7 +17478,7 @@
       <c r="V4" s="231" t="s">
         <v>108</v>
       </c>
-      <c r="W4" s="352"/>
+      <c r="W4" s="353"/>
       <c r="X4" s="232" t="s">
         <v>107</v>
       </c>
@@ -17488,7 +17491,7 @@
       <c r="AA4" s="232" t="s">
         <v>104</v>
       </c>
-      <c r="AB4" s="352"/>
+      <c r="AB4" s="353"/>
     </row>
     <row r="5" spans="1:28" ht="196" x14ac:dyDescent="0.2">
       <c r="A5" s="233" t="s">
@@ -18382,16 +18385,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="355" t="s">
+      <c r="A1" s="356" t="s">
         <v>228</v>
       </c>
-      <c r="B1" s="355"/>
-      <c r="C1" s="355"/>
-      <c r="D1" s="355"/>
-      <c r="E1" s="355"/>
-      <c r="F1" s="355"/>
-      <c r="G1" s="355"/>
-      <c r="H1" s="355"/>
+      <c r="B1" s="356"/>
+      <c r="C1" s="356"/>
+      <c r="D1" s="356"/>
+      <c r="E1" s="356"/>
+      <c r="F1" s="356"/>
+      <c r="G1" s="356"/>
+      <c r="H1" s="356"/>
       <c r="I1" s="273"/>
       <c r="J1" s="273"/>
       <c r="K1" s="273"/>
@@ -18416,7 +18419,7 @@
       <c r="G2" s="275" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="354" t="s">
+      <c r="H2" s="355" t="s">
         <v>182</v>
       </c>
       <c r="I2" s="275" t="s">
@@ -18449,13 +18452,13 @@
       <c r="R2" s="275" t="s">
         <v>181</v>
       </c>
-      <c r="S2" s="354" t="s">
+      <c r="S2" s="355" t="s">
         <v>180</v>
       </c>
       <c r="T2" s="275" t="s">
         <v>45</v>
       </c>
-      <c r="U2" s="354" t="s">
+      <c r="U2" s="355" t="s">
         <v>179</v>
       </c>
     </row>
@@ -18469,7 +18472,7 @@
       <c r="G3" s="275" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="354"/>
+      <c r="H3" s="355"/>
       <c r="I3" s="275" t="s">
         <v>224</v>
       </c>
@@ -18500,11 +18503,11 @@
       <c r="R3" s="275" t="s">
         <v>159</v>
       </c>
-      <c r="S3" s="354"/>
+      <c r="S3" s="355"/>
       <c r="T3" s="275" t="s">
         <v>156</v>
       </c>
-      <c r="U3" s="354"/>
+      <c r="U3" s="355"/>
     </row>
     <row r="4" spans="1:21" ht="112" x14ac:dyDescent="0.2">
       <c r="A4" s="272"/>
@@ -18526,7 +18529,7 @@
       <c r="G4" s="275" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="354"/>
+      <c r="H4" s="355"/>
       <c r="I4" s="275" t="s">
         <v>205</v>
       </c>
@@ -18557,11 +18560,11 @@
       <c r="R4" s="275" t="s">
         <v>108</v>
       </c>
-      <c r="S4" s="354"/>
+      <c r="S4" s="355"/>
       <c r="T4" s="275" t="s">
         <v>104</v>
       </c>
-      <c r="U4" s="354"/>
+      <c r="U4" s="355"/>
     </row>
     <row r="5" spans="1:21" ht="196" x14ac:dyDescent="0.2">
       <c r="A5" s="278" t="s">
@@ -19252,13 +19255,13 @@
       <c r="K2" s="203" t="s">
         <v>181</v>
       </c>
-      <c r="L2" s="351" t="s">
+      <c r="L2" s="352" t="s">
         <v>180</v>
       </c>
       <c r="M2" s="203" t="s">
         <v>45</v>
       </c>
-      <c r="N2" s="351" t="s">
+      <c r="N2" s="352" t="s">
         <v>179</v>
       </c>
     </row>
@@ -19276,11 +19279,11 @@
       <c r="K3" s="203" t="s">
         <v>159</v>
       </c>
-      <c r="L3" s="351"/>
+      <c r="L3" s="352"/>
       <c r="M3" s="203" t="s">
         <v>156</v>
       </c>
-      <c r="N3" s="351"/>
+      <c r="N3" s="352"/>
     </row>
     <row r="4" spans="1:14" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="256"/>
@@ -19306,11 +19309,11 @@
       <c r="K4" s="203" t="s">
         <v>108</v>
       </c>
-      <c r="L4" s="351"/>
+      <c r="L4" s="352"/>
       <c r="M4" s="203" t="s">
         <v>104</v>
       </c>
-      <c r="N4" s="351"/>
+      <c r="N4" s="352"/>
     </row>
     <row r="5" spans="1:14" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="258"/>
@@ -19962,7 +19965,7 @@
   <sheetPr codeName="Feuil13">
     <tabColor rgb="FF2C45E0"/>
   </sheetPr>
-  <dimension ref="A1:FI4"/>
+  <dimension ref="A1:FJ4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.6640625" customWidth="1"/>
@@ -19975,11 +19978,11 @@
     <col min="157" max="157" width="60.6640625" bestFit="1" customWidth="1"/>
     <col min="161" max="161" width="52" bestFit="1" customWidth="1"/>
     <col min="162" max="162" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="169" max="169" width="45.1640625" bestFit="1" customWidth="1"/>
-    <col min="170" max="170" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="170" max="170" width="45.1640625" bestFit="1" customWidth="1"/>
+    <col min="171" max="171" width="15.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:165" s="4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:166" s="4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>232</v>
       </c>
@@ -19999,13 +20002,14 @@
       <c r="FD1" s="338"/>
       <c r="FE1" s="338"/>
       <c r="FF1" s="338"/>
-      <c r="FG1" s="356"/>
-      <c r="FH1" s="356"/>
-      <c r="FI1" s="4" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:165" ht="66" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="FG1" s="339"/>
+      <c r="FH1" s="339"/>
+      <c r="FI1" s="339"/>
+      <c r="FJ1" s="4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:166" ht="66" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="22" t="s">
         <v>8</v>
       </c>
@@ -20031,13 +20035,16 @@
         <v>39</v>
       </c>
       <c r="FG2" s="126" t="s">
+        <v>437</v>
+      </c>
+      <c r="FH2" s="126" t="s">
         <v>435</v>
       </c>
-      <c r="FH2" s="126" t="s">
+      <c r="FI2" s="126" t="s">
         <v>436</v>
       </c>
     </row>
-    <row r="3" spans="1:165" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:166" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="s">
         <v>11</v>
       </c>
@@ -20045,7 +20052,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:165" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:166" x14ac:dyDescent="0.2">
       <c r="B4" s="27" t="s">
         <v>7</v>
       </c>
@@ -20054,7 +20061,7 @@
   </sheetData>
   <autoFilter ref="A2:DT2" xr:uid="{3B89445B-6ECC-4440-B85C-E593AE209933}"/>
   <mergeCells count="1">
-    <mergeCell ref="FA1:FH1"/>
+    <mergeCell ref="FA1:FI1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -20144,28 +20151,28 @@
       <c r="D4" s="294"/>
       <c r="E4" s="294"/>
       <c r="F4" s="294"/>
-      <c r="G4" s="339" t="s">
+      <c r="G4" s="340" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="340"/>
-      <c r="I4" s="340"/>
-      <c r="J4" s="340"/>
-      <c r="K4" s="340"/>
-      <c r="L4" s="341"/>
-      <c r="M4" s="342"/>
-      <c r="N4" s="343" t="s">
+      <c r="H4" s="341"/>
+      <c r="I4" s="341"/>
+      <c r="J4" s="341"/>
+      <c r="K4" s="341"/>
+      <c r="L4" s="342"/>
+      <c r="M4" s="343"/>
+      <c r="N4" s="344" t="s">
         <v>27</v>
       </c>
-      <c r="O4" s="341"/>
-      <c r="P4" s="341"/>
-      <c r="Q4" s="341"/>
-      <c r="R4" s="341"/>
-      <c r="S4" s="341"/>
-      <c r="T4" s="344"/>
-      <c r="U4" s="339" t="s">
+      <c r="O4" s="342"/>
+      <c r="P4" s="342"/>
+      <c r="Q4" s="342"/>
+      <c r="R4" s="342"/>
+      <c r="S4" s="342"/>
+      <c r="T4" s="345"/>
+      <c r="U4" s="340" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="342"/>
+      <c r="V4" s="343"/>
       <c r="W4" s="301"/>
       <c r="X4" t="s">
         <v>0</v>
@@ -20243,7 +20250,7 @@
         <v>399</v>
       </c>
       <c r="G6" s="19" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"M-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="H6" s="298" t="str">
@@ -20251,11 +20258,11 @@
         <v/>
       </c>
       <c r="I6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"M-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="J6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"M-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"M-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="K6" s="18" t="e">
@@ -20263,7 +20270,7 @@
 INDEX('ETPT Format DDG'!$A:$DU,
 ,
 IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
-),'ETPT Format DDG'!$I:$I,"C",
+),'ETPT Format DDG'!$FG:$FG,"C",
 'ETPT Format DDG'!$C:$C,$A$3,
 'ETPT Format DDG'!$G:$G,"Magistrat")</f>
         <v>#N/A</v>
@@ -20283,7 +20290,7 @@
         <v/>
       </c>
       <c r="N6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"F-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"F-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="O6" s="298" t="str">
@@ -20291,15 +20298,15 @@
         <v/>
       </c>
       <c r="P6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"F-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"F-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="Q6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"F-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"F-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="R6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$I:$I,"C",'ETPT Format DDG'!$C:$C,$A$3,'ETPT Format DDG'!$G:$G,"Greffe")</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"C",'ETPT Format DDG'!$C:$C,$A$3,'ETPT Format DDG'!$G:$G,"Greffe")</f>
         <v>#N/A</v>
       </c>
       <c r="S6" s="19" t="e">
@@ -20321,7 +20328,7 @@
 INDEX('ETPT Format DDG'!$A:$DU,
 ,
 IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
-),'ETPT Format DDG'!$I:$I,"C",
+),'ETPT Format DDG'!$FG:$FG,"C",
 'ETPT Format DDG'!$C:$C,$A$3,
 'ETPT Format DDG'!$G:$G,"Autour du magistrat")</f>
         <v>#N/A</v>
@@ -20744,16 +20751,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:62" s="44" customFormat="1" ht="23.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B1" s="346" t="s">
+      <c r="B1" s="347" t="s">
         <v>184</v>
       </c>
-      <c r="C1" s="346"/>
-      <c r="D1" s="346"/>
-      <c r="E1" s="346"/>
-      <c r="F1" s="346"/>
-      <c r="G1" s="346"/>
-      <c r="H1" s="346"/>
-      <c r="I1" s="346"/>
+      <c r="C1" s="347"/>
+      <c r="D1" s="347"/>
+      <c r="E1" s="347"/>
+      <c r="F1" s="347"/>
+      <c r="G1" s="347"/>
+      <c r="H1" s="347"/>
+      <c r="I1" s="347"/>
     </row>
     <row r="2" spans="1:62" s="44" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="90"/>
@@ -20765,7 +20772,7 @@
       <c r="G2" s="87" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="345" t="s">
+      <c r="H2" s="346" t="s">
         <v>182</v>
       </c>
       <c r="I2" s="86" t="s">
@@ -20810,7 +20817,7 @@
       <c r="V2" s="86" t="s">
         <v>181</v>
       </c>
-      <c r="W2" s="345" t="s">
+      <c r="W2" s="346" t="s">
         <v>180</v>
       </c>
       <c r="X2" s="87" t="s">
@@ -20825,7 +20832,7 @@
       <c r="AA2" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="AB2" s="345" t="s">
+      <c r="AB2" s="346" t="s">
         <v>179</v>
       </c>
       <c r="AC2" s="84" t="s">
@@ -20855,7 +20862,7 @@
       <c r="AK2" s="84" t="s">
         <v>178</v>
       </c>
-      <c r="AL2" s="345" t="s">
+      <c r="AL2" s="346" t="s">
         <v>177</v>
       </c>
       <c r="AM2" s="84" t="s">
@@ -20897,7 +20904,7 @@
       <c r="AY2" s="84" t="s">
         <v>176</v>
       </c>
-      <c r="AZ2" s="345" t="s">
+      <c r="AZ2" s="346" t="s">
         <v>175</v>
       </c>
       <c r="BA2" s="83" t="s">
@@ -20927,7 +20934,7 @@
       <c r="BI2" s="83" t="s">
         <v>174</v>
       </c>
-      <c r="BJ2" s="345" t="s">
+      <c r="BJ2" s="346" t="s">
         <v>173</v>
       </c>
     </row>
@@ -20941,7 +20948,7 @@
       <c r="G3" s="87" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="345"/>
+      <c r="H3" s="346"/>
       <c r="I3" s="86" t="s">
         <v>171</v>
       </c>
@@ -20982,7 +20989,7 @@
       <c r="V3" s="86" t="s">
         <v>159</v>
       </c>
-      <c r="W3" s="345"/>
+      <c r="W3" s="346"/>
       <c r="X3" s="82"/>
       <c r="Y3" s="87" t="s">
         <v>158</v>
@@ -20993,7 +21000,7 @@
       <c r="AA3" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="AB3" s="345"/>
+      <c r="AB3" s="346"/>
       <c r="AC3" s="84" t="s">
         <v>155</v>
       </c>
@@ -21021,7 +21028,7 @@
       <c r="AK3" s="84" t="s">
         <v>149</v>
       </c>
-      <c r="AL3" s="345"/>
+      <c r="AL3" s="346"/>
       <c r="AM3" s="84" t="s">
         <v>148</v>
       </c>
@@ -21061,7 +21068,7 @@
       <c r="AY3" s="84" t="s">
         <v>136</v>
       </c>
-      <c r="AZ3" s="345"/>
+      <c r="AZ3" s="346"/>
       <c r="BA3" s="83" t="s">
         <v>135</v>
       </c>
@@ -21089,7 +21096,7 @@
       <c r="BI3" s="83" t="s">
         <v>127</v>
       </c>
-      <c r="BJ3" s="345"/>
+      <c r="BJ3" s="346"/>
     </row>
     <row r="4" spans="1:62" s="44" customFormat="1" ht="60" x14ac:dyDescent="0.15">
       <c r="A4" s="89"/>
@@ -21111,7 +21118,7 @@
       <c r="G4" s="87" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="345"/>
+      <c r="H4" s="346"/>
       <c r="I4" s="86" t="s">
         <v>121</v>
       </c>
@@ -21154,7 +21161,7 @@
       <c r="V4" s="86" t="s">
         <v>108</v>
       </c>
-      <c r="W4" s="345"/>
+      <c r="W4" s="346"/>
       <c r="X4" s="85" t="s">
         <v>107</v>
       </c>
@@ -21167,7 +21174,7 @@
       <c r="AA4" s="85" t="s">
         <v>104</v>
       </c>
-      <c r="AB4" s="345"/>
+      <c r="AB4" s="346"/>
       <c r="AC4" s="84" t="s">
         <v>103</v>
       </c>
@@ -21195,7 +21202,7 @@
       <c r="AK4" s="84" t="s">
         <v>96</v>
       </c>
-      <c r="AL4" s="345"/>
+      <c r="AL4" s="346"/>
       <c r="AM4" s="84" t="s">
         <v>95</v>
       </c>
@@ -21235,7 +21242,7 @@
       <c r="AY4" s="84" t="s">
         <v>83</v>
       </c>
-      <c r="AZ4" s="345"/>
+      <c r="AZ4" s="346"/>
       <c r="BA4" s="83" t="s">
         <v>82</v>
       </c>
@@ -21263,7 +21270,7 @@
       <c r="BI4" s="83" t="s">
         <v>74</v>
       </c>
-      <c r="BJ4" s="345"/>
+      <c r="BJ4" s="346"/>
     </row>
     <row r="5" spans="1:62" s="44" customFormat="1" ht="11" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="54" t="s">
@@ -23452,16 +23459,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A1" s="347" t="s">
+      <c r="A1" s="348" t="s">
         <v>228</v>
       </c>
-      <c r="B1" s="347"/>
-      <c r="C1" s="347"/>
-      <c r="D1" s="347"/>
-      <c r="E1" s="347"/>
-      <c r="F1" s="347"/>
-      <c r="G1" s="347"/>
-      <c r="H1" s="347"/>
+      <c r="B1" s="348"/>
+      <c r="C1" s="348"/>
+      <c r="D1" s="348"/>
+      <c r="E1" s="348"/>
+      <c r="F1" s="348"/>
+      <c r="G1" s="348"/>
+      <c r="H1" s="348"/>
       <c r="I1" s="44"/>
       <c r="J1" s="44"/>
       <c r="K1" s="44"/>
@@ -23500,7 +23507,7 @@
       <c r="G2" s="87" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="345" t="s">
+      <c r="H2" s="346" t="s">
         <v>182</v>
       </c>
       <c r="I2" s="87" t="s">
@@ -23533,13 +23540,13 @@
       <c r="R2" s="87" t="s">
         <v>181</v>
       </c>
-      <c r="S2" s="345" t="s">
+      <c r="S2" s="346" t="s">
         <v>180</v>
       </c>
       <c r="T2" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="U2" s="345" t="s">
+      <c r="U2" s="346" t="s">
         <v>179</v>
       </c>
       <c r="V2" s="87" t="s">
@@ -23569,7 +23576,7 @@
       <c r="AD2" s="87" t="s">
         <v>178</v>
       </c>
-      <c r="AE2" s="345" t="s">
+      <c r="AE2" s="346" t="s">
         <v>227</v>
       </c>
       <c r="AF2" s="87" t="s">
@@ -23581,7 +23588,7 @@
       <c r="AH2" s="87" t="s">
         <v>226</v>
       </c>
-      <c r="AI2" s="345" t="s">
+      <c r="AI2" s="346" t="s">
         <v>225</v>
       </c>
     </row>
@@ -23595,7 +23602,7 @@
       <c r="G3" s="87" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="345"/>
+      <c r="H3" s="346"/>
       <c r="I3" s="87" t="s">
         <v>224</v>
       </c>
@@ -23626,11 +23633,11 @@
       <c r="R3" s="87" t="s">
         <v>159</v>
       </c>
-      <c r="S3" s="345"/>
+      <c r="S3" s="346"/>
       <c r="T3" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="U3" s="345"/>
+      <c r="U3" s="346"/>
       <c r="V3" s="87" t="s">
         <v>215</v>
       </c>
@@ -23658,7 +23665,7 @@
       <c r="AD3" s="87" t="s">
         <v>207</v>
       </c>
-      <c r="AE3" s="345"/>
+      <c r="AE3" s="346"/>
       <c r="AF3" s="87" t="s">
         <v>206</v>
       </c>
@@ -23668,7 +23675,7 @@
       <c r="AH3" s="87" t="s">
         <v>136</v>
       </c>
-      <c r="AI3" s="345"/>
+      <c r="AI3" s="346"/>
     </row>
     <row r="4" spans="1:35" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="90"/>
@@ -23690,7 +23697,7 @@
       <c r="G4" s="87" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="345"/>
+      <c r="H4" s="346"/>
       <c r="I4" s="87" t="s">
         <v>205</v>
       </c>
@@ -23721,11 +23728,11 @@
       <c r="R4" s="87" t="s">
         <v>108</v>
       </c>
-      <c r="S4" s="345"/>
+      <c r="S4" s="346"/>
       <c r="T4" s="87" t="s">
         <v>104</v>
       </c>
-      <c r="U4" s="345"/>
+      <c r="U4" s="346"/>
       <c r="V4" s="87" t="s">
         <v>196</v>
       </c>
@@ -23753,7 +23760,7 @@
       <c r="AD4" s="87" t="s">
         <v>188</v>
       </c>
-      <c r="AE4" s="345"/>
+      <c r="AE4" s="346"/>
       <c r="AF4" s="87" t="s">
         <v>187</v>
       </c>
@@ -23763,7 +23770,7 @@
       <c r="AH4" s="87" t="s">
         <v>83</v>
       </c>
-      <c r="AI4" s="345"/>
+      <c r="AI4" s="346"/>
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A5" s="93" t="s">

</xml_diff>

<commit_message>
update extractor CA Indispo counter
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7302EF8-8DE6-1A43-8AD2-8669F817114E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D77EB23-DE49-7A4C-AAEA-EFF1BADE4F3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" activeTab="3" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -7156,7 +7156,3047 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
     <cellStyle name="Normal 3" xfId="4" xr:uid="{6BD57324-3FD5-D341-A299-730D14794802}"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="314">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -20437,45 +23477,71 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="9" priority="10">
+    <cfRule type="expression" dxfId="31" priority="16">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="8" priority="12">
+    <cfRule type="expression" dxfId="30" priority="18">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="7" priority="1">
-      <formula>AND($D1="5. TOTAL JLD CIVIL",OR(_xlfn.NUMBERVALUE($L1-$L2-$L3)-_xlfn.NUMBERVALUE($L4)&lt;&gt;0,_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)&lt;&gt;0,_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)&lt;&gt;0))</formula>
+    <cfRule type="expression" dxfId="16" priority="7">
+      <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3)-_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)-_xlfn.NUMBERVALUE($L6)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="6">
+    <cfRule type="expression" dxfId="29" priority="12">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",OR(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3)&lt;&gt;0,_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)&lt;&gt;0,_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)&lt;&gt;0))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="28" priority="2">
+      <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)&lt;&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="27" priority="1" stopIfTrue="1">
+      <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)&lt;&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D7:F7">
+    <cfRule type="expression" dxfId="26" priority="6">
+      <formula>OR(_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6),_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6),_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="5" priority="5">
-      <formula>AND($D1="5. TOTAL JLD CIVIL",_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3)-_xlfn.NUMBERVALUE($L4)&lt;&gt;0)</formula>
+    <cfRule type="expression" dxfId="25" priority="11" stopIfTrue="1">
+      <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3)-_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="9">
+    <cfRule type="expression" dxfId="24" priority="15" stopIfTrue="1">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G7:M7">
+    <cfRule type="expression" dxfId="23" priority="5">
+      <formula>_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="3" priority="4">
-      <formula>AND($D1="5. TOTAL JLD CIVIL",_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)&lt;&gt;0)</formula>
+    <cfRule type="expression" dxfId="22" priority="10" stopIfTrue="1">
+      <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="8">
+    <cfRule type="expression" dxfId="21" priority="14" stopIfTrue="1">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="N7:T7">
+    <cfRule type="expression" dxfId="20" priority="4">
+      <formula>_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="1" priority="3">
-      <formula>AND($D1="5. TOTAL JLD CIVIL",_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)&lt;&gt;0)</formula>
+    <cfRule type="expression" dxfId="19" priority="9" stopIfTrue="1">
+      <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="7">
+    <cfRule type="expression" dxfId="18" priority="13" stopIfTrue="1">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)&lt;&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U7:V7">
+    <cfRule type="expression" dxfId="17" priority="3">
+      <formula>_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
update validation conditionnelle agregats
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D77EB23-DE49-7A4C-AAEA-EFF1BADE4F3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E3095B4-999B-FB46-9889-DD77E8729181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" activeTab="3" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -7156,7 +7156,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
     <cellStyle name="Normal 3" xfId="4" xr:uid="{6BD57324-3FD5-D341-A299-730D14794802}"/>
   </cellStyles>
-  <dxfs count="314">
+  <dxfs count="240">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -8878,6 +8878,26 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill>
           <fgColor theme="5" tint="0.79998168889431442"/>
@@ -8896,6 +8916,26 @@
       <font>
         <color theme="0"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -9158,6 +9198,26 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill>
           <fgColor theme="5" tint="0.79998168889431442"/>
@@ -9176,6 +9236,26 @@
       <font>
         <color theme="0"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -9336,826 +9416,6 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -23384,13 +22644,13 @@
         <v>#N/A</v>
       </c>
       <c r="L6" s="19" t="e">
-        <f>SUMIFS(
+        <f>ROUND(SUMIFS(
 INDEX('ETPT Format DDG'!$A:$DU,
 ,
 IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
 ),
 'ETPT Format DDG'!$C:$C,$A$3,
-'ETPT Format DDG'!$G:$G,"Magistrat")</f>
+'ETPT Format DDG'!$G:$G,"Magistrat"),3)</f>
         <v>#N/A</v>
       </c>
       <c r="M6" s="299" t="str">
@@ -23418,13 +22678,13 @@
         <v>#N/A</v>
       </c>
       <c r="S6" s="19" t="e">
-        <f>SUMIFS(
+        <f>ROUND(SUMIFS(
 INDEX('ETPT Format DDG'!$A:$DU,
 ,
 IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
 ),
 'ETPT Format DDG'!$C:$C,$A$3,
-'ETPT Format DDG'!$G:$G,"Greffe")</f>
+'ETPT Format DDG'!$G:$G,"Greffe"),3)</f>
         <v>#N/A</v>
       </c>
       <c r="T6" s="298" t="str">
@@ -23432,13 +22692,13 @@
         <v/>
       </c>
       <c r="U6" s="19" t="e">
-        <f>SUMIFS(
+        <f>ROUND(SUMIFS(
 INDEX('ETPT Format DDG'!$A:$DU,
 ,
 IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
 ),'ETPT Format DDG'!$FG:$FG,"C",
 'ETPT Format DDG'!$C:$C,$A$3,
-'ETPT Format DDG'!$G:$G,"Autour du magistrat")</f>
+'ETPT Format DDG'!$G:$G,"Autour du magistrat"),3)</f>
         <v>#N/A</v>
       </c>
       <c r="V6" s="299" t="str">
@@ -23487,60 +22747,60 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="16" priority="7">
-      <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3)-_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)-_xlfn.NUMBERVALUE($L6)&lt;&gt;0)</formula>
+    <cfRule type="expression" dxfId="16" priority="1" stopIfTrue="1">
+      <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3)+_xlfn.NUMBERVALUE($U4)+_xlfn.NUMBERVALUE($U5)+_xlfn.NUMBERVALUE($U6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="29" priority="12">
-      <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",OR(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3)&lt;&gt;0,_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)&lt;&gt;0,_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)&lt;&gt;0))</formula>
+    <cfRule type="expression" dxfId="17" priority="2" stopIfTrue="1">
+      <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3)+_xlfn.NUMBERVALUE($S4)+_xlfn.NUMBERVALUE($S5)+_xlfn.NUMBERVALUE($S6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="28" priority="2">
-      <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)&lt;&gt;0)</formula>
+    <cfRule type="expression" dxfId="18" priority="7" stopIfTrue="1">
+      <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="1" stopIfTrue="1">
-      <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)&lt;&gt;0)</formula>
+    <cfRule type="expression" dxfId="19" priority="12" stopIfTrue="1">
+      <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",OR(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0,_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0,_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="26" priority="6">
+    <cfRule type="expression" dxfId="29" priority="6" stopIfTrue="1">
       <formula>OR(_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6),_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6),_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="25" priority="11" stopIfTrue="1">
-      <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3)-_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)&lt;&gt;0)</formula>
+    <cfRule type="expression" dxfId="28" priority="11" stopIfTrue="1">
+      <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)+_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="15" stopIfTrue="1">
-      <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3)&lt;&gt;0)</formula>
+    <cfRule type="expression" dxfId="27" priority="15">
+      <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="23" priority="5">
+    <cfRule type="expression" dxfId="26" priority="5">
       <formula>_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="22" priority="10" stopIfTrue="1">
-      <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)&lt;&gt;0)</formula>
+    <cfRule type="expression" dxfId="25" priority="10" stopIfTrue="1">
+      <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3)+_xlfn.NUMBERVALUE($S4)+_xlfn.NUMBERVALUE($S5)+_xlfn.NUMBERVALUE($S6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="14" stopIfTrue="1">
-      <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)&lt;&gt;0)</formula>
+    <cfRule type="expression" dxfId="24" priority="14">
+      <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="20" priority="4">
+    <cfRule type="expression" dxfId="23" priority="4">
       <formula>_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="19" priority="9" stopIfTrue="1">
-      <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)&lt;&gt;0)</formula>
+    <cfRule type="expression" dxfId="22" priority="9">
+      <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3)+_xlfn.NUMBERVALUE($U4)+_xlfn.NUMBERVALUE($U5)+_xlfn.NUMBERVALUE($U6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="13" stopIfTrue="1">
-      <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)&lt;&gt;0)</formula>
+    <cfRule type="expression" dxfId="21" priority="13">
+      <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="17" priority="3">
+    <cfRule type="expression" dxfId="20" priority="3">
       <formula>_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6)</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
add CA indicator for red flags aggregats and add message for TJ and CA
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E3095B4-999B-FB46-9889-DD77E8729181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59FC65B3-C932-D543-B071-ECABC4D66B10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" activeTab="3" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -5955,7 +5955,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="357">
+  <cellXfs count="358">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -7025,6 +7025,9 @@
     </xf>
     <xf numFmtId="0" fontId="70" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -7156,2247 +7159,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
     <cellStyle name="Normal 3" xfId="4" xr:uid="{6BD57324-3FD5-D341-A299-730D14794802}"/>
   </cellStyles>
-  <dxfs count="240">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
+  <dxfs count="16">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -10330,11 +8093,11 @@
       <c r="B1" s="129" t="s">
         <v>239</v>
       </c>
-      <c r="C1" s="319" t="s">
+      <c r="C1" s="320" t="s">
         <v>240</v>
       </c>
-      <c r="D1" s="319"/>
-      <c r="E1" s="319"/>
+      <c r="D1" s="320"/>
+      <c r="E1" s="320"/>
       <c r="F1" s="130"/>
       <c r="H1" s="26" t="s">
         <v>0</v>
@@ -10343,11 +8106,11 @@
     <row r="2" spans="1:8" s="134" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="131"/>
       <c r="B2" s="132"/>
-      <c r="C2" s="320" t="s">
+      <c r="C2" s="321" t="s">
         <v>241</v>
       </c>
-      <c r="D2" s="320"/>
-      <c r="E2" s="320"/>
+      <c r="D2" s="321"/>
+      <c r="E2" s="321"/>
       <c r="F2" s="133"/>
       <c r="H2" s="26" t="s">
         <v>0</v>
@@ -10371,10 +8134,10 @@
       <c r="D4" s="139" t="s">
         <v>244</v>
       </c>
-      <c r="E4" s="326" t="s">
+      <c r="E4" s="327" t="s">
         <v>245</v>
       </c>
-      <c r="F4" s="327"/>
+      <c r="F4" s="328"/>
       <c r="G4" s="148"/>
       <c r="H4" s="26" t="s">
         <v>0</v>
@@ -10391,10 +8154,10 @@
       <c r="D5" s="145" t="s">
         <v>248</v>
       </c>
-      <c r="E5" s="328" t="s">
+      <c r="E5" s="329" t="s">
         <v>261</v>
       </c>
-      <c r="F5" s="329"/>
+      <c r="F5" s="330"/>
       <c r="G5" s="147"/>
       <c r="H5" s="26" t="s">
         <v>0</v>
@@ -10411,10 +8174,10 @@
       <c r="D6" s="146" t="s">
         <v>251</v>
       </c>
-      <c r="E6" s="330" t="s">
+      <c r="E6" s="331" t="s">
         <v>262</v>
       </c>
-      <c r="F6" s="331"/>
+      <c r="F6" s="332"/>
       <c r="G6" s="147"/>
       <c r="H6" s="26" t="s">
         <v>0</v>
@@ -10431,10 +8194,10 @@
       <c r="D7" s="146" t="s">
         <v>254</v>
       </c>
-      <c r="E7" s="330" t="s">
+      <c r="E7" s="331" t="s">
         <v>261</v>
       </c>
-      <c r="F7" s="331"/>
+      <c r="F7" s="332"/>
       <c r="G7" s="147"/>
       <c r="H7" s="26" t="s">
         <v>0</v>
@@ -10445,16 +8208,16 @@
       <c r="B8" s="155" t="s">
         <v>255</v>
       </c>
-      <c r="C8" s="321" t="s">
+      <c r="C8" s="322" t="s">
         <v>256</v>
       </c>
-      <c r="D8" s="321" t="s">
+      <c r="D8" s="322" t="s">
         <v>257</v>
       </c>
-      <c r="E8" s="332" t="s">
+      <c r="E8" s="333" t="s">
         <v>263</v>
       </c>
-      <c r="F8" s="333"/>
+      <c r="F8" s="334"/>
       <c r="G8" s="147"/>
       <c r="H8" s="26" t="s">
         <v>0</v>
@@ -10465,10 +8228,10 @@
       <c r="B9" s="156" t="s">
         <v>258</v>
       </c>
-      <c r="C9" s="321"/>
-      <c r="D9" s="321"/>
-      <c r="E9" s="334"/>
-      <c r="F9" s="335"/>
+      <c r="C9" s="322"/>
+      <c r="D9" s="322"/>
+      <c r="E9" s="335"/>
+      <c r="F9" s="336"/>
       <c r="G9" s="147"/>
       <c r="H9" s="26" t="s">
         <v>0</v>
@@ -10479,10 +8242,10 @@
       <c r="B10" s="157" t="s">
         <v>259</v>
       </c>
-      <c r="C10" s="322"/>
-      <c r="D10" s="322"/>
-      <c r="E10" s="336"/>
-      <c r="F10" s="337"/>
+      <c r="C10" s="323"/>
+      <c r="D10" s="323"/>
+      <c r="E10" s="337"/>
+      <c r="F10" s="338"/>
       <c r="G10" s="147"/>
       <c r="H10" s="26" t="s">
         <v>0</v>
@@ -10502,11 +8265,11 @@
     <row r="12" spans="1:8" s="26" customFormat="1" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="135"/>
       <c r="B12" s="149"/>
-      <c r="C12" s="325" t="s">
+      <c r="C12" s="326" t="s">
         <v>260</v>
       </c>
-      <c r="D12" s="325"/>
-      <c r="E12" s="325"/>
+      <c r="D12" s="326"/>
+      <c r="E12" s="326"/>
       <c r="F12" s="150"/>
       <c r="H12" s="26" t="s">
         <v>0</v>
@@ -10520,14 +8283,14 @@
       </c>
     </row>
     <row r="14" spans="1:8" s="26" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="323" t="s">
+      <c r="A14" s="324" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="323"/>
-      <c r="C14" s="323"/>
-      <c r="D14" s="323"/>
-      <c r="E14" s="323"/>
-      <c r="F14" s="324"/>
+      <c r="B14" s="324"/>
+      <c r="C14" s="324"/>
+      <c r="D14" s="324"/>
+      <c r="E14" s="324"/>
+      <c r="F14" s="325"/>
       <c r="H14" s="26" t="s">
         <v>0</v>
       </c>
@@ -10595,13 +8358,13 @@
       <c r="G2" s="87" t="s">
         <v>181</v>
       </c>
-      <c r="H2" s="346" t="s">
+      <c r="H2" s="347" t="s">
         <v>180</v>
       </c>
       <c r="I2" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="J2" s="346" t="s">
+      <c r="J2" s="347" t="s">
         <v>179</v>
       </c>
     </row>
@@ -10615,11 +8378,11 @@
       <c r="G3" s="87" t="s">
         <v>159</v>
       </c>
-      <c r="H3" s="346"/>
+      <c r="H3" s="347"/>
       <c r="I3" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="J3" s="346"/>
+      <c r="J3" s="347"/>
     </row>
     <row r="4" spans="1:10" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="109"/>
@@ -10641,11 +8404,11 @@
       <c r="G4" s="87" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="346"/>
+      <c r="H4" s="347"/>
       <c r="I4" s="87" t="s">
         <v>104</v>
       </c>
-      <c r="J4" s="346"/>
+      <c r="J4" s="347"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="103" t="s">
@@ -11044,7 +8807,7 @@
       <c r="G2" s="87" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="346" t="s">
+      <c r="H2" s="347" t="s">
         <v>182</v>
       </c>
       <c r="I2" s="86" t="s">
@@ -11089,7 +8852,7 @@
       <c r="V2" s="86" t="s">
         <v>181</v>
       </c>
-      <c r="W2" s="346" t="s">
+      <c r="W2" s="347" t="s">
         <v>180</v>
       </c>
       <c r="X2" s="87" t="s">
@@ -11104,7 +8867,7 @@
       <c r="AA2" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="AB2" s="346" t="s">
+      <c r="AB2" s="347" t="s">
         <v>179</v>
       </c>
       <c r="AC2" s="84" t="s">
@@ -11134,7 +8897,7 @@
       <c r="AK2" s="84" t="s">
         <v>178</v>
       </c>
-      <c r="AL2" s="346" t="s">
+      <c r="AL2" s="347" t="s">
         <v>177</v>
       </c>
       <c r="AM2" s="84" t="s">
@@ -11176,7 +8939,7 @@
       <c r="AY2" s="84" t="s">
         <v>176</v>
       </c>
-      <c r="AZ2" s="346" t="s">
+      <c r="AZ2" s="347" t="s">
         <v>175</v>
       </c>
       <c r="BA2" s="83" t="s">
@@ -11206,7 +8969,7 @@
       <c r="BI2" s="83" t="s">
         <v>174</v>
       </c>
-      <c r="BJ2" s="346" t="s">
+      <c r="BJ2" s="347" t="s">
         <v>173</v>
       </c>
       <c r="BK2"/>
@@ -11221,7 +8984,7 @@
       <c r="G3" s="87" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="346"/>
+      <c r="H3" s="347"/>
       <c r="I3" s="86" t="s">
         <v>171</v>
       </c>
@@ -11262,7 +9025,7 @@
       <c r="V3" s="86" t="s">
         <v>159</v>
       </c>
-      <c r="W3" s="346"/>
+      <c r="W3" s="347"/>
       <c r="X3" s="82"/>
       <c r="Y3" s="87" t="s">
         <v>158</v>
@@ -11273,7 +9036,7 @@
       <c r="AA3" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="AB3" s="346"/>
+      <c r="AB3" s="347"/>
       <c r="AC3" s="84" t="s">
         <v>155</v>
       </c>
@@ -11301,7 +9064,7 @@
       <c r="AK3" s="84" t="s">
         <v>149</v>
       </c>
-      <c r="AL3" s="346"/>
+      <c r="AL3" s="347"/>
       <c r="AM3" s="84" t="s">
         <v>148</v>
       </c>
@@ -11341,7 +9104,7 @@
       <c r="AY3" s="84" t="s">
         <v>136</v>
       </c>
-      <c r="AZ3" s="346"/>
+      <c r="AZ3" s="347"/>
       <c r="BA3" s="83" t="s">
         <v>135</v>
       </c>
@@ -11369,7 +9132,7 @@
       <c r="BI3" s="83" t="s">
         <v>127</v>
       </c>
-      <c r="BJ3" s="346"/>
+      <c r="BJ3" s="347"/>
     </row>
     <row r="4" spans="1:63" s="44" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="89"/>
@@ -11391,7 +9154,7 @@
       <c r="G4" s="87" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="346"/>
+      <c r="H4" s="347"/>
       <c r="I4" s="86" t="s">
         <v>121</v>
       </c>
@@ -11434,7 +9197,7 @@
       <c r="V4" s="86" t="s">
         <v>108</v>
       </c>
-      <c r="W4" s="346"/>
+      <c r="W4" s="347"/>
       <c r="X4" s="85" t="s">
         <v>107</v>
       </c>
@@ -11447,7 +9210,7 @@
       <c r="AA4" s="85" t="s">
         <v>104</v>
       </c>
-      <c r="AB4" s="346"/>
+      <c r="AB4" s="347"/>
       <c r="AC4" s="84" t="s">
         <v>103</v>
       </c>
@@ -11475,7 +9238,7 @@
       <c r="AK4" s="84" t="s">
         <v>96</v>
       </c>
-      <c r="AL4" s="346"/>
+      <c r="AL4" s="347"/>
       <c r="AM4" s="84" t="s">
         <v>95</v>
       </c>
@@ -11515,7 +9278,7 @@
       <c r="AY4" s="84" t="s">
         <v>83</v>
       </c>
-      <c r="AZ4" s="346"/>
+      <c r="AZ4" s="347"/>
       <c r="BA4" s="83" t="s">
         <v>82</v>
       </c>
@@ -11543,7 +9306,7 @@
       <c r="BI4" s="83" t="s">
         <v>74</v>
       </c>
-      <c r="BJ4" s="346"/>
+      <c r="BJ4" s="347"/>
       <c r="BK4"/>
     </row>
     <row r="5" spans="1:63" s="44" customFormat="1" ht="15" x14ac:dyDescent="0.2">
@@ -14288,7 +12051,7 @@
       <c r="G2" s="87" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="346" t="s">
+      <c r="H2" s="347" t="s">
         <v>182</v>
       </c>
       <c r="I2" s="87" t="s">
@@ -14321,13 +12084,13 @@
       <c r="R2" s="87" t="s">
         <v>181</v>
       </c>
-      <c r="S2" s="346" t="s">
+      <c r="S2" s="347" t="s">
         <v>180</v>
       </c>
       <c r="T2" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="U2" s="346" t="s">
+      <c r="U2" s="347" t="s">
         <v>179</v>
       </c>
       <c r="V2" s="87" t="s">
@@ -14357,7 +12120,7 @@
       <c r="AD2" s="87" t="s">
         <v>178</v>
       </c>
-      <c r="AE2" s="346" t="s">
+      <c r="AE2" s="347" t="s">
         <v>227</v>
       </c>
       <c r="AF2" s="87" t="s">
@@ -14369,7 +12132,7 @@
       <c r="AH2" s="87" t="s">
         <v>226</v>
       </c>
-      <c r="AI2" s="346" t="s">
+      <c r="AI2" s="347" t="s">
         <v>225</v>
       </c>
     </row>
@@ -14383,7 +12146,7 @@
       <c r="G3" s="87" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="346"/>
+      <c r="H3" s="347"/>
       <c r="I3" s="87" t="s">
         <v>224</v>
       </c>
@@ -14414,11 +12177,11 @@
       <c r="R3" s="87" t="s">
         <v>159</v>
       </c>
-      <c r="S3" s="346"/>
+      <c r="S3" s="347"/>
       <c r="T3" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="U3" s="346"/>
+      <c r="U3" s="347"/>
       <c r="V3" s="87" t="s">
         <v>215</v>
       </c>
@@ -14446,7 +12209,7 @@
       <c r="AD3" s="87" t="s">
         <v>207</v>
       </c>
-      <c r="AE3" s="346"/>
+      <c r="AE3" s="347"/>
       <c r="AF3" s="87" t="s">
         <v>206</v>
       </c>
@@ -14456,7 +12219,7 @@
       <c r="AH3" s="87" t="s">
         <v>136</v>
       </c>
-      <c r="AI3" s="346"/>
+      <c r="AI3" s="347"/>
     </row>
     <row r="4" spans="1:62" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="90"/>
@@ -14478,7 +12241,7 @@
       <c r="G4" s="87" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="346"/>
+      <c r="H4" s="347"/>
       <c r="I4" s="87" t="s">
         <v>205</v>
       </c>
@@ -14509,11 +12272,11 @@
       <c r="R4" s="87" t="s">
         <v>108</v>
       </c>
-      <c r="S4" s="346"/>
+      <c r="S4" s="347"/>
       <c r="T4" s="87" t="s">
         <v>104</v>
       </c>
-      <c r="U4" s="346"/>
+      <c r="U4" s="347"/>
       <c r="V4" s="87" t="s">
         <v>196</v>
       </c>
@@ -14541,7 +12304,7 @@
       <c r="AD4" s="87" t="s">
         <v>188</v>
       </c>
-      <c r="AE4" s="346"/>
+      <c r="AE4" s="347"/>
       <c r="AF4" s="87" t="s">
         <v>187</v>
       </c>
@@ -14551,7 +12314,7 @@
       <c r="AH4" s="87" t="s">
         <v>83</v>
       </c>
-      <c r="AI4" s="346"/>
+      <c r="AI4" s="347"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="93" t="s">
@@ -16303,13 +14066,13 @@
       <c r="G2" s="87" t="s">
         <v>181</v>
       </c>
-      <c r="H2" s="346" t="s">
+      <c r="H2" s="347" t="s">
         <v>180</v>
       </c>
       <c r="I2" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="J2" s="346" t="s">
+      <c r="J2" s="347" t="s">
         <v>179</v>
       </c>
     </row>
@@ -16323,11 +14086,11 @@
       <c r="G3" s="87" t="s">
         <v>159</v>
       </c>
-      <c r="H3" s="346"/>
+      <c r="H3" s="347"/>
       <c r="I3" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="J3" s="346"/>
+      <c r="J3" s="347"/>
     </row>
     <row r="4" spans="1:62" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="109"/>
@@ -16349,11 +14112,11 @@
       <c r="G4" s="87" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="346"/>
+      <c r="H4" s="347"/>
       <c r="I4" s="87" t="s">
         <v>104</v>
       </c>
-      <c r="J4" s="346"/>
+      <c r="J4" s="347"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="103" t="s">
@@ -16740,13 +14503,13 @@
   <sheetData>
     <row r="1" spans="1:61" s="168" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="167"/>
-      <c r="B1" s="350" t="s">
+      <c r="B1" s="351" t="s">
         <v>184</v>
       </c>
-      <c r="C1" s="350"/>
-      <c r="D1" s="350"/>
-      <c r="E1" s="350"/>
-      <c r="F1" s="350"/>
+      <c r="C1" s="351"/>
+      <c r="D1" s="351"/>
+      <c r="E1" s="351"/>
+      <c r="F1" s="351"/>
       <c r="G1" s="169"/>
       <c r="H1" s="169"/>
       <c r="I1" s="169"/>
@@ -16791,7 +14554,7 @@
       <c r="O2" s="171" t="s">
         <v>178</v>
       </c>
-      <c r="P2" s="349" t="s">
+      <c r="P2" s="350" t="s">
         <v>177</v>
       </c>
       <c r="Q2" s="171" t="s">
@@ -16833,7 +14596,7 @@
       <c r="AC2" s="171" t="s">
         <v>176</v>
       </c>
-      <c r="AD2" s="349" t="s">
+      <c r="AD2" s="350" t="s">
         <v>175</v>
       </c>
       <c r="AE2" s="172" t="s">
@@ -16863,7 +14626,7 @@
       <c r="AM2" s="172" t="s">
         <v>174</v>
       </c>
-      <c r="AN2" s="349" t="s">
+      <c r="AN2" s="350" t="s">
         <v>173</v>
       </c>
       <c r="AQ2" s="171"/>
@@ -16874,7 +14637,7 @@
       <c r="AV2" s="171"/>
       <c r="AW2" s="171"/>
       <c r="AX2" s="171"/>
-      <c r="AY2" s="349"/>
+      <c r="AY2" s="350"/>
       <c r="AZ2" s="172"/>
       <c r="BA2" s="172"/>
       <c r="BB2" s="172"/>
@@ -16884,7 +14647,7 @@
       <c r="BF2" s="172"/>
       <c r="BG2" s="172"/>
       <c r="BH2" s="172"/>
-      <c r="BI2" s="349"/>
+      <c r="BI2" s="350"/>
     </row>
     <row r="3" spans="1:61" s="168" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="170"/>
@@ -16920,7 +14683,7 @@
       <c r="O3" s="171" t="s">
         <v>149</v>
       </c>
-      <c r="P3" s="349"/>
+      <c r="P3" s="350"/>
       <c r="Q3" s="171" t="s">
         <v>148</v>
       </c>
@@ -16960,7 +14723,7 @@
       <c r="AC3" s="171" t="s">
         <v>136</v>
       </c>
-      <c r="AD3" s="349"/>
+      <c r="AD3" s="350"/>
       <c r="AE3" s="172" t="s">
         <v>135</v>
       </c>
@@ -16988,7 +14751,7 @@
       <c r="AM3" s="172" t="s">
         <v>127</v>
       </c>
-      <c r="AN3" s="349"/>
+      <c r="AN3" s="350"/>
       <c r="AQ3" s="171"/>
       <c r="AR3" s="171"/>
       <c r="AS3" s="171"/>
@@ -16997,7 +14760,7 @@
       <c r="AV3" s="171"/>
       <c r="AW3" s="171"/>
       <c r="AX3" s="171"/>
-      <c r="AY3" s="349"/>
+      <c r="AY3" s="350"/>
       <c r="AZ3" s="172"/>
       <c r="BA3" s="172"/>
       <c r="BB3" s="172"/>
@@ -17007,7 +14770,7 @@
       <c r="BF3" s="172"/>
       <c r="BG3" s="172"/>
       <c r="BH3" s="172"/>
-      <c r="BI3" s="349"/>
+      <c r="BI3" s="350"/>
     </row>
     <row r="4" spans="1:61" s="168" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="173"/>
@@ -17053,7 +14816,7 @@
       <c r="O4" s="171" t="s">
         <v>96</v>
       </c>
-      <c r="P4" s="349"/>
+      <c r="P4" s="350"/>
       <c r="Q4" s="171" t="s">
         <v>95</v>
       </c>
@@ -17093,7 +14856,7 @@
       <c r="AC4" s="171" t="s">
         <v>83</v>
       </c>
-      <c r="AD4" s="349"/>
+      <c r="AD4" s="350"/>
       <c r="AE4" s="172" t="s">
         <v>82</v>
       </c>
@@ -17121,7 +14884,7 @@
       <c r="AM4" s="172" t="s">
         <v>74</v>
       </c>
-      <c r="AN4" s="349"/>
+      <c r="AN4" s="350"/>
       <c r="AQ4" s="171"/>
       <c r="AR4" s="171"/>
       <c r="AS4" s="171"/>
@@ -17130,7 +14893,7 @@
       <c r="AV4" s="171"/>
       <c r="AW4" s="171"/>
       <c r="AX4" s="171"/>
-      <c r="AY4" s="349"/>
+      <c r="AY4" s="350"/>
       <c r="AZ4" s="172"/>
       <c r="BA4" s="172"/>
       <c r="BB4" s="172"/>
@@ -17140,7 +14903,7 @@
       <c r="BF4" s="172"/>
       <c r="BG4" s="172"/>
       <c r="BH4" s="172"/>
-      <c r="BI4" s="349"/>
+      <c r="BI4" s="350"/>
     </row>
     <row r="5" spans="1:61" s="168" customFormat="1" ht="144" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="175" t="s">
@@ -18862,14 +16625,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="351" t="s">
+      <c r="A1" s="352" t="s">
         <v>228</v>
       </c>
-      <c r="B1" s="351"/>
-      <c r="C1" s="351"/>
-      <c r="D1" s="351"/>
-      <c r="E1" s="351"/>
-      <c r="F1" s="351"/>
+      <c r="B1" s="352"/>
+      <c r="C1" s="352"/>
+      <c r="D1" s="352"/>
+      <c r="E1" s="352"/>
+      <c r="F1" s="352"/>
       <c r="G1" s="200"/>
       <c r="H1" s="200"/>
       <c r="I1" s="200"/>
@@ -18919,7 +16682,7 @@
       <c r="O2" s="203" t="s">
         <v>178</v>
       </c>
-      <c r="P2" s="352" t="s">
+      <c r="P2" s="353" t="s">
         <v>227</v>
       </c>
       <c r="Q2" s="203" t="s">
@@ -18931,7 +16694,7 @@
       <c r="S2" s="203" t="s">
         <v>226</v>
       </c>
-      <c r="T2" s="352" t="s">
+      <c r="T2" s="353" t="s">
         <v>225</v>
       </c>
     </row>
@@ -18969,7 +16732,7 @@
       <c r="O3" s="203" t="s">
         <v>207</v>
       </c>
-      <c r="P3" s="352"/>
+      <c r="P3" s="353"/>
       <c r="Q3" s="203" t="s">
         <v>206</v>
       </c>
@@ -18979,7 +16742,7 @@
       <c r="S3" s="203" t="s">
         <v>136</v>
       </c>
-      <c r="T3" s="352"/>
+      <c r="T3" s="353"/>
     </row>
     <row r="4" spans="1:20" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="202"/>
@@ -19025,7 +16788,7 @@
       <c r="O4" s="203" t="s">
         <v>188</v>
       </c>
-      <c r="P4" s="352"/>
+      <c r="P4" s="353"/>
       <c r="Q4" s="203" t="s">
         <v>187</v>
       </c>
@@ -19035,7 +16798,7 @@
       <c r="S4" s="203" t="s">
         <v>83</v>
       </c>
-      <c r="T4" s="352"/>
+      <c r="T4" s="353"/>
     </row>
     <row r="5" spans="1:20" ht="317" x14ac:dyDescent="0.2">
       <c r="A5" s="206" t="s">
@@ -19621,16 +17384,16 @@
   <sheetData>
     <row r="1" spans="1:28" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="226"/>
-      <c r="B1" s="354" t="s">
+      <c r="B1" s="355" t="s">
         <v>184</v>
       </c>
-      <c r="C1" s="354"/>
-      <c r="D1" s="354"/>
-      <c r="E1" s="354"/>
-      <c r="F1" s="354"/>
-      <c r="G1" s="354"/>
-      <c r="H1" s="354"/>
-      <c r="I1" s="354"/>
+      <c r="C1" s="355"/>
+      <c r="D1" s="355"/>
+      <c r="E1" s="355"/>
+      <c r="F1" s="355"/>
+      <c r="G1" s="355"/>
+      <c r="H1" s="355"/>
+      <c r="I1" s="355"/>
       <c r="J1" s="223"/>
       <c r="K1" s="223"/>
       <c r="L1" s="223"/>
@@ -19661,7 +17424,7 @@
       <c r="G2" s="225" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="353" t="s">
+      <c r="H2" s="354" t="s">
         <v>182</v>
       </c>
       <c r="I2" s="228" t="s">
@@ -19706,7 +17469,7 @@
       <c r="V2" s="228" t="s">
         <v>181</v>
       </c>
-      <c r="W2" s="353" t="s">
+      <c r="W2" s="354" t="s">
         <v>180</v>
       </c>
       <c r="X2" s="225" t="s">
@@ -19721,7 +17484,7 @@
       <c r="AA2" s="225" t="s">
         <v>45</v>
       </c>
-      <c r="AB2" s="353" t="s">
+      <c r="AB2" s="354" t="s">
         <v>179</v>
       </c>
     </row>
@@ -19735,7 +17498,7 @@
       <c r="G3" s="225" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="353"/>
+      <c r="H3" s="354"/>
       <c r="I3" s="228" t="s">
         <v>171</v>
       </c>
@@ -19776,7 +17539,7 @@
       <c r="V3" s="228" t="s">
         <v>159</v>
       </c>
-      <c r="W3" s="353"/>
+      <c r="W3" s="354"/>
       <c r="X3" s="227"/>
       <c r="Y3" s="225" t="s">
         <v>158</v>
@@ -19787,7 +17550,7 @@
       <c r="AA3" s="225" t="s">
         <v>156</v>
       </c>
-      <c r="AB3" s="353"/>
+      <c r="AB3" s="354"/>
     </row>
     <row r="4" spans="1:28" ht="98" x14ac:dyDescent="0.2">
       <c r="A4" s="229"/>
@@ -19809,7 +17572,7 @@
       <c r="G4" s="225" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="353"/>
+      <c r="H4" s="354"/>
       <c r="I4" s="228" t="s">
         <v>121</v>
       </c>
@@ -19852,7 +17615,7 @@
       <c r="V4" s="231" t="s">
         <v>108</v>
       </c>
-      <c r="W4" s="353"/>
+      <c r="W4" s="354"/>
       <c r="X4" s="232" t="s">
         <v>107</v>
       </c>
@@ -19865,7 +17628,7 @@
       <c r="AA4" s="232" t="s">
         <v>104</v>
       </c>
-      <c r="AB4" s="353"/>
+      <c r="AB4" s="354"/>
     </row>
     <row r="5" spans="1:28" ht="196" x14ac:dyDescent="0.2">
       <c r="A5" s="233" t="s">
@@ -20759,16 +18522,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="356" t="s">
+      <c r="A1" s="357" t="s">
         <v>228</v>
       </c>
-      <c r="B1" s="356"/>
-      <c r="C1" s="356"/>
-      <c r="D1" s="356"/>
-      <c r="E1" s="356"/>
-      <c r="F1" s="356"/>
-      <c r="G1" s="356"/>
-      <c r="H1" s="356"/>
+      <c r="B1" s="357"/>
+      <c r="C1" s="357"/>
+      <c r="D1" s="357"/>
+      <c r="E1" s="357"/>
+      <c r="F1" s="357"/>
+      <c r="G1" s="357"/>
+      <c r="H1" s="357"/>
       <c r="I1" s="273"/>
       <c r="J1" s="273"/>
       <c r="K1" s="273"/>
@@ -20793,7 +18556,7 @@
       <c r="G2" s="275" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="355" t="s">
+      <c r="H2" s="356" t="s">
         <v>182</v>
       </c>
       <c r="I2" s="275" t="s">
@@ -20826,13 +18589,13 @@
       <c r="R2" s="275" t="s">
         <v>181</v>
       </c>
-      <c r="S2" s="355" t="s">
+      <c r="S2" s="356" t="s">
         <v>180</v>
       </c>
       <c r="T2" s="275" t="s">
         <v>45</v>
       </c>
-      <c r="U2" s="355" t="s">
+      <c r="U2" s="356" t="s">
         <v>179</v>
       </c>
     </row>
@@ -20846,7 +18609,7 @@
       <c r="G3" s="275" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="355"/>
+      <c r="H3" s="356"/>
       <c r="I3" s="275" t="s">
         <v>224</v>
       </c>
@@ -20877,11 +18640,11 @@
       <c r="R3" s="275" t="s">
         <v>159</v>
       </c>
-      <c r="S3" s="355"/>
+      <c r="S3" s="356"/>
       <c r="T3" s="275" t="s">
         <v>156</v>
       </c>
-      <c r="U3" s="355"/>
+      <c r="U3" s="356"/>
     </row>
     <row r="4" spans="1:21" ht="112" x14ac:dyDescent="0.2">
       <c r="A4" s="272"/>
@@ -20903,7 +18666,7 @@
       <c r="G4" s="275" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="355"/>
+      <c r="H4" s="356"/>
       <c r="I4" s="275" t="s">
         <v>205</v>
       </c>
@@ -20934,11 +18697,11 @@
       <c r="R4" s="275" t="s">
         <v>108</v>
       </c>
-      <c r="S4" s="355"/>
+      <c r="S4" s="356"/>
       <c r="T4" s="275" t="s">
         <v>104</v>
       </c>
-      <c r="U4" s="355"/>
+      <c r="U4" s="356"/>
     </row>
     <row r="5" spans="1:21" ht="196" x14ac:dyDescent="0.2">
       <c r="A5" s="278" t="s">
@@ -21629,13 +19392,13 @@
       <c r="K2" s="203" t="s">
         <v>181</v>
       </c>
-      <c r="L2" s="352" t="s">
+      <c r="L2" s="353" t="s">
         <v>180</v>
       </c>
       <c r="M2" s="203" t="s">
         <v>45</v>
       </c>
-      <c r="N2" s="352" t="s">
+      <c r="N2" s="353" t="s">
         <v>179</v>
       </c>
     </row>
@@ -21653,11 +19416,11 @@
       <c r="K3" s="203" t="s">
         <v>159</v>
       </c>
-      <c r="L3" s="352"/>
+      <c r="L3" s="353"/>
       <c r="M3" s="203" t="s">
         <v>156</v>
       </c>
-      <c r="N3" s="352"/>
+      <c r="N3" s="353"/>
     </row>
     <row r="4" spans="1:14" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="256"/>
@@ -21683,11 +19446,11 @@
       <c r="K4" s="203" t="s">
         <v>108</v>
       </c>
-      <c r="L4" s="352"/>
+      <c r="L4" s="353"/>
       <c r="M4" s="203" t="s">
         <v>104</v>
       </c>
-      <c r="N4" s="352"/>
+      <c r="N4" s="353"/>
     </row>
     <row r="5" spans="1:14" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="258"/>
@@ -22368,17 +20131,17 @@
       <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="FA1" s="338" t="s">
+      <c r="FA1" s="339" t="s">
         <v>237</v>
       </c>
-      <c r="FB1" s="338"/>
-      <c r="FC1" s="338"/>
-      <c r="FD1" s="338"/>
-      <c r="FE1" s="338"/>
-      <c r="FF1" s="338"/>
-      <c r="FG1" s="339"/>
-      <c r="FH1" s="339"/>
-      <c r="FI1" s="339"/>
+      <c r="FB1" s="339"/>
+      <c r="FC1" s="339"/>
+      <c r="FD1" s="339"/>
+      <c r="FE1" s="339"/>
+      <c r="FF1" s="339"/>
+      <c r="FG1" s="340"/>
+      <c r="FH1" s="340"/>
+      <c r="FI1" s="340"/>
       <c r="FJ1" s="4" t="s">
         <v>0</v>
       </c>
@@ -22519,28 +20282,28 @@
       <c r="D4" s="294"/>
       <c r="E4" s="294"/>
       <c r="F4" s="294"/>
-      <c r="G4" s="340" t="s">
+      <c r="G4" s="341" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="341"/>
-      <c r="I4" s="341"/>
-      <c r="J4" s="341"/>
-      <c r="K4" s="341"/>
-      <c r="L4" s="342"/>
-      <c r="M4" s="343"/>
-      <c r="N4" s="344" t="s">
+      <c r="H4" s="342"/>
+      <c r="I4" s="342"/>
+      <c r="J4" s="342"/>
+      <c r="K4" s="342"/>
+      <c r="L4" s="343"/>
+      <c r="M4" s="344"/>
+      <c r="N4" s="345" t="s">
         <v>27</v>
       </c>
-      <c r="O4" s="342"/>
-      <c r="P4" s="342"/>
-      <c r="Q4" s="342"/>
-      <c r="R4" s="342"/>
-      <c r="S4" s="342"/>
-      <c r="T4" s="345"/>
-      <c r="U4" s="340" t="s">
+      <c r="O4" s="343"/>
+      <c r="P4" s="343"/>
+      <c r="Q4" s="343"/>
+      <c r="R4" s="343"/>
+      <c r="S4" s="343"/>
+      <c r="T4" s="346"/>
+      <c r="U4" s="341" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="343"/>
+      <c r="V4" s="344"/>
       <c r="W4" s="301"/>
       <c r="X4" t="s">
         <v>0</v>
@@ -22603,7 +20366,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:24" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="13"/>
       <c r="C6" s="17" t="s">
         <v>23</v>
@@ -22614,7 +20377,7 @@
       <c r="E6" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="16" t="s">
+      <c r="F6" s="319" t="s">
         <v>399</v>
       </c>
       <c r="G6" s="19" t="e">
@@ -22737,70 +20500,70 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="31" priority="16">
+    <cfRule type="expression" dxfId="15" priority="16">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="30" priority="18">
+    <cfRule type="expression" dxfId="14" priority="18">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="16" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="1" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3)+_xlfn.NUMBERVALUE($U4)+_xlfn.NUMBERVALUE($U5)+_xlfn.NUMBERVALUE($U6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="2" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3)+_xlfn.NUMBERVALUE($S4)+_xlfn.NUMBERVALUE($S5)+_xlfn.NUMBERVALUE($S6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="7" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="12" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="12" stopIfTrue="1">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",OR(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0,_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0,_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="29" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
       <formula>OR(_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6),_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6),_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="28" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="8" priority="11" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)+_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="15">
+    <cfRule type="expression" dxfId="7" priority="15">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="26" priority="5">
+    <cfRule type="expression" dxfId="6" priority="5">
       <formula>_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="25" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="10" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3)+_xlfn.NUMBERVALUE($S4)+_xlfn.NUMBERVALUE($S5)+_xlfn.NUMBERVALUE($S6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="14">
+    <cfRule type="expression" dxfId="4" priority="14">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="23" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="22" priority="9">
+    <cfRule type="expression" dxfId="2" priority="9">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3)+_xlfn.NUMBERVALUE($U4)+_xlfn.NUMBERVALUE($U5)+_xlfn.NUMBERVALUE($U6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="13">
+    <cfRule type="expression" dxfId="1" priority="13">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="20" priority="3">
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -23177,16 +20940,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:62" s="44" customFormat="1" ht="23.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B1" s="347" t="s">
+      <c r="B1" s="348" t="s">
         <v>184</v>
       </c>
-      <c r="C1" s="347"/>
-      <c r="D1" s="347"/>
-      <c r="E1" s="347"/>
-      <c r="F1" s="347"/>
-      <c r="G1" s="347"/>
-      <c r="H1" s="347"/>
-      <c r="I1" s="347"/>
+      <c r="C1" s="348"/>
+      <c r="D1" s="348"/>
+      <c r="E1" s="348"/>
+      <c r="F1" s="348"/>
+      <c r="G1" s="348"/>
+      <c r="H1" s="348"/>
+      <c r="I1" s="348"/>
     </row>
     <row r="2" spans="1:62" s="44" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="90"/>
@@ -23198,7 +20961,7 @@
       <c r="G2" s="87" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="346" t="s">
+      <c r="H2" s="347" t="s">
         <v>182</v>
       </c>
       <c r="I2" s="86" t="s">
@@ -23243,7 +21006,7 @@
       <c r="V2" s="86" t="s">
         <v>181</v>
       </c>
-      <c r="W2" s="346" t="s">
+      <c r="W2" s="347" t="s">
         <v>180</v>
       </c>
       <c r="X2" s="87" t="s">
@@ -23258,7 +21021,7 @@
       <c r="AA2" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="AB2" s="346" t="s">
+      <c r="AB2" s="347" t="s">
         <v>179</v>
       </c>
       <c r="AC2" s="84" t="s">
@@ -23288,7 +21051,7 @@
       <c r="AK2" s="84" t="s">
         <v>178</v>
       </c>
-      <c r="AL2" s="346" t="s">
+      <c r="AL2" s="347" t="s">
         <v>177</v>
       </c>
       <c r="AM2" s="84" t="s">
@@ -23330,7 +21093,7 @@
       <c r="AY2" s="84" t="s">
         <v>176</v>
       </c>
-      <c r="AZ2" s="346" t="s">
+      <c r="AZ2" s="347" t="s">
         <v>175</v>
       </c>
       <c r="BA2" s="83" t="s">
@@ -23360,7 +21123,7 @@
       <c r="BI2" s="83" t="s">
         <v>174</v>
       </c>
-      <c r="BJ2" s="346" t="s">
+      <c r="BJ2" s="347" t="s">
         <v>173</v>
       </c>
     </row>
@@ -23374,7 +21137,7 @@
       <c r="G3" s="87" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="346"/>
+      <c r="H3" s="347"/>
       <c r="I3" s="86" t="s">
         <v>171</v>
       </c>
@@ -23415,7 +21178,7 @@
       <c r="V3" s="86" t="s">
         <v>159</v>
       </c>
-      <c r="W3" s="346"/>
+      <c r="W3" s="347"/>
       <c r="X3" s="82"/>
       <c r="Y3" s="87" t="s">
         <v>158</v>
@@ -23426,7 +21189,7 @@
       <c r="AA3" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="AB3" s="346"/>
+      <c r="AB3" s="347"/>
       <c r="AC3" s="84" t="s">
         <v>155</v>
       </c>
@@ -23454,7 +21217,7 @@
       <c r="AK3" s="84" t="s">
         <v>149</v>
       </c>
-      <c r="AL3" s="346"/>
+      <c r="AL3" s="347"/>
       <c r="AM3" s="84" t="s">
         <v>148</v>
       </c>
@@ -23494,7 +21257,7 @@
       <c r="AY3" s="84" t="s">
         <v>136</v>
       </c>
-      <c r="AZ3" s="346"/>
+      <c r="AZ3" s="347"/>
       <c r="BA3" s="83" t="s">
         <v>135</v>
       </c>
@@ -23522,7 +21285,7 @@
       <c r="BI3" s="83" t="s">
         <v>127</v>
       </c>
-      <c r="BJ3" s="346"/>
+      <c r="BJ3" s="347"/>
     </row>
     <row r="4" spans="1:62" s="44" customFormat="1" ht="60" x14ac:dyDescent="0.15">
       <c r="A4" s="89"/>
@@ -23544,7 +21307,7 @@
       <c r="G4" s="87" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="346"/>
+      <c r="H4" s="347"/>
       <c r="I4" s="86" t="s">
         <v>121</v>
       </c>
@@ -23587,7 +21350,7 @@
       <c r="V4" s="86" t="s">
         <v>108</v>
       </c>
-      <c r="W4" s="346"/>
+      <c r="W4" s="347"/>
       <c r="X4" s="85" t="s">
         <v>107</v>
       </c>
@@ -23600,7 +21363,7 @@
       <c r="AA4" s="85" t="s">
         <v>104</v>
       </c>
-      <c r="AB4" s="346"/>
+      <c r="AB4" s="347"/>
       <c r="AC4" s="84" t="s">
         <v>103</v>
       </c>
@@ -23628,7 +21391,7 @@
       <c r="AK4" s="84" t="s">
         <v>96</v>
       </c>
-      <c r="AL4" s="346"/>
+      <c r="AL4" s="347"/>
       <c r="AM4" s="84" t="s">
         <v>95</v>
       </c>
@@ -23668,7 +21431,7 @@
       <c r="AY4" s="84" t="s">
         <v>83</v>
       </c>
-      <c r="AZ4" s="346"/>
+      <c r="AZ4" s="347"/>
       <c r="BA4" s="83" t="s">
         <v>82</v>
       </c>
@@ -23696,7 +21459,7 @@
       <c r="BI4" s="83" t="s">
         <v>74</v>
       </c>
-      <c r="BJ4" s="346"/>
+      <c r="BJ4" s="347"/>
     </row>
     <row r="5" spans="1:62" s="44" customFormat="1" ht="11" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="54" t="s">
@@ -25885,16 +23648,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A1" s="348" t="s">
+      <c r="A1" s="349" t="s">
         <v>228</v>
       </c>
-      <c r="B1" s="348"/>
-      <c r="C1" s="348"/>
-      <c r="D1" s="348"/>
-      <c r="E1" s="348"/>
-      <c r="F1" s="348"/>
-      <c r="G1" s="348"/>
-      <c r="H1" s="348"/>
+      <c r="B1" s="349"/>
+      <c r="C1" s="349"/>
+      <c r="D1" s="349"/>
+      <c r="E1" s="349"/>
+      <c r="F1" s="349"/>
+      <c r="G1" s="349"/>
+      <c r="H1" s="349"/>
       <c r="I1" s="44"/>
       <c r="J1" s="44"/>
       <c r="K1" s="44"/>
@@ -25933,7 +23696,7 @@
       <c r="G2" s="87" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="346" t="s">
+      <c r="H2" s="347" t="s">
         <v>182</v>
       </c>
       <c r="I2" s="87" t="s">
@@ -25966,13 +23729,13 @@
       <c r="R2" s="87" t="s">
         <v>181</v>
       </c>
-      <c r="S2" s="346" t="s">
+      <c r="S2" s="347" t="s">
         <v>180</v>
       </c>
       <c r="T2" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="U2" s="346" t="s">
+      <c r="U2" s="347" t="s">
         <v>179</v>
       </c>
       <c r="V2" s="87" t="s">
@@ -26002,7 +23765,7 @@
       <c r="AD2" s="87" t="s">
         <v>178</v>
       </c>
-      <c r="AE2" s="346" t="s">
+      <c r="AE2" s="347" t="s">
         <v>227</v>
       </c>
       <c r="AF2" s="87" t="s">
@@ -26014,7 +23777,7 @@
       <c r="AH2" s="87" t="s">
         <v>226</v>
       </c>
-      <c r="AI2" s="346" t="s">
+      <c r="AI2" s="347" t="s">
         <v>225</v>
       </c>
     </row>
@@ -26028,7 +23791,7 @@
       <c r="G3" s="87" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="346"/>
+      <c r="H3" s="347"/>
       <c r="I3" s="87" t="s">
         <v>224</v>
       </c>
@@ -26059,11 +23822,11 @@
       <c r="R3" s="87" t="s">
         <v>159</v>
       </c>
-      <c r="S3" s="346"/>
+      <c r="S3" s="347"/>
       <c r="T3" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="U3" s="346"/>
+      <c r="U3" s="347"/>
       <c r="V3" s="87" t="s">
         <v>215</v>
       </c>
@@ -26091,7 +23854,7 @@
       <c r="AD3" s="87" t="s">
         <v>207</v>
       </c>
-      <c r="AE3" s="346"/>
+      <c r="AE3" s="347"/>
       <c r="AF3" s="87" t="s">
         <v>206</v>
       </c>
@@ -26101,7 +23864,7 @@
       <c r="AH3" s="87" t="s">
         <v>136</v>
       </c>
-      <c r="AI3" s="346"/>
+      <c r="AI3" s="347"/>
     </row>
     <row r="4" spans="1:35" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="90"/>
@@ -26123,7 +23886,7 @@
       <c r="G4" s="87" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="346"/>
+      <c r="H4" s="347"/>
       <c r="I4" s="87" t="s">
         <v>205</v>
       </c>
@@ -26154,11 +23917,11 @@
       <c r="R4" s="87" t="s">
         <v>108</v>
       </c>
-      <c r="S4" s="346"/>
+      <c r="S4" s="347"/>
       <c r="T4" s="87" t="s">
         <v>104</v>
       </c>
-      <c r="U4" s="346"/>
+      <c r="U4" s="347"/>
       <c r="V4" s="87" t="s">
         <v>196</v>
       </c>
@@ -26186,7 +23949,7 @@
       <c r="AD4" s="87" t="s">
         <v>188</v>
       </c>
-      <c r="AE4" s="346"/>
+      <c r="AE4" s="347"/>
       <c r="AF4" s="87" t="s">
         <v>187</v>
       </c>
@@ -26196,7 +23959,7 @@
       <c r="AH4" s="87" t="s">
         <v>83</v>
       </c>
-      <c r="AI4" s="346"/>
+      <c r="AI4" s="347"/>
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A5" s="93" t="s">

</xml_diff>

<commit_message>
update underline red extractor for gap cases
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10112"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59FC65B3-C932-D543-B071-ECABC4D66B10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57A7E359-D53B-D241-8BBF-656D9D6D4728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" activeTab="3" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" activeTab="2" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -5955,7 +5955,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="358">
+  <cellXfs count="357">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -7029,6 +7029,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="37" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="39" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -7085,12 +7088,6 @@
     </xf>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -7159,7 +7156,27 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
     <cellStyle name="Normal 3" xfId="4" xr:uid="{6BD57324-3FD5-D341-A299-730D14794802}"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="18">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -8093,11 +8110,11 @@
       <c r="B1" s="129" t="s">
         <v>239</v>
       </c>
-      <c r="C1" s="320" t="s">
+      <c r="C1" s="321" t="s">
         <v>240</v>
       </c>
-      <c r="D1" s="320"/>
-      <c r="E1" s="320"/>
+      <c r="D1" s="321"/>
+      <c r="E1" s="321"/>
       <c r="F1" s="130"/>
       <c r="H1" s="26" t="s">
         <v>0</v>
@@ -8106,11 +8123,11 @@
     <row r="2" spans="1:8" s="134" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="131"/>
       <c r="B2" s="132"/>
-      <c r="C2" s="321" t="s">
+      <c r="C2" s="322" t="s">
         <v>241</v>
       </c>
-      <c r="D2" s="321"/>
-      <c r="E2" s="321"/>
+      <c r="D2" s="322"/>
+      <c r="E2" s="322"/>
       <c r="F2" s="133"/>
       <c r="H2" s="26" t="s">
         <v>0</v>
@@ -8134,10 +8151,10 @@
       <c r="D4" s="139" t="s">
         <v>244</v>
       </c>
-      <c r="E4" s="327" t="s">
+      <c r="E4" s="328" t="s">
         <v>245</v>
       </c>
-      <c r="F4" s="328"/>
+      <c r="F4" s="329"/>
       <c r="G4" s="148"/>
       <c r="H4" s="26" t="s">
         <v>0</v>
@@ -8154,10 +8171,10 @@
       <c r="D5" s="145" t="s">
         <v>248</v>
       </c>
-      <c r="E5" s="329" t="s">
+      <c r="E5" s="330" t="s">
         <v>261</v>
       </c>
-      <c r="F5" s="330"/>
+      <c r="F5" s="331"/>
       <c r="G5" s="147"/>
       <c r="H5" s="26" t="s">
         <v>0</v>
@@ -8174,10 +8191,10 @@
       <c r="D6" s="146" t="s">
         <v>251</v>
       </c>
-      <c r="E6" s="331" t="s">
+      <c r="E6" s="332" t="s">
         <v>262</v>
       </c>
-      <c r="F6" s="332"/>
+      <c r="F6" s="333"/>
       <c r="G6" s="147"/>
       <c r="H6" s="26" t="s">
         <v>0</v>
@@ -8194,10 +8211,10 @@
       <c r="D7" s="146" t="s">
         <v>254</v>
       </c>
-      <c r="E7" s="331" t="s">
+      <c r="E7" s="332" t="s">
         <v>261</v>
       </c>
-      <c r="F7" s="332"/>
+      <c r="F7" s="333"/>
       <c r="G7" s="147"/>
       <c r="H7" s="26" t="s">
         <v>0</v>
@@ -8208,16 +8225,16 @@
       <c r="B8" s="155" t="s">
         <v>255</v>
       </c>
-      <c r="C8" s="322" t="s">
+      <c r="C8" s="323" t="s">
         <v>256</v>
       </c>
-      <c r="D8" s="322" t="s">
+      <c r="D8" s="323" t="s">
         <v>257</v>
       </c>
-      <c r="E8" s="333" t="s">
+      <c r="E8" s="334" t="s">
         <v>263</v>
       </c>
-      <c r="F8" s="334"/>
+      <c r="F8" s="335"/>
       <c r="G8" s="147"/>
       <c r="H8" s="26" t="s">
         <v>0</v>
@@ -8228,10 +8245,10 @@
       <c r="B9" s="156" t="s">
         <v>258</v>
       </c>
-      <c r="C9" s="322"/>
-      <c r="D9" s="322"/>
-      <c r="E9" s="335"/>
-      <c r="F9" s="336"/>
+      <c r="C9" s="323"/>
+      <c r="D9" s="323"/>
+      <c r="E9" s="336"/>
+      <c r="F9" s="337"/>
       <c r="G9" s="147"/>
       <c r="H9" s="26" t="s">
         <v>0</v>
@@ -8242,10 +8259,10 @@
       <c r="B10" s="157" t="s">
         <v>259</v>
       </c>
-      <c r="C10" s="323"/>
-      <c r="D10" s="323"/>
-      <c r="E10" s="337"/>
-      <c r="F10" s="338"/>
+      <c r="C10" s="324"/>
+      <c r="D10" s="324"/>
+      <c r="E10" s="338"/>
+      <c r="F10" s="339"/>
       <c r="G10" s="147"/>
       <c r="H10" s="26" t="s">
         <v>0</v>
@@ -8265,11 +8282,11 @@
     <row r="12" spans="1:8" s="26" customFormat="1" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="135"/>
       <c r="B12" s="149"/>
-      <c r="C12" s="326" t="s">
+      <c r="C12" s="327" t="s">
         <v>260</v>
       </c>
-      <c r="D12" s="326"/>
-      <c r="E12" s="326"/>
+      <c r="D12" s="327"/>
+      <c r="E12" s="327"/>
       <c r="F12" s="150"/>
       <c r="H12" s="26" t="s">
         <v>0</v>
@@ -8283,14 +8300,14 @@
       </c>
     </row>
     <row r="14" spans="1:8" s="26" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="324" t="s">
+      <c r="A14" s="325" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="324"/>
-      <c r="C14" s="324"/>
-      <c r="D14" s="324"/>
-      <c r="E14" s="324"/>
-      <c r="F14" s="325"/>
+      <c r="B14" s="325"/>
+      <c r="C14" s="325"/>
+      <c r="D14" s="325"/>
+      <c r="E14" s="325"/>
+      <c r="F14" s="326"/>
       <c r="H14" s="26" t="s">
         <v>0</v>
       </c>
@@ -8358,13 +8375,13 @@
       <c r="G2" s="87" t="s">
         <v>181</v>
       </c>
-      <c r="H2" s="347" t="s">
+      <c r="H2" s="346" t="s">
         <v>180</v>
       </c>
       <c r="I2" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="J2" s="347" t="s">
+      <c r="J2" s="346" t="s">
         <v>179</v>
       </c>
     </row>
@@ -8378,11 +8395,11 @@
       <c r="G3" s="87" t="s">
         <v>159</v>
       </c>
-      <c r="H3" s="347"/>
+      <c r="H3" s="346"/>
       <c r="I3" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="J3" s="347"/>
+      <c r="J3" s="346"/>
     </row>
     <row r="4" spans="1:10" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="109"/>
@@ -8404,11 +8421,11 @@
       <c r="G4" s="87" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="347"/>
+      <c r="H4" s="346"/>
       <c r="I4" s="87" t="s">
         <v>104</v>
       </c>
-      <c r="J4" s="347"/>
+      <c r="J4" s="346"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="103" t="s">
@@ -8807,7 +8824,7 @@
       <c r="G2" s="87" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="347" t="s">
+      <c r="H2" s="346" t="s">
         <v>182</v>
       </c>
       <c r="I2" s="86" t="s">
@@ -8852,7 +8869,7 @@
       <c r="V2" s="86" t="s">
         <v>181</v>
       </c>
-      <c r="W2" s="347" t="s">
+      <c r="W2" s="346" t="s">
         <v>180</v>
       </c>
       <c r="X2" s="87" t="s">
@@ -8867,7 +8884,7 @@
       <c r="AA2" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="AB2" s="347" t="s">
+      <c r="AB2" s="346" t="s">
         <v>179</v>
       </c>
       <c r="AC2" s="84" t="s">
@@ -8897,7 +8914,7 @@
       <c r="AK2" s="84" t="s">
         <v>178</v>
       </c>
-      <c r="AL2" s="347" t="s">
+      <c r="AL2" s="346" t="s">
         <v>177</v>
       </c>
       <c r="AM2" s="84" t="s">
@@ -8939,7 +8956,7 @@
       <c r="AY2" s="84" t="s">
         <v>176</v>
       </c>
-      <c r="AZ2" s="347" t="s">
+      <c r="AZ2" s="346" t="s">
         <v>175</v>
       </c>
       <c r="BA2" s="83" t="s">
@@ -8969,7 +8986,7 @@
       <c r="BI2" s="83" t="s">
         <v>174</v>
       </c>
-      <c r="BJ2" s="347" t="s">
+      <c r="BJ2" s="346" t="s">
         <v>173</v>
       </c>
       <c r="BK2"/>
@@ -8984,7 +9001,7 @@
       <c r="G3" s="87" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="347"/>
+      <c r="H3" s="346"/>
       <c r="I3" s="86" t="s">
         <v>171</v>
       </c>
@@ -9025,7 +9042,7 @@
       <c r="V3" s="86" t="s">
         <v>159</v>
       </c>
-      <c r="W3" s="347"/>
+      <c r="W3" s="346"/>
       <c r="X3" s="82"/>
       <c r="Y3" s="87" t="s">
         <v>158</v>
@@ -9036,7 +9053,7 @@
       <c r="AA3" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="AB3" s="347"/>
+      <c r="AB3" s="346"/>
       <c r="AC3" s="84" t="s">
         <v>155</v>
       </c>
@@ -9064,7 +9081,7 @@
       <c r="AK3" s="84" t="s">
         <v>149</v>
       </c>
-      <c r="AL3" s="347"/>
+      <c r="AL3" s="346"/>
       <c r="AM3" s="84" t="s">
         <v>148</v>
       </c>
@@ -9104,7 +9121,7 @@
       <c r="AY3" s="84" t="s">
         <v>136</v>
       </c>
-      <c r="AZ3" s="347"/>
+      <c r="AZ3" s="346"/>
       <c r="BA3" s="83" t="s">
         <v>135</v>
       </c>
@@ -9132,7 +9149,7 @@
       <c r="BI3" s="83" t="s">
         <v>127</v>
       </c>
-      <c r="BJ3" s="347"/>
+      <c r="BJ3" s="346"/>
     </row>
     <row r="4" spans="1:63" s="44" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="89"/>
@@ -9154,7 +9171,7 @@
       <c r="G4" s="87" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="347"/>
+      <c r="H4" s="346"/>
       <c r="I4" s="86" t="s">
         <v>121</v>
       </c>
@@ -9197,7 +9214,7 @@
       <c r="V4" s="86" t="s">
         <v>108</v>
       </c>
-      <c r="W4" s="347"/>
+      <c r="W4" s="346"/>
       <c r="X4" s="85" t="s">
         <v>107</v>
       </c>
@@ -9210,7 +9227,7 @@
       <c r="AA4" s="85" t="s">
         <v>104</v>
       </c>
-      <c r="AB4" s="347"/>
+      <c r="AB4" s="346"/>
       <c r="AC4" s="84" t="s">
         <v>103</v>
       </c>
@@ -9238,7 +9255,7 @@
       <c r="AK4" s="84" t="s">
         <v>96</v>
       </c>
-      <c r="AL4" s="347"/>
+      <c r="AL4" s="346"/>
       <c r="AM4" s="84" t="s">
         <v>95</v>
       </c>
@@ -9278,7 +9295,7 @@
       <c r="AY4" s="84" t="s">
         <v>83</v>
       </c>
-      <c r="AZ4" s="347"/>
+      <c r="AZ4" s="346"/>
       <c r="BA4" s="83" t="s">
         <v>82</v>
       </c>
@@ -9306,7 +9323,7 @@
       <c r="BI4" s="83" t="s">
         <v>74</v>
       </c>
-      <c r="BJ4" s="347"/>
+      <c r="BJ4" s="346"/>
       <c r="BK4"/>
     </row>
     <row r="5" spans="1:63" s="44" customFormat="1" ht="15" x14ac:dyDescent="0.2">
@@ -12051,7 +12068,7 @@
       <c r="G2" s="87" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="347" t="s">
+      <c r="H2" s="346" t="s">
         <v>182</v>
       </c>
       <c r="I2" s="87" t="s">
@@ -12084,13 +12101,13 @@
       <c r="R2" s="87" t="s">
         <v>181</v>
       </c>
-      <c r="S2" s="347" t="s">
+      <c r="S2" s="346" t="s">
         <v>180</v>
       </c>
       <c r="T2" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="U2" s="347" t="s">
+      <c r="U2" s="346" t="s">
         <v>179</v>
       </c>
       <c r="V2" s="87" t="s">
@@ -12120,7 +12137,7 @@
       <c r="AD2" s="87" t="s">
         <v>178</v>
       </c>
-      <c r="AE2" s="347" t="s">
+      <c r="AE2" s="346" t="s">
         <v>227</v>
       </c>
       <c r="AF2" s="87" t="s">
@@ -12132,7 +12149,7 @@
       <c r="AH2" s="87" t="s">
         <v>226</v>
       </c>
-      <c r="AI2" s="347" t="s">
+      <c r="AI2" s="346" t="s">
         <v>225</v>
       </c>
     </row>
@@ -12146,7 +12163,7 @@
       <c r="G3" s="87" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="347"/>
+      <c r="H3" s="346"/>
       <c r="I3" s="87" t="s">
         <v>224</v>
       </c>
@@ -12177,11 +12194,11 @@
       <c r="R3" s="87" t="s">
         <v>159</v>
       </c>
-      <c r="S3" s="347"/>
+      <c r="S3" s="346"/>
       <c r="T3" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="U3" s="347"/>
+      <c r="U3" s="346"/>
       <c r="V3" s="87" t="s">
         <v>215</v>
       </c>
@@ -12209,7 +12226,7 @@
       <c r="AD3" s="87" t="s">
         <v>207</v>
       </c>
-      <c r="AE3" s="347"/>
+      <c r="AE3" s="346"/>
       <c r="AF3" s="87" t="s">
         <v>206</v>
       </c>
@@ -12219,7 +12236,7 @@
       <c r="AH3" s="87" t="s">
         <v>136</v>
       </c>
-      <c r="AI3" s="347"/>
+      <c r="AI3" s="346"/>
     </row>
     <row r="4" spans="1:62" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="90"/>
@@ -12241,7 +12258,7 @@
       <c r="G4" s="87" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="347"/>
+      <c r="H4" s="346"/>
       <c r="I4" s="87" t="s">
         <v>205</v>
       </c>
@@ -12272,11 +12289,11 @@
       <c r="R4" s="87" t="s">
         <v>108</v>
       </c>
-      <c r="S4" s="347"/>
+      <c r="S4" s="346"/>
       <c r="T4" s="87" t="s">
         <v>104</v>
       </c>
-      <c r="U4" s="347"/>
+      <c r="U4" s="346"/>
       <c r="V4" s="87" t="s">
         <v>196</v>
       </c>
@@ -12304,7 +12321,7 @@
       <c r="AD4" s="87" t="s">
         <v>188</v>
       </c>
-      <c r="AE4" s="347"/>
+      <c r="AE4" s="346"/>
       <c r="AF4" s="87" t="s">
         <v>187</v>
       </c>
@@ -12314,7 +12331,7 @@
       <c r="AH4" s="87" t="s">
         <v>83</v>
       </c>
-      <c r="AI4" s="347"/>
+      <c r="AI4" s="346"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="93" t="s">
@@ -14066,13 +14083,13 @@
       <c r="G2" s="87" t="s">
         <v>181</v>
       </c>
-      <c r="H2" s="347" t="s">
+      <c r="H2" s="346" t="s">
         <v>180</v>
       </c>
       <c r="I2" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="J2" s="347" t="s">
+      <c r="J2" s="346" t="s">
         <v>179</v>
       </c>
     </row>
@@ -14086,11 +14103,11 @@
       <c r="G3" s="87" t="s">
         <v>159</v>
       </c>
-      <c r="H3" s="347"/>
+      <c r="H3" s="346"/>
       <c r="I3" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="J3" s="347"/>
+      <c r="J3" s="346"/>
     </row>
     <row r="4" spans="1:62" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="109"/>
@@ -14112,11 +14129,11 @@
       <c r="G4" s="87" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="347"/>
+      <c r="H4" s="346"/>
       <c r="I4" s="87" t="s">
         <v>104</v>
       </c>
-      <c r="J4" s="347"/>
+      <c r="J4" s="346"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="103" t="s">
@@ -14503,13 +14520,13 @@
   <sheetData>
     <row r="1" spans="1:61" s="168" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="167"/>
-      <c r="B1" s="351" t="s">
+      <c r="B1" s="350" t="s">
         <v>184</v>
       </c>
-      <c r="C1" s="351"/>
-      <c r="D1" s="351"/>
-      <c r="E1" s="351"/>
-      <c r="F1" s="351"/>
+      <c r="C1" s="350"/>
+      <c r="D1" s="350"/>
+      <c r="E1" s="350"/>
+      <c r="F1" s="350"/>
       <c r="G1" s="169"/>
       <c r="H1" s="169"/>
       <c r="I1" s="169"/>
@@ -14554,7 +14571,7 @@
       <c r="O2" s="171" t="s">
         <v>178</v>
       </c>
-      <c r="P2" s="350" t="s">
+      <c r="P2" s="349" t="s">
         <v>177</v>
       </c>
       <c r="Q2" s="171" t="s">
@@ -14596,7 +14613,7 @@
       <c r="AC2" s="171" t="s">
         <v>176</v>
       </c>
-      <c r="AD2" s="350" t="s">
+      <c r="AD2" s="349" t="s">
         <v>175</v>
       </c>
       <c r="AE2" s="172" t="s">
@@ -14626,7 +14643,7 @@
       <c r="AM2" s="172" t="s">
         <v>174</v>
       </c>
-      <c r="AN2" s="350" t="s">
+      <c r="AN2" s="349" t="s">
         <v>173</v>
       </c>
       <c r="AQ2" s="171"/>
@@ -14637,7 +14654,7 @@
       <c r="AV2" s="171"/>
       <c r="AW2" s="171"/>
       <c r="AX2" s="171"/>
-      <c r="AY2" s="350"/>
+      <c r="AY2" s="349"/>
       <c r="AZ2" s="172"/>
       <c r="BA2" s="172"/>
       <c r="BB2" s="172"/>
@@ -14647,7 +14664,7 @@
       <c r="BF2" s="172"/>
       <c r="BG2" s="172"/>
       <c r="BH2" s="172"/>
-      <c r="BI2" s="350"/>
+      <c r="BI2" s="349"/>
     </row>
     <row r="3" spans="1:61" s="168" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="170"/>
@@ -14683,7 +14700,7 @@
       <c r="O3" s="171" t="s">
         <v>149</v>
       </c>
-      <c r="P3" s="350"/>
+      <c r="P3" s="349"/>
       <c r="Q3" s="171" t="s">
         <v>148</v>
       </c>
@@ -14723,7 +14740,7 @@
       <c r="AC3" s="171" t="s">
         <v>136</v>
       </c>
-      <c r="AD3" s="350"/>
+      <c r="AD3" s="349"/>
       <c r="AE3" s="172" t="s">
         <v>135</v>
       </c>
@@ -14751,7 +14768,7 @@
       <c r="AM3" s="172" t="s">
         <v>127</v>
       </c>
-      <c r="AN3" s="350"/>
+      <c r="AN3" s="349"/>
       <c r="AQ3" s="171"/>
       <c r="AR3" s="171"/>
       <c r="AS3" s="171"/>
@@ -14760,7 +14777,7 @@
       <c r="AV3" s="171"/>
       <c r="AW3" s="171"/>
       <c r="AX3" s="171"/>
-      <c r="AY3" s="350"/>
+      <c r="AY3" s="349"/>
       <c r="AZ3" s="172"/>
       <c r="BA3" s="172"/>
       <c r="BB3" s="172"/>
@@ -14770,7 +14787,7 @@
       <c r="BF3" s="172"/>
       <c r="BG3" s="172"/>
       <c r="BH3" s="172"/>
-      <c r="BI3" s="350"/>
+      <c r="BI3" s="349"/>
     </row>
     <row r="4" spans="1:61" s="168" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="173"/>
@@ -14816,7 +14833,7 @@
       <c r="O4" s="171" t="s">
         <v>96</v>
       </c>
-      <c r="P4" s="350"/>
+      <c r="P4" s="349"/>
       <c r="Q4" s="171" t="s">
         <v>95</v>
       </c>
@@ -14856,7 +14873,7 @@
       <c r="AC4" s="171" t="s">
         <v>83</v>
       </c>
-      <c r="AD4" s="350"/>
+      <c r="AD4" s="349"/>
       <c r="AE4" s="172" t="s">
         <v>82</v>
       </c>
@@ -14884,7 +14901,7 @@
       <c r="AM4" s="172" t="s">
         <v>74</v>
       </c>
-      <c r="AN4" s="350"/>
+      <c r="AN4" s="349"/>
       <c r="AQ4" s="171"/>
       <c r="AR4" s="171"/>
       <c r="AS4" s="171"/>
@@ -14893,7 +14910,7 @@
       <c r="AV4" s="171"/>
       <c r="AW4" s="171"/>
       <c r="AX4" s="171"/>
-      <c r="AY4" s="350"/>
+      <c r="AY4" s="349"/>
       <c r="AZ4" s="172"/>
       <c r="BA4" s="172"/>
       <c r="BB4" s="172"/>
@@ -14903,7 +14920,7 @@
       <c r="BF4" s="172"/>
       <c r="BG4" s="172"/>
       <c r="BH4" s="172"/>
-      <c r="BI4" s="350"/>
+      <c r="BI4" s="349"/>
     </row>
     <row r="5" spans="1:61" s="168" customFormat="1" ht="144" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="175" t="s">
@@ -16625,14 +16642,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="352" t="s">
+      <c r="A1" s="351" t="s">
         <v>228</v>
       </c>
-      <c r="B1" s="352"/>
-      <c r="C1" s="352"/>
-      <c r="D1" s="352"/>
-      <c r="E1" s="352"/>
-      <c r="F1" s="352"/>
+      <c r="B1" s="351"/>
+      <c r="C1" s="351"/>
+      <c r="D1" s="351"/>
+      <c r="E1" s="351"/>
+      <c r="F1" s="351"/>
       <c r="G1" s="200"/>
       <c r="H1" s="200"/>
       <c r="I1" s="200"/>
@@ -16682,7 +16699,7 @@
       <c r="O2" s="203" t="s">
         <v>178</v>
       </c>
-      <c r="P2" s="353" t="s">
+      <c r="P2" s="352" t="s">
         <v>227</v>
       </c>
       <c r="Q2" s="203" t="s">
@@ -16694,7 +16711,7 @@
       <c r="S2" s="203" t="s">
         <v>226</v>
       </c>
-      <c r="T2" s="353" t="s">
+      <c r="T2" s="352" t="s">
         <v>225</v>
       </c>
     </row>
@@ -16732,7 +16749,7 @@
       <c r="O3" s="203" t="s">
         <v>207</v>
       </c>
-      <c r="P3" s="353"/>
+      <c r="P3" s="352"/>
       <c r="Q3" s="203" t="s">
         <v>206</v>
       </c>
@@ -16742,7 +16759,7 @@
       <c r="S3" s="203" t="s">
         <v>136</v>
       </c>
-      <c r="T3" s="353"/>
+      <c r="T3" s="352"/>
     </row>
     <row r="4" spans="1:20" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="202"/>
@@ -16788,7 +16805,7 @@
       <c r="O4" s="203" t="s">
         <v>188</v>
       </c>
-      <c r="P4" s="353"/>
+      <c r="P4" s="352"/>
       <c r="Q4" s="203" t="s">
         <v>187</v>
       </c>
@@ -16798,7 +16815,7 @@
       <c r="S4" s="203" t="s">
         <v>83</v>
       </c>
-      <c r="T4" s="353"/>
+      <c r="T4" s="352"/>
     </row>
     <row r="5" spans="1:20" ht="317" x14ac:dyDescent="0.2">
       <c r="A5" s="206" t="s">
@@ -17384,16 +17401,16 @@
   <sheetData>
     <row r="1" spans="1:28" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="226"/>
-      <c r="B1" s="355" t="s">
+      <c r="B1" s="354" t="s">
         <v>184</v>
       </c>
-      <c r="C1" s="355"/>
-      <c r="D1" s="355"/>
-      <c r="E1" s="355"/>
-      <c r="F1" s="355"/>
-      <c r="G1" s="355"/>
-      <c r="H1" s="355"/>
-      <c r="I1" s="355"/>
+      <c r="C1" s="354"/>
+      <c r="D1" s="354"/>
+      <c r="E1" s="354"/>
+      <c r="F1" s="354"/>
+      <c r="G1" s="354"/>
+      <c r="H1" s="354"/>
+      <c r="I1" s="354"/>
       <c r="J1" s="223"/>
       <c r="K1" s="223"/>
       <c r="L1" s="223"/>
@@ -17424,7 +17441,7 @@
       <c r="G2" s="225" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="354" t="s">
+      <c r="H2" s="353" t="s">
         <v>182</v>
       </c>
       <c r="I2" s="228" t="s">
@@ -17469,7 +17486,7 @@
       <c r="V2" s="228" t="s">
         <v>181</v>
       </c>
-      <c r="W2" s="354" t="s">
+      <c r="W2" s="353" t="s">
         <v>180</v>
       </c>
       <c r="X2" s="225" t="s">
@@ -17484,7 +17501,7 @@
       <c r="AA2" s="225" t="s">
         <v>45</v>
       </c>
-      <c r="AB2" s="354" t="s">
+      <c r="AB2" s="353" t="s">
         <v>179</v>
       </c>
     </row>
@@ -17498,7 +17515,7 @@
       <c r="G3" s="225" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="354"/>
+      <c r="H3" s="353"/>
       <c r="I3" s="228" t="s">
         <v>171</v>
       </c>
@@ -17539,7 +17556,7 @@
       <c r="V3" s="228" t="s">
         <v>159</v>
       </c>
-      <c r="W3" s="354"/>
+      <c r="W3" s="353"/>
       <c r="X3" s="227"/>
       <c r="Y3" s="225" t="s">
         <v>158</v>
@@ -17550,7 +17567,7 @@
       <c r="AA3" s="225" t="s">
         <v>156</v>
       </c>
-      <c r="AB3" s="354"/>
+      <c r="AB3" s="353"/>
     </row>
     <row r="4" spans="1:28" ht="98" x14ac:dyDescent="0.2">
       <c r="A4" s="229"/>
@@ -17572,7 +17589,7 @@
       <c r="G4" s="225" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="354"/>
+      <c r="H4" s="353"/>
       <c r="I4" s="228" t="s">
         <v>121</v>
       </c>
@@ -17615,7 +17632,7 @@
       <c r="V4" s="231" t="s">
         <v>108</v>
       </c>
-      <c r="W4" s="354"/>
+      <c r="W4" s="353"/>
       <c r="X4" s="232" t="s">
         <v>107</v>
       </c>
@@ -17628,7 +17645,7 @@
       <c r="AA4" s="232" t="s">
         <v>104</v>
       </c>
-      <c r="AB4" s="354"/>
+      <c r="AB4" s="353"/>
     </row>
     <row r="5" spans="1:28" ht="196" x14ac:dyDescent="0.2">
       <c r="A5" s="233" t="s">
@@ -18522,16 +18539,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="357" t="s">
+      <c r="A1" s="356" t="s">
         <v>228</v>
       </c>
-      <c r="B1" s="357"/>
-      <c r="C1" s="357"/>
-      <c r="D1" s="357"/>
-      <c r="E1" s="357"/>
-      <c r="F1" s="357"/>
-      <c r="G1" s="357"/>
-      <c r="H1" s="357"/>
+      <c r="B1" s="356"/>
+      <c r="C1" s="356"/>
+      <c r="D1" s="356"/>
+      <c r="E1" s="356"/>
+      <c r="F1" s="356"/>
+      <c r="G1" s="356"/>
+      <c r="H1" s="356"/>
       <c r="I1" s="273"/>
       <c r="J1" s="273"/>
       <c r="K1" s="273"/>
@@ -18556,7 +18573,7 @@
       <c r="G2" s="275" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="356" t="s">
+      <c r="H2" s="355" t="s">
         <v>182</v>
       </c>
       <c r="I2" s="275" t="s">
@@ -18589,13 +18606,13 @@
       <c r="R2" s="275" t="s">
         <v>181</v>
       </c>
-      <c r="S2" s="356" t="s">
+      <c r="S2" s="355" t="s">
         <v>180</v>
       </c>
       <c r="T2" s="275" t="s">
         <v>45</v>
       </c>
-      <c r="U2" s="356" t="s">
+      <c r="U2" s="355" t="s">
         <v>179</v>
       </c>
     </row>
@@ -18609,7 +18626,7 @@
       <c r="G3" s="275" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="356"/>
+      <c r="H3" s="355"/>
       <c r="I3" s="275" t="s">
         <v>224</v>
       </c>
@@ -18640,11 +18657,11 @@
       <c r="R3" s="275" t="s">
         <v>159</v>
       </c>
-      <c r="S3" s="356"/>
+      <c r="S3" s="355"/>
       <c r="T3" s="275" t="s">
         <v>156</v>
       </c>
-      <c r="U3" s="356"/>
+      <c r="U3" s="355"/>
     </row>
     <row r="4" spans="1:21" ht="112" x14ac:dyDescent="0.2">
       <c r="A4" s="272"/>
@@ -18666,7 +18683,7 @@
       <c r="G4" s="275" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="356"/>
+      <c r="H4" s="355"/>
       <c r="I4" s="275" t="s">
         <v>205</v>
       </c>
@@ -18697,11 +18714,11 @@
       <c r="R4" s="275" t="s">
         <v>108</v>
       </c>
-      <c r="S4" s="356"/>
+      <c r="S4" s="355"/>
       <c r="T4" s="275" t="s">
         <v>104</v>
       </c>
-      <c r="U4" s="356"/>
+      <c r="U4" s="355"/>
     </row>
     <row r="5" spans="1:21" ht="196" x14ac:dyDescent="0.2">
       <c r="A5" s="278" t="s">
@@ -19392,13 +19409,13 @@
       <c r="K2" s="203" t="s">
         <v>181</v>
       </c>
-      <c r="L2" s="353" t="s">
+      <c r="L2" s="352" t="s">
         <v>180</v>
       </c>
       <c r="M2" s="203" t="s">
         <v>45</v>
       </c>
-      <c r="N2" s="353" t="s">
+      <c r="N2" s="352" t="s">
         <v>179</v>
       </c>
     </row>
@@ -19416,11 +19433,11 @@
       <c r="K3" s="203" t="s">
         <v>159</v>
       </c>
-      <c r="L3" s="353"/>
+      <c r="L3" s="352"/>
       <c r="M3" s="203" t="s">
         <v>156</v>
       </c>
-      <c r="N3" s="353"/>
+      <c r="N3" s="352"/>
     </row>
     <row r="4" spans="1:14" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="256"/>
@@ -19446,11 +19463,11 @@
       <c r="K4" s="203" t="s">
         <v>108</v>
       </c>
-      <c r="L4" s="353"/>
+      <c r="L4" s="352"/>
       <c r="M4" s="203" t="s">
         <v>104</v>
       </c>
-      <c r="N4" s="353"/>
+      <c r="N4" s="352"/>
     </row>
     <row r="5" spans="1:14" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="258"/>
@@ -20131,17 +20148,17 @@
       <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="FA1" s="339" t="s">
+      <c r="FA1" s="320" t="s">
         <v>237</v>
       </c>
-      <c r="FB1" s="339"/>
-      <c r="FC1" s="339"/>
-      <c r="FD1" s="339"/>
-      <c r="FE1" s="339"/>
-      <c r="FF1" s="339"/>
-      <c r="FG1" s="340"/>
-      <c r="FH1" s="340"/>
-      <c r="FI1" s="340"/>
+      <c r="FB1" s="320"/>
+      <c r="FC1" s="320"/>
+      <c r="FD1" s="320"/>
+      <c r="FE1" s="320"/>
+      <c r="FF1" s="320"/>
+      <c r="FG1" s="320"/>
+      <c r="FH1"/>
+      <c r="FI1"/>
       <c r="FJ1" s="4" t="s">
         <v>0</v>
       </c>
@@ -20191,9 +20208,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A2:DT2" xr:uid="{3B89445B-6ECC-4440-B85C-E593AE209933}"/>
-  <mergeCells count="1">
-    <mergeCell ref="FA1:FI1"/>
-  </mergeCells>
+  <conditionalFormatting sqref="A1:FG1048576">
+    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+      <formula>AND(OR($N1&lt;&gt;"-",$O1&lt;&gt;0,$P1&lt;&gt;0),ROW()&gt;2,$A1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
@@ -20282,28 +20301,28 @@
       <c r="D4" s="294"/>
       <c r="E4" s="294"/>
       <c r="F4" s="294"/>
-      <c r="G4" s="341" t="s">
+      <c r="G4" s="340" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="342"/>
-      <c r="I4" s="342"/>
-      <c r="J4" s="342"/>
-      <c r="K4" s="342"/>
-      <c r="L4" s="343"/>
-      <c r="M4" s="344"/>
-      <c r="N4" s="345" t="s">
+      <c r="H4" s="341"/>
+      <c r="I4" s="341"/>
+      <c r="J4" s="341"/>
+      <c r="K4" s="341"/>
+      <c r="L4" s="342"/>
+      <c r="M4" s="343"/>
+      <c r="N4" s="344" t="s">
         <v>27</v>
       </c>
-      <c r="O4" s="343"/>
-      <c r="P4" s="343"/>
-      <c r="Q4" s="343"/>
-      <c r="R4" s="343"/>
-      <c r="S4" s="343"/>
-      <c r="T4" s="346"/>
-      <c r="U4" s="341" t="s">
+      <c r="O4" s="342"/>
+      <c r="P4" s="342"/>
+      <c r="Q4" s="342"/>
+      <c r="R4" s="342"/>
+      <c r="S4" s="342"/>
+      <c r="T4" s="345"/>
+      <c r="U4" s="340" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="344"/>
+      <c r="V4" s="343"/>
       <c r="W4" s="301"/>
       <c r="X4" t="s">
         <v>0</v>
@@ -20500,70 +20519,70 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="15" priority="16">
+    <cfRule type="expression" dxfId="17" priority="16">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="14" priority="18">
+    <cfRule type="expression" dxfId="16" priority="18">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="13" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="15" priority="1" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3)+_xlfn.NUMBERVALUE($U4)+_xlfn.NUMBERVALUE($U5)+_xlfn.NUMBERVALUE($U6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="2" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3)+_xlfn.NUMBERVALUE($S4)+_xlfn.NUMBERVALUE($S5)+_xlfn.NUMBERVALUE($S6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="7" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="12" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="12" stopIfTrue="1">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",OR(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0,_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0,_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="6" stopIfTrue="1">
       <formula>OR(_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6),_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6),_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="8" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="11" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)+_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="15">
+    <cfRule type="expression" dxfId="9" priority="15">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="6" priority="5">
+    <cfRule type="expression" dxfId="8" priority="5">
       <formula>_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="5" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="10" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3)+_xlfn.NUMBERVALUE($S4)+_xlfn.NUMBERVALUE($S5)+_xlfn.NUMBERVALUE($S6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="14">
+    <cfRule type="expression" dxfId="6" priority="14">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="5" priority="4">
       <formula>_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="2" priority="9">
+    <cfRule type="expression" dxfId="4" priority="9">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3)+_xlfn.NUMBERVALUE($U4)+_xlfn.NUMBERVALUE($U5)+_xlfn.NUMBERVALUE($U6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="13">
+    <cfRule type="expression" dxfId="3" priority="13">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -20940,16 +20959,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:62" s="44" customFormat="1" ht="23.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B1" s="348" t="s">
+      <c r="B1" s="347" t="s">
         <v>184</v>
       </c>
-      <c r="C1" s="348"/>
-      <c r="D1" s="348"/>
-      <c r="E1" s="348"/>
-      <c r="F1" s="348"/>
-      <c r="G1" s="348"/>
-      <c r="H1" s="348"/>
-      <c r="I1" s="348"/>
+      <c r="C1" s="347"/>
+      <c r="D1" s="347"/>
+      <c r="E1" s="347"/>
+      <c r="F1" s="347"/>
+      <c r="G1" s="347"/>
+      <c r="H1" s="347"/>
+      <c r="I1" s="347"/>
     </row>
     <row r="2" spans="1:62" s="44" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="90"/>
@@ -20961,7 +20980,7 @@
       <c r="G2" s="87" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="347" t="s">
+      <c r="H2" s="346" t="s">
         <v>182</v>
       </c>
       <c r="I2" s="86" t="s">
@@ -21006,7 +21025,7 @@
       <c r="V2" s="86" t="s">
         <v>181</v>
       </c>
-      <c r="W2" s="347" t="s">
+      <c r="W2" s="346" t="s">
         <v>180</v>
       </c>
       <c r="X2" s="87" t="s">
@@ -21021,7 +21040,7 @@
       <c r="AA2" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="AB2" s="347" t="s">
+      <c r="AB2" s="346" t="s">
         <v>179</v>
       </c>
       <c r="AC2" s="84" t="s">
@@ -21051,7 +21070,7 @@
       <c r="AK2" s="84" t="s">
         <v>178</v>
       </c>
-      <c r="AL2" s="347" t="s">
+      <c r="AL2" s="346" t="s">
         <v>177</v>
       </c>
       <c r="AM2" s="84" t="s">
@@ -21093,7 +21112,7 @@
       <c r="AY2" s="84" t="s">
         <v>176</v>
       </c>
-      <c r="AZ2" s="347" t="s">
+      <c r="AZ2" s="346" t="s">
         <v>175</v>
       </c>
       <c r="BA2" s="83" t="s">
@@ -21123,7 +21142,7 @@
       <c r="BI2" s="83" t="s">
         <v>174</v>
       </c>
-      <c r="BJ2" s="347" t="s">
+      <c r="BJ2" s="346" t="s">
         <v>173</v>
       </c>
     </row>
@@ -21137,7 +21156,7 @@
       <c r="G3" s="87" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="347"/>
+      <c r="H3" s="346"/>
       <c r="I3" s="86" t="s">
         <v>171</v>
       </c>
@@ -21178,7 +21197,7 @@
       <c r="V3" s="86" t="s">
         <v>159</v>
       </c>
-      <c r="W3" s="347"/>
+      <c r="W3" s="346"/>
       <c r="X3" s="82"/>
       <c r="Y3" s="87" t="s">
         <v>158</v>
@@ -21189,7 +21208,7 @@
       <c r="AA3" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="AB3" s="347"/>
+      <c r="AB3" s="346"/>
       <c r="AC3" s="84" t="s">
         <v>155</v>
       </c>
@@ -21217,7 +21236,7 @@
       <c r="AK3" s="84" t="s">
         <v>149</v>
       </c>
-      <c r="AL3" s="347"/>
+      <c r="AL3" s="346"/>
       <c r="AM3" s="84" t="s">
         <v>148</v>
       </c>
@@ -21257,7 +21276,7 @@
       <c r="AY3" s="84" t="s">
         <v>136</v>
       </c>
-      <c r="AZ3" s="347"/>
+      <c r="AZ3" s="346"/>
       <c r="BA3" s="83" t="s">
         <v>135</v>
       </c>
@@ -21285,7 +21304,7 @@
       <c r="BI3" s="83" t="s">
         <v>127</v>
       </c>
-      <c r="BJ3" s="347"/>
+      <c r="BJ3" s="346"/>
     </row>
     <row r="4" spans="1:62" s="44" customFormat="1" ht="60" x14ac:dyDescent="0.15">
       <c r="A4" s="89"/>
@@ -21307,7 +21326,7 @@
       <c r="G4" s="87" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="347"/>
+      <c r="H4" s="346"/>
       <c r="I4" s="86" t="s">
         <v>121</v>
       </c>
@@ -21350,7 +21369,7 @@
       <c r="V4" s="86" t="s">
         <v>108</v>
       </c>
-      <c r="W4" s="347"/>
+      <c r="W4" s="346"/>
       <c r="X4" s="85" t="s">
         <v>107</v>
       </c>
@@ -21363,7 +21382,7 @@
       <c r="AA4" s="85" t="s">
         <v>104</v>
       </c>
-      <c r="AB4" s="347"/>
+      <c r="AB4" s="346"/>
       <c r="AC4" s="84" t="s">
         <v>103</v>
       </c>
@@ -21391,7 +21410,7 @@
       <c r="AK4" s="84" t="s">
         <v>96</v>
       </c>
-      <c r="AL4" s="347"/>
+      <c r="AL4" s="346"/>
       <c r="AM4" s="84" t="s">
         <v>95</v>
       </c>
@@ -21431,7 +21450,7 @@
       <c r="AY4" s="84" t="s">
         <v>83</v>
       </c>
-      <c r="AZ4" s="347"/>
+      <c r="AZ4" s="346"/>
       <c r="BA4" s="83" t="s">
         <v>82</v>
       </c>
@@ -21459,7 +21478,7 @@
       <c r="BI4" s="83" t="s">
         <v>74</v>
       </c>
-      <c r="BJ4" s="347"/>
+      <c r="BJ4" s="346"/>
     </row>
     <row r="5" spans="1:62" s="44" customFormat="1" ht="11" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="54" t="s">
@@ -23648,16 +23667,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A1" s="349" t="s">
+      <c r="A1" s="348" t="s">
         <v>228</v>
       </c>
-      <c r="B1" s="349"/>
-      <c r="C1" s="349"/>
-      <c r="D1" s="349"/>
-      <c r="E1" s="349"/>
-      <c r="F1" s="349"/>
-      <c r="G1" s="349"/>
-      <c r="H1" s="349"/>
+      <c r="B1" s="348"/>
+      <c r="C1" s="348"/>
+      <c r="D1" s="348"/>
+      <c r="E1" s="348"/>
+      <c r="F1" s="348"/>
+      <c r="G1" s="348"/>
+      <c r="H1" s="348"/>
       <c r="I1" s="44"/>
       <c r="J1" s="44"/>
       <c r="K1" s="44"/>
@@ -23696,7 +23715,7 @@
       <c r="G2" s="87" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="347" t="s">
+      <c r="H2" s="346" t="s">
         <v>182</v>
       </c>
       <c r="I2" s="87" t="s">
@@ -23729,13 +23748,13 @@
       <c r="R2" s="87" t="s">
         <v>181</v>
       </c>
-      <c r="S2" s="347" t="s">
+      <c r="S2" s="346" t="s">
         <v>180</v>
       </c>
       <c r="T2" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="U2" s="347" t="s">
+      <c r="U2" s="346" t="s">
         <v>179</v>
       </c>
       <c r="V2" s="87" t="s">
@@ -23765,7 +23784,7 @@
       <c r="AD2" s="87" t="s">
         <v>178</v>
       </c>
-      <c r="AE2" s="347" t="s">
+      <c r="AE2" s="346" t="s">
         <v>227</v>
       </c>
       <c r="AF2" s="87" t="s">
@@ -23777,7 +23796,7 @@
       <c r="AH2" s="87" t="s">
         <v>226</v>
       </c>
-      <c r="AI2" s="347" t="s">
+      <c r="AI2" s="346" t="s">
         <v>225</v>
       </c>
     </row>
@@ -23791,7 +23810,7 @@
       <c r="G3" s="87" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="347"/>
+      <c r="H3" s="346"/>
       <c r="I3" s="87" t="s">
         <v>224</v>
       </c>
@@ -23822,11 +23841,11 @@
       <c r="R3" s="87" t="s">
         <v>159</v>
       </c>
-      <c r="S3" s="347"/>
+      <c r="S3" s="346"/>
       <c r="T3" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="U3" s="347"/>
+      <c r="U3" s="346"/>
       <c r="V3" s="87" t="s">
         <v>215</v>
       </c>
@@ -23854,7 +23873,7 @@
       <c r="AD3" s="87" t="s">
         <v>207</v>
       </c>
-      <c r="AE3" s="347"/>
+      <c r="AE3" s="346"/>
       <c r="AF3" s="87" t="s">
         <v>206</v>
       </c>
@@ -23864,7 +23883,7 @@
       <c r="AH3" s="87" t="s">
         <v>136</v>
       </c>
-      <c r="AI3" s="347"/>
+      <c r="AI3" s="346"/>
     </row>
     <row r="4" spans="1:35" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="90"/>
@@ -23886,7 +23905,7 @@
       <c r="G4" s="87" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="347"/>
+      <c r="H4" s="346"/>
       <c r="I4" s="87" t="s">
         <v>205</v>
       </c>
@@ -23917,11 +23936,11 @@
       <c r="R4" s="87" t="s">
         <v>108</v>
       </c>
-      <c r="S4" s="347"/>
+      <c r="S4" s="346"/>
       <c r="T4" s="87" t="s">
         <v>104</v>
       </c>
-      <c r="U4" s="347"/>
+      <c r="U4" s="346"/>
       <c r="V4" s="87" t="s">
         <v>196</v>
       </c>
@@ -23949,7 +23968,7 @@
       <c r="AD4" s="87" t="s">
         <v>188</v>
       </c>
-      <c r="AE4" s="347"/>
+      <c r="AE4" s="346"/>
       <c r="AF4" s="87" t="s">
         <v>187</v>
       </c>
@@ -23959,7 +23978,7 @@
       <c r="AH4" s="87" t="s">
         <v>83</v>
       </c>
-      <c r="AI4" s="347"/>
+      <c r="AI4" s="346"/>
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A5" s="93" t="s">

</xml_diff>

<commit_message>
update mme DE JONG full matrice
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57A7E359-D53B-D241-8BBF-656D9D6D4728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3995F21F-6950-954B-9481-B601979F7EA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" activeTab="2" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -5289,7 +5289,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="32">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5473,6 +5473,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -5955,7 +5961,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="357">
+  <cellXfs count="359">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -7145,6 +7151,14 @@
     </xf>
     <xf numFmtId="0" fontId="53" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="32" borderId="12" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="65" fillId="13" borderId="12" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
       <protection hidden="1"/>
     </xf>
   </cellXfs>
@@ -7156,27 +7170,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
     <cellStyle name="Normal 3" xfId="4" xr:uid="{6BD57324-3FD5-D341-A299-730D14794802}"/>
   </cellStyles>
-  <dxfs count="18">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="17">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -7336,6 +7330,16 @@
       <font>
         <color theme="0"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -20209,7 +20213,7 @@
   </sheetData>
   <autoFilter ref="A2:DT2" xr:uid="{3B89445B-6ECC-4440-B85C-E593AE209933}"/>
   <conditionalFormatting sqref="A1:FG1048576">
-    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="16" priority="1" stopIfTrue="1">
       <formula>AND(OR($N1&lt;&gt;"-",$O1&lt;&gt;0,$P1&lt;&gt;0),ROW()&gt;2,$A1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -20400,7 +20404,7 @@
         <v>399</v>
       </c>
       <c r="G6" s="19" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"M-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FG,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"M-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="H6" s="298" t="str">
@@ -20408,16 +20412,16 @@
         <v/>
       </c>
       <c r="I6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"M-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FG,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"M-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="J6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"M-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FG,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"M-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="K6" s="18" t="e">
         <f>SUMIFS(
-INDEX('ETPT Format DDG'!$A:$DU,
+INDEX('ETPT Format DDG'!$A:$FG,
 ,
 IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
 ),'ETPT Format DDG'!$FG:$FG,"C",
@@ -20427,7 +20431,7 @@
       </c>
       <c r="L6" s="19" t="e">
         <f>ROUND(SUMIFS(
-INDEX('ETPT Format DDG'!$A:$DU,
+INDEX('ETPT Format DDG'!$A:$FG,
 ,
 IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
 ),
@@ -20440,7 +20444,7 @@
         <v/>
       </c>
       <c r="N6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"F-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FG,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"F-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="O6" s="298" t="str">
@@ -20448,20 +20452,20 @@
         <v/>
       </c>
       <c r="P6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"F-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FG,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"F-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="Q6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"F-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FG,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"F-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="R6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$DU,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"C",'ETPT Format DDG'!$C:$C,$A$3,'ETPT Format DDG'!$G:$G,"Greffe")</f>
+        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FG,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FG:$FG,"C",'ETPT Format DDG'!$C:$C,$A$3,'ETPT Format DDG'!$G:$G,"Greffe")</f>
         <v>#N/A</v>
       </c>
       <c r="S6" s="19" t="e">
         <f>ROUND(SUMIFS(
-INDEX('ETPT Format DDG'!$A:$DU,
+INDEX('ETPT Format DDG'!$A:$FG,
 ,
 IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
 ),
@@ -20475,7 +20479,7 @@
       </c>
       <c r="U6" s="19" t="e">
         <f>ROUND(SUMIFS(
-INDEX('ETPT Format DDG'!$A:$DU,
+INDEX('ETPT Format DDG'!$A:$FG,
 ,
 IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
 ),'ETPT Format DDG'!$FG:$FG,"C",
@@ -20519,70 +20523,70 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="17" priority="16">
+    <cfRule type="expression" dxfId="15" priority="16">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="16" priority="18">
+    <cfRule type="expression" dxfId="14" priority="18">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="15" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="1" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3)+_xlfn.NUMBERVALUE($U4)+_xlfn.NUMBERVALUE($U5)+_xlfn.NUMBERVALUE($U6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="2" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3)+_xlfn.NUMBERVALUE($S4)+_xlfn.NUMBERVALUE($S5)+_xlfn.NUMBERVALUE($S6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="7" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="12" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="12" stopIfTrue="1">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",OR(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0,_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0,_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="11" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
       <formula>OR(_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6),_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6),_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="10" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="8" priority="11" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)+_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="15">
+    <cfRule type="expression" dxfId="7" priority="15">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="8" priority="5">
+    <cfRule type="expression" dxfId="6" priority="5">
       <formula>_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="7" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="10" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3)+_xlfn.NUMBERVALUE($S4)+_xlfn.NUMBERVALUE($S5)+_xlfn.NUMBERVALUE($S6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="14">
+    <cfRule type="expression" dxfId="4" priority="14">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="5" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="4" priority="9">
+    <cfRule type="expression" dxfId="2" priority="9">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3)+_xlfn.NUMBERVALUE($U4)+_xlfn.NUMBERVALUE($U5)+_xlfn.NUMBERVALUE($U6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="13">
+    <cfRule type="expression" dxfId="1" priority="13">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -21613,46 +21617,42 @@
       <c r="AQ5" s="75"/>
       <c r="AR5" s="75"/>
       <c r="AS5" s="58" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1.1. DÉPARTAGE PRUD'HOMAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1.1. DÉPARTAGE PRUD'HOMAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1.1. DÉPARTAGE PRUD'HOMAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
         <v>#N/A</v>
       </c>
       <c r="AT5" s="56" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
         <v>#N/A</v>
       </c>
       <c r="AU5" s="56" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")</f>
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
         <v>#N/A</v>
       </c>
       <c r="AV5" s="56" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1.1. DÉPARTAGE PRUD'HOMAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1.1. DÉPARTAGE PRUD'HOMAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1.1. DÉPARTAGE PRUD'HOMAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
         <v>#N/A</v>
       </c>
       <c r="AW5" s="165" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("2. TOTAL CONTENTIEUX JAF",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("2. TOTAL CONTENTIEUX JAF",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("2. TOTAL CONTENTIEUX JAF",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
         <v>#N/A</v>
       </c>
       <c r="AX5" s="58" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (contentieux civils et sociaux)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3. TOTAL CONTENTIEUX DE LA PROTECTION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("6.1. ACTIVITÉ CIVILE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("5. TOTAL JLD CIVIL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("4. TOTAL CIVIL NON SPÉCIALISÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
         <v>#N/A</v>
       </c>
       <c r="AY5" s="58" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (contentieux civils et sociaux)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
-(SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3. TOTAL CONTENTIEUX DE LA PROTECTION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS"))-
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("6.1. ACTIVITÉ CIVILE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("5. TOTAL JLD CIVIL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
-SUM(AS5:AW5)</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("4. TOTAL CIVIL NON SPÉCIALISÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")</f>
         <v>#N/A</v>
       </c>
       <c r="AZ5" s="49" t="e">
@@ -21852,7 +21852,15 @@
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("8.4. AUTRES SECTIONS SPÉCIALISÉES",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9. TOTAL JAP",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("6.2. ACTIVITÉ PÉNALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("10. TOTAL JLD PÉNAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("10. TOTAL JLD PÉNAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("7.5. COUR D'ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("7.51. COUR D'ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("7.52. COUR CRIMINELLE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("7.121. COLLÉGIALES JIRS ECO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("7.12. COLLÉGIALES JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("7.122. COLLÉGIALES AUTRES SECTIONS SPÉCIALISÉES",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("7.6. TRIBUNAL DE POLICE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("7.7. OP CONTRAVENTIONNELLES",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
         <v>#N/A</v>
       </c>
       <c r="AY6" s="74" t="e">
@@ -21864,7 +21872,14 @@
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("9. TOTAL JAP",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("6.2. ACTIVITÉ PÉNALE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("10. TOTAL JLD PÉNAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
-SUM(AM6:AW6)</f>
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("7.5. COUR D'ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("7.51. COUR D'ASSISES JIRS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("7.52. COUR CRIMINELLE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("7.121. COLLÉGIALES JIRS ECO-FI",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("7.12. COLLÉGIALES JIRS CRIM-ORG",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("7.122. COLLÉGIALES AUTRES SECTIONS SPÉCIALISÉES",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("7.6. TRIBUNAL DE POLICE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("7.7. OP CONTRAVENTIONNELLES",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")</f>
         <v>#N/A</v>
       </c>
       <c r="AZ6" s="49" t="e">
@@ -22638,13 +22653,19 @@
       <c r="AD12" s="56" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"JCP")+
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"VPCP")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPCP")</f>
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPCP")-
+(SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"JCP")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"VPCP")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPCP"))</f>
         <v>#N/A</v>
       </c>
       <c r="AE12" s="56" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"JI")+
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"VPI")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPI")</f>
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPI")-
+(SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"JI")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"VPI")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AF12" s="66"/>
@@ -22653,18 +22674,26 @@
       <c r="AI12" s="56" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"JAP")+
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"VPAP")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPAP")</f>
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPAP")-
+(SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"JAP")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"VPAP")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPAP"))</f>
         <v>#N/A</v>
       </c>
       <c r="AJ12" s="56" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"JE")+
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"VPE")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPE")</f>
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPE")-
+(SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"JE")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"VPE")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPE"))</f>
         <v>#N/A</v>
       </c>
       <c r="AK12" s="56" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"VPLD")+
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPLD")</f>
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPLD")-
+(SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"VPLD")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"1VPLD"))</f>
         <v>#N/A</v>
       </c>
       <c r="AL12" s="49" t="e">
@@ -22684,7 +22713,8 @@
       <c r="AW12" s="66"/>
       <c r="AX12" s="66"/>
       <c r="AY12" s="56" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")</f>
         <v>#N/A</v>
       </c>
       <c r="AZ12" s="49" t="e">
@@ -22820,7 +22850,7 @@
       <c r="AW13" s="66"/>
       <c r="AX13" s="66"/>
       <c r="AY13" s="303" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$H:$H,"Magistrat SIEGE NS")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")</f>
         <v>#N/A</v>
       </c>
       <c r="AZ13" s="49" t="e">
@@ -22857,13 +22887,13 @@
       <c r="F14" s="64" t="s">
         <v>54</v>
       </c>
-      <c r="G14" s="63">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilé sur la période (y.c. indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé ADD")</f>
-        <v>0</v>
-      </c>
-      <c r="H14" s="62">
+      <c r="G14" s="63" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("ETPT sur la période hors indisponibilités",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé ADD")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H14" s="62" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>#N/A</v>
       </c>
       <c r="I14" s="61" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.8. FONCTIONNAIRES AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")</f>
@@ -22931,7 +22961,7 @@
         <v>#N/A</v>
       </c>
       <c r="V14" s="166" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilé sur la période (y.c. indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")-
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("ETPT sur la période hors indisponibilités",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")-
 SUM(I14:U14)-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.7. FONCTIONNAIRES AFFECTÉS AU CPH",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé ADD")</f>
         <v>#N/A</v>
       </c>
@@ -23042,7 +23072,7 @@
       </c>
       <c r="AX14" s="57"/>
       <c r="AY14" s="56" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilé sur la période (y.c. indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")-SUM(AC14:AK14)-SUM(AM14:AX14)</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("ETPT sur la période hors indisponibilités",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")-SUM(AC14:AK14)-SUM(AM14:AX14)</f>
         <v>#N/A</v>
       </c>
       <c r="AZ14" s="49" t="e">
@@ -23079,13 +23109,13 @@
       <c r="F15" s="64" t="s">
         <v>51</v>
       </c>
-      <c r="G15" s="63">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilé sur la période (y.c. indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé SUB")</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="62">
+      <c r="G15" s="63" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("ETPT sur la période hors indisponibilités",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé SUB")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H15" s="62" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>#N/A</v>
       </c>
       <c r="I15" s="61" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.8. FONCTIONNAIRES AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")</f>
@@ -23153,7 +23183,7 @@
         <v>#N/A</v>
       </c>
       <c r="V15" s="166" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilé sur la période (y.c. indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")-
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("ETPT sur la période hors indisponibilités",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")-
 SUM(I15:U15)-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.7. FONCTIONNAIRES AFFECTÉS AU CPH",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé SUB")</f>
         <v>#N/A</v>
       </c>
@@ -23264,7 +23294,7 @@
       </c>
       <c r="AX15" s="57"/>
       <c r="AY15" s="56" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilé sur la période (y.c. indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")-SUM(AC15:AK15)-SUM(AM15:AX15)</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("ETPT sur la période hors indisponibilités",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")-SUM(AC15:AK15)-SUM(AM15:AX15)</f>
         <v>#N/A</v>
       </c>
       <c r="AZ15" s="49" t="e">
@@ -24059,8 +24089,8 @@
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
         <v>#N/A</v>
       </c>
-      <c r="Z5" s="164"/>
-      <c r="AA5" s="164"/>
+      <c r="Z5" s="57"/>
+      <c r="AA5" s="57"/>
       <c r="AB5" s="57"/>
       <c r="AC5" s="57"/>
       <c r="AD5" s="57"/>
@@ -24074,7 +24104,11 @@
         <v>#N/A</v>
       </c>
       <c r="AH5" s="56" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (contentieux civils et sociaux)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-SUM(V5:AD5)-AF5-AG5-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("6.1. ACTIVITÉ CIVILE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("5. TOTAL JLD CIVIL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("2. TOTAL CONTENTIEUX JAF",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilés sur la période (contentieux civils et sociaux)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3. TOTAL CONTENTIEUX DE LA PROTECTION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1.1. DÉPARTAGE PRUD'HOMAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("6.1. ACTIVITÉ CIVILE",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("5. TOTAL JLD CIVIL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("2. TOTAL CONTENTIEUX JAF",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
         <v>#N/A</v>
       </c>
       <c r="AI5" s="94" t="e">
@@ -24187,8 +24221,8 @@
       <c r="W7" s="66"/>
       <c r="X7" s="66"/>
       <c r="Y7" s="66"/>
-      <c r="Z7" s="66"/>
-      <c r="AA7" s="66"/>
+      <c r="Z7" s="57"/>
+      <c r="AA7" s="57"/>
       <c r="AB7" s="57"/>
       <c r="AC7" s="57"/>
       <c r="AD7" s="57"/>
@@ -24257,8 +24291,8 @@
       <c r="W8" s="66"/>
       <c r="X8" s="66"/>
       <c r="Y8" s="66"/>
-      <c r="Z8" s="66"/>
-      <c r="AA8" s="66"/>
+      <c r="Z8" s="57"/>
+      <c r="AA8" s="57"/>
       <c r="AB8" s="57"/>
       <c r="AC8" s="57"/>
       <c r="AD8" s="57"/>
@@ -24268,13 +24302,10 @@
       </c>
       <c r="AF8" s="66"/>
       <c r="AG8" s="66"/>
-      <c r="AH8" s="61" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.51. ACCUEIL DU JUSTICIABLE (DONT SAUJ)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AI8" s="94" t="e">
+      <c r="AH8" s="66"/>
+      <c r="AI8" s="94">
         <f t="shared" si="4"/>
-        <v>#N/A</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:35" x14ac:dyDescent="0.2">
@@ -24337,8 +24368,8 @@
       <c r="W9" s="66"/>
       <c r="X9" s="66"/>
       <c r="Y9" s="66"/>
-      <c r="Z9" s="66"/>
-      <c r="AA9" s="66"/>
+      <c r="Z9" s="57"/>
+      <c r="AA9" s="57"/>
       <c r="AB9" s="57"/>
       <c r="AC9" s="57"/>
       <c r="AD9" s="57"/>
@@ -24412,8 +24443,8 @@
       <c r="W10" s="66"/>
       <c r="X10" s="66"/>
       <c r="Y10" s="66"/>
-      <c r="Z10" s="66"/>
-      <c r="AA10" s="66"/>
+      <c r="Z10" s="57"/>
+      <c r="AA10" s="57"/>
       <c r="AB10" s="57"/>
       <c r="AC10" s="57"/>
       <c r="AD10" s="57"/>
@@ -24485,8 +24516,8 @@
       <c r="W11" s="66"/>
       <c r="X11" s="66"/>
       <c r="Y11" s="66"/>
-      <c r="Z11" s="66"/>
-      <c r="AA11" s="66"/>
+      <c r="Z11" s="57"/>
+      <c r="AA11" s="57"/>
       <c r="AB11" s="57"/>
       <c r="AC11" s="57"/>
       <c r="AD11" s="57"/>
@@ -24561,8 +24592,8 @@
       <c r="W12" s="66"/>
       <c r="X12" s="66"/>
       <c r="Y12" s="66"/>
-      <c r="Z12" s="66"/>
-      <c r="AA12" s="66"/>
+      <c r="Z12" s="57"/>
+      <c r="AA12" s="57"/>
       <c r="AB12" s="57"/>
       <c r="AC12" s="57"/>
       <c r="AD12" s="57"/>
@@ -24573,7 +24604,8 @@
       <c r="AF12" s="66"/>
       <c r="AG12" s="66"/>
       <c r="AH12" s="56" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12. TOTAL INDISPONIBILITÉ",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
         <v>#N/A</v>
       </c>
       <c r="AI12" s="94" t="e">
@@ -24634,8 +24666,8 @@
       <c r="W13" s="66"/>
       <c r="X13" s="66"/>
       <c r="Y13" s="66"/>
-      <c r="Z13" s="66"/>
-      <c r="AA13" s="66"/>
+      <c r="Z13" s="57"/>
+      <c r="AA13" s="57"/>
       <c r="AB13" s="57"/>
       <c r="AC13" s="57"/>
       <c r="AD13" s="57"/>
@@ -24645,7 +24677,7 @@
       </c>
       <c r="AF13" s="66"/>
       <c r="AG13" s="66"/>
-      <c r="AH13" s="303" t="e">
+      <c r="AH13" s="358" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
         <v>#N/A</v>
       </c>
@@ -24670,13 +24702,13 @@
       <c r="F14" s="65" t="s">
         <v>54</v>
       </c>
-      <c r="G14" s="63">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilé sur la période (y.c. indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé ADD")</f>
-        <v>0</v>
-      </c>
-      <c r="H14" s="94">
+      <c r="G14" s="63" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("ETPT sur la période hors indisponibilités",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé ADD")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H14" s="94" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>#N/A</v>
       </c>
       <c r="I14" s="95"/>
       <c r="J14" s="61" t="e">
@@ -24700,8 +24732,9 @@
       <c r="O14" s="57"/>
       <c r="P14" s="57"/>
       <c r="Q14" s="66"/>
-      <c r="R14" s="166" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilé sur la période (y.c. indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")-SUM(I14:Q14)-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.7. FONCTIONNAIRES AFFECTÉS AU CPH",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé ADD")</f>
+      <c r="R14" s="357" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("ETPT sur la période hors indisponibilités",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé ADD")-SUM(I14:Q14)-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.7. FONCTIONNAIRES AFFECTÉS AU CPH",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé ADD")</f>
         <v>#N/A</v>
       </c>
       <c r="S14" s="49" t="e">
@@ -24730,13 +24763,13 @@
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")</f>
         <v>#N/A</v>
       </c>
-      <c r="Z14" s="164"/>
-      <c r="AA14" s="164"/>
+      <c r="Z14" s="57"/>
+      <c r="AA14" s="57"/>
       <c r="AB14" s="57"/>
       <c r="AC14" s="57"/>
       <c r="AD14" s="57"/>
       <c r="AE14" s="94" t="e">
-        <f t="shared" si="3"/>
+        <f>SUM(V14:AD14)</f>
         <v>#N/A</v>
       </c>
       <c r="AF14" s="57"/>
@@ -24744,8 +24777,8 @@
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1.1. DÉPARTAGE PRUD'HOMAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")</f>
         <v>#N/A</v>
       </c>
-      <c r="AH14" s="165" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilé sur la période (y.c. indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")-SUM(AE14:AG14)</f>
+      <c r="AH14" s="56" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("ETPT sur la période hors indisponibilités",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé ADD")-SUM(V14:AD14)-SUM(AF14:AG14)</f>
         <v>#N/A</v>
       </c>
       <c r="AI14" s="94" t="e">
@@ -24769,13 +24802,13 @@
       <c r="F15" s="65" t="s">
         <v>51</v>
       </c>
-      <c r="G15" s="63">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilé sur la période (y.c. indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé SUB")</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="94">
+      <c r="G15" s="63" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("ETPT sur la période hors indisponibilités",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé SUB")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H15" s="94" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>#N/A</v>
       </c>
       <c r="I15" s="95"/>
       <c r="J15" s="61" t="e">
@@ -24799,8 +24832,9 @@
       <c r="O15" s="57"/>
       <c r="P15" s="57"/>
       <c r="Q15" s="66"/>
-      <c r="R15" s="166" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilé sur la période (y.c. indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")-SUM(I15:Q15)-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.7. FONCTIONNAIRES AFFECTÉS AU CPH",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé SUB")</f>
+      <c r="R15" s="357" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("ETPT sur la période hors indisponibilités",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire A-B-CBUR placé SUB")-SUM(I15:Q15)-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("11.7. FONCTIONNAIRES AFFECTÉS AU CPH",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Fonctionnaire CTECH placé SUB")</f>
         <v>#N/A</v>
       </c>
       <c r="S15" s="49" t="e">
@@ -24829,8 +24863,8 @@
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")</f>
         <v>#N/A</v>
       </c>
-      <c r="Z15" s="164"/>
-      <c r="AA15" s="164"/>
+      <c r="Z15" s="57"/>
+      <c r="AA15" s="57"/>
       <c r="AB15" s="57"/>
       <c r="AC15" s="57"/>
       <c r="AD15" s="57"/>
@@ -24843,8 +24877,8 @@
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("1.1. DÉPARTAGE PRUD'HOMAL",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")</f>
         <v>#N/A</v>
       </c>
-      <c r="AH15" s="165" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("Temps ventilé sur la période (y.c. indisponibilité)",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")-SUM(AE15:AG15)</f>
+      <c r="AH15" s="56" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("ETPT sur la période hors indisponibilités",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat placé SUB")-SUM(V15:AD15)-SUM(AF15:AG15)</f>
         <v>#N/A</v>
       </c>
       <c r="AI15" s="94" t="e">

</xml_diff>

<commit_message>
extractor add ns tprox W X Y col
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3995F21F-6950-954B-9481-B601979F7EA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C54CD53-D25B-7142-9BDF-EB6E9B501194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -24075,18 +24075,25 @@
       <c r="V5" s="60"/>
       <c r="W5" s="61" t="e">
         <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="X5" s="61" t="e">
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3. TOTAL CONTENTIEUX DE LA PROTECTION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3. TOTAL CONTENTIEUX DE LA PROTECTION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")-
 SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
         <v>#N/A</v>
       </c>
-      <c r="X5" s="61" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3. TOTAL CONTENTIEUX DE LA PROTECTION",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")-
-SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
-        <v>#N/A</v>
-      </c>
       <c r="Y5" s="61" t="e">
-        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")</f>
+        <f>SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE S")+
+SUMIFS( INDEX( 'ETPT Format DDG'!$A:$FF,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),'ETPT Format DDG'!$C:$C,$D$5,'ETPT Format DDG'!$FA:$FA,"Magistrat SIEGE NS")</f>
         <v>#N/A</v>
       </c>
       <c r="Z5" s="57"/>

</xml_diff>

<commit_message>
automatisation des formules CA
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,29 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BD38D8C-2855-4A4F-8DA1-232A21640553}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26444862-8F27-8C4D-A082-DAFA947950F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="2" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
     <sheet name="ETPT A-JUST" sheetId="1" r:id="rId2"/>
     <sheet name="ETPT Format DDG" sheetId="9" r:id="rId3"/>
     <sheet name="Agrégats DDG" sheetId="10" r:id="rId4"/>
-    <sheet name="codage tribunal" sheetId="12" r:id="rId5"/>
-    <sheet name="Juridictions" sheetId="17" r:id="rId6"/>
-    <sheet name="Table_Fonctions" sheetId="19" r:id="rId7"/>
-    <sheet name="ETPT_TJ" sheetId="25" r:id="rId8"/>
-    <sheet name="ETPT_TPRX" sheetId="26" r:id="rId9"/>
-    <sheet name="ETPT_CPH" sheetId="27" r:id="rId10"/>
+    <sheet name="codage tribunal" sheetId="12" state="hidden" r:id="rId5"/>
+    <sheet name="Juridictions" sheetId="17" state="hidden" r:id="rId6"/>
+    <sheet name="Table_Fonctions" sheetId="19" state="hidden" r:id="rId7"/>
+    <sheet name="ETPT_TJ" sheetId="25" state="hidden" r:id="rId8"/>
+    <sheet name="ETPT_TPRX" sheetId="26" state="hidden" r:id="rId9"/>
+    <sheet name="ETPT_CPH" sheetId="27" state="hidden" r:id="rId10"/>
     <sheet name="ETPT_TJ_DDG" sheetId="28" r:id="rId11"/>
     <sheet name="ETPT_TPRX_DDG" sheetId="29" r:id="rId12"/>
     <sheet name="ETPT_CPH_DDG" sheetId="30" r:id="rId13"/>
-    <sheet name="ETPT_TJ_corresp-SIEGE-TJ" sheetId="24" r:id="rId14"/>
-    <sheet name="ETPT_TPROX_corresp-SIEGE-TPROX" sheetId="34" r:id="rId15"/>
-    <sheet name="ETPT_TJ_corresp-GREFFE-TJ" sheetId="35" r:id="rId16"/>
-    <sheet name="ETPT_TROX_corresp-GREFFE-TPROX" sheetId="36" r:id="rId17"/>
-    <sheet name="ETPT_CPH_corresp-GREFFE-CPH" sheetId="37" r:id="rId18"/>
+    <sheet name="ETPT_TJ_corresp-SIEGE-TJ" sheetId="24" state="hidden" r:id="rId14"/>
+    <sheet name="ETPT_TPROX_corresp-SIEGE-TPROX" sheetId="34" state="hidden" r:id="rId15"/>
+    <sheet name="ETPT_TJ_corresp-GREFFE-TJ" sheetId="35" state="hidden" r:id="rId16"/>
+    <sheet name="ETPT_TROX_corresp-GREFFE-TPROX" sheetId="36" state="hidden" r:id="rId17"/>
+    <sheet name="ETPT_CPH_corresp-GREFFE-CPH" sheetId="37" state="hidden" r:id="rId18"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ETPT A-JUST'!$A$2:$DN$2</definedName>

</xml_diff>

<commit_message>
maj mise en forme onglet agregat ddg
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26444862-8F27-8C4D-A082-DAFA947950F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F68F44F-B77B-2C4A-9B96-14988F96AD57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1584" uniqueCount="431">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1584" uniqueCount="432">
   <si>
     <t>#! END_ROW</t>
   </si>
@@ -4762,6 +4762,9 @@
   </si>
   <si>
     <t>Fonction agrégat</t>
+  </si>
+  <si>
+    <t>#! DUMP_COLS subtitles1</t>
   </si>
 </sst>
 </file>
@@ -20133,7 +20136,7 @@
       <c r="E1" s="7"/>
       <c r="F1" s="6"/>
       <c r="G1" s="6" t="s">
-        <v>6</v>
+        <v>431</v>
       </c>
       <c r="FA1" s="320" t="s">
         <v>232</v>

</xml_diff>

<commit_message>
size of column extractor resize
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F68F44F-B77B-2C4A-9B96-14988F96AD57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1CFD4B4-6148-7D41-8052-F1C174D564C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" activeTab="2" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -5949,7 +5949,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="359">
+  <cellXfs count="360">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -7148,6 +7148,9 @@
     <xf numFmtId="0" fontId="53" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -20169,6 +20172,9 @@
       <c r="B3" t="s">
         <v>10</v>
       </c>
+      <c r="N3" s="359"/>
+      <c r="O3" s="359"/>
+      <c r="P3" s="359"/>
     </row>
     <row r="4" spans="1:161" x14ac:dyDescent="0.2">
       <c r="B4" s="27" t="s">

</xml_diff>

<commit_message>
update nomenclature for extractor add jirs param
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B904EEE-7121-DA47-B624-F62FF37BCC9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89872010-548C-AA4A-A687-CB1FFA214E05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" activeTab="2" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -7129,7 +7129,27 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
     <cellStyle name="Normal 3" xfId="4" xr:uid="{6BD57324-3FD5-D341-A299-730D14794802}"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="18">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -7289,16 +7309,6 @@
       <font>
         <color theme="0"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -20146,8 +20156,8 @@
   </sheetData>
   <autoFilter ref="A2:DT2" xr:uid="{3B89445B-6ECC-4440-B85C-E593AE209933}"/>
   <conditionalFormatting sqref="A1:G1 I1:EY1 A2:EZ2 A3:FB1048576">
-    <cfRule type="expression" dxfId="16" priority="1">
-      <formula>AND(OR($P1&lt;&gt;"-",$Q1&lt;&gt;0,$R1&lt;&gt;0),ROW()&gt;2,$A1&lt;&gt;"")</formula>
+    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+      <formula>AND(OR($Q1&lt;&gt;"-",$R1&lt;&gt;0,$S1&lt;&gt;0),ROW()&gt;2,$A1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -20337,7 +20347,10 @@
         <v>387</v>
       </c>
       <c r="G6" s="19" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FB,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FB:$FB,"M-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction agrégat",'ETPT Format DDG'!2:2,0)),"M-TIT",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="H6" s="294" t="str">
@@ -20345,31 +20358,32 @@
         <v/>
       </c>
       <c r="I6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FB,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FB:$FB,"M-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction agrégat",'ETPT Format DDG'!2:2,0)),"M-PLAC-ADD",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="J6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FB,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FB:$FB,"M-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction agrégat",'ETPT Format DDG'!2:2,0)),"M-PLAC-SUB",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="K6" s="18" t="e">
         <f>SUMIFS(
-INDEX('ETPT Format DDG'!$A:$FB,
-,
-IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
-),'ETPT Format DDG'!$FB:$FB,"C",
-'ETPT Format DDG'!$C:$C,$A$3,
-'ETPT Format DDG'!$G:$G,"Magistrat")</f>
+INDEX('ETPT Format DDG'!$A:$ZZ,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction agrégat",'ETPT Format DDG'!2:2,0)),"C",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$A$3,
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Catégorie",'ETPT Format DDG'!2:2,0)),"Magistrat")</f>
         <v>#N/A</v>
       </c>
       <c r="L6" s="19" t="e">
         <f>ROUND(SUMIFS(
-INDEX('ETPT Format DDG'!$A:$FB,
-,
-IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
-),
-'ETPT Format DDG'!$C:$C,$A$3,
-'ETPT Format DDG'!$G:$G,"Magistrat"),3)</f>
+INDEX('ETPT Format DDG'!$A:$ZZ,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$A$3,
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Catégorie",'ETPT Format DDG'!2:2,0)),"Magistrat"),3)</f>
         <v>#N/A</v>
       </c>
       <c r="M6" s="295" t="str">
@@ -20377,7 +20391,10 @@
         <v/>
       </c>
       <c r="N6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FB,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FB:$FB,"F-TIT",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(
+INDEX('ETPT Format DDG'!$A:$ZZ,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction agrégat",'ETPT Format DDG'!2:2,0)),"F-TIT",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="O6" s="294" t="str">
@@ -20385,25 +20402,32 @@
         <v/>
       </c>
       <c r="P6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FB,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FB:$FB,"F-PLAC-ADD",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(
+INDEX('ETPT Format DDG'!$A:$FB,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction agrégat",'ETPT Format DDG'!2:2,0)),"F-PLAC-ADD",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="Q6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FB,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FB:$FB,"F-PLAC-SUB",'ETPT Format DDG'!$C:$C,$A$3)</f>
+        <f>SUMIFS(
+INDEX('ETPT Format DDG'!$A:$FB,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction agrégat",'ETPT Format DDG'!2:2,0)),"F-PLAC-SUB",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="R6" s="18" t="e">
-        <f>SUMIFS(INDEX('ETPT Format DDG'!$A:$FB,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),'ETPT Format DDG'!$FB:$FB,"C",'ETPT Format DDG'!$C:$C,$A$3,'ETPT Format DDG'!$G:$G,"Greffe")</f>
+        <f>SUMIFS(
+INDEX('ETPT Format DDG'!$A:$FB,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction agrégat",'ETPT Format DDG'!2:2,0)),"C",
+'ETPT Format DDG'!$G:$G,"Greffe",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$A$3)</f>
         <v>#N/A</v>
       </c>
       <c r="S6" s="19" t="e">
         <f>ROUND(SUMIFS(
-INDEX('ETPT Format DDG'!$A:$FB,
-,
-IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
-),
-'ETPT Format DDG'!$C:$C,$A$3,
-'ETPT Format DDG'!$G:$G,"Greffe"),3)</f>
+INDEX('ETPT Format DDG'!$A:$FB,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Catégorie",'ETPT Format DDG'!2:2,0)),"Greffe",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$A$3),3)</f>
         <v>#N/A</v>
       </c>
       <c r="T6" s="294" t="str">
@@ -20412,12 +20436,10 @@
       </c>
       <c r="U6" s="19" t="e">
         <f>ROUND(SUMIFS(
-INDEX('ETPT Format DDG'!$A:$FB,
-,
-IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))
-),'ETPT Format DDG'!$FB:$FB,"C",
-'ETPT Format DDG'!$C:$C,$A$3,
-'ETPT Format DDG'!$G:$G,"Autour du magistrat"),3)</f>
+INDEX('ETPT Format DDG'!$A:$FB,,IFERROR(MATCH(E6,'ETPT Format DDG'!$2:$2,0),MATCH(C6,'ETPT Format DDG'!$2:$2,0))),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction agrégat",'ETPT Format DDG'!2:2,0)),"C",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$A$3,
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Catégorie",'ETPT Format DDG'!2:2,0)),"Autour du magistrat"),3)</f>
         <v>#N/A</v>
       </c>
       <c r="V6" s="295" t="str">
@@ -20456,70 +20478,70 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="15" priority="16">
+    <cfRule type="expression" dxfId="17" priority="16">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="14" priority="18">
+    <cfRule type="expression" dxfId="16" priority="18">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="13" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="15" priority="1" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3)+_xlfn.NUMBERVALUE($U4)+_xlfn.NUMBERVALUE($U5)+_xlfn.NUMBERVALUE($U6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="2" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3)+_xlfn.NUMBERVALUE($S4)+_xlfn.NUMBERVALUE($S5)+_xlfn.NUMBERVALUE($S6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="7" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="12" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="12" stopIfTrue="1">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",OR(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0,_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0,_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="6" stopIfTrue="1">
       <formula>OR(_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6),_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6),_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="8" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="11" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)+_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="15">
+    <cfRule type="expression" dxfId="9" priority="15">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="6" priority="5">
+    <cfRule type="expression" dxfId="8" priority="5">
       <formula>_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="5" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="10" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3)+_xlfn.NUMBERVALUE($S4)+_xlfn.NUMBERVALUE($S5)+_xlfn.NUMBERVALUE($S6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="14">
+    <cfRule type="expression" dxfId="6" priority="14">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="5" priority="4">
       <formula>_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="2" priority="9">
+    <cfRule type="expression" dxfId="4" priority="9">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3)+_xlfn.NUMBERVALUE($U4)+_xlfn.NUMBERVALUE($U5)+_xlfn.NUMBERVALUE($U6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="13">
+    <cfRule type="expression" dxfId="3" priority="13">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6)</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
create Extractor CA VF
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C3A6E75-74D1-5945-8006-EE38F7EEDD36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3CA5426-8F3A-E749-BA9A-8EB3AEE04FDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -9690,6 +9690,21 @@
     <xf numFmtId="0" fontId="23" fillId="19" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="38" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -9808,23 +9823,8 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="49" fontId="30" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="53" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -10877,11 +10877,11 @@
       <c r="B1" s="115" t="s">
         <v>227</v>
       </c>
-      <c r="C1" s="334" t="s">
+      <c r="C1" s="339" t="s">
         <v>228</v>
       </c>
-      <c r="D1" s="334"/>
-      <c r="E1" s="334"/>
+      <c r="D1" s="339"/>
+      <c r="E1" s="339"/>
       <c r="F1" s="116"/>
       <c r="H1" s="26" t="s">
         <v>0</v>
@@ -10890,11 +10890,11 @@
     <row r="2" spans="1:8" s="120" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="117"/>
       <c r="B2" s="118"/>
-      <c r="C2" s="335" t="s">
+      <c r="C2" s="340" t="s">
         <v>229</v>
       </c>
-      <c r="D2" s="335"/>
-      <c r="E2" s="335"/>
+      <c r="D2" s="340"/>
+      <c r="E2" s="340"/>
       <c r="F2" s="119"/>
       <c r="H2" s="26" t="s">
         <v>0</v>
@@ -10918,10 +10918,10 @@
       <c r="D4" s="125" t="s">
         <v>232</v>
       </c>
-      <c r="E4" s="341" t="s">
+      <c r="E4" s="346" t="s">
         <v>233</v>
       </c>
-      <c r="F4" s="342"/>
+      <c r="F4" s="347"/>
       <c r="G4" s="134"/>
       <c r="H4" s="26" t="s">
         <v>0</v>
@@ -10938,10 +10938,10 @@
       <c r="D5" s="131" t="s">
         <v>236</v>
       </c>
-      <c r="E5" s="343" t="s">
+      <c r="E5" s="348" t="s">
         <v>249</v>
       </c>
-      <c r="F5" s="344"/>
+      <c r="F5" s="349"/>
       <c r="G5" s="133"/>
       <c r="H5" s="26" t="s">
         <v>0</v>
@@ -10958,10 +10958,10 @@
       <c r="D6" s="132" t="s">
         <v>239</v>
       </c>
-      <c r="E6" s="345" t="s">
+      <c r="E6" s="350" t="s">
         <v>250</v>
       </c>
-      <c r="F6" s="346"/>
+      <c r="F6" s="351"/>
       <c r="G6" s="133"/>
       <c r="H6" s="26" t="s">
         <v>0</v>
@@ -10978,10 +10978,10 @@
       <c r="D7" s="132" t="s">
         <v>242</v>
       </c>
-      <c r="E7" s="345" t="s">
+      <c r="E7" s="350" t="s">
         <v>249</v>
       </c>
-      <c r="F7" s="346"/>
+      <c r="F7" s="351"/>
       <c r="G7" s="133"/>
       <c r="H7" s="26" t="s">
         <v>0</v>
@@ -10992,16 +10992,16 @@
       <c r="B8" s="141" t="s">
         <v>243</v>
       </c>
-      <c r="C8" s="336" t="s">
+      <c r="C8" s="341" t="s">
         <v>244</v>
       </c>
-      <c r="D8" s="336" t="s">
+      <c r="D8" s="341" t="s">
         <v>245</v>
       </c>
-      <c r="E8" s="347" t="s">
+      <c r="E8" s="352" t="s">
         <v>251</v>
       </c>
-      <c r="F8" s="348"/>
+      <c r="F8" s="353"/>
       <c r="G8" s="133"/>
       <c r="H8" s="26" t="s">
         <v>0</v>
@@ -11012,10 +11012,10 @@
       <c r="B9" s="142" t="s">
         <v>246</v>
       </c>
-      <c r="C9" s="336"/>
-      <c r="D9" s="336"/>
-      <c r="E9" s="349"/>
-      <c r="F9" s="350"/>
+      <c r="C9" s="341"/>
+      <c r="D9" s="341"/>
+      <c r="E9" s="354"/>
+      <c r="F9" s="355"/>
       <c r="G9" s="133"/>
       <c r="H9" s="26" t="s">
         <v>0</v>
@@ -11026,10 +11026,10 @@
       <c r="B10" s="143" t="s">
         <v>247</v>
       </c>
-      <c r="C10" s="337"/>
-      <c r="D10" s="337"/>
-      <c r="E10" s="351"/>
-      <c r="F10" s="352"/>
+      <c r="C10" s="342"/>
+      <c r="D10" s="342"/>
+      <c r="E10" s="356"/>
+      <c r="F10" s="357"/>
       <c r="G10" s="133"/>
       <c r="H10" s="26" t="s">
         <v>0</v>
@@ -11049,11 +11049,11 @@
     <row r="12" spans="1:8" s="26" customFormat="1" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="121"/>
       <c r="B12" s="135"/>
-      <c r="C12" s="340" t="s">
+      <c r="C12" s="345" t="s">
         <v>248</v>
       </c>
-      <c r="D12" s="340"/>
-      <c r="E12" s="340"/>
+      <c r="D12" s="345"/>
+      <c r="E12" s="345"/>
       <c r="F12" s="136"/>
       <c r="H12" s="26" t="s">
         <v>0</v>
@@ -11067,14 +11067,14 @@
       </c>
     </row>
     <row r="14" spans="1:8" s="26" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="338" t="s">
+      <c r="A14" s="343" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="338"/>
-      <c r="C14" s="338"/>
-      <c r="D14" s="338"/>
-      <c r="E14" s="338"/>
-      <c r="F14" s="339"/>
+      <c r="B14" s="343"/>
+      <c r="C14" s="343"/>
+      <c r="D14" s="343"/>
+      <c r="E14" s="343"/>
+      <c r="F14" s="344"/>
       <c r="H14" s="26" t="s">
         <v>0</v>
       </c>
@@ -11202,7 +11202,7 @@
       <c r="G2" s="75" t="s">
         <v>172</v>
       </c>
-      <c r="H2" s="359" t="s">
+      <c r="H2" s="364" t="s">
         <v>171</v>
       </c>
       <c r="I2" s="74" t="s">
@@ -11247,7 +11247,7 @@
       <c r="V2" s="74" t="s">
         <v>170</v>
       </c>
-      <c r="W2" s="359" t="s">
+      <c r="W2" s="364" t="s">
         <v>169</v>
       </c>
       <c r="X2" s="73" t="s">
@@ -11277,7 +11277,7 @@
       <c r="AF2" s="73" t="s">
         <v>167</v>
       </c>
-      <c r="AG2" s="359" t="s">
+      <c r="AG2" s="364" t="s">
         <v>166</v>
       </c>
       <c r="AH2" s="73" t="s">
@@ -11319,7 +11319,7 @@
       <c r="AT2" s="73" t="s">
         <v>165</v>
       </c>
-      <c r="AU2" s="359" t="s">
+      <c r="AU2" s="364" t="s">
         <v>164</v>
       </c>
       <c r="AV2" s="72" t="s">
@@ -11349,7 +11349,7 @@
       <c r="BD2" s="72" t="s">
         <v>163</v>
       </c>
-      <c r="BE2" s="359" t="s">
+      <c r="BE2" s="364" t="s">
         <v>162</v>
       </c>
       <c r="BF2"/>
@@ -11364,7 +11364,7 @@
       <c r="G3" s="75" t="s">
         <v>161</v>
       </c>
-      <c r="H3" s="359"/>
+      <c r="H3" s="364"/>
       <c r="I3" s="74" t="s">
         <v>160</v>
       </c>
@@ -11405,7 +11405,7 @@
       <c r="V3" s="74" t="s">
         <v>148</v>
       </c>
-      <c r="W3" s="359"/>
+      <c r="W3" s="364"/>
       <c r="X3" s="73" t="s">
         <v>144</v>
       </c>
@@ -11433,7 +11433,7 @@
       <c r="AF3" s="73" t="s">
         <v>138</v>
       </c>
-      <c r="AG3" s="359"/>
+      <c r="AG3" s="364"/>
       <c r="AH3" s="73" t="s">
         <v>137</v>
       </c>
@@ -11473,7 +11473,7 @@
       <c r="AT3" s="73" t="s">
         <v>125</v>
       </c>
-      <c r="AU3" s="359"/>
+      <c r="AU3" s="364"/>
       <c r="AV3" s="72" t="s">
         <v>124</v>
       </c>
@@ -11501,7 +11501,7 @@
       <c r="BD3" s="72" t="s">
         <v>116</v>
       </c>
-      <c r="BE3" s="359"/>
+      <c r="BE3" s="364"/>
     </row>
     <row r="4" spans="1:58" s="41" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="77"/>
@@ -11523,7 +11523,7 @@
       <c r="G4" s="75" t="s">
         <v>111</v>
       </c>
-      <c r="H4" s="359"/>
+      <c r="H4" s="364"/>
       <c r="I4" s="74" t="s">
         <v>110</v>
       </c>
@@ -11566,7 +11566,7 @@
       <c r="V4" s="74" t="s">
         <v>97</v>
       </c>
-      <c r="W4" s="359"/>
+      <c r="W4" s="364"/>
       <c r="X4" s="73" t="s">
         <v>92</v>
       </c>
@@ -11594,7 +11594,7 @@
       <c r="AF4" s="73" t="s">
         <v>85</v>
       </c>
-      <c r="AG4" s="359"/>
+      <c r="AG4" s="364"/>
       <c r="AH4" s="73" t="s">
         <v>84</v>
       </c>
@@ -11634,7 +11634,7 @@
       <c r="AT4" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="AU4" s="359"/>
+      <c r="AU4" s="364"/>
       <c r="AV4" s="72" t="s">
         <v>71</v>
       </c>
@@ -11662,7 +11662,7 @@
       <c r="BD4" s="72" t="s">
         <v>63</v>
       </c>
-      <c r="BE4" s="359"/>
+      <c r="BE4" s="364"/>
       <c r="BF4"/>
     </row>
     <row r="5" spans="1:58" s="41" customFormat="1" ht="15" x14ac:dyDescent="0.2">
@@ -14161,7 +14161,7 @@
       <c r="G2" s="75" t="s">
         <v>172</v>
       </c>
-      <c r="H2" s="359" t="s">
+      <c r="H2" s="364" t="s">
         <v>171</v>
       </c>
       <c r="I2" s="75" t="s">
@@ -14194,7 +14194,7 @@
       <c r="R2" s="75" t="s">
         <v>170</v>
       </c>
-      <c r="S2" s="359" t="s">
+      <c r="S2" s="364" t="s">
         <v>169</v>
       </c>
       <c r="T2" s="75" t="s">
@@ -14224,7 +14224,7 @@
       <c r="AB2" s="75" t="s">
         <v>167</v>
       </c>
-      <c r="AC2" s="359" t="s">
+      <c r="AC2" s="364" t="s">
         <v>216</v>
       </c>
       <c r="AD2" s="75" t="s">
@@ -14236,7 +14236,7 @@
       <c r="AF2" s="75" t="s">
         <v>215</v>
       </c>
-      <c r="AG2" s="359" t="s">
+      <c r="AG2" s="364" t="s">
         <v>214</v>
       </c>
     </row>
@@ -14247,7 +14247,7 @@
       <c r="G3" s="75" t="s">
         <v>161</v>
       </c>
-      <c r="H3" s="359"/>
+      <c r="H3" s="364"/>
       <c r="I3" s="75" t="s">
         <v>213</v>
       </c>
@@ -14278,7 +14278,7 @@
       <c r="R3" s="75" t="s">
         <v>148</v>
       </c>
-      <c r="S3" s="359"/>
+      <c r="S3" s="364"/>
       <c r="T3" s="75" t="s">
         <v>204</v>
       </c>
@@ -14306,7 +14306,7 @@
       <c r="AB3" s="75" t="s">
         <v>196</v>
       </c>
-      <c r="AC3" s="359"/>
+      <c r="AC3" s="364"/>
       <c r="AD3" s="75" t="s">
         <v>195</v>
       </c>
@@ -14316,7 +14316,7 @@
       <c r="AF3" s="75" t="s">
         <v>125</v>
       </c>
-      <c r="AG3" s="359"/>
+      <c r="AG3" s="364"/>
     </row>
     <row r="4" spans="1:60" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="78"/>
@@ -14338,7 +14338,7 @@
       <c r="G4" s="75" t="s">
         <v>111</v>
       </c>
-      <c r="H4" s="359"/>
+      <c r="H4" s="364"/>
       <c r="I4" s="75" t="s">
         <v>194</v>
       </c>
@@ -14369,7 +14369,7 @@
       <c r="R4" s="75" t="s">
         <v>97</v>
       </c>
-      <c r="S4" s="359"/>
+      <c r="S4" s="364"/>
       <c r="T4" s="75" t="s">
         <v>185</v>
       </c>
@@ -14397,7 +14397,7 @@
       <c r="AB4" s="75" t="s">
         <v>177</v>
       </c>
-      <c r="AC4" s="359"/>
+      <c r="AC4" s="364"/>
       <c r="AD4" s="75" t="s">
         <v>176</v>
       </c>
@@ -14407,7 +14407,7 @@
       <c r="AF4" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="AG4" s="359"/>
+      <c r="AG4" s="364"/>
     </row>
     <row r="5" spans="1:60" x14ac:dyDescent="0.2">
       <c r="A5" s="81" t="s">
@@ -16057,13 +16057,13 @@
       <c r="G2" s="75" t="s">
         <v>170</v>
       </c>
-      <c r="H2" s="359" t="s">
+      <c r="H2" s="364" t="s">
         <v>169</v>
       </c>
       <c r="I2" s="75" t="s">
         <v>38</v>
       </c>
-      <c r="J2" s="359" t="s">
+      <c r="J2" s="364" t="s">
         <v>168</v>
       </c>
     </row>
@@ -16071,11 +16071,11 @@
       <c r="G3" s="75" t="s">
         <v>148</v>
       </c>
-      <c r="H3" s="359"/>
+      <c r="H3" s="364"/>
       <c r="I3" s="75" t="s">
         <v>145</v>
       </c>
-      <c r="J3" s="359"/>
+      <c r="J3" s="364"/>
     </row>
     <row r="4" spans="1:62" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="97"/>
@@ -16097,11 +16097,11 @@
       <c r="G4" s="75" t="s">
         <v>97</v>
       </c>
-      <c r="H4" s="359"/>
+      <c r="H4" s="364"/>
       <c r="I4" s="75" t="s">
         <v>93</v>
       </c>
-      <c r="J4" s="359"/>
+      <c r="J4" s="364"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="91" t="s">
@@ -16570,7 +16570,7 @@
       <c r="P2" s="316" t="s">
         <v>38</v>
       </c>
-      <c r="Q2" s="362" t="s">
+      <c r="Q2" s="367" t="s">
         <v>434</v>
       </c>
     </row>
@@ -16611,7 +16611,7 @@
       <c r="P3" s="316" t="s">
         <v>441</v>
       </c>
-      <c r="Q3" s="362"/>
+      <c r="Q3" s="367"/>
     </row>
     <row r="4" spans="1:62" ht="70" x14ac:dyDescent="0.2">
       <c r="A4" s="317"/>
@@ -16660,7 +16660,7 @@
       <c r="P4" s="319" t="s">
         <v>452</v>
       </c>
-      <c r="Q4" s="362"/>
+      <c r="Q4" s="367"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="320" t="s">
@@ -17510,13 +17510,13 @@
   <sheetData>
     <row r="1" spans="1:61" s="151" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="150"/>
-      <c r="B1" s="364" t="s">
+      <c r="B1" s="369" t="s">
         <v>173</v>
       </c>
-      <c r="C1" s="364"/>
-      <c r="D1" s="364"/>
-      <c r="E1" s="364"/>
-      <c r="F1" s="364"/>
+      <c r="C1" s="369"/>
+      <c r="D1" s="369"/>
+      <c r="E1" s="369"/>
+      <c r="F1" s="369"/>
       <c r="G1" s="152"/>
       <c r="H1" s="152"/>
       <c r="I1" s="152"/>
@@ -17561,7 +17561,7 @@
       <c r="O2" s="154" t="s">
         <v>167</v>
       </c>
-      <c r="P2" s="363" t="s">
+      <c r="P2" s="368" t="s">
         <v>166</v>
       </c>
       <c r="Q2" s="154" t="s">
@@ -17603,7 +17603,7 @@
       <c r="AC2" s="154" t="s">
         <v>165</v>
       </c>
-      <c r="AD2" s="363" t="s">
+      <c r="AD2" s="368" t="s">
         <v>164</v>
       </c>
       <c r="AE2" s="155" t="s">
@@ -17633,7 +17633,7 @@
       <c r="AM2" s="155" t="s">
         <v>163</v>
       </c>
-      <c r="AN2" s="363" t="s">
+      <c r="AN2" s="368" t="s">
         <v>162</v>
       </c>
       <c r="AQ2" s="154"/>
@@ -17644,7 +17644,7 @@
       <c r="AV2" s="154"/>
       <c r="AW2" s="154"/>
       <c r="AX2" s="154"/>
-      <c r="AY2" s="363"/>
+      <c r="AY2" s="368"/>
       <c r="AZ2" s="155"/>
       <c r="BA2" s="155"/>
       <c r="BB2" s="155"/>
@@ -17654,7 +17654,7 @@
       <c r="BF2" s="155"/>
       <c r="BG2" s="155"/>
       <c r="BH2" s="155"/>
-      <c r="BI2" s="363"/>
+      <c r="BI2" s="368"/>
     </row>
     <row r="3" spans="1:61" s="151" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="153"/>
@@ -17690,7 +17690,7 @@
       <c r="O3" s="154" t="s">
         <v>138</v>
       </c>
-      <c r="P3" s="363"/>
+      <c r="P3" s="368"/>
       <c r="Q3" s="154" t="s">
         <v>137</v>
       </c>
@@ -17730,7 +17730,7 @@
       <c r="AC3" s="154" t="s">
         <v>125</v>
       </c>
-      <c r="AD3" s="363"/>
+      <c r="AD3" s="368"/>
       <c r="AE3" s="155" t="s">
         <v>124</v>
       </c>
@@ -17758,7 +17758,7 @@
       <c r="AM3" s="155" t="s">
         <v>116</v>
       </c>
-      <c r="AN3" s="363"/>
+      <c r="AN3" s="368"/>
       <c r="AQ3" s="154"/>
       <c r="AR3" s="154"/>
       <c r="AS3" s="154"/>
@@ -17767,7 +17767,7 @@
       <c r="AV3" s="154"/>
       <c r="AW3" s="154"/>
       <c r="AX3" s="154"/>
-      <c r="AY3" s="363"/>
+      <c r="AY3" s="368"/>
       <c r="AZ3" s="155"/>
       <c r="BA3" s="155"/>
       <c r="BB3" s="155"/>
@@ -17777,7 +17777,7 @@
       <c r="BF3" s="155"/>
       <c r="BG3" s="155"/>
       <c r="BH3" s="155"/>
-      <c r="BI3" s="363"/>
+      <c r="BI3" s="368"/>
     </row>
     <row r="4" spans="1:61" s="151" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="156"/>
@@ -17823,7 +17823,7 @@
       <c r="O4" s="154" t="s">
         <v>85</v>
       </c>
-      <c r="P4" s="363"/>
+      <c r="P4" s="368"/>
       <c r="Q4" s="154" t="s">
         <v>84</v>
       </c>
@@ -17863,7 +17863,7 @@
       <c r="AC4" s="154" t="s">
         <v>72</v>
       </c>
-      <c r="AD4" s="363"/>
+      <c r="AD4" s="368"/>
       <c r="AE4" s="155" t="s">
         <v>71</v>
       </c>
@@ -17891,7 +17891,7 @@
       <c r="AM4" s="155" t="s">
         <v>63</v>
       </c>
-      <c r="AN4" s="363"/>
+      <c r="AN4" s="368"/>
       <c r="AQ4" s="154"/>
       <c r="AR4" s="154"/>
       <c r="AS4" s="154"/>
@@ -17900,7 +17900,7 @@
       <c r="AV4" s="154"/>
       <c r="AW4" s="154"/>
       <c r="AX4" s="154"/>
-      <c r="AY4" s="363"/>
+      <c r="AY4" s="368"/>
       <c r="AZ4" s="155"/>
       <c r="BA4" s="155"/>
       <c r="BB4" s="155"/>
@@ -17910,7 +17910,7 @@
       <c r="BF4" s="155"/>
       <c r="BG4" s="155"/>
       <c r="BH4" s="155"/>
-      <c r="BI4" s="363"/>
+      <c r="BI4" s="368"/>
     </row>
     <row r="5" spans="1:61" s="151" customFormat="1" ht="144" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="158" t="s">
@@ -19632,14 +19632,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="365" t="s">
+      <c r="A1" s="370" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="365"/>
-      <c r="C1" s="365"/>
-      <c r="D1" s="365"/>
-      <c r="E1" s="365"/>
-      <c r="F1" s="365"/>
+      <c r="B1" s="370"/>
+      <c r="C1" s="370"/>
+      <c r="D1" s="370"/>
+      <c r="E1" s="370"/>
+      <c r="F1" s="370"/>
       <c r="G1" s="183"/>
       <c r="H1" s="183"/>
       <c r="I1" s="183"/>
@@ -19689,7 +19689,7 @@
       <c r="O2" s="186" t="s">
         <v>167</v>
       </c>
-      <c r="P2" s="366" t="s">
+      <c r="P2" s="371" t="s">
         <v>216</v>
       </c>
       <c r="Q2" s="186" t="s">
@@ -19701,7 +19701,7 @@
       <c r="S2" s="186" t="s">
         <v>215</v>
       </c>
-      <c r="T2" s="366" t="s">
+      <c r="T2" s="371" t="s">
         <v>214</v>
       </c>
     </row>
@@ -19739,7 +19739,7 @@
       <c r="O3" s="186" t="s">
         <v>196</v>
       </c>
-      <c r="P3" s="366"/>
+      <c r="P3" s="371"/>
       <c r="Q3" s="186" t="s">
         <v>195</v>
       </c>
@@ -19749,7 +19749,7 @@
       <c r="S3" s="186" t="s">
         <v>125</v>
       </c>
-      <c r="T3" s="366"/>
+      <c r="T3" s="371"/>
     </row>
     <row r="4" spans="1:20" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="185"/>
@@ -19795,7 +19795,7 @@
       <c r="O4" s="186" t="s">
         <v>177</v>
       </c>
-      <c r="P4" s="366"/>
+      <c r="P4" s="371"/>
       <c r="Q4" s="186" t="s">
         <v>176</v>
       </c>
@@ -19805,7 +19805,7 @@
       <c r="S4" s="186" t="s">
         <v>72</v>
       </c>
-      <c r="T4" s="366"/>
+      <c r="T4" s="371"/>
     </row>
     <row r="5" spans="1:20" ht="317" x14ac:dyDescent="0.2">
       <c r="A5" s="189" t="s">
@@ -20391,16 +20391,16 @@
   <sheetData>
     <row r="1" spans="1:28" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="209"/>
-      <c r="B1" s="368" t="s">
+      <c r="B1" s="373" t="s">
         <v>173</v>
       </c>
-      <c r="C1" s="368"/>
-      <c r="D1" s="368"/>
-      <c r="E1" s="368"/>
-      <c r="F1" s="368"/>
-      <c r="G1" s="368"/>
-      <c r="H1" s="368"/>
-      <c r="I1" s="368"/>
+      <c r="C1" s="373"/>
+      <c r="D1" s="373"/>
+      <c r="E1" s="373"/>
+      <c r="F1" s="373"/>
+      <c r="G1" s="373"/>
+      <c r="H1" s="373"/>
+      <c r="I1" s="373"/>
       <c r="J1" s="206"/>
       <c r="K1" s="206"/>
       <c r="L1" s="206"/>
@@ -20431,7 +20431,7 @@
       <c r="G2" s="208" t="s">
         <v>172</v>
       </c>
-      <c r="H2" s="367" t="s">
+      <c r="H2" s="372" t="s">
         <v>171</v>
       </c>
       <c r="I2" s="211" t="s">
@@ -20476,7 +20476,7 @@
       <c r="V2" s="211" t="s">
         <v>170</v>
       </c>
-      <c r="W2" s="367" t="s">
+      <c r="W2" s="372" t="s">
         <v>169</v>
       </c>
       <c r="X2" s="208" t="s">
@@ -20491,7 +20491,7 @@
       <c r="AA2" s="208" t="s">
         <v>38</v>
       </c>
-      <c r="AB2" s="367" t="s">
+      <c r="AB2" s="372" t="s">
         <v>168</v>
       </c>
     </row>
@@ -20505,7 +20505,7 @@
       <c r="G3" s="208" t="s">
         <v>161</v>
       </c>
-      <c r="H3" s="367"/>
+      <c r="H3" s="372"/>
       <c r="I3" s="211" t="s">
         <v>160</v>
       </c>
@@ -20546,7 +20546,7 @@
       <c r="V3" s="211" t="s">
         <v>148</v>
       </c>
-      <c r="W3" s="367"/>
+      <c r="W3" s="372"/>
       <c r="X3" s="210"/>
       <c r="Y3" s="208" t="s">
         <v>147</v>
@@ -20557,7 +20557,7 @@
       <c r="AA3" s="208" t="s">
         <v>145</v>
       </c>
-      <c r="AB3" s="367"/>
+      <c r="AB3" s="372"/>
     </row>
     <row r="4" spans="1:28" ht="98" x14ac:dyDescent="0.2">
       <c r="A4" s="212"/>
@@ -20579,7 +20579,7 @@
       <c r="G4" s="208" t="s">
         <v>111</v>
       </c>
-      <c r="H4" s="367"/>
+      <c r="H4" s="372"/>
       <c r="I4" s="211" t="s">
         <v>110</v>
       </c>
@@ -20622,7 +20622,7 @@
       <c r="V4" s="214" t="s">
         <v>97</v>
       </c>
-      <c r="W4" s="367"/>
+      <c r="W4" s="372"/>
       <c r="X4" s="215" t="s">
         <v>96</v>
       </c>
@@ -20635,7 +20635,7 @@
       <c r="AA4" s="215" t="s">
         <v>93</v>
       </c>
-      <c r="AB4" s="367"/>
+      <c r="AB4" s="372"/>
     </row>
     <row r="5" spans="1:28" ht="196" x14ac:dyDescent="0.2">
       <c r="A5" s="216" t="s">
@@ -21529,16 +21529,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="370" t="s">
+      <c r="A1" s="375" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="370"/>
-      <c r="C1" s="370"/>
-      <c r="D1" s="370"/>
-      <c r="E1" s="370"/>
-      <c r="F1" s="370"/>
-      <c r="G1" s="370"/>
-      <c r="H1" s="370"/>
+      <c r="B1" s="375"/>
+      <c r="C1" s="375"/>
+      <c r="D1" s="375"/>
+      <c r="E1" s="375"/>
+      <c r="F1" s="375"/>
+      <c r="G1" s="375"/>
+      <c r="H1" s="375"/>
       <c r="I1" s="256"/>
       <c r="J1" s="256"/>
       <c r="K1" s="256"/>
@@ -21563,7 +21563,7 @@
       <c r="G2" s="258" t="s">
         <v>172</v>
       </c>
-      <c r="H2" s="369" t="s">
+      <c r="H2" s="374" t="s">
         <v>171</v>
       </c>
       <c r="I2" s="258" t="s">
@@ -21596,13 +21596,13 @@
       <c r="R2" s="258" t="s">
         <v>170</v>
       </c>
-      <c r="S2" s="369" t="s">
+      <c r="S2" s="374" t="s">
         <v>169</v>
       </c>
       <c r="T2" s="258" t="s">
         <v>38</v>
       </c>
-      <c r="U2" s="369" t="s">
+      <c r="U2" s="374" t="s">
         <v>168</v>
       </c>
     </row>
@@ -21616,7 +21616,7 @@
       <c r="G3" s="258" t="s">
         <v>161</v>
       </c>
-      <c r="H3" s="369"/>
+      <c r="H3" s="374"/>
       <c r="I3" s="258" t="s">
         <v>213</v>
       </c>
@@ -21647,11 +21647,11 @@
       <c r="R3" s="258" t="s">
         <v>148</v>
       </c>
-      <c r="S3" s="369"/>
+      <c r="S3" s="374"/>
       <c r="T3" s="258" t="s">
         <v>145</v>
       </c>
-      <c r="U3" s="369"/>
+      <c r="U3" s="374"/>
     </row>
     <row r="4" spans="1:21" ht="112" x14ac:dyDescent="0.2">
       <c r="A4" s="255"/>
@@ -21673,7 +21673,7 @@
       <c r="G4" s="258" t="s">
         <v>111</v>
       </c>
-      <c r="H4" s="369"/>
+      <c r="H4" s="374"/>
       <c r="I4" s="258" t="s">
         <v>194</v>
       </c>
@@ -21704,11 +21704,11 @@
       <c r="R4" s="258" t="s">
         <v>97</v>
       </c>
-      <c r="S4" s="369"/>
+      <c r="S4" s="374"/>
       <c r="T4" s="258" t="s">
         <v>93</v>
       </c>
-      <c r="U4" s="369"/>
+      <c r="U4" s="374"/>
     </row>
     <row r="5" spans="1:21" ht="196" x14ac:dyDescent="0.2">
       <c r="A5" s="261" t="s">
@@ -22399,13 +22399,13 @@
       <c r="K2" s="186" t="s">
         <v>170</v>
       </c>
-      <c r="L2" s="366" t="s">
+      <c r="L2" s="371" t="s">
         <v>169</v>
       </c>
       <c r="M2" s="186" t="s">
         <v>38</v>
       </c>
-      <c r="N2" s="366" t="s">
+      <c r="N2" s="371" t="s">
         <v>168</v>
       </c>
     </row>
@@ -22423,11 +22423,11 @@
       <c r="K3" s="186" t="s">
         <v>148</v>
       </c>
-      <c r="L3" s="366"/>
+      <c r="L3" s="371"/>
       <c r="M3" s="186" t="s">
         <v>145</v>
       </c>
-      <c r="N3" s="366"/>
+      <c r="N3" s="371"/>
     </row>
     <row r="4" spans="1:14" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="239"/>
@@ -22453,11 +22453,11 @@
       <c r="K4" s="186" t="s">
         <v>97</v>
       </c>
-      <c r="L4" s="366"/>
+      <c r="L4" s="371"/>
       <c r="M4" s="186" t="s">
         <v>93</v>
       </c>
-      <c r="N4" s="366"/>
+      <c r="N4" s="371"/>
     </row>
     <row r="5" spans="1:14" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="241"/>
@@ -23121,25 +23121,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A1" s="371"/>
-      <c r="B1" s="372" t="s">
+      <c r="A1" s="334"/>
+      <c r="B1" s="376" t="s">
         <v>455</v>
       </c>
-      <c r="C1" s="372"/>
-      <c r="D1" s="372"/>
-      <c r="E1" s="372"/>
-      <c r="F1" s="373"/>
-      <c r="G1" s="371"/>
-      <c r="H1" s="371"/>
-      <c r="I1" s="371"/>
-      <c r="J1" s="371"/>
-      <c r="K1" s="371"/>
-      <c r="L1" s="371"/>
-      <c r="M1" s="371"/>
-      <c r="N1" s="371"/>
-      <c r="O1" s="371"/>
-      <c r="P1" s="371"/>
-      <c r="Q1" s="371"/>
+      <c r="C1" s="376"/>
+      <c r="D1" s="376"/>
+      <c r="E1" s="376"/>
+      <c r="F1" s="335"/>
+      <c r="G1" s="334"/>
+      <c r="H1" s="334"/>
+      <c r="I1" s="334"/>
+      <c r="J1" s="334"/>
+      <c r="K1" s="334"/>
+      <c r="L1" s="334"/>
+      <c r="M1" s="334"/>
+      <c r="N1" s="334"/>
+      <c r="O1" s="334"/>
+      <c r="P1" s="334"/>
+      <c r="Q1" s="334"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="313"/>
@@ -23178,7 +23178,7 @@
       <c r="P2" s="316" t="s">
         <v>38</v>
       </c>
-      <c r="Q2" s="362" t="s">
+      <c r="Q2" s="367" t="s">
         <v>434</v>
       </c>
     </row>
@@ -23219,9 +23219,9 @@
       <c r="P3" s="316" t="s">
         <v>441</v>
       </c>
-      <c r="Q3" s="362"/>
-    </row>
-    <row r="4" spans="1:17" ht="98" x14ac:dyDescent="0.2">
+      <c r="Q3" s="367"/>
+    </row>
+    <row r="4" spans="1:17" ht="70" x14ac:dyDescent="0.2">
       <c r="A4" s="317"/>
       <c r="B4" s="318" t="s">
         <v>115</v>
@@ -23268,9 +23268,9 @@
       <c r="P4" s="319" t="s">
         <v>452</v>
       </c>
-      <c r="Q4" s="362"/>
-    </row>
-    <row r="5" spans="1:17" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="Q4" s="367"/>
+    </row>
+    <row r="5" spans="1:17" ht="398" x14ac:dyDescent="0.2">
       <c r="A5" s="320" t="s">
         <v>453</v>
       </c>
@@ -23314,7 +23314,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" ht="266" x14ac:dyDescent="0.2">
       <c r="A6" s="320" t="s">
         <v>453</v>
       </c>
@@ -23358,7 +23358,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="252" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17" ht="224" x14ac:dyDescent="0.2">
       <c r="A7" s="320" t="s">
         <v>453</v>
       </c>
@@ -23404,7 +23404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="371" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" ht="345" x14ac:dyDescent="0.2">
       <c r="A8" s="320" t="s">
         <v>453</v>
       </c>
@@ -23450,7 +23450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="238" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" ht="210" x14ac:dyDescent="0.2">
       <c r="A9" s="320" t="s">
         <v>453</v>
       </c>
@@ -23496,7 +23496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="224" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" ht="196" x14ac:dyDescent="0.2">
       <c r="A10" s="320" t="s">
         <v>453</v>
       </c>
@@ -23542,7 +23542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="306" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" ht="280" x14ac:dyDescent="0.2">
       <c r="A11" s="320" t="s">
         <v>453</v>
       </c>
@@ -23588,7 +23588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="306" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" ht="280" x14ac:dyDescent="0.2">
       <c r="A12" s="320" t="s">
         <v>453</v>
       </c>
@@ -23635,11 +23635,11 @@
       </c>
     </row>
     <row r="13" spans="1:17" ht="28" x14ac:dyDescent="0.2">
-      <c r="A13" s="374"/>
-      <c r="B13" s="375"/>
-      <c r="C13" s="375"/>
-      <c r="D13" s="376"/>
-      <c r="E13" s="375"/>
+      <c r="A13" s="336"/>
+      <c r="B13" s="337"/>
+      <c r="C13" s="337"/>
+      <c r="D13" s="338"/>
+      <c r="E13" s="337"/>
       <c r="F13" s="328" t="s">
         <v>39</v>
       </c>
@@ -23859,28 +23859,28 @@
       <c r="D4" s="277"/>
       <c r="E4" s="277"/>
       <c r="F4" s="277"/>
-      <c r="G4" s="353" t="s">
+      <c r="G4" s="358" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="354"/>
-      <c r="I4" s="354"/>
-      <c r="J4" s="354"/>
-      <c r="K4" s="354"/>
-      <c r="L4" s="355"/>
-      <c r="M4" s="356"/>
-      <c r="N4" s="357" t="s">
+      <c r="H4" s="359"/>
+      <c r="I4" s="359"/>
+      <c r="J4" s="359"/>
+      <c r="K4" s="359"/>
+      <c r="L4" s="360"/>
+      <c r="M4" s="361"/>
+      <c r="N4" s="362" t="s">
         <v>27</v>
       </c>
-      <c r="O4" s="355"/>
-      <c r="P4" s="355"/>
-      <c r="Q4" s="355"/>
-      <c r="R4" s="355"/>
-      <c r="S4" s="355"/>
-      <c r="T4" s="358"/>
-      <c r="U4" s="353" t="s">
+      <c r="O4" s="360"/>
+      <c r="P4" s="360"/>
+      <c r="Q4" s="360"/>
+      <c r="R4" s="360"/>
+      <c r="S4" s="360"/>
+      <c r="T4" s="363"/>
+      <c r="U4" s="358" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="356"/>
+      <c r="V4" s="361"/>
       <c r="W4" s="284"/>
       <c r="X4" t="s">
         <v>0</v>
@@ -23965,7 +23965,7 @@
         <v>#N/A</v>
       </c>
       <c r="H6" s="281" t="str">
-        <f>IF(AND(OR(LEFT(C6,3)="12.",LEFT(E6,3)="12.",LEFT(E6,5)="CET &gt;",IFERROR(G6/$G$6,"")=0),NOT(AND(LEFT(E6,5)="12.31",IFERROR(G6/$G$6,"")&lt;&gt;0)),NOT(AND(LEFT(E6,5)="12.32",IFERROR(G6/$G$6,"")&lt;&gt;0))),"", IFERROR(G6/$G$6,""))</f>
+        <f>IF(AND(OR(LEFT(C6,3)="12.",LEFT(E6,3)="12.",LEFT(E6,5)="CET &gt;",IFERROR(G6/$G$6,"")=0),NOT(AND(LEFT(E6,4)="12.8",IFERROR(G6/$G$6,"")&lt;&gt;0)),NOT(AND(LEFT(E6,5)="12.31",IFERROR(G6/$G$6,"")&lt;&gt;0)),NOT(AND(LEFT(E6,5)="12.32",IFERROR(G6/$G$6,"")&lt;&gt;0))),"", IFERROR(G6/$G$6,""))</f>
         <v/>
       </c>
       <c r="I6" s="18" t="e">
@@ -23998,7 +23998,7 @@
         <v>#N/A</v>
       </c>
       <c r="M6" s="282" t="str">
-        <f>IF(AND(OR(LEFT(C6,3)="12.",LEFT(E6,3)="12.",LEFT(E6,5)="CET &gt;", IFERROR(L6/$L$6,"")=0),NOT(AND(LEFT(E6,5)="12.31",IFERROR(L6/$G$6,"")&lt;&gt;0)),NOT(AND(LEFT(E6,5)="12.32",IFERROR(L6/$G$6,"")&lt;&gt;0))),"", IFERROR(L6/$L$6,""))</f>
+        <f>IF(AND(OR(LEFT(C6,3)="12.",LEFT(E6,3)="12.",LEFT(E6,5)="CET &gt;", IFERROR(L6/$L$6,"")=0),NOT(AND(LEFT(E6,4)="12.8",IFERROR(G6/$G$6,"")&lt;&gt;0)),NOT(AND(LEFT(E6,5)="12.31",IFERROR(L6/$G$6,"")&lt;&gt;0)),NOT(AND(LEFT(E6,5)="12.32",IFERROR(L6/$G$6,"")&lt;&gt;0))),"", IFERROR(L6/$L$6,""))</f>
         <v/>
       </c>
       <c r="N6" s="18" t="e">
@@ -24009,7 +24009,7 @@
         <v>#N/A</v>
       </c>
       <c r="O6" s="281" t="str">
-        <f>IF(AND(OR(LEFT(C6,3)="12.",LEFT(E6,3)="12.",LEFT(E6,5)="CET &gt;",IFERROR(N6/$N$6,"")=0),NOT(AND(LEFT(E6,5)="12.31",IFERROR(N6/$G$6,"")&lt;&gt;0)),NOT(AND(LEFT(E6,5)="12.32",IFERROR(N6/$G$6,"")&lt;&gt;0))),"",IFERROR(N6/$N$6,""))</f>
+        <f>IF(AND(OR(LEFT(C6,3)="12.",LEFT(E6,3)="12.",LEFT(E6,5)="CET &gt;",IFERROR(N6/$N$6,"")=0),NOT(AND(LEFT(E6,4)="12.8",IFERROR(G6/$G$6,"")&lt;&gt;0)),NOT(AND(LEFT(E6,5)="12.31",IFERROR(N6/$G$6,"")&lt;&gt;0)),NOT(AND(LEFT(E6,5)="12.32",IFERROR(N6/$G$6,"")&lt;&gt;0))),"",IFERROR(N6/$N$6,""))</f>
         <v/>
       </c>
       <c r="P6" s="18" t="e">
@@ -24042,7 +24042,7 @@
         <v>#N/A</v>
       </c>
       <c r="T6" s="281" t="str">
-        <f>IF(AND(OR(LEFT(C6,3)="12.",LEFT(E6,3)="12.",LEFT(E6,5)="CET &gt;",IFERROR(S6/$S$6,"")=0),NOT(AND(LEFT(E6,5)="12.31",IFERROR(S6/$G$6,"")&lt;&gt;0)),NOT(AND(LEFT(E6,5)="12.32",IFERROR(S6/$G$6,"")&lt;&gt;0))),"", IFERROR(S6/$S$6,""))</f>
+        <f>IF(AND(OR(LEFT(C6,3)="12.",LEFT(E6,3)="12.",LEFT(E6,5)="CET &gt;",IFERROR(S6/$S$6,"")=0),NOT(AND(LEFT(E6,4)="12.8",IFERROR(G6/$G$6,"")&lt;&gt;0)),NOT(AND(LEFT(E6,5)="12.31",IFERROR(S6/$G$6,"")&lt;&gt;0)),NOT(AND(LEFT(E6,5)="12.32",IFERROR(S6/$G$6,"")&lt;&gt;0))),"", IFERROR(S6/$S$6,""))</f>
         <v/>
       </c>
       <c r="U6" s="19" t="e">
@@ -24054,7 +24054,7 @@
         <v>#N/A</v>
       </c>
       <c r="V6" s="282" t="str">
-        <f>IF(AND(OR(LEFT(C6,3)="12.",LEFT(E6,3)="12.",LEFT(E6,5)="CET &gt;",IFERROR(U6/$U$6,"")=0),NOT(AND(LEFT(E6,5)="12.31",IFERROR(U6/$G$6,"")&lt;&gt;0)),NOT(AND(LEFT(E6,5)="12.32",IFERROR(U6/$G$6,"")&lt;&gt;0))),"", IFERROR(U6/$U$6,""))</f>
+        <f>IF(AND(OR(LEFT(C6,3)="12.",LEFT(E6,3)="12.",LEFT(E6,5)="CET &gt;",IFERROR(U6/$U$6,"")=0),NOT(AND(LEFT(E6,4)="12.8",IFERROR(G6/$G$6,"")&lt;&gt;0)),NOT(AND(LEFT(E6,5)="12.31",IFERROR(U6/$G$6,"")&lt;&gt;0)),NOT(AND(LEFT(E6,5)="12.32",IFERROR(U6/$G$6,"")&lt;&gt;0))),"", IFERROR(U6/$U$6,""))</f>
         <v/>
       </c>
       <c r="W6" t="s">
@@ -24295,16 +24295,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:57" s="41" customFormat="1" ht="23.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B1" s="360" t="s">
+      <c r="B1" s="365" t="s">
         <v>173</v>
       </c>
-      <c r="C1" s="360"/>
-      <c r="D1" s="360"/>
-      <c r="E1" s="360"/>
-      <c r="F1" s="360"/>
-      <c r="G1" s="360"/>
-      <c r="H1" s="360"/>
-      <c r="I1" s="360"/>
+      <c r="C1" s="365"/>
+      <c r="D1" s="365"/>
+      <c r="E1" s="365"/>
+      <c r="F1" s="365"/>
+      <c r="G1" s="365"/>
+      <c r="H1" s="365"/>
+      <c r="I1" s="365"/>
     </row>
     <row r="2" spans="1:57" s="41" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="78"/>
@@ -24316,7 +24316,7 @@
       <c r="G2" s="75" t="s">
         <v>172</v>
       </c>
-      <c r="H2" s="359" t="s">
+      <c r="H2" s="364" t="s">
         <v>171</v>
       </c>
       <c r="I2" s="74" t="s">
@@ -24361,7 +24361,7 @@
       <c r="V2" s="74" t="s">
         <v>170</v>
       </c>
-      <c r="W2" s="359" t="s">
+      <c r="W2" s="364" t="s">
         <v>169</v>
       </c>
       <c r="X2" s="73" t="s">
@@ -24391,7 +24391,7 @@
       <c r="AF2" s="73" t="s">
         <v>167</v>
       </c>
-      <c r="AG2" s="359" t="s">
+      <c r="AG2" s="364" t="s">
         <v>166</v>
       </c>
       <c r="AH2" s="73" t="s">
@@ -24433,7 +24433,7 @@
       <c r="AT2" s="73" t="s">
         <v>165</v>
       </c>
-      <c r="AU2" s="359" t="s">
+      <c r="AU2" s="364" t="s">
         <v>164</v>
       </c>
       <c r="AV2" s="72" t="s">
@@ -24463,7 +24463,7 @@
       <c r="BD2" s="72" t="s">
         <v>163</v>
       </c>
-      <c r="BE2" s="359" t="s">
+      <c r="BE2" s="364" t="s">
         <v>162</v>
       </c>
     </row>
@@ -24477,7 +24477,7 @@
       <c r="G3" s="75" t="s">
         <v>161</v>
       </c>
-      <c r="H3" s="359"/>
+      <c r="H3" s="364"/>
       <c r="I3" s="74" t="s">
         <v>160</v>
       </c>
@@ -24518,7 +24518,7 @@
       <c r="V3" s="74" t="s">
         <v>148</v>
       </c>
-      <c r="W3" s="359"/>
+      <c r="W3" s="364"/>
       <c r="X3" s="73" t="s">
         <v>144</v>
       </c>
@@ -24546,7 +24546,7 @@
       <c r="AF3" s="73" t="s">
         <v>138</v>
       </c>
-      <c r="AG3" s="359"/>
+      <c r="AG3" s="364"/>
       <c r="AH3" s="73" t="s">
         <v>137</v>
       </c>
@@ -24586,7 +24586,7 @@
       <c r="AT3" s="73" t="s">
         <v>125</v>
       </c>
-      <c r="AU3" s="359"/>
+      <c r="AU3" s="364"/>
       <c r="AV3" s="72" t="s">
         <v>124</v>
       </c>
@@ -24614,7 +24614,7 @@
       <c r="BD3" s="72" t="s">
         <v>116</v>
       </c>
-      <c r="BE3" s="359"/>
+      <c r="BE3" s="364"/>
     </row>
     <row r="4" spans="1:57" s="41" customFormat="1" ht="60" x14ac:dyDescent="0.15">
       <c r="A4" s="77"/>
@@ -24636,7 +24636,7 @@
       <c r="G4" s="75" t="s">
         <v>111</v>
       </c>
-      <c r="H4" s="359"/>
+      <c r="H4" s="364"/>
       <c r="I4" s="74" t="s">
         <v>110</v>
       </c>
@@ -24679,7 +24679,7 @@
       <c r="V4" s="74" t="s">
         <v>97</v>
       </c>
-      <c r="W4" s="359"/>
+      <c r="W4" s="364"/>
       <c r="X4" s="73" t="s">
         <v>92</v>
       </c>
@@ -24707,7 +24707,7 @@
       <c r="AF4" s="73" t="s">
         <v>85</v>
       </c>
-      <c r="AG4" s="359"/>
+      <c r="AG4" s="364"/>
       <c r="AH4" s="73" t="s">
         <v>84</v>
       </c>
@@ -24747,7 +24747,7 @@
       <c r="AT4" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="AU4" s="359"/>
+      <c r="AU4" s="364"/>
       <c r="AV4" s="72" t="s">
         <v>71</v>
       </c>
@@ -24775,7 +24775,7 @@
       <c r="BD4" s="72" t="s">
         <v>63</v>
       </c>
-      <c r="BE4" s="359"/>
+      <c r="BE4" s="364"/>
     </row>
     <row r="5" spans="1:57" s="41" customFormat="1" ht="11" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="51" t="s">
@@ -27634,16 +27634,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" x14ac:dyDescent="0.2">
-      <c r="A1" s="361" t="s">
+      <c r="A1" s="366" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="361"/>
-      <c r="C1" s="361"/>
-      <c r="D1" s="361"/>
-      <c r="E1" s="361"/>
-      <c r="F1" s="361"/>
-      <c r="G1" s="361"/>
-      <c r="H1" s="361"/>
+      <c r="B1" s="366"/>
+      <c r="C1" s="366"/>
+      <c r="D1" s="366"/>
+      <c r="E1" s="366"/>
+      <c r="F1" s="366"/>
+      <c r="G1" s="366"/>
+      <c r="H1" s="366"/>
       <c r="I1" s="41"/>
       <c r="J1" s="41"/>
       <c r="K1" s="41"/>
@@ -27680,7 +27680,7 @@
       <c r="G2" s="75" t="s">
         <v>172</v>
       </c>
-      <c r="H2" s="359" t="s">
+      <c r="H2" s="364" t="s">
         <v>171</v>
       </c>
       <c r="I2" s="75" t="s">
@@ -27713,7 +27713,7 @@
       <c r="R2" s="75" t="s">
         <v>170</v>
       </c>
-      <c r="S2" s="359" t="s">
+      <c r="S2" s="364" t="s">
         <v>169</v>
       </c>
       <c r="T2" s="75" t="s">
@@ -27743,7 +27743,7 @@
       <c r="AB2" s="75" t="s">
         <v>167</v>
       </c>
-      <c r="AC2" s="359" t="s">
+      <c r="AC2" s="364" t="s">
         <v>216</v>
       </c>
       <c r="AD2" s="75" t="s">
@@ -27755,7 +27755,7 @@
       <c r="AF2" s="75" t="s">
         <v>215</v>
       </c>
-      <c r="AG2" s="359" t="s">
+      <c r="AG2" s="364" t="s">
         <v>214</v>
       </c>
     </row>
@@ -27769,7 +27769,7 @@
       <c r="G3" s="75" t="s">
         <v>161</v>
       </c>
-      <c r="H3" s="359"/>
+      <c r="H3" s="364"/>
       <c r="I3" s="75" t="s">
         <v>213</v>
       </c>
@@ -27800,7 +27800,7 @@
       <c r="R3" s="75" t="s">
         <v>148</v>
       </c>
-      <c r="S3" s="359"/>
+      <c r="S3" s="364"/>
       <c r="T3" s="75" t="s">
         <v>204</v>
       </c>
@@ -27828,7 +27828,7 @@
       <c r="AB3" s="75" t="s">
         <v>196</v>
       </c>
-      <c r="AC3" s="359"/>
+      <c r="AC3" s="364"/>
       <c r="AD3" s="75" t="s">
         <v>195</v>
       </c>
@@ -27838,7 +27838,7 @@
       <c r="AF3" s="75" t="s">
         <v>125</v>
       </c>
-      <c r="AG3" s="359"/>
+      <c r="AG3" s="364"/>
     </row>
     <row r="4" spans="1:33" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="78"/>
@@ -27860,7 +27860,7 @@
       <c r="G4" s="75" t="s">
         <v>111</v>
       </c>
-      <c r="H4" s="359"/>
+      <c r="H4" s="364"/>
       <c r="I4" s="75" t="s">
         <v>194</v>
       </c>
@@ -27891,7 +27891,7 @@
       <c r="R4" s="75" t="s">
         <v>97</v>
       </c>
-      <c r="S4" s="359"/>
+      <c r="S4" s="364"/>
       <c r="T4" s="75" t="s">
         <v>185</v>
       </c>
@@ -27919,7 +27919,7 @@
       <c r="AB4" s="75" t="s">
         <v>177</v>
       </c>
-      <c r="AC4" s="359"/>
+      <c r="AC4" s="364"/>
       <c r="AD4" s="75" t="s">
         <v>176</v>
       </c>
@@ -27929,7 +27929,7 @@
       <c r="AF4" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="AG4" s="359"/>
+      <c r="AG4" s="364"/>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A5" s="81" t="s">
@@ -29299,13 +29299,13 @@
       <c r="G2" s="75" t="s">
         <v>170</v>
       </c>
-      <c r="H2" s="359" t="s">
+      <c r="H2" s="364" t="s">
         <v>169</v>
       </c>
       <c r="I2" s="75" t="s">
         <v>38</v>
       </c>
-      <c r="J2" s="359" t="s">
+      <c r="J2" s="364" t="s">
         <v>168</v>
       </c>
     </row>
@@ -29319,11 +29319,11 @@
       <c r="G3" s="75" t="s">
         <v>148</v>
       </c>
-      <c r="H3" s="359"/>
+      <c r="H3" s="364"/>
       <c r="I3" s="75" t="s">
         <v>145</v>
       </c>
-      <c r="J3" s="359"/>
+      <c r="J3" s="364"/>
     </row>
     <row r="4" spans="1:10" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="97"/>
@@ -29345,11 +29345,11 @@
       <c r="G4" s="75" t="s">
         <v>97</v>
       </c>
-      <c r="H4" s="359"/>
+      <c r="H4" s="364"/>
       <c r="I4" s="75" t="s">
         <v>93</v>
       </c>
-      <c r="J4" s="359"/>
+      <c r="J4" s="364"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="91" t="s">
@@ -29770,7 +29770,7 @@
       <c r="P2" s="316" t="s">
         <v>38</v>
       </c>
-      <c r="Q2" s="362" t="s">
+      <c r="Q2" s="367" t="s">
         <v>434</v>
       </c>
     </row>
@@ -29811,7 +29811,7 @@
       <c r="P3" s="316" t="s">
         <v>441</v>
       </c>
-      <c r="Q3" s="362"/>
+      <c r="Q3" s="367"/>
     </row>
     <row r="4" spans="1:62" ht="70" x14ac:dyDescent="0.2">
       <c r="A4" s="317"/>
@@ -29860,7 +29860,7 @@
       <c r="P4" s="319" t="s">
         <v>452</v>
       </c>
-      <c r="Q4" s="362"/>
+      <c r="Q4" s="367"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="320" t="s">

</xml_diff>

<commit_message>
extractor lines switch tj
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71A4DF08-A0BA-A74B-A3A3-DB14EF00192D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D885D31A-70B3-374B-89AB-98BEDBE8ACC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -15817,6 +15817,50 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="81" fillId="0" borderId="0" xfId="4" applyFont="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="28" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="40" fontId="37" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="81" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="83" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="29" fillId="8" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="24" fillId="8" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="84" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="23" fillId="10" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="67" fillId="28" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="169" fontId="48" fillId="28" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="81" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="39" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -15974,50 +16018,6 @@
     </xf>
     <xf numFmtId="49" fontId="31" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="81" fillId="0" borderId="0" xfId="4" applyFont="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="28" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="40" fontId="37" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="81" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="81" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="81" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="83" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="81" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="29" fillId="8" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="8" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="84" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="23" fillId="10" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="67" fillId="28" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="48" fillId="28" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="81" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -17080,11 +17080,11 @@
       <c r="B1" s="115" t="s">
         <v>223</v>
       </c>
-      <c r="C1" s="347" t="s">
+      <c r="C1" s="363" t="s">
         <v>224</v>
       </c>
-      <c r="D1" s="347"/>
-      <c r="E1" s="347"/>
+      <c r="D1" s="363"/>
+      <c r="E1" s="363"/>
       <c r="F1" s="116"/>
       <c r="H1" s="26" t="s">
         <v>0</v>
@@ -17093,11 +17093,11 @@
     <row r="2" spans="1:8" s="120" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="117"/>
       <c r="B2" s="118"/>
-      <c r="C2" s="348" t="s">
+      <c r="C2" s="364" t="s">
         <v>225</v>
       </c>
-      <c r="D2" s="348"/>
-      <c r="E2" s="348"/>
+      <c r="D2" s="364"/>
+      <c r="E2" s="364"/>
       <c r="F2" s="119"/>
       <c r="H2" s="26" t="s">
         <v>0</v>
@@ -17121,10 +17121,10 @@
       <c r="D4" s="125" t="s">
         <v>228</v>
       </c>
-      <c r="E4" s="352" t="s">
+      <c r="E4" s="368" t="s">
         <v>229</v>
       </c>
-      <c r="F4" s="353"/>
+      <c r="F4" s="369"/>
       <c r="G4" s="134"/>
       <c r="H4" s="26" t="s">
         <v>0</v>
@@ -17141,10 +17141,10 @@
       <c r="D5" s="131" t="s">
         <v>232</v>
       </c>
-      <c r="E5" s="354" t="s">
+      <c r="E5" s="370" t="s">
         <v>245</v>
       </c>
-      <c r="F5" s="355"/>
+      <c r="F5" s="371"/>
       <c r="G5" s="133"/>
       <c r="H5" s="26" t="s">
         <v>0</v>
@@ -17161,10 +17161,10 @@
       <c r="D6" s="132" t="s">
         <v>235</v>
       </c>
-      <c r="E6" s="356" t="s">
+      <c r="E6" s="372" t="s">
         <v>246</v>
       </c>
-      <c r="F6" s="357"/>
+      <c r="F6" s="373"/>
       <c r="G6" s="133"/>
       <c r="H6" s="26" t="s">
         <v>0</v>
@@ -17181,10 +17181,10 @@
       <c r="D7" s="132" t="s">
         <v>238</v>
       </c>
-      <c r="E7" s="356" t="s">
+      <c r="E7" s="372" t="s">
         <v>245</v>
       </c>
-      <c r="F7" s="357"/>
+      <c r="F7" s="373"/>
       <c r="G7" s="133"/>
       <c r="H7" s="26" t="s">
         <v>0</v>
@@ -17195,16 +17195,16 @@
       <c r="B8" s="138" t="s">
         <v>239</v>
       </c>
-      <c r="C8" s="358" t="s">
+      <c r="C8" s="374" t="s">
         <v>240</v>
       </c>
-      <c r="D8" s="358" t="s">
+      <c r="D8" s="374" t="s">
         <v>241</v>
       </c>
-      <c r="E8" s="361" t="s">
+      <c r="E8" s="377" t="s">
         <v>247</v>
       </c>
-      <c r="F8" s="361"/>
+      <c r="F8" s="377"/>
       <c r="G8" s="133"/>
       <c r="H8" s="26" t="s">
         <v>0</v>
@@ -17215,10 +17215,10 @@
       <c r="B9" s="304" t="s">
         <v>242</v>
       </c>
-      <c r="C9" s="359"/>
-      <c r="D9" s="359"/>
-      <c r="E9" s="362"/>
-      <c r="F9" s="362"/>
+      <c r="C9" s="375"/>
+      <c r="D9" s="375"/>
+      <c r="E9" s="378"/>
+      <c r="F9" s="378"/>
       <c r="G9" s="133"/>
       <c r="H9" s="26" t="s">
         <v>0</v>
@@ -17229,10 +17229,10 @@
       <c r="B10" s="305" t="s">
         <v>243</v>
       </c>
-      <c r="C10" s="359"/>
-      <c r="D10" s="359"/>
-      <c r="E10" s="362"/>
-      <c r="F10" s="362"/>
+      <c r="C10" s="375"/>
+      <c r="D10" s="375"/>
+      <c r="E10" s="378"/>
+      <c r="F10" s="378"/>
       <c r="G10" s="133"/>
       <c r="H10" s="26" t="s">
         <v>0</v>
@@ -17243,10 +17243,10 @@
       <c r="B11" s="300" t="s">
         <v>367</v>
       </c>
-      <c r="C11" s="360"/>
-      <c r="D11" s="360"/>
-      <c r="E11" s="363"/>
-      <c r="F11" s="363"/>
+      <c r="C11" s="376"/>
+      <c r="D11" s="376"/>
+      <c r="E11" s="379"/>
+      <c r="F11" s="379"/>
       <c r="G11" s="133"/>
       <c r="H11" s="26" t="s">
         <v>0</v>
@@ -17266,11 +17266,11 @@
     <row r="13" spans="1:8" s="26" customFormat="1" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="121"/>
       <c r="B13" s="302"/>
-      <c r="C13" s="351" t="s">
+      <c r="C13" s="367" t="s">
         <v>244</v>
       </c>
-      <c r="D13" s="351"/>
-      <c r="E13" s="351"/>
+      <c r="D13" s="367"/>
+      <c r="E13" s="367"/>
       <c r="F13" s="303"/>
       <c r="H13" s="26" t="s">
         <v>0</v>
@@ -17284,14 +17284,14 @@
       </c>
     </row>
     <row r="15" spans="1:8" s="26" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="349" t="s">
+      <c r="A15" s="365" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="349"/>
-      <c r="C15" s="349"/>
-      <c r="D15" s="349"/>
-      <c r="E15" s="349"/>
-      <c r="F15" s="350"/>
+      <c r="B15" s="365"/>
+      <c r="C15" s="365"/>
+      <c r="D15" s="365"/>
+      <c r="E15" s="365"/>
+      <c r="F15" s="366"/>
       <c r="H15" s="26" t="s">
         <v>0</v>
       </c>
@@ -17415,13 +17415,13 @@
       <c r="A2" s="78"/>
       <c r="B2" s="78"/>
       <c r="C2" s="78"/>
-      <c r="D2" s="395"/>
-      <c r="E2" s="395"/>
-      <c r="F2" s="395"/>
+      <c r="D2" s="347"/>
+      <c r="E2" s="347"/>
+      <c r="F2" s="347"/>
       <c r="G2" s="75" t="s">
         <v>169</v>
       </c>
-      <c r="H2" s="373" t="s">
+      <c r="H2" s="389" t="s">
         <v>168</v>
       </c>
       <c r="I2" s="74" t="s">
@@ -17466,7 +17466,7 @@
       <c r="V2" s="74" t="s">
         <v>167</v>
       </c>
-      <c r="W2" s="373" t="s">
+      <c r="W2" s="389" t="s">
         <v>166</v>
       </c>
       <c r="X2" s="73" t="s">
@@ -17496,7 +17496,7 @@
       <c r="AF2" s="73" t="s">
         <v>164</v>
       </c>
-      <c r="AG2" s="373" t="s">
+      <c r="AG2" s="389" t="s">
         <v>163</v>
       </c>
       <c r="AH2" s="73" t="s">
@@ -17538,7 +17538,7 @@
       <c r="AT2" s="73" t="s">
         <v>162</v>
       </c>
-      <c r="AU2" s="373" t="s">
+      <c r="AU2" s="389" t="s">
         <v>161</v>
       </c>
       <c r="AV2" s="72" t="s">
@@ -17568,7 +17568,7 @@
       <c r="BD2" s="72" t="s">
         <v>160</v>
       </c>
-      <c r="BE2" s="373" t="s">
+      <c r="BE2" s="389" t="s">
         <v>159</v>
       </c>
       <c r="BF2"/>
@@ -17583,7 +17583,7 @@
       <c r="G3" s="75" t="s">
         <v>158</v>
       </c>
-      <c r="H3" s="373"/>
+      <c r="H3" s="389"/>
       <c r="I3" s="74" t="s">
         <v>157</v>
       </c>
@@ -17624,7 +17624,7 @@
       <c r="V3" s="74" t="s">
         <v>145</v>
       </c>
-      <c r="W3" s="373"/>
+      <c r="W3" s="389"/>
       <c r="X3" s="73" t="s">
         <v>141</v>
       </c>
@@ -17652,7 +17652,7 @@
       <c r="AF3" s="73" t="s">
         <v>135</v>
       </c>
-      <c r="AG3" s="373"/>
+      <c r="AG3" s="389"/>
       <c r="AH3" s="73" t="s">
         <v>134</v>
       </c>
@@ -17692,7 +17692,7 @@
       <c r="AT3" s="73" t="s">
         <v>122</v>
       </c>
-      <c r="AU3" s="373"/>
+      <c r="AU3" s="389"/>
       <c r="AV3" s="72" t="s">
         <v>121</v>
       </c>
@@ -17720,7 +17720,7 @@
       <c r="BD3" s="72" t="s">
         <v>113</v>
       </c>
-      <c r="BE3" s="373"/>
+      <c r="BE3" s="389"/>
     </row>
     <row r="4" spans="1:58" s="41" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="77"/>
@@ -17742,7 +17742,7 @@
       <c r="G4" s="75" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="373"/>
+      <c r="H4" s="389"/>
       <c r="I4" s="74" t="s">
         <v>107</v>
       </c>
@@ -17785,7 +17785,7 @@
       <c r="V4" s="74" t="s">
         <v>94</v>
       </c>
-      <c r="W4" s="373"/>
+      <c r="W4" s="389"/>
       <c r="X4" s="73" t="s">
         <v>92</v>
       </c>
@@ -17813,7 +17813,7 @@
       <c r="AF4" s="73" t="s">
         <v>85</v>
       </c>
-      <c r="AG4" s="373"/>
+      <c r="AG4" s="389"/>
       <c r="AH4" s="73" t="s">
         <v>611</v>
       </c>
@@ -17853,7 +17853,7 @@
       <c r="AT4" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="AU4" s="373"/>
+      <c r="AU4" s="389"/>
       <c r="AV4" s="72" t="s">
         <v>71</v>
       </c>
@@ -17881,7 +17881,7 @@
       <c r="BD4" s="72" t="s">
         <v>63</v>
       </c>
-      <c r="BE4" s="373"/>
+      <c r="BE4" s="389"/>
       <c r="BF4"/>
     </row>
     <row r="5" spans="1:58" s="41" customFormat="1" ht="15" x14ac:dyDescent="0.2">
@@ -20231,273 +20231,273 @@
       </c>
     </row>
     <row r="17" spans="4:57" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D17" s="395"/>
-      <c r="E17" s="395"/>
-      <c r="F17" s="395"/>
-      <c r="G17" s="395"/>
-      <c r="H17" s="395"/>
-      <c r="I17" s="395"/>
-      <c r="J17" s="395"/>
-      <c r="K17" s="395"/>
-      <c r="L17" s="395"/>
-      <c r="M17" s="395"/>
-      <c r="N17" s="395"/>
-      <c r="O17" s="395"/>
-      <c r="P17" s="395"/>
-      <c r="Q17" s="395"/>
-      <c r="R17" s="395"/>
-      <c r="S17" s="395"/>
-      <c r="T17" s="395"/>
-      <c r="U17" s="395"/>
-      <c r="V17" s="395"/>
-      <c r="W17" s="396"/>
-      <c r="X17" s="395"/>
-      <c r="Y17" s="395"/>
-      <c r="Z17" s="395"/>
-      <c r="AA17" s="395"/>
-      <c r="AB17" s="395"/>
-      <c r="AC17" s="395"/>
-      <c r="AD17" s="395"/>
-      <c r="AE17" s="395"/>
-      <c r="AF17" s="395"/>
-      <c r="AG17" s="395"/>
-      <c r="AH17" s="395"/>
-      <c r="AI17" s="395"/>
-      <c r="AJ17" s="395"/>
-      <c r="AK17" s="395"/>
-      <c r="AL17" s="395"/>
-      <c r="AM17" s="395"/>
-      <c r="AN17" s="395"/>
-      <c r="AO17" s="395"/>
-      <c r="AP17" s="395"/>
-      <c r="AQ17" s="395"/>
-      <c r="AR17" s="395"/>
-      <c r="AS17" s="395"/>
-      <c r="AT17" s="395"/>
-      <c r="AU17" s="396"/>
-      <c r="AV17" s="395"/>
-      <c r="AW17" s="395"/>
-      <c r="AX17" s="395"/>
-      <c r="AY17" s="395"/>
-      <c r="AZ17" s="395"/>
-      <c r="BA17" s="395"/>
-      <c r="BB17" s="395"/>
-      <c r="BC17" s="395"/>
-      <c r="BD17" s="395"/>
-      <c r="BE17" s="395"/>
+      <c r="D17" s="347"/>
+      <c r="E17" s="347"/>
+      <c r="F17" s="347"/>
+      <c r="G17" s="347"/>
+      <c r="H17" s="347"/>
+      <c r="I17" s="347"/>
+      <c r="J17" s="347"/>
+      <c r="K17" s="347"/>
+      <c r="L17" s="347"/>
+      <c r="M17" s="347"/>
+      <c r="N17" s="347"/>
+      <c r="O17" s="347"/>
+      <c r="P17" s="347"/>
+      <c r="Q17" s="347"/>
+      <c r="R17" s="347"/>
+      <c r="S17" s="347"/>
+      <c r="T17" s="347"/>
+      <c r="U17" s="347"/>
+      <c r="V17" s="347"/>
+      <c r="W17" s="348"/>
+      <c r="X17" s="347"/>
+      <c r="Y17" s="347"/>
+      <c r="Z17" s="347"/>
+      <c r="AA17" s="347"/>
+      <c r="AB17" s="347"/>
+      <c r="AC17" s="347"/>
+      <c r="AD17" s="347"/>
+      <c r="AE17" s="347"/>
+      <c r="AF17" s="347"/>
+      <c r="AG17" s="347"/>
+      <c r="AH17" s="347"/>
+      <c r="AI17" s="347"/>
+      <c r="AJ17" s="347"/>
+      <c r="AK17" s="347"/>
+      <c r="AL17" s="347"/>
+      <c r="AM17" s="347"/>
+      <c r="AN17" s="347"/>
+      <c r="AO17" s="347"/>
+      <c r="AP17" s="347"/>
+      <c r="AQ17" s="347"/>
+      <c r="AR17" s="347"/>
+      <c r="AS17" s="347"/>
+      <c r="AT17" s="347"/>
+      <c r="AU17" s="348"/>
+      <c r="AV17" s="347"/>
+      <c r="AW17" s="347"/>
+      <c r="AX17" s="347"/>
+      <c r="AY17" s="347"/>
+      <c r="AZ17" s="347"/>
+      <c r="BA17" s="347"/>
+      <c r="BB17" s="347"/>
+      <c r="BC17" s="347"/>
+      <c r="BD17" s="347"/>
+      <c r="BE17" s="347"/>
     </row>
     <row r="18" spans="4:57" hidden="1" x14ac:dyDescent="0.2">
-      <c r="D18" s="395"/>
-      <c r="E18" s="395"/>
-      <c r="F18" s="395"/>
-      <c r="G18" s="395"/>
-      <c r="H18" s="395"/>
-      <c r="I18" s="395"/>
-      <c r="J18" s="395"/>
-      <c r="K18" s="395"/>
-      <c r="L18" s="395"/>
-      <c r="M18" s="395"/>
-      <c r="N18" s="395"/>
-      <c r="O18" s="395"/>
-      <c r="P18" s="395"/>
-      <c r="Q18" s="395"/>
-      <c r="R18" s="395"/>
-      <c r="S18" s="395"/>
-      <c r="T18" s="395"/>
-      <c r="U18" s="395"/>
-      <c r="V18" s="395"/>
-      <c r="W18" s="397"/>
-      <c r="X18" s="395"/>
-      <c r="Y18" s="395"/>
-      <c r="Z18" s="395"/>
-      <c r="AA18" s="395"/>
-      <c r="AB18" s="395"/>
-      <c r="AC18" s="395"/>
-      <c r="AD18" s="395"/>
-      <c r="AE18" s="395"/>
-      <c r="AF18" s="395"/>
-      <c r="AG18" s="395"/>
-      <c r="AH18" s="395"/>
-      <c r="AI18" s="395"/>
-      <c r="AJ18" s="395"/>
-      <c r="AK18" s="395"/>
-      <c r="AL18" s="395"/>
-      <c r="AM18" s="395"/>
-      <c r="AN18" s="395"/>
-      <c r="AO18" s="395"/>
-      <c r="AP18" s="395"/>
-      <c r="AQ18" s="395"/>
-      <c r="AR18" s="395"/>
-      <c r="AS18" s="395"/>
-      <c r="AT18" s="395"/>
-      <c r="AU18" s="397">
+      <c r="D18" s="347"/>
+      <c r="E18" s="347"/>
+      <c r="F18" s="347"/>
+      <c r="G18" s="347"/>
+      <c r="H18" s="347"/>
+      <c r="I18" s="347"/>
+      <c r="J18" s="347"/>
+      <c r="K18" s="347"/>
+      <c r="L18" s="347"/>
+      <c r="M18" s="347"/>
+      <c r="N18" s="347"/>
+      <c r="O18" s="347"/>
+      <c r="P18" s="347"/>
+      <c r="Q18" s="347"/>
+      <c r="R18" s="347"/>
+      <c r="S18" s="347"/>
+      <c r="T18" s="347"/>
+      <c r="U18" s="347"/>
+      <c r="V18" s="347"/>
+      <c r="W18" s="349"/>
+      <c r="X18" s="347"/>
+      <c r="Y18" s="347"/>
+      <c r="Z18" s="347"/>
+      <c r="AA18" s="347"/>
+      <c r="AB18" s="347"/>
+      <c r="AC18" s="347"/>
+      <c r="AD18" s="347"/>
+      <c r="AE18" s="347"/>
+      <c r="AF18" s="347"/>
+      <c r="AG18" s="347"/>
+      <c r="AH18" s="347"/>
+      <c r="AI18" s="347"/>
+      <c r="AJ18" s="347"/>
+      <c r="AK18" s="347"/>
+      <c r="AL18" s="347"/>
+      <c r="AM18" s="347"/>
+      <c r="AN18" s="347"/>
+      <c r="AO18" s="347"/>
+      <c r="AP18" s="347"/>
+      <c r="AQ18" s="347"/>
+      <c r="AR18" s="347"/>
+      <c r="AS18" s="347"/>
+      <c r="AT18" s="347"/>
+      <c r="AU18" s="349">
         <f>AU16+AG16-AU14-AG14-AU13-AU12-AG13-AG12</f>
         <v>0</v>
       </c>
-      <c r="AV18" s="395"/>
-      <c r="AW18" s="395"/>
-      <c r="AX18" s="395"/>
-      <c r="AY18" s="395"/>
-      <c r="AZ18" s="395"/>
-      <c r="BA18" s="395"/>
-      <c r="BB18" s="395"/>
-      <c r="BC18" s="395"/>
-      <c r="BD18" s="395"/>
-      <c r="BE18" s="395"/>
+      <c r="AV18" s="347"/>
+      <c r="AW18" s="347"/>
+      <c r="AX18" s="347"/>
+      <c r="AY18" s="347"/>
+      <c r="AZ18" s="347"/>
+      <c r="BA18" s="347"/>
+      <c r="BB18" s="347"/>
+      <c r="BC18" s="347"/>
+      <c r="BD18" s="347"/>
+      <c r="BE18" s="347"/>
     </row>
     <row r="19" spans="4:57" x14ac:dyDescent="0.2">
-      <c r="D19" s="395"/>
-      <c r="E19" s="395"/>
-      <c r="F19" s="395"/>
-      <c r="G19" s="395"/>
-      <c r="H19" s="395"/>
-      <c r="I19" s="395"/>
-      <c r="J19" s="395"/>
-      <c r="K19" s="395"/>
-      <c r="L19" s="395"/>
-      <c r="M19" s="395"/>
-      <c r="N19" s="395"/>
-      <c r="O19" s="395"/>
-      <c r="P19" s="395"/>
-      <c r="Q19" s="395"/>
-      <c r="R19" s="395"/>
-      <c r="S19" s="395"/>
-      <c r="T19" s="395"/>
-      <c r="U19" s="395"/>
-      <c r="V19" s="395"/>
-      <c r="W19" s="395"/>
-      <c r="X19" s="395"/>
-      <c r="Y19" s="395"/>
-      <c r="Z19" s="395"/>
-      <c r="AA19" s="395"/>
-      <c r="AB19" s="395"/>
-      <c r="AC19" s="395"/>
-      <c r="AD19" s="395"/>
-      <c r="AE19" s="395"/>
-      <c r="AF19" s="395"/>
-      <c r="AG19" s="395"/>
-      <c r="AH19" s="395"/>
-      <c r="AI19" s="395"/>
-      <c r="AJ19" s="395"/>
-      <c r="AK19" s="395"/>
-      <c r="AL19" s="395"/>
-      <c r="AM19" s="395"/>
-      <c r="AN19" s="395"/>
-      <c r="AO19" s="395"/>
-      <c r="AP19" s="395"/>
-      <c r="AQ19" s="395"/>
-      <c r="AR19" s="395"/>
-      <c r="AS19" s="395"/>
-      <c r="AT19" s="395"/>
-      <c r="AU19" s="395"/>
-      <c r="AV19" s="395"/>
-      <c r="AW19" s="395"/>
-      <c r="AX19" s="395"/>
-      <c r="AY19" s="395"/>
-      <c r="AZ19" s="395"/>
-      <c r="BA19" s="395"/>
-      <c r="BB19" s="395"/>
-      <c r="BC19" s="395"/>
-      <c r="BD19" s="395"/>
-      <c r="BE19" s="395"/>
+      <c r="D19" s="347"/>
+      <c r="E19" s="347"/>
+      <c r="F19" s="347"/>
+      <c r="G19" s="347"/>
+      <c r="H19" s="347"/>
+      <c r="I19" s="347"/>
+      <c r="J19" s="347"/>
+      <c r="K19" s="347"/>
+      <c r="L19" s="347"/>
+      <c r="M19" s="347"/>
+      <c r="N19" s="347"/>
+      <c r="O19" s="347"/>
+      <c r="P19" s="347"/>
+      <c r="Q19" s="347"/>
+      <c r="R19" s="347"/>
+      <c r="S19" s="347"/>
+      <c r="T19" s="347"/>
+      <c r="U19" s="347"/>
+      <c r="V19" s="347"/>
+      <c r="W19" s="347"/>
+      <c r="X19" s="347"/>
+      <c r="Y19" s="347"/>
+      <c r="Z19" s="347"/>
+      <c r="AA19" s="347"/>
+      <c r="AB19" s="347"/>
+      <c r="AC19" s="347"/>
+      <c r="AD19" s="347"/>
+      <c r="AE19" s="347"/>
+      <c r="AF19" s="347"/>
+      <c r="AG19" s="347"/>
+      <c r="AH19" s="347"/>
+      <c r="AI19" s="347"/>
+      <c r="AJ19" s="347"/>
+      <c r="AK19" s="347"/>
+      <c r="AL19" s="347"/>
+      <c r="AM19" s="347"/>
+      <c r="AN19" s="347"/>
+      <c r="AO19" s="347"/>
+      <c r="AP19" s="347"/>
+      <c r="AQ19" s="347"/>
+      <c r="AR19" s="347"/>
+      <c r="AS19" s="347"/>
+      <c r="AT19" s="347"/>
+      <c r="AU19" s="347"/>
+      <c r="AV19" s="347"/>
+      <c r="AW19" s="347"/>
+      <c r="AX19" s="347"/>
+      <c r="AY19" s="347"/>
+      <c r="AZ19" s="347"/>
+      <c r="BA19" s="347"/>
+      <c r="BB19" s="347"/>
+      <c r="BC19" s="347"/>
+      <c r="BD19" s="347"/>
+      <c r="BE19" s="347"/>
     </row>
     <row r="20" spans="4:57" ht="24" x14ac:dyDescent="0.2">
-      <c r="D20" s="395"/>
-      <c r="E20" s="395"/>
-      <c r="F20" s="398" t="s">
+      <c r="D20" s="347"/>
+      <c r="E20" s="347"/>
+      <c r="F20" s="350" t="s">
         <v>253</v>
       </c>
       <c r="G20" s="152" t="str">
         <f>IF(ISBLANK(ETPT_TJ_DDG!$D$5),"",IF(ISERROR(ETPT_TJ!G20),"",IF(ETPT_TJ!G20=0,"",ETPT_TJ!G20)))</f>
         <v/>
       </c>
-      <c r="H20" s="395"/>
-      <c r="I20" s="395"/>
-      <c r="J20" s="395"/>
-      <c r="K20" s="395"/>
-      <c r="L20" s="395"/>
-      <c r="M20" s="395"/>
-      <c r="N20" s="395"/>
-      <c r="O20" s="395"/>
-      <c r="P20" s="395"/>
-      <c r="Q20" s="395"/>
-      <c r="R20" s="395"/>
-      <c r="S20" s="395"/>
-      <c r="T20" s="395"/>
-      <c r="U20" s="399" t="s">
+      <c r="H20" s="347"/>
+      <c r="I20" s="347"/>
+      <c r="J20" s="347"/>
+      <c r="K20" s="347"/>
+      <c r="L20" s="347"/>
+      <c r="M20" s="347"/>
+      <c r="N20" s="347"/>
+      <c r="O20" s="347"/>
+      <c r="P20" s="347"/>
+      <c r="Q20" s="347"/>
+      <c r="R20" s="347"/>
+      <c r="S20" s="347"/>
+      <c r="T20" s="347"/>
+      <c r="U20" s="351" t="s">
         <v>254</v>
       </c>
       <c r="V20" s="152" t="str">
         <f>IF(ISBLANK(ETPT_TJ_DDG!$D$5),"",IF(ISERROR(ETPT_TJ!V20),"",IF(ETPT_TJ!V20=0,"",ETPT_TJ!V20)))</f>
         <v/>
       </c>
-      <c r="W20" s="395"/>
-      <c r="X20" s="395"/>
-      <c r="Y20" s="395"/>
-      <c r="Z20" s="395"/>
-      <c r="AA20" s="395"/>
-      <c r="AB20" s="395"/>
-      <c r="AC20" s="400"/>
-      <c r="AD20" s="395"/>
-      <c r="AE20" s="395"/>
-      <c r="AF20" s="395"/>
-      <c r="AG20" s="395"/>
-      <c r="AH20" s="395"/>
-      <c r="AI20" s="395"/>
-      <c r="AJ20" s="395"/>
-      <c r="AK20" s="395"/>
-      <c r="AL20" s="395"/>
-      <c r="AM20" s="395"/>
-      <c r="AN20" s="395"/>
-      <c r="AO20" s="395"/>
-      <c r="AP20" s="395"/>
-      <c r="AQ20" s="395"/>
-      <c r="AR20" s="395"/>
-      <c r="AS20" s="399" t="s">
+      <c r="W20" s="347"/>
+      <c r="X20" s="347"/>
+      <c r="Y20" s="347"/>
+      <c r="Z20" s="347"/>
+      <c r="AA20" s="347"/>
+      <c r="AB20" s="347"/>
+      <c r="AC20" s="352"/>
+      <c r="AD20" s="347"/>
+      <c r="AE20" s="347"/>
+      <c r="AF20" s="347"/>
+      <c r="AG20" s="347"/>
+      <c r="AH20" s="347"/>
+      <c r="AI20" s="347"/>
+      <c r="AJ20" s="347"/>
+      <c r="AK20" s="347"/>
+      <c r="AL20" s="347"/>
+      <c r="AM20" s="347"/>
+      <c r="AN20" s="347"/>
+      <c r="AO20" s="347"/>
+      <c r="AP20" s="347"/>
+      <c r="AQ20" s="347"/>
+      <c r="AR20" s="347"/>
+      <c r="AS20" s="351" t="s">
         <v>252</v>
       </c>
       <c r="AT20" s="152" t="str">
         <f>IF(ISBLANK(ETPT_TJ_DDG!$D$5),"",IF(ISERROR(ETPT_TJ!AT20),"",IF(ETPT_TJ!AT20=0,"",ETPT_TJ!AT20)))</f>
         <v/>
       </c>
-      <c r="AU20" s="395"/>
-      <c r="AV20" s="395"/>
-      <c r="AW20" s="395"/>
-      <c r="AX20" s="395"/>
-      <c r="AY20" s="395"/>
-      <c r="AZ20" s="395"/>
-      <c r="BA20" s="395"/>
-      <c r="BB20" s="395"/>
-      <c r="BC20" s="395"/>
-      <c r="BD20" s="395"/>
-      <c r="BE20" s="395"/>
+      <c r="AU20" s="347"/>
+      <c r="AV20" s="347"/>
+      <c r="AW20" s="347"/>
+      <c r="AX20" s="347"/>
+      <c r="AY20" s="347"/>
+      <c r="AZ20" s="347"/>
+      <c r="BA20" s="347"/>
+      <c r="BB20" s="347"/>
+      <c r="BC20" s="347"/>
+      <c r="BD20" s="347"/>
+      <c r="BE20" s="347"/>
     </row>
     <row r="21" spans="4:57" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="E21" s="39"/>
     </row>
     <row r="22" spans="4:57" ht="69" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E22" s="377" t="s">
+      <c r="E22" s="393" t="s">
         <v>370</v>
       </c>
-      <c r="F22" s="378"/>
-      <c r="G22" s="378"/>
-      <c r="H22" s="378"/>
-      <c r="I22" s="378"/>
-      <c r="J22" s="378"/>
-      <c r="K22" s="378"/>
-      <c r="L22" s="378"/>
-      <c r="M22" s="378"/>
-      <c r="N22" s="378"/>
-      <c r="O22" s="378"/>
-      <c r="P22" s="378"/>
-      <c r="Q22" s="378"/>
-      <c r="R22" s="378"/>
-      <c r="S22" s="378"/>
-      <c r="T22" s="378"/>
-      <c r="U22" s="378"/>
-      <c r="V22" s="378"/>
-      <c r="W22" s="378"/>
-      <c r="X22" s="379"/>
+      <c r="F22" s="394"/>
+      <c r="G22" s="394"/>
+      <c r="H22" s="394"/>
+      <c r="I22" s="394"/>
+      <c r="J22" s="394"/>
+      <c r="K22" s="394"/>
+      <c r="L22" s="394"/>
+      <c r="M22" s="394"/>
+      <c r="N22" s="394"/>
+      <c r="O22" s="394"/>
+      <c r="P22" s="394"/>
+      <c r="Q22" s="394"/>
+      <c r="R22" s="394"/>
+      <c r="S22" s="394"/>
+      <c r="T22" s="394"/>
+      <c r="U22" s="394"/>
+      <c r="V22" s="394"/>
+      <c r="W22" s="394"/>
+      <c r="X22" s="395"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -20598,13 +20598,13 @@
       <c r="A2" s="78"/>
       <c r="B2" s="78"/>
       <c r="C2" s="78"/>
-      <c r="D2" s="395"/>
-      <c r="E2" s="395"/>
-      <c r="F2" s="395"/>
+      <c r="D2" s="347"/>
+      <c r="E2" s="347"/>
+      <c r="F2" s="347"/>
       <c r="G2" s="75" t="s">
         <v>169</v>
       </c>
-      <c r="H2" s="373" t="s">
+      <c r="H2" s="389" t="s">
         <v>168</v>
       </c>
       <c r="I2" s="75" t="s">
@@ -20637,7 +20637,7 @@
       <c r="R2" s="75" t="s">
         <v>167</v>
       </c>
-      <c r="S2" s="373" t="s">
+      <c r="S2" s="389" t="s">
         <v>166</v>
       </c>
       <c r="T2" s="75" t="s">
@@ -20667,7 +20667,7 @@
       <c r="AB2" s="75" t="s">
         <v>164</v>
       </c>
-      <c r="AC2" s="373" t="s">
+      <c r="AC2" s="389" t="s">
         <v>213</v>
       </c>
       <c r="AD2" s="75" t="s">
@@ -20679,7 +20679,7 @@
       <c r="AF2" s="75" t="s">
         <v>212</v>
       </c>
-      <c r="AG2" s="373" t="s">
+      <c r="AG2" s="389" t="s">
         <v>211</v>
       </c>
     </row>
@@ -20687,13 +20687,13 @@
       <c r="A3" s="78"/>
       <c r="B3" s="78"/>
       <c r="C3" s="78"/>
-      <c r="D3" s="395"/>
-      <c r="E3" s="395"/>
-      <c r="F3" s="395"/>
+      <c r="D3" s="347"/>
+      <c r="E3" s="347"/>
+      <c r="F3" s="347"/>
       <c r="G3" s="75" t="s">
         <v>158</v>
       </c>
-      <c r="H3" s="373"/>
+      <c r="H3" s="389"/>
       <c r="I3" s="75" t="s">
         <v>210</v>
       </c>
@@ -20724,7 +20724,7 @@
       <c r="R3" s="75" t="s">
         <v>145</v>
       </c>
-      <c r="S3" s="373"/>
+      <c r="S3" s="389"/>
       <c r="T3" s="75" t="s">
         <v>201</v>
       </c>
@@ -20752,7 +20752,7 @@
       <c r="AB3" s="75" t="s">
         <v>193</v>
       </c>
-      <c r="AC3" s="373"/>
+      <c r="AC3" s="389"/>
       <c r="AD3" s="75" t="s">
         <v>192</v>
       </c>
@@ -20762,7 +20762,7 @@
       <c r="AF3" s="75" t="s">
         <v>122</v>
       </c>
-      <c r="AG3" s="373"/>
+      <c r="AG3" s="389"/>
     </row>
     <row r="4" spans="1:60" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="78"/>
@@ -20784,7 +20784,7 @@
       <c r="G4" s="75" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="373"/>
+      <c r="H4" s="389"/>
       <c r="I4" s="75" t="s">
         <v>191</v>
       </c>
@@ -20815,7 +20815,7 @@
       <c r="R4" s="75" t="s">
         <v>94</v>
       </c>
-      <c r="S4" s="373"/>
+      <c r="S4" s="389"/>
       <c r="T4" s="75" t="s">
         <v>182</v>
       </c>
@@ -20843,7 +20843,7 @@
       <c r="AB4" s="75" t="s">
         <v>174</v>
       </c>
-      <c r="AC4" s="373"/>
+      <c r="AC4" s="389"/>
       <c r="AD4" s="75" t="s">
         <v>616</v>
       </c>
@@ -20853,7 +20853,7 @@
       <c r="AF4" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="AG4" s="373"/>
+      <c r="AG4" s="389"/>
     </row>
     <row r="5" spans="1:60" x14ac:dyDescent="0.2">
       <c r="A5" s="81" t="s">
@@ -22346,83 +22346,83 @@
       </c>
     </row>
     <row r="17" spans="4:33" x14ac:dyDescent="0.2">
-      <c r="D17" s="395"/>
-      <c r="E17" s="395"/>
-      <c r="F17" s="395"/>
-      <c r="G17" s="395"/>
-      <c r="H17" s="395"/>
-      <c r="I17" s="395"/>
-      <c r="J17" s="395"/>
-      <c r="K17" s="395"/>
-      <c r="L17" s="395"/>
-      <c r="M17" s="395"/>
-      <c r="N17" s="395"/>
-      <c r="O17" s="395"/>
-      <c r="P17" s="395"/>
-      <c r="Q17" s="395"/>
-      <c r="R17" s="395"/>
-      <c r="S17" s="396"/>
-      <c r="T17" s="395"/>
-      <c r="U17" s="395"/>
-      <c r="V17" s="395"/>
-      <c r="W17" s="395"/>
-      <c r="X17" s="395"/>
-      <c r="Y17" s="395"/>
-      <c r="Z17" s="395"/>
-      <c r="AA17" s="395"/>
-      <c r="AB17" s="395"/>
-      <c r="AC17" s="395"/>
-      <c r="AD17" s="395"/>
-      <c r="AE17" s="395"/>
-      <c r="AF17" s="395"/>
-      <c r="AG17" s="395"/>
+      <c r="D17" s="347"/>
+      <c r="E17" s="347"/>
+      <c r="F17" s="347"/>
+      <c r="G17" s="347"/>
+      <c r="H17" s="347"/>
+      <c r="I17" s="347"/>
+      <c r="J17" s="347"/>
+      <c r="K17" s="347"/>
+      <c r="L17" s="347"/>
+      <c r="M17" s="347"/>
+      <c r="N17" s="347"/>
+      <c r="O17" s="347"/>
+      <c r="P17" s="347"/>
+      <c r="Q17" s="347"/>
+      <c r="R17" s="347"/>
+      <c r="S17" s="348"/>
+      <c r="T17" s="347"/>
+      <c r="U17" s="347"/>
+      <c r="V17" s="347"/>
+      <c r="W17" s="347"/>
+      <c r="X17" s="347"/>
+      <c r="Y17" s="347"/>
+      <c r="Z17" s="347"/>
+      <c r="AA17" s="347"/>
+      <c r="AB17" s="347"/>
+      <c r="AC17" s="347"/>
+      <c r="AD17" s="347"/>
+      <c r="AE17" s="347"/>
+      <c r="AF17" s="347"/>
+      <c r="AG17" s="347"/>
     </row>
     <row r="18" spans="4:33" ht="24" x14ac:dyDescent="0.2">
-      <c r="D18" s="401"/>
-      <c r="E18" s="402"/>
-      <c r="F18" s="398" t="s">
+      <c r="D18" s="353"/>
+      <c r="E18" s="354"/>
+      <c r="F18" s="350" t="s">
         <v>253</v>
       </c>
       <c r="G18" s="152" t="str">
         <f>IF(ISBLANK(ETPT_TPRX_DDG!$D$5),"",IF(ISERROR(ETPT_TPRX!G18),"",IF(ETPT_TPRX!G18=0,"",ETPT_TPRX!G18)))</f>
         <v/>
       </c>
-      <c r="H18" s="402"/>
-      <c r="I18" s="402"/>
-      <c r="J18" s="402"/>
-      <c r="K18" s="402"/>
-      <c r="L18" s="395"/>
-      <c r="M18" s="395"/>
-      <c r="N18" s="395"/>
-      <c r="O18" s="395"/>
-      <c r="P18" s="395"/>
-      <c r="Q18" s="399" t="s">
+      <c r="H18" s="354"/>
+      <c r="I18" s="354"/>
+      <c r="J18" s="354"/>
+      <c r="K18" s="354"/>
+      <c r="L18" s="347"/>
+      <c r="M18" s="347"/>
+      <c r="N18" s="347"/>
+      <c r="O18" s="347"/>
+      <c r="P18" s="347"/>
+      <c r="Q18" s="351" t="s">
         <v>254</v>
       </c>
       <c r="R18" s="152" t="str">
         <f>IF(ISBLANK(ETPT_TPRX_DDG!$D$5),"",IF(ISERROR(ETPT_TPRX!R18),"",IF(ETPT_TPRX!R18=0,"",ETPT_TPRX!R18)))</f>
         <v/>
       </c>
-      <c r="S18" s="395"/>
-      <c r="T18" s="395"/>
-      <c r="U18" s="395"/>
-      <c r="V18" s="395"/>
-      <c r="W18" s="395"/>
-      <c r="X18" s="395"/>
-      <c r="Y18" s="395"/>
-      <c r="Z18" s="395"/>
-      <c r="AA18" s="395"/>
-      <c r="AB18" s="395"/>
-      <c r="AC18" s="395"/>
-      <c r="AD18" s="402"/>
-      <c r="AE18" s="399" t="s">
+      <c r="S18" s="347"/>
+      <c r="T18" s="347"/>
+      <c r="U18" s="347"/>
+      <c r="V18" s="347"/>
+      <c r="W18" s="347"/>
+      <c r="X18" s="347"/>
+      <c r="Y18" s="347"/>
+      <c r="Z18" s="347"/>
+      <c r="AA18" s="347"/>
+      <c r="AB18" s="347"/>
+      <c r="AC18" s="347"/>
+      <c r="AD18" s="354"/>
+      <c r="AE18" s="351" t="s">
         <v>252</v>
       </c>
       <c r="AF18" s="152" t="str">
         <f>IF(ISBLANK(ETPT_TPRX_DDG!$D$5),"",IF(ISERROR(ETPT_TPRX!AF18),"",IF(ETPT_TPRX!AF18=0,"",ETPT_TPRX!AF18)))</f>
         <v/>
       </c>
-      <c r="AG18" s="395"/>
+      <c r="AG18" s="347"/>
     </row>
     <row r="20" spans="4:33" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="E20" s="139" t="s">
@@ -22436,32 +22436,32 @@
       <c r="K20" s="140"/>
     </row>
     <row r="21" spans="4:33" ht="50" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E21" s="380" t="s">
+      <c r="E21" s="396" t="s">
         <v>371</v>
       </c>
-      <c r="F21" s="381"/>
-      <c r="G21" s="381"/>
-      <c r="H21" s="381"/>
-      <c r="I21" s="381"/>
-      <c r="J21" s="381"/>
-      <c r="K21" s="381"/>
-      <c r="L21" s="381"/>
-      <c r="M21" s="381"/>
-      <c r="N21" s="381"/>
-      <c r="O21" s="381"/>
-      <c r="P21" s="381"/>
-      <c r="Q21" s="381"/>
-      <c r="R21" s="381"/>
-      <c r="S21" s="381"/>
-      <c r="T21" s="381"/>
-      <c r="U21" s="381"/>
-      <c r="V21" s="381"/>
-      <c r="W21" s="381"/>
-      <c r="X21" s="381"/>
-      <c r="Y21" s="381"/>
-      <c r="Z21" s="381"/>
-      <c r="AA21" s="381"/>
-      <c r="AB21" s="382"/>
+      <c r="F21" s="397"/>
+      <c r="G21" s="397"/>
+      <c r="H21" s="397"/>
+      <c r="I21" s="397"/>
+      <c r="J21" s="397"/>
+      <c r="K21" s="397"/>
+      <c r="L21" s="397"/>
+      <c r="M21" s="397"/>
+      <c r="N21" s="397"/>
+      <c r="O21" s="397"/>
+      <c r="P21" s="397"/>
+      <c r="Q21" s="397"/>
+      <c r="R21" s="397"/>
+      <c r="S21" s="397"/>
+      <c r="T21" s="397"/>
+      <c r="U21" s="397"/>
+      <c r="V21" s="397"/>
+      <c r="W21" s="397"/>
+      <c r="X21" s="397"/>
+      <c r="Y21" s="397"/>
+      <c r="Z21" s="397"/>
+      <c r="AA21" s="397"/>
+      <c r="AB21" s="398"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -22564,7 +22564,7 @@
       <c r="G2" s="75" t="s">
         <v>167</v>
       </c>
-      <c r="H2" s="373" t="s">
+      <c r="H2" s="389" t="s">
         <v>166</v>
       </c>
     </row>
@@ -22572,7 +22572,7 @@
       <c r="G3" s="75" t="s">
         <v>145</v>
       </c>
-      <c r="H3" s="373"/>
+      <c r="H3" s="389"/>
     </row>
     <row r="4" spans="1:62" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="97"/>
@@ -22594,7 +22594,7 @@
       <c r="G4" s="75" t="s">
         <v>94</v>
       </c>
-      <c r="H4" s="373"/>
+      <c r="H4" s="389"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="91" t="s">
@@ -22848,15 +22848,15 @@
       <c r="J16" s="21"/>
     </row>
     <row r="17" spans="4:10" ht="99" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D17" s="383" t="s">
+      <c r="D17" s="399" t="s">
         <v>372</v>
       </c>
-      <c r="E17" s="384"/>
-      <c r="F17" s="384"/>
-      <c r="G17" s="384"/>
-      <c r="H17" s="384"/>
-      <c r="I17" s="384"/>
-      <c r="J17" s="385"/>
+      <c r="E17" s="400"/>
+      <c r="F17" s="400"/>
+      <c r="G17" s="400"/>
+      <c r="H17" s="400"/>
+      <c r="I17" s="400"/>
+      <c r="J17" s="401"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -22985,7 +22985,7 @@
       <c r="P2" s="277" t="s">
         <v>38</v>
       </c>
-      <c r="Q2" s="376" t="s">
+      <c r="Q2" s="392" t="s">
         <v>274</v>
       </c>
     </row>
@@ -23026,7 +23026,7 @@
       <c r="P3" s="277" t="s">
         <v>281</v>
       </c>
-      <c r="Q3" s="376"/>
+      <c r="Q3" s="392"/>
     </row>
     <row r="4" spans="1:62" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="278"/>
@@ -23036,13 +23036,13 @@
       <c r="C4" s="279" t="s">
         <v>111</v>
       </c>
-      <c r="D4" s="403" t="s">
+      <c r="D4" s="355" t="s">
         <v>32</v>
       </c>
-      <c r="E4" s="403" t="s">
+      <c r="E4" s="355" t="s">
         <v>282</v>
       </c>
-      <c r="F4" s="403" t="s">
+      <c r="F4" s="355" t="s">
         <v>109</v>
       </c>
       <c r="G4" s="277" t="s">
@@ -23075,7 +23075,7 @@
       <c r="P4" s="277" t="s">
         <v>292</v>
       </c>
-      <c r="Q4" s="376"/>
+      <c r="Q4" s="392"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="281" t="s">
@@ -23087,43 +23087,43 @@
       <c r="E5" s="282" t="s">
         <v>62</v>
       </c>
-      <c r="F5" s="404" t="s">
+      <c r="F5" s="356" t="s">
         <v>61</v>
       </c>
-      <c r="G5" s="409"/>
-      <c r="H5" s="410" t="str">
+      <c r="G5" s="361"/>
+      <c r="H5" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!H5),"",IF(ISERROR(ETPT_JUR_ASS!H5),"",IF(ETPT_JUR_ASS!H5=0,"",ETPT_JUR_ASS!H5)))</f>
         <v/>
       </c>
-      <c r="I5" s="410" t="str">
+      <c r="I5" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!I5),"",IF(ISERROR(ETPT_JUR_ASS!I5),"",IF(ETPT_JUR_ASS!I5=0,"",ETPT_JUR_ASS!I5)))</f>
         <v/>
       </c>
-      <c r="J5" s="410" t="str">
+      <c r="J5" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!J5),"",IF(ISERROR(ETPT_JUR_ASS!J5),"",IF(ETPT_JUR_ASS!J5=0,"",ETPT_JUR_ASS!J5)))</f>
         <v/>
       </c>
-      <c r="K5" s="410" t="str">
+      <c r="K5" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!K5),"",IF(ISERROR(ETPT_JUR_ASS!K5),"",IF(ETPT_JUR_ASS!K5=0,"",ETPT_JUR_ASS!K5)))</f>
         <v/>
       </c>
-      <c r="L5" s="410" t="str">
+      <c r="L5" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!L5),"",IF(ISERROR(ETPT_JUR_ASS!L5),"",IF(ETPT_JUR_ASS!L5=0,"",ETPT_JUR_ASS!L5)))</f>
         <v/>
       </c>
-      <c r="M5" s="410" t="str">
+      <c r="M5" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!M5),"",IF(ISERROR(ETPT_JUR_ASS!M5),"",IF(ETPT_JUR_ASS!M5=0,"",ETPT_JUR_ASS!M5)))</f>
         <v/>
       </c>
-      <c r="N5" s="410" t="str">
+      <c r="N5" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!N5),"",IF(ISERROR(ETPT_JUR_ASS!N5),"",IF(ETPT_JUR_ASS!N5=0,"",ETPT_JUR_ASS!N5)))</f>
         <v/>
       </c>
-      <c r="O5" s="410" t="str">
+      <c r="O5" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!O5),"",IF(ISERROR(ETPT_JUR_ASS!O5),"",IF(ETPT_JUR_ASS!O5=0,"",ETPT_JUR_ASS!O5)))</f>
         <v/>
       </c>
-      <c r="P5" s="410" t="str">
+      <c r="P5" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!P5),"",IF(ISERROR(ETPT_JUR_ASS!P5),"",IF(ETPT_JUR_ASS!P5=0,"",ETPT_JUR_ASS!P5)))</f>
         <v/>
       </c>
@@ -23145,43 +23145,43 @@
       <c r="E6" s="282" t="s">
         <v>60</v>
       </c>
-      <c r="F6" s="404" t="s">
+      <c r="F6" s="356" t="s">
         <v>59</v>
       </c>
-      <c r="G6" s="408"/>
-      <c r="H6" s="410" t="str">
+      <c r="G6" s="360"/>
+      <c r="H6" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!H6),"",IF(ISERROR(ETPT_JUR_ASS!H6),"",IF(ETPT_JUR_ASS!H6=0,"",ETPT_JUR_ASS!H6)))</f>
         <v/>
       </c>
-      <c r="I6" s="410" t="str">
+      <c r="I6" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!I6),"",IF(ISERROR(ETPT_JUR_ASS!I6),"",IF(ETPT_JUR_ASS!I6=0,"",ETPT_JUR_ASS!I6)))</f>
         <v/>
       </c>
-      <c r="J6" s="410" t="str">
+      <c r="J6" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!J6),"",IF(ISERROR(ETPT_JUR_ASS!J6),"",IF(ETPT_JUR_ASS!J6=0,"",ETPT_JUR_ASS!J6)))</f>
         <v/>
       </c>
-      <c r="K6" s="410" t="str">
+      <c r="K6" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!K6),"",IF(ISERROR(ETPT_JUR_ASS!K6),"",IF(ETPT_JUR_ASS!K6=0,"",ETPT_JUR_ASS!K6)))</f>
         <v/>
       </c>
-      <c r="L6" s="410" t="str">
+      <c r="L6" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!L6),"",IF(ISERROR(ETPT_JUR_ASS!L6),"",IF(ETPT_JUR_ASS!L6=0,"",ETPT_JUR_ASS!L6)))</f>
         <v/>
       </c>
-      <c r="M6" s="410" t="str">
+      <c r="M6" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!M6),"",IF(ISERROR(ETPT_JUR_ASS!M6),"",IF(ETPT_JUR_ASS!M6=0,"",ETPT_JUR_ASS!M6)))</f>
         <v/>
       </c>
-      <c r="N6" s="410" t="str">
+      <c r="N6" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!N6),"",IF(ISERROR(ETPT_JUR_ASS!N6),"",IF(ETPT_JUR_ASS!N6=0,"",ETPT_JUR_ASS!N6)))</f>
         <v/>
       </c>
-      <c r="O6" s="410" t="str">
+      <c r="O6" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!O6),"",IF(ISERROR(ETPT_JUR_ASS!O6),"",IF(ETPT_JUR_ASS!O6=0,"",ETPT_JUR_ASS!O6)))</f>
         <v/>
       </c>
-      <c r="P6" s="410" t="str">
+      <c r="P6" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!P6),"",IF(ISERROR(ETPT_JUR_ASS!P6),"",IF(ETPT_JUR_ASS!P6=0,"",ETPT_JUR_ASS!P6)))</f>
         <v/>
       </c>
@@ -23203,43 +23203,43 @@
       <c r="E7" s="282" t="s">
         <v>56</v>
       </c>
-      <c r="F7" s="404" t="s">
+      <c r="F7" s="356" t="s">
         <v>55</v>
       </c>
-      <c r="G7" s="408"/>
-      <c r="H7" s="410" t="str">
+      <c r="G7" s="360"/>
+      <c r="H7" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!H7),"",IF(ISERROR(ETPT_JUR_ASS!H7),"",IF(ETPT_JUR_ASS!H7=0,"",ETPT_JUR_ASS!H7)))</f>
         <v/>
       </c>
-      <c r="I7" s="410" t="str">
+      <c r="I7" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!I7),"",IF(ISERROR(ETPT_JUR_ASS!I7),"",IF(ETPT_JUR_ASS!I7=0,"",ETPT_JUR_ASS!I7)))</f>
         <v/>
       </c>
-      <c r="J7" s="410" t="str">
+      <c r="J7" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!J7),"",IF(ISERROR(ETPT_JUR_ASS!J7),"",IF(ETPT_JUR_ASS!J7=0,"",ETPT_JUR_ASS!J7)))</f>
         <v/>
       </c>
-      <c r="K7" s="410" t="str">
+      <c r="K7" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!K7),"",IF(ISERROR(ETPT_JUR_ASS!K7),"",IF(ETPT_JUR_ASS!K7=0,"",ETPT_JUR_ASS!K7)))</f>
         <v/>
       </c>
-      <c r="L7" s="410" t="str">
+      <c r="L7" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!L7),"",IF(ISERROR(ETPT_JUR_ASS!L7),"",IF(ETPT_JUR_ASS!L7=0,"",ETPT_JUR_ASS!L7)))</f>
         <v/>
       </c>
-      <c r="M7" s="410" t="str">
+      <c r="M7" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!M7),"",IF(ISERROR(ETPT_JUR_ASS!M7),"",IF(ETPT_JUR_ASS!M7=0,"",ETPT_JUR_ASS!M7)))</f>
         <v/>
       </c>
-      <c r="N7" s="410" t="str">
+      <c r="N7" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!N7),"",IF(ISERROR(ETPT_JUR_ASS!N7),"",IF(ETPT_JUR_ASS!N7=0,"",ETPT_JUR_ASS!N7)))</f>
         <v/>
       </c>
-      <c r="O7" s="410" t="str">
+      <c r="O7" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!O7),"",IF(ISERROR(ETPT_JUR_ASS!O7),"",IF(ETPT_JUR_ASS!O7=0,"",ETPT_JUR_ASS!O7)))</f>
         <v/>
       </c>
-      <c r="P7" s="410" t="str">
+      <c r="P7" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!P7),"",IF(ISERROR(ETPT_JUR_ASS!P7),"",IF(ETPT_JUR_ASS!P7=0,"",ETPT_JUR_ASS!P7)))</f>
         <v/>
       </c>
@@ -23261,43 +23261,43 @@
       <c r="E8" s="282" t="s">
         <v>54</v>
       </c>
-      <c r="F8" s="404" t="s">
+      <c r="F8" s="356" t="s">
         <v>53</v>
       </c>
-      <c r="G8" s="408"/>
-      <c r="H8" s="410" t="str">
+      <c r="G8" s="360"/>
+      <c r="H8" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!H8),"",IF(ISERROR(ETPT_JUR_ASS!H8),"",IF(ETPT_JUR_ASS!H8=0,"",ETPT_JUR_ASS!H8)))</f>
         <v/>
       </c>
-      <c r="I8" s="410" t="str">
+      <c r="I8" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!I8),"",IF(ISERROR(ETPT_JUR_ASS!I8),"",IF(ETPT_JUR_ASS!I8=0,"",ETPT_JUR_ASS!I8)))</f>
         <v/>
       </c>
-      <c r="J8" s="410" t="str">
+      <c r="J8" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!J8),"",IF(ISERROR(ETPT_JUR_ASS!J8),"",IF(ETPT_JUR_ASS!J8=0,"",ETPT_JUR_ASS!J8)))</f>
         <v/>
       </c>
-      <c r="K8" s="410" t="str">
+      <c r="K8" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!K8),"",IF(ISERROR(ETPT_JUR_ASS!K8),"",IF(ETPT_JUR_ASS!K8=0,"",ETPT_JUR_ASS!K8)))</f>
         <v/>
       </c>
-      <c r="L8" s="410" t="str">
+      <c r="L8" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!L8),"",IF(ISERROR(ETPT_JUR_ASS!L8),"",IF(ETPT_JUR_ASS!L8=0,"",ETPT_JUR_ASS!L8)))</f>
         <v/>
       </c>
-      <c r="M8" s="410" t="str">
+      <c r="M8" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!M8),"",IF(ISERROR(ETPT_JUR_ASS!M8),"",IF(ETPT_JUR_ASS!M8=0,"",ETPT_JUR_ASS!M8)))</f>
         <v/>
       </c>
-      <c r="N8" s="410" t="str">
+      <c r="N8" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!N8),"",IF(ISERROR(ETPT_JUR_ASS!N8),"",IF(ETPT_JUR_ASS!N8=0,"",ETPT_JUR_ASS!N8)))</f>
         <v/>
       </c>
-      <c r="O8" s="410" t="str">
+      <c r="O8" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!O8),"",IF(ISERROR(ETPT_JUR_ASS!O8),"",IF(ETPT_JUR_ASS!O8=0,"",ETPT_JUR_ASS!O8)))</f>
         <v/>
       </c>
-      <c r="P8" s="410" t="str">
+      <c r="P8" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!P8),"",IF(ISERROR(ETPT_JUR_ASS!P8),"",IF(ETPT_JUR_ASS!P8=0,"",ETPT_JUR_ASS!P8)))</f>
         <v/>
       </c>
@@ -23319,43 +23319,43 @@
       <c r="E9" s="282" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="404" t="s">
+      <c r="F9" s="356" t="s">
         <v>51</v>
       </c>
-      <c r="G9" s="408"/>
-      <c r="H9" s="410" t="str">
+      <c r="G9" s="360"/>
+      <c r="H9" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!H9),"",IF(ISERROR(ETPT_JUR_ASS!H9),"",IF(ETPT_JUR_ASS!H9=0,"",ETPT_JUR_ASS!H9)))</f>
         <v/>
       </c>
-      <c r="I9" s="410" t="str">
+      <c r="I9" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!I9),"",IF(ISERROR(ETPT_JUR_ASS!I9),"",IF(ETPT_JUR_ASS!I9=0,"",ETPT_JUR_ASS!I9)))</f>
         <v/>
       </c>
-      <c r="J9" s="410" t="str">
+      <c r="J9" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!J9),"",IF(ISERROR(ETPT_JUR_ASS!J9),"",IF(ETPT_JUR_ASS!J9=0,"",ETPT_JUR_ASS!J9)))</f>
         <v/>
       </c>
-      <c r="K9" s="410" t="str">
+      <c r="K9" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!K9),"",IF(ISERROR(ETPT_JUR_ASS!K9),"",IF(ETPT_JUR_ASS!K9=0,"",ETPT_JUR_ASS!K9)))</f>
         <v/>
       </c>
-      <c r="L9" s="410" t="str">
+      <c r="L9" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!L9),"",IF(ISERROR(ETPT_JUR_ASS!L9),"",IF(ETPT_JUR_ASS!L9=0,"",ETPT_JUR_ASS!L9)))</f>
         <v/>
       </c>
-      <c r="M9" s="410" t="str">
+      <c r="M9" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!M9),"",IF(ISERROR(ETPT_JUR_ASS!M9),"",IF(ETPT_JUR_ASS!M9=0,"",ETPT_JUR_ASS!M9)))</f>
         <v/>
       </c>
-      <c r="N9" s="410" t="str">
+      <c r="N9" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!N9),"",IF(ISERROR(ETPT_JUR_ASS!N9),"",IF(ETPT_JUR_ASS!N9=0,"",ETPT_JUR_ASS!N9)))</f>
         <v/>
       </c>
-      <c r="O9" s="410" t="str">
+      <c r="O9" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!O9),"",IF(ISERROR(ETPT_JUR_ASS!O9),"",IF(ETPT_JUR_ASS!O9=0,"",ETPT_JUR_ASS!O9)))</f>
         <v/>
       </c>
-      <c r="P9" s="410" t="str">
+      <c r="P9" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!P9),"",IF(ISERROR(ETPT_JUR_ASS!P9),"",IF(ETPT_JUR_ASS!P9=0,"",ETPT_JUR_ASS!P9)))</f>
         <v/>
       </c>
@@ -23377,43 +23377,43 @@
       <c r="E10" s="282" t="s">
         <v>50</v>
       </c>
-      <c r="F10" s="404" t="s">
+      <c r="F10" s="356" t="s">
         <v>49</v>
       </c>
-      <c r="G10" s="408"/>
-      <c r="H10" s="410" t="str">
+      <c r="G10" s="360"/>
+      <c r="H10" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!H10),"",IF(ISERROR(ETPT_JUR_ASS!H10),"",IF(ETPT_JUR_ASS!H10=0,"",ETPT_JUR_ASS!H10)))</f>
         <v/>
       </c>
-      <c r="I10" s="410" t="str">
+      <c r="I10" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!I10),"",IF(ISERROR(ETPT_JUR_ASS!I10),"",IF(ETPT_JUR_ASS!I10=0,"",ETPT_JUR_ASS!I10)))</f>
         <v/>
       </c>
-      <c r="J10" s="410" t="str">
+      <c r="J10" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!J10),"",IF(ISERROR(ETPT_JUR_ASS!J10),"",IF(ETPT_JUR_ASS!J10=0,"",ETPT_JUR_ASS!J10)))</f>
         <v/>
       </c>
-      <c r="K10" s="410" t="str">
+      <c r="K10" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!K10),"",IF(ISERROR(ETPT_JUR_ASS!K10),"",IF(ETPT_JUR_ASS!K10=0,"",ETPT_JUR_ASS!K10)))</f>
         <v/>
       </c>
-      <c r="L10" s="410" t="str">
+      <c r="L10" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!L10),"",IF(ISERROR(ETPT_JUR_ASS!L10),"",IF(ETPT_JUR_ASS!L10=0,"",ETPT_JUR_ASS!L10)))</f>
         <v/>
       </c>
-      <c r="M10" s="410" t="str">
+      <c r="M10" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!M10),"",IF(ISERROR(ETPT_JUR_ASS!M10),"",IF(ETPT_JUR_ASS!M10=0,"",ETPT_JUR_ASS!M10)))</f>
         <v/>
       </c>
-      <c r="N10" s="410" t="str">
+      <c r="N10" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!N10),"",IF(ISERROR(ETPT_JUR_ASS!N10),"",IF(ETPT_JUR_ASS!N10=0,"",ETPT_JUR_ASS!N10)))</f>
         <v/>
       </c>
-      <c r="O10" s="410" t="str">
+      <c r="O10" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!O10),"",IF(ISERROR(ETPT_JUR_ASS!O10),"",IF(ETPT_JUR_ASS!O10=0,"",ETPT_JUR_ASS!O10)))</f>
         <v/>
       </c>
-      <c r="P10" s="410" t="str">
+      <c r="P10" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!P10),"",IF(ISERROR(ETPT_JUR_ASS!P10),"",IF(ETPT_JUR_ASS!P10=0,"",ETPT_JUR_ASS!P10)))</f>
         <v/>
       </c>
@@ -23435,43 +23435,43 @@
       <c r="E11" s="282" t="s">
         <v>48</v>
       </c>
-      <c r="F11" s="404" t="s">
+      <c r="F11" s="356" t="s">
         <v>47</v>
       </c>
-      <c r="G11" s="408"/>
-      <c r="H11" s="410" t="str">
+      <c r="G11" s="360"/>
+      <c r="H11" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!H11),"",IF(ISERROR(ETPT_JUR_ASS!H11),"",IF(ETPT_JUR_ASS!H11=0,"",ETPT_JUR_ASS!H11)))</f>
         <v/>
       </c>
-      <c r="I11" s="410" t="str">
+      <c r="I11" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!I11),"",IF(ISERROR(ETPT_JUR_ASS!I11),"",IF(ETPT_JUR_ASS!I11=0,"",ETPT_JUR_ASS!I11)))</f>
         <v/>
       </c>
-      <c r="J11" s="410" t="str">
+      <c r="J11" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!J11),"",IF(ISERROR(ETPT_JUR_ASS!J11),"",IF(ETPT_JUR_ASS!J11=0,"",ETPT_JUR_ASS!J11)))</f>
         <v/>
       </c>
-      <c r="K11" s="410" t="str">
+      <c r="K11" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!K11),"",IF(ISERROR(ETPT_JUR_ASS!K11),"",IF(ETPT_JUR_ASS!K11=0,"",ETPT_JUR_ASS!K11)))</f>
         <v/>
       </c>
-      <c r="L11" s="410" t="str">
+      <c r="L11" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!L11),"",IF(ISERROR(ETPT_JUR_ASS!L11),"",IF(ETPT_JUR_ASS!L11=0,"",ETPT_JUR_ASS!L11)))</f>
         <v/>
       </c>
-      <c r="M11" s="410" t="str">
+      <c r="M11" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!M11),"",IF(ISERROR(ETPT_JUR_ASS!M11),"",IF(ETPT_JUR_ASS!M11=0,"",ETPT_JUR_ASS!M11)))</f>
         <v/>
       </c>
-      <c r="N11" s="410" t="str">
+      <c r="N11" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!N11),"",IF(ISERROR(ETPT_JUR_ASS!N11),"",IF(ETPT_JUR_ASS!N11=0,"",ETPT_JUR_ASS!N11)))</f>
         <v/>
       </c>
-      <c r="O11" s="410" t="str">
+      <c r="O11" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!O11),"",IF(ISERROR(ETPT_JUR_ASS!O11),"",IF(ETPT_JUR_ASS!O11=0,"",ETPT_JUR_ASS!O11)))</f>
         <v/>
       </c>
-      <c r="P11" s="410" t="str">
+      <c r="P11" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!P11),"",IF(ISERROR(ETPT_JUR_ASS!P11),"",IF(ETPT_JUR_ASS!P11=0,"",ETPT_JUR_ASS!P11)))</f>
         <v/>
       </c>
@@ -23493,43 +23493,43 @@
       <c r="E12" s="282" t="s">
         <v>46</v>
       </c>
-      <c r="F12" s="404" t="s">
+      <c r="F12" s="356" t="s">
         <v>45</v>
       </c>
-      <c r="G12" s="408"/>
-      <c r="H12" s="410" t="str">
+      <c r="G12" s="360"/>
+      <c r="H12" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!H12),"",IF(ISERROR(ETPT_JUR_ASS!H12),"",IF(ETPT_JUR_ASS!H12=0,"",ETPT_JUR_ASS!H12)))</f>
         <v/>
       </c>
-      <c r="I12" s="410" t="str">
+      <c r="I12" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!I12),"",IF(ISERROR(ETPT_JUR_ASS!I12),"",IF(ETPT_JUR_ASS!I12=0,"",ETPT_JUR_ASS!I12)))</f>
         <v/>
       </c>
-      <c r="J12" s="410" t="str">
+      <c r="J12" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!J12),"",IF(ISERROR(ETPT_JUR_ASS!J12),"",IF(ETPT_JUR_ASS!J12=0,"",ETPT_JUR_ASS!J12)))</f>
         <v/>
       </c>
-      <c r="K12" s="410" t="str">
+      <c r="K12" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!K12),"",IF(ISERROR(ETPT_JUR_ASS!K12),"",IF(ETPT_JUR_ASS!K12=0,"",ETPT_JUR_ASS!K12)))</f>
         <v/>
       </c>
-      <c r="L12" s="410" t="str">
+      <c r="L12" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!L12),"",IF(ISERROR(ETPT_JUR_ASS!L12),"",IF(ETPT_JUR_ASS!L12=0,"",ETPT_JUR_ASS!L12)))</f>
         <v/>
       </c>
-      <c r="M12" s="410" t="str">
+      <c r="M12" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!M12),"",IF(ISERROR(ETPT_JUR_ASS!M12),"",IF(ETPT_JUR_ASS!M12=0,"",ETPT_JUR_ASS!M12)))</f>
         <v/>
       </c>
-      <c r="N12" s="410" t="str">
+      <c r="N12" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!N12),"",IF(ISERROR(ETPT_JUR_ASS!N12),"",IF(ETPT_JUR_ASS!N12=0,"",ETPT_JUR_ASS!N12)))</f>
         <v/>
       </c>
-      <c r="O12" s="410" t="str">
+      <c r="O12" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!O12),"",IF(ISERROR(ETPT_JUR_ASS!O12),"",IF(ETPT_JUR_ASS!O12=0,"",ETPT_JUR_ASS!O12)))</f>
         <v/>
       </c>
-      <c r="P12" s="410" t="str">
+      <c r="P12" s="362" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!P12),"",IF(ISERROR(ETPT_JUR_ASS!P12),"",IF(ETPT_JUR_ASS!P12=0,"",ETPT_JUR_ASS!P12)))</f>
         <v/>
       </c>
@@ -23542,9 +23542,9 @@
       <c r="A13" s="291"/>
       <c r="B13" s="291"/>
       <c r="C13" s="291"/>
-      <c r="D13" s="405"/>
-      <c r="E13" s="406"/>
-      <c r="F13" s="407" t="s">
+      <c r="D13" s="357"/>
+      <c r="E13" s="358"/>
+      <c r="F13" s="359" t="s">
         <v>39</v>
       </c>
       <c r="G13" s="287">
@@ -23925,13 +23925,13 @@
   <sheetData>
     <row r="1" spans="1:61" s="142" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="141"/>
-      <c r="B1" s="387" t="s">
+      <c r="B1" s="403" t="s">
         <v>170</v>
       </c>
-      <c r="C1" s="387"/>
-      <c r="D1" s="387"/>
-      <c r="E1" s="387"/>
-      <c r="F1" s="387"/>
+      <c r="C1" s="403"/>
+      <c r="D1" s="403"/>
+      <c r="E1" s="403"/>
+      <c r="F1" s="403"/>
       <c r="G1" s="143"/>
       <c r="H1" s="143"/>
       <c r="I1" s="143"/>
@@ -23976,7 +23976,7 @@
       <c r="O2" s="145" t="s">
         <v>164</v>
       </c>
-      <c r="P2" s="386" t="s">
+      <c r="P2" s="402" t="s">
         <v>163</v>
       </c>
       <c r="Q2" s="145" t="s">
@@ -24018,7 +24018,7 @@
       <c r="AC2" s="145" t="s">
         <v>162</v>
       </c>
-      <c r="AD2" s="386" t="s">
+      <c r="AD2" s="402" t="s">
         <v>161</v>
       </c>
       <c r="AE2" s="146" t="s">
@@ -24048,7 +24048,7 @@
       <c r="AM2" s="146" t="s">
         <v>160</v>
       </c>
-      <c r="AN2" s="386" t="s">
+      <c r="AN2" s="402" t="s">
         <v>159</v>
       </c>
       <c r="AZ2" s="146"/>
@@ -24060,7 +24060,7 @@
       <c r="BF2" s="146"/>
       <c r="BG2" s="146"/>
       <c r="BH2" s="146"/>
-      <c r="BI2" s="386"/>
+      <c r="BI2" s="402"/>
     </row>
     <row r="3" spans="1:61" s="142" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="144"/>
@@ -24096,7 +24096,7 @@
       <c r="O3" s="145" t="s">
         <v>135</v>
       </c>
-      <c r="P3" s="386"/>
+      <c r="P3" s="402"/>
       <c r="Q3" s="145" t="s">
         <v>134</v>
       </c>
@@ -24136,7 +24136,7 @@
       <c r="AC3" s="145" t="s">
         <v>122</v>
       </c>
-      <c r="AD3" s="386"/>
+      <c r="AD3" s="402"/>
       <c r="AE3" s="146" t="s">
         <v>121</v>
       </c>
@@ -24164,7 +24164,7 @@
       <c r="AM3" s="146" t="s">
         <v>113</v>
       </c>
-      <c r="AN3" s="386"/>
+      <c r="AN3" s="402"/>
       <c r="AZ3" s="146"/>
       <c r="BA3" s="146"/>
       <c r="BB3" s="146"/>
@@ -24174,7 +24174,7 @@
       <c r="BF3" s="146"/>
       <c r="BG3" s="146"/>
       <c r="BH3" s="146"/>
-      <c r="BI3" s="386"/>
+      <c r="BI3" s="402"/>
     </row>
     <row r="4" spans="1:61" s="142" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="147"/>
@@ -24220,7 +24220,7 @@
       <c r="O4" s="145" t="s">
         <v>85</v>
       </c>
-      <c r="P4" s="386"/>
+      <c r="P4" s="402"/>
       <c r="Q4" s="145" t="s">
         <v>84</v>
       </c>
@@ -24260,7 +24260,7 @@
       <c r="AC4" s="145" t="s">
         <v>72</v>
       </c>
-      <c r="AD4" s="386"/>
+      <c r="AD4" s="402"/>
       <c r="AE4" s="146" t="s">
         <v>71</v>
       </c>
@@ -24288,7 +24288,7 @@
       <c r="AM4" s="146" t="s">
         <v>63</v>
       </c>
-      <c r="AN4" s="386"/>
+      <c r="AN4" s="402"/>
       <c r="AZ4" s="146"/>
       <c r="BA4" s="146"/>
       <c r="BB4" s="146"/>
@@ -24298,7 +24298,7 @@
       <c r="BF4" s="146"/>
       <c r="BG4" s="146"/>
       <c r="BH4" s="146"/>
-      <c r="BI4" s="386"/>
+      <c r="BI4" s="402"/>
     </row>
     <row r="5" spans="1:61" s="142" customFormat="1" ht="144" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="149" t="s">
@@ -25934,14 +25934,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="388" t="s">
+      <c r="A1" s="404" t="s">
         <v>214</v>
       </c>
-      <c r="B1" s="388"/>
-      <c r="C1" s="388"/>
-      <c r="D1" s="388"/>
-      <c r="E1" s="388"/>
-      <c r="F1" s="388"/>
+      <c r="B1" s="404"/>
+      <c r="C1" s="404"/>
+      <c r="D1" s="404"/>
+      <c r="E1" s="404"/>
+      <c r="F1" s="404"/>
       <c r="G1" s="319"/>
       <c r="H1" s="319"/>
       <c r="I1" s="319"/>
@@ -25991,7 +25991,7 @@
       <c r="O2" s="173" t="s">
         <v>164</v>
       </c>
-      <c r="P2" s="389" t="s">
+      <c r="P2" s="405" t="s">
         <v>213</v>
       </c>
       <c r="Q2" s="173" t="s">
@@ -26003,7 +26003,7 @@
       <c r="S2" s="173" t="s">
         <v>212</v>
       </c>
-      <c r="T2" s="389" t="s">
+      <c r="T2" s="405" t="s">
         <v>211</v>
       </c>
     </row>
@@ -26041,7 +26041,7 @@
       <c r="O3" s="173" t="s">
         <v>193</v>
       </c>
-      <c r="P3" s="389"/>
+      <c r="P3" s="405"/>
       <c r="Q3" s="173" t="s">
         <v>192</v>
       </c>
@@ -26051,7 +26051,7 @@
       <c r="S3" s="173" t="s">
         <v>122</v>
       </c>
-      <c r="T3" s="389"/>
+      <c r="T3" s="405"/>
     </row>
     <row r="4" spans="1:20" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="172"/>
@@ -26097,7 +26097,7 @@
       <c r="O4" s="173" t="s">
         <v>174</v>
       </c>
-      <c r="P4" s="389"/>
+      <c r="P4" s="405"/>
       <c r="Q4" s="173" t="s">
         <v>173</v>
       </c>
@@ -26107,7 +26107,7 @@
       <c r="S4" s="173" t="s">
         <v>72</v>
       </c>
-      <c r="T4" s="389"/>
+      <c r="T4" s="405"/>
     </row>
     <row r="5" spans="1:20" ht="204" x14ac:dyDescent="0.2">
       <c r="A5" s="321" t="s">
@@ -26701,16 +26701,16 @@
   <sheetData>
     <row r="1" spans="1:23" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="181"/>
-      <c r="B1" s="390" t="s">
+      <c r="B1" s="406" t="s">
         <v>170</v>
       </c>
-      <c r="C1" s="390"/>
-      <c r="D1" s="390"/>
-      <c r="E1" s="390"/>
-      <c r="F1" s="390"/>
-      <c r="G1" s="390"/>
-      <c r="H1" s="390"/>
-      <c r="I1" s="390"/>
+      <c r="C1" s="406"/>
+      <c r="D1" s="406"/>
+      <c r="E1" s="406"/>
+      <c r="F1" s="406"/>
+      <c r="G1" s="406"/>
+      <c r="H1" s="406"/>
+      <c r="I1" s="406"/>
       <c r="J1" s="178"/>
       <c r="K1" s="178"/>
       <c r="L1" s="178"/>
@@ -26736,7 +26736,7 @@
       <c r="G2" s="180" t="s">
         <v>169</v>
       </c>
-      <c r="H2" s="391" t="s">
+      <c r="H2" s="407" t="s">
         <v>168</v>
       </c>
       <c r="I2" s="182" t="s">
@@ -26781,7 +26781,7 @@
       <c r="V2" s="182" t="s">
         <v>167</v>
       </c>
-      <c r="W2" s="391" t="s">
+      <c r="W2" s="407" t="s">
         <v>166</v>
       </c>
     </row>
@@ -26795,7 +26795,7 @@
       <c r="G3" s="180" t="s">
         <v>158</v>
       </c>
-      <c r="H3" s="391"/>
+      <c r="H3" s="407"/>
       <c r="I3" s="182" t="s">
         <v>157</v>
       </c>
@@ -26836,7 +26836,7 @@
       <c r="V3" s="182" t="s">
         <v>145</v>
       </c>
-      <c r="W3" s="391"/>
+      <c r="W3" s="407"/>
     </row>
     <row r="4" spans="1:23" ht="98" x14ac:dyDescent="0.2">
       <c r="A4" s="183"/>
@@ -26858,7 +26858,7 @@
       <c r="G4" s="180" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="391"/>
+      <c r="H4" s="407"/>
       <c r="I4" s="182" t="s">
         <v>107</v>
       </c>
@@ -26901,7 +26901,7 @@
       <c r="V4" s="185" t="s">
         <v>94</v>
       </c>
-      <c r="W4" s="391"/>
+      <c r="W4" s="407"/>
     </row>
     <row r="5" spans="1:23" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A5" s="186" t="s">
@@ -27607,16 +27607,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="393" t="s">
+      <c r="A1" s="409" t="s">
         <v>214</v>
       </c>
-      <c r="B1" s="393"/>
-      <c r="C1" s="393"/>
-      <c r="D1" s="393"/>
-      <c r="E1" s="393"/>
-      <c r="F1" s="393"/>
-      <c r="G1" s="393"/>
-      <c r="H1" s="393"/>
+      <c r="B1" s="409"/>
+      <c r="C1" s="409"/>
+      <c r="D1" s="409"/>
+      <c r="E1" s="409"/>
+      <c r="F1" s="409"/>
+      <c r="G1" s="409"/>
+      <c r="H1" s="409"/>
       <c r="I1" s="220"/>
       <c r="J1" s="220"/>
       <c r="K1" s="220"/>
@@ -27641,7 +27641,7 @@
       <c r="G2" s="222" t="s">
         <v>169</v>
       </c>
-      <c r="H2" s="392" t="s">
+      <c r="H2" s="408" t="s">
         <v>168</v>
       </c>
       <c r="I2" s="222" t="s">
@@ -27674,7 +27674,7 @@
       <c r="R2" s="222" t="s">
         <v>167</v>
       </c>
-      <c r="S2" s="392" t="s">
+      <c r="S2" s="408" t="s">
         <v>166</v>
       </c>
     </row>
@@ -27688,7 +27688,7 @@
       <c r="G3" s="222" t="s">
         <v>158</v>
       </c>
-      <c r="H3" s="392"/>
+      <c r="H3" s="408"/>
       <c r="I3" s="222" t="s">
         <v>210</v>
       </c>
@@ -27719,7 +27719,7 @@
       <c r="R3" s="222" t="s">
         <v>145</v>
       </c>
-      <c r="S3" s="392"/>
+      <c r="S3" s="408"/>
     </row>
     <row r="4" spans="1:21" ht="112" x14ac:dyDescent="0.2">
       <c r="A4" s="219"/>
@@ -27741,7 +27741,7 @@
       <c r="G4" s="222" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="392"/>
+      <c r="H4" s="408"/>
       <c r="I4" s="222" t="s">
         <v>191</v>
       </c>
@@ -27772,7 +27772,7 @@
       <c r="R4" s="222" t="s">
         <v>94</v>
       </c>
-      <c r="S4" s="392"/>
+      <c r="S4" s="408"/>
     </row>
     <row r="5" spans="1:21" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A5" s="225" t="s">
@@ -28403,13 +28403,13 @@
       <c r="K2" s="173" t="s">
         <v>167</v>
       </c>
-      <c r="L2" s="389" t="s">
+      <c r="L2" s="405" t="s">
         <v>166</v>
       </c>
       <c r="M2" s="173" t="s">
         <v>38</v>
       </c>
-      <c r="N2" s="389" t="s">
+      <c r="N2" s="405" t="s">
         <v>165</v>
       </c>
     </row>
@@ -28427,11 +28427,11 @@
       <c r="K3" s="173" t="s">
         <v>145</v>
       </c>
-      <c r="L3" s="389"/>
+      <c r="L3" s="405"/>
       <c r="M3" s="173" t="s">
         <v>142</v>
       </c>
-      <c r="N3" s="389"/>
+      <c r="N3" s="405"/>
     </row>
     <row r="4" spans="1:14" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="204"/>
@@ -28457,11 +28457,11 @@
       <c r="K4" s="173" t="s">
         <v>94</v>
       </c>
-      <c r="L4" s="389"/>
+      <c r="L4" s="405"/>
       <c r="M4" s="173" t="s">
         <v>93</v>
       </c>
-      <c r="N4" s="389"/>
+      <c r="N4" s="405"/>
     </row>
     <row r="5" spans="1:14" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="206"/>
@@ -29124,12 +29124,12 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" s="294"/>
-      <c r="B1" s="394" t="s">
+      <c r="B1" s="410" t="s">
         <v>295</v>
       </c>
-      <c r="C1" s="394"/>
-      <c r="D1" s="394"/>
-      <c r="E1" s="394"/>
+      <c r="C1" s="410"/>
+      <c r="D1" s="410"/>
+      <c r="E1" s="410"/>
       <c r="F1" s="295"/>
       <c r="G1" s="294"/>
       <c r="H1" s="294"/>
@@ -29180,7 +29180,7 @@
       <c r="P2" s="277" t="s">
         <v>38</v>
       </c>
-      <c r="Q2" s="376" t="s">
+      <c r="Q2" s="392" t="s">
         <v>274</v>
       </c>
     </row>
@@ -29221,7 +29221,7 @@
       <c r="P3" s="277" t="s">
         <v>281</v>
       </c>
-      <c r="Q3" s="376"/>
+      <c r="Q3" s="392"/>
     </row>
     <row r="4" spans="1:17" ht="70" x14ac:dyDescent="0.2">
       <c r="A4" s="278"/>
@@ -29270,7 +29270,7 @@
       <c r="P4" s="280" t="s">
         <v>292</v>
       </c>
-      <c r="Q4" s="376"/>
+      <c r="Q4" s="392"/>
     </row>
     <row r="5" spans="1:17" ht="398" x14ac:dyDescent="0.2">
       <c r="A5" s="281" t="s">
@@ -29725,22 +29725,22 @@
       <c r="A1" s="3"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
-      <c r="D1" s="364" t="s">
+      <c r="D1" s="380" t="s">
         <v>368</v>
       </c>
-      <c r="E1" s="365"/>
-      <c r="F1" s="365"/>
-      <c r="G1" s="365"/>
-      <c r="H1" s="365"/>
-      <c r="I1" s="365"/>
-      <c r="J1" s="366"/>
-      <c r="K1" s="366"/>
-      <c r="L1" s="366"/>
-      <c r="M1" s="366"/>
-      <c r="N1" s="366"/>
-      <c r="O1" s="366"/>
-      <c r="P1" s="366"/>
-      <c r="Q1" s="366"/>
+      <c r="E1" s="381"/>
+      <c r="F1" s="381"/>
+      <c r="G1" s="381"/>
+      <c r="H1" s="381"/>
+      <c r="I1" s="381"/>
+      <c r="J1" s="382"/>
+      <c r="K1" s="382"/>
+      <c r="L1" s="382"/>
+      <c r="M1" s="382"/>
+      <c r="N1" s="382"/>
+      <c r="O1" s="382"/>
+      <c r="P1" s="382"/>
+      <c r="Q1" s="382"/>
       <c r="R1" s="6" t="s">
         <v>263</v>
       </c>
@@ -29885,28 +29885,28 @@
       <c r="D4" s="239"/>
       <c r="E4" s="239"/>
       <c r="F4" s="239"/>
-      <c r="G4" s="367" t="s">
+      <c r="G4" s="383" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="368"/>
-      <c r="I4" s="368"/>
-      <c r="J4" s="368"/>
-      <c r="K4" s="368"/>
-      <c r="L4" s="369"/>
-      <c r="M4" s="370"/>
-      <c r="N4" s="371" t="s">
+      <c r="H4" s="384"/>
+      <c r="I4" s="384"/>
+      <c r="J4" s="384"/>
+      <c r="K4" s="384"/>
+      <c r="L4" s="385"/>
+      <c r="M4" s="386"/>
+      <c r="N4" s="387" t="s">
         <v>27</v>
       </c>
-      <c r="O4" s="369"/>
-      <c r="P4" s="369"/>
-      <c r="Q4" s="369"/>
-      <c r="R4" s="369"/>
-      <c r="S4" s="369"/>
-      <c r="T4" s="372"/>
-      <c r="U4" s="367" t="s">
+      <c r="O4" s="385"/>
+      <c r="P4" s="385"/>
+      <c r="Q4" s="385"/>
+      <c r="R4" s="385"/>
+      <c r="S4" s="385"/>
+      <c r="T4" s="388"/>
+      <c r="U4" s="383" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="370"/>
+      <c r="V4" s="386"/>
       <c r="W4" s="246"/>
       <c r="X4" t="s">
         <v>0</v>
@@ -30321,16 +30321,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:57" s="41" customFormat="1" ht="23.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B1" s="374" t="s">
+      <c r="B1" s="390" t="s">
         <v>170</v>
       </c>
-      <c r="C1" s="374"/>
-      <c r="D1" s="374"/>
-      <c r="E1" s="374"/>
-      <c r="F1" s="374"/>
-      <c r="G1" s="374"/>
-      <c r="H1" s="374"/>
-      <c r="I1" s="374"/>
+      <c r="C1" s="390"/>
+      <c r="D1" s="390"/>
+      <c r="E1" s="390"/>
+      <c r="F1" s="390"/>
+      <c r="G1" s="390"/>
+      <c r="H1" s="390"/>
+      <c r="I1" s="390"/>
     </row>
     <row r="2" spans="1:57" s="41" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="78"/>
@@ -30342,7 +30342,7 @@
       <c r="G2" s="75" t="s">
         <v>169</v>
       </c>
-      <c r="H2" s="373" t="s">
+      <c r="H2" s="389" t="s">
         <v>168</v>
       </c>
       <c r="I2" s="74" t="s">
@@ -30387,7 +30387,7 @@
       <c r="V2" s="74" t="s">
         <v>167</v>
       </c>
-      <c r="W2" s="373" t="s">
+      <c r="W2" s="389" t="s">
         <v>166</v>
       </c>
       <c r="X2" s="73" t="s">
@@ -30417,7 +30417,7 @@
       <c r="AF2" s="73" t="s">
         <v>164</v>
       </c>
-      <c r="AG2" s="373" t="s">
+      <c r="AG2" s="389" t="s">
         <v>163</v>
       </c>
       <c r="AH2" s="73" t="s">
@@ -30459,7 +30459,7 @@
       <c r="AT2" s="73" t="s">
         <v>162</v>
       </c>
-      <c r="AU2" s="373" t="s">
+      <c r="AU2" s="389" t="s">
         <v>161</v>
       </c>
       <c r="AV2" s="72" t="s">
@@ -30489,7 +30489,7 @@
       <c r="BD2" s="72" t="s">
         <v>160</v>
       </c>
-      <c r="BE2" s="373" t="s">
+      <c r="BE2" s="389" t="s">
         <v>159</v>
       </c>
     </row>
@@ -30503,7 +30503,7 @@
       <c r="G3" s="75" t="s">
         <v>158</v>
       </c>
-      <c r="H3" s="373"/>
+      <c r="H3" s="389"/>
       <c r="I3" s="74" t="s">
         <v>157</v>
       </c>
@@ -30544,7 +30544,7 @@
       <c r="V3" s="74" t="s">
         <v>145</v>
       </c>
-      <c r="W3" s="373"/>
+      <c r="W3" s="389"/>
       <c r="X3" s="73" t="s">
         <v>141</v>
       </c>
@@ -30572,7 +30572,7 @@
       <c r="AF3" s="73" t="s">
         <v>135</v>
       </c>
-      <c r="AG3" s="373"/>
+      <c r="AG3" s="389"/>
       <c r="AH3" s="73" t="s">
         <v>134</v>
       </c>
@@ -30612,7 +30612,7 @@
       <c r="AT3" s="73" t="s">
         <v>122</v>
       </c>
-      <c r="AU3" s="373"/>
+      <c r="AU3" s="389"/>
       <c r="AV3" s="72" t="s">
         <v>121</v>
       </c>
@@ -30640,7 +30640,7 @@
       <c r="BD3" s="72" t="s">
         <v>113</v>
       </c>
-      <c r="BE3" s="373"/>
+      <c r="BE3" s="389"/>
     </row>
     <row r="4" spans="1:57" s="41" customFormat="1" ht="60" x14ac:dyDescent="0.15">
       <c r="A4" s="77"/>
@@ -30662,7 +30662,7 @@
       <c r="G4" s="75" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="373"/>
+      <c r="H4" s="389"/>
       <c r="I4" s="74" t="s">
         <v>107</v>
       </c>
@@ -30705,7 +30705,7 @@
       <c r="V4" s="74" t="s">
         <v>94</v>
       </c>
-      <c r="W4" s="373"/>
+      <c r="W4" s="389"/>
       <c r="X4" s="73" t="s">
         <v>92</v>
       </c>
@@ -30733,7 +30733,7 @@
       <c r="AF4" s="73" t="s">
         <v>85</v>
       </c>
-      <c r="AG4" s="373"/>
+      <c r="AG4" s="389"/>
       <c r="AH4" s="73" t="s">
         <v>84</v>
       </c>
@@ -30773,7 +30773,7 @@
       <c r="AT4" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="AU4" s="373"/>
+      <c r="AU4" s="389"/>
       <c r="AV4" s="72" t="s">
         <v>71</v>
       </c>
@@ -30801,7 +30801,7 @@
       <c r="BD4" s="72" t="s">
         <v>63</v>
       </c>
-      <c r="BE4" s="373"/>
+      <c r="BE4" s="389"/>
     </row>
     <row r="5" spans="1:57" s="41" customFormat="1" ht="11" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="51" t="s">
@@ -33660,16 +33660,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" x14ac:dyDescent="0.2">
-      <c r="A1" s="375" t="s">
+      <c r="A1" s="391" t="s">
         <v>214</v>
       </c>
-      <c r="B1" s="375"/>
-      <c r="C1" s="375"/>
-      <c r="D1" s="375"/>
-      <c r="E1" s="375"/>
-      <c r="F1" s="375"/>
-      <c r="G1" s="375"/>
-      <c r="H1" s="375"/>
+      <c r="B1" s="391"/>
+      <c r="C1" s="391"/>
+      <c r="D1" s="391"/>
+      <c r="E1" s="391"/>
+      <c r="F1" s="391"/>
+      <c r="G1" s="391"/>
+      <c r="H1" s="391"/>
       <c r="I1" s="41"/>
       <c r="J1" s="41"/>
       <c r="K1" s="41"/>
@@ -33706,7 +33706,7 @@
       <c r="G2" s="75" t="s">
         <v>169</v>
       </c>
-      <c r="H2" s="373" t="s">
+      <c r="H2" s="389" t="s">
         <v>168</v>
       </c>
       <c r="I2" s="75" t="s">
@@ -33739,7 +33739,7 @@
       <c r="R2" s="75" t="s">
         <v>167</v>
       </c>
-      <c r="S2" s="373" t="s">
+      <c r="S2" s="389" t="s">
         <v>166</v>
       </c>
       <c r="T2" s="75" t="s">
@@ -33769,7 +33769,7 @@
       <c r="AB2" s="75" t="s">
         <v>164</v>
       </c>
-      <c r="AC2" s="373" t="s">
+      <c r="AC2" s="389" t="s">
         <v>213</v>
       </c>
       <c r="AD2" s="75" t="s">
@@ -33781,7 +33781,7 @@
       <c r="AF2" s="75" t="s">
         <v>212</v>
       </c>
-      <c r="AG2" s="373" t="s">
+      <c r="AG2" s="389" t="s">
         <v>211</v>
       </c>
     </row>
@@ -33795,7 +33795,7 @@
       <c r="G3" s="75" t="s">
         <v>158</v>
       </c>
-      <c r="H3" s="373"/>
+      <c r="H3" s="389"/>
       <c r="I3" s="75" t="s">
         <v>210</v>
       </c>
@@ -33826,7 +33826,7 @@
       <c r="R3" s="75" t="s">
         <v>145</v>
       </c>
-      <c r="S3" s="373"/>
+      <c r="S3" s="389"/>
       <c r="T3" s="75" t="s">
         <v>201</v>
       </c>
@@ -33854,7 +33854,7 @@
       <c r="AB3" s="75" t="s">
         <v>193</v>
       </c>
-      <c r="AC3" s="373"/>
+      <c r="AC3" s="389"/>
       <c r="AD3" s="75" t="s">
         <v>192</v>
       </c>
@@ -33864,7 +33864,7 @@
       <c r="AF3" s="75" t="s">
         <v>122</v>
       </c>
-      <c r="AG3" s="373"/>
+      <c r="AG3" s="389"/>
     </row>
     <row r="4" spans="1:33" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="78"/>
@@ -33886,7 +33886,7 @@
       <c r="G4" s="75" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="373"/>
+      <c r="H4" s="389"/>
       <c r="I4" s="75" t="s">
         <v>191</v>
       </c>
@@ -33917,7 +33917,7 @@
       <c r="R4" s="75" t="s">
         <v>94</v>
       </c>
-      <c r="S4" s="373"/>
+      <c r="S4" s="389"/>
       <c r="T4" s="75" t="s">
         <v>182</v>
       </c>
@@ -33945,7 +33945,7 @@
       <c r="AB4" s="75" t="s">
         <v>174</v>
       </c>
-      <c r="AC4" s="373"/>
+      <c r="AC4" s="389"/>
       <c r="AD4" s="75" t="s">
         <v>173</v>
       </c>
@@ -33955,7 +33955,7 @@
       <c r="AF4" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="AG4" s="373"/>
+      <c r="AG4" s="389"/>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A5" s="81" t="s">
@@ -35325,13 +35325,13 @@
       <c r="G2" s="75" t="s">
         <v>167</v>
       </c>
-      <c r="H2" s="373" t="s">
+      <c r="H2" s="389" t="s">
         <v>166</v>
       </c>
       <c r="I2" s="75" t="s">
         <v>38</v>
       </c>
-      <c r="J2" s="373" t="s">
+      <c r="J2" s="389" t="s">
         <v>165</v>
       </c>
     </row>
@@ -35345,11 +35345,11 @@
       <c r="G3" s="75" t="s">
         <v>145</v>
       </c>
-      <c r="H3" s="373"/>
+      <c r="H3" s="389"/>
       <c r="I3" s="75" t="s">
         <v>142</v>
       </c>
-      <c r="J3" s="373"/>
+      <c r="J3" s="389"/>
     </row>
     <row r="4" spans="1:10" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="97"/>
@@ -35371,11 +35371,11 @@
       <c r="G4" s="75" t="s">
         <v>94</v>
       </c>
-      <c r="H4" s="373"/>
+      <c r="H4" s="389"/>
       <c r="I4" s="75" t="s">
         <v>93</v>
       </c>
-      <c r="J4" s="373"/>
+      <c r="J4" s="389"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="91" t="s">
@@ -35796,7 +35796,7 @@
       <c r="P2" s="277" t="s">
         <v>38</v>
       </c>
-      <c r="Q2" s="376" t="s">
+      <c r="Q2" s="392" t="s">
         <v>274</v>
       </c>
     </row>
@@ -35837,7 +35837,7 @@
       <c r="P3" s="277" t="s">
         <v>281</v>
       </c>
-      <c r="Q3" s="376"/>
+      <c r="Q3" s="392"/>
     </row>
     <row r="4" spans="1:62" ht="70" x14ac:dyDescent="0.2">
       <c r="A4" s="278"/>
@@ -35886,7 +35886,7 @@
       <c r="P4" s="280" t="s">
         <v>292</v>
       </c>
-      <c r="Q4" s="376"/>
+      <c r="Q4" s="392"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="281" t="s">

</xml_diff>

<commit_message>
fix cph multifactor formulas extractors
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3164879A-4450-2D4C-ACDA-E91C3253F07B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1408546-923B-464B-9BAC-DB85FD1D9A2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -15900,6 +15900,52 @@
     <xf numFmtId="0" fontId="24" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="24" fillId="10" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="30" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="30" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="0" xfId="4" applyFont="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="35" fillId="8" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="24" fillId="10" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="8" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="85" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="40" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -16058,52 +16104,6 @@
     <xf numFmtId="49" fontId="32" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="25" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="10" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="30" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="30" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="85" fillId="0" borderId="0" xfId="4" applyFont="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="35" fillId="8" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="10" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="25" fillId="8" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="85" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma 2" xfId="2" xr:uid="{C877C5E8-FCBF-114F-9ECB-F75EF7C9C0EB}"/>
@@ -17165,11 +17165,11 @@
       <c r="B1" s="115" t="s">
         <v>220</v>
       </c>
-      <c r="C1" s="360" t="s">
+      <c r="C1" s="376" t="s">
         <v>221</v>
       </c>
-      <c r="D1" s="360"/>
-      <c r="E1" s="360"/>
+      <c r="D1" s="376"/>
+      <c r="E1" s="376"/>
       <c r="F1" s="116"/>
       <c r="H1" s="26" t="s">
         <v>0</v>
@@ -17178,11 +17178,11 @@
     <row r="2" spans="1:8" s="120" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="117"/>
       <c r="B2" s="118"/>
-      <c r="C2" s="361" t="s">
+      <c r="C2" s="377" t="s">
         <v>222</v>
       </c>
-      <c r="D2" s="361"/>
-      <c r="E2" s="361"/>
+      <c r="D2" s="377"/>
+      <c r="E2" s="377"/>
       <c r="F2" s="119"/>
       <c r="H2" s="26" t="s">
         <v>0</v>
@@ -17206,10 +17206,10 @@
       <c r="D4" s="125" t="s">
         <v>225</v>
       </c>
-      <c r="E4" s="365" t="s">
+      <c r="E4" s="381" t="s">
         <v>226</v>
       </c>
-      <c r="F4" s="366"/>
+      <c r="F4" s="382"/>
       <c r="G4" s="134"/>
       <c r="H4" s="26" t="s">
         <v>0</v>
@@ -17226,10 +17226,10 @@
       <c r="D5" s="131" t="s">
         <v>229</v>
       </c>
-      <c r="E5" s="367" t="s">
+      <c r="E5" s="383" t="s">
         <v>242</v>
       </c>
-      <c r="F5" s="368"/>
+      <c r="F5" s="384"/>
       <c r="G5" s="133"/>
       <c r="H5" s="26" t="s">
         <v>0</v>
@@ -17246,10 +17246,10 @@
       <c r="D6" s="132" t="s">
         <v>232</v>
       </c>
-      <c r="E6" s="369" t="s">
+      <c r="E6" s="385" t="s">
         <v>243</v>
       </c>
-      <c r="F6" s="370"/>
+      <c r="F6" s="386"/>
       <c r="G6" s="133"/>
       <c r="H6" s="26" t="s">
         <v>0</v>
@@ -17266,10 +17266,10 @@
       <c r="D7" s="132" t="s">
         <v>235</v>
       </c>
-      <c r="E7" s="369" t="s">
+      <c r="E7" s="385" t="s">
         <v>242</v>
       </c>
-      <c r="F7" s="370"/>
+      <c r="F7" s="386"/>
       <c r="G7" s="133"/>
       <c r="H7" s="26" t="s">
         <v>0</v>
@@ -17280,16 +17280,16 @@
       <c r="B8" s="138" t="s">
         <v>236</v>
       </c>
-      <c r="C8" s="371" t="s">
+      <c r="C8" s="387" t="s">
         <v>237</v>
       </c>
-      <c r="D8" s="371" t="s">
+      <c r="D8" s="387" t="s">
         <v>238</v>
       </c>
-      <c r="E8" s="374" t="s">
+      <c r="E8" s="390" t="s">
         <v>244</v>
       </c>
-      <c r="F8" s="374"/>
+      <c r="F8" s="390"/>
       <c r="G8" s="133"/>
       <c r="H8" s="26" t="s">
         <v>0</v>
@@ -17300,10 +17300,10 @@
       <c r="B9" s="304" t="s">
         <v>239</v>
       </c>
-      <c r="C9" s="372"/>
-      <c r="D9" s="372"/>
-      <c r="E9" s="375"/>
-      <c r="F9" s="375"/>
+      <c r="C9" s="388"/>
+      <c r="D9" s="388"/>
+      <c r="E9" s="391"/>
+      <c r="F9" s="391"/>
       <c r="G9" s="133"/>
       <c r="H9" s="26" t="s">
         <v>0</v>
@@ -17314,10 +17314,10 @@
       <c r="B10" s="305" t="s">
         <v>240</v>
       </c>
-      <c r="C10" s="372"/>
-      <c r="D10" s="372"/>
-      <c r="E10" s="375"/>
-      <c r="F10" s="375"/>
+      <c r="C10" s="388"/>
+      <c r="D10" s="388"/>
+      <c r="E10" s="391"/>
+      <c r="F10" s="391"/>
       <c r="G10" s="133"/>
       <c r="H10" s="26" t="s">
         <v>0</v>
@@ -17328,10 +17328,10 @@
       <c r="B11" s="300" t="s">
         <v>364</v>
       </c>
-      <c r="C11" s="373"/>
-      <c r="D11" s="373"/>
-      <c r="E11" s="376"/>
-      <c r="F11" s="376"/>
+      <c r="C11" s="389"/>
+      <c r="D11" s="389"/>
+      <c r="E11" s="392"/>
+      <c r="F11" s="392"/>
       <c r="G11" s="133"/>
       <c r="H11" s="26" t="s">
         <v>0</v>
@@ -17351,11 +17351,11 @@
     <row r="13" spans="1:8" s="26" customFormat="1" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="121"/>
       <c r="B13" s="302"/>
-      <c r="C13" s="364" t="s">
+      <c r="C13" s="380" t="s">
         <v>241</v>
       </c>
-      <c r="D13" s="364"/>
-      <c r="E13" s="364"/>
+      <c r="D13" s="380"/>
+      <c r="E13" s="380"/>
       <c r="F13" s="303"/>
       <c r="H13" s="26" t="s">
         <v>0</v>
@@ -17369,14 +17369,14 @@
       </c>
     </row>
     <row r="15" spans="1:8" s="26" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="362" t="s">
+      <c r="A15" s="378" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="362"/>
-      <c r="C15" s="362"/>
-      <c r="D15" s="362"/>
-      <c r="E15" s="362"/>
-      <c r="F15" s="363"/>
+      <c r="B15" s="378"/>
+      <c r="C15" s="378"/>
+      <c r="D15" s="378"/>
+      <c r="E15" s="378"/>
+      <c r="F15" s="379"/>
       <c r="H15" s="26" t="s">
         <v>0</v>
       </c>
@@ -17506,7 +17506,7 @@
       <c r="G2" s="75" t="s">
         <v>169</v>
       </c>
-      <c r="H2" s="386" t="s">
+      <c r="H2" s="402" t="s">
         <v>168</v>
       </c>
       <c r="I2" s="74" t="s">
@@ -17551,7 +17551,7 @@
       <c r="V2" s="74" t="s">
         <v>167</v>
       </c>
-      <c r="W2" s="386" t="s">
+      <c r="W2" s="402" t="s">
         <v>166</v>
       </c>
       <c r="X2" s="73" t="s">
@@ -17581,7 +17581,7 @@
       <c r="AF2" s="73" t="s">
         <v>164</v>
       </c>
-      <c r="AG2" s="386" t="s">
+      <c r="AG2" s="402" t="s">
         <v>163</v>
       </c>
       <c r="AH2" s="73" t="s">
@@ -17623,7 +17623,7 @@
       <c r="AT2" s="73" t="s">
         <v>162</v>
       </c>
-      <c r="AU2" s="386" t="s">
+      <c r="AU2" s="402" t="s">
         <v>161</v>
       </c>
       <c r="AV2" s="72" t="s">
@@ -17653,7 +17653,7 @@
       <c r="BD2" s="72" t="s">
         <v>160</v>
       </c>
-      <c r="BE2" s="386" t="s">
+      <c r="BE2" s="402" t="s">
         <v>159</v>
       </c>
       <c r="BF2"/>
@@ -17668,7 +17668,7 @@
       <c r="G3" s="75" t="s">
         <v>158</v>
       </c>
-      <c r="H3" s="386"/>
+      <c r="H3" s="402"/>
       <c r="I3" s="74" t="s">
         <v>157</v>
       </c>
@@ -17709,7 +17709,7 @@
       <c r="V3" s="74" t="s">
         <v>145</v>
       </c>
-      <c r="W3" s="386"/>
+      <c r="W3" s="402"/>
       <c r="X3" s="73" t="s">
         <v>141</v>
       </c>
@@ -17737,7 +17737,7 @@
       <c r="AF3" s="73" t="s">
         <v>135</v>
       </c>
-      <c r="AG3" s="386"/>
+      <c r="AG3" s="402"/>
       <c r="AH3" s="73" t="s">
         <v>134</v>
       </c>
@@ -17777,7 +17777,7 @@
       <c r="AT3" s="73" t="s">
         <v>122</v>
       </c>
-      <c r="AU3" s="386"/>
+      <c r="AU3" s="402"/>
       <c r="AV3" s="72" t="s">
         <v>121</v>
       </c>
@@ -17805,7 +17805,7 @@
       <c r="BD3" s="72" t="s">
         <v>113</v>
       </c>
-      <c r="BE3" s="386"/>
+      <c r="BE3" s="402"/>
     </row>
     <row r="4" spans="1:58" s="41" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="77"/>
@@ -17827,7 +17827,7 @@
       <c r="G4" s="75" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="386"/>
+      <c r="H4" s="402"/>
       <c r="I4" s="74" t="s">
         <v>107</v>
       </c>
@@ -17870,7 +17870,7 @@
       <c r="V4" s="74" t="s">
         <v>94</v>
       </c>
-      <c r="W4" s="386"/>
+      <c r="W4" s="402"/>
       <c r="X4" s="73" t="s">
         <v>92</v>
       </c>
@@ -17898,7 +17898,7 @@
       <c r="AF4" s="73" t="s">
         <v>85</v>
       </c>
-      <c r="AG4" s="386"/>
+      <c r="AG4" s="402"/>
       <c r="AH4" s="73" t="s">
         <v>608</v>
       </c>
@@ -17938,7 +17938,7 @@
       <c r="AT4" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="AU4" s="386"/>
+      <c r="AU4" s="402"/>
       <c r="AV4" s="72" t="s">
         <v>71</v>
       </c>
@@ -17966,7 +17966,7 @@
       <c r="BD4" s="72" t="s">
         <v>63</v>
       </c>
-      <c r="BE4" s="386"/>
+      <c r="BE4" s="402"/>
       <c r="BF4"/>
     </row>
     <row r="5" spans="1:58" s="41" customFormat="1" ht="15" x14ac:dyDescent="0.2">
@@ -20561,28 +20561,28 @@
       <c r="E21" s="39"/>
     </row>
     <row r="22" spans="4:57" ht="69" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E22" s="390" t="s">
+      <c r="E22" s="406" t="s">
         <v>367</v>
       </c>
-      <c r="F22" s="391"/>
-      <c r="G22" s="391"/>
-      <c r="H22" s="391"/>
-      <c r="I22" s="391"/>
-      <c r="J22" s="391"/>
-      <c r="K22" s="391"/>
-      <c r="L22" s="391"/>
-      <c r="M22" s="391"/>
-      <c r="N22" s="391"/>
-      <c r="O22" s="391"/>
-      <c r="P22" s="391"/>
-      <c r="Q22" s="391"/>
-      <c r="R22" s="391"/>
-      <c r="S22" s="391"/>
-      <c r="T22" s="391"/>
-      <c r="U22" s="391"/>
-      <c r="V22" s="391"/>
-      <c r="W22" s="391"/>
-      <c r="X22" s="392"/>
+      <c r="F22" s="407"/>
+      <c r="G22" s="407"/>
+      <c r="H22" s="407"/>
+      <c r="I22" s="407"/>
+      <c r="J22" s="407"/>
+      <c r="K22" s="407"/>
+      <c r="L22" s="407"/>
+      <c r="M22" s="407"/>
+      <c r="N22" s="407"/>
+      <c r="O22" s="407"/>
+      <c r="P22" s="407"/>
+      <c r="Q22" s="407"/>
+      <c r="R22" s="407"/>
+      <c r="S22" s="407"/>
+      <c r="T22" s="407"/>
+      <c r="U22" s="407"/>
+      <c r="V22" s="407"/>
+      <c r="W22" s="407"/>
+      <c r="X22" s="408"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -20686,82 +20686,82 @@
       <c r="D2" s="347"/>
       <c r="E2" s="347"/>
       <c r="F2" s="347"/>
-      <c r="G2" s="408" t="s">
+      <c r="G2" s="360" t="s">
         <v>108</v>
       </c>
       <c r="H2" s="359" t="s">
         <v>168</v>
       </c>
-      <c r="I2" s="408" t="s">
+      <c r="I2" s="360" t="s">
         <v>191</v>
       </c>
-      <c r="J2" s="408" t="s">
+      <c r="J2" s="360" t="s">
         <v>190</v>
       </c>
-      <c r="K2" s="408" t="s">
+      <c r="K2" s="360" t="s">
         <v>189</v>
       </c>
-      <c r="L2" s="408" t="s">
+      <c r="L2" s="360" t="s">
         <v>188</v>
       </c>
-      <c r="M2" s="408" t="s">
+      <c r="M2" s="360" t="s">
         <v>187</v>
       </c>
-      <c r="N2" s="408" t="s">
+      <c r="N2" s="360" t="s">
         <v>186</v>
       </c>
-      <c r="O2" s="408" t="s">
+      <c r="O2" s="360" t="s">
         <v>185</v>
       </c>
-      <c r="P2" s="408" t="s">
+      <c r="P2" s="360" t="s">
         <v>184</v>
       </c>
-      <c r="Q2" s="408" t="s">
+      <c r="Q2" s="360" t="s">
         <v>183</v>
       </c>
-      <c r="R2" s="408" t="s">
+      <c r="R2" s="360" t="s">
         <v>624</v>
       </c>
       <c r="S2" s="359" t="s">
         <v>166</v>
       </c>
-      <c r="T2" s="408" t="s">
+      <c r="T2" s="360" t="s">
         <v>182</v>
       </c>
-      <c r="U2" s="408" t="s">
+      <c r="U2" s="360" t="s">
         <v>181</v>
       </c>
-      <c r="V2" s="408" t="s">
+      <c r="V2" s="360" t="s">
         <v>625</v>
       </c>
-      <c r="W2" s="408" t="s">
+      <c r="W2" s="360" t="s">
         <v>179</v>
       </c>
-      <c r="X2" s="408" t="s">
+      <c r="X2" s="360" t="s">
         <v>178</v>
       </c>
-      <c r="Y2" s="408" t="s">
+      <c r="Y2" s="360" t="s">
         <v>177</v>
       </c>
-      <c r="Z2" s="408" t="s">
+      <c r="Z2" s="360" t="s">
         <v>176</v>
       </c>
-      <c r="AA2" s="408" t="s">
+      <c r="AA2" s="360" t="s">
         <v>175</v>
       </c>
-      <c r="AB2" s="408" t="s">
+      <c r="AB2" s="360" t="s">
         <v>174</v>
       </c>
       <c r="AC2" s="359" t="s">
         <v>213</v>
       </c>
-      <c r="AD2" s="408" t="s">
+      <c r="AD2" s="360" t="s">
         <v>613</v>
       </c>
-      <c r="AE2" s="408" t="s">
+      <c r="AE2" s="360" t="s">
         <v>78</v>
       </c>
-      <c r="AF2" s="408" t="s">
+      <c r="AF2" s="360" t="s">
         <v>72</v>
       </c>
       <c r="AG2" s="359" t="s">
@@ -20775,82 +20775,82 @@
       <c r="D3" s="347"/>
       <c r="E3" s="347"/>
       <c r="F3" s="347"/>
-      <c r="G3" s="408" t="s">
+      <c r="G3" s="360" t="s">
         <v>108</v>
       </c>
       <c r="H3" s="359" t="s">
         <v>168</v>
       </c>
-      <c r="I3" s="408" t="s">
+      <c r="I3" s="360" t="s">
         <v>191</v>
       </c>
-      <c r="J3" s="408" t="s">
+      <c r="J3" s="360" t="s">
         <v>190</v>
       </c>
-      <c r="K3" s="408" t="s">
+      <c r="K3" s="360" t="s">
         <v>189</v>
       </c>
-      <c r="L3" s="408" t="s">
+      <c r="L3" s="360" t="s">
         <v>188</v>
       </c>
-      <c r="M3" s="408" t="s">
+      <c r="M3" s="360" t="s">
         <v>187</v>
       </c>
-      <c r="N3" s="408" t="s">
+      <c r="N3" s="360" t="s">
         <v>186</v>
       </c>
-      <c r="O3" s="408" t="s">
+      <c r="O3" s="360" t="s">
         <v>185</v>
       </c>
-      <c r="P3" s="408" t="s">
+      <c r="P3" s="360" t="s">
         <v>184</v>
       </c>
-      <c r="Q3" s="408" t="s">
+      <c r="Q3" s="360" t="s">
         <v>183</v>
       </c>
-      <c r="R3" s="408" t="s">
+      <c r="R3" s="360" t="s">
         <v>624</v>
       </c>
       <c r="S3" s="359" t="s">
         <v>166</v>
       </c>
-      <c r="T3" s="408" t="s">
+      <c r="T3" s="360" t="s">
         <v>182</v>
       </c>
-      <c r="U3" s="408" t="s">
+      <c r="U3" s="360" t="s">
         <v>181</v>
       </c>
-      <c r="V3" s="408" t="s">
+      <c r="V3" s="360" t="s">
         <v>625</v>
       </c>
-      <c r="W3" s="408" t="s">
+      <c r="W3" s="360" t="s">
         <v>179</v>
       </c>
-      <c r="X3" s="408" t="s">
+      <c r="X3" s="360" t="s">
         <v>178</v>
       </c>
-      <c r="Y3" s="408" t="s">
+      <c r="Y3" s="360" t="s">
         <v>177</v>
       </c>
-      <c r="Z3" s="408" t="s">
+      <c r="Z3" s="360" t="s">
         <v>176</v>
       </c>
-      <c r="AA3" s="408" t="s">
+      <c r="AA3" s="360" t="s">
         <v>175</v>
       </c>
-      <c r="AB3" s="408" t="s">
+      <c r="AB3" s="360" t="s">
         <v>174</v>
       </c>
       <c r="AC3" s="359" t="s">
         <v>213</v>
       </c>
-      <c r="AD3" s="408" t="s">
+      <c r="AD3" s="360" t="s">
         <v>613</v>
       </c>
-      <c r="AE3" s="408" t="s">
+      <c r="AE3" s="360" t="s">
         <v>78</v>
       </c>
-      <c r="AF3" s="408" t="s">
+      <c r="AF3" s="360" t="s">
         <v>72</v>
       </c>
       <c r="AG3" s="359" t="s">
@@ -20874,82 +20874,82 @@
       <c r="F4" s="76" t="s">
         <v>109</v>
       </c>
-      <c r="G4" s="408" t="s">
+      <c r="G4" s="360" t="s">
         <v>108</v>
       </c>
       <c r="H4" s="359" t="s">
         <v>168</v>
       </c>
-      <c r="I4" s="408" t="s">
+      <c r="I4" s="360" t="s">
         <v>191</v>
       </c>
-      <c r="J4" s="408" t="s">
+      <c r="J4" s="360" t="s">
         <v>190</v>
       </c>
-      <c r="K4" s="408" t="s">
+      <c r="K4" s="360" t="s">
         <v>189</v>
       </c>
-      <c r="L4" s="408" t="s">
+      <c r="L4" s="360" t="s">
         <v>188</v>
       </c>
-      <c r="M4" s="408" t="s">
+      <c r="M4" s="360" t="s">
         <v>187</v>
       </c>
-      <c r="N4" s="408" t="s">
+      <c r="N4" s="360" t="s">
         <v>186</v>
       </c>
-      <c r="O4" s="408" t="s">
+      <c r="O4" s="360" t="s">
         <v>185</v>
       </c>
-      <c r="P4" s="408" t="s">
+      <c r="P4" s="360" t="s">
         <v>184</v>
       </c>
-      <c r="Q4" s="408" t="s">
+      <c r="Q4" s="360" t="s">
         <v>183</v>
       </c>
-      <c r="R4" s="408" t="s">
+      <c r="R4" s="360" t="s">
         <v>624</v>
       </c>
       <c r="S4" s="359" t="s">
         <v>166</v>
       </c>
-      <c r="T4" s="408" t="s">
+      <c r="T4" s="360" t="s">
         <v>182</v>
       </c>
-      <c r="U4" s="408" t="s">
+      <c r="U4" s="360" t="s">
         <v>181</v>
       </c>
-      <c r="V4" s="408" t="s">
+      <c r="V4" s="360" t="s">
         <v>625</v>
       </c>
-      <c r="W4" s="408" t="s">
+      <c r="W4" s="360" t="s">
         <v>179</v>
       </c>
-      <c r="X4" s="408" t="s">
+      <c r="X4" s="360" t="s">
         <v>178</v>
       </c>
-      <c r="Y4" s="408" t="s">
+      <c r="Y4" s="360" t="s">
         <v>177</v>
       </c>
-      <c r="Z4" s="408" t="s">
+      <c r="Z4" s="360" t="s">
         <v>176</v>
       </c>
-      <c r="AA4" s="408" t="s">
+      <c r="AA4" s="360" t="s">
         <v>175</v>
       </c>
-      <c r="AB4" s="408" t="s">
+      <c r="AB4" s="360" t="s">
         <v>174</v>
       </c>
       <c r="AC4" s="359" t="s">
         <v>213</v>
       </c>
-      <c r="AD4" s="408" t="s">
+      <c r="AD4" s="360" t="s">
         <v>613</v>
       </c>
-      <c r="AE4" s="408" t="s">
+      <c r="AE4" s="360" t="s">
         <v>78</v>
       </c>
-      <c r="AF4" s="408" t="s">
+      <c r="AF4" s="360" t="s">
         <v>72</v>
       </c>
       <c r="AG4" s="359" t="s">
@@ -20966,7 +20966,7 @@
       <c r="E5" s="61" t="s">
         <v>62</v>
       </c>
-      <c r="F5" s="411" t="s">
+      <c r="F5" s="363" t="s">
         <v>61</v>
       </c>
       <c r="G5" s="106" t="str">
@@ -21091,7 +21091,7 @@
       <c r="E6" s="61" t="s">
         <v>60</v>
       </c>
-      <c r="F6" s="411" t="s">
+      <c r="F6" s="363" t="s">
         <v>59</v>
       </c>
       <c r="G6" s="106" t="str">
@@ -21216,7 +21216,7 @@
       <c r="E7" s="61" t="s">
         <v>58</v>
       </c>
-      <c r="F7" s="411" t="s">
+      <c r="F7" s="363" t="s">
         <v>57</v>
       </c>
       <c r="G7" s="106" t="str">
@@ -21341,7 +21341,7 @@
       <c r="E8" s="61" t="s">
         <v>56</v>
       </c>
-      <c r="F8" s="411" t="s">
+      <c r="F8" s="363" t="s">
         <v>55</v>
       </c>
       <c r="G8" s="106" t="str">
@@ -21466,7 +21466,7 @@
       <c r="E9" s="61" t="s">
         <v>54</v>
       </c>
-      <c r="F9" s="411" t="s">
+      <c r="F9" s="363" t="s">
         <v>53</v>
       </c>
       <c r="G9" s="106" t="str">
@@ -21591,7 +21591,7 @@
       <c r="E10" s="61" t="s">
         <v>52</v>
       </c>
-      <c r="F10" s="411" t="s">
+      <c r="F10" s="363" t="s">
         <v>51</v>
       </c>
       <c r="G10" s="106" t="str">
@@ -21716,7 +21716,7 @@
       <c r="E11" s="61" t="s">
         <v>50</v>
       </c>
-      <c r="F11" s="411" t="s">
+      <c r="F11" s="363" t="s">
         <v>49</v>
       </c>
       <c r="G11" s="106" t="str">
@@ -21841,7 +21841,7 @@
       <c r="E12" s="61" t="s">
         <v>48</v>
       </c>
-      <c r="F12" s="411" t="s">
+      <c r="F12" s="363" t="s">
         <v>47</v>
       </c>
       <c r="G12" s="106" t="str">
@@ -21966,7 +21966,7 @@
       <c r="E13" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="F13" s="411" t="s">
+      <c r="F13" s="363" t="s">
         <v>45</v>
       </c>
       <c r="G13" s="106" t="str">
@@ -22091,7 +22091,7 @@
       <c r="E14" s="61" t="s">
         <v>44</v>
       </c>
-      <c r="F14" s="411" t="s">
+      <c r="F14" s="363" t="s">
         <v>43</v>
       </c>
       <c r="G14" s="106" t="str">
@@ -22216,7 +22216,7 @@
       <c r="E15" s="61" t="s">
         <v>41</v>
       </c>
-      <c r="F15" s="411" t="s">
+      <c r="F15" s="363" t="s">
         <v>40</v>
       </c>
       <c r="G15" s="106" t="str">
@@ -22334,7 +22334,7 @@
       <c r="C16" s="80"/>
       <c r="D16" s="80"/>
       <c r="E16" s="80"/>
-      <c r="F16" s="412" t="s">
+      <c r="F16" s="364" t="s">
         <v>39</v>
       </c>
       <c r="G16" s="46">
@@ -22537,32 +22537,32 @@
       <c r="K20" s="140"/>
     </row>
     <row r="21" spans="4:33" ht="50" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E21" s="393" t="s">
+      <c r="E21" s="409" t="s">
         <v>368</v>
       </c>
-      <c r="F21" s="394"/>
-      <c r="G21" s="394"/>
-      <c r="H21" s="394"/>
-      <c r="I21" s="394"/>
-      <c r="J21" s="394"/>
-      <c r="K21" s="394"/>
-      <c r="L21" s="394"/>
-      <c r="M21" s="394"/>
-      <c r="N21" s="394"/>
-      <c r="O21" s="394"/>
-      <c r="P21" s="394"/>
-      <c r="Q21" s="394"/>
-      <c r="R21" s="394"/>
-      <c r="S21" s="394"/>
-      <c r="T21" s="394"/>
-      <c r="U21" s="394"/>
-      <c r="V21" s="394"/>
-      <c r="W21" s="394"/>
-      <c r="X21" s="394"/>
-      <c r="Y21" s="394"/>
-      <c r="Z21" s="394"/>
-      <c r="AA21" s="394"/>
-      <c r="AB21" s="395"/>
+      <c r="F21" s="410"/>
+      <c r="G21" s="410"/>
+      <c r="H21" s="410"/>
+      <c r="I21" s="410"/>
+      <c r="J21" s="410"/>
+      <c r="K21" s="410"/>
+      <c r="L21" s="410"/>
+      <c r="M21" s="410"/>
+      <c r="N21" s="410"/>
+      <c r="O21" s="410"/>
+      <c r="P21" s="410"/>
+      <c r="Q21" s="410"/>
+      <c r="R21" s="410"/>
+      <c r="S21" s="410"/>
+      <c r="T21" s="410"/>
+      <c r="U21" s="410"/>
+      <c r="V21" s="410"/>
+      <c r="W21" s="410"/>
+      <c r="X21" s="410"/>
+      <c r="Y21" s="410"/>
+      <c r="Z21" s="410"/>
+      <c r="AA21" s="410"/>
+      <c r="AB21" s="411"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -22658,33 +22658,33 @@
       <c r="BJ1" s="37"/>
     </row>
     <row r="2" spans="1:62" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="416"/>
-      <c r="B2" s="416"/>
-      <c r="C2" s="416"/>
-      <c r="D2" s="416"/>
-      <c r="E2" s="416"/>
-      <c r="F2" s="416"/>
+      <c r="A2" s="368"/>
+      <c r="B2" s="368"/>
+      <c r="C2" s="368"/>
+      <c r="D2" s="368"/>
+      <c r="E2" s="368"/>
+      <c r="F2" s="368"/>
       <c r="G2" s="75" t="s">
         <v>167</v>
       </c>
-      <c r="H2" s="386" t="s">
+      <c r="H2" s="402" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="3" spans="1:62" ht="36" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="416"/>
-      <c r="B3" s="416"/>
-      <c r="C3" s="416"/>
-      <c r="D3" s="416"/>
-      <c r="E3" s="416"/>
-      <c r="F3" s="416"/>
+      <c r="A3" s="368"/>
+      <c r="B3" s="368"/>
+      <c r="C3" s="368"/>
+      <c r="D3" s="368"/>
+      <c r="E3" s="368"/>
+      <c r="F3" s="368"/>
       <c r="G3" s="75" t="s">
         <v>145</v>
       </c>
-      <c r="H3" s="386"/>
+      <c r="H3" s="402"/>
     </row>
     <row r="4" spans="1:62" ht="36" x14ac:dyDescent="0.2">
-      <c r="A4" s="417"/>
+      <c r="A4" s="369"/>
       <c r="B4" s="96" t="s">
         <v>112</v>
       </c>
@@ -22703,7 +22703,7 @@
       <c r="G4" s="75" t="s">
         <v>94</v>
       </c>
-      <c r="H4" s="386"/>
+      <c r="H4" s="402"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="91" t="s">
@@ -22715,7 +22715,7 @@
       <c r="E5" s="90" t="s">
         <v>62</v>
       </c>
-      <c r="F5" s="409" t="s">
+      <c r="F5" s="361" t="s">
         <v>61</v>
       </c>
       <c r="G5" s="105" t="str">
@@ -22740,7 +22740,7 @@
       <c r="E6" s="90" t="s">
         <v>56</v>
       </c>
-      <c r="F6" s="409" t="s">
+      <c r="F6" s="361" t="s">
         <v>55</v>
       </c>
       <c r="G6" s="105" t="str">
@@ -22765,7 +22765,7 @@
       <c r="E7" s="90" t="s">
         <v>54</v>
       </c>
-      <c r="F7" s="409" t="s">
+      <c r="F7" s="361" t="s">
         <v>53</v>
       </c>
       <c r="G7" s="105" t="str">
@@ -22790,7 +22790,7 @@
       <c r="E8" s="90" t="s">
         <v>52</v>
       </c>
-      <c r="F8" s="409" t="s">
+      <c r="F8" s="361" t="s">
         <v>51</v>
       </c>
       <c r="G8" s="105" t="str">
@@ -22815,7 +22815,7 @@
       <c r="E9" s="90" t="s">
         <v>50</v>
       </c>
-      <c r="F9" s="409" t="s">
+      <c r="F9" s="361" t="s">
         <v>49</v>
       </c>
       <c r="G9" s="105" t="str">
@@ -22840,7 +22840,7 @@
       <c r="E10" s="90" t="s">
         <v>48</v>
       </c>
-      <c r="F10" s="409" t="s">
+      <c r="F10" s="361" t="s">
         <v>47</v>
       </c>
       <c r="G10" s="105" t="str">
@@ -22865,7 +22865,7 @@
       <c r="E11" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="F11" s="409" t="s">
+      <c r="F11" s="361" t="s">
         <v>45</v>
       </c>
       <c r="G11" s="105" t="str">
@@ -22890,7 +22890,7 @@
       <c r="E12" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="F12" s="409" t="s">
+      <c r="F12" s="361" t="s">
         <v>43</v>
       </c>
       <c r="G12" s="105" t="str">
@@ -22915,7 +22915,7 @@
       <c r="E13" s="90" t="s">
         <v>41</v>
       </c>
-      <c r="F13" s="409" t="s">
+      <c r="F13" s="361" t="s">
         <v>40</v>
       </c>
       <c r="G13" s="105" t="str">
@@ -22928,12 +22928,12 @@
       </c>
     </row>
     <row r="14" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="A14" s="418"/>
+      <c r="A14" s="370"/>
       <c r="B14" s="61"/>
       <c r="C14" s="61"/>
       <c r="D14" s="61"/>
       <c r="E14" s="80"/>
-      <c r="F14" s="410" t="s">
+      <c r="F14" s="362" t="s">
         <v>39</v>
       </c>
       <c r="G14" s="84">
@@ -22957,15 +22957,15 @@
       <c r="J16" s="21"/>
     </row>
     <row r="17" spans="4:10" ht="99" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D17" s="396" t="s">
+      <c r="D17" s="412" t="s">
         <v>369</v>
       </c>
-      <c r="E17" s="397"/>
-      <c r="F17" s="397"/>
-      <c r="G17" s="397"/>
-      <c r="H17" s="397"/>
-      <c r="I17" s="397"/>
-      <c r="J17" s="398"/>
+      <c r="E17" s="413"/>
+      <c r="F17" s="413"/>
+      <c r="G17" s="413"/>
+      <c r="H17" s="413"/>
+      <c r="I17" s="413"/>
+      <c r="J17" s="414"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -23058,7 +23058,7 @@
       <c r="BJ1"/>
     </row>
     <row r="2" spans="1:62" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="414"/>
+      <c r="A2" s="366"/>
       <c r="B2" s="275"/>
       <c r="C2" s="275"/>
       <c r="D2" s="275"/>
@@ -23094,12 +23094,12 @@
       <c r="P2" s="277" t="s">
         <v>38</v>
       </c>
-      <c r="Q2" s="389" t="s">
+      <c r="Q2" s="405" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="3" spans="1:62" ht="24" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="414"/>
+      <c r="A3" s="366"/>
       <c r="B3" s="275"/>
       <c r="C3" s="275"/>
       <c r="D3" s="275"/>
@@ -23135,10 +23135,10 @@
       <c r="P3" s="277" t="s">
         <v>278</v>
       </c>
-      <c r="Q3" s="389"/>
+      <c r="Q3" s="405"/>
     </row>
     <row r="4" spans="1:62" ht="36" x14ac:dyDescent="0.2">
-      <c r="A4" s="415"/>
+      <c r="A4" s="367"/>
       <c r="B4" s="355" t="s">
         <v>112</v>
       </c>
@@ -23154,37 +23154,37 @@
       <c r="F4" s="355" t="s">
         <v>109</v>
       </c>
-      <c r="G4" s="408" t="s">
+      <c r="G4" s="360" t="s">
         <v>614</v>
       </c>
-      <c r="H4" s="408" t="s">
+      <c r="H4" s="360" t="s">
         <v>615</v>
       </c>
-      <c r="I4" s="408" t="s">
+      <c r="I4" s="360" t="s">
         <v>616</v>
       </c>
-      <c r="J4" s="408" t="s">
+      <c r="J4" s="360" t="s">
         <v>93</v>
       </c>
-      <c r="K4" s="408" t="s">
+      <c r="K4" s="360" t="s">
         <v>617</v>
       </c>
-      <c r="L4" s="408" t="s">
+      <c r="L4" s="360" t="s">
         <v>618</v>
       </c>
-      <c r="M4" s="408" t="s">
+      <c r="M4" s="360" t="s">
         <v>619</v>
       </c>
-      <c r="N4" s="408" t="s">
+      <c r="N4" s="360" t="s">
         <v>620</v>
       </c>
-      <c r="O4" s="408" t="s">
+      <c r="O4" s="360" t="s">
         <v>621</v>
       </c>
-      <c r="P4" s="408" t="s">
+      <c r="P4" s="360" t="s">
         <v>622</v>
       </c>
-      <c r="Q4" s="389"/>
+      <c r="Q4" s="405"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="281" t="s">
@@ -23616,11 +23616,11 @@
       </c>
       <c r="B12" s="282"/>
       <c r="C12" s="282"/>
-      <c r="D12" s="420">
+      <c r="D12" s="372">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E12" s="421" t="s">
+      <c r="E12" s="373" t="s">
         <v>46</v>
       </c>
       <c r="F12" s="356" t="s">
@@ -23675,9 +23675,9 @@
       <c r="A13" s="357"/>
       <c r="B13" s="357"/>
       <c r="C13" s="357"/>
-      <c r="D13" s="422"/>
-      <c r="E13" s="423"/>
-      <c r="F13" s="419" t="s">
+      <c r="D13" s="374"/>
+      <c r="E13" s="375"/>
+      <c r="F13" s="371" t="s">
         <v>39</v>
       </c>
       <c r="G13" s="287">
@@ -24058,13 +24058,13 @@
   <sheetData>
     <row r="1" spans="1:61" s="142" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="141"/>
-      <c r="B1" s="400" t="s">
+      <c r="B1" s="416" t="s">
         <v>170</v>
       </c>
-      <c r="C1" s="400"/>
-      <c r="D1" s="400"/>
-      <c r="E1" s="400"/>
-      <c r="F1" s="400"/>
+      <c r="C1" s="416"/>
+      <c r="D1" s="416"/>
+      <c r="E1" s="416"/>
+      <c r="F1" s="416"/>
       <c r="G1" s="143"/>
       <c r="H1" s="143"/>
       <c r="I1" s="143"/>
@@ -24109,7 +24109,7 @@
       <c r="O2" s="145" t="s">
         <v>164</v>
       </c>
-      <c r="P2" s="399" t="s">
+      <c r="P2" s="415" t="s">
         <v>163</v>
       </c>
       <c r="Q2" s="145" t="s">
@@ -24151,7 +24151,7 @@
       <c r="AC2" s="145" t="s">
         <v>162</v>
       </c>
-      <c r="AD2" s="399" t="s">
+      <c r="AD2" s="415" t="s">
         <v>161</v>
       </c>
       <c r="AE2" s="146" t="s">
@@ -24181,7 +24181,7 @@
       <c r="AM2" s="146" t="s">
         <v>160</v>
       </c>
-      <c r="AN2" s="399" t="s">
+      <c r="AN2" s="415" t="s">
         <v>159</v>
       </c>
       <c r="AZ2" s="146"/>
@@ -24193,7 +24193,7 @@
       <c r="BF2" s="146"/>
       <c r="BG2" s="146"/>
       <c r="BH2" s="146"/>
-      <c r="BI2" s="399"/>
+      <c r="BI2" s="415"/>
     </row>
     <row r="3" spans="1:61" s="142" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="144"/>
@@ -24229,7 +24229,7 @@
       <c r="O3" s="145" t="s">
         <v>135</v>
       </c>
-      <c r="P3" s="399"/>
+      <c r="P3" s="415"/>
       <c r="Q3" s="145" t="s">
         <v>134</v>
       </c>
@@ -24269,7 +24269,7 @@
       <c r="AC3" s="145" t="s">
         <v>122</v>
       </c>
-      <c r="AD3" s="399"/>
+      <c r="AD3" s="415"/>
       <c r="AE3" s="146" t="s">
         <v>121</v>
       </c>
@@ -24297,7 +24297,7 @@
       <c r="AM3" s="146" t="s">
         <v>113</v>
       </c>
-      <c r="AN3" s="399"/>
+      <c r="AN3" s="415"/>
       <c r="AZ3" s="146"/>
       <c r="BA3" s="146"/>
       <c r="BB3" s="146"/>
@@ -24307,7 +24307,7 @@
       <c r="BF3" s="146"/>
       <c r="BG3" s="146"/>
       <c r="BH3" s="146"/>
-      <c r="BI3" s="399"/>
+      <c r="BI3" s="415"/>
     </row>
     <row r="4" spans="1:61" s="142" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="147"/>
@@ -24353,7 +24353,7 @@
       <c r="O4" s="145" t="s">
         <v>85</v>
       </c>
-      <c r="P4" s="399"/>
+      <c r="P4" s="415"/>
       <c r="Q4" s="145" t="s">
         <v>84</v>
       </c>
@@ -24393,7 +24393,7 @@
       <c r="AC4" s="145" t="s">
         <v>72</v>
       </c>
-      <c r="AD4" s="399"/>
+      <c r="AD4" s="415"/>
       <c r="AE4" s="146" t="s">
         <v>71</v>
       </c>
@@ -24421,7 +24421,7 @@
       <c r="AM4" s="146" t="s">
         <v>63</v>
       </c>
-      <c r="AN4" s="399"/>
+      <c r="AN4" s="415"/>
       <c r="AZ4" s="146"/>
       <c r="BA4" s="146"/>
       <c r="BB4" s="146"/>
@@ -24431,7 +24431,7 @@
       <c r="BF4" s="146"/>
       <c r="BG4" s="146"/>
       <c r="BH4" s="146"/>
-      <c r="BI4" s="399"/>
+      <c r="BI4" s="415"/>
     </row>
     <row r="5" spans="1:61" s="142" customFormat="1" ht="144" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="149" t="s">
@@ -26067,14 +26067,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="401" t="s">
+      <c r="A1" s="417" t="s">
         <v>214</v>
       </c>
-      <c r="B1" s="401"/>
-      <c r="C1" s="401"/>
-      <c r="D1" s="401"/>
-      <c r="E1" s="401"/>
-      <c r="F1" s="401"/>
+      <c r="B1" s="417"/>
+      <c r="C1" s="417"/>
+      <c r="D1" s="417"/>
+      <c r="E1" s="417"/>
+      <c r="F1" s="417"/>
       <c r="G1" s="319"/>
       <c r="H1" s="319"/>
       <c r="I1" s="319"/>
@@ -26124,7 +26124,7 @@
       <c r="O2" s="173" t="s">
         <v>164</v>
       </c>
-      <c r="P2" s="402" t="s">
+      <c r="P2" s="418" t="s">
         <v>213</v>
       </c>
       <c r="Q2" s="173" t="s">
@@ -26136,7 +26136,7 @@
       <c r="S2" s="173" t="s">
         <v>212</v>
       </c>
-      <c r="T2" s="402" t="s">
+      <c r="T2" s="418" t="s">
         <v>211</v>
       </c>
     </row>
@@ -26174,7 +26174,7 @@
       <c r="O3" s="173" t="s">
         <v>193</v>
       </c>
-      <c r="P3" s="402"/>
+      <c r="P3" s="418"/>
       <c r="Q3" s="173" t="s">
         <v>192</v>
       </c>
@@ -26184,7 +26184,7 @@
       <c r="S3" s="173" t="s">
         <v>122</v>
       </c>
-      <c r="T3" s="402"/>
+      <c r="T3" s="418"/>
     </row>
     <row r="4" spans="1:20" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="172"/>
@@ -26230,7 +26230,7 @@
       <c r="O4" s="173" t="s">
         <v>174</v>
       </c>
-      <c r="P4" s="402"/>
+      <c r="P4" s="418"/>
       <c r="Q4" s="173" t="s">
         <v>173</v>
       </c>
@@ -26240,7 +26240,7 @@
       <c r="S4" s="173" t="s">
         <v>72</v>
       </c>
-      <c r="T4" s="402"/>
+      <c r="T4" s="418"/>
     </row>
     <row r="5" spans="1:20" ht="204" x14ac:dyDescent="0.2">
       <c r="A5" s="321" t="s">
@@ -26834,16 +26834,16 @@
   <sheetData>
     <row r="1" spans="1:23" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="181"/>
-      <c r="B1" s="403" t="s">
+      <c r="B1" s="419" t="s">
         <v>170</v>
       </c>
-      <c r="C1" s="403"/>
-      <c r="D1" s="403"/>
-      <c r="E1" s="403"/>
-      <c r="F1" s="403"/>
-      <c r="G1" s="403"/>
-      <c r="H1" s="403"/>
-      <c r="I1" s="403"/>
+      <c r="C1" s="419"/>
+      <c r="D1" s="419"/>
+      <c r="E1" s="419"/>
+      <c r="F1" s="419"/>
+      <c r="G1" s="419"/>
+      <c r="H1" s="419"/>
+      <c r="I1" s="419"/>
       <c r="J1" s="178"/>
       <c r="K1" s="178"/>
       <c r="L1" s="178"/>
@@ -26869,7 +26869,7 @@
       <c r="G2" s="180" t="s">
         <v>169</v>
       </c>
-      <c r="H2" s="404" t="s">
+      <c r="H2" s="420" t="s">
         <v>168</v>
       </c>
       <c r="I2" s="182" t="s">
@@ -26914,7 +26914,7 @@
       <c r="V2" s="182" t="s">
         <v>167</v>
       </c>
-      <c r="W2" s="404" t="s">
+      <c r="W2" s="420" t="s">
         <v>166</v>
       </c>
     </row>
@@ -26928,7 +26928,7 @@
       <c r="G3" s="180" t="s">
         <v>158</v>
       </c>
-      <c r="H3" s="404"/>
+      <c r="H3" s="420"/>
       <c r="I3" s="182" t="s">
         <v>157</v>
       </c>
@@ -26969,7 +26969,7 @@
       <c r="V3" s="182" t="s">
         <v>145</v>
       </c>
-      <c r="W3" s="404"/>
+      <c r="W3" s="420"/>
     </row>
     <row r="4" spans="1:23" ht="98" x14ac:dyDescent="0.2">
       <c r="A4" s="183"/>
@@ -26991,7 +26991,7 @@
       <c r="G4" s="180" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="404"/>
+      <c r="H4" s="420"/>
       <c r="I4" s="182" t="s">
         <v>107</v>
       </c>
@@ -27034,7 +27034,7 @@
       <c r="V4" s="185" t="s">
         <v>94</v>
       </c>
-      <c r="W4" s="404"/>
+      <c r="W4" s="420"/>
     </row>
     <row r="5" spans="1:23" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A5" s="186" t="s">
@@ -27740,16 +27740,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="406" t="s">
+      <c r="A1" s="422" t="s">
         <v>214</v>
       </c>
-      <c r="B1" s="406"/>
-      <c r="C1" s="406"/>
-      <c r="D1" s="406"/>
-      <c r="E1" s="406"/>
-      <c r="F1" s="406"/>
-      <c r="G1" s="406"/>
-      <c r="H1" s="406"/>
+      <c r="B1" s="422"/>
+      <c r="C1" s="422"/>
+      <c r="D1" s="422"/>
+      <c r="E1" s="422"/>
+      <c r="F1" s="422"/>
+      <c r="G1" s="422"/>
+      <c r="H1" s="422"/>
       <c r="I1" s="220"/>
       <c r="J1" s="220"/>
       <c r="K1" s="220"/>
@@ -27774,7 +27774,7 @@
       <c r="G2" s="222" t="s">
         <v>169</v>
       </c>
-      <c r="H2" s="405" t="s">
+      <c r="H2" s="421" t="s">
         <v>168</v>
       </c>
       <c r="I2" s="222" t="s">
@@ -27807,7 +27807,7 @@
       <c r="R2" s="222" t="s">
         <v>167</v>
       </c>
-      <c r="S2" s="405" t="s">
+      <c r="S2" s="421" t="s">
         <v>166</v>
       </c>
     </row>
@@ -27821,7 +27821,7 @@
       <c r="G3" s="222" t="s">
         <v>158</v>
       </c>
-      <c r="H3" s="405"/>
+      <c r="H3" s="421"/>
       <c r="I3" s="222" t="s">
         <v>210</v>
       </c>
@@ -27852,7 +27852,7 @@
       <c r="R3" s="222" t="s">
         <v>145</v>
       </c>
-      <c r="S3" s="405"/>
+      <c r="S3" s="421"/>
     </row>
     <row r="4" spans="1:21" ht="112" x14ac:dyDescent="0.2">
       <c r="A4" s="219"/>
@@ -27874,7 +27874,7 @@
       <c r="G4" s="222" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="405"/>
+      <c r="H4" s="421"/>
       <c r="I4" s="222" t="s">
         <v>191</v>
       </c>
@@ -27905,7 +27905,7 @@
       <c r="R4" s="222" t="s">
         <v>94</v>
       </c>
-      <c r="S4" s="405"/>
+      <c r="S4" s="421"/>
     </row>
     <row r="5" spans="1:21" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A5" s="225" t="s">
@@ -28536,13 +28536,13 @@
       <c r="K2" s="173" t="s">
         <v>167</v>
       </c>
-      <c r="L2" s="402" t="s">
+      <c r="L2" s="418" t="s">
         <v>166</v>
       </c>
       <c r="M2" s="173" t="s">
         <v>38</v>
       </c>
-      <c r="N2" s="402" t="s">
+      <c r="N2" s="418" t="s">
         <v>165</v>
       </c>
     </row>
@@ -28560,11 +28560,11 @@
       <c r="K3" s="173" t="s">
         <v>145</v>
       </c>
-      <c r="L3" s="402"/>
+      <c r="L3" s="418"/>
       <c r="M3" s="173" t="s">
         <v>142</v>
       </c>
-      <c r="N3" s="402"/>
+      <c r="N3" s="418"/>
     </row>
     <row r="4" spans="1:14" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="204"/>
@@ -28590,11 +28590,11 @@
       <c r="K4" s="173" t="s">
         <v>94</v>
       </c>
-      <c r="L4" s="402"/>
+      <c r="L4" s="418"/>
       <c r="M4" s="173" t="s">
         <v>93</v>
       </c>
-      <c r="N4" s="402"/>
+      <c r="N4" s="418"/>
     </row>
     <row r="5" spans="1:14" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="206"/>
@@ -29257,12 +29257,12 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" s="294"/>
-      <c r="B1" s="407" t="s">
+      <c r="B1" s="423" t="s">
         <v>292</v>
       </c>
-      <c r="C1" s="407"/>
-      <c r="D1" s="407"/>
-      <c r="E1" s="407"/>
+      <c r="C1" s="423"/>
+      <c r="D1" s="423"/>
+      <c r="E1" s="423"/>
       <c r="F1" s="295"/>
       <c r="G1" s="294"/>
       <c r="H1" s="294"/>
@@ -29313,7 +29313,7 @@
       <c r="P2" s="277" t="s">
         <v>38</v>
       </c>
-      <c r="Q2" s="389" t="s">
+      <c r="Q2" s="405" t="s">
         <v>271</v>
       </c>
     </row>
@@ -29354,7 +29354,7 @@
       <c r="P3" s="277" t="s">
         <v>278</v>
       </c>
-      <c r="Q3" s="389"/>
+      <c r="Q3" s="405"/>
     </row>
     <row r="4" spans="1:17" ht="70" x14ac:dyDescent="0.2">
       <c r="A4" s="278"/>
@@ -29403,7 +29403,7 @@
       <c r="P4" s="280" t="s">
         <v>289</v>
       </c>
-      <c r="Q4" s="389"/>
+      <c r="Q4" s="405"/>
     </row>
     <row r="5" spans="1:17" ht="398" x14ac:dyDescent="0.2">
       <c r="A5" s="281" t="s">
@@ -29858,22 +29858,22 @@
       <c r="A1" s="3"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
-      <c r="D1" s="377" t="s">
+      <c r="D1" s="393" t="s">
         <v>365</v>
       </c>
-      <c r="E1" s="378"/>
-      <c r="F1" s="378"/>
-      <c r="G1" s="378"/>
-      <c r="H1" s="378"/>
-      <c r="I1" s="378"/>
-      <c r="J1" s="379"/>
-      <c r="K1" s="379"/>
-      <c r="L1" s="379"/>
-      <c r="M1" s="379"/>
-      <c r="N1" s="379"/>
-      <c r="O1" s="379"/>
-      <c r="P1" s="379"/>
-      <c r="Q1" s="379"/>
+      <c r="E1" s="394"/>
+      <c r="F1" s="394"/>
+      <c r="G1" s="394"/>
+      <c r="H1" s="394"/>
+      <c r="I1" s="394"/>
+      <c r="J1" s="395"/>
+      <c r="K1" s="395"/>
+      <c r="L1" s="395"/>
+      <c r="M1" s="395"/>
+      <c r="N1" s="395"/>
+      <c r="O1" s="395"/>
+      <c r="P1" s="395"/>
+      <c r="Q1" s="395"/>
       <c r="R1" s="6" t="s">
         <v>260</v>
       </c>
@@ -30018,28 +30018,28 @@
       <c r="D4" s="239"/>
       <c r="E4" s="239"/>
       <c r="F4" s="239"/>
-      <c r="G4" s="380" t="s">
+      <c r="G4" s="396" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="381"/>
-      <c r="I4" s="381"/>
-      <c r="J4" s="381"/>
-      <c r="K4" s="381"/>
-      <c r="L4" s="382"/>
-      <c r="M4" s="383"/>
-      <c r="N4" s="384" t="s">
+      <c r="H4" s="397"/>
+      <c r="I4" s="397"/>
+      <c r="J4" s="397"/>
+      <c r="K4" s="397"/>
+      <c r="L4" s="398"/>
+      <c r="M4" s="399"/>
+      <c r="N4" s="400" t="s">
         <v>27</v>
       </c>
-      <c r="O4" s="382"/>
-      <c r="P4" s="382"/>
-      <c r="Q4" s="382"/>
-      <c r="R4" s="382"/>
-      <c r="S4" s="382"/>
-      <c r="T4" s="385"/>
-      <c r="U4" s="380" t="s">
+      <c r="O4" s="398"/>
+      <c r="P4" s="398"/>
+      <c r="Q4" s="398"/>
+      <c r="R4" s="398"/>
+      <c r="S4" s="398"/>
+      <c r="T4" s="401"/>
+      <c r="U4" s="396" t="s">
         <v>28</v>
       </c>
-      <c r="V4" s="383"/>
+      <c r="V4" s="399"/>
       <c r="W4" s="246"/>
       <c r="X4" t="s">
         <v>0</v>
@@ -30454,16 +30454,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:57" s="41" customFormat="1" ht="23.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B1" s="387" t="s">
+      <c r="B1" s="403" t="s">
         <v>170</v>
       </c>
-      <c r="C1" s="387"/>
-      <c r="D1" s="387"/>
-      <c r="E1" s="387"/>
-      <c r="F1" s="387"/>
-      <c r="G1" s="387"/>
-      <c r="H1" s="387"/>
-      <c r="I1" s="387"/>
+      <c r="C1" s="403"/>
+      <c r="D1" s="403"/>
+      <c r="E1" s="403"/>
+      <c r="F1" s="403"/>
+      <c r="G1" s="403"/>
+      <c r="H1" s="403"/>
+      <c r="I1" s="403"/>
     </row>
     <row r="2" spans="1:57" s="41" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="78"/>
@@ -30475,7 +30475,7 @@
       <c r="G2" s="75" t="s">
         <v>169</v>
       </c>
-      <c r="H2" s="386" t="s">
+      <c r="H2" s="402" t="s">
         <v>168</v>
       </c>
       <c r="I2" s="74" t="s">
@@ -30520,7 +30520,7 @@
       <c r="V2" s="74" t="s">
         <v>167</v>
       </c>
-      <c r="W2" s="386" t="s">
+      <c r="W2" s="402" t="s">
         <v>166</v>
       </c>
       <c r="X2" s="73" t="s">
@@ -30550,7 +30550,7 @@
       <c r="AF2" s="73" t="s">
         <v>164</v>
       </c>
-      <c r="AG2" s="386" t="s">
+      <c r="AG2" s="402" t="s">
         <v>163</v>
       </c>
       <c r="AH2" s="73" t="s">
@@ -30592,7 +30592,7 @@
       <c r="AT2" s="73" t="s">
         <v>162</v>
       </c>
-      <c r="AU2" s="386" t="s">
+      <c r="AU2" s="402" t="s">
         <v>161</v>
       </c>
       <c r="AV2" s="72" t="s">
@@ -30622,7 +30622,7 @@
       <c r="BD2" s="72" t="s">
         <v>160</v>
       </c>
-      <c r="BE2" s="386" t="s">
+      <c r="BE2" s="402" t="s">
         <v>159</v>
       </c>
     </row>
@@ -30636,7 +30636,7 @@
       <c r="G3" s="75" t="s">
         <v>158</v>
       </c>
-      <c r="H3" s="386"/>
+      <c r="H3" s="402"/>
       <c r="I3" s="74" t="s">
         <v>157</v>
       </c>
@@ -30677,7 +30677,7 @@
       <c r="V3" s="74" t="s">
         <v>145</v>
       </c>
-      <c r="W3" s="386"/>
+      <c r="W3" s="402"/>
       <c r="X3" s="73" t="s">
         <v>141</v>
       </c>
@@ -30705,7 +30705,7 @@
       <c r="AF3" s="73" t="s">
         <v>135</v>
       </c>
-      <c r="AG3" s="386"/>
+      <c r="AG3" s="402"/>
       <c r="AH3" s="73" t="s">
         <v>134</v>
       </c>
@@ -30745,7 +30745,7 @@
       <c r="AT3" s="73" t="s">
         <v>122</v>
       </c>
-      <c r="AU3" s="386"/>
+      <c r="AU3" s="402"/>
       <c r="AV3" s="72" t="s">
         <v>121</v>
       </c>
@@ -30773,7 +30773,7 @@
       <c r="BD3" s="72" t="s">
         <v>113</v>
       </c>
-      <c r="BE3" s="386"/>
+      <c r="BE3" s="402"/>
     </row>
     <row r="4" spans="1:57" s="41" customFormat="1" ht="60" x14ac:dyDescent="0.15">
       <c r="A4" s="77"/>
@@ -30795,7 +30795,7 @@
       <c r="G4" s="75" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="386"/>
+      <c r="H4" s="402"/>
       <c r="I4" s="74" t="s">
         <v>107</v>
       </c>
@@ -30838,7 +30838,7 @@
       <c r="V4" s="74" t="s">
         <v>94</v>
       </c>
-      <c r="W4" s="386"/>
+      <c r="W4" s="402"/>
       <c r="X4" s="73" t="s">
         <v>92</v>
       </c>
@@ -30866,7 +30866,7 @@
       <c r="AF4" s="73" t="s">
         <v>85</v>
       </c>
-      <c r="AG4" s="386"/>
+      <c r="AG4" s="402"/>
       <c r="AH4" s="73" t="s">
         <v>84</v>
       </c>
@@ -30906,7 +30906,7 @@
       <c r="AT4" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="AU4" s="386"/>
+      <c r="AU4" s="402"/>
       <c r="AV4" s="72" t="s">
         <v>71</v>
       </c>
@@ -30934,7 +30934,7 @@
       <c r="BD4" s="72" t="s">
         <v>63</v>
       </c>
-      <c r="BE4" s="386"/>
+      <c r="BE4" s="402"/>
     </row>
     <row r="5" spans="1:57" s="41" customFormat="1" ht="11" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="51" t="s">
@@ -30952,50 +30952,50 @@
       <c r="F5" s="60" t="s">
         <v>61</v>
       </c>
-      <c r="G5" s="101" t="e" cm="1">
-        <f t="array" ref="G5">SUM(SUMIFS(
+      <c r="G5" s="101" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("2. TOTAL CONTENTIEUX JAF",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3. TOTAL CONTENTIEUX DE LA PROTECTION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4. TOTAL CIVIL NON SPÉCIALISÉ",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("5. TOTAL JLD CIVIL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("6.1. ACTIVITÉ CIVILE",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.7. FONCTIONNAIRES AFFECTÉS AU CPH",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.8. FONCTIONNAIRES AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="H5" s="59" t="e">
         <f t="shared" ref="H5:H15" si="0">SUM(G5)</f>
         <v>#N/A</v>
       </c>
-      <c r="I5" s="58" t="e" cm="1">
-        <f t="array" ref="I5">SUM(SUMIFS(
+      <c r="I5" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.8. FONCTIONNAIRES AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="J5" s="70"/>
@@ -31004,81 +31004,81 @@
       <c r="M5" s="70"/>
       <c r="N5" s="70"/>
       <c r="O5" s="70"/>
-      <c r="P5" s="58" t="e" cm="1">
-        <f t="array" ref="P5">SUM(SUMIFS(
+      <c r="P5" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="Q5" s="58" t="e" cm="1">
-        <f t="array" ref="Q5">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q5" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3. TOTAL CONTENTIEUX DE LA PROTECTION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="R5" s="58" t="e" cm="1">
-        <f t="array" ref="R5">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="R5" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("5. TOTAL JLD CIVIL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("6.1. ACTIVITÉ CIVILE",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="S5" s="58" t="e" cm="1">
-        <f t="array" ref="S5">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="S5" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="T5" s="58" t="e" cm="1">
-        <f t="array" ref="T5">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="T5" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="U5" s="58" t="e" cm="1">
-        <f t="array" ref="U5">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="U5" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="V5" s="58" t="e" cm="1">
-        <f t="array" ref="V5">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="V5" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("2. TOTAL CONTENTIEUX JAF",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4. TOTAL CIVIL NON SPÉCIALISÉ",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="W5" s="46" t="e">
@@ -31089,26 +31089,26 @@
         <f t="array" ref="X5">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"Magistrat SIEGE S";"Magistrat SIEGE NS"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="Y5" s="53" t="e" cm="1">
         <f t="array" ref="Y5">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3. TOTAL CONTENTIEUX DE LA PROTECTION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"Magistrat SIEGE S";"Magistrat SIEGE NS"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"Magistrat SIEGE S";"Magistrat SIEGE NS"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"Magistrat SIEGE S";"Magistrat SIEGE NS"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"Magistrat SIEGE S";"Magistrat SIEGE NS"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="Z5" s="68"/>
@@ -31142,36 +31142,36 @@
         <f t="array" ref="AN5">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("1.1. DÉPARTAGE PRUD'HOMAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"Magistrat SIEGE S";"Magistrat SIEGE NS"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AO5" s="53" t="e" cm="1">
         <f t="array" ref="AO5">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"Magistrat SIEGE S";"Magistrat SIEGE NS"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AP5" s="53" t="e" cm="1">
         <f t="array" ref="AP5">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"Magistrat SIEGE S";"Magistrat SIEGE NS"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"Magistrat SIEGE S";"Magistrat SIEGE NS"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AQ5" s="53" t="e" cm="1">
         <f t="array" ref="AQ5">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"Magistrat SIEGE S";"Magistrat SIEGE NS"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("1.1. DÉPARTAGE PRUD'HOMAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"Magistrat SIEGE S";"Magistrat SIEGE NS"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AR5" s="55" t="e" cm="1">
@@ -31180,26 +31180,26 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"Magistrat SIEGE S";"Magistrat SIEGE NS"}))</f>
         <v>#N/A</v>
       </c>
-      <c r="AS5" s="55" t="e" cm="1">
-        <f t="array" ref="AS5">SUM(SUMIFS(
+      <c r="AS5" s="55" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4. TOTAL CIVIL NON SPÉCIALISÉ",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE S",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE S",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AT5" s="55" t="e" cm="1">
-        <f t="array" ref="AT5">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="AT5" s="55" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4. TOTAL CIVIL NON SPÉCIALISÉ",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AU5" s="46" t="e">
@@ -31600,14 +31600,14 @@
         <f t="array" ref="Y7">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.5. CSM",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JCP";"VPCP";"1VPCP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="Z7" s="53" t="e" cm="1">
         <f t="array" ref="Z7">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.5. CSM",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JI";"VPI";"1VPI"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AA7" s="62"/>
@@ -31617,21 +31617,21 @@
         <f t="array" ref="AD7">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.5. CSM",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JAP";"VPAP";"1VPAP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AE7" s="53" t="e" cm="1">
         <f t="array" ref="AE7">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.5. CSM",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JE";"VPE";"1VPE"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AF7" s="53" t="e" cm="1">
         <f t="array" ref="AF7">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.5. CSM",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"VPLD";"1VPLD"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AG7" s="46" t="e">
@@ -31650,11 +31650,11 @@
       <c r="AQ7" s="62"/>
       <c r="AR7" s="266"/>
       <c r="AS7" s="62"/>
-      <c r="AT7" s="53" t="e" cm="1">
-        <f t="array" ref="AT7">SUM(SUMIFS(
+      <c r="AT7" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.5. CSM",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AU7" s="46" t="e">
@@ -31691,11 +31691,11 @@
       <c r="F8" s="60" t="s">
         <v>55</v>
       </c>
-      <c r="G8" s="101" t="e" cm="1">
-        <f t="array" ref="G8">SUM(SUMIFS(
+      <c r="G8" s="101" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.51. ACCUEIL DU JUSTICIABLE (DONT SAUJ)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="H8" s="59" t="e">
@@ -31715,11 +31715,11 @@
       <c r="S8" s="62"/>
       <c r="T8" s="62"/>
       <c r="U8" s="62"/>
-      <c r="V8" s="53" t="e" cm="1">
-        <f t="array" ref="V8">SUM(SUMIFS(
+      <c r="V8" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.51. ACCUEIL DU JUSTICIABLE (DONT SAUJ)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="W8" s="46" t="e">
@@ -31731,14 +31731,14 @@
         <f t="array" ref="Y8">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.51. ACCUEIL DU JUSTICIABLE (DONT SAUJ)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JCP";"VPCP";"1VPCP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="Z8" s="53" t="e" cm="1">
         <f t="array" ref="Z8">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.51. ACCUEIL DU JUSTICIABLE (DONT SAUJ)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JI";"VPI";"1VPI"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AA8" s="62"/>
@@ -31748,21 +31748,21 @@
         <f t="array" ref="AD8">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.51. ACCUEIL DU JUSTICIABLE (DONT SAUJ)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JAP";"VPAP";"1VPAP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AE8" s="53" t="e" cm="1">
         <f t="array" ref="AE8">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.51. ACCUEIL DU JUSTICIABLE (DONT SAUJ)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JE";"VPE";"1VPE"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AF8" s="53" t="e" cm="1">
         <f t="array" ref="AF8">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.51. ACCUEIL DU JUSTICIABLE (DONT SAUJ)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"VPLD";"1VPLD"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AG8" s="46" t="e">
@@ -31781,11 +31781,11 @@
       <c r="AQ8" s="62"/>
       <c r="AR8" s="62"/>
       <c r="AS8" s="62"/>
-      <c r="AT8" s="53" t="e" cm="1">
-        <f t="array" ref="AT8">SUM(SUMIFS(
+      <c r="AT8" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.51. ACCUEIL DU JUSTICIABLE (DONT SAUJ)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AU8" s="46" t="e">
@@ -31822,19 +31822,19 @@
       <c r="F9" s="60" t="s">
         <v>53</v>
       </c>
-      <c r="G9" s="101" t="e" cm="1">
-        <f t="array" ref="G9">SUM(SUMIFS(
+      <c r="G9" s="101" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.1. SOUTIEN (HORS FORMATIONS SUIVIES)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.2. FORMATIONS SUIVIES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.6. AUTRES ACTIVITÉS NON JURIDICTIONNELLES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="H9" s="59" t="e">
@@ -31854,19 +31854,19 @@
       <c r="S9" s="62"/>
       <c r="T9" s="62"/>
       <c r="U9" s="62"/>
-      <c r="V9" s="53" t="e" cm="1">
-        <f t="array" ref="V9">SUM(SUMIFS(
+      <c r="V9" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.1. SOUTIEN (HORS FORMATIONS SUIVIES)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.2. FORMATIONS SUIVIES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.6. AUTRES ACTIVITÉS NON JURIDICTIONNELLES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="W9" s="46" t="e">
@@ -31878,30 +31878,30 @@
         <f t="array" ref="Y9">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.1. SOUTIEN (HORS FORMATIONS SUIVIES)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JCP";"VPCP";"1VPCP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.2. FORMATIONS SUIVIES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JCP";"VPCP";"1VPCP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.6. AUTRES ACTIVITÉS NON JURIDICTIONNELLES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JCP";"VPCP";"1VPCP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="Z9" s="53" t="e" cm="1">
         <f t="array" ref="Z9">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.1. SOUTIEN (HORS FORMATIONS SUIVIES)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JI";"VPI";"1VPI"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.2. FORMATIONS SUIVIES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JI";"VPI";"1VPI"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.6. AUTRES ACTIVITÉS NON JURIDICTIONNELLES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JI";"VPI";"1VPI"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AA9" s="62"/>
@@ -31911,45 +31911,45 @@
         <f t="array" ref="AD9">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.1. SOUTIEN (HORS FORMATIONS SUIVIES)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JAP";"VPAP";"1VPAP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.2. FORMATIONS SUIVIES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JAP";"VPAP";"1VPAP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.6. AUTRES ACTIVITÉS NON JURIDICTIONNELLES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JAP";"VPAP";"1VPAP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AE9" s="53" t="e" cm="1">
         <f t="array" ref="AE9">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.1. SOUTIEN (HORS FORMATIONS SUIVIES)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JE";"VPE";"1VPE"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.2. FORMATIONS SUIVIES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JE";"VPE";"1VPE"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.6. AUTRES ACTIVITÉS NON JURIDICTIONNELLES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JE";"VPE";"1VPE"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AF9" s="53" t="e" cm="1">
         <f t="array" ref="AF9">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.1. SOUTIEN (HORS FORMATIONS SUIVIES)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"VPLD";"1VPLD"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.2. FORMATIONS SUIVIES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"VPLD";"1VPLD"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.6. AUTRES ACTIVITÉS NON JURIDICTIONNELLES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"VPLD";"1VPLD"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AG9" s="46" t="e">
@@ -31968,19 +31968,19 @@
       <c r="AQ9" s="62"/>
       <c r="AR9" s="62"/>
       <c r="AS9" s="62"/>
-      <c r="AT9" s="53" t="e" cm="1">
-        <f t="array" ref="AT9">SUM(SUMIFS(
+      <c r="AT9" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.1. SOUTIEN (HORS FORMATIONS SUIVIES)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.2. FORMATIONS SUIVIES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.6. AUTRES ACTIVITÉS NON JURIDICTIONNELLES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AU9" s="46" t="e">
@@ -32017,11 +32017,11 @@
       <c r="F10" s="60" t="s">
         <v>51</v>
       </c>
-      <c r="G10" s="101" t="e" cm="1">
-        <f t="array" ref="G10">SUM(SUMIFS(
+      <c r="G10" s="101" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="H10" s="59" t="e">
@@ -32041,11 +32041,11 @@
       <c r="S10" s="62"/>
       <c r="T10" s="62"/>
       <c r="U10" s="62"/>
-      <c r="V10" s="53" t="e" cm="1">
-        <f t="array" ref="V10">SUM(SUMIFS(
+      <c r="V10" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="W10" s="46" t="e">
@@ -32057,14 +32057,14 @@
         <f t="array" ref="Y10">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JCP";"VPCP";"1VPCP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="Z10" s="53" t="e" cm="1">
         <f t="array" ref="Z10">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JI";"VPI";"1VPI"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AA10" s="62"/>
@@ -32074,21 +32074,21 @@
         <f t="array" ref="AD10">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JAP";"VPAP";"1VPAP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AE10" s="53" t="e" cm="1">
         <f t="array" ref="AE10">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JE";"VPE";"1VPE"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AF10" s="53" t="e" cm="1">
         <f t="array" ref="AF10">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"VPLD";"1VPLD"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AG10" s="46" t="e">
@@ -32107,11 +32107,11 @@
       <c r="AQ10" s="62"/>
       <c r="AR10" s="62"/>
       <c r="AS10" s="62"/>
-      <c r="AT10" s="53" t="e" cm="1">
-        <f t="array" ref="AT10">SUM(SUMIFS(
+      <c r="AT10" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AU10" s="46" t="e">
@@ -32148,11 +32148,11 @@
       <c r="F11" s="60" t="s">
         <v>49</v>
       </c>
-      <c r="G11" s="101" t="e" cm="1">
-        <f t="array" ref="G11">SUM(SUMIFS(
+      <c r="G11" s="101" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.4. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="H11" s="59" t="e">
@@ -32172,11 +32172,11 @@
       <c r="S11" s="62"/>
       <c r="T11" s="62"/>
       <c r="U11" s="62"/>
-      <c r="V11" s="53" t="e" cm="1">
-        <f t="array" ref="V11">SUM(SUMIFS(
+      <c r="V11" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.4. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="W11" s="46" t="e">
@@ -32188,14 +32188,14 @@
         <f t="array" ref="Y11">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.4. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JCP";"VPCP";"1VPCP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="Z11" s="53" t="e" cm="1">
         <f t="array" ref="Z11">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.4. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JI";"VPI";"1VPI"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AA11" s="64"/>
@@ -32205,21 +32205,21 @@
         <f t="array" ref="AD11">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.4. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JAP";"VPAP";"1VPAP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AE11" s="53" t="e" cm="1">
         <f t="array" ref="AE11">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.4. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JE";"VPE";"1VPE"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AF11" s="53" t="e" cm="1">
         <f t="array" ref="AF11">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.4. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"VPLD";"1VPLD"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AG11" s="59" t="e">
@@ -32238,11 +32238,11 @@
       <c r="AQ11" s="62"/>
       <c r="AR11" s="62"/>
       <c r="AS11" s="62"/>
-      <c r="AT11" s="53" t="e" cm="1">
-        <f t="array" ref="AT11">SUM(SUMIFS(
+      <c r="AT11" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.4. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AU11" s="46" t="e">
@@ -32279,15 +32279,15 @@
       <c r="F12" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="G12" s="101" t="e" cm="1">
-        <f t="array" ref="G12">SUM(SUMIFS(
+      <c r="G12" s="101" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="H12" s="59" t="e">
@@ -32307,15 +32307,15 @@
       <c r="S12" s="62"/>
       <c r="T12" s="62"/>
       <c r="U12" s="62"/>
-      <c r="V12" s="53" t="e" cm="1">
-        <f t="array" ref="V12">SUM(SUMIFS(
+      <c r="V12" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="W12" s="46" t="e">
@@ -32327,22 +32327,22 @@
         <f t="array" ref="Y12">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JCP";"VPCP";"1VPCP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JCP";"VPCP";"1VPCP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="Z12" s="53" t="e" cm="1">
         <f t="array" ref="Z12">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JI";"VPI";"1VPI"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JI";"VPI";"1VPI"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AA12" s="62"/>
@@ -32352,33 +32352,33 @@
         <f t="array" ref="AD12">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JAP";"VPAP";"1VPAP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JAP";"VPAP";"1VPAP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AE12" s="53" t="e" cm="1">
         <f t="array" ref="AE12">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JE";"VPE";"1VPE"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JE";"VPE";"1VPE"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AF12" s="53" t="e" cm="1">
         <f t="array" ref="AF12">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"VPLD";"1VPLD"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"VPLD";"1VPLD"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AG12" s="46" t="e">
@@ -32397,15 +32397,15 @@
       <c r="AQ12" s="62"/>
       <c r="AR12" s="62"/>
       <c r="AS12" s="62"/>
-      <c r="AT12" s="53" t="e" cm="1">
-        <f t="array" ref="AT12">SUM(SUMIFS(
+      <c r="AT12" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AU12" s="46" t="e">
@@ -32442,15 +32442,15 @@
       <c r="F13" s="60" t="s">
         <v>45</v>
       </c>
-      <c r="G13" s="101" t="e" cm="1">
-        <f t="array" ref="G13">SUM(SUMIFS(
+      <c r="G13" s="101" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13. TOTAL CONTENTIEUX LOCAUX SPÉCIFIQUES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="H13" s="59" t="e">
@@ -32470,15 +32470,15 @@
       <c r="S13" s="62"/>
       <c r="T13" s="62"/>
       <c r="U13" s="62"/>
-      <c r="V13" s="53" t="e" cm="1">
-        <f t="array" ref="V13">SUM(SUMIFS(
+      <c r="V13" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13. TOTAL CONTENTIEUX LOCAUX SPÉCIFIQUES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="W13" s="46" t="e">
@@ -32490,14 +32490,14 @@
         <f t="array" ref="Y13">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JCP";"VPCP";"1VPCP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="Z13" s="53" t="e" cm="1">
         <f t="array" ref="Z13">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JI";"VPI";"1VPI"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AA13" s="62"/>
@@ -32507,21 +32507,21 @@
         <f t="array" ref="AD13">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JAP";"VPAP";"1VPAP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AE13" s="53" t="e" cm="1">
         <f t="array" ref="AE13">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JE";"VPE";"1VPE"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AF13" s="53" t="e" cm="1">
         <f t="array" ref="AF13">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"VPLD";"1VPLD"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AG13" s="46" t="e">
@@ -32539,22 +32539,22 @@
       <c r="AP13" s="62"/>
       <c r="AQ13" s="62"/>
       <c r="AR13" s="62"/>
-      <c r="AS13" s="53" t="e" cm="1">
-        <f t="array" ref="AS13">SUM(SUMIFS(
+      <c r="AS13" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13. TOTAL CONTENTIEUX LOCAUX SPÉCIFIQUES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE S",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AT13" s="53" t="e" cm="1">
-        <f t="array" ref="AT13">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="AT13" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13. TOTAL CONTENTIEUX LOCAUX SPÉCIFIQUES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AU13" s="46" t="e">
@@ -32591,22 +32591,22 @@
       <c r="F14" s="60" t="s">
         <v>43</v>
       </c>
-      <c r="G14" s="101" t="e" cm="1">
-        <f t="array" ref="G14">SUM(SUMIFS(
+      <c r="G14" s="101" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Temps ventilés sur la période (hors action 99)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="H14" s="59" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
       </c>
-      <c r="I14" s="58" t="e" cm="1">
-        <f t="array" ref="I14">SUM(SUMIFS(
+      <c r="I14" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.8. FONCTIONNAIRES AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="J14" s="58" t="e">
@@ -32653,30 +32653,30 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Jirs",'ETPT Format DDG'!2:2,0)),""))</f>
         <v>#N/A</v>
       </c>
-      <c r="P14" s="58" t="e" cm="1">
-        <f t="array" ref="P14">SUM(SUMIFS(
+      <c r="P14" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="Q14" s="58" t="e" cm="1">
-        <f t="array" ref="Q14">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q14" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3. TOTAL CONTENTIEUX DE LA PROTECTION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="R14" s="58" t="e">
@@ -32697,52 +32697,52 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD"))</f>
         <v>#N/A</v>
       </c>
-      <c r="S14" s="58" t="e" cm="1">
-        <f t="array" ref="S14">SUM(SUMIFS(
+      <c r="S14" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="T14" s="58" t="e" cm="1">
-        <f t="array" ref="T14">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="T14" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="U14" s="58" t="e" cm="1">
-        <f t="array" ref="U14">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="U14" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="V14" s="53" t="e" cm="1">
-        <f t="array" ref="V14">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="V14" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("2. TOTAL CONTENTIEUX JAF",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4. TOTAL CIVIL NON SPÉCIALISÉ",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("6.1. ACTIVITÉ CIVILE",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13. TOTAL CONTENTIEUX LOCAUX SPÉCIFIQUES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.1. COLLÉGIALES HORS JIRS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD")+
@@ -32782,30 +32782,30 @@
         <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
-      <c r="X14" s="53" t="e" cm="1">
-        <f t="array" ref="X14">SUM(SUMIFS(
+      <c r="X14" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="Y14" s="53" t="e" cm="1">
-        <f t="array" ref="Y14">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Y14" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3. TOTAL CONTENTIEUX DE LA PROTECTION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="Z14" s="53" t="e">
@@ -32910,40 +32910,40 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé ADD"))</f>
         <v>#N/A</v>
       </c>
-      <c r="AN14" s="53" t="e" cm="1">
-        <f t="array" ref="AN14">SUM(SUMIFS(
+      <c r="AN14" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("1.1. DÉPARTAGE PRUD'HOMAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AO14" s="53" t="e" cm="1">
-        <f t="array" ref="AO14">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="AO14" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AP14" s="53" t="e" cm="1">
-        <f t="array" ref="AP14">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="AP14" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AQ14" s="53" t="e" cm="1">
-        <f t="array" ref="AQ14">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="AQ14" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("1.1. DÉPARTAGE PRUD'HOMAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AR14" s="53" t="e">
@@ -32953,15 +32953,15 @@
         <v>#N/A</v>
       </c>
       <c r="AS14" s="54"/>
-      <c r="AT14" s="53" t="e" cm="1">
-        <f t="array" ref="AT14">SUM(SUMIFS(
+      <c r="AT14" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4. TOTAL CIVIL NON SPÉCIALISÉ",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé ADD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.1. COLLÉGIALES HORS JIRS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé ADD")+
@@ -33022,22 +33022,22 @@
       <c r="F15" s="60" t="s">
         <v>40</v>
       </c>
-      <c r="G15" s="101" t="e" cm="1">
-        <f t="array" ref="G15">SUM(SUMIFS(
+      <c r="G15" s="101" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Temps ventilés sur la période (hors action 99)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="H15" s="59" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
       </c>
-      <c r="I15" s="58" t="e" cm="1">
-        <f t="array" ref="I15">SUM(SUMIFS(
+      <c r="I15" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.8. FONCTIONNAIRES AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="J15" s="58" t="e">
@@ -33084,30 +33084,30 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Jirs",'ETPT Format DDG'!2:2,0)),""))</f>
         <v>#N/A</v>
       </c>
-      <c r="P15" s="58" t="e" cm="1">
-        <f t="array" ref="P15">SUM(SUMIFS(
+      <c r="P15" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="Q15" s="58" t="e" cm="1">
-        <f t="array" ref="Q15">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q15" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3. TOTAL CONTENTIEUX DE LA PROTECTION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="R15" s="58" t="e">
@@ -33128,52 +33128,52 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB"))</f>
         <v>#N/A</v>
       </c>
-      <c r="S15" s="58" t="e" cm="1">
-        <f t="array" ref="S15">SUM(SUMIFS(
+      <c r="S15" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="T15" s="58" t="e" cm="1">
-        <f t="array" ref="T15">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="T15" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="U15" s="58" t="e" cm="1">
-        <f t="array" ref="U15">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="U15" s="58" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="V15" s="53" t="e" cm="1">
-        <f t="array" ref="V15">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="V15" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("2. TOTAL CONTENTIEUX JAF",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4. TOTAL CIVIL NON SPÉCIALISÉ",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("6.1. ACTIVITÉ CIVILE",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13. TOTAL CONTENTIEUX LOCAUX SPÉCIFIQUES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.1. COLLÉGIALES HORS JIRS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB")+
@@ -33213,30 +33213,30 @@
         <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
-      <c r="X15" s="53" t="e" cm="1">
-        <f t="array" ref="X15">SUM(SUMIFS(
+      <c r="X15" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="Y15" s="53" t="e" cm="1">
-        <f t="array" ref="Y15">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Y15" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3. TOTAL CONTENTIEUX DE LA PROTECTION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.2. PROTECTION DES MAJEURS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="Z15" s="53" t="e">
@@ -33341,40 +33341,40 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé SUB"))</f>
         <v>#N/A</v>
       </c>
-      <c r="AN15" s="53" t="e" cm="1">
-        <f t="array" ref="AN15">SUM(SUMIFS(
+      <c r="AN15" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("1.1. DÉPARTAGE PRUD'HOMAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AO15" s="53" t="e" cm="1">
-        <f t="array" ref="AO15">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="AO15" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AP15" s="53" t="e" cm="1">
-        <f t="array" ref="AP15">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="AP15" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.43. INJONCTIONS DE PAYER",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AQ15" s="53" t="e" cm="1">
-        <f t="array" ref="AQ15">SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="AQ15" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("1.1. DÉPARTAGE PRUD'HOMAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AR15" s="53" t="e">
@@ -33384,15 +33384,15 @@
         <v>#N/A</v>
       </c>
       <c r="AS15" s="54"/>
-      <c r="AT15" s="53" t="e" cm="1">
-        <f t="array" ref="AT15">SUM(SUMIFS(
+      <c r="AT15" s="53" t="e">
+        <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4. TOTAL CIVIL NON SPÉCIALISÉ",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))-
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé SUB",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))+
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))+
 SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.1. COLLÉGIALES HORS JIRS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat placé SUB")+
@@ -33728,7 +33728,7 @@
         <f t="array" ref="G20">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"Fonctionnaire CTECH placé ADD";"Fonctionnaire CTECH placé SUB"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="U20" s="250" t="s">
@@ -33738,7 +33738,7 @@
         <f t="array" ref="V20">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"Fonctionnaire A-B-CBUR placé ADD";"Fonctionnaire A-B-CBUR placé SUB"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="W20" s="38"/>
@@ -33749,7 +33749,7 @@
         <f t="array" ref="AT20">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"Magistrat placé ADD";"Magistrat placé SUB"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),TJCPH))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
         <v>#N/A</v>
       </c>
       <c r="AU20" s="38"/>
@@ -33793,16 +33793,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" x14ac:dyDescent="0.2">
-      <c r="A1" s="388" t="s">
+      <c r="A1" s="404" t="s">
         <v>214</v>
       </c>
-      <c r="B1" s="388"/>
-      <c r="C1" s="388"/>
-      <c r="D1" s="388"/>
-      <c r="E1" s="388"/>
-      <c r="F1" s="388"/>
-      <c r="G1" s="388"/>
-      <c r="H1" s="388"/>
+      <c r="B1" s="404"/>
+      <c r="C1" s="404"/>
+      <c r="D1" s="404"/>
+      <c r="E1" s="404"/>
+      <c r="F1" s="404"/>
+      <c r="G1" s="404"/>
+      <c r="H1" s="404"/>
       <c r="I1" s="41"/>
       <c r="J1" s="41"/>
       <c r="K1" s="41"/>
@@ -33839,7 +33839,7 @@
       <c r="G2" s="75" t="s">
         <v>169</v>
       </c>
-      <c r="H2" s="386" t="s">
+      <c r="H2" s="402" t="s">
         <v>168</v>
       </c>
       <c r="I2" s="75" t="s">
@@ -33872,7 +33872,7 @@
       <c r="R2" s="75" t="s">
         <v>167</v>
       </c>
-      <c r="S2" s="386" t="s">
+      <c r="S2" s="402" t="s">
         <v>166</v>
       </c>
       <c r="T2" s="75" t="s">
@@ -33902,7 +33902,7 @@
       <c r="AB2" s="75" t="s">
         <v>164</v>
       </c>
-      <c r="AC2" s="386" t="s">
+      <c r="AC2" s="402" t="s">
         <v>213</v>
       </c>
       <c r="AD2" s="75" t="s">
@@ -33914,7 +33914,7 @@
       <c r="AF2" s="75" t="s">
         <v>212</v>
       </c>
-      <c r="AG2" s="386" t="s">
+      <c r="AG2" s="402" t="s">
         <v>211</v>
       </c>
     </row>
@@ -33928,7 +33928,7 @@
       <c r="G3" s="75" t="s">
         <v>158</v>
       </c>
-      <c r="H3" s="386"/>
+      <c r="H3" s="402"/>
       <c r="I3" s="75" t="s">
         <v>210</v>
       </c>
@@ -33959,7 +33959,7 @@
       <c r="R3" s="75" t="s">
         <v>145</v>
       </c>
-      <c r="S3" s="386"/>
+      <c r="S3" s="402"/>
       <c r="T3" s="75" t="s">
         <v>201</v>
       </c>
@@ -33987,7 +33987,7 @@
       <c r="AB3" s="75" t="s">
         <v>193</v>
       </c>
-      <c r="AC3" s="386"/>
+      <c r="AC3" s="402"/>
       <c r="AD3" s="75" t="s">
         <v>192</v>
       </c>
@@ -33997,7 +33997,7 @@
       <c r="AF3" s="75" t="s">
         <v>122</v>
       </c>
-      <c r="AG3" s="386"/>
+      <c r="AG3" s="402"/>
     </row>
     <row r="4" spans="1:33" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="78"/>
@@ -34019,7 +34019,7 @@
       <c r="G4" s="75" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="386"/>
+      <c r="H4" s="402"/>
       <c r="I4" s="75" t="s">
         <v>191</v>
       </c>
@@ -34050,7 +34050,7 @@
       <c r="R4" s="75" t="s">
         <v>94</v>
       </c>
-      <c r="S4" s="386"/>
+      <c r="S4" s="402"/>
       <c r="T4" s="75" t="s">
         <v>182</v>
       </c>
@@ -34078,7 +34078,7 @@
       <c r="AB4" s="75" t="s">
         <v>174</v>
       </c>
-      <c r="AC4" s="386"/>
+      <c r="AC4" s="402"/>
       <c r="AD4" s="75" t="s">
         <v>173</v>
       </c>
@@ -34088,7 +34088,7 @@
       <c r="AF4" s="75" t="s">
         <v>72</v>
       </c>
-      <c r="AG4" s="386"/>
+      <c r="AG4" s="402"/>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A5" s="81" t="s">
@@ -35458,13 +35458,13 @@
       <c r="G2" s="75" t="s">
         <v>167</v>
       </c>
-      <c r="H2" s="386" t="s">
+      <c r="H2" s="402" t="s">
         <v>166</v>
       </c>
       <c r="I2" s="75" t="s">
         <v>38</v>
       </c>
-      <c r="J2" s="386" t="s">
+      <c r="J2" s="402" t="s">
         <v>165</v>
       </c>
     </row>
@@ -35478,11 +35478,11 @@
       <c r="G3" s="75" t="s">
         <v>145</v>
       </c>
-      <c r="H3" s="386"/>
+      <c r="H3" s="402"/>
       <c r="I3" s="75" t="s">
         <v>142</v>
       </c>
-      <c r="J3" s="386"/>
+      <c r="J3" s="402"/>
     </row>
     <row r="4" spans="1:10" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="97"/>
@@ -35504,11 +35504,11 @@
       <c r="G4" s="75" t="s">
         <v>94</v>
       </c>
-      <c r="H4" s="386"/>
+      <c r="H4" s="402"/>
       <c r="I4" s="75" t="s">
         <v>93</v>
       </c>
-      <c r="J4" s="386"/>
+      <c r="J4" s="402"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="91" t="s">
@@ -35929,7 +35929,7 @@
       <c r="P2" s="277" t="s">
         <v>38</v>
       </c>
-      <c r="Q2" s="389" t="s">
+      <c r="Q2" s="405" t="s">
         <v>271</v>
       </c>
     </row>
@@ -35970,7 +35970,7 @@
       <c r="P3" s="277" t="s">
         <v>278</v>
       </c>
-      <c r="Q3" s="389"/>
+      <c r="Q3" s="405"/>
     </row>
     <row r="4" spans="1:62" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="278"/>
@@ -35989,37 +35989,37 @@
       <c r="F4" s="355" t="s">
         <v>109</v>
       </c>
-      <c r="G4" s="408" t="s">
+      <c r="G4" s="360" t="s">
         <v>614</v>
       </c>
-      <c r="H4" s="408" t="s">
+      <c r="H4" s="360" t="s">
         <v>615</v>
       </c>
-      <c r="I4" s="408" t="s">
+      <c r="I4" s="360" t="s">
         <v>616</v>
       </c>
-      <c r="J4" s="408" t="s">
+      <c r="J4" s="360" t="s">
         <v>93</v>
       </c>
-      <c r="K4" s="408" t="s">
+      <c r="K4" s="360" t="s">
         <v>617</v>
       </c>
-      <c r="L4" s="408" t="s">
+      <c r="L4" s="360" t="s">
         <v>618</v>
       </c>
-      <c r="M4" s="408" t="s">
+      <c r="M4" s="360" t="s">
         <v>619</v>
       </c>
-      <c r="N4" s="408" t="s">
+      <c r="N4" s="360" t="s">
         <v>620</v>
       </c>
-      <c r="O4" s="408" t="s">
+      <c r="O4" s="360" t="s">
         <v>621</v>
       </c>
-      <c r="P4" s="408" t="s">
+      <c r="P4" s="360" t="s">
         <v>622</v>
       </c>
-      <c r="Q4" s="389"/>
+      <c r="Q4" s="405"/>
     </row>
     <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="281" t="s">
@@ -36997,7 +36997,7 @@
       <c r="F17" s="291"/>
       <c r="G17" s="291"/>
       <c r="H17" s="291"/>
-      <c r="I17" s="413" t="s">
+      <c r="I17" s="365" t="s">
         <v>626</v>
       </c>
       <c r="J17" s="290"/>
@@ -37018,7 +37018,7 @@
       <c r="F18" s="291"/>
       <c r="G18" s="291"/>
       <c r="H18" s="291"/>
-      <c r="I18" s="413" t="s">
+      <c r="I18" s="365" t="s">
         <v>627</v>
       </c>
       <c r="J18" s="290"/>

</xml_diff>

<commit_message>
update gaps condition for TJ extractor
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1408546-923B-464B-9BAC-DB85FD1D9A2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A9A3B61-4C4A-7C4E-91AA-DFD07D02FBFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -3626,21 +3626,6 @@
     <t>ETPT_ATTACHES_JUSTICE_DDG</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">                  Extracteur de données d'effectifs - Format DDG (avec réintégration de l'absentéisme)
-                  </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri (Corps)"/>
-      </rPr>
-      <t>Les lignes en rouge invitent à des vérifications dans les colonnes Q, R et S</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">                     Agrégats DDG</t>
   </si>
   <si>
@@ -13482,6 +13467,21 @@
   </si>
   <si>
     <t xml:space="preserve">                 DÉCLARATION ETPT TJ</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">                  Extracteur de données d'effectifs - Format DDG (avec réintégration de l'absentéisme)
+                  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri (Corps)"/>
+      </rPr>
+      <t>Les lignes en rouge invitent à des vérifications dans les colonnes R, S et T</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -16255,6 +16255,26 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill>
           <fgColor theme="5" tint="0.79998168889431442"/>
@@ -16273,26 +16293,6 @@
       <font>
         <color theme="0"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -17440,7 +17440,7 @@
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
       <c r="D1" s="3" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="E1" s="7"/>
       <c r="F1" s="6"/>
@@ -17835,7 +17835,7 @@
         <v>106</v>
       </c>
       <c r="K4" s="74" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="L4" s="74" t="s">
         <v>104</v>
@@ -17900,7 +17900,7 @@
       </c>
       <c r="AG4" s="402"/>
       <c r="AH4" s="73" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="AI4" s="73" t="s">
         <v>83</v>
@@ -17946,16 +17946,16 @@
         <v>70</v>
       </c>
       <c r="AX4" s="72" t="s">
+        <v>608</v>
+      </c>
+      <c r="AY4" s="72" t="s">
         <v>609</v>
       </c>
-      <c r="AY4" s="72" t="s">
+      <c r="AZ4" s="72" t="s">
         <v>610</v>
       </c>
-      <c r="AZ4" s="72" t="s">
+      <c r="BA4" s="72" t="s">
         <v>611</v>
-      </c>
-      <c r="BA4" s="72" t="s">
-        <v>612</v>
       </c>
       <c r="BB4" s="72" t="s">
         <v>65</v>
@@ -20562,7 +20562,7 @@
     </row>
     <row r="22" spans="4:57" ht="69" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="E22" s="406" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="F22" s="407"/>
       <c r="G22" s="407"/>
@@ -20620,7 +20620,7 @@
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
       <c r="D1" s="3" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="E1" s="7"/>
       <c r="F1" s="6"/>
@@ -20720,7 +20720,7 @@
         <v>183</v>
       </c>
       <c r="R2" s="360" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="S2" s="359" t="s">
         <v>166</v>
@@ -20732,7 +20732,7 @@
         <v>181</v>
       </c>
       <c r="V2" s="360" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="W2" s="360" t="s">
         <v>179</v>
@@ -20756,7 +20756,7 @@
         <v>213</v>
       </c>
       <c r="AD2" s="360" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="AE2" s="360" t="s">
         <v>78</v>
@@ -20809,7 +20809,7 @@
         <v>183</v>
       </c>
       <c r="R3" s="360" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="S3" s="359" t="s">
         <v>166</v>
@@ -20821,7 +20821,7 @@
         <v>181</v>
       </c>
       <c r="V3" s="360" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="W3" s="360" t="s">
         <v>179</v>
@@ -20845,7 +20845,7 @@
         <v>213</v>
       </c>
       <c r="AD3" s="360" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="AE3" s="360" t="s">
         <v>78</v>
@@ -20908,7 +20908,7 @@
         <v>183</v>
       </c>
       <c r="R4" s="360" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="S4" s="359" t="s">
         <v>166</v>
@@ -20920,7 +20920,7 @@
         <v>181</v>
       </c>
       <c r="V4" s="360" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="W4" s="360" t="s">
         <v>179</v>
@@ -20944,7 +20944,7 @@
         <v>213</v>
       </c>
       <c r="AD4" s="360" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="AE4" s="360" t="s">
         <v>78</v>
@@ -22538,7 +22538,7 @@
     </row>
     <row r="21" spans="4:33" ht="50" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="E21" s="409" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="F21" s="410"/>
       <c r="G21" s="410"/>
@@ -22596,7 +22596,7 @@
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
       <c r="D1" s="3" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="E1" s="7"/>
       <c r="F1" s="6"/>
@@ -22958,7 +22958,7 @@
     </row>
     <row r="17" spans="4:10" ht="99" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D17" s="412" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E17" s="413"/>
       <c r="F17" s="413"/>
@@ -22996,7 +22996,7 @@
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
       <c r="D1" s="3" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="E1" s="7"/>
       <c r="F1" s="6"/>
@@ -23155,34 +23155,34 @@
         <v>109</v>
       </c>
       <c r="G4" s="360" t="s">
+        <v>613</v>
+      </c>
+      <c r="H4" s="360" t="s">
         <v>614</v>
       </c>
-      <c r="H4" s="360" t="s">
+      <c r="I4" s="360" t="s">
         <v>615</v>
-      </c>
-      <c r="I4" s="360" t="s">
-        <v>616</v>
       </c>
       <c r="J4" s="360" t="s">
         <v>93</v>
       </c>
       <c r="K4" s="360" t="s">
+        <v>616</v>
+      </c>
+      <c r="L4" s="360" t="s">
         <v>617</v>
       </c>
-      <c r="L4" s="360" t="s">
+      <c r="M4" s="360" t="s">
         <v>618</v>
       </c>
-      <c r="M4" s="360" t="s">
+      <c r="N4" s="360" t="s">
         <v>619</v>
       </c>
-      <c r="N4" s="360" t="s">
+      <c r="O4" s="360" t="s">
         <v>620</v>
       </c>
-      <c r="O4" s="360" t="s">
+      <c r="P4" s="360" t="s">
         <v>621</v>
-      </c>
-      <c r="P4" s="360" t="s">
-        <v>622</v>
       </c>
       <c r="Q4" s="405"/>
     </row>
@@ -24447,10 +24447,10 @@
         <v>61</v>
       </c>
       <c r="G5" s="152" t="s">
+        <v>494</v>
+      </c>
+      <c r="H5" s="152" t="s">
         <v>495</v>
-      </c>
-      <c r="H5" s="152" t="s">
-        <v>496</v>
       </c>
       <c r="I5" s="154"/>
       <c r="J5" s="154"/>
@@ -24458,10 +24458,10 @@
       <c r="L5" s="154"/>
       <c r="M5" s="155"/>
       <c r="N5" s="152" t="s">
+        <v>496</v>
+      </c>
+      <c r="O5" s="152" t="s">
         <v>497</v>
-      </c>
-      <c r="O5" s="152" t="s">
-        <v>498</v>
       </c>
       <c r="P5" s="153">
         <f>SUMIF($G$2:O$2,O$2,$G5:O5)</f>
@@ -24474,25 +24474,25 @@
       <c r="U5" s="154"/>
       <c r="V5" s="154"/>
       <c r="W5" s="325" t="s">
+        <v>498</v>
+      </c>
+      <c r="X5" s="325" t="s">
         <v>499</v>
       </c>
-      <c r="X5" s="325" t="s">
+      <c r="Y5" s="325" t="s">
         <v>500</v>
       </c>
-      <c r="Y5" s="325" t="s">
+      <c r="Z5" s="325" t="s">
         <v>501</v>
       </c>
-      <c r="Z5" s="325" t="s">
+      <c r="AA5" s="325" t="s">
         <v>502</v>
       </c>
-      <c r="AA5" s="325" t="s">
+      <c r="AB5" s="325" t="s">
         <v>503</v>
       </c>
-      <c r="AB5" s="325" t="s">
+      <c r="AC5" s="325" t="s">
         <v>504</v>
-      </c>
-      <c r="AC5" s="325" t="s">
-        <v>505</v>
       </c>
       <c r="AD5" s="153">
         <f>SUMIF($G$2:AC$2,Y$2,$G5:AC5)</f>
@@ -24538,47 +24538,47 @@
       <c r="G6" s="154"/>
       <c r="H6" s="154"/>
       <c r="I6" s="152" t="s">
+        <v>505</v>
+      </c>
+      <c r="J6" s="152" t="s">
         <v>506</v>
       </c>
-      <c r="J6" s="152" t="s">
+      <c r="K6" s="152" t="s">
         <v>507</v>
       </c>
-      <c r="K6" s="152" t="s">
+      <c r="L6" s="341" t="s">
         <v>508</v>
       </c>
-      <c r="L6" s="341" t="s">
+      <c r="M6" s="152" t="s">
         <v>509</v>
       </c>
-      <c r="M6" s="152" t="s">
+      <c r="N6" s="152" t="s">
         <v>510</v>
       </c>
-      <c r="N6" s="152" t="s">
+      <c r="O6" s="152" t="s">
         <v>511</v>
-      </c>
-      <c r="O6" s="152" t="s">
-        <v>512</v>
       </c>
       <c r="P6" s="153">
         <f>SUMIF($G$2:O$2,O$2,$G6:O6)</f>
         <v>0</v>
       </c>
       <c r="Q6" s="325" t="s">
+        <v>512</v>
+      </c>
+      <c r="R6" s="325" t="s">
         <v>513</v>
       </c>
-      <c r="R6" s="325" t="s">
+      <c r="S6" s="342" t="s">
         <v>514</v>
       </c>
-      <c r="S6" s="342" t="s">
+      <c r="T6" s="325" t="s">
         <v>515</v>
       </c>
-      <c r="T6" s="325" t="s">
+      <c r="U6" s="343" t="s">
         <v>516</v>
       </c>
-      <c r="U6" s="343" t="s">
+      <c r="V6" s="325" t="s">
         <v>517</v>
-      </c>
-      <c r="V6" s="325" t="s">
-        <v>518</v>
       </c>
       <c r="W6" s="154"/>
       <c r="X6" s="154"/>
@@ -24586,10 +24586,10 @@
       <c r="Z6" s="154"/>
       <c r="AA6" s="154"/>
       <c r="AB6" s="325" t="s">
+        <v>518</v>
+      </c>
+      <c r="AC6" s="325" t="s">
         <v>519</v>
-      </c>
-      <c r="AC6" s="325" t="s">
-        <v>520</v>
       </c>
       <c r="AD6" s="153">
         <f>SUMIF($G$2:AC$2,Y$2,$G6:AC6)</f>
@@ -24634,22 +24634,22 @@
       </c>
       <c r="G7" s="158"/>
       <c r="H7" s="152" t="s">
+        <v>520</v>
+      </c>
+      <c r="I7" s="152" t="s">
         <v>521</v>
-      </c>
-      <c r="I7" s="152" t="s">
-        <v>522</v>
       </c>
       <c r="J7" s="158"/>
       <c r="K7" s="158"/>
       <c r="L7" s="158"/>
       <c r="M7" s="152" t="s">
+        <v>522</v>
+      </c>
+      <c r="N7" s="152" t="s">
         <v>523</v>
       </c>
-      <c r="N7" s="152" t="s">
+      <c r="O7" s="152" t="s">
         <v>524</v>
-      </c>
-      <c r="O7" s="152" t="s">
-        <v>525</v>
       </c>
       <c r="P7" s="153">
         <f>SUMIF($G$2:O$2,O$2,$G7:O7)</f>
@@ -24668,7 +24668,7 @@
       <c r="AA7" s="158"/>
       <c r="AB7" s="158"/>
       <c r="AC7" s="152" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="AD7" s="153">
         <f>SUMIF($G$2:AC$2,Y$2,$G7:AC7)</f>
@@ -24713,22 +24713,22 @@
       </c>
       <c r="G8" s="344"/>
       <c r="H8" s="341" t="s">
+        <v>526</v>
+      </c>
+      <c r="I8" s="341" t="s">
         <v>527</v>
-      </c>
-      <c r="I8" s="341" t="s">
-        <v>528</v>
       </c>
       <c r="J8" s="344"/>
       <c r="K8" s="344"/>
       <c r="L8" s="344"/>
       <c r="M8" s="341" t="s">
+        <v>528</v>
+      </c>
+      <c r="N8" s="341" t="s">
         <v>529</v>
       </c>
-      <c r="N8" s="341" t="s">
+      <c r="O8" s="341" t="s">
         <v>530</v>
-      </c>
-      <c r="O8" s="341" t="s">
-        <v>531</v>
       </c>
       <c r="P8" s="153">
         <f>SUMIF($G$2:O$2,O$2,$G8:O8)</f>
@@ -24747,7 +24747,7 @@
       <c r="AA8" s="165"/>
       <c r="AB8" s="165"/>
       <c r="AC8" s="341" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="AD8" s="153">
         <f>SUMIF($G$2:AC$2,Y$2,$G8:AC8)</f>
@@ -24792,22 +24792,22 @@
       </c>
       <c r="G9" s="160"/>
       <c r="H9" s="325" t="s">
+        <v>532</v>
+      </c>
+      <c r="I9" s="325" t="s">
         <v>533</v>
-      </c>
-      <c r="I9" s="325" t="s">
-        <v>534</v>
       </c>
       <c r="J9" s="161"/>
       <c r="K9" s="161"/>
       <c r="L9" s="161"/>
       <c r="M9" s="325" t="s">
+        <v>534</v>
+      </c>
+      <c r="N9" s="325" t="s">
         <v>535</v>
       </c>
-      <c r="N9" s="325" t="s">
+      <c r="O9" s="325" t="s">
         <v>536</v>
-      </c>
-      <c r="O9" s="325" t="s">
-        <v>537</v>
       </c>
       <c r="P9" s="162">
         <f>SUMIF($G$2:O$2,O$2,$G9:O9)</f>
@@ -24826,7 +24826,7 @@
       <c r="AA9" s="158"/>
       <c r="AB9" s="158"/>
       <c r="AC9" s="325" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="AD9" s="153">
         <f>SUMIF($G$2:AC$2,Y$2,$G9:AC9)</f>
@@ -24871,22 +24871,22 @@
       </c>
       <c r="G10" s="160"/>
       <c r="H10" s="152" t="s">
+        <v>538</v>
+      </c>
+      <c r="I10" s="152" t="s">
         <v>539</v>
-      </c>
-      <c r="I10" s="152" t="s">
-        <v>540</v>
       </c>
       <c r="J10" s="161"/>
       <c r="K10" s="161"/>
       <c r="L10" s="161"/>
       <c r="M10" s="152" t="s">
+        <v>540</v>
+      </c>
+      <c r="N10" s="152" t="s">
         <v>541</v>
       </c>
-      <c r="N10" s="152" t="s">
+      <c r="O10" s="152" t="s">
         <v>542</v>
-      </c>
-      <c r="O10" s="152" t="s">
-        <v>543</v>
       </c>
       <c r="P10" s="162">
         <f>SUMIF($G$2:O$2,O$2,$G10:O10)</f>
@@ -24905,7 +24905,7 @@
       <c r="AA10" s="158"/>
       <c r="AB10" s="158"/>
       <c r="AC10" s="152" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="AD10" s="153">
         <f>SUMIF($G$2:AC$2,Y$2,$G10:AC10)</f>
@@ -24950,22 +24950,22 @@
       </c>
       <c r="G11" s="160"/>
       <c r="H11" s="152" t="s">
+        <v>544</v>
+      </c>
+      <c r="I11" s="152" t="s">
         <v>545</v>
-      </c>
-      <c r="I11" s="152" t="s">
-        <v>546</v>
       </c>
       <c r="J11" s="161"/>
       <c r="K11" s="161"/>
       <c r="L11" s="161"/>
       <c r="M11" s="152" t="s">
+        <v>546</v>
+      </c>
+      <c r="N11" s="152" t="s">
         <v>547</v>
       </c>
-      <c r="N11" s="152" t="s">
+      <c r="O11" s="152" t="s">
         <v>548</v>
-      </c>
-      <c r="O11" s="152" t="s">
-        <v>549</v>
       </c>
       <c r="P11" s="162">
         <f>SUMIF($G$2:O$2,O$2,$G11:O11)</f>
@@ -24984,7 +24984,7 @@
       <c r="AA11" s="158"/>
       <c r="AB11" s="158"/>
       <c r="AC11" s="152" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="AD11" s="153">
         <f>SUMIF($G$2:AC$2,Y$2,$G11:AC11)</f>
@@ -25029,22 +25029,22 @@
       </c>
       <c r="G12" s="160"/>
       <c r="H12" s="325" t="s">
+        <v>550</v>
+      </c>
+      <c r="I12" s="325" t="s">
         <v>551</v>
-      </c>
-      <c r="I12" s="325" t="s">
-        <v>552</v>
       </c>
       <c r="J12" s="161"/>
       <c r="K12" s="161"/>
       <c r="L12" s="161"/>
       <c r="M12" s="325" t="s">
+        <v>552</v>
+      </c>
+      <c r="N12" s="325" t="s">
         <v>553</v>
       </c>
-      <c r="N12" s="325" t="s">
+      <c r="O12" s="325" t="s">
         <v>554</v>
-      </c>
-      <c r="O12" s="325" t="s">
-        <v>555</v>
       </c>
       <c r="P12" s="162">
         <f>SUMIF($G$2:O$2,O$2,$G12:O12)</f>
@@ -25063,7 +25063,7 @@
       <c r="AA12" s="158"/>
       <c r="AB12" s="158"/>
       <c r="AC12" s="325" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="AD12" s="153">
         <f>SUMIF($G$2:AC$2,Y$2,$G12:AC12)</f>
@@ -25108,22 +25108,22 @@
       </c>
       <c r="G13" s="163"/>
       <c r="H13" s="325" t="s">
+        <v>556</v>
+      </c>
+      <c r="I13" s="325" t="s">
         <v>557</v>
-      </c>
-      <c r="I13" s="325" t="s">
-        <v>558</v>
       </c>
       <c r="J13" s="161"/>
       <c r="K13" s="161"/>
       <c r="L13" s="161"/>
       <c r="M13" s="325" t="s">
+        <v>558</v>
+      </c>
+      <c r="N13" s="325" t="s">
         <v>559</v>
       </c>
-      <c r="N13" s="325" t="s">
+      <c r="O13" s="325" t="s">
         <v>560</v>
-      </c>
-      <c r="O13" s="325" t="s">
-        <v>561</v>
       </c>
       <c r="P13" s="153">
         <f>SUMIF($G$2:O$2,O$2,$G13:O13)</f>
@@ -25141,10 +25141,10 @@
       <c r="Z13" s="158"/>
       <c r="AA13" s="158"/>
       <c r="AB13" s="325" t="s">
+        <v>561</v>
+      </c>
+      <c r="AC13" s="325" t="s">
         <v>562</v>
-      </c>
-      <c r="AC13" s="325" t="s">
-        <v>563</v>
       </c>
       <c r="AD13" s="153">
         <f>SUMIF($G$2:AC$2,Y$2,$G13:AC13)</f>
@@ -25188,72 +25188,72 @@
         <v>43</v>
       </c>
       <c r="G14" s="152" t="s">
+        <v>563</v>
+      </c>
+      <c r="H14" s="152" t="s">
         <v>564</v>
       </c>
-      <c r="H14" s="152" t="s">
+      <c r="I14" s="152" t="s">
         <v>565</v>
       </c>
-      <c r="I14" s="152" t="s">
+      <c r="J14" s="152" t="s">
         <v>566</v>
       </c>
-      <c r="J14" s="152" t="s">
+      <c r="K14" s="152" t="s">
         <v>567</v>
       </c>
-      <c r="K14" s="152" t="s">
+      <c r="L14" s="341" t="s">
         <v>568</v>
       </c>
-      <c r="L14" s="341" t="s">
+      <c r="M14" s="152" t="s">
         <v>569</v>
       </c>
-      <c r="M14" s="152" t="s">
+      <c r="N14" s="152" t="s">
         <v>570</v>
       </c>
-      <c r="N14" s="152" t="s">
+      <c r="O14" s="152" t="s">
         <v>571</v>
-      </c>
-      <c r="O14" s="152" t="s">
-        <v>572</v>
       </c>
       <c r="P14" s="153">
         <f>SUMIF($G$2:O$2,O$2,$G14:O14)</f>
         <v>0</v>
       </c>
       <c r="Q14" s="325" t="s">
+        <v>572</v>
+      </c>
+      <c r="R14" s="325" t="s">
         <v>573</v>
       </c>
-      <c r="R14" s="325" t="s">
+      <c r="S14" s="342" t="s">
         <v>574</v>
       </c>
-      <c r="S14" s="342" t="s">
+      <c r="T14" s="325" t="s">
         <v>575</v>
       </c>
-      <c r="T14" s="325" t="s">
+      <c r="U14" s="343" t="s">
         <v>576</v>
       </c>
-      <c r="U14" s="343" t="s">
+      <c r="V14" s="325" t="s">
         <v>577</v>
       </c>
-      <c r="V14" s="325" t="s">
+      <c r="W14" s="325" t="s">
         <v>578</v>
       </c>
-      <c r="W14" s="325" t="s">
+      <c r="X14" s="325" t="s">
         <v>579</v>
       </c>
-      <c r="X14" s="325" t="s">
+      <c r="Y14" s="325" t="s">
         <v>580</v>
       </c>
-      <c r="Y14" s="325" t="s">
+      <c r="Z14" s="325" t="s">
         <v>581</v>
       </c>
-      <c r="Z14" s="325" t="s">
+      <c r="AA14" s="325" t="s">
         <v>582</v>
-      </c>
-      <c r="AA14" s="325" t="s">
-        <v>583</v>
       </c>
       <c r="AB14" s="165"/>
       <c r="AC14" s="341" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="AD14" s="153">
         <f>SUMIF($G$2:AC$2,Y$2,$G14:AC14)</f>
@@ -25297,72 +25297,72 @@
         <v>40</v>
       </c>
       <c r="G15" s="152" t="s">
+        <v>584</v>
+      </c>
+      <c r="H15" s="152" t="s">
         <v>585</v>
       </c>
-      <c r="H15" s="152" t="s">
+      <c r="I15" s="152" t="s">
         <v>586</v>
       </c>
-      <c r="I15" s="152" t="s">
+      <c r="J15" s="152" t="s">
         <v>587</v>
       </c>
-      <c r="J15" s="152" t="s">
+      <c r="K15" s="152" t="s">
         <v>588</v>
       </c>
-      <c r="K15" s="152" t="s">
+      <c r="L15" s="341" t="s">
         <v>589</v>
       </c>
-      <c r="L15" s="341" t="s">
+      <c r="M15" s="152" t="s">
         <v>590</v>
       </c>
-      <c r="M15" s="152" t="s">
+      <c r="N15" s="152" t="s">
         <v>591</v>
       </c>
-      <c r="N15" s="152" t="s">
+      <c r="O15" s="152" t="s">
         <v>592</v>
-      </c>
-      <c r="O15" s="152" t="s">
-        <v>593</v>
       </c>
       <c r="P15" s="153">
         <f>SUMIF($G$2:O$2,O$2,$G15:O15)</f>
         <v>0</v>
       </c>
       <c r="Q15" s="325" t="s">
+        <v>593</v>
+      </c>
+      <c r="R15" s="325" t="s">
         <v>594</v>
       </c>
-      <c r="R15" s="325" t="s">
+      <c r="S15" s="342" t="s">
         <v>595</v>
       </c>
-      <c r="S15" s="342" t="s">
+      <c r="T15" s="325" t="s">
         <v>596</v>
       </c>
-      <c r="T15" s="325" t="s">
+      <c r="U15" s="343" t="s">
         <v>597</v>
       </c>
-      <c r="U15" s="343" t="s">
+      <c r="V15" s="325" t="s">
         <v>598</v>
       </c>
-      <c r="V15" s="325" t="s">
+      <c r="W15" s="325" t="s">
         <v>599</v>
       </c>
-      <c r="W15" s="325" t="s">
+      <c r="X15" s="325" t="s">
         <v>600</v>
       </c>
-      <c r="X15" s="325" t="s">
+      <c r="Y15" s="325" t="s">
         <v>601</v>
       </c>
-      <c r="Y15" s="325" t="s">
+      <c r="Z15" s="325" t="s">
         <v>602</v>
       </c>
-      <c r="Z15" s="325" t="s">
+      <c r="AA15" s="325" t="s">
         <v>603</v>
-      </c>
-      <c r="AA15" s="325" t="s">
-        <v>604</v>
       </c>
       <c r="AB15" s="165"/>
       <c r="AC15" s="341" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="AD15" s="153">
         <f>SUMIF($G$2:AC$2,Y$2,$G15:AC15)</f>
@@ -25677,7 +25677,7 @@
         <v>249</v>
       </c>
       <c r="AC19" s="325" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="AD19" s="346"/>
       <c r="AE19" s="251"/>
@@ -26257,37 +26257,37 @@
       </c>
       <c r="G5" s="324"/>
       <c r="H5" s="325" t="s">
+        <v>465</v>
+      </c>
+      <c r="I5" s="325" t="s">
         <v>466</v>
       </c>
-      <c r="I5" s="325" t="s">
+      <c r="J5" s="325" t="s">
         <v>467</v>
       </c>
-      <c r="J5" s="325" t="s">
+      <c r="K5" s="326" t="s">
         <v>468</v>
       </c>
-      <c r="K5" s="326" t="s">
-        <v>469</v>
-      </c>
       <c r="L5" s="326" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="M5" s="177"/>
       <c r="N5" s="177"/>
       <c r="O5" s="326" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="P5" s="327">
         <f t="shared" ref="P5:P15" si="0">SUM(G5:O5)</f>
         <v>0</v>
       </c>
       <c r="Q5" s="326" t="s">
+        <v>469</v>
+      </c>
+      <c r="R5" s="325" t="s">
         <v>470</v>
       </c>
-      <c r="R5" s="325" t="s">
+      <c r="S5" s="328" t="s">
         <v>471</v>
-      </c>
-      <c r="S5" s="328" t="s">
-        <v>472</v>
       </c>
       <c r="T5" s="327">
         <f t="shared" ref="T5:T15" si="1">SUM(Q5:S5)</f>
@@ -26314,20 +26314,20 @@
       <c r="K6" s="331"/>
       <c r="L6" s="331"/>
       <c r="M6" s="326" t="s">
+        <v>472</v>
+      </c>
+      <c r="N6" s="326" t="s">
         <v>473</v>
       </c>
-      <c r="N6" s="326" t="s">
-        <v>474</v>
-      </c>
       <c r="O6" s="326" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="P6" s="327">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q6" s="326" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="R6" s="331"/>
       <c r="S6" s="177"/>
@@ -26365,7 +26365,7 @@
       <c r="Q7" s="331"/>
       <c r="R7" s="331"/>
       <c r="S7" s="325" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="T7" s="327">
         <f>SUM(Q7:S7)</f>
@@ -26401,7 +26401,7 @@
       <c r="Q8" s="334"/>
       <c r="R8" s="164"/>
       <c r="S8" s="325" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="T8" s="327">
         <f>SUM(Q8:R8)</f>
@@ -26437,7 +26437,7 @@
       <c r="Q9" s="334"/>
       <c r="R9" s="164"/>
       <c r="S9" s="325" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="T9" s="327">
         <f>SUM(Q9:R9)</f>
@@ -26473,7 +26473,7 @@
       <c r="Q10" s="334"/>
       <c r="R10" s="334"/>
       <c r="S10" s="325" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="T10" s="327">
         <f t="shared" si="1"/>
@@ -26509,7 +26509,7 @@
       <c r="Q11" s="334"/>
       <c r="R11" s="164"/>
       <c r="S11" s="325" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="T11" s="327">
         <f>SUM(Q11:R11)</f>
@@ -26545,7 +26545,7 @@
       <c r="Q12" s="334"/>
       <c r="R12" s="334"/>
       <c r="S12" s="325" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="T12" s="327">
         <f t="shared" si="1"/>
@@ -26566,7 +26566,7 @@
         <v>45</v>
       </c>
       <c r="G13" s="335" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="H13" s="334"/>
       <c r="I13" s="334"/>
@@ -26583,7 +26583,7 @@
       <c r="Q13" s="334"/>
       <c r="R13" s="334"/>
       <c r="S13" s="325" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="T13" s="327">
         <f t="shared" si="1"/>
@@ -26605,13 +26605,13 @@
       </c>
       <c r="G14" s="324"/>
       <c r="H14" s="325" t="s">
+        <v>483</v>
+      </c>
+      <c r="I14" s="325" t="s">
         <v>484</v>
       </c>
-      <c r="I14" s="325" t="s">
+      <c r="J14" s="325" t="s">
         <v>485</v>
-      </c>
-      <c r="J14" s="325" t="s">
-        <v>486</v>
       </c>
       <c r="K14" s="336"/>
       <c r="L14" s="336"/>
@@ -26624,10 +26624,10 @@
       </c>
       <c r="Q14" s="331"/>
       <c r="R14" s="325" t="s">
+        <v>486</v>
+      </c>
+      <c r="S14" s="325" t="s">
         <v>487</v>
-      </c>
-      <c r="S14" s="325" t="s">
-        <v>488</v>
       </c>
       <c r="T14" s="327">
         <f t="shared" si="1"/>
@@ -26649,13 +26649,13 @@
       </c>
       <c r="G15" s="324"/>
       <c r="H15" s="325" t="s">
+        <v>488</v>
+      </c>
+      <c r="I15" s="325" t="s">
         <v>489</v>
       </c>
-      <c r="I15" s="325" t="s">
+      <c r="J15" s="325" t="s">
         <v>490</v>
-      </c>
-      <c r="J15" s="325" t="s">
-        <v>491</v>
       </c>
       <c r="K15" s="336"/>
       <c r="L15" s="336"/>
@@ -26668,10 +26668,10 @@
       </c>
       <c r="Q15" s="334"/>
       <c r="R15" s="325" t="s">
+        <v>491</v>
+      </c>
+      <c r="S15" s="325" t="s">
         <v>492</v>
-      </c>
-      <c r="S15" s="325" t="s">
-        <v>493</v>
       </c>
       <c r="T15" s="327">
         <f t="shared" si="1"/>
@@ -26810,7 +26810,7 @@
         <v>249</v>
       </c>
       <c r="S19" s="325" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="T19" s="26"/>
     </row>
@@ -27050,14 +27050,14 @@
         <v>61</v>
       </c>
       <c r="G5" s="313" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="H5" s="190">
         <f>SUMIF($G$2:G$2,G$2,$G5:G5)</f>
         <v>0</v>
       </c>
       <c r="I5" s="307" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="J5" s="191"/>
       <c r="K5" s="192"/>
@@ -27066,25 +27066,25 @@
       <c r="N5" s="192"/>
       <c r="O5" s="192"/>
       <c r="P5" s="307" t="s">
+        <v>405</v>
+      </c>
+      <c r="Q5" s="307" t="s">
         <v>406</v>
       </c>
-      <c r="Q5" s="307" t="s">
+      <c r="R5" s="307" t="s">
         <v>407</v>
       </c>
-      <c r="R5" s="307" t="s">
+      <c r="S5" s="307" t="s">
         <v>408</v>
       </c>
-      <c r="S5" s="307" t="s">
+      <c r="T5" s="307" t="s">
         <v>409</v>
       </c>
-      <c r="T5" s="307" t="s">
+      <c r="U5" s="307" t="s">
         <v>410</v>
       </c>
-      <c r="U5" s="307" t="s">
+      <c r="V5" s="313" t="s">
         <v>411</v>
-      </c>
-      <c r="V5" s="313" t="s">
-        <v>412</v>
       </c>
       <c r="W5" s="190">
         <f>SUMIF($G$2:V$2,V$2,$G5:V5)</f>
@@ -27105,7 +27105,7 @@
         <v>59</v>
       </c>
       <c r="G6" s="307" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="H6" s="190">
         <f>SUMIF($G$2:G$2,G$2,$G6:G6)</f>
@@ -27113,33 +27113,33 @@
       </c>
       <c r="I6" s="191"/>
       <c r="J6" s="307" t="s">
+        <v>413</v>
+      </c>
+      <c r="K6" s="307" t="s">
         <v>414</v>
       </c>
-      <c r="K6" s="307" t="s">
+      <c r="L6" s="307" t="s">
         <v>415</v>
       </c>
-      <c r="L6" s="307" t="s">
+      <c r="M6" s="316" t="s">
         <v>416</v>
       </c>
-      <c r="M6" s="316" t="s">
+      <c r="N6" s="307" t="s">
         <v>417</v>
       </c>
-      <c r="N6" s="307" t="s">
+      <c r="O6" s="317" t="s">
         <v>418</v>
-      </c>
-      <c r="O6" s="317" t="s">
-        <v>419</v>
       </c>
       <c r="P6" s="192"/>
       <c r="Q6" s="192"/>
       <c r="R6" s="307" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="S6" s="192"/>
       <c r="T6" s="192"/>
       <c r="U6" s="192"/>
       <c r="V6" s="318" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="W6" s="190">
         <f>SUMIF($G$2:V$2,V$2,$G6:V6)</f>
@@ -27197,7 +27197,7 @@
         <v>55</v>
       </c>
       <c r="G8" s="307" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="H8" s="190">
         <f>SUMIF($G$2:G$2,G$2,$G8:G8)</f>
@@ -27217,7 +27217,7 @@
       <c r="T8" s="194"/>
       <c r="U8" s="194"/>
       <c r="V8" s="307" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="W8" s="190">
         <f>SUMIF($G$2:V$2,V$2,$G8:V8)</f>
@@ -27238,7 +27238,7 @@
         <v>53</v>
       </c>
       <c r="G9" s="307" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="H9" s="190">
         <f>SUMIF($G$2:G$2,G$2,$G9:G9)</f>
@@ -27258,7 +27258,7 @@
       <c r="T9" s="194"/>
       <c r="U9" s="194"/>
       <c r="V9" s="313" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="W9" s="190">
         <f>SUMIF($G$2:V$2,V$2,$G9:V9)</f>
@@ -27279,7 +27279,7 @@
         <v>51</v>
       </c>
       <c r="G10" s="307" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="H10" s="190">
         <f>SUMIF($G$2:G$2,G$2,$G10:G10)</f>
@@ -27298,7 +27298,7 @@
       <c r="T10" s="194"/>
       <c r="U10" s="194"/>
       <c r="V10" s="307" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="W10" s="190">
         <f>SUMIF($G$2:V$2,V$2,$G10:V10)</f>
@@ -27319,7 +27319,7 @@
         <v>49</v>
       </c>
       <c r="G11" s="307" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="H11" s="190">
         <f>SUMIF($G$2:G$2,G$2,$G11:G11)</f>
@@ -27339,7 +27339,7 @@
       <c r="T11" s="194"/>
       <c r="U11" s="194"/>
       <c r="V11" s="307" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="W11" s="190">
         <f>SUMIF($G$2:V$2,V$2,$G11:V11)</f>
@@ -27360,7 +27360,7 @@
         <v>47</v>
       </c>
       <c r="G12" s="307" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="H12" s="190">
         <f>SUMIF($G$2:G$2,G$2,$G12:G12)</f>
@@ -27380,7 +27380,7 @@
       <c r="T12" s="194"/>
       <c r="U12" s="194"/>
       <c r="V12" s="307" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="W12" s="190">
         <f>SUMIF($G$2:V$2,V$2,$G12:V12)</f>
@@ -27401,7 +27401,7 @@
         <v>45</v>
       </c>
       <c r="G13" s="313" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="H13" s="190">
         <f>SUMIF($G$2:G$2,G$2,$G13:G13)</f>
@@ -27421,7 +27421,7 @@
       <c r="T13" s="194"/>
       <c r="U13" s="194"/>
       <c r="V13" s="313" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="W13" s="190">
         <f>SUMIF($G$2:V$2,V$2,$G13:V13)</f>
@@ -27442,53 +27442,53 @@
         <v>43</v>
       </c>
       <c r="G14" s="307" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="H14" s="190">
         <f>SUMIF($G$2:G$2,G$2,$G14:G14)</f>
         <v>0</v>
       </c>
       <c r="I14" s="307" t="s">
+        <v>434</v>
+      </c>
+      <c r="J14" s="313" t="s">
         <v>435</v>
       </c>
-      <c r="J14" s="313" t="s">
+      <c r="K14" s="313" t="s">
         <v>436</v>
       </c>
-      <c r="K14" s="313" t="s">
+      <c r="L14" s="313" t="s">
         <v>437</v>
       </c>
-      <c r="L14" s="313" t="s">
+      <c r="M14" s="316" t="s">
         <v>438</v>
       </c>
-      <c r="M14" s="316" t="s">
+      <c r="N14" s="313" t="s">
         <v>439</v>
       </c>
-      <c r="N14" s="313" t="s">
+      <c r="O14" s="317" t="s">
         <v>440</v>
       </c>
-      <c r="O14" s="317" t="s">
+      <c r="P14" s="307" t="s">
         <v>441</v>
       </c>
-      <c r="P14" s="307" t="s">
+      <c r="Q14" s="307" t="s">
         <v>442</v>
       </c>
-      <c r="Q14" s="307" t="s">
+      <c r="R14" s="313" t="s">
         <v>443</v>
       </c>
-      <c r="R14" s="313" t="s">
+      <c r="S14" s="307" t="s">
         <v>444</v>
       </c>
-      <c r="S14" s="307" t="s">
+      <c r="T14" s="307" t="s">
         <v>445</v>
       </c>
-      <c r="T14" s="307" t="s">
+      <c r="U14" s="307" t="s">
         <v>446</v>
       </c>
-      <c r="U14" s="307" t="s">
+      <c r="V14" s="313" t="s">
         <v>447</v>
-      </c>
-      <c r="V14" s="313" t="s">
-        <v>448</v>
       </c>
       <c r="W14" s="190">
         <f>SUMIF($G$2:V$2,V$2,$G14:V14)</f>
@@ -27509,53 +27509,53 @@
         <v>40</v>
       </c>
       <c r="G15" s="307" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="H15" s="190">
         <f>SUMIF($G$2:G$2,G$2,$G15:G15)</f>
         <v>0</v>
       </c>
       <c r="I15" s="307" t="s">
+        <v>449</v>
+      </c>
+      <c r="J15" s="313" t="s">
         <v>450</v>
       </c>
-      <c r="J15" s="313" t="s">
+      <c r="K15" s="313" t="s">
         <v>451</v>
       </c>
-      <c r="K15" s="313" t="s">
+      <c r="L15" s="313" t="s">
         <v>452</v>
       </c>
-      <c r="L15" s="313" t="s">
+      <c r="M15" s="316" t="s">
         <v>453</v>
       </c>
-      <c r="M15" s="316" t="s">
+      <c r="N15" s="313" t="s">
         <v>454</v>
       </c>
-      <c r="N15" s="313" t="s">
+      <c r="O15" s="317" t="s">
         <v>455</v>
       </c>
-      <c r="O15" s="317" t="s">
+      <c r="P15" s="307" t="s">
         <v>456</v>
       </c>
-      <c r="P15" s="307" t="s">
+      <c r="Q15" s="307" t="s">
         <v>457</v>
       </c>
-      <c r="Q15" s="307" t="s">
+      <c r="R15" s="313" t="s">
         <v>458</v>
       </c>
-      <c r="R15" s="313" t="s">
+      <c r="S15" s="307" t="s">
         <v>459</v>
       </c>
-      <c r="S15" s="307" t="s">
+      <c r="T15" s="307" t="s">
         <v>460</v>
       </c>
-      <c r="T15" s="307" t="s">
+      <c r="U15" s="307" t="s">
         <v>461</v>
       </c>
-      <c r="U15" s="307" t="s">
+      <c r="V15" s="313" t="s">
         <v>462</v>
-      </c>
-      <c r="V15" s="313" t="s">
-        <v>463</v>
       </c>
       <c r="W15" s="190">
         <f>SUMIF($G$2:V$2,V$2,$G15:V15)</f>
@@ -27697,7 +27697,7 @@
         <v>250</v>
       </c>
       <c r="G19" s="307" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="H19" s="254"/>
       <c r="I19" s="254"/>
@@ -27716,7 +27716,7 @@
         <v>251</v>
       </c>
       <c r="V19" s="307" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="W19" s="254"/>
     </row>
@@ -27921,7 +27921,7 @@
         <v>61</v>
       </c>
       <c r="G5" s="307" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="H5" s="228">
         <f t="shared" ref="H5:H15" si="0">SUM(G5)</f>
@@ -27929,27 +27929,27 @@
       </c>
       <c r="I5" s="229"/>
       <c r="J5" s="307" t="s">
+        <v>373</v>
+      </c>
+      <c r="K5" s="307" t="s">
         <v>374</v>
       </c>
-      <c r="K5" s="307" t="s">
+      <c r="L5" s="307" t="s">
         <v>375</v>
       </c>
-      <c r="L5" s="307" t="s">
+      <c r="M5" s="308" t="s">
         <v>376</v>
       </c>
-      <c r="M5" s="308" t="s">
-        <v>377</v>
-      </c>
       <c r="N5" s="308" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="O5" s="309"/>
       <c r="P5" s="309"/>
       <c r="Q5" s="308" t="s">
+        <v>376</v>
+      </c>
+      <c r="R5" s="307" t="s">
         <v>377</v>
-      </c>
-      <c r="R5" s="307" t="s">
-        <v>378</v>
       </c>
       <c r="S5" s="228">
         <f t="shared" ref="S5:S15" si="1">SUM(I5:R5)</f>
@@ -27981,16 +27981,16 @@
       <c r="M6" s="311"/>
       <c r="N6" s="312"/>
       <c r="O6" s="308" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="P6" s="308" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="Q6" s="308" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="R6" s="308" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="S6" s="234">
         <f t="shared" si="1"/>
@@ -28044,7 +28044,7 @@
         <v>55</v>
       </c>
       <c r="G8" s="307" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="H8" s="228">
         <f t="shared" si="0"/>
@@ -28060,7 +28060,7 @@
       <c r="P8" s="231"/>
       <c r="Q8" s="232"/>
       <c r="R8" s="307" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="S8" s="228">
         <f t="shared" si="1"/>
@@ -28081,7 +28081,7 @@
         <v>53</v>
       </c>
       <c r="G9" s="307" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H9" s="228">
         <f t="shared" si="0"/>
@@ -28097,7 +28097,7 @@
       <c r="P9" s="231"/>
       <c r="Q9" s="232"/>
       <c r="R9" s="307" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="S9" s="228">
         <f t="shared" si="1"/>
@@ -28118,7 +28118,7 @@
         <v>51</v>
       </c>
       <c r="G10" s="307" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="H10" s="228">
         <f>SUM(G10)</f>
@@ -28134,7 +28134,7 @@
       <c r="P10" s="231"/>
       <c r="Q10" s="232"/>
       <c r="R10" s="307" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="S10" s="228">
         <f t="shared" si="1"/>
@@ -28155,7 +28155,7 @@
         <v>49</v>
       </c>
       <c r="G11" s="307" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="H11" s="228">
         <f>SUM(G11)</f>
@@ -28171,7 +28171,7 @@
       <c r="P11" s="231"/>
       <c r="Q11" s="232"/>
       <c r="R11" s="307" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="S11" s="228">
         <f t="shared" si="1"/>
@@ -28192,7 +28192,7 @@
         <v>47</v>
       </c>
       <c r="G12" s="307" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="H12" s="228">
         <f t="shared" si="0"/>
@@ -28208,7 +28208,7 @@
       <c r="P12" s="231"/>
       <c r="Q12" s="232"/>
       <c r="R12" s="307" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="S12" s="228">
         <f t="shared" si="1"/>
@@ -28229,14 +28229,14 @@
         <v>45</v>
       </c>
       <c r="G13" s="307" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H13" s="228">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I13" s="313" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="J13" s="232"/>
       <c r="K13" s="232"/>
@@ -28247,7 +28247,7 @@
       <c r="P13" s="231"/>
       <c r="Q13" s="232"/>
       <c r="R13" s="307" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="S13" s="228">
         <f t="shared" si="1"/>
@@ -28268,7 +28268,7 @@
         <v>43</v>
       </c>
       <c r="G14" s="307" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="H14" s="228">
         <f t="shared" si="0"/>
@@ -28276,13 +28276,13 @@
       </c>
       <c r="I14" s="229"/>
       <c r="J14" s="307" t="s">
+        <v>392</v>
+      </c>
+      <c r="K14" s="307" t="s">
         <v>393</v>
       </c>
-      <c r="K14" s="307" t="s">
+      <c r="L14" s="307" t="s">
         <v>394</v>
-      </c>
-      <c r="L14" s="307" t="s">
-        <v>395</v>
       </c>
       <c r="M14" s="230"/>
       <c r="N14" s="230"/>
@@ -28290,7 +28290,7 @@
       <c r="P14" s="231"/>
       <c r="Q14" s="232"/>
       <c r="R14" s="307" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="S14" s="228">
         <f t="shared" si="1"/>
@@ -28311,7 +28311,7 @@
         <v>40</v>
       </c>
       <c r="G15" s="307" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="H15" s="228">
         <f t="shared" si="0"/>
@@ -28319,13 +28319,13 @@
       </c>
       <c r="I15" s="229"/>
       <c r="J15" s="307" t="s">
+        <v>397</v>
+      </c>
+      <c r="K15" s="307" t="s">
         <v>398</v>
       </c>
-      <c r="K15" s="307" t="s">
+      <c r="L15" s="307" t="s">
         <v>399</v>
-      </c>
-      <c r="L15" s="307" t="s">
-        <v>400</v>
       </c>
       <c r="M15" s="230"/>
       <c r="N15" s="230"/>
@@ -28333,7 +28333,7 @@
       <c r="P15" s="231"/>
       <c r="Q15" s="232"/>
       <c r="R15" s="307" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="S15" s="228">
         <f t="shared" si="1"/>
@@ -28456,7 +28456,7 @@
         <v>250</v>
       </c>
       <c r="G19" s="307" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H19" s="258"/>
       <c r="I19" s="258"/>
@@ -28471,7 +28471,7 @@
         <v>251</v>
       </c>
       <c r="R19" s="307" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="S19" s="258"/>
       <c r="T19" s="258"/>
@@ -28614,7 +28614,7 @@
         <v>61</v>
       </c>
       <c r="K5" s="306" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="L5" s="209">
         <f t="shared" ref="L5:L13" si="0">SUM(K5)</f>
@@ -28812,7 +28812,7 @@
         <v>43</v>
       </c>
       <c r="K12" s="306" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="L12" s="209">
         <f t="shared" si="0"/>
@@ -28842,7 +28842,7 @@
         <v>40</v>
       </c>
       <c r="K13" s="306" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="L13" s="209">
         <f t="shared" si="0"/>
@@ -29859,7 +29859,7 @@
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="393" t="s">
-        <v>365</v>
+        <v>630</v>
       </c>
       <c r="E1" s="394"/>
       <c r="F1" s="394"/>
@@ -29916,14 +29916,9 @@
   <mergeCells count="1">
     <mergeCell ref="D1:Q1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A1:D1 R1 T1:EY1">
-    <cfRule type="expression" dxfId="17" priority="19" stopIfTrue="1">
-      <formula>AND(OR($Q1&lt;&gt;"-",#REF!&lt;&gt;0,#REF!&lt;&gt;0),ROW()&gt;2,$A1&lt;&gt;"")</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="A2:EZ2 A3:FB1048576">
-    <cfRule type="expression" dxfId="16" priority="1" stopIfTrue="1">
-      <formula>AND(OR($Q2&lt;&gt;"-",$R2&lt;&gt;0,$S2&lt;&gt;0),ROW()&gt;2,$A2&lt;&gt;"")</formula>
+    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+      <formula>AND(OR($R1&lt;&gt;"-",$S1&lt;&gt;0,$T1&lt;&gt;0),ROW()&gt;2,$A1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -29957,7 +29952,7 @@
   <sheetData>
     <row r="1" spans="1:24" s="4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="128" t="s">
@@ -30248,70 +30243,70 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="15" priority="16">
+    <cfRule type="expression" dxfId="17" priority="16">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="14" priority="18">
+    <cfRule type="expression" dxfId="16" priority="18">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="13" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="15" priority="1" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3)+_xlfn.NUMBERVALUE($U4)+_xlfn.NUMBERVALUE($U5)+_xlfn.NUMBERVALUE($U6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="2" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3)+_xlfn.NUMBERVALUE($S4)+_xlfn.NUMBERVALUE($S5)+_xlfn.NUMBERVALUE($S6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="7" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="12" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="12" stopIfTrue="1">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",OR(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0,_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0,_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="6" stopIfTrue="1">
       <formula>OR(_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6),_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6),_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="8" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="11" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)+_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="15">
+    <cfRule type="expression" dxfId="9" priority="15">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="6" priority="5">
+    <cfRule type="expression" dxfId="8" priority="5">
       <formula>_xlfn.NUMBERVALUE($L7)&lt;&gt;_xlfn.NUMBERVALUE($L6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="5" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="10" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3)+_xlfn.NUMBERVALUE($S4)+_xlfn.NUMBERVALUE($S5)+_xlfn.NUMBERVALUE($S6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="14">
+    <cfRule type="expression" dxfId="6" priority="14">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($S1)-(_xlfn.NUMBERVALUE($S2)+_xlfn.NUMBERVALUE($S3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="5" priority="4">
       <formula>_xlfn.NUMBERVALUE($S7)&lt;&gt;_xlfn.NUMBERVALUE($S6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="2" priority="9">
+    <cfRule type="expression" dxfId="4" priority="9">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3)+_xlfn.NUMBERVALUE($U4)+_xlfn.NUMBERVALUE($U5)+_xlfn.NUMBERVALUE($U6))&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="13">
+    <cfRule type="expression" dxfId="3" priority="13">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",_xlfn.NUMBERVALUE($U1)-(_xlfn.NUMBERVALUE($U2)+_xlfn.NUMBERVALUE($U3))&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>_xlfn.NUMBERVALUE($U7)&lt;&gt;_xlfn.NUMBERVALUE($U6)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -35990,34 +35985,34 @@
         <v>109</v>
       </c>
       <c r="G4" s="360" t="s">
+        <v>613</v>
+      </c>
+      <c r="H4" s="360" t="s">
         <v>614</v>
       </c>
-      <c r="H4" s="360" t="s">
+      <c r="I4" s="360" t="s">
         <v>615</v>
-      </c>
-      <c r="I4" s="360" t="s">
-        <v>616</v>
       </c>
       <c r="J4" s="360" t="s">
         <v>93</v>
       </c>
       <c r="K4" s="360" t="s">
+        <v>616</v>
+      </c>
+      <c r="L4" s="360" t="s">
         <v>617</v>
       </c>
-      <c r="L4" s="360" t="s">
+      <c r="M4" s="360" t="s">
         <v>618</v>
       </c>
-      <c r="M4" s="360" t="s">
+      <c r="N4" s="360" t="s">
         <v>619</v>
       </c>
-      <c r="N4" s="360" t="s">
+      <c r="O4" s="360" t="s">
         <v>620</v>
       </c>
-      <c r="O4" s="360" t="s">
+      <c r="P4" s="360" t="s">
         <v>621</v>
-      </c>
-      <c r="P4" s="360" t="s">
-        <v>622</v>
       </c>
       <c r="Q4" s="405"/>
     </row>
@@ -36998,7 +36993,7 @@
       <c r="G17" s="291"/>
       <c r="H17" s="291"/>
       <c r="I17" s="365" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="J17" s="290"/>
       <c r="L17" s="290"/>
@@ -37019,7 +37014,7 @@
       <c r="G18" s="291"/>
       <c r="H18" s="291"/>
       <c r="I18" s="365" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="J18" s="290"/>
       <c r="L18" s="290"/>

</xml_diff>

<commit_message>
update zoom for tj et ca extractor
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC793514-3200-1142-B289-DAE449AC69D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D163E9F-EF9A-EB49-A9BD-BFEE7DA6ED22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17740" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -18814,807 +18814,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
     <cellStyle name="Normal 3" xfId="4" xr:uid="{6BD57324-3FD5-D341-A299-730D14794802}"/>
   </cellStyles>
-  <dxfs count="97">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="5" tint="0.79998168889431442"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
+  <dxfs count="17">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -20642,7 +19842,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="1.1640625" style="21" customWidth="1"/>
-    <col min="2" max="2" width="27.1640625" style="21" customWidth="1"/>
+    <col min="2" max="2" width="30" style="21" customWidth="1"/>
     <col min="3" max="3" width="102.1640625" style="21" customWidth="1"/>
     <col min="4" max="4" width="56.33203125" style="21" customWidth="1"/>
     <col min="5" max="5" width="14" style="21" customWidth="1"/>
@@ -33465,7 +32665,7 @@
     <mergeCell ref="D1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2:EZ2 A3:FB1048576">
-    <cfRule type="expression" dxfId="96" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="16" priority="1" stopIfTrue="1">
       <formula>AND(OR($R1&lt;&gt;"-",$S1&lt;&gt;0,$T1&lt;&gt;0),ROW()&gt;2,$A1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -33791,70 +32991,70 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="31" priority="16">
+    <cfRule type="expression" dxfId="15" priority="16">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="30" priority="18" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="18" stopIfTrue="1">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="29" priority="1">
+    <cfRule type="expression" dxfId="13" priority="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)-_xlfn.NUMBERVALUE($U6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="28" priority="2">
+    <cfRule type="expression" dxfId="12" priority="2">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)-_xlfn.NUMBERVALUE($S6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="7" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3)-_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)-_xlfn.NUMBERVALUE($L6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="12">
+    <cfRule type="expression" dxfId="10" priority="12">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",OR(ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="25" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
       <formula>OR(ROUND(_xlfn.NUMBERVALUE($L7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($L6),3),ROUND(_xlfn.NUMBERVALUE($S7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($S6),3),ROUND(_xlfn.NUMBERVALUE($U7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($U6),3))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="24" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="8" priority="11" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)+_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6)),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="23" priority="15">
+    <cfRule type="expression" dxfId="7" priority="15">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="22" priority="5">
+    <cfRule type="expression" dxfId="6" priority="5">
       <formula>ROUND(_xlfn.NUMBERVALUE($L7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($L6),3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="21" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="10" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)-_xlfn.NUMBERVALUE($S6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="14">
+    <cfRule type="expression" dxfId="4" priority="14">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="19" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>ROUND(_xlfn.NUMBERVALUE($S7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($S6),3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="17" priority="9">
+    <cfRule type="expression" dxfId="2" priority="9">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)-_xlfn.NUMBERVALUE($U6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="13">
+    <cfRule type="expression" dxfId="1" priority="13">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="18" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="0" priority="3" stopIfTrue="1">
       <formula>ROUND(_xlfn.NUMBERVALUE($U7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($U6),3)</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
update extractor red underline while no etpt
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D163E9F-EF9A-EB49-A9BD-BFEE7DA6ED22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81C1F9DA-37DD-2E45-BE7A-648C2291B142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17740" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -18814,7 +18814,27 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
     <cellStyle name="Normal 3" xfId="4" xr:uid="{6BD57324-3FD5-D341-A299-730D14794802}"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="18">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -18974,16 +18994,6 @@
       <font>
         <color theme="0"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -32665,8 +32675,8 @@
     <mergeCell ref="D1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2:EZ2 A3:FB1048576">
-    <cfRule type="expression" dxfId="16" priority="1" stopIfTrue="1">
-      <formula>AND(OR($R1&lt;&gt;"-",$S1&lt;&gt;0,$T1&lt;&gt;0),ROW()&gt;2,$A1&lt;&gt;"")</formula>
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>AND(OR($R1&lt;&gt;"-",$S1&lt;&gt;0,$T1&lt;&gt;0,ISBLANK($P1)),ROW()&gt;2,$A1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -32991,70 +33001,70 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="15" priority="16">
+    <cfRule type="expression" dxfId="17" priority="16">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="14" priority="18" stopIfTrue="1">
+    <cfRule type="expression" dxfId="16" priority="18" stopIfTrue="1">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="13" priority="1">
+    <cfRule type="expression" dxfId="15" priority="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)-_xlfn.NUMBERVALUE($U6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="2">
+    <cfRule type="expression" dxfId="14" priority="2">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)-_xlfn.NUMBERVALUE($S6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="7" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3)-_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)-_xlfn.NUMBERVALUE($L6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="12">
+    <cfRule type="expression" dxfId="12" priority="12">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",OR(ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="6" stopIfTrue="1">
       <formula>OR(ROUND(_xlfn.NUMBERVALUE($L7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($L6),3),ROUND(_xlfn.NUMBERVALUE($S7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($S6),3),ROUND(_xlfn.NUMBERVALUE($U7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($U6),3))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="8" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="11" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)+_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6)),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="15">
+    <cfRule type="expression" dxfId="9" priority="15">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="6" priority="5">
+    <cfRule type="expression" dxfId="8" priority="5">
       <formula>ROUND(_xlfn.NUMBERVALUE($L7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($L6),3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="5" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="10" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)-_xlfn.NUMBERVALUE($S6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="14">
+    <cfRule type="expression" dxfId="6" priority="14">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="5" priority="4">
       <formula>ROUND(_xlfn.NUMBERVALUE($S7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($S6),3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="2" priority="9">
+    <cfRule type="expression" dxfId="4" priority="9">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)-_xlfn.NUMBERVALUE($U6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="13">
+    <cfRule type="expression" dxfId="3" priority="13">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="0" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="2" priority="3" stopIfTrue="1">
       <formula>ROUND(_xlfn.NUMBERVALUE($U7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($U6),3)</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
update lock for dropdown
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimmychevallier/Documents/GitHub/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{748ECCA0-6141-774D-B98C-4C33A9F8161B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CF57EE2-9FE9-4949-9C0C-EC386BD939CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15720" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -36691,7 +36691,7 @@
       <c r="FA4" s="21"/>
     </row>
   </sheetData>
-  <sheetProtection sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" autoFilter="0"/>
   <autoFilter ref="A2:DT2" xr:uid="{3B89445B-6ECC-4440-B85C-E593AE209933}"/>
   <mergeCells count="1">
     <mergeCell ref="D1:Q1"/>

</xml_diff>

<commit_message>
feat: Update Excel template with new Attaché de Justice formulas
- Add formulas for 3 new recoded functions in ETPT_JUR_ASS tab:
  * JA/AttJ Siege Assises
  * JA/AttJ Siege CCD
  * JA/AttJ JLD PÉNAL

- Update formula arrays to include new function variants
- Ensures proper calculation of ETPT for new Attaché de Justice roles
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-clean/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF0681A9-AC29-A745-9551-49B4DCC99555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F6B9269-C0E1-5A4D-A26F-754C1F2A9340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11060" yWindow="760" windowWidth="30240" windowHeight="17700" firstSheet="4" activeTab="6" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" firstSheet="1" activeTab="9" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -112,7 +112,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1828" uniqueCount="684">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1832" uniqueCount="686">
   <si>
     <t>#! END_ROW</t>
   </si>
@@ -16485,6 +16485,12 @@
       <t xml:space="preserve">
 *figurant dans l'onglet ETPT A-JUST</t>
     </r>
+  </si>
+  <si>
+    <t>Attachés de justice parquet affectés aux assises</t>
+  </si>
+  <si>
+    <t>Attachés de justice parquet affectés aux CDD</t>
   </si>
 </sst>
 </file>
@@ -20544,16 +20550,16 @@
   <sheetPr>
     <tabColor rgb="FF002060"/>
   </sheetPr>
-  <dimension ref="A1:BJ145"/>
+  <dimension ref="A1:BL145"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="10.83203125" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="9.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="73.83203125" customWidth="1"/>
-    <col min="7" max="16" width="13.33203125" customWidth="1"/>
+    <col min="7" max="18" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:62" s="4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:64" s="4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>217</v>
       </c>
@@ -20620,8 +20626,10 @@
       <c r="BH1" s="7"/>
       <c r="BI1" s="7"/>
       <c r="BJ1" s="7"/>
-    </row>
-    <row r="2" spans="1:62" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="BK1" s="7"/>
+      <c r="BL1" s="7"/>
+    </row>
+    <row r="2" spans="1:64" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="206"/>
       <c r="B2" s="207"/>
       <c r="C2" s="207"/>
@@ -20642,23 +20650,25 @@
       <c r="L2" s="208" t="s">
         <v>38</v>
       </c>
-      <c r="M2" s="208" t="s">
-        <v>38</v>
-      </c>
-      <c r="N2" s="208" t="s">
-        <v>38</v>
-      </c>
+      <c r="M2" s="208"/>
+      <c r="N2" s="208"/>
       <c r="O2" s="208" t="s">
         <v>38</v>
       </c>
       <c r="P2" s="208" t="s">
         <v>38</v>
       </c>
-      <c r="Q2" s="418" t="s">
+      <c r="Q2" s="208" t="s">
+        <v>38</v>
+      </c>
+      <c r="R2" s="208" t="s">
+        <v>38</v>
+      </c>
+      <c r="S2" s="418" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="3" spans="1:62" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:64" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="206"/>
       <c r="B3" s="207"/>
       <c r="C3" s="207"/>
@@ -20679,21 +20689,23 @@
       <c r="L3" s="208" t="s">
         <v>144</v>
       </c>
-      <c r="M3" s="208" t="s">
+      <c r="M3" s="208"/>
+      <c r="N3" s="208"/>
+      <c r="O3" s="208" t="s">
         <v>275</v>
       </c>
-      <c r="N3" s="208" t="s">
+      <c r="P3" s="208" t="s">
         <v>276</v>
       </c>
-      <c r="O3" s="208" t="s">
+      <c r="Q3" s="208" t="s">
         <v>277</v>
       </c>
-      <c r="P3" s="208" t="s">
+      <c r="R3" s="208" t="s">
         <v>278</v>
       </c>
-      <c r="Q3" s="418"/>
-    </row>
-    <row r="4" spans="1:62" ht="36" x14ac:dyDescent="0.2">
+      <c r="S3" s="418"/>
+    </row>
+    <row r="4" spans="1:64" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="209"/>
       <c r="B4" s="210" t="s">
         <v>112</v>
@@ -20729,20 +20741,26 @@
         <v>677</v>
       </c>
       <c r="M4" s="249" t="s">
+        <v>684</v>
+      </c>
+      <c r="N4" s="249" t="s">
+        <v>685</v>
+      </c>
+      <c r="O4" s="249" t="s">
         <v>678</v>
       </c>
-      <c r="N4" s="249" t="s">
+      <c r="P4" s="249" t="s">
         <v>679</v>
       </c>
-      <c r="O4" s="249" t="s">
+      <c r="Q4" s="249" t="s">
         <v>680</v>
       </c>
-      <c r="P4" s="249" t="s">
+      <c r="R4" s="249" t="s">
         <v>676</v>
       </c>
-      <c r="Q4" s="418"/>
-    </row>
-    <row r="5" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="S4" s="418"/>
+    </row>
+    <row r="5" spans="1:64" x14ac:dyDescent="0.2">
       <c r="A5" s="211" t="s">
         <v>290</v>
       </c>
@@ -20799,19 +20817,19 @@
       <c r="I5" s="280" t="e" cm="1">
         <f t="array" ref="I5">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("2. TOTAL CONTENTIEUX JAF",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Social"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD";"JA/AttJ Social"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3. TOTAL CONTENTIEUX DE LA PROTECTION",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Social"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD";"JA/AttJ Social"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4. TOTAL CIVIL NON SPÉCIALISÉ",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Social"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD";"JA/AttJ Social"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.7. FONCTIONNAIRES AFFECTÉS AU CPH",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Social"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD";"JA/AttJ Social"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
@@ -20820,26 +20838,28 @@
       <c r="L5" s="280" t="e" cm="1">
         <f t="array" ref="L5">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.8. FONCTIONNAIRES AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Social"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD";"JA/AttJ Social"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
       <c r="M5" s="280"/>
-      <c r="N5" s="280" t="e" cm="1">
-        <f t="array" ref="N5">SUM(SUMIFS(
+      <c r="N5" s="280"/>
+      <c r="O5" s="280"/>
+      <c r="P5" s="280" t="e" cm="1">
+        <f t="array" ref="P5">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("6.1. ACTIVITÉ CIVILE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Social"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD";"JA/AttJ Social"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="O5" s="280"/>
-      <c r="P5" s="280"/>
-      <c r="Q5" s="278">
-        <f>_xlfn.AGGREGATE(9,6,G5:P5)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="Q5" s="280"/>
+      <c r="R5" s="280"/>
+      <c r="S5" s="278">
+        <f>_xlfn.AGGREGATE(9,6,G5:R5)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:64" x14ac:dyDescent="0.2">
       <c r="A6" s="211" t="s">
         <v>290</v>
       </c>
@@ -20892,7 +20912,7 @@
       <c r="I6" s="280" t="e" cm="1">
         <f t="array" ref="I6">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7. TOTAL SIÈGE PÉNAL",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Social"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD";"JA/AttJ Social"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
@@ -20901,48 +20921,50 @@
       <c r="L6" s="280" t="e" cm="1">
         <f t="array" ref="L6">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.9. FONCTIONNAIRES AFFECTÉS À L'EXÉCUTION DES PEINES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Social"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD";"JA/AttJ Social"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.10. AUTRES FONCTIONNAIRES AFFECTÉS AU PARQUET",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Social"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD";"JA/AttJ Social"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="M6" s="280" t="e" cm="1">
-        <f t="array" ref="M6">SUM(SUMIFS(
+      <c r="M6" s="280"/>
+      <c r="N6" s="280"/>
+      <c r="O6" s="280" t="e" cm="1">
+        <f t="array" ref="O6">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("9. TOTAL JAP",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Social"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD";"JA/AttJ Social"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="N6" s="280" t="e" cm="1">
-        <f t="array" ref="N6">SUM(SUMIFS(
+      <c r="P6" s="280" t="e" cm="1">
+        <f t="array" ref="P6">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("6.2. ACTIVITÉ PÉNALE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Social"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD";"JA/AttJ Social"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="O6" s="280" t="e" cm="1">
-        <f t="array" ref="O6">SUM(SUMIFS(
+      <c r="Q6" s="280" t="e" cm="1">
+        <f t="array" ref="Q6">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("8. TOTAL JUGES D'INSTRUCTION",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Social"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD";"JA/AttJ Social"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="P6" s="280" t="e" cm="1">
-        <f t="array" ref="P6">SUM(SUMIFS(
+      <c r="R6" s="280" t="e" cm="1">
+        <f t="array" ref="R6">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("10. TOTAL JLD PÉNAL",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Social"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD";"JA/AttJ Social"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="Q6" s="278">
-        <f>_xlfn.AGGREGATE(9,6,G6:P6)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="S6" s="278">
+        <f>_xlfn.AGGREGATE(9,6,G6:R6)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:64" x14ac:dyDescent="0.2">
       <c r="A7" s="211" t="s">
         <v>290</v>
       </c>
@@ -20988,40 +21010,42 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="M7" s="280" t="e">
+      <c r="M7" s="280"/>
+      <c r="N7" s="280"/>
+      <c r="O7" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.51. ACCUEIL DU JUSTICIABLE (DONT SAUJ)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JAP",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="N7" s="280" t="e">
+      <c r="P7" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.51. ACCUEIL DU JUSTICIABLE (DONT SAUJ)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JE",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="O7" s="280" t="e">
+      <c r="Q7" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.51. ACCUEIL DU JUSTICIABLE (DONT SAUJ)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JI",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="P7" s="280" t="e">
+      <c r="R7" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.51. ACCUEIL DU JUSTICIABLE (DONT SAUJ)",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD PÉNAL",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="Q7" s="278">
-        <f>_xlfn.AGGREGATE(9,6,G7:P7)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="S7" s="278">
+        <f>_xlfn.AGGREGATE(9,6,G7:R7)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:64" x14ac:dyDescent="0.2">
       <c r="A8" s="211" t="s">
         <v>290</v>
       </c>
@@ -21099,7 +21123,9 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="M8" s="280" t="e">
+      <c r="M8" s="280"/>
+      <c r="N8" s="280"/>
+      <c r="O8" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.1. SOUTIEN (HORS FORMATIONS SUIVIES)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JAP",
@@ -21114,7 +21140,7 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="N8" s="280" t="e">
+      <c r="P8" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.1. SOUTIEN (HORS FORMATIONS SUIVIES)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JE",
@@ -21129,7 +21155,7 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="O8" s="280" t="e">
+      <c r="Q8" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.1. SOUTIEN (HORS FORMATIONS SUIVIES)",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JI",
@@ -21144,27 +21170,27 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="P8" s="280" t="e">
+      <c r="R8" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.1. SOUTIEN (HORS FORMATIONS SUIVIES)",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD PÉNAL",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.2. FORMATIONS SUIVIES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD PÉNAL",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.6. AUTRES ACTIVITÉS NON JURIDICTIONNELLES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD PÉNAL",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="Q8" s="278">
-        <f>_xlfn.AGGREGATE(9,6,G8:P8)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="S8" s="278">
+        <f>_xlfn.AGGREGATE(9,6,G8:R8)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:64" x14ac:dyDescent="0.2">
       <c r="A9" s="211" t="s">
         <v>290</v>
       </c>
@@ -21210,40 +21236,42 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="M9" s="280" t="e">
+      <c r="M9" s="280"/>
+      <c r="N9" s="280"/>
+      <c r="O9" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JAP",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="N9" s="280" t="e">
+      <c r="P9" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JE",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="O9" s="280" t="e">
+      <c r="Q9" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JI",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="P9" s="280" t="e">
+      <c r="R9" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.3. FORMATIONS DISPENSÉES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD PÉNAL",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="Q9" s="278">
-        <f>_xlfn.AGGREGATE(9,6,G9:P9)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="S9" s="278">
+        <f>_xlfn.AGGREGATE(9,6,G9:R9)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:64" x14ac:dyDescent="0.2">
       <c r="A10" s="211" t="s">
         <v>290</v>
       </c>
@@ -21289,40 +21317,42 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="M10" s="280" t="e">
+      <c r="M10" s="280"/>
+      <c r="N10" s="280"/>
+      <c r="O10" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.4. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JAP",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="N10" s="280" t="e">
+      <c r="P10" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.4. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JE",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="O10" s="280" t="e">
+      <c r="Q10" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.4. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JI",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="P10" s="280" t="e">
+      <c r="R10" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.4. ACCÈS AU DROIT ET À LA JUSTICE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD PÉNAL",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="Q10" s="278">
-        <f>_xlfn.AGGREGATE(9,6,G10:P10)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="S10" s="278">
+        <f>_xlfn.AGGREGATE(9,6,G10:R10)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:64" x14ac:dyDescent="0.2">
       <c r="A11" s="211" t="s">
         <v>290</v>
       </c>
@@ -21384,7 +21414,9 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="M11" s="280" t="e">
+      <c r="M11" s="280"/>
+      <c r="N11" s="280"/>
+      <c r="O11" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JAP",
@@ -21395,7 +21427,7 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="N11" s="280" t="e">
+      <c r="P11" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JE",
@@ -21406,7 +21438,7 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="O11" s="280" t="e">
+      <c r="Q11" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JI",
@@ -21417,23 +21449,23 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="P11" s="280" t="e">
+      <c r="R11" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD PÉNAL",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD PÉNAL",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
-      <c r="Q11" s="278">
-        <f>_xlfn.AGGREGATE(9,6,G11:P11)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="S11" s="278">
+        <f>_xlfn.AGGREGATE(9,6,G11:R11)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:64" x14ac:dyDescent="0.2">
       <c r="A12" s="211" t="s">
         <v>290</v>
       </c>
@@ -21495,7 +21527,9 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)),0)</f>
         <v>#N/A</v>
       </c>
-      <c r="M12" s="280" t="e">
+      <c r="M12" s="280"/>
+      <c r="N12" s="280"/>
+      <c r="O12" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JAP",
@@ -21506,7 +21540,7 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)),0)</f>
         <v>#N/A</v>
       </c>
-      <c r="N12" s="280" t="e">
+      <c r="P12" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JE",
@@ -21517,7 +21551,7 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)),0)</f>
         <v>#N/A</v>
       </c>
-      <c r="O12" s="280" t="e">
+      <c r="Q12" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JI",
@@ -21528,23 +21562,23 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)),0)</f>
         <v>#N/A</v>
       </c>
-      <c r="P12" s="280" t="e">
+      <c r="R12" s="280" t="e">
         <f>SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD PÉNAL",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))+
 _xlfn.IFNA(SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("13. TOTAL CONTENTIEUX LOCAUX SPÉCIFIQUES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD",
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD PÉNAL",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)),0)</f>
         <v>#N/A</v>
       </c>
-      <c r="Q12" s="278">
-        <f>_xlfn.AGGREGATE(9,6,G12:P12)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+      <c r="S12" s="278">
+        <f>_xlfn.AGGREGATE(9,6,G12:R12)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:64" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="217"/>
       <c r="B13" s="217"/>
       <c r="C13" s="217"/>
@@ -21562,7 +21596,7 @@
         <v>0</v>
       </c>
       <c r="I13" s="278">
-        <f t="shared" ref="I13:P13" si="0">_xlfn.AGGREGATE(9,6,I5:I12)</f>
+        <f t="shared" ref="I13:R13" si="0">_xlfn.AGGREGATE(9,6,I5:I12)</f>
         <v>0</v>
       </c>
       <c r="J13" s="278">
@@ -21594,11 +21628,19 @@
         <v>0</v>
       </c>
       <c r="Q13" s="278">
-        <f>_xlfn.AGGREGATE(9,6,Q5:Q12)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R13" s="278">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="S13" s="278">
+        <f>_xlfn.AGGREGATE(9,6,S5:S12)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:64" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="217"/>
       <c r="B14" s="217"/>
       <c r="C14" s="217"/>
@@ -21616,8 +21658,10 @@
       <c r="O14" s="216"/>
       <c r="P14" s="216"/>
       <c r="Q14" s="216"/>
-    </row>
-    <row r="15" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+      <c r="R14" s="216"/>
+      <c r="S14" s="216"/>
+    </row>
+    <row r="15" spans="1:64" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="217"/>
       <c r="B15" s="217"/>
       <c r="C15" s="217"/>
@@ -21629,13 +21673,13 @@
       <c r="I15" s="216"/>
       <c r="J15" s="216"/>
       <c r="K15" s="216"/>
-      <c r="M15" s="216"/>
-      <c r="N15" s="216"/>
       <c r="O15" s="216"/>
       <c r="P15" s="216"/>
       <c r="Q15" s="216"/>
-    </row>
-    <row r="16" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+      <c r="R15" s="216"/>
+      <c r="S15" s="216"/>
+    </row>
+    <row r="16" spans="1:64" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="217"/>
       <c r="B16" s="217"/>
       <c r="C16" s="217"/>
@@ -21647,13 +21691,13 @@
       <c r="I16" s="216"/>
       <c r="J16" s="216"/>
       <c r="K16" s="216"/>
-      <c r="M16" s="216"/>
-      <c r="N16" s="216"/>
       <c r="O16" s="216"/>
       <c r="P16" s="216"/>
       <c r="Q16" s="216"/>
-    </row>
-    <row r="17" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="R16" s="216"/>
+      <c r="S16" s="216"/>
+    </row>
+    <row r="17" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="217"/>
       <c r="B17" s="217"/>
       <c r="C17" s="217"/>
@@ -21665,14 +21709,14 @@
       <c r="I17" s="216"/>
       <c r="J17" s="216"/>
       <c r="K17" s="216"/>
-      <c r="M17" s="216"/>
-      <c r="N17" s="216"/>
       <c r="O17" s="216"/>
       <c r="P17" s="216"/>
       <c r="Q17" s="216"/>
       <c r="R17" s="216"/>
-    </row>
-    <row r="18" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S17" s="216"/>
+      <c r="T17" s="216"/>
+    </row>
+    <row r="18" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="217"/>
       <c r="B18" s="217"/>
       <c r="C18" s="217"/>
@@ -21684,14 +21728,14 @@
       <c r="I18" s="216"/>
       <c r="J18" s="216"/>
       <c r="K18" s="216"/>
-      <c r="M18" s="216"/>
-      <c r="N18" s="216"/>
       <c r="O18" s="216"/>
       <c r="P18" s="216"/>
       <c r="Q18" s="216"/>
       <c r="R18" s="216"/>
-    </row>
-    <row r="19" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S18" s="216"/>
+      <c r="T18" s="216"/>
+    </row>
+    <row r="19" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="217"/>
       <c r="B19" s="217"/>
       <c r="C19" s="217"/>
@@ -21703,14 +21747,14 @@
       <c r="I19" s="216"/>
       <c r="J19" s="216"/>
       <c r="K19" s="216"/>
-      <c r="M19" s="216"/>
-      <c r="N19" s="216"/>
       <c r="O19" s="216"/>
       <c r="P19" s="216"/>
       <c r="Q19" s="216"/>
       <c r="R19" s="216"/>
-    </row>
-    <row r="20" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S19" s="216"/>
+      <c r="T19" s="216"/>
+    </row>
+    <row r="20" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="217"/>
       <c r="B20" s="217"/>
       <c r="C20" s="217"/>
@@ -21722,14 +21766,14 @@
       <c r="I20" s="216"/>
       <c r="J20" s="216"/>
       <c r="K20" s="216"/>
-      <c r="M20" s="216"/>
-      <c r="N20" s="216"/>
       <c r="O20" s="216"/>
       <c r="P20" s="216"/>
       <c r="Q20" s="216"/>
       <c r="R20" s="216"/>
-    </row>
-    <row r="21" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S20" s="216"/>
+      <c r="T20" s="216"/>
+    </row>
+    <row r="21" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="217"/>
       <c r="B21" s="217"/>
       <c r="C21" s="217"/>
@@ -21741,14 +21785,14 @@
       <c r="I21" s="216"/>
       <c r="J21" s="216"/>
       <c r="K21" s="216"/>
-      <c r="M21" s="216"/>
-      <c r="N21" s="216"/>
       <c r="O21" s="216"/>
       <c r="P21" s="216"/>
       <c r="Q21" s="216"/>
       <c r="R21" s="216"/>
-    </row>
-    <row r="22" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S21" s="216"/>
+      <c r="T21" s="216"/>
+    </row>
+    <row r="22" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="217"/>
       <c r="B22" s="217"/>
       <c r="C22" s="217"/>
@@ -21760,14 +21804,14 @@
       <c r="I22" s="216"/>
       <c r="J22" s="216"/>
       <c r="K22" s="216"/>
-      <c r="M22" s="216"/>
-      <c r="N22" s="216"/>
       <c r="O22" s="216"/>
       <c r="P22" s="216"/>
       <c r="Q22" s="216"/>
       <c r="R22" s="216"/>
-    </row>
-    <row r="23" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S22" s="216"/>
+      <c r="T22" s="216"/>
+    </row>
+    <row r="23" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="217"/>
       <c r="B23" s="217"/>
       <c r="C23" s="217"/>
@@ -21786,8 +21830,10 @@
       <c r="P23" s="216"/>
       <c r="Q23" s="216"/>
       <c r="R23" s="216"/>
-    </row>
-    <row r="24" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S23" s="216"/>
+      <c r="T23" s="216"/>
+    </row>
+    <row r="24" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="217"/>
       <c r="B24" s="217"/>
       <c r="C24" s="217"/>
@@ -21806,8 +21852,10 @@
       <c r="P24" s="216"/>
       <c r="Q24" s="216"/>
       <c r="R24" s="216"/>
-    </row>
-    <row r="25" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S24" s="216"/>
+      <c r="T24" s="216"/>
+    </row>
+    <row r="25" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="217"/>
       <c r="B25" s="217"/>
       <c r="C25" s="217"/>
@@ -21826,8 +21874,10 @@
       <c r="P25" s="216"/>
       <c r="Q25" s="216"/>
       <c r="R25" s="216"/>
-    </row>
-    <row r="26" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S25" s="216"/>
+      <c r="T25" s="216"/>
+    </row>
+    <row r="26" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="217"/>
       <c r="B26" s="217"/>
       <c r="C26" s="217"/>
@@ -21846,8 +21896,10 @@
       <c r="P26" s="216"/>
       <c r="Q26" s="216"/>
       <c r="R26" s="216"/>
-    </row>
-    <row r="27" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S26" s="216"/>
+      <c r="T26" s="216"/>
+    </row>
+    <row r="27" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="217"/>
       <c r="B27" s="217"/>
       <c r="C27" s="217"/>
@@ -21866,8 +21918,10 @@
       <c r="P27" s="216"/>
       <c r="Q27" s="216"/>
       <c r="R27" s="216"/>
-    </row>
-    <row r="28" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S27" s="216"/>
+      <c r="T27" s="216"/>
+    </row>
+    <row r="28" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="217"/>
       <c r="B28" s="217"/>
       <c r="C28" s="217"/>
@@ -21886,8 +21940,10 @@
       <c r="P28" s="216"/>
       <c r="Q28" s="216"/>
       <c r="R28" s="216"/>
-    </row>
-    <row r="29" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S28" s="216"/>
+      <c r="T28" s="216"/>
+    </row>
+    <row r="29" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="217"/>
       <c r="B29" s="217"/>
       <c r="C29" s="217"/>
@@ -21906,8 +21962,10 @@
       <c r="P29" s="216"/>
       <c r="Q29" s="216"/>
       <c r="R29" s="216"/>
-    </row>
-    <row r="30" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S29" s="216"/>
+      <c r="T29" s="216"/>
+    </row>
+    <row r="30" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="217"/>
       <c r="B30" s="217"/>
       <c r="C30" s="217"/>
@@ -21926,8 +21984,10 @@
       <c r="P30" s="216"/>
       <c r="Q30" s="216"/>
       <c r="R30" s="216"/>
-    </row>
-    <row r="31" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S30" s="216"/>
+      <c r="T30" s="216"/>
+    </row>
+    <row r="31" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="217"/>
       <c r="B31" s="217"/>
       <c r="C31" s="217"/>
@@ -21946,8 +22006,10 @@
       <c r="P31" s="216"/>
       <c r="Q31" s="216"/>
       <c r="R31" s="216"/>
-    </row>
-    <row r="32" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S31" s="216"/>
+      <c r="T31" s="216"/>
+    </row>
+    <row r="32" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="217"/>
       <c r="B32" s="217"/>
       <c r="C32" s="217"/>
@@ -21966,8 +22028,10 @@
       <c r="P32" s="216"/>
       <c r="Q32" s="216"/>
       <c r="R32" s="216"/>
-    </row>
-    <row r="33" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S32" s="216"/>
+      <c r="T32" s="216"/>
+    </row>
+    <row r="33" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="217"/>
       <c r="B33" s="217"/>
       <c r="C33" s="217"/>
@@ -21986,8 +22050,10 @@
       <c r="P33" s="216"/>
       <c r="Q33" s="216"/>
       <c r="R33" s="216"/>
-    </row>
-    <row r="34" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S33" s="216"/>
+      <c r="T33" s="216"/>
+    </row>
+    <row r="34" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="217"/>
       <c r="B34" s="217"/>
       <c r="C34" s="217"/>
@@ -22006,8 +22072,10 @@
       <c r="P34" s="216"/>
       <c r="Q34" s="216"/>
       <c r="R34" s="216"/>
-    </row>
-    <row r="35" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S34" s="216"/>
+      <c r="T34" s="216"/>
+    </row>
+    <row r="35" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="217"/>
       <c r="B35" s="217"/>
       <c r="C35" s="217"/>
@@ -22026,8 +22094,10 @@
       <c r="P35" s="216"/>
       <c r="Q35" s="216"/>
       <c r="R35" s="216"/>
-    </row>
-    <row r="36" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S35" s="216"/>
+      <c r="T35" s="216"/>
+    </row>
+    <row r="36" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="217"/>
       <c r="B36" s="217"/>
       <c r="C36" s="217"/>
@@ -22046,8 +22116,10 @@
       <c r="P36" s="216"/>
       <c r="Q36" s="216"/>
       <c r="R36" s="216"/>
-    </row>
-    <row r="37" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S36" s="216"/>
+      <c r="T36" s="216"/>
+    </row>
+    <row r="37" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="217"/>
       <c r="B37" s="217"/>
       <c r="C37" s="217"/>
@@ -22066,8 +22138,10 @@
       <c r="P37" s="216"/>
       <c r="Q37" s="216"/>
       <c r="R37" s="216"/>
-    </row>
-    <row r="38" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S37" s="216"/>
+      <c r="T37" s="216"/>
+    </row>
+    <row r="38" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="217"/>
       <c r="B38" s="217"/>
       <c r="C38" s="217"/>
@@ -22086,8 +22160,10 @@
       <c r="P38" s="216"/>
       <c r="Q38" s="216"/>
       <c r="R38" s="216"/>
-    </row>
-    <row r="39" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S38" s="216"/>
+      <c r="T38" s="216"/>
+    </row>
+    <row r="39" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="217"/>
       <c r="B39" s="217"/>
       <c r="C39" s="217"/>
@@ -22106,8 +22182,10 @@
       <c r="P39" s="216"/>
       <c r="Q39" s="216"/>
       <c r="R39" s="216"/>
-    </row>
-    <row r="40" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S39" s="216"/>
+      <c r="T39" s="216"/>
+    </row>
+    <row r="40" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="217"/>
       <c r="B40" s="217"/>
       <c r="C40" s="217"/>
@@ -22126,8 +22204,10 @@
       <c r="P40" s="216"/>
       <c r="Q40" s="216"/>
       <c r="R40" s="216"/>
-    </row>
-    <row r="41" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S40" s="216"/>
+      <c r="T40" s="216"/>
+    </row>
+    <row r="41" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="217"/>
       <c r="B41" s="217"/>
       <c r="C41" s="217"/>
@@ -22146,8 +22226,10 @@
       <c r="P41" s="216"/>
       <c r="Q41" s="216"/>
       <c r="R41" s="216"/>
-    </row>
-    <row r="42" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S41" s="216"/>
+      <c r="T41" s="216"/>
+    </row>
+    <row r="42" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="217"/>
       <c r="B42" s="217"/>
       <c r="C42" s="217"/>
@@ -22166,8 +22248,10 @@
       <c r="P42" s="216"/>
       <c r="Q42" s="216"/>
       <c r="R42" s="216"/>
-    </row>
-    <row r="43" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S42" s="216"/>
+      <c r="T42" s="216"/>
+    </row>
+    <row r="43" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="217"/>
       <c r="B43" s="217"/>
       <c r="C43" s="217"/>
@@ -22186,8 +22270,10 @@
       <c r="P43" s="216"/>
       <c r="Q43" s="216"/>
       <c r="R43" s="216"/>
-    </row>
-    <row r="44" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S43" s="216"/>
+      <c r="T43" s="216"/>
+    </row>
+    <row r="44" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="217"/>
       <c r="B44" s="217"/>
       <c r="C44" s="217"/>
@@ -22206,8 +22292,10 @@
       <c r="P44" s="216"/>
       <c r="Q44" s="216"/>
       <c r="R44" s="216"/>
-    </row>
-    <row r="45" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S44" s="216"/>
+      <c r="T44" s="216"/>
+    </row>
+    <row r="45" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="217"/>
       <c r="B45" s="217"/>
       <c r="C45" s="217"/>
@@ -22226,8 +22314,10 @@
       <c r="P45" s="216"/>
       <c r="Q45" s="216"/>
       <c r="R45" s="216"/>
-    </row>
-    <row r="46" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S45" s="216"/>
+      <c r="T45" s="216"/>
+    </row>
+    <row r="46" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="217"/>
       <c r="B46" s="217"/>
       <c r="C46" s="217"/>
@@ -22246,8 +22336,10 @@
       <c r="P46" s="216"/>
       <c r="Q46" s="216"/>
       <c r="R46" s="216"/>
-    </row>
-    <row r="47" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S46" s="216"/>
+      <c r="T46" s="216"/>
+    </row>
+    <row r="47" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" s="217"/>
       <c r="B47" s="217"/>
       <c r="C47" s="217"/>
@@ -22266,8 +22358,10 @@
       <c r="P47" s="216"/>
       <c r="Q47" s="216"/>
       <c r="R47" s="216"/>
-    </row>
-    <row r="48" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S47" s="216"/>
+      <c r="T47" s="216"/>
+    </row>
+    <row r="48" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" s="217"/>
       <c r="B48" s="217"/>
       <c r="C48" s="217"/>
@@ -22286,8 +22380,10 @@
       <c r="P48" s="216"/>
       <c r="Q48" s="216"/>
       <c r="R48" s="216"/>
-    </row>
-    <row r="49" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S48" s="216"/>
+      <c r="T48" s="216"/>
+    </row>
+    <row r="49" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" s="217"/>
       <c r="B49" s="217"/>
       <c r="C49" s="217"/>
@@ -22306,8 +22402,10 @@
       <c r="P49" s="216"/>
       <c r="Q49" s="216"/>
       <c r="R49" s="216"/>
-    </row>
-    <row r="50" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S49" s="216"/>
+      <c r="T49" s="216"/>
+    </row>
+    <row r="50" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" s="217"/>
       <c r="B50" s="217"/>
       <c r="C50" s="217"/>
@@ -22326,8 +22424,10 @@
       <c r="P50" s="216"/>
       <c r="Q50" s="216"/>
       <c r="R50" s="216"/>
-    </row>
-    <row r="51" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S50" s="216"/>
+      <c r="T50" s="216"/>
+    </row>
+    <row r="51" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" s="217"/>
       <c r="B51" s="217"/>
       <c r="C51" s="217"/>
@@ -22346,8 +22446,10 @@
       <c r="P51" s="216"/>
       <c r="Q51" s="216"/>
       <c r="R51" s="216"/>
-    </row>
-    <row r="52" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S51" s="216"/>
+      <c r="T51" s="216"/>
+    </row>
+    <row r="52" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" s="217"/>
       <c r="B52" s="217"/>
       <c r="C52" s="217"/>
@@ -22366,8 +22468,10 @@
       <c r="P52" s="216"/>
       <c r="Q52" s="216"/>
       <c r="R52" s="216"/>
-    </row>
-    <row r="53" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S52" s="216"/>
+      <c r="T52" s="216"/>
+    </row>
+    <row r="53" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" s="217"/>
       <c r="B53" s="217"/>
       <c r="C53" s="217"/>
@@ -22386,8 +22490,10 @@
       <c r="P53" s="216"/>
       <c r="Q53" s="216"/>
       <c r="R53" s="216"/>
-    </row>
-    <row r="54" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S53" s="216"/>
+      <c r="T53" s="216"/>
+    </row>
+    <row r="54" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A54" s="217"/>
       <c r="B54" s="217"/>
       <c r="C54" s="217"/>
@@ -22406,8 +22512,10 @@
       <c r="P54" s="216"/>
       <c r="Q54" s="216"/>
       <c r="R54" s="216"/>
-    </row>
-    <row r="55" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S54" s="216"/>
+      <c r="T54" s="216"/>
+    </row>
+    <row r="55" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" s="217"/>
       <c r="B55" s="217"/>
       <c r="C55" s="217"/>
@@ -22426,8 +22534,10 @@
       <c r="P55" s="216"/>
       <c r="Q55" s="216"/>
       <c r="R55" s="216"/>
-    </row>
-    <row r="56" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S55" s="216"/>
+      <c r="T55" s="216"/>
+    </row>
+    <row r="56" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" s="217"/>
       <c r="B56" s="217"/>
       <c r="C56" s="217"/>
@@ -22446,8 +22556,10 @@
       <c r="P56" s="216"/>
       <c r="Q56" s="216"/>
       <c r="R56" s="216"/>
-    </row>
-    <row r="57" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S56" s="216"/>
+      <c r="T56" s="216"/>
+    </row>
+    <row r="57" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A57" s="217"/>
       <c r="B57" s="217"/>
       <c r="C57" s="217"/>
@@ -22466,8 +22578,10 @@
       <c r="P57" s="216"/>
       <c r="Q57" s="216"/>
       <c r="R57" s="216"/>
-    </row>
-    <row r="58" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S57" s="216"/>
+      <c r="T57" s="216"/>
+    </row>
+    <row r="58" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A58" s="217"/>
       <c r="B58" s="217"/>
       <c r="C58" s="217"/>
@@ -22486,8 +22600,10 @@
       <c r="P58" s="216"/>
       <c r="Q58" s="216"/>
       <c r="R58" s="216"/>
-    </row>
-    <row r="59" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S58" s="216"/>
+      <c r="T58" s="216"/>
+    </row>
+    <row r="59" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" s="217"/>
       <c r="B59" s="217"/>
       <c r="C59" s="217"/>
@@ -22506,8 +22622,10 @@
       <c r="P59" s="216"/>
       <c r="Q59" s="216"/>
       <c r="R59" s="216"/>
-    </row>
-    <row r="60" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S59" s="216"/>
+      <c r="T59" s="216"/>
+    </row>
+    <row r="60" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A60" s="217"/>
       <c r="B60" s="217"/>
       <c r="C60" s="217"/>
@@ -22526,8 +22644,10 @@
       <c r="P60" s="216"/>
       <c r="Q60" s="216"/>
       <c r="R60" s="216"/>
-    </row>
-    <row r="61" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S60" s="216"/>
+      <c r="T60" s="216"/>
+    </row>
+    <row r="61" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A61" s="217"/>
       <c r="B61" s="217"/>
       <c r="C61" s="217"/>
@@ -22546,8 +22666,10 @@
       <c r="P61" s="216"/>
       <c r="Q61" s="216"/>
       <c r="R61" s="216"/>
-    </row>
-    <row r="62" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S61" s="216"/>
+      <c r="T61" s="216"/>
+    </row>
+    <row r="62" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A62" s="217"/>
       <c r="B62" s="217"/>
       <c r="C62" s="217"/>
@@ -22566,8 +22688,10 @@
       <c r="P62" s="216"/>
       <c r="Q62" s="216"/>
       <c r="R62" s="216"/>
-    </row>
-    <row r="63" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S62" s="216"/>
+      <c r="T62" s="216"/>
+    </row>
+    <row r="63" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A63" s="217"/>
       <c r="B63" s="217"/>
       <c r="C63" s="217"/>
@@ -22586,8 +22710,10 @@
       <c r="P63" s="216"/>
       <c r="Q63" s="216"/>
       <c r="R63" s="216"/>
-    </row>
-    <row r="64" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S63" s="216"/>
+      <c r="T63" s="216"/>
+    </row>
+    <row r="64" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A64" s="217"/>
       <c r="B64" s="217"/>
       <c r="C64" s="217"/>
@@ -22606,8 +22732,10 @@
       <c r="P64" s="216"/>
       <c r="Q64" s="216"/>
       <c r="R64" s="216"/>
-    </row>
-    <row r="65" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S64" s="216"/>
+      <c r="T64" s="216"/>
+    </row>
+    <row r="65" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A65" s="217"/>
       <c r="B65" s="217"/>
       <c r="C65" s="217"/>
@@ -22626,8 +22754,10 @@
       <c r="P65" s="216"/>
       <c r="Q65" s="216"/>
       <c r="R65" s="216"/>
-    </row>
-    <row r="66" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S65" s="216"/>
+      <c r="T65" s="216"/>
+    </row>
+    <row r="66" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A66" s="217"/>
       <c r="B66" s="217"/>
       <c r="C66" s="217"/>
@@ -22646,8 +22776,10 @@
       <c r="P66" s="216"/>
       <c r="Q66" s="216"/>
       <c r="R66" s="216"/>
-    </row>
-    <row r="67" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S66" s="216"/>
+      <c r="T66" s="216"/>
+    </row>
+    <row r="67" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A67" s="217"/>
       <c r="B67" s="217"/>
       <c r="C67" s="217"/>
@@ -22666,8 +22798,10 @@
       <c r="P67" s="216"/>
       <c r="Q67" s="216"/>
       <c r="R67" s="216"/>
-    </row>
-    <row r="68" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S67" s="216"/>
+      <c r="T67" s="216"/>
+    </row>
+    <row r="68" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A68" s="217"/>
       <c r="B68" s="217"/>
       <c r="C68" s="217"/>
@@ -22686,8 +22820,10 @@
       <c r="P68" s="216"/>
       <c r="Q68" s="216"/>
       <c r="R68" s="216"/>
-    </row>
-    <row r="69" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S68" s="216"/>
+      <c r="T68" s="216"/>
+    </row>
+    <row r="69" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A69" s="217"/>
       <c r="B69" s="217"/>
       <c r="C69" s="217"/>
@@ -22706,8 +22842,10 @@
       <c r="P69" s="216"/>
       <c r="Q69" s="216"/>
       <c r="R69" s="216"/>
-    </row>
-    <row r="70" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S69" s="216"/>
+      <c r="T69" s="216"/>
+    </row>
+    <row r="70" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A70" s="217"/>
       <c r="B70" s="217"/>
       <c r="C70" s="217"/>
@@ -22726,8 +22864,10 @@
       <c r="P70" s="216"/>
       <c r="Q70" s="216"/>
       <c r="R70" s="216"/>
-    </row>
-    <row r="71" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S70" s="216"/>
+      <c r="T70" s="216"/>
+    </row>
+    <row r="71" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A71" s="217"/>
       <c r="B71" s="217"/>
       <c r="C71" s="217"/>
@@ -22746,8 +22886,10 @@
       <c r="P71" s="216"/>
       <c r="Q71" s="216"/>
       <c r="R71" s="216"/>
-    </row>
-    <row r="72" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S71" s="216"/>
+      <c r="T71" s="216"/>
+    </row>
+    <row r="72" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A72" s="217"/>
       <c r="B72" s="217"/>
       <c r="C72" s="217"/>
@@ -22766,8 +22908,10 @@
       <c r="P72" s="216"/>
       <c r="Q72" s="216"/>
       <c r="R72" s="216"/>
-    </row>
-    <row r="73" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S72" s="216"/>
+      <c r="T72" s="216"/>
+    </row>
+    <row r="73" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A73" s="217"/>
       <c r="B73" s="217"/>
       <c r="C73" s="217"/>
@@ -22786,8 +22930,10 @@
       <c r="P73" s="216"/>
       <c r="Q73" s="216"/>
       <c r="R73" s="216"/>
-    </row>
-    <row r="74" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S73" s="216"/>
+      <c r="T73" s="216"/>
+    </row>
+    <row r="74" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A74" s="217"/>
       <c r="B74" s="217"/>
       <c r="C74" s="217"/>
@@ -22806,8 +22952,10 @@
       <c r="P74" s="216"/>
       <c r="Q74" s="216"/>
       <c r="R74" s="216"/>
-    </row>
-    <row r="75" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S74" s="216"/>
+      <c r="T74" s="216"/>
+    </row>
+    <row r="75" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A75" s="217"/>
       <c r="B75" s="217"/>
       <c r="C75" s="217"/>
@@ -22826,8 +22974,10 @@
       <c r="P75" s="216"/>
       <c r="Q75" s="216"/>
       <c r="R75" s="216"/>
-    </row>
-    <row r="76" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S75" s="216"/>
+      <c r="T75" s="216"/>
+    </row>
+    <row r="76" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A76" s="217"/>
       <c r="B76" s="217"/>
       <c r="C76" s="217"/>
@@ -22846,8 +22996,10 @@
       <c r="P76" s="216"/>
       <c r="Q76" s="216"/>
       <c r="R76" s="216"/>
-    </row>
-    <row r="77" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S76" s="216"/>
+      <c r="T76" s="216"/>
+    </row>
+    <row r="77" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A77" s="217"/>
       <c r="B77" s="217"/>
       <c r="C77" s="217"/>
@@ -22866,8 +23018,10 @@
       <c r="P77" s="216"/>
       <c r="Q77" s="216"/>
       <c r="R77" s="216"/>
-    </row>
-    <row r="78" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S77" s="216"/>
+      <c r="T77" s="216"/>
+    </row>
+    <row r="78" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A78" s="217"/>
       <c r="B78" s="217"/>
       <c r="C78" s="217"/>
@@ -22886,8 +23040,10 @@
       <c r="P78" s="216"/>
       <c r="Q78" s="216"/>
       <c r="R78" s="216"/>
-    </row>
-    <row r="79" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S78" s="216"/>
+      <c r="T78" s="216"/>
+    </row>
+    <row r="79" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A79" s="217"/>
       <c r="B79" s="217"/>
       <c r="C79" s="217"/>
@@ -22906,8 +23062,10 @@
       <c r="P79" s="216"/>
       <c r="Q79" s="216"/>
       <c r="R79" s="216"/>
-    </row>
-    <row r="80" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S79" s="216"/>
+      <c r="T79" s="216"/>
+    </row>
+    <row r="80" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A80" s="217"/>
       <c r="B80" s="217"/>
       <c r="C80" s="217"/>
@@ -22926,8 +23084,10 @@
       <c r="P80" s="216"/>
       <c r="Q80" s="216"/>
       <c r="R80" s="216"/>
-    </row>
-    <row r="81" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S80" s="216"/>
+      <c r="T80" s="216"/>
+    </row>
+    <row r="81" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A81" s="217"/>
       <c r="B81" s="217"/>
       <c r="C81" s="217"/>
@@ -22946,8 +23106,10 @@
       <c r="P81" s="216"/>
       <c r="Q81" s="216"/>
       <c r="R81" s="216"/>
-    </row>
-    <row r="82" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S81" s="216"/>
+      <c r="T81" s="216"/>
+    </row>
+    <row r="82" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A82" s="217"/>
       <c r="B82" s="217"/>
       <c r="C82" s="217"/>
@@ -22966,8 +23128,10 @@
       <c r="P82" s="216"/>
       <c r="Q82" s="216"/>
       <c r="R82" s="216"/>
-    </row>
-    <row r="83" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S82" s="216"/>
+      <c r="T82" s="216"/>
+    </row>
+    <row r="83" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A83" s="217"/>
       <c r="B83" s="217"/>
       <c r="C83" s="217"/>
@@ -22986,8 +23150,10 @@
       <c r="P83" s="216"/>
       <c r="Q83" s="216"/>
       <c r="R83" s="216"/>
-    </row>
-    <row r="84" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S83" s="216"/>
+      <c r="T83" s="216"/>
+    </row>
+    <row r="84" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A84" s="217"/>
       <c r="B84" s="217"/>
       <c r="C84" s="217"/>
@@ -23006,8 +23172,10 @@
       <c r="P84" s="216"/>
       <c r="Q84" s="216"/>
       <c r="R84" s="216"/>
-    </row>
-    <row r="85" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S84" s="216"/>
+      <c r="T84" s="216"/>
+    </row>
+    <row r="85" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A85" s="217"/>
       <c r="B85" s="217"/>
       <c r="C85" s="217"/>
@@ -23026,8 +23194,10 @@
       <c r="P85" s="216"/>
       <c r="Q85" s="216"/>
       <c r="R85" s="216"/>
-    </row>
-    <row r="86" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S85" s="216"/>
+      <c r="T85" s="216"/>
+    </row>
+    <row r="86" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A86" s="217"/>
       <c r="B86" s="217"/>
       <c r="C86" s="217"/>
@@ -23046,8 +23216,10 @@
       <c r="P86" s="216"/>
       <c r="Q86" s="216"/>
       <c r="R86" s="216"/>
-    </row>
-    <row r="87" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S86" s="216"/>
+      <c r="T86" s="216"/>
+    </row>
+    <row r="87" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A87" s="217"/>
       <c r="B87" s="217"/>
       <c r="C87" s="217"/>
@@ -23066,8 +23238,10 @@
       <c r="P87" s="216"/>
       <c r="Q87" s="216"/>
       <c r="R87" s="216"/>
-    </row>
-    <row r="88" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S87" s="216"/>
+      <c r="T87" s="216"/>
+    </row>
+    <row r="88" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A88" s="217"/>
       <c r="B88" s="217"/>
       <c r="C88" s="217"/>
@@ -23086,8 +23260,10 @@
       <c r="P88" s="216"/>
       <c r="Q88" s="216"/>
       <c r="R88" s="216"/>
-    </row>
-    <row r="89" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S88" s="216"/>
+      <c r="T88" s="216"/>
+    </row>
+    <row r="89" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A89" s="217"/>
       <c r="B89" s="217"/>
       <c r="C89" s="217"/>
@@ -23106,8 +23282,10 @@
       <c r="P89" s="216"/>
       <c r="Q89" s="216"/>
       <c r="R89" s="216"/>
-    </row>
-    <row r="90" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S89" s="216"/>
+      <c r="T89" s="216"/>
+    </row>
+    <row r="90" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A90" s="217"/>
       <c r="B90" s="217"/>
       <c r="C90" s="217"/>
@@ -23126,8 +23304,10 @@
       <c r="P90" s="216"/>
       <c r="Q90" s="216"/>
       <c r="R90" s="216"/>
-    </row>
-    <row r="91" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S90" s="216"/>
+      <c r="T90" s="216"/>
+    </row>
+    <row r="91" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A91" s="217"/>
       <c r="B91" s="217"/>
       <c r="C91" s="217"/>
@@ -23146,8 +23326,10 @@
       <c r="P91" s="216"/>
       <c r="Q91" s="216"/>
       <c r="R91" s="216"/>
-    </row>
-    <row r="92" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S91" s="216"/>
+      <c r="T91" s="216"/>
+    </row>
+    <row r="92" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A92" s="217"/>
       <c r="B92" s="217"/>
       <c r="C92" s="217"/>
@@ -23166,8 +23348,10 @@
       <c r="P92" s="216"/>
       <c r="Q92" s="216"/>
       <c r="R92" s="216"/>
-    </row>
-    <row r="93" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S92" s="216"/>
+      <c r="T92" s="216"/>
+    </row>
+    <row r="93" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A93" s="217"/>
       <c r="B93" s="217"/>
       <c r="C93" s="217"/>
@@ -23186,8 +23370,10 @@
       <c r="P93" s="216"/>
       <c r="Q93" s="216"/>
       <c r="R93" s="216"/>
-    </row>
-    <row r="94" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S93" s="216"/>
+      <c r="T93" s="216"/>
+    </row>
+    <row r="94" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A94" s="217"/>
       <c r="B94" s="217"/>
       <c r="C94" s="217"/>
@@ -23206,8 +23392,10 @@
       <c r="P94" s="216"/>
       <c r="Q94" s="216"/>
       <c r="R94" s="216"/>
-    </row>
-    <row r="95" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S94" s="216"/>
+      <c r="T94" s="216"/>
+    </row>
+    <row r="95" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A95" s="217"/>
       <c r="B95" s="217"/>
       <c r="C95" s="217"/>
@@ -23226,8 +23414,10 @@
       <c r="P95" s="216"/>
       <c r="Q95" s="216"/>
       <c r="R95" s="216"/>
-    </row>
-    <row r="96" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S95" s="216"/>
+      <c r="T95" s="216"/>
+    </row>
+    <row r="96" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A96" s="217"/>
       <c r="B96" s="217"/>
       <c r="C96" s="217"/>
@@ -23246,8 +23436,10 @@
       <c r="P96" s="216"/>
       <c r="Q96" s="216"/>
       <c r="R96" s="216"/>
-    </row>
-    <row r="97" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S96" s="216"/>
+      <c r="T96" s="216"/>
+    </row>
+    <row r="97" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A97" s="217"/>
       <c r="B97" s="217"/>
       <c r="C97" s="217"/>
@@ -23266,8 +23458,10 @@
       <c r="P97" s="216"/>
       <c r="Q97" s="216"/>
       <c r="R97" s="216"/>
-    </row>
-    <row r="98" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S97" s="216"/>
+      <c r="T97" s="216"/>
+    </row>
+    <row r="98" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A98" s="217"/>
       <c r="B98" s="217"/>
       <c r="C98" s="217"/>
@@ -23286,8 +23480,10 @@
       <c r="P98" s="216"/>
       <c r="Q98" s="216"/>
       <c r="R98" s="216"/>
-    </row>
-    <row r="99" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S98" s="216"/>
+      <c r="T98" s="216"/>
+    </row>
+    <row r="99" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A99" s="217"/>
       <c r="B99" s="217"/>
       <c r="C99" s="217"/>
@@ -23306,8 +23502,10 @@
       <c r="P99" s="216"/>
       <c r="Q99" s="216"/>
       <c r="R99" s="216"/>
-    </row>
-    <row r="100" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S99" s="216"/>
+      <c r="T99" s="216"/>
+    </row>
+    <row r="100" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A100" s="217"/>
       <c r="B100" s="217"/>
       <c r="C100" s="217"/>
@@ -23326,8 +23524,10 @@
       <c r="P100" s="216"/>
       <c r="Q100" s="216"/>
       <c r="R100" s="216"/>
-    </row>
-    <row r="101" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S100" s="216"/>
+      <c r="T100" s="216"/>
+    </row>
+    <row r="101" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A101" s="217"/>
       <c r="B101" s="217"/>
       <c r="C101" s="217"/>
@@ -23346,8 +23546,10 @@
       <c r="P101" s="216"/>
       <c r="Q101" s="216"/>
       <c r="R101" s="216"/>
-    </row>
-    <row r="102" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S101" s="216"/>
+      <c r="T101" s="216"/>
+    </row>
+    <row r="102" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A102" s="217"/>
       <c r="B102" s="217"/>
       <c r="C102" s="217"/>
@@ -23366,8 +23568,10 @@
       <c r="P102" s="216"/>
       <c r="Q102" s="216"/>
       <c r="R102" s="216"/>
-    </row>
-    <row r="103" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S102" s="216"/>
+      <c r="T102" s="216"/>
+    </row>
+    <row r="103" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A103" s="217"/>
       <c r="B103" s="217"/>
       <c r="C103" s="217"/>
@@ -23386,8 +23590,10 @@
       <c r="P103" s="216"/>
       <c r="Q103" s="216"/>
       <c r="R103" s="216"/>
-    </row>
-    <row r="104" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S103" s="216"/>
+      <c r="T103" s="216"/>
+    </row>
+    <row r="104" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A104" s="217"/>
       <c r="B104" s="217"/>
       <c r="C104" s="217"/>
@@ -23406,8 +23612,10 @@
       <c r="P104" s="216"/>
       <c r="Q104" s="216"/>
       <c r="R104" s="216"/>
-    </row>
-    <row r="105" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S104" s="216"/>
+      <c r="T104" s="216"/>
+    </row>
+    <row r="105" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A105" s="217"/>
       <c r="B105" s="217"/>
       <c r="C105" s="217"/>
@@ -23426,8 +23634,10 @@
       <c r="P105" s="216"/>
       <c r="Q105" s="216"/>
       <c r="R105" s="216"/>
-    </row>
-    <row r="106" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S105" s="216"/>
+      <c r="T105" s="216"/>
+    </row>
+    <row r="106" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A106" s="217"/>
       <c r="B106" s="217"/>
       <c r="C106" s="217"/>
@@ -23446,8 +23656,10 @@
       <c r="P106" s="216"/>
       <c r="Q106" s="216"/>
       <c r="R106" s="216"/>
-    </row>
-    <row r="107" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S106" s="216"/>
+      <c r="T106" s="216"/>
+    </row>
+    <row r="107" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A107" s="217"/>
       <c r="B107" s="217"/>
       <c r="C107" s="217"/>
@@ -23466,8 +23678,10 @@
       <c r="P107" s="216"/>
       <c r="Q107" s="216"/>
       <c r="R107" s="216"/>
-    </row>
-    <row r="108" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S107" s="216"/>
+      <c r="T107" s="216"/>
+    </row>
+    <row r="108" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A108" s="217"/>
       <c r="B108" s="217"/>
       <c r="C108" s="217"/>
@@ -23486,8 +23700,10 @@
       <c r="P108" s="216"/>
       <c r="Q108" s="216"/>
       <c r="R108" s="216"/>
-    </row>
-    <row r="109" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S108" s="216"/>
+      <c r="T108" s="216"/>
+    </row>
+    <row r="109" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A109" s="217"/>
       <c r="B109" s="217"/>
       <c r="C109" s="217"/>
@@ -23506,8 +23722,10 @@
       <c r="P109" s="216"/>
       <c r="Q109" s="216"/>
       <c r="R109" s="216"/>
-    </row>
-    <row r="110" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S109" s="216"/>
+      <c r="T109" s="216"/>
+    </row>
+    <row r="110" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A110" s="217"/>
       <c r="B110" s="217"/>
       <c r="C110" s="217"/>
@@ -23526,8 +23744,10 @@
       <c r="P110" s="216"/>
       <c r="Q110" s="216"/>
       <c r="R110" s="216"/>
-    </row>
-    <row r="111" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S110" s="216"/>
+      <c r="T110" s="216"/>
+    </row>
+    <row r="111" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A111" s="217"/>
       <c r="B111" s="217"/>
       <c r="C111" s="217"/>
@@ -23546,8 +23766,10 @@
       <c r="P111" s="216"/>
       <c r="Q111" s="216"/>
       <c r="R111" s="216"/>
-    </row>
-    <row r="112" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S111" s="216"/>
+      <c r="T111" s="216"/>
+    </row>
+    <row r="112" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A112" s="217"/>
       <c r="B112" s="217"/>
       <c r="C112" s="217"/>
@@ -23566,8 +23788,10 @@
       <c r="P112" s="216"/>
       <c r="Q112" s="216"/>
       <c r="R112" s="216"/>
-    </row>
-    <row r="113" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S112" s="216"/>
+      <c r="T112" s="216"/>
+    </row>
+    <row r="113" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A113" s="217"/>
       <c r="B113" s="217"/>
       <c r="C113" s="217"/>
@@ -23586,8 +23810,10 @@
       <c r="P113" s="216"/>
       <c r="Q113" s="216"/>
       <c r="R113" s="216"/>
-    </row>
-    <row r="114" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S113" s="216"/>
+      <c r="T113" s="216"/>
+    </row>
+    <row r="114" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A114" s="217"/>
       <c r="B114" s="217"/>
       <c r="C114" s="217"/>
@@ -23606,8 +23832,10 @@
       <c r="P114" s="216"/>
       <c r="Q114" s="216"/>
       <c r="R114" s="216"/>
-    </row>
-    <row r="115" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S114" s="216"/>
+      <c r="T114" s="216"/>
+    </row>
+    <row r="115" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A115" s="217"/>
       <c r="B115" s="217"/>
       <c r="C115" s="217"/>
@@ -23626,8 +23854,10 @@
       <c r="P115" s="216"/>
       <c r="Q115" s="216"/>
       <c r="R115" s="216"/>
-    </row>
-    <row r="116" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S115" s="216"/>
+      <c r="T115" s="216"/>
+    </row>
+    <row r="116" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A116" s="217"/>
       <c r="B116" s="217"/>
       <c r="C116" s="217"/>
@@ -23646,8 +23876,10 @@
       <c r="P116" s="216"/>
       <c r="Q116" s="216"/>
       <c r="R116" s="216"/>
-    </row>
-    <row r="117" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S116" s="216"/>
+      <c r="T116" s="216"/>
+    </row>
+    <row r="117" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A117" s="217"/>
       <c r="B117" s="217"/>
       <c r="C117" s="217"/>
@@ -23666,8 +23898,10 @@
       <c r="P117" s="216"/>
       <c r="Q117" s="216"/>
       <c r="R117" s="216"/>
-    </row>
-    <row r="118" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S117" s="216"/>
+      <c r="T117" s="216"/>
+    </row>
+    <row r="118" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A118" s="217"/>
       <c r="B118" s="217"/>
       <c r="C118" s="217"/>
@@ -23686,8 +23920,10 @@
       <c r="P118" s="216"/>
       <c r="Q118" s="216"/>
       <c r="R118" s="216"/>
-    </row>
-    <row r="119" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S118" s="216"/>
+      <c r="T118" s="216"/>
+    </row>
+    <row r="119" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A119" s="217"/>
       <c r="B119" s="217"/>
       <c r="C119" s="217"/>
@@ -23706,8 +23942,10 @@
       <c r="P119" s="216"/>
       <c r="Q119" s="216"/>
       <c r="R119" s="216"/>
-    </row>
-    <row r="120" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S119" s="216"/>
+      <c r="T119" s="216"/>
+    </row>
+    <row r="120" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A120" s="217"/>
       <c r="B120" s="217"/>
       <c r="C120" s="217"/>
@@ -23726,8 +23964,10 @@
       <c r="P120" s="216"/>
       <c r="Q120" s="216"/>
       <c r="R120" s="216"/>
-    </row>
-    <row r="121" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S120" s="216"/>
+      <c r="T120" s="216"/>
+    </row>
+    <row r="121" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A121" s="217"/>
       <c r="B121" s="217"/>
       <c r="C121" s="217"/>
@@ -23746,8 +23986,10 @@
       <c r="P121" s="216"/>
       <c r="Q121" s="216"/>
       <c r="R121" s="216"/>
-    </row>
-    <row r="122" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S121" s="216"/>
+      <c r="T121" s="216"/>
+    </row>
+    <row r="122" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A122" s="217"/>
       <c r="B122" s="217"/>
       <c r="C122" s="217"/>
@@ -23766,8 +24008,10 @@
       <c r="P122" s="216"/>
       <c r="Q122" s="216"/>
       <c r="R122" s="216"/>
-    </row>
-    <row r="123" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S122" s="216"/>
+      <c r="T122" s="216"/>
+    </row>
+    <row r="123" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A123" s="217"/>
       <c r="B123" s="217"/>
       <c r="C123" s="217"/>
@@ -23786,8 +24030,10 @@
       <c r="P123" s="216"/>
       <c r="Q123" s="216"/>
       <c r="R123" s="216"/>
-    </row>
-    <row r="124" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S123" s="216"/>
+      <c r="T123" s="216"/>
+    </row>
+    <row r="124" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A124" s="217"/>
       <c r="B124" s="217"/>
       <c r="C124" s="217"/>
@@ -23806,8 +24052,10 @@
       <c r="P124" s="216"/>
       <c r="Q124" s="216"/>
       <c r="R124" s="216"/>
-    </row>
-    <row r="125" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S124" s="216"/>
+      <c r="T124" s="216"/>
+    </row>
+    <row r="125" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A125" s="217"/>
       <c r="B125" s="217"/>
       <c r="C125" s="217"/>
@@ -23826,8 +24074,10 @@
       <c r="P125" s="216"/>
       <c r="Q125" s="216"/>
       <c r="R125" s="216"/>
-    </row>
-    <row r="126" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S125" s="216"/>
+      <c r="T125" s="216"/>
+    </row>
+    <row r="126" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A126" s="217"/>
       <c r="B126" s="217"/>
       <c r="C126" s="217"/>
@@ -23846,8 +24096,10 @@
       <c r="P126" s="216"/>
       <c r="Q126" s="216"/>
       <c r="R126" s="216"/>
-    </row>
-    <row r="127" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S126" s="216"/>
+      <c r="T126" s="216"/>
+    </row>
+    <row r="127" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A127" s="217"/>
       <c r="B127" s="217"/>
       <c r="C127" s="217"/>
@@ -23866,8 +24118,10 @@
       <c r="P127" s="216"/>
       <c r="Q127" s="216"/>
       <c r="R127" s="216"/>
-    </row>
-    <row r="128" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S127" s="216"/>
+      <c r="T127" s="216"/>
+    </row>
+    <row r="128" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A128" s="217"/>
       <c r="B128" s="217"/>
       <c r="C128" s="217"/>
@@ -23886,8 +24140,10 @@
       <c r="P128" s="216"/>
       <c r="Q128" s="216"/>
       <c r="R128" s="216"/>
-    </row>
-    <row r="129" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S128" s="216"/>
+      <c r="T128" s="216"/>
+    </row>
+    <row r="129" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A129" s="217"/>
       <c r="B129" s="217"/>
       <c r="C129" s="217"/>
@@ -23906,8 +24162,10 @@
       <c r="P129" s="216"/>
       <c r="Q129" s="216"/>
       <c r="R129" s="216"/>
-    </row>
-    <row r="130" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S129" s="216"/>
+      <c r="T129" s="216"/>
+    </row>
+    <row r="130" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A130" s="217"/>
       <c r="B130" s="217"/>
       <c r="C130" s="217"/>
@@ -23926,8 +24184,10 @@
       <c r="P130" s="216"/>
       <c r="Q130" s="216"/>
       <c r="R130" s="216"/>
-    </row>
-    <row r="131" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S130" s="216"/>
+      <c r="T130" s="216"/>
+    </row>
+    <row r="131" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A131" s="217"/>
       <c r="B131" s="217"/>
       <c r="C131" s="217"/>
@@ -23946,8 +24206,10 @@
       <c r="P131" s="216"/>
       <c r="Q131" s="216"/>
       <c r="R131" s="216"/>
-    </row>
-    <row r="132" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S131" s="216"/>
+      <c r="T131" s="216"/>
+    </row>
+    <row r="132" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A132" s="217"/>
       <c r="B132" s="217"/>
       <c r="C132" s="217"/>
@@ -23966,8 +24228,10 @@
       <c r="P132" s="216"/>
       <c r="Q132" s="216"/>
       <c r="R132" s="216"/>
-    </row>
-    <row r="133" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S132" s="216"/>
+      <c r="T132" s="216"/>
+    </row>
+    <row r="133" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A133" s="217"/>
       <c r="B133" s="217"/>
       <c r="C133" s="217"/>
@@ -23986,8 +24250,10 @@
       <c r="P133" s="216"/>
       <c r="Q133" s="216"/>
       <c r="R133" s="216"/>
-    </row>
-    <row r="134" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S133" s="216"/>
+      <c r="T133" s="216"/>
+    </row>
+    <row r="134" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A134" s="217"/>
       <c r="B134" s="217"/>
       <c r="C134" s="217"/>
@@ -24006,8 +24272,10 @@
       <c r="P134" s="216"/>
       <c r="Q134" s="216"/>
       <c r="R134" s="216"/>
-    </row>
-    <row r="135" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S134" s="216"/>
+      <c r="T134" s="216"/>
+    </row>
+    <row r="135" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A135" s="217"/>
       <c r="B135" s="217"/>
       <c r="C135" s="217"/>
@@ -24026,8 +24294,10 @@
       <c r="P135" s="216"/>
       <c r="Q135" s="216"/>
       <c r="R135" s="216"/>
-    </row>
-    <row r="136" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S135" s="216"/>
+      <c r="T135" s="216"/>
+    </row>
+    <row r="136" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A136" s="217"/>
       <c r="B136" s="217"/>
       <c r="C136" s="217"/>
@@ -24046,8 +24316,10 @@
       <c r="P136" s="216"/>
       <c r="Q136" s="216"/>
       <c r="R136" s="216"/>
-    </row>
-    <row r="137" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S136" s="216"/>
+      <c r="T136" s="216"/>
+    </row>
+    <row r="137" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A137" s="217"/>
       <c r="B137" s="217"/>
       <c r="C137" s="217"/>
@@ -24066,8 +24338,10 @@
       <c r="P137" s="216"/>
       <c r="Q137" s="216"/>
       <c r="R137" s="216"/>
-    </row>
-    <row r="138" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S137" s="216"/>
+      <c r="T137" s="216"/>
+    </row>
+    <row r="138" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A138" s="217"/>
       <c r="B138" s="217"/>
       <c r="C138" s="217"/>
@@ -24086,8 +24360,10 @@
       <c r="P138" s="216"/>
       <c r="Q138" s="216"/>
       <c r="R138" s="216"/>
-    </row>
-    <row r="139" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S138" s="216"/>
+      <c r="T138" s="216"/>
+    </row>
+    <row r="139" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A139" s="217"/>
       <c r="B139" s="217"/>
       <c r="C139" s="217"/>
@@ -24106,8 +24382,10 @@
       <c r="P139" s="216"/>
       <c r="Q139" s="216"/>
       <c r="R139" s="216"/>
-    </row>
-    <row r="140" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S139" s="216"/>
+      <c r="T139" s="216"/>
+    </row>
+    <row r="140" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A140" s="217"/>
       <c r="B140" s="217"/>
       <c r="C140" s="217"/>
@@ -24126,8 +24404,10 @@
       <c r="P140" s="216"/>
       <c r="Q140" s="216"/>
       <c r="R140" s="216"/>
-    </row>
-    <row r="141" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S140" s="216"/>
+      <c r="T140" s="216"/>
+    </row>
+    <row r="141" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A141" s="217"/>
       <c r="B141" s="217"/>
       <c r="C141" s="217"/>
@@ -24146,8 +24426,10 @@
       <c r="P141" s="216"/>
       <c r="Q141" s="216"/>
       <c r="R141" s="216"/>
-    </row>
-    <row r="142" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S141" s="216"/>
+      <c r="T141" s="216"/>
+    </row>
+    <row r="142" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A142" s="217"/>
       <c r="B142" s="217"/>
       <c r="C142" s="217"/>
@@ -24166,8 +24448,10 @@
       <c r="P142" s="216"/>
       <c r="Q142" s="216"/>
       <c r="R142" s="216"/>
-    </row>
-    <row r="143" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S142" s="216"/>
+      <c r="T142" s="216"/>
+    </row>
+    <row r="143" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A143" s="217"/>
       <c r="B143" s="217"/>
       <c r="C143" s="217"/>
@@ -24186,8 +24470,10 @@
       <c r="P143" s="216"/>
       <c r="Q143" s="216"/>
       <c r="R143" s="216"/>
-    </row>
-    <row r="144" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="S143" s="216"/>
+      <c r="T143" s="216"/>
+    </row>
+    <row r="144" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A144" s="217"/>
       <c r="B144" s="217"/>
       <c r="C144" s="217"/>
@@ -24206,6 +24492,8 @@
       <c r="P144" s="216"/>
       <c r="Q144" s="216"/>
       <c r="R144" s="216"/>
+      <c r="S144" s="216"/>
+      <c r="T144" s="216"/>
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A145" s="217"/>
@@ -24219,7 +24507,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="Q2:Q4"/>
+    <mergeCell ref="S2:S4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -29846,16 +30134,16 @@
   <sheetPr>
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:BJ17"/>
+  <dimension ref="A1:BL17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="3" width="0" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="16.83203125" customWidth="1"/>
     <col min="6" max="6" width="68.83203125" customWidth="1"/>
-    <col min="7" max="16" width="13.5" customWidth="1"/>
+    <col min="7" max="18" width="13.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:62" s="4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:64" s="4" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3"/>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -29875,8 +30163,8 @@
       <c r="O1" s="7"/>
       <c r="P1" s="7"/>
       <c r="Q1" s="7"/>
-      <c r="R1"/>
-      <c r="S1"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="7"/>
       <c r="T1"/>
       <c r="U1"/>
       <c r="V1"/>
@@ -29920,8 +30208,10 @@
       <c r="BH1"/>
       <c r="BI1"/>
       <c r="BJ1"/>
-    </row>
-    <row r="2" spans="1:62" hidden="1" x14ac:dyDescent="0.2">
+      <c r="BK1"/>
+      <c r="BL1"/>
+    </row>
+    <row r="2" spans="1:64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" s="254"/>
       <c r="B2" s="207"/>
       <c r="C2" s="207"/>
@@ -29942,23 +30232,25 @@
       <c r="L2" s="208" t="s">
         <v>38</v>
       </c>
-      <c r="M2" s="208" t="s">
-        <v>38</v>
-      </c>
-      <c r="N2" s="208" t="s">
-        <v>38</v>
-      </c>
+      <c r="M2" s="208"/>
+      <c r="N2" s="208"/>
       <c r="O2" s="208" t="s">
         <v>38</v>
       </c>
       <c r="P2" s="208" t="s">
         <v>38</v>
       </c>
-      <c r="Q2" s="418" t="s">
+      <c r="Q2" s="208" t="s">
+        <v>38</v>
+      </c>
+      <c r="R2" s="208" t="s">
+        <v>38</v>
+      </c>
+      <c r="S2" s="418" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="3" spans="1:62" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" s="254"/>
       <c r="B3" s="207"/>
       <c r="C3" s="207"/>
@@ -29979,21 +30271,23 @@
       <c r="L3" s="208" t="s">
         <v>144</v>
       </c>
-      <c r="M3" s="208" t="s">
+      <c r="M3" s="208"/>
+      <c r="N3" s="208"/>
+      <c r="O3" s="208" t="s">
         <v>275</v>
       </c>
-      <c r="N3" s="208" t="s">
+      <c r="P3" s="208" t="s">
         <v>276</v>
       </c>
-      <c r="O3" s="208" t="s">
+      <c r="Q3" s="208" t="s">
         <v>277</v>
       </c>
-      <c r="P3" s="208" t="s">
+      <c r="R3" s="208" t="s">
         <v>278</v>
       </c>
-      <c r="Q3" s="418"/>
-    </row>
-    <row r="4" spans="1:62" ht="36" x14ac:dyDescent="0.2">
+      <c r="S3" s="418"/>
+    </row>
+    <row r="4" spans="1:64" ht="36" x14ac:dyDescent="0.2">
       <c r="A4" s="255"/>
       <c r="B4" s="244" t="s">
         <v>112</v>
@@ -30029,20 +30323,26 @@
         <v>677</v>
       </c>
       <c r="M4" s="249" t="s">
+        <v>684</v>
+      </c>
+      <c r="N4" s="249" t="s">
+        <v>685</v>
+      </c>
+      <c r="O4" s="249" t="s">
         <v>678</v>
       </c>
-      <c r="N4" s="249" t="s">
+      <c r="P4" s="249" t="s">
         <v>679</v>
       </c>
-      <c r="O4" s="249" t="s">
+      <c r="Q4" s="249" t="s">
         <v>680</v>
       </c>
-      <c r="P4" s="249" t="s">
+      <c r="R4" s="249" t="s">
         <v>676</v>
       </c>
-      <c r="Q4" s="418"/>
-    </row>
-    <row r="5" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="S4" s="418"/>
+    </row>
+    <row r="5" spans="1:64" x14ac:dyDescent="0.2">
       <c r="A5" s="211" t="s">
         <v>290</v>
       </c>
@@ -30079,14 +30379,8 @@
         <f>IF(ISBLANK(ETPT_JUR_ASS!L5),"",IF(ISERROR(ETPT_JUR_ASS!L5),"",IF(ETPT_JUR_ASS!L5=0,"",ETPT_JUR_ASS!L5)))</f>
         <v/>
       </c>
-      <c r="M5" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_JUR_ASS!M5),"",IF(ISERROR(ETPT_JUR_ASS!M5),"",IF(ETPT_JUR_ASS!M5=0,"",ETPT_JUR_ASS!M5)))</f>
-        <v/>
-      </c>
-      <c r="N5" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_JUR_ASS!N5),"",IF(ISERROR(ETPT_JUR_ASS!N5),"",IF(ETPT_JUR_ASS!N5=0,"",ETPT_JUR_ASS!N5)))</f>
-        <v/>
-      </c>
+      <c r="M5" s="247"/>
+      <c r="N5" s="247"/>
       <c r="O5" s="247" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!O5),"",IF(ISERROR(ETPT_JUR_ASS!O5),"",IF(ETPT_JUR_ASS!O5=0,"",ETPT_JUR_ASS!O5)))</f>
         <v/>
@@ -30095,12 +30389,20 @@
         <f>IF(ISBLANK(ETPT_JUR_ASS!P5),"",IF(ISERROR(ETPT_JUR_ASS!P5),"",IF(ETPT_JUR_ASS!P5=0,"",ETPT_JUR_ASS!P5)))</f>
         <v/>
       </c>
-      <c r="Q5" s="214">
-        <f>ETPT_JUR_ASS!Q5</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="Q5" s="247" t="str">
+        <f>IF(ISBLANK(ETPT_JUR_ASS!Q5),"",IF(ISERROR(ETPT_JUR_ASS!Q5),"",IF(ETPT_JUR_ASS!Q5=0,"",ETPT_JUR_ASS!Q5)))</f>
+        <v/>
+      </c>
+      <c r="R5" s="247" t="str">
+        <f>IF(ISBLANK(ETPT_JUR_ASS!R5),"",IF(ISERROR(ETPT_JUR_ASS!R5),"",IF(ETPT_JUR_ASS!R5=0,"",ETPT_JUR_ASS!R5)))</f>
+        <v/>
+      </c>
+      <c r="S5" s="214">
+        <f>ETPT_JUR_ASS!S5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:64" x14ac:dyDescent="0.2">
       <c r="A6" s="211" t="s">
         <v>290</v>
       </c>
@@ -30134,14 +30436,8 @@
         <f>IF(ISBLANK(ETPT_JUR_ASS!L6),"",IF(ISERROR(ETPT_JUR_ASS!L6),"",IF(ETPT_JUR_ASS!L6=0,"",ETPT_JUR_ASS!L6)))</f>
         <v/>
       </c>
-      <c r="M6" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_JUR_ASS!M6),"",IF(ISERROR(ETPT_JUR_ASS!M6),"",IF(ETPT_JUR_ASS!M6=0,"",ETPT_JUR_ASS!M6)))</f>
-        <v/>
-      </c>
-      <c r="N6" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_JUR_ASS!N6),"",IF(ISERROR(ETPT_JUR_ASS!N6),"",IF(ETPT_JUR_ASS!N6=0,"",ETPT_JUR_ASS!N6)))</f>
-        <v/>
-      </c>
+      <c r="M6" s="247"/>
+      <c r="N6" s="247"/>
       <c r="O6" s="247" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!O6),"",IF(ISERROR(ETPT_JUR_ASS!O6),"",IF(ETPT_JUR_ASS!O6=0,"",ETPT_JUR_ASS!O6)))</f>
         <v/>
@@ -30150,12 +30446,20 @@
         <f>IF(ISBLANK(ETPT_JUR_ASS!P6),"",IF(ISERROR(ETPT_JUR_ASS!P6),"",IF(ETPT_JUR_ASS!P6=0,"",ETPT_JUR_ASS!P6)))</f>
         <v/>
       </c>
-      <c r="Q6" s="214">
-        <f>ETPT_JUR_ASS!Q6</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="Q6" s="247" t="str">
+        <f>IF(ISBLANK(ETPT_JUR_ASS!Q6),"",IF(ISERROR(ETPT_JUR_ASS!Q6),"",IF(ETPT_JUR_ASS!Q6=0,"",ETPT_JUR_ASS!Q6)))</f>
+        <v/>
+      </c>
+      <c r="R6" s="247" t="str">
+        <f>IF(ISBLANK(ETPT_JUR_ASS!R6),"",IF(ISERROR(ETPT_JUR_ASS!R6),"",IF(ETPT_JUR_ASS!R6=0,"",ETPT_JUR_ASS!R6)))</f>
+        <v/>
+      </c>
+      <c r="S6" s="214">
+        <f>ETPT_JUR_ASS!S6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:64" x14ac:dyDescent="0.2">
       <c r="A7" s="211" t="s">
         <v>290</v>
       </c>
@@ -30189,14 +30493,8 @@
         <f>IF(ISBLANK(ETPT_JUR_ASS!L7),"",IF(ISERROR(ETPT_JUR_ASS!L7),"",IF(ETPT_JUR_ASS!L7=0,"",ETPT_JUR_ASS!L7)))</f>
         <v/>
       </c>
-      <c r="M7" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_JUR_ASS!M7),"",IF(ISERROR(ETPT_JUR_ASS!M7),"",IF(ETPT_JUR_ASS!M7=0,"",ETPT_JUR_ASS!M7)))</f>
-        <v/>
-      </c>
-      <c r="N7" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_JUR_ASS!N7),"",IF(ISERROR(ETPT_JUR_ASS!N7),"",IF(ETPT_JUR_ASS!N7=0,"",ETPT_JUR_ASS!N7)))</f>
-        <v/>
-      </c>
+      <c r="M7" s="247"/>
+      <c r="N7" s="247"/>
       <c r="O7" s="247" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!O7),"",IF(ISERROR(ETPT_JUR_ASS!O7),"",IF(ETPT_JUR_ASS!O7=0,"",ETPT_JUR_ASS!O7)))</f>
         <v/>
@@ -30205,12 +30503,20 @@
         <f>IF(ISBLANK(ETPT_JUR_ASS!P7),"",IF(ISERROR(ETPT_JUR_ASS!P7),"",IF(ETPT_JUR_ASS!P7=0,"",ETPT_JUR_ASS!P7)))</f>
         <v/>
       </c>
-      <c r="Q7" s="214">
-        <f>ETPT_JUR_ASS!Q7</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="Q7" s="247" t="str">
+        <f>IF(ISBLANK(ETPT_JUR_ASS!Q7),"",IF(ISERROR(ETPT_JUR_ASS!Q7),"",IF(ETPT_JUR_ASS!Q7=0,"",ETPT_JUR_ASS!Q7)))</f>
+        <v/>
+      </c>
+      <c r="R7" s="247" t="str">
+        <f>IF(ISBLANK(ETPT_JUR_ASS!R7),"",IF(ISERROR(ETPT_JUR_ASS!R7),"",IF(ETPT_JUR_ASS!R7=0,"",ETPT_JUR_ASS!R7)))</f>
+        <v/>
+      </c>
+      <c r="S7" s="214">
+        <f>ETPT_JUR_ASS!S7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:64" x14ac:dyDescent="0.2">
       <c r="A8" s="211" t="s">
         <v>290</v>
       </c>
@@ -30244,14 +30550,8 @@
         <f>IF(ISBLANK(ETPT_JUR_ASS!L8),"",IF(ISERROR(ETPT_JUR_ASS!L8),"",IF(ETPT_JUR_ASS!L8=0,"",ETPT_JUR_ASS!L8)))</f>
         <v/>
       </c>
-      <c r="M8" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_JUR_ASS!M8),"",IF(ISERROR(ETPT_JUR_ASS!M8),"",IF(ETPT_JUR_ASS!M8=0,"",ETPT_JUR_ASS!M8)))</f>
-        <v/>
-      </c>
-      <c r="N8" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_JUR_ASS!N8),"",IF(ISERROR(ETPT_JUR_ASS!N8),"",IF(ETPT_JUR_ASS!N8=0,"",ETPT_JUR_ASS!N8)))</f>
-        <v/>
-      </c>
+      <c r="M8" s="247"/>
+      <c r="N8" s="247"/>
       <c r="O8" s="247" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!O8),"",IF(ISERROR(ETPT_JUR_ASS!O8),"",IF(ETPT_JUR_ASS!O8=0,"",ETPT_JUR_ASS!O8)))</f>
         <v/>
@@ -30260,12 +30560,20 @@
         <f>IF(ISBLANK(ETPT_JUR_ASS!P8),"",IF(ISERROR(ETPT_JUR_ASS!P8),"",IF(ETPT_JUR_ASS!P8=0,"",ETPT_JUR_ASS!P8)))</f>
         <v/>
       </c>
-      <c r="Q8" s="214">
-        <f>ETPT_JUR_ASS!Q8</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="Q8" s="247" t="str">
+        <f>IF(ISBLANK(ETPT_JUR_ASS!Q8),"",IF(ISERROR(ETPT_JUR_ASS!Q8),"",IF(ETPT_JUR_ASS!Q8=0,"",ETPT_JUR_ASS!Q8)))</f>
+        <v/>
+      </c>
+      <c r="R8" s="247" t="str">
+        <f>IF(ISBLANK(ETPT_JUR_ASS!R8),"",IF(ISERROR(ETPT_JUR_ASS!R8),"",IF(ETPT_JUR_ASS!R8=0,"",ETPT_JUR_ASS!R8)))</f>
+        <v/>
+      </c>
+      <c r="S8" s="214">
+        <f>ETPT_JUR_ASS!S8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:64" x14ac:dyDescent="0.2">
       <c r="A9" s="211" t="s">
         <v>290</v>
       </c>
@@ -30299,14 +30607,8 @@
         <f>IF(ISBLANK(ETPT_JUR_ASS!L9),"",IF(ISERROR(ETPT_JUR_ASS!L9),"",IF(ETPT_JUR_ASS!L9=0,"",ETPT_JUR_ASS!L9)))</f>
         <v/>
       </c>
-      <c r="M9" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_JUR_ASS!M9),"",IF(ISERROR(ETPT_JUR_ASS!M9),"",IF(ETPT_JUR_ASS!M9=0,"",ETPT_JUR_ASS!M9)))</f>
-        <v/>
-      </c>
-      <c r="N9" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_JUR_ASS!N9),"",IF(ISERROR(ETPT_JUR_ASS!N9),"",IF(ETPT_JUR_ASS!N9=0,"",ETPT_JUR_ASS!N9)))</f>
-        <v/>
-      </c>
+      <c r="M9" s="247"/>
+      <c r="N9" s="247"/>
       <c r="O9" s="247" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!O9),"",IF(ISERROR(ETPT_JUR_ASS!O9),"",IF(ETPT_JUR_ASS!O9=0,"",ETPT_JUR_ASS!O9)))</f>
         <v/>
@@ -30315,12 +30617,20 @@
         <f>IF(ISBLANK(ETPT_JUR_ASS!P9),"",IF(ISERROR(ETPT_JUR_ASS!P9),"",IF(ETPT_JUR_ASS!P9=0,"",ETPT_JUR_ASS!P9)))</f>
         <v/>
       </c>
-      <c r="Q9" s="214">
-        <f>ETPT_JUR_ASS!Q9</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="Q9" s="247" t="str">
+        <f>IF(ISBLANK(ETPT_JUR_ASS!Q9),"",IF(ISERROR(ETPT_JUR_ASS!Q9),"",IF(ETPT_JUR_ASS!Q9=0,"",ETPT_JUR_ASS!Q9)))</f>
+        <v/>
+      </c>
+      <c r="R9" s="247" t="str">
+        <f>IF(ISBLANK(ETPT_JUR_ASS!R9),"",IF(ISERROR(ETPT_JUR_ASS!R9),"",IF(ETPT_JUR_ASS!R9=0,"",ETPT_JUR_ASS!R9)))</f>
+        <v/>
+      </c>
+      <c r="S9" s="214">
+        <f>ETPT_JUR_ASS!S9</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:64" x14ac:dyDescent="0.2">
       <c r="A10" s="211" t="s">
         <v>290</v>
       </c>
@@ -30354,14 +30664,8 @@
         <f>IF(ISBLANK(ETPT_JUR_ASS!L10),"",IF(ISERROR(ETPT_JUR_ASS!L10),"",IF(ETPT_JUR_ASS!L10=0,"",ETPT_JUR_ASS!L10)))</f>
         <v/>
       </c>
-      <c r="M10" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_JUR_ASS!M10),"",IF(ISERROR(ETPT_JUR_ASS!M10),"",IF(ETPT_JUR_ASS!M10=0,"",ETPT_JUR_ASS!M10)))</f>
-        <v/>
-      </c>
-      <c r="N10" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_JUR_ASS!N10),"",IF(ISERROR(ETPT_JUR_ASS!N10),"",IF(ETPT_JUR_ASS!N10=0,"",ETPT_JUR_ASS!N10)))</f>
-        <v/>
-      </c>
+      <c r="M10" s="247"/>
+      <c r="N10" s="247"/>
       <c r="O10" s="247" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!O10),"",IF(ISERROR(ETPT_JUR_ASS!O10),"",IF(ETPT_JUR_ASS!O10=0,"",ETPT_JUR_ASS!O10)))</f>
         <v/>
@@ -30370,12 +30674,20 @@
         <f>IF(ISBLANK(ETPT_JUR_ASS!P10),"",IF(ISERROR(ETPT_JUR_ASS!P10),"",IF(ETPT_JUR_ASS!P10=0,"",ETPT_JUR_ASS!P10)))</f>
         <v/>
       </c>
-      <c r="Q10" s="214">
-        <f>ETPT_JUR_ASS!Q10</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="Q10" s="247" t="str">
+        <f>IF(ISBLANK(ETPT_JUR_ASS!Q10),"",IF(ISERROR(ETPT_JUR_ASS!Q10),"",IF(ETPT_JUR_ASS!Q10=0,"",ETPT_JUR_ASS!Q10)))</f>
+        <v/>
+      </c>
+      <c r="R10" s="247" t="str">
+        <f>IF(ISBLANK(ETPT_JUR_ASS!R10),"",IF(ISERROR(ETPT_JUR_ASS!R10),"",IF(ETPT_JUR_ASS!R10=0,"",ETPT_JUR_ASS!R10)))</f>
+        <v/>
+      </c>
+      <c r="S10" s="214">
+        <f>ETPT_JUR_ASS!S10</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:64" x14ac:dyDescent="0.2">
       <c r="A11" s="211" t="s">
         <v>290</v>
       </c>
@@ -30409,14 +30721,8 @@
         <f>IF(ISBLANK(ETPT_JUR_ASS!L11),"",IF(ISERROR(ETPT_JUR_ASS!L11),"",IF(ETPT_JUR_ASS!L11=0,"",ETPT_JUR_ASS!L11)))</f>
         <v/>
       </c>
-      <c r="M11" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_JUR_ASS!M11),"",IF(ISERROR(ETPT_JUR_ASS!M11),"",IF(ETPT_JUR_ASS!M11=0,"",ETPT_JUR_ASS!M11)))</f>
-        <v/>
-      </c>
-      <c r="N11" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_JUR_ASS!N11),"",IF(ISERROR(ETPT_JUR_ASS!N11),"",IF(ETPT_JUR_ASS!N11=0,"",ETPT_JUR_ASS!N11)))</f>
-        <v/>
-      </c>
+      <c r="M11" s="247"/>
+      <c r="N11" s="247"/>
       <c r="O11" s="247" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!O11),"",IF(ISERROR(ETPT_JUR_ASS!O11),"",IF(ETPT_JUR_ASS!O11=0,"",ETPT_JUR_ASS!O11)))</f>
         <v/>
@@ -30425,12 +30731,20 @@
         <f>IF(ISBLANK(ETPT_JUR_ASS!P11),"",IF(ISERROR(ETPT_JUR_ASS!P11),"",IF(ETPT_JUR_ASS!P11=0,"",ETPT_JUR_ASS!P11)))</f>
         <v/>
       </c>
-      <c r="Q11" s="214">
-        <f>ETPT_JUR_ASS!Q11</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="Q11" s="247" t="str">
+        <f>IF(ISBLANK(ETPT_JUR_ASS!Q11),"",IF(ISERROR(ETPT_JUR_ASS!Q11),"",IF(ETPT_JUR_ASS!Q11=0,"",ETPT_JUR_ASS!Q11)))</f>
+        <v/>
+      </c>
+      <c r="R11" s="247" t="str">
+        <f>IF(ISBLANK(ETPT_JUR_ASS!R11),"",IF(ISERROR(ETPT_JUR_ASS!R11),"",IF(ETPT_JUR_ASS!R11=0,"",ETPT_JUR_ASS!R11)))</f>
+        <v/>
+      </c>
+      <c r="S11" s="214">
+        <f>ETPT_JUR_ASS!S11</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:64" x14ac:dyDescent="0.2">
       <c r="A12" s="211" t="s">
         <v>290</v>
       </c>
@@ -30464,14 +30778,8 @@
         <f>IF(ISBLANK(ETPT_JUR_ASS!L12),"",IF(ISERROR(ETPT_JUR_ASS!L12),"",IF(ETPT_JUR_ASS!L12=0,"",ETPT_JUR_ASS!L12)))</f>
         <v/>
       </c>
-      <c r="M12" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_JUR_ASS!M12),"",IF(ISERROR(ETPT_JUR_ASS!M12),"",IF(ETPT_JUR_ASS!M12=0,"",ETPT_JUR_ASS!M12)))</f>
-        <v/>
-      </c>
-      <c r="N12" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_JUR_ASS!N12),"",IF(ISERROR(ETPT_JUR_ASS!N12),"",IF(ETPT_JUR_ASS!N12=0,"",ETPT_JUR_ASS!N12)))</f>
-        <v/>
-      </c>
+      <c r="M12" s="247"/>
+      <c r="N12" s="247"/>
       <c r="O12" s="247" t="str">
         <f>IF(ISBLANK(ETPT_JUR_ASS!O12),"",IF(ISERROR(ETPT_JUR_ASS!O12),"",IF(ETPT_JUR_ASS!O12=0,"",ETPT_JUR_ASS!O12)))</f>
         <v/>
@@ -30480,12 +30788,20 @@
         <f>IF(ISBLANK(ETPT_JUR_ASS!P12),"",IF(ISERROR(ETPT_JUR_ASS!P12),"",IF(ETPT_JUR_ASS!P12=0,"",ETPT_JUR_ASS!P12)))</f>
         <v/>
       </c>
-      <c r="Q12" s="214">
-        <f>ETPT_JUR_ASS!Q12</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="Q12" s="247" t="str">
+        <f>IF(ISBLANK(ETPT_JUR_ASS!Q12),"",IF(ISERROR(ETPT_JUR_ASS!Q12),"",IF(ETPT_JUR_ASS!Q12=0,"",ETPT_JUR_ASS!Q12)))</f>
+        <v/>
+      </c>
+      <c r="R12" s="247" t="str">
+        <f>IF(ISBLANK(ETPT_JUR_ASS!R12),"",IF(ISERROR(ETPT_JUR_ASS!R12),"",IF(ETPT_JUR_ASS!R12=0,"",ETPT_JUR_ASS!R12)))</f>
+        <v/>
+      </c>
+      <c r="S12" s="214">
+        <f>ETPT_JUR_ASS!S12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:64" x14ac:dyDescent="0.2">
       <c r="A13" s="246"/>
       <c r="B13" s="246"/>
       <c r="C13" s="246"/>
@@ -30518,14 +30834,8 @@
         <f>ETPT_JUR_ASS!L13</f>
         <v>0</v>
       </c>
-      <c r="M13" s="214">
-        <f>ETPT_JUR_ASS!M13</f>
-        <v>0</v>
-      </c>
-      <c r="N13" s="214">
-        <f>ETPT_JUR_ASS!N13</f>
-        <v>0</v>
-      </c>
+      <c r="M13" s="214"/>
+      <c r="N13" s="214"/>
       <c r="O13" s="214">
         <f>ETPT_JUR_ASS!O13</f>
         <v>0</v>
@@ -30538,8 +30848,16 @@
         <f>ETPT_JUR_ASS!Q13</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+      <c r="R13" s="214">
+        <f>ETPT_JUR_ASS!R13</f>
+        <v>0</v>
+      </c>
+      <c r="S13" s="214">
+        <f>ETPT_JUR_ASS!S13</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:64" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="217"/>
       <c r="B14" s="217"/>
       <c r="C14" s="217"/>
@@ -30558,8 +30876,10 @@
       <c r="P14" s="216"/>
       <c r="Q14" s="216"/>
       <c r="R14" s="216"/>
-    </row>
-    <row r="15" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+      <c r="S14" s="216"/>
+      <c r="T14" s="216"/>
+    </row>
+    <row r="15" spans="1:64" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="217"/>
       <c r="B15" s="217"/>
       <c r="C15" s="217"/>
@@ -30579,8 +30899,10 @@
       <c r="P15" s="216"/>
       <c r="Q15" s="216"/>
       <c r="R15" s="216"/>
-    </row>
-    <row r="16" spans="1:62" ht="16" x14ac:dyDescent="0.2">
+      <c r="S15" s="216"/>
+      <c r="T15" s="216"/>
+    </row>
+    <row r="16" spans="1:64" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="217"/>
       <c r="B16" s="217"/>
       <c r="C16" s="217"/>
@@ -30598,8 +30920,10 @@
       <c r="O16" s="216"/>
       <c r="P16" s="216"/>
       <c r="Q16" s="216"/>
-    </row>
-    <row r="17" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="R16" s="216"/>
+      <c r="S16" s="216"/>
+    </row>
+    <row r="17" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="217"/>
       <c r="B17" s="217"/>
       <c r="C17" s="217"/>
@@ -30618,10 +30942,12 @@
       <c r="P17" s="216"/>
       <c r="Q17" s="216"/>
       <c r="R17" s="216"/>
+      <c r="S17" s="216"/>
+      <c r="T17" s="216"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="Q2:Q4"/>
+    <mergeCell ref="S2:S4"/>
   </mergeCells>
   <phoneticPr fontId="68" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -37985,7 +38311,7 @@
         <v>86</v>
       </c>
       <c r="AF4" s="69" t="s">
-        <v>85</v>
+        <v>670</v>
       </c>
       <c r="AG4" s="415"/>
       <c r="AH4" s="69" t="s">

</xml_diff>

<commit_message>
Update tab names in template4.xlsx
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69B3E188-CE49-144E-96BF-F010583622E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FF01C49-2529-E649-9666-9B966F986BA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="13" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="1" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -22,11 +22,11 @@
     <sheet name="ETPT_TJ" sheetId="25" state="hidden" r:id="rId7"/>
     <sheet name="ETPT_TPRX" sheetId="26" state="hidden" r:id="rId8"/>
     <sheet name="ETPT_CPH" sheetId="27" state="hidden" r:id="rId9"/>
-    <sheet name="ETPT_ATT_JUR" sheetId="38" state="hidden" r:id="rId10"/>
+    <sheet name="ETPT_ATTJ" sheetId="38" r:id="rId10"/>
     <sheet name="ETPT_TJ_DDG" sheetId="28" r:id="rId11"/>
     <sheet name="ETPT_TPRX_DDG" sheetId="29" r:id="rId12"/>
     <sheet name="ETPT_CPH_DDG" sheetId="30" r:id="rId13"/>
-    <sheet name="ETPT_ATT_JUR_DDG" sheetId="39" r:id="rId14"/>
+    <sheet name="ETPT_ATTJ_DDG" sheetId="39" r:id="rId14"/>
     <sheet name="Juridictions" sheetId="17" state="hidden" r:id="rId15"/>
     <sheet name="ETPT_TJ_corresp-SIEGE-TJ" sheetId="24" state="hidden" r:id="rId16"/>
     <sheet name="ETPT_TPROX_corresp-SIEGE-TPROX" sheetId="34" state="hidden" r:id="rId17"/>
@@ -20877,7 +20877,7 @@
       <c r="B5" s="212"/>
       <c r="C5" s="212"/>
       <c r="D5" s="212">
-        <f>ETPT_ATT_JUR_DDG!D5</f>
+        <f>ETPT_ATTJ_DDG!D5</f>
         <v>0</v>
       </c>
       <c r="E5" s="212" t="s">
@@ -20980,7 +20980,7 @@
       <c r="B6" s="212"/>
       <c r="C6" s="212"/>
       <c r="D6" s="212">
-        <f>ETPT_ATT_JUR_DDG!D6</f>
+        <f>ETPT_ATTJ_DDG!D6</f>
         <v>0</v>
       </c>
       <c r="E6" s="212" t="s">
@@ -21113,7 +21113,7 @@
       <c r="B7" s="212"/>
       <c r="C7" s="212"/>
       <c r="D7" s="212">
-        <f>ETPT_ATT_JUR_DDG!D7</f>
+        <f>ETPT_ATTJ_DDG!D7</f>
         <v>0</v>
       </c>
       <c r="E7" s="212" t="s">
@@ -21206,7 +21206,7 @@
       <c r="B8" s="212"/>
       <c r="C8" s="212"/>
       <c r="D8" s="212">
-        <f>ETPT_ATT_JUR_DDG!D8</f>
+        <f>ETPT_ATTJ_DDG!D8</f>
         <v>0</v>
       </c>
       <c r="E8" s="212" t="s">
@@ -21379,7 +21379,7 @@
       <c r="B9" s="212"/>
       <c r="C9" s="212"/>
       <c r="D9" s="212">
-        <f>ETPT_ATT_JUR_DDG!D9</f>
+        <f>ETPT_ATTJ_DDG!D9</f>
         <v>0</v>
       </c>
       <c r="E9" s="212" t="s">
@@ -21472,7 +21472,7 @@
       <c r="B10" s="212"/>
       <c r="C10" s="212"/>
       <c r="D10" s="212">
-        <f>ETPT_ATT_JUR_DDG!D10</f>
+        <f>ETPT_ATTJ_DDG!D10</f>
         <v>0</v>
       </c>
       <c r="E10" s="212" t="s">
@@ -21565,7 +21565,7 @@
       <c r="B11" s="212"/>
       <c r="C11" s="212"/>
       <c r="D11" s="212">
-        <f>ETPT_ATT_JUR_DDG!D11</f>
+        <f>ETPT_ATTJ_DDG!D11</f>
         <v>0</v>
       </c>
       <c r="E11" s="212" t="s">
@@ -21698,7 +21698,7 @@
       <c r="B12" s="212"/>
       <c r="C12" s="212"/>
       <c r="D12" s="212">
-        <f>ETPT_ATT_JUR_DDG!D12</f>
+        <f>ETPT_ATTJ_DDG!D12</f>
         <v>0</v>
       </c>
       <c r="E12" s="212" t="s">
@@ -30602,43 +30602,43 @@
         <v>61</v>
       </c>
       <c r="G5" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!G5),"",IF(ISERROR(ETPT_ATT_JUR!G5),"",IF(ETPT_ATT_JUR!G5=0,"",ETPT_ATT_JUR!G5)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!G5),"",IF(ISERROR(ETPT_ATTJ!G5),"",IF(ETPT_ATTJ!G5=0,"",ETPT_ATTJ!G5)))</f>
         <v/>
       </c>
       <c r="H5" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!H5),"",IF(ISERROR(ETPT_ATT_JUR!H5),"",IF(ETPT_ATT_JUR!H5=0,"",ETPT_ATT_JUR!H5)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!H5),"",IF(ISERROR(ETPT_ATTJ!H5),"",IF(ETPT_ATTJ!H5=0,"",ETPT_ATTJ!H5)))</f>
         <v/>
       </c>
       <c r="I5" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!I5),"",IF(ISERROR(ETPT_ATT_JUR!I5),"",IF(ETPT_ATT_JUR!I5=0,"",ETPT_ATT_JUR!I5)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!I5),"",IF(ISERROR(ETPT_ATTJ!I5),"",IF(ETPT_ATTJ!I5=0,"",ETPT_ATTJ!I5)))</f>
         <v/>
       </c>
       <c r="J5" s="247"/>
       <c r="K5" s="247"/>
       <c r="L5" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!L5),"",IF(ISERROR(ETPT_ATT_JUR!L5),"",IF(ETPT_ATT_JUR!L5=0,"",ETPT_ATT_JUR!L5)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!L5),"",IF(ISERROR(ETPT_ATTJ!L5),"",IF(ETPT_ATTJ!L5=0,"",ETPT_ATTJ!L5)))</f>
         <v/>
       </c>
       <c r="M5" s="247"/>
       <c r="N5" s="247"/>
       <c r="O5" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!O5),"",IF(ISERROR(ETPT_ATT_JUR!O5),"",IF(ETPT_ATT_JUR!O5=0,"",ETPT_ATT_JUR!O5)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!O5),"",IF(ISERROR(ETPT_ATTJ!O5),"",IF(ETPT_ATTJ!O5=0,"",ETPT_ATTJ!O5)))</f>
         <v/>
       </c>
       <c r="P5" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!P5),"",IF(ISERROR(ETPT_ATT_JUR!P5),"",IF(ETPT_ATT_JUR!P5=0,"",ETPT_ATT_JUR!P5)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!P5),"",IF(ISERROR(ETPT_ATTJ!P5),"",IF(ETPT_ATTJ!P5=0,"",ETPT_ATTJ!P5)))</f>
         <v/>
       </c>
       <c r="Q5" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!Q5),"",IF(ISERROR(ETPT_ATT_JUR!Q5),"",IF(ETPT_ATT_JUR!Q5=0,"",ETPT_ATT_JUR!Q5)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!Q5),"",IF(ISERROR(ETPT_ATTJ!Q5),"",IF(ETPT_ATTJ!Q5=0,"",ETPT_ATTJ!Q5)))</f>
         <v/>
       </c>
       <c r="R5" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!R5),"",IF(ISERROR(ETPT_ATT_JUR!R5),"",IF(ETPT_ATT_JUR!R5=0,"",ETPT_ATT_JUR!R5)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!R5),"",IF(ISERROR(ETPT_ATTJ!R5),"",IF(ETPT_ATTJ!R5=0,"",ETPT_ATTJ!R5)))</f>
         <v/>
       </c>
       <c r="S5" s="214">
-        <f>ETPT_ATT_JUR!S5</f>
+        <f>ETPT_ATTJ!S5</f>
         <v>0</v>
       </c>
     </row>
@@ -30659,49 +30659,49 @@
         <v>59</v>
       </c>
       <c r="G6" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!G6),"",IF(ISERROR(ETPT_ATT_JUR!G6),"",IF(ETPT_ATT_JUR!G6=0,"",ETPT_ATT_JUR!G6)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!G6),"",IF(ISERROR(ETPT_ATTJ!G6),"",IF(ETPT_ATTJ!G6=0,"",ETPT_ATTJ!G6)))</f>
         <v/>
       </c>
       <c r="H6" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!H6),"",IF(ISERROR(ETPT_ATT_JUR!H6),"",IF(ETPT_ATT_JUR!H6=0,"",ETPT_ATT_JUR!H6)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!H6),"",IF(ISERROR(ETPT_ATTJ!H6),"",IF(ETPT_ATTJ!H6=0,"",ETPT_ATTJ!H6)))</f>
         <v/>
       </c>
       <c r="I6" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!I6),"",IF(ISERROR(ETPT_ATT_JUR!I6),"",IF(ETPT_ATT_JUR!I6=0,"",ETPT_ATT_JUR!I6)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!I6),"",IF(ISERROR(ETPT_ATTJ!I6),"",IF(ETPT_ATTJ!I6=0,"",ETPT_ATTJ!I6)))</f>
         <v/>
       </c>
       <c r="J6" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!J6),"",IF(ISERROR(ETPT_ATT_JUR!J6),"",IF(ETPT_ATT_JUR!J6=0,"",ETPT_ATT_JUR!J6)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!J6),"",IF(ISERROR(ETPT_ATTJ!J6),"",IF(ETPT_ATTJ!J6=0,"",ETPT_ATTJ!J6)))</f>
         <v/>
       </c>
       <c r="K6" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!K6),"",IF(ISERROR(ETPT_ATT_JUR!K6),"",IF(ETPT_ATT_JUR!K6=0,"",ETPT_ATT_JUR!K6)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!K6),"",IF(ISERROR(ETPT_ATTJ!K6),"",IF(ETPT_ATTJ!K6=0,"",ETPT_ATTJ!K6)))</f>
         <v/>
       </c>
       <c r="L6" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!L6),"",IF(ISERROR(ETPT_ATT_JUR!L6),"",IF(ETPT_ATT_JUR!L6=0,"",ETPT_ATT_JUR!L6)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!L6),"",IF(ISERROR(ETPT_ATTJ!L6),"",IF(ETPT_ATTJ!L6=0,"",ETPT_ATTJ!L6)))</f>
         <v/>
       </c>
       <c r="M6" s="247"/>
       <c r="N6" s="247"/>
       <c r="O6" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!O6),"",IF(ISERROR(ETPT_ATT_JUR!O6),"",IF(ETPT_ATT_JUR!O6=0,"",ETPT_ATT_JUR!O6)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!O6),"",IF(ISERROR(ETPT_ATTJ!O6),"",IF(ETPT_ATTJ!O6=0,"",ETPT_ATTJ!O6)))</f>
         <v/>
       </c>
       <c r="P6" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!P6),"",IF(ISERROR(ETPT_ATT_JUR!P6),"",IF(ETPT_ATT_JUR!P6=0,"",ETPT_ATT_JUR!P6)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!P6),"",IF(ISERROR(ETPT_ATTJ!P6),"",IF(ETPT_ATTJ!P6=0,"",ETPT_ATTJ!P6)))</f>
         <v/>
       </c>
       <c r="Q6" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!Q6),"",IF(ISERROR(ETPT_ATT_JUR!Q6),"",IF(ETPT_ATT_JUR!Q6=0,"",ETPT_ATT_JUR!Q6)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!Q6),"",IF(ISERROR(ETPT_ATTJ!Q6),"",IF(ETPT_ATTJ!Q6=0,"",ETPT_ATTJ!Q6)))</f>
         <v/>
       </c>
       <c r="R6" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!R6),"",IF(ISERROR(ETPT_ATT_JUR!R6),"",IF(ETPT_ATT_JUR!R6=0,"",ETPT_ATT_JUR!R6)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!R6),"",IF(ISERROR(ETPT_ATTJ!R6),"",IF(ETPT_ATTJ!R6=0,"",ETPT_ATTJ!R6)))</f>
         <v/>
       </c>
       <c r="S6" s="214">
-        <f>ETPT_ATT_JUR!S6</f>
+        <f>ETPT_ATTJ!S6</f>
         <v>0</v>
       </c>
     </row>
@@ -30722,43 +30722,43 @@
         <v>55</v>
       </c>
       <c r="G7" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!G7),"",IF(ISERROR(ETPT_ATT_JUR!G7),"",IF(ETPT_ATT_JUR!G7=0,"",ETPT_ATT_JUR!G7)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!G7),"",IF(ISERROR(ETPT_ATTJ!G7),"",IF(ETPT_ATTJ!G7=0,"",ETPT_ATTJ!G7)))</f>
         <v/>
       </c>
       <c r="H7" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!H7),"",IF(ISERROR(ETPT_ATT_JUR!H7),"",IF(ETPT_ATT_JUR!H7=0,"",ETPT_ATT_JUR!H7)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!H7),"",IF(ISERROR(ETPT_ATTJ!H7),"",IF(ETPT_ATTJ!H7=0,"",ETPT_ATTJ!H7)))</f>
         <v/>
       </c>
       <c r="I7" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!I7),"",IF(ISERROR(ETPT_ATT_JUR!I7),"",IF(ETPT_ATT_JUR!I7=0,"",ETPT_ATT_JUR!I7)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!I7),"",IF(ISERROR(ETPT_ATTJ!I7),"",IF(ETPT_ATTJ!I7=0,"",ETPT_ATTJ!I7)))</f>
         <v/>
       </c>
       <c r="J7" s="247"/>
       <c r="K7" s="247"/>
       <c r="L7" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!L7),"",IF(ISERROR(ETPT_ATT_JUR!L7),"",IF(ETPT_ATT_JUR!L7=0,"",ETPT_ATT_JUR!L7)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!L7),"",IF(ISERROR(ETPT_ATTJ!L7),"",IF(ETPT_ATTJ!L7=0,"",ETPT_ATTJ!L7)))</f>
         <v/>
       </c>
       <c r="M7" s="247"/>
       <c r="N7" s="247"/>
       <c r="O7" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!O7),"",IF(ISERROR(ETPT_ATT_JUR!O7),"",IF(ETPT_ATT_JUR!O7=0,"",ETPT_ATT_JUR!O7)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!O7),"",IF(ISERROR(ETPT_ATTJ!O7),"",IF(ETPT_ATTJ!O7=0,"",ETPT_ATTJ!O7)))</f>
         <v/>
       </c>
       <c r="P7" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!P7),"",IF(ISERROR(ETPT_ATT_JUR!P7),"",IF(ETPT_ATT_JUR!P7=0,"",ETPT_ATT_JUR!P7)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!P7),"",IF(ISERROR(ETPT_ATTJ!P7),"",IF(ETPT_ATTJ!P7=0,"",ETPT_ATTJ!P7)))</f>
         <v/>
       </c>
       <c r="Q7" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!Q7),"",IF(ISERROR(ETPT_ATT_JUR!Q7),"",IF(ETPT_ATT_JUR!Q7=0,"",ETPT_ATT_JUR!Q7)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!Q7),"",IF(ISERROR(ETPT_ATTJ!Q7),"",IF(ETPT_ATTJ!Q7=0,"",ETPT_ATTJ!Q7)))</f>
         <v/>
       </c>
       <c r="R7" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!R7),"",IF(ISERROR(ETPT_ATT_JUR!R7),"",IF(ETPT_ATT_JUR!R7=0,"",ETPT_ATT_JUR!R7)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!R7),"",IF(ISERROR(ETPT_ATTJ!R7),"",IF(ETPT_ATTJ!R7=0,"",ETPT_ATTJ!R7)))</f>
         <v/>
       </c>
       <c r="S7" s="214">
-        <f>ETPT_ATT_JUR!S7</f>
+        <f>ETPT_ATTJ!S7</f>
         <v>0</v>
       </c>
     </row>
@@ -30779,43 +30779,43 @@
         <v>53</v>
       </c>
       <c r="G8" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!G8),"",IF(ISERROR(ETPT_ATT_JUR!G8),"",IF(ETPT_ATT_JUR!G8=0,"",ETPT_ATT_JUR!G8)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!G8),"",IF(ISERROR(ETPT_ATTJ!G8),"",IF(ETPT_ATTJ!G8=0,"",ETPT_ATTJ!G8)))</f>
         <v/>
       </c>
       <c r="H8" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!H8),"",IF(ISERROR(ETPT_ATT_JUR!H8),"",IF(ETPT_ATT_JUR!H8=0,"",ETPT_ATT_JUR!H8)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!H8),"",IF(ISERROR(ETPT_ATTJ!H8),"",IF(ETPT_ATTJ!H8=0,"",ETPT_ATTJ!H8)))</f>
         <v/>
       </c>
       <c r="I8" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!I8),"",IF(ISERROR(ETPT_ATT_JUR!I8),"",IF(ETPT_ATT_JUR!I8=0,"",ETPT_ATT_JUR!I8)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!I8),"",IF(ISERROR(ETPT_ATTJ!I8),"",IF(ETPT_ATTJ!I8=0,"",ETPT_ATTJ!I8)))</f>
         <v/>
       </c>
       <c r="J8" s="247"/>
       <c r="K8" s="247"/>
       <c r="L8" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!L8),"",IF(ISERROR(ETPT_ATT_JUR!L8),"",IF(ETPT_ATT_JUR!L8=0,"",ETPT_ATT_JUR!L8)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!L8),"",IF(ISERROR(ETPT_ATTJ!L8),"",IF(ETPT_ATTJ!L8=0,"",ETPT_ATTJ!L8)))</f>
         <v/>
       </c>
       <c r="M8" s="247"/>
       <c r="N8" s="247"/>
       <c r="O8" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!O8),"",IF(ISERROR(ETPT_ATT_JUR!O8),"",IF(ETPT_ATT_JUR!O8=0,"",ETPT_ATT_JUR!O8)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!O8),"",IF(ISERROR(ETPT_ATTJ!O8),"",IF(ETPT_ATTJ!O8=0,"",ETPT_ATTJ!O8)))</f>
         <v/>
       </c>
       <c r="P8" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!P8),"",IF(ISERROR(ETPT_ATT_JUR!P8),"",IF(ETPT_ATT_JUR!P8=0,"",ETPT_ATT_JUR!P8)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!P8),"",IF(ISERROR(ETPT_ATTJ!P8),"",IF(ETPT_ATTJ!P8=0,"",ETPT_ATTJ!P8)))</f>
         <v/>
       </c>
       <c r="Q8" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!Q8),"",IF(ISERROR(ETPT_ATT_JUR!Q8),"",IF(ETPT_ATT_JUR!Q8=0,"",ETPT_ATT_JUR!Q8)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!Q8),"",IF(ISERROR(ETPT_ATTJ!Q8),"",IF(ETPT_ATTJ!Q8=0,"",ETPT_ATTJ!Q8)))</f>
         <v/>
       </c>
       <c r="R8" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!R8),"",IF(ISERROR(ETPT_ATT_JUR!R8),"",IF(ETPT_ATT_JUR!R8=0,"",ETPT_ATT_JUR!R8)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!R8),"",IF(ISERROR(ETPT_ATTJ!R8),"",IF(ETPT_ATTJ!R8=0,"",ETPT_ATTJ!R8)))</f>
         <v/>
       </c>
       <c r="S8" s="214">
-        <f>ETPT_ATT_JUR!S8</f>
+        <f>ETPT_ATTJ!S8</f>
         <v>0</v>
       </c>
     </row>
@@ -30836,43 +30836,43 @@
         <v>51</v>
       </c>
       <c r="G9" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!G9),"",IF(ISERROR(ETPT_ATT_JUR!G9),"",IF(ETPT_ATT_JUR!G9=0,"",ETPT_ATT_JUR!G9)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!G9),"",IF(ISERROR(ETPT_ATTJ!G9),"",IF(ETPT_ATTJ!G9=0,"",ETPT_ATTJ!G9)))</f>
         <v/>
       </c>
       <c r="H9" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!H9),"",IF(ISERROR(ETPT_ATT_JUR!H9),"",IF(ETPT_ATT_JUR!H9=0,"",ETPT_ATT_JUR!H9)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!H9),"",IF(ISERROR(ETPT_ATTJ!H9),"",IF(ETPT_ATTJ!H9=0,"",ETPT_ATTJ!H9)))</f>
         <v/>
       </c>
       <c r="I9" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!I9),"",IF(ISERROR(ETPT_ATT_JUR!I9),"",IF(ETPT_ATT_JUR!I9=0,"",ETPT_ATT_JUR!I9)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!I9),"",IF(ISERROR(ETPT_ATTJ!I9),"",IF(ETPT_ATTJ!I9=0,"",ETPT_ATTJ!I9)))</f>
         <v/>
       </c>
       <c r="J9" s="247"/>
       <c r="K9" s="247"/>
       <c r="L9" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!L9),"",IF(ISERROR(ETPT_ATT_JUR!L9),"",IF(ETPT_ATT_JUR!L9=0,"",ETPT_ATT_JUR!L9)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!L9),"",IF(ISERROR(ETPT_ATTJ!L9),"",IF(ETPT_ATTJ!L9=0,"",ETPT_ATTJ!L9)))</f>
         <v/>
       </c>
       <c r="M9" s="247"/>
       <c r="N9" s="247"/>
       <c r="O9" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!O9),"",IF(ISERROR(ETPT_ATT_JUR!O9),"",IF(ETPT_ATT_JUR!O9=0,"",ETPT_ATT_JUR!O9)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!O9),"",IF(ISERROR(ETPT_ATTJ!O9),"",IF(ETPT_ATTJ!O9=0,"",ETPT_ATTJ!O9)))</f>
         <v/>
       </c>
       <c r="P9" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!P9),"",IF(ISERROR(ETPT_ATT_JUR!P9),"",IF(ETPT_ATT_JUR!P9=0,"",ETPT_ATT_JUR!P9)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!P9),"",IF(ISERROR(ETPT_ATTJ!P9),"",IF(ETPT_ATTJ!P9=0,"",ETPT_ATTJ!P9)))</f>
         <v/>
       </c>
       <c r="Q9" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!Q9),"",IF(ISERROR(ETPT_ATT_JUR!Q9),"",IF(ETPT_ATT_JUR!Q9=0,"",ETPT_ATT_JUR!Q9)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!Q9),"",IF(ISERROR(ETPT_ATTJ!Q9),"",IF(ETPT_ATTJ!Q9=0,"",ETPT_ATTJ!Q9)))</f>
         <v/>
       </c>
       <c r="R9" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!R9),"",IF(ISERROR(ETPT_ATT_JUR!R9),"",IF(ETPT_ATT_JUR!R9=0,"",ETPT_ATT_JUR!R9)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!R9),"",IF(ISERROR(ETPT_ATTJ!R9),"",IF(ETPT_ATTJ!R9=0,"",ETPT_ATTJ!R9)))</f>
         <v/>
       </c>
       <c r="S9" s="214">
-        <f>ETPT_ATT_JUR!S9</f>
+        <f>ETPT_ATTJ!S9</f>
         <v>0</v>
       </c>
     </row>
@@ -30893,43 +30893,43 @@
         <v>49</v>
       </c>
       <c r="G10" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!G10),"",IF(ISERROR(ETPT_ATT_JUR!G10),"",IF(ETPT_ATT_JUR!G10=0,"",ETPT_ATT_JUR!G10)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!G10),"",IF(ISERROR(ETPT_ATTJ!G10),"",IF(ETPT_ATTJ!G10=0,"",ETPT_ATTJ!G10)))</f>
         <v/>
       </c>
       <c r="H10" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!H10),"",IF(ISERROR(ETPT_ATT_JUR!H10),"",IF(ETPT_ATT_JUR!H10=0,"",ETPT_ATT_JUR!H10)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!H10),"",IF(ISERROR(ETPT_ATTJ!H10),"",IF(ETPT_ATTJ!H10=0,"",ETPT_ATTJ!H10)))</f>
         <v/>
       </c>
       <c r="I10" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!I10),"",IF(ISERROR(ETPT_ATT_JUR!I10),"",IF(ETPT_ATT_JUR!I10=0,"",ETPT_ATT_JUR!I10)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!I10),"",IF(ISERROR(ETPT_ATTJ!I10),"",IF(ETPT_ATTJ!I10=0,"",ETPT_ATTJ!I10)))</f>
         <v/>
       </c>
       <c r="J10" s="247"/>
       <c r="K10" s="247"/>
       <c r="L10" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!L10),"",IF(ISERROR(ETPT_ATT_JUR!L10),"",IF(ETPT_ATT_JUR!L10=0,"",ETPT_ATT_JUR!L10)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!L10),"",IF(ISERROR(ETPT_ATTJ!L10),"",IF(ETPT_ATTJ!L10=0,"",ETPT_ATTJ!L10)))</f>
         <v/>
       </c>
       <c r="M10" s="247"/>
       <c r="N10" s="247"/>
       <c r="O10" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!O10),"",IF(ISERROR(ETPT_ATT_JUR!O10),"",IF(ETPT_ATT_JUR!O10=0,"",ETPT_ATT_JUR!O10)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!O10),"",IF(ISERROR(ETPT_ATTJ!O10),"",IF(ETPT_ATTJ!O10=0,"",ETPT_ATTJ!O10)))</f>
         <v/>
       </c>
       <c r="P10" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!P10),"",IF(ISERROR(ETPT_ATT_JUR!P10),"",IF(ETPT_ATT_JUR!P10=0,"",ETPT_ATT_JUR!P10)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!P10),"",IF(ISERROR(ETPT_ATTJ!P10),"",IF(ETPT_ATTJ!P10=0,"",ETPT_ATTJ!P10)))</f>
         <v/>
       </c>
       <c r="Q10" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!Q10),"",IF(ISERROR(ETPT_ATT_JUR!Q10),"",IF(ETPT_ATT_JUR!Q10=0,"",ETPT_ATT_JUR!Q10)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!Q10),"",IF(ISERROR(ETPT_ATTJ!Q10),"",IF(ETPT_ATTJ!Q10=0,"",ETPT_ATTJ!Q10)))</f>
         <v/>
       </c>
       <c r="R10" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!R10),"",IF(ISERROR(ETPT_ATT_JUR!R10),"",IF(ETPT_ATT_JUR!R10=0,"",ETPT_ATT_JUR!R10)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!R10),"",IF(ISERROR(ETPT_ATTJ!R10),"",IF(ETPT_ATTJ!R10=0,"",ETPT_ATTJ!R10)))</f>
         <v/>
       </c>
       <c r="S10" s="214">
-        <f>ETPT_ATT_JUR!S10</f>
+        <f>ETPT_ATTJ!S10</f>
         <v>0</v>
       </c>
     </row>
@@ -30950,43 +30950,43 @@
         <v>47</v>
       </c>
       <c r="G11" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!G11),"",IF(ISERROR(ETPT_ATT_JUR!G11),"",IF(ETPT_ATT_JUR!G11=0,"",ETPT_ATT_JUR!G11)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!G11),"",IF(ISERROR(ETPT_ATTJ!G11),"",IF(ETPT_ATTJ!G11=0,"",ETPT_ATTJ!G11)))</f>
         <v/>
       </c>
       <c r="H11" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!H11),"",IF(ISERROR(ETPT_ATT_JUR!H11),"",IF(ETPT_ATT_JUR!H11=0,"",ETPT_ATT_JUR!H11)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!H11),"",IF(ISERROR(ETPT_ATTJ!H11),"",IF(ETPT_ATTJ!H11=0,"",ETPT_ATTJ!H11)))</f>
         <v/>
       </c>
       <c r="I11" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!I11),"",IF(ISERROR(ETPT_ATT_JUR!I11),"",IF(ETPT_ATT_JUR!I11=0,"",ETPT_ATT_JUR!I11)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!I11),"",IF(ISERROR(ETPT_ATTJ!I11),"",IF(ETPT_ATTJ!I11=0,"",ETPT_ATTJ!I11)))</f>
         <v/>
       </c>
       <c r="J11" s="247"/>
       <c r="K11" s="247"/>
       <c r="L11" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!L11),"",IF(ISERROR(ETPT_ATT_JUR!L11),"",IF(ETPT_ATT_JUR!L11=0,"",ETPT_ATT_JUR!L11)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!L11),"",IF(ISERROR(ETPT_ATTJ!L11),"",IF(ETPT_ATTJ!L11=0,"",ETPT_ATTJ!L11)))</f>
         <v/>
       </c>
       <c r="M11" s="247"/>
       <c r="N11" s="247"/>
       <c r="O11" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!O11),"",IF(ISERROR(ETPT_ATT_JUR!O11),"",IF(ETPT_ATT_JUR!O11=0,"",ETPT_ATT_JUR!O11)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!O11),"",IF(ISERROR(ETPT_ATTJ!O11),"",IF(ETPT_ATTJ!O11=0,"",ETPT_ATTJ!O11)))</f>
         <v/>
       </c>
       <c r="P11" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!P11),"",IF(ISERROR(ETPT_ATT_JUR!P11),"",IF(ETPT_ATT_JUR!P11=0,"",ETPT_ATT_JUR!P11)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!P11),"",IF(ISERROR(ETPT_ATTJ!P11),"",IF(ETPT_ATTJ!P11=0,"",ETPT_ATTJ!P11)))</f>
         <v/>
       </c>
       <c r="Q11" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!Q11),"",IF(ISERROR(ETPT_ATT_JUR!Q11),"",IF(ETPT_ATT_JUR!Q11=0,"",ETPT_ATT_JUR!Q11)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!Q11),"",IF(ISERROR(ETPT_ATTJ!Q11),"",IF(ETPT_ATTJ!Q11=0,"",ETPT_ATTJ!Q11)))</f>
         <v/>
       </c>
       <c r="R11" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!R11),"",IF(ISERROR(ETPT_ATT_JUR!R11),"",IF(ETPT_ATT_JUR!R11=0,"",ETPT_ATT_JUR!R11)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!R11),"",IF(ISERROR(ETPT_ATTJ!R11),"",IF(ETPT_ATTJ!R11=0,"",ETPT_ATTJ!R11)))</f>
         <v/>
       </c>
       <c r="S11" s="214">
-        <f>ETPT_ATT_JUR!S11</f>
+        <f>ETPT_ATTJ!S11</f>
         <v>0</v>
       </c>
     </row>
@@ -31007,43 +31007,43 @@
         <v>45</v>
       </c>
       <c r="G12" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!G12),"",IF(ISERROR(ETPT_ATT_JUR!G12),"",IF(ETPT_ATT_JUR!G12=0,"",ETPT_ATT_JUR!G12)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!G12),"",IF(ISERROR(ETPT_ATTJ!G12),"",IF(ETPT_ATTJ!G12=0,"",ETPT_ATTJ!G12)))</f>
         <v/>
       </c>
       <c r="H12" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!H12),"",IF(ISERROR(ETPT_ATT_JUR!H12),"",IF(ETPT_ATT_JUR!H12=0,"",ETPT_ATT_JUR!H12)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!H12),"",IF(ISERROR(ETPT_ATTJ!H12),"",IF(ETPT_ATTJ!H12=0,"",ETPT_ATTJ!H12)))</f>
         <v/>
       </c>
       <c r="I12" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!I12),"",IF(ISERROR(ETPT_ATT_JUR!I12),"",IF(ETPT_ATT_JUR!I12=0,"",ETPT_ATT_JUR!I12)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!I12),"",IF(ISERROR(ETPT_ATTJ!I12),"",IF(ETPT_ATTJ!I12=0,"",ETPT_ATTJ!I12)))</f>
         <v/>
       </c>
       <c r="J12" s="247"/>
       <c r="K12" s="247"/>
       <c r="L12" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!L12),"",IF(ISERROR(ETPT_ATT_JUR!L12),"",IF(ETPT_ATT_JUR!L12=0,"",ETPT_ATT_JUR!L12)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!L12),"",IF(ISERROR(ETPT_ATTJ!L12),"",IF(ETPT_ATTJ!L12=0,"",ETPT_ATTJ!L12)))</f>
         <v/>
       </c>
       <c r="M12" s="247"/>
       <c r="N12" s="247"/>
       <c r="O12" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!O12),"",IF(ISERROR(ETPT_ATT_JUR!O12),"",IF(ETPT_ATT_JUR!O12=0,"",ETPT_ATT_JUR!O12)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!O12),"",IF(ISERROR(ETPT_ATTJ!O12),"",IF(ETPT_ATTJ!O12=0,"",ETPT_ATTJ!O12)))</f>
         <v/>
       </c>
       <c r="P12" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!P12),"",IF(ISERROR(ETPT_ATT_JUR!P12),"",IF(ETPT_ATT_JUR!P12=0,"",ETPT_ATT_JUR!P12)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!P12),"",IF(ISERROR(ETPT_ATTJ!P12),"",IF(ETPT_ATTJ!P12=0,"",ETPT_ATTJ!P12)))</f>
         <v/>
       </c>
       <c r="Q12" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!Q12),"",IF(ISERROR(ETPT_ATT_JUR!Q12),"",IF(ETPT_ATT_JUR!Q12=0,"",ETPT_ATT_JUR!Q12)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!Q12),"",IF(ISERROR(ETPT_ATTJ!Q12),"",IF(ETPT_ATTJ!Q12=0,"",ETPT_ATTJ!Q12)))</f>
         <v/>
       </c>
       <c r="R12" s="247" t="str">
-        <f>IF(ISBLANK(ETPT_ATT_JUR!R12),"",IF(ISERROR(ETPT_ATT_JUR!R12),"",IF(ETPT_ATT_JUR!R12=0,"",ETPT_ATT_JUR!R12)))</f>
+        <f>IF(ISBLANK(ETPT_ATTJ!R12),"",IF(ISERROR(ETPT_ATTJ!R12),"",IF(ETPT_ATTJ!R12=0,"",ETPT_ATTJ!R12)))</f>
         <v/>
       </c>
       <c r="S12" s="214">
-        <f>ETPT_ATT_JUR!S12</f>
+        <f>ETPT_ATTJ!S12</f>
         <v>0</v>
       </c>
     </row>
@@ -31057,55 +31057,55 @@
         <v>39</v>
       </c>
       <c r="G13" s="214">
-        <f>ETPT_ATT_JUR!G13</f>
+        <f>ETPT_ATTJ!G13</f>
         <v>0</v>
       </c>
       <c r="H13" s="214">
-        <f>ETPT_ATT_JUR!H13</f>
+        <f>ETPT_ATTJ!H13</f>
         <v>0</v>
       </c>
       <c r="I13" s="214">
-        <f>ETPT_ATT_JUR!I13</f>
+        <f>ETPT_ATTJ!I13</f>
         <v>0</v>
       </c>
       <c r="J13" s="214">
-        <f>ETPT_ATT_JUR!J13</f>
+        <f>ETPT_ATTJ!J13</f>
         <v>0</v>
       </c>
       <c r="K13" s="214">
-        <f>ETPT_ATT_JUR!K13</f>
+        <f>ETPT_ATTJ!K13</f>
         <v>0</v>
       </c>
       <c r="L13" s="214">
-        <f>ETPT_ATT_JUR!L13</f>
+        <f>ETPT_ATTJ!L13</f>
         <v>0</v>
       </c>
       <c r="M13" s="214">
-        <f>ETPT_ATT_JUR!M13</f>
+        <f>ETPT_ATTJ!M13</f>
         <v>0</v>
       </c>
       <c r="N13" s="214">
-        <f>ETPT_ATT_JUR!N13</f>
+        <f>ETPT_ATTJ!N13</f>
         <v>0</v>
       </c>
       <c r="O13" s="214">
-        <f>ETPT_ATT_JUR!O13</f>
+        <f>ETPT_ATTJ!O13</f>
         <v>0</v>
       </c>
       <c r="P13" s="214">
-        <f>ETPT_ATT_JUR!P13</f>
+        <f>ETPT_ATTJ!P13</f>
         <v>0</v>
       </c>
       <c r="Q13" s="214">
-        <f>ETPT_ATT_JUR!Q13</f>
+        <f>ETPT_ATTJ!Q13</f>
         <v>0</v>
       </c>
       <c r="R13" s="214">
-        <f>ETPT_ATT_JUR!R13</f>
+        <f>ETPT_ATTJ!R13</f>
         <v>0</v>
       </c>
       <c r="S13" s="214">
-        <f>ETPT_ATT_JUR!S13</f>
+        <f>ETPT_ATTJ!S13</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix recodedFunction values for Att. J Siege Assises and CCD to match Excel formulas
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67451E94-B29C-274D-8918-FE32A7FB46CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8633B384-6001-964A-B82D-5903BEEB9204}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="9" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -20929,27 +20929,27 @@
       <c r="I5" s="280" t="e" cm="1">
         <f t="array" ref="I5">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("2. TOTAL CONTENTIEUX JAF",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("3. TOTAL CONTENTIEUX DE LA PROTECTION",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4. TOTAL CIVIL NON SPÉCIALISÉ",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))+
 SUM(SUMIFS(
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("5. TOTAL JLD CIVIL",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4. TOTAL CIVIL NON SPÉCIALISÉ",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.7. FONCTIONNAIRES AFFECTÉS AU CPH",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
@@ -20958,7 +20958,7 @@
       <c r="L5" s="280" t="e" cm="1">
         <f t="array" ref="L5">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.8. FONCTIONNAIRES AFFECTÉS AUX ACTIVITÉS CIVILES ET COMMERCIALES DU PARQUET",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
@@ -20968,7 +20968,7 @@
       <c r="P5" s="280" t="e" cm="1">
         <f t="array" ref="P5">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("6.1. ACTIVITÉ CIVILE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
@@ -21032,48 +21032,48 @@
       <c r="I6" s="280" t="e" cm="1">
         <f t="array" ref="I6">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7. TOTAL SIÈGE PÉNAL",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)) -
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.51. COUR D'ASSISES JIRS",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)) -
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.52. COUR CRIMINELLE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.5. COUR D'ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
       <c r="J6" s="280" t="e" cm="1">
         <f t="array" ref="J6">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.5. COUR D'ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.51. COUR D'ASSISES JIRS",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
       <c r="K6" s="280" t="e" cm="1">
         <f t="array" ref="K6">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.52. COUR CRIMINELLE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
       <c r="L6" s="280" t="e" cm="1">
         <f t="array" ref="L6">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.9. FONCTIONNAIRES AFFECTÉS À L'EXÉCUTION DES PEINES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))+
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.10. AUTRES FONCTIONNAIRES AFFECTÉS AU PARQUET",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
@@ -21082,28 +21082,28 @@
       <c r="O6" s="280" t="e" cm="1">
         <f t="array" ref="O6">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("9. TOTAL JAP",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
       <c r="P6" s="280" t="e" cm="1">
         <f t="array" ref="P6">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("6.2. ACTIVITÉ PÉNALE",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
       <c r="Q6" s="280" t="e" cm="1">
         <f t="array" ref="Q6">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("8. TOTAL JUGES D'INSTRUCTION",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>
       <c r="R6" s="280" t="e" cm="1">
         <f t="array" ref="R6">SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("10. TOTAL JLD PÉNAL",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
         <v>#N/A</v>
       </c>

</xml_diff>

<commit_message>
Add conditional formatting rule to highlight rows where function code starts with 'JA'
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{519EB016-6E2B-BF45-B5E5-B4BC372EEBC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D9017EF-062B-544A-8703-0F0C6A643CA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="9" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="2" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -22,7 +22,7 @@
     <sheet name="ETPT_TJ" sheetId="25" state="hidden" r:id="rId7"/>
     <sheet name="ETPT_TPRX" sheetId="26" state="hidden" r:id="rId8"/>
     <sheet name="ETPT_CPH" sheetId="27" state="hidden" r:id="rId9"/>
-    <sheet name="ETPT_ATTJ" sheetId="38" r:id="rId10"/>
+    <sheet name="ETPT_ATTJ" sheetId="38" state="hidden" r:id="rId10"/>
     <sheet name="ETPT_TJ_DDG" sheetId="28" r:id="rId11"/>
     <sheet name="ETPT_TPRX_DDG" sheetId="29" r:id="rId12"/>
     <sheet name="ETPT_CPH_DDG" sheetId="30" r:id="rId13"/>
@@ -19281,6 +19281,16 @@
   </cellStyles>
   <dxfs count="28">
     <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill>
           <bgColor theme="9" tint="0.79998168889431442"/>
@@ -19519,16 +19529,6 @@
       <font>
         <color theme="0"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -20944,6 +20944,10 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))+
 SUM(SUMIFS(
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("5. TOTAL JLD CIVIL",'ETPT Format DDG'!2:2,0)),
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))+
+SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("11.7. FONCTIONNAIRES AFFECTÉS AU CPH",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
@@ -37421,8 +37425,8 @@
     <mergeCell ref="D1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2:EZ2 A3:FB1048576">
-    <cfRule type="expression" dxfId="27" priority="1" stopIfTrue="1">
-      <formula>AND(OR($R1&lt;&gt;0,$S1&lt;&gt;0,$T1&lt;&gt;0,ISBLANK($P1)),ROW()&gt;2,$A1&lt;&gt;"")</formula>
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>OR(AND(OR($R1&lt;&gt;0,$S1&lt;&gt;0,$T1&lt;&gt;0,ISBLANK($P1)),ROW()&gt;2,$A1&lt;&gt;""),LEFT($F2,2)="JA")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -37747,70 +37751,70 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="26" priority="16">
+    <cfRule type="expression" dxfId="27" priority="16">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="25" priority="18" stopIfTrue="1">
+    <cfRule type="expression" dxfId="26" priority="18" stopIfTrue="1">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="24" priority="1">
+    <cfRule type="expression" dxfId="25" priority="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)-_xlfn.NUMBERVALUE($U6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="23" priority="2">
+    <cfRule type="expression" dxfId="24" priority="2">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)-_xlfn.NUMBERVALUE($S6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="23" priority="7" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3)-_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)-_xlfn.NUMBERVALUE($L6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="12">
+    <cfRule type="expression" dxfId="22" priority="12">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",OR(ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="20" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="21" priority="6" stopIfTrue="1">
       <formula>OR(ROUND(_xlfn.NUMBERVALUE($L7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($L6),3),ROUND(_xlfn.NUMBERVALUE($S7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($S6),3),ROUND(_xlfn.NUMBERVALUE($U7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($U6),3))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="19" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="20" priority="11" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)+_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6)),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="15">
+    <cfRule type="expression" dxfId="19" priority="15">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="17" priority="5">
+    <cfRule type="expression" dxfId="18" priority="5">
       <formula>ROUND(_xlfn.NUMBERVALUE($L7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($L6),3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="16" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="17" priority="10" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)-_xlfn.NUMBERVALUE($S6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="14">
+    <cfRule type="expression" dxfId="16" priority="14">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="14" priority="4">
+    <cfRule type="expression" dxfId="15" priority="4">
       <formula>ROUND(_xlfn.NUMBERVALUE($S7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($S6),3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="13" priority="9">
+    <cfRule type="expression" dxfId="14" priority="9">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)-_xlfn.NUMBERVALUE($U6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="13">
+    <cfRule type="expression" dxfId="13" priority="13">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="11" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="3" stopIfTrue="1">
       <formula>ROUND(_xlfn.NUMBERVALUE($U7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($U6),3)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -38102,57 +38106,57 @@
   </sheetData>
   <autoFilter ref="A1:V1" xr:uid="{02AF4949-5E39-2D4C-AD07-A4D8FB117F56}"/>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="10" priority="30">
+    <cfRule type="expression" dxfId="11" priority="30">
       <formula>AND(OR($I1&lt;&gt;"-",#REF!&lt;&gt;0,#REF!&lt;&gt;0,ISBLANK($M1)),ROW()&gt;2,$A1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:F2">
-    <cfRule type="expression" dxfId="9" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="11" stopIfTrue="1">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:N2">
-    <cfRule type="expression" dxfId="8" priority="5">
+    <cfRule type="expression" dxfId="9" priority="5">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:K2">
-    <cfRule type="expression" dxfId="7" priority="6">
+    <cfRule type="expression" dxfId="8" priority="6">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2">
-    <cfRule type="expression" dxfId="6" priority="8">
+    <cfRule type="expression" dxfId="7" priority="8">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2">
-    <cfRule type="expression" dxfId="5" priority="7">
+    <cfRule type="expression" dxfId="6" priority="7">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2">
-    <cfRule type="expression" dxfId="4" priority="9">
+    <cfRule type="expression" dxfId="5" priority="9">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:V2">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q2:R2">
-    <cfRule type="expression" dxfId="2" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S2:T2">
-    <cfRule type="expression" dxfId="1" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V2">
-    <cfRule type="expression" dxfId="0" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Fix conditional formatting column reference for function code check
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D9017EF-062B-544A-8703-0F0C6A643CA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D3A3F79-72D7-E047-84AC-5E68FF6DA48A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="2" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -19279,7 +19279,17 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
     <cellStyle name="Normal 3" xfId="4" xr:uid="{6BD57324-3FD5-D341-A299-730D14794802}"/>
   </cellStyles>
-  <dxfs count="28">
+  <dxfs count="29">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -37419,14 +37429,14 @@
       <c r="FA4" s="21"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" autoFilter="0"/>
+  <sheetProtection autoFilter="0"/>
   <autoFilter ref="A2:DT2" xr:uid="{3B89445B-6ECC-4440-B85C-E593AE209933}"/>
   <mergeCells count="1">
     <mergeCell ref="D1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2:EZ2 A3:FB1048576">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>OR(AND(OR($R1&lt;&gt;0,$S1&lt;&gt;0,$T1&lt;&gt;0,ISBLANK($P1)),ROW()&gt;2,$A1&lt;&gt;""),LEFT($F2,2)="JA")</formula>
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>OR(AND(OR($R1&lt;&gt;0,$S1&lt;&gt;0,$T1&lt;&gt;0,ISBLANK($P1)),ROW()&gt;2,$A1&lt;&gt;""),LEFT($I2,2)="JA")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -37751,70 +37761,70 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="27" priority="16">
+    <cfRule type="expression" dxfId="28" priority="16">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="26" priority="18" stopIfTrue="1">
+    <cfRule type="expression" dxfId="27" priority="18" stopIfTrue="1">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="25" priority="1">
+    <cfRule type="expression" dxfId="26" priority="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)-_xlfn.NUMBERVALUE($U6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="2">
+    <cfRule type="expression" dxfId="25" priority="2">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)-_xlfn.NUMBERVALUE($S6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="23" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="24" priority="7" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3)-_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)-_xlfn.NUMBERVALUE($L6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="12">
+    <cfRule type="expression" dxfId="23" priority="12">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",OR(ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="21" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="22" priority="6" stopIfTrue="1">
       <formula>OR(ROUND(_xlfn.NUMBERVALUE($L7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($L6),3),ROUND(_xlfn.NUMBERVALUE($S7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($S6),3),ROUND(_xlfn.NUMBERVALUE($U7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($U6),3))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="20" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="21" priority="11" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)+_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6)),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="15">
+    <cfRule type="expression" dxfId="20" priority="15">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="18" priority="5">
+    <cfRule type="expression" dxfId="19" priority="5">
       <formula>ROUND(_xlfn.NUMBERVALUE($L7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($L6),3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="17" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="18" priority="10" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)-_xlfn.NUMBERVALUE($S6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="14">
+    <cfRule type="expression" dxfId="17" priority="14">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="15" priority="4">
+    <cfRule type="expression" dxfId="16" priority="4">
       <formula>ROUND(_xlfn.NUMBERVALUE($S7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($S6),3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="14" priority="9">
+    <cfRule type="expression" dxfId="15" priority="9">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)-_xlfn.NUMBERVALUE($U6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="13">
+    <cfRule type="expression" dxfId="14" priority="13">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="12" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="3" stopIfTrue="1">
       <formula>ROUND(_xlfn.NUMBERVALUE($U7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($U6),3)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -38106,57 +38116,57 @@
   </sheetData>
   <autoFilter ref="A1:V1" xr:uid="{02AF4949-5E39-2D4C-AD07-A4D8FB117F56}"/>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="11" priority="30">
+    <cfRule type="expression" dxfId="12" priority="30">
       <formula>AND(OR($I1&lt;&gt;"-",#REF!&lt;&gt;0,#REF!&lt;&gt;0,ISBLANK($M1)),ROW()&gt;2,$A1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:F2">
-    <cfRule type="expression" dxfId="10" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="11" stopIfTrue="1">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:N2">
-    <cfRule type="expression" dxfId="9" priority="5">
+    <cfRule type="expression" dxfId="10" priority="5">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:K2">
-    <cfRule type="expression" dxfId="8" priority="6">
+    <cfRule type="expression" dxfId="9" priority="6">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2">
-    <cfRule type="expression" dxfId="7" priority="8">
+    <cfRule type="expression" dxfId="8" priority="8">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2">
-    <cfRule type="expression" dxfId="6" priority="7">
+    <cfRule type="expression" dxfId="7" priority="7">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2">
-    <cfRule type="expression" dxfId="5" priority="9">
+    <cfRule type="expression" dxfId="6" priority="9">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:V2">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="5" priority="1">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q2:R2">
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="4" priority="4">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S2:T2">
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V2">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Fix conditional formatting row offset - check current row instead of row below for JA function code
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D3A3F79-72D7-E047-84AC-5E68FF6DA48A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EFF9B49-A96E-E448-8B02-56262FDE8ECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="2" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -19279,17 +19279,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
     <cellStyle name="Normal 3" xfId="4" xr:uid="{6BD57324-3FD5-D341-A299-730D14794802}"/>
   </cellStyles>
-  <dxfs count="29">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="28">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -37429,14 +37419,14 @@
       <c r="FA4" s="21"/>
     </row>
   </sheetData>
-  <sheetProtection autoFilter="0"/>
+  <sheetProtection sheet="1" autoFilter="0"/>
   <autoFilter ref="A2:DT2" xr:uid="{3B89445B-6ECC-4440-B85C-E593AE209933}"/>
   <mergeCells count="1">
     <mergeCell ref="D1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2:EZ2 A3:FB1048576">
-    <cfRule type="expression" dxfId="1" priority="1">
-      <formula>OR(AND(OR($R1&lt;&gt;0,$S1&lt;&gt;0,$T1&lt;&gt;0,ISBLANK($P1)),ROW()&gt;2,$A1&lt;&gt;""),LEFT($I2,2)="JA")</formula>
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>OR(AND(OR($R1&lt;&gt;0,$S1&lt;&gt;0,$T1&lt;&gt;0,ISBLANK($P1)),ROW()&gt;2,$A1&lt;&gt;""),LEFT($I1,2)="JA")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -37761,70 +37751,70 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="28" priority="16">
+    <cfRule type="expression" dxfId="27" priority="16">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="27" priority="18" stopIfTrue="1">
+    <cfRule type="expression" dxfId="26" priority="18" stopIfTrue="1">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="26" priority="1">
+    <cfRule type="expression" dxfId="25" priority="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)-_xlfn.NUMBERVALUE($U6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="25" priority="2">
+    <cfRule type="expression" dxfId="24" priority="2">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)-_xlfn.NUMBERVALUE($S6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="23" priority="7" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3)-_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)-_xlfn.NUMBERVALUE($L6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="23" priority="12">
+    <cfRule type="expression" dxfId="22" priority="12">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",OR(ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="22" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="21" priority="6" stopIfTrue="1">
       <formula>OR(ROUND(_xlfn.NUMBERVALUE($L7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($L6),3),ROUND(_xlfn.NUMBERVALUE($S7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($S6),3),ROUND(_xlfn.NUMBERVALUE($U7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($U6),3))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="21" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="20" priority="11" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)+_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6)),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="15">
+    <cfRule type="expression" dxfId="19" priority="15">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="19" priority="5">
+    <cfRule type="expression" dxfId="18" priority="5">
       <formula>ROUND(_xlfn.NUMBERVALUE($L7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($L6),3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="18" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="17" priority="10" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)-_xlfn.NUMBERVALUE($S6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="14">
+    <cfRule type="expression" dxfId="16" priority="14">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="16" priority="4">
+    <cfRule type="expression" dxfId="15" priority="4">
       <formula>ROUND(_xlfn.NUMBERVALUE($S7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($S6),3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="15" priority="9">
+    <cfRule type="expression" dxfId="14" priority="9">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)-_xlfn.NUMBERVALUE($U6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="13">
+    <cfRule type="expression" dxfId="13" priority="13">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="13" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="3" stopIfTrue="1">
       <formula>ROUND(_xlfn.NUMBERVALUE($U7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($U6),3)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -38116,57 +38106,57 @@
   </sheetData>
   <autoFilter ref="A1:V1" xr:uid="{02AF4949-5E39-2D4C-AD07-A4D8FB117F56}"/>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="12" priority="30">
+    <cfRule type="expression" dxfId="11" priority="30">
       <formula>AND(OR($I1&lt;&gt;"-",#REF!&lt;&gt;0,#REF!&lt;&gt;0,ISBLANK($M1)),ROW()&gt;2,$A1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:F2">
-    <cfRule type="expression" dxfId="11" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="11" stopIfTrue="1">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:N2">
-    <cfRule type="expression" dxfId="10" priority="5">
+    <cfRule type="expression" dxfId="9" priority="5">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:K2">
-    <cfRule type="expression" dxfId="9" priority="6">
+    <cfRule type="expression" dxfId="8" priority="6">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2">
-    <cfRule type="expression" dxfId="8" priority="8">
+    <cfRule type="expression" dxfId="7" priority="8">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2">
-    <cfRule type="expression" dxfId="7" priority="7">
+    <cfRule type="expression" dxfId="6" priority="7">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2">
-    <cfRule type="expression" dxfId="6" priority="9">
+    <cfRule type="expression" dxfId="5" priority="9">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:V2">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q2:R2">
-    <cfRule type="expression" dxfId="4" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S2:T2">
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V2">
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Refine conditional formatting to match 'JA ' (with space) to exclude JAP function
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EFF9B49-A96E-E448-8B02-56262FDE8ECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81FCE37C-F06D-D34D-9018-EB66181FA98A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="2" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -19279,7 +19279,27 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
     <cellStyle name="Normal 3" xfId="4" xr:uid="{6BD57324-3FD5-D341-A299-730D14794802}"/>
   </cellStyles>
-  <dxfs count="28">
+  <dxfs count="30">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -37419,14 +37439,14 @@
       <c r="FA4" s="21"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" autoFilter="0"/>
+  <sheetProtection autoFilter="0"/>
   <autoFilter ref="A2:DT2" xr:uid="{3B89445B-6ECC-4440-B85C-E593AE209933}"/>
   <mergeCells count="1">
     <mergeCell ref="D1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2:EZ2 A3:FB1048576">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>OR(AND(OR($R1&lt;&gt;0,$S1&lt;&gt;0,$T1&lt;&gt;0,ISBLANK($P1)),ROW()&gt;2,$A1&lt;&gt;""),LEFT($I1,2)="JA")</formula>
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>OR(AND(OR($R1&lt;&gt;0,$S1&lt;&gt;0,$T1&lt;&gt;0,ISBLANK($P1)),ROW()&gt;2,$A1&lt;&gt;""),LEFT($I1,2)="JA ")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -37751,70 +37771,70 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="27" priority="16">
+    <cfRule type="expression" dxfId="29" priority="16">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="26" priority="18" stopIfTrue="1">
+    <cfRule type="expression" dxfId="28" priority="18" stopIfTrue="1">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="25" priority="1">
+    <cfRule type="expression" dxfId="27" priority="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)-_xlfn.NUMBERVALUE($U6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="2">
+    <cfRule type="expression" dxfId="26" priority="2">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)-_xlfn.NUMBERVALUE($S6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="23" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="25" priority="7" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3)-_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)-_xlfn.NUMBERVALUE($L6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="12">
+    <cfRule type="expression" dxfId="24" priority="12">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",OR(ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="21" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="23" priority="6" stopIfTrue="1">
       <formula>OR(ROUND(_xlfn.NUMBERVALUE($L7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($L6),3),ROUND(_xlfn.NUMBERVALUE($S7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($S6),3),ROUND(_xlfn.NUMBERVALUE($U7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($U6),3))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="20" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="22" priority="11" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)+_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6)),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="15">
+    <cfRule type="expression" dxfId="21" priority="15">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="18" priority="5">
+    <cfRule type="expression" dxfId="20" priority="5">
       <formula>ROUND(_xlfn.NUMBERVALUE($L7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($L6),3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="17" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="19" priority="10" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)-_xlfn.NUMBERVALUE($S6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="14">
+    <cfRule type="expression" dxfId="18" priority="14">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="15" priority="4">
+    <cfRule type="expression" dxfId="17" priority="4">
       <formula>ROUND(_xlfn.NUMBERVALUE($S7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($S6),3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="14" priority="9">
+    <cfRule type="expression" dxfId="16" priority="9">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)-_xlfn.NUMBERVALUE($U6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="13">
+    <cfRule type="expression" dxfId="15" priority="13">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="12" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="3" stopIfTrue="1">
       <formula>ROUND(_xlfn.NUMBERVALUE($U7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($U6),3)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -38106,57 +38126,57 @@
   </sheetData>
   <autoFilter ref="A1:V1" xr:uid="{02AF4949-5E39-2D4C-AD07-A4D8FB117F56}"/>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="11" priority="30">
+    <cfRule type="expression" dxfId="13" priority="30">
       <formula>AND(OR($I1&lt;&gt;"-",#REF!&lt;&gt;0,#REF!&lt;&gt;0,ISBLANK($M1)),ROW()&gt;2,$A1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:F2">
-    <cfRule type="expression" dxfId="10" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="11" stopIfTrue="1">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:N2">
-    <cfRule type="expression" dxfId="9" priority="5">
+    <cfRule type="expression" dxfId="11" priority="5">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:K2">
-    <cfRule type="expression" dxfId="8" priority="6">
+    <cfRule type="expression" dxfId="10" priority="6">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2">
-    <cfRule type="expression" dxfId="7" priority="8">
+    <cfRule type="expression" dxfId="9" priority="8">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2">
-    <cfRule type="expression" dxfId="6" priority="7">
+    <cfRule type="expression" dxfId="8" priority="7">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2">
-    <cfRule type="expression" dxfId="5" priority="9">
+    <cfRule type="expression" dxfId="7" priority="9">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:V2">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="6" priority="1">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q2:R2">
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="5" priority="4">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S2:T2">
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="4" priority="3">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V2">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Fix GAUCHE to extract 3 characters for JA space check in conditional formatting
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81FCE37C-F06D-D34D-9018-EB66181FA98A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E1CB723-D4D5-6E4C-980E-5BC547F985EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="2" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
@@ -19279,7 +19279,27 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6FC886D6-2077-B34D-B1DF-739B068A66D1}"/>
     <cellStyle name="Normal 3" xfId="4" xr:uid="{6BD57324-3FD5-D341-A299-730D14794802}"/>
   </cellStyles>
-  <dxfs count="30">
+  <dxfs count="32">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -37446,7 +37466,7 @@
   </mergeCells>
   <conditionalFormatting sqref="A2:EZ2 A3:FB1048576">
     <cfRule type="expression" dxfId="1" priority="1">
-      <formula>OR(AND(OR($R1&lt;&gt;0,$S1&lt;&gt;0,$T1&lt;&gt;0,ISBLANK($P1)),ROW()&gt;2,$A1&lt;&gt;""),LEFT($I1,2)="JA ")</formula>
+      <formula>OR(AND(OR($R1&lt;&gt;0,$S1&lt;&gt;0,$T1&lt;&gt;0,ISBLANK($P1)),ROW()&gt;2,$A1&lt;&gt;""),LEFT($I1,3)="JA ")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -37771,70 +37791,70 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="29" priority="16">
+    <cfRule type="expression" dxfId="31" priority="16">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="28" priority="18" stopIfTrue="1">
+    <cfRule type="expression" dxfId="30" priority="18" stopIfTrue="1">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="27" priority="1">
+    <cfRule type="expression" dxfId="29" priority="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)-_xlfn.NUMBERVALUE($U6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="2">
+    <cfRule type="expression" dxfId="28" priority="2">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)-_xlfn.NUMBERVALUE($S6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="25" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="27" priority="7" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3)-_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)-_xlfn.NUMBERVALUE($L6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="12">
+    <cfRule type="expression" dxfId="26" priority="12">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",OR(ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="23" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="25" priority="6" stopIfTrue="1">
       <formula>OR(ROUND(_xlfn.NUMBERVALUE($L7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($L6),3),ROUND(_xlfn.NUMBERVALUE($S7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($S6),3),ROUND(_xlfn.NUMBERVALUE($U7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($U6),3))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="22" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="24" priority="11" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)+_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6)),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="15">
+    <cfRule type="expression" dxfId="23" priority="15">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="20" priority="5">
+    <cfRule type="expression" dxfId="22" priority="5">
       <formula>ROUND(_xlfn.NUMBERVALUE($L7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($L6),3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="19" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="21" priority="10" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)-_xlfn.NUMBERVALUE($S6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="14">
+    <cfRule type="expression" dxfId="20" priority="14">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="17" priority="4">
+    <cfRule type="expression" dxfId="19" priority="4">
       <formula>ROUND(_xlfn.NUMBERVALUE($S7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($S6),3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="16" priority="9">
+    <cfRule type="expression" dxfId="18" priority="9">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)-_xlfn.NUMBERVALUE($U6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="13">
+    <cfRule type="expression" dxfId="17" priority="13">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="14" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="16" priority="3" stopIfTrue="1">
       <formula>ROUND(_xlfn.NUMBERVALUE($U7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($U6),3)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -38126,57 +38146,57 @@
   </sheetData>
   <autoFilter ref="A1:V1" xr:uid="{02AF4949-5E39-2D4C-AD07-A4D8FB117F56}"/>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="13" priority="30">
+    <cfRule type="expression" dxfId="15" priority="30">
       <formula>AND(OR($I1&lt;&gt;"-",#REF!&lt;&gt;0,#REF!&lt;&gt;0,ISBLANK($M1)),ROW()&gt;2,$A1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:F2">
-    <cfRule type="expression" dxfId="12" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="11" stopIfTrue="1">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:N2">
-    <cfRule type="expression" dxfId="11" priority="5">
+    <cfRule type="expression" dxfId="13" priority="5">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:K2">
-    <cfRule type="expression" dxfId="10" priority="6">
+    <cfRule type="expression" dxfId="12" priority="6">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2">
-    <cfRule type="expression" dxfId="9" priority="8">
+    <cfRule type="expression" dxfId="11" priority="8">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2">
-    <cfRule type="expression" dxfId="8" priority="7">
+    <cfRule type="expression" dxfId="10" priority="7">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2">
-    <cfRule type="expression" dxfId="7" priority="9">
+    <cfRule type="expression" dxfId="9" priority="9">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:V2">
-    <cfRule type="expression" dxfId="6" priority="1">
+    <cfRule type="expression" dxfId="8" priority="1">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q2:R2">
-    <cfRule type="expression" dxfId="5" priority="4">
+    <cfRule type="expression" dxfId="7" priority="4">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S2:T2">
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="6" priority="3">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V2">
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="5" priority="2">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Add additional MAX(0; flooring to more formulas in template4
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E1CB723-D4D5-6E4C-980E-5BC547F985EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A63A948-13E0-4949-B8D2-2BA472C0F735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="2" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="9" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -19,10 +19,10 @@
     <sheet name="Synthèse ETPT" sheetId="10" r:id="rId4"/>
     <sheet name="Table_Fonctions" sheetId="19" state="hidden" r:id="rId5"/>
     <sheet name="ETPT Format DDG DETAIL" sheetId="41" state="hidden" r:id="rId6"/>
-    <sheet name="ETPT_TJ" sheetId="25" state="hidden" r:id="rId7"/>
+    <sheet name="ETPT_TJ" sheetId="25" r:id="rId7"/>
     <sheet name="ETPT_TPRX" sheetId="26" state="hidden" r:id="rId8"/>
     <sheet name="ETPT_CPH" sheetId="27" state="hidden" r:id="rId9"/>
-    <sheet name="ETPT_ATTJ" sheetId="38" state="hidden" r:id="rId10"/>
+    <sheet name="ETPT_ATTJ" sheetId="38" r:id="rId10"/>
     <sheet name="ETPT_TJ_DDG" sheetId="28" r:id="rId11"/>
     <sheet name="ETPT_TPRX_DDG" sheetId="29" r:id="rId12"/>
     <sheet name="ETPT_CPH_DDG" sheetId="30" r:id="rId13"/>
@@ -21070,7 +21070,7 @@
         <v>#N/A</v>
       </c>
       <c r="I6" s="280" t="e" cm="1">
-        <f t="array" ref="I6">SUM(SUMIFS(
+        <f t="array" ref="I6">MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7. TOTAL SIÈGE PÉNAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)) -
@@ -21085,7 +21085,7 @@
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.5. COUR D'ASSISES HORS JIRS",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"JA/AttJ JAP";"JA/AttJ JE";"JA/AttJ JI";"JA/AttJ JLD PÉNAL";"JA/AttJ Parquet";"JA/AttJ Siège autres";"JA/AttJ Siege Assises";"JA/AttJ Siege CCD"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)))</f>
         <v>#N/A</v>
       </c>
       <c r="J6" s="280" t="e" cm="1">
@@ -21621,115 +21621,115 @@
         <v>47</v>
       </c>
       <c r="G11" s="279" t="e" cm="1">
-        <f t="array" ref="G11">SUM(SUMIFS(
+        <f t="array" ref="G11">MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"CONT A JP Siège";"CONT A VIF Siège"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"CONT A JP Siège";"CONT A VIF Siège"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)))</f>
         <v>#N/A</v>
       </c>
       <c r="H11" s="279" t="e" cm="1">
-        <f t="array" ref="H11">SUM(SUMIFS(
+        <f t="array" ref="H11">MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"CONT A JP Parquet";"CONT A VIF Parquet"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),{"CONT A JP Parquet";"CONT A VIF Parquet"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)))</f>
         <v>#N/A</v>
       </c>
       <c r="I11" s="280" t="e">
-        <f>SUM(SUMIFS(
+        <f>MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siège autres",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)))</f>
         <v>#N/A</v>
       </c>
       <c r="J11" s="280" t="e">
-        <f>SUM(SUMIFS(
+        <f>MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siege Assises",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siege Assises",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)))</f>
         <v>#N/A</v>
       </c>
       <c r="K11" s="280" t="e">
-        <f>SUM(SUMIFS(
+        <f>MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siege CCD",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Siege CCD",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)))</f>
         <v>#N/A</v>
       </c>
       <c r="L11" s="280" t="e">
-        <f>SUM(SUMIFS(
+        <f>MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Parquet",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ Parquet",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)))</f>
         <v>#N/A</v>
       </c>
       <c r="M11" s="280"/>
       <c r="N11" s="280"/>
       <c r="O11" s="280" t="e">
-        <f>SUM(SUMIFS(
+        <f>MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JAP",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JAP",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)))</f>
         <v>#N/A</v>
       </c>
       <c r="P11" s="280" t="e">
-        <f>SUM(SUMIFS(
+        <f>MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JE",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JE",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)))</f>
         <v>#N/A</v>
       </c>
       <c r="Q11" s="280" t="e">
-        <f>SUM(SUMIFS(
+        <f>MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JI",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JI",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)))</f>
         <v>#N/A</v>
       </c>
       <c r="R11" s="280" t="e">
-        <f>SUM(SUMIFS(
+        <f>MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD PÉNAL",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"JA/AttJ JLD PÉNAL",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Juridiction",'ETPT Format DDG'!2:2,0)),$D$5)))</f>
         <v>#N/A</v>
       </c>
       <c r="S11" s="278">
@@ -38960,14 +38960,14 @@
         <v>#N/A</v>
       </c>
       <c r="AS5" s="54" t="e">
-        <f>SUM(SUMIFS(
+        <f>MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4. TOTAL CIVIL NON SPÉCIALISÉ",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE S",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE S",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI")))</f>
         <v>#N/A</v>
       </c>
       <c r="AT5" s="54" t="e" cm="1">
@@ -38977,14 +38977,14 @@
         <v>#N/A</v>
       </c>
       <c r="AU5" s="54" t="e">
-        <f>SUM(SUMIFS(
+        <f>MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4. TOTAL CIVIL NON SPÉCIALISÉ",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("4.0. CONTENTIEUX GÉNÉRAL &lt;10.000€",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI")))</f>
         <v>#N/A</v>
       </c>
       <c r="AV5" s="46">
@@ -39123,7 +39123,7 @@
         <v>270</v>
       </c>
       <c r="V6" s="202" t="e">
-        <f>SUM(SUMIFS(
+        <f>MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7. TOTAL SIÈGE PÉNAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR"))+
 SUM(SUMIFS(
@@ -39146,7 +39146,7 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.122. COLLÉGIALES AUTRES SECTIONS SPÉCIALISÉES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR"))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR")))</f>
         <v>#N/A</v>
       </c>
       <c r="W6" s="46">
@@ -39257,7 +39257,7 @@
       <c r="AQ6" s="64"/>
       <c r="AR6" s="64"/>
       <c r="AS6" s="54" t="e">
-        <f>SUMIFS(
+        <f>MAX(0,SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7. TOTAL SIÈGE PÉNAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE S")-
 SUMIFS(
@@ -39283,12 +39283,12 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE S")-
 SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.7. OP CONTRAVENTIONNELLES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE S")</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE S"))</f>
         <v>#N/A</v>
       </c>
       <c r="AT6" s="54"/>
       <c r="AU6" s="63" t="e">
-        <f>SUMIFS(
+        <f>MAX(0,SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7. TOTAL SIÈGE PÉNAL",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS")-
 SUMIFS(
@@ -39314,7 +39314,7 @@
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS")-
 SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("7.7. OP CONTRAVENTIONNELLES",'ETPT Format DDG'!2:2,0)),
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS")</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS"))</f>
         <v>#N/A</v>
       </c>
       <c r="AV6" s="46">
@@ -40068,14 +40068,14 @@
         <v>47</v>
       </c>
       <c r="G12" s="89" t="e">
-        <f>SUM(SUMIFS(
+        <f>MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire CTECH",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI")))</f>
         <v>#N/A</v>
       </c>
       <c r="H12" s="57">
@@ -40096,14 +40096,14 @@
       <c r="T12" s="60"/>
       <c r="U12" s="60"/>
       <c r="V12" s="52" t="e">
-        <f>SUM(SUMIFS(
+        <f>MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Fonctionnaire A-B-CBUR",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI")))</f>
         <v>#N/A</v>
       </c>
       <c r="W12" s="46">
@@ -40123,50 +40123,50 @@
         <v>#N/A</v>
       </c>
       <c r="Z12" s="52" t="e" cm="1">
-        <f t="array" ref="Z12">SUM(SUMIFS(
+        <f t="array" ref="Z12">MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JI";"VPI";"1VPI"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JI";"VPI";"1VPI"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI")))</f>
         <v>#N/A</v>
       </c>
       <c r="AA12" s="60"/>
       <c r="AB12" s="60"/>
       <c r="AC12" s="60"/>
       <c r="AD12" s="52" t="e" cm="1">
-        <f t="array" ref="AD12">SUM(SUMIFS(
+        <f t="array" ref="AD12">MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JAP";"VPAP";"1VPAP"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JAP";"VPAP";"1VPAP"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI")))</f>
         <v>#N/A</v>
       </c>
       <c r="AE12" s="52" t="e" cm="1">
-        <f t="array" ref="AE12">SUM(SUMIFS(
+        <f t="array" ref="AE12">MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JE";"VPE";"1VPE"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"JE";"VPE";"1VPE"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI")))</f>
         <v>#N/A</v>
       </c>
       <c r="AF12" s="52" t="e" cm="1">
-        <f t="array" ref="AF12">SUM(SUMIFS(
+        <f t="array" ref="AF12">MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"VPLD";"1VPLD"},
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction",'ETPT Format DDG'!2:2,0)),{"VPLD";"1VPLD"},
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI")))</f>
         <v>#N/A</v>
       </c>
       <c r="AG12" s="46">
@@ -40187,14 +40187,14 @@
       <c r="AS12" s="60"/>
       <c r="AT12" s="60"/>
       <c r="AU12" s="52" t="e">
-        <f>SUM(SUMIFS(
+        <f>MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12. TOTAL des INDISPONIBILITÉS relevant de l'action 99",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS",
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("12.5. MISE À DISPOSITION",'ETPT Format DDG'!2:2,0)),
 INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT Format DDG'!2:2,0)),"Magistrat SIEGE NS",
-INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI"))</f>
+INDEX( 'ETPT Format DDG'!$A:$ZZ,,MATCH("TJCPH",'ETPT Format DDG'!2:2,0)),"OUI")))</f>
         <v>#N/A</v>
       </c>
       <c r="AV12" s="46">
@@ -40738,14 +40738,14 @@
         <v>#N/A</v>
       </c>
       <c r="AQ14" s="52" t="e">
-        <f>SUM(SUMIFS(
+        <f>MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT A-JUST'!2:2,0)),
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),"Magistrat placé ADD",
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("TJCPH",'ETPT A-JUST'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("1.1. DÉPARTAGE PRUD'HOMAL",'ETPT A-JUST'!2:2,0)),
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),"Magistrat placé ADD",
-INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("TJCPH",'ETPT A-JUST'!2:2,0)),"OUI"))</f>
+INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("TJCPH",'ETPT A-JUST'!2:2,0)),"OUI")))</f>
         <v>#N/A</v>
       </c>
       <c r="AR14" s="52" t="e">
@@ -40762,7 +40762,7 @@
         <v>#N/A</v>
       </c>
       <c r="AU14" s="265" t="e">
-        <f>SUM(SUMIFS(
+        <f>MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("4. TOTAL CIVIL NON SPÉCIALISÉ",'ETPT A-JUST'!2:2,0)),
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),"Magistrat placé ADD",
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("TJCPH",'ETPT A-JUST'!2:2,0)),"OUI"))-
@@ -40829,7 +40829,7 @@
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),"Magistrat placé ADD"))-
 SUM(SUMIFS(
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("7.7. OP CONTRAVENTIONNELLES",'ETPT A-JUST'!2:2,0)),
-INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),"Magistrat placé ADD"))</f>
+INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),"Magistrat placé ADD")))</f>
         <v>#N/A</v>
       </c>
       <c r="AV14" s="46">
@@ -41080,7 +41080,7 @@
         <v>#N/A</v>
       </c>
       <c r="Y15" s="52" t="e">
-        <f>SUM(SUMIFS(
+        <f>MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("3. TOTAL CONTENTIEUX DE LA PROTECTION",'ETPT A-JUST'!2:2,0)),
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),"Magistrat placé SUB",
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("TJCPH",'ETPT A-JUST'!2:2,0)),"OUI"))-
@@ -41095,7 +41095,7 @@
 SUM(SUMIFS(
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("3.44. SAISIE DES RÉMUNÉRATIONS",'ETPT A-JUST'!2:2,0)),
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),"Magistrat placé SUB",
-INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("TJCPH",'ETPT A-JUST'!2:2,0)),"OUI"))</f>
+INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("TJCPH",'ETPT A-JUST'!2:2,0)),"OUI")))</f>
         <v>#N/A</v>
       </c>
       <c r="Z15" s="52" t="e">
@@ -41223,14 +41223,14 @@
         <v>#N/A</v>
       </c>
       <c r="AQ15" s="52" t="e">
-        <f>SUM(SUMIFS(
+        <f>MAX(0,SUM(SUMIFS(
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("1. TOTAL CONTENTIEUX SOCIAL",'ETPT A-JUST'!2:2,0)),
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),"Magistrat placé SUB",
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("TJCPH",'ETPT A-JUST'!2:2,0)),"OUI"))-
 SUM(SUMIFS(
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("1.1. DÉPARTAGE PRUD'HOMAL",'ETPT A-JUST'!2:2,0)),
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),"Magistrat placé SUB",
-INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("TJCPH",'ETPT A-JUST'!2:2,0)),"OUI"))</f>
+INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("TJCPH",'ETPT A-JUST'!2:2,0)),"OUI")))</f>
         <v>#N/A</v>
       </c>
       <c r="AR15" s="52" t="e">

</xml_diff>

<commit_message>
fix calcul of ept saisi
</commit_message>
<xml_diff>
--- a/front/src/assets/template4.xlsx
+++ b/front/src/assets/template4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinum-327809/Documents/a-just-dev/a-just/front/src/assets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francois-xaviermontigny/git/beta.gouv.fr/a-just/front/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E22D660-49FE-F145-B00B-8BAE396A4F8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A3A0383-DF44-9D41-90A4-F5AE55CC880F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17400" xr2:uid="{50CB0F02-73D8-432D-BA19-0D33B1FE1838}"/>
   </bookViews>
   <sheets>
     <sheet name="ACCUEIL" sheetId="33" r:id="rId1"/>
@@ -19281,16 +19281,6 @@
   </cellStyles>
   <dxfs count="28">
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill>
           <bgColor theme="9" tint="0.79998168889431442"/>
@@ -19529,6 +19519,16 @@
       <font>
         <color theme="0"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -37494,7 +37494,7 @@
     <mergeCell ref="D1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2:EZ2 A3:FB1048576">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="27" priority="1">
       <formula>OR(AND(OR($R1&lt;&gt;0,$S1&lt;&gt;0,$T1&lt;&gt;0,ISBLANK($P1)),ROW()&gt;2,$A1&lt;&gt;""),LEFT($I1,3)="JA ")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -37820,70 +37820,70 @@
     <mergeCell ref="U4:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:F4">
-    <cfRule type="expression" dxfId="27" priority="16">
+    <cfRule type="expression" dxfId="26" priority="16">
       <formula>IF(LEFT($A$3,2)&lt;&gt;"TJ",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:V151">
-    <cfRule type="expression" dxfId="26" priority="18" stopIfTrue="1">
+    <cfRule type="expression" dxfId="25" priority="18" stopIfTrue="1">
       <formula>AND(ISBLANK($C6)=FALSE,ISBLANK($E6)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:F1048576">
-    <cfRule type="expression" dxfId="25" priority="1">
+    <cfRule type="expression" dxfId="24" priority="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)-_xlfn.NUMBERVALUE($U6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="2">
+    <cfRule type="expression" dxfId="23" priority="2">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)-_xlfn.NUMBERVALUE($S6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="23" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="22" priority="7" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3)-_xlfn.NUMBERVALUE($L4)-_xlfn.NUMBERVALUE($L5)-_xlfn.NUMBERVALUE($L6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="12">
+    <cfRule type="expression" dxfId="21" priority="12">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",OR(ROUND(_xlfn.NUMBERVALUE($L1)-_xlfn.NUMBERVALUE($L2)-_xlfn.NUMBERVALUE($L3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0,ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:F7">
-    <cfRule type="expression" dxfId="21" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="20" priority="6" stopIfTrue="1">
       <formula>OR(ROUND(_xlfn.NUMBERVALUE($L7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($L6),3),ROUND(_xlfn.NUMBERVALUE($S7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($S6),3),ROUND(_xlfn.NUMBERVALUE($U7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($U6),3))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:M1048576">
-    <cfRule type="expression" dxfId="20" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="19" priority="11" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)+_xlfn.NUMBERVALUE($L4)+_xlfn.NUMBERVALUE($L5)+_xlfn.NUMBERVALUE($L6)),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="15">
+    <cfRule type="expression" dxfId="18" priority="15">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($L1)-(_xlfn.NUMBERVALUE($L2)+_xlfn.NUMBERVALUE($L3)),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:M7">
-    <cfRule type="expression" dxfId="18" priority="5">
+    <cfRule type="expression" dxfId="17" priority="5">
       <formula>ROUND(_xlfn.NUMBERVALUE($L7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($L6),3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1048576">
-    <cfRule type="expression" dxfId="17" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="16" priority="10" stopIfTrue="1">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3)-_xlfn.NUMBERVALUE($S4)-_xlfn.NUMBERVALUE($S5)-_xlfn.NUMBERVALUE($S6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="14">
+    <cfRule type="expression" dxfId="15" priority="14">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($S1)-_xlfn.NUMBERVALUE($S2)-_xlfn.NUMBERVALUE($S3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N7:T7">
-    <cfRule type="expression" dxfId="15" priority="4">
+    <cfRule type="expression" dxfId="14" priority="4">
       <formula>ROUND(_xlfn.NUMBERVALUE($S7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($S6),3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:V1048576">
-    <cfRule type="expression" dxfId="14" priority="9">
+    <cfRule type="expression" dxfId="13" priority="9">
       <formula>AND($D1="8. TOTAL JUGES D'INSTRUCTION",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3)-_xlfn.NUMBERVALUE($U4)-_xlfn.NUMBERVALUE($U5)-_xlfn.NUMBERVALUE($U6),3)&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="13">
+    <cfRule type="expression" dxfId="12" priority="13">
       <formula>AND($D1="6. TOTAL JUGES DES ENFANTS",ROUND(_xlfn.NUMBERVALUE($U1)-_xlfn.NUMBERVALUE($U2)-_xlfn.NUMBERVALUE($U3),3)&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:V7">
-    <cfRule type="expression" dxfId="12" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="3" stopIfTrue="1">
       <formula>ROUND(_xlfn.NUMBERVALUE($U7),3)&lt;&gt;ROUND(_xlfn.NUMBERVALUE($U6),3)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -38175,57 +38175,57 @@
   </sheetData>
   <autoFilter ref="A1:V1" xr:uid="{02AF4949-5E39-2D4C-AD07-A4D8FB117F56}"/>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="11" priority="30">
+    <cfRule type="expression" dxfId="10" priority="30">
       <formula>AND(OR($I1&lt;&gt;"-",#REF!&lt;&gt;0,#REF!&lt;&gt;0,ISBLANK($M1)),ROW()&gt;2,$A1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:F2">
-    <cfRule type="expression" dxfId="10" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="11" stopIfTrue="1">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:N2">
-    <cfRule type="expression" dxfId="9" priority="5">
+    <cfRule type="expression" dxfId="8" priority="5">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:K2">
-    <cfRule type="expression" dxfId="8" priority="6">
+    <cfRule type="expression" dxfId="7" priority="6">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2">
-    <cfRule type="expression" dxfId="7" priority="8">
+    <cfRule type="expression" dxfId="6" priority="8">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2">
-    <cfRule type="expression" dxfId="6" priority="7">
+    <cfRule type="expression" dxfId="5" priority="7">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2">
-    <cfRule type="expression" dxfId="5" priority="9">
+    <cfRule type="expression" dxfId="4" priority="9">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:V2">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>$F2="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q2:R2">
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="2" priority="4">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S2:T2">
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="1" priority="3">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V2">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>1=1</formula>
     </cfRule>
   </conditionalFormatting>
@@ -40550,10 +40550,6 @@
 SUM(SUMIFS(
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("5. TOTAL JLD CIVIL",'ETPT A-JUST'!2:2,0)),
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD"))+
-SUM(SUMIFS(
-INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("6.1. ACTIVITÉ CIVILE",'ETPT A-JUST'!2:2,0)),
-INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD",
-INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("TJCPH",'ETPT A-JUST'!2:2,0)),"OUI"))+
 _xlfn.IFNA(SUM(SUMIFS(
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("13. TOTAL CONTENTIEUX LOCAUX SPÉCIFIQUES",'ETPT A-JUST'!2:2,0)),
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),"Fonctionnaire A-B-CBUR placé ADD",
@@ -41035,10 +41031,6 @@
 SUM(SUMIFS(
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("5. TOTAL JLD CIVIL",'ETPT A-JUST'!2:2,0)),
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB"))+
-SUM(SUMIFS(
-INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("6.1. ACTIVITÉ CIVILE",'ETPT A-JUST'!2:2,0)),
-INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB",
-INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("TJCPH",'ETPT A-JUST'!2:2,0)),"OUI"))+
 _xlfn.IFNA(SUM(SUMIFS(
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("13. TOTAL CONTENTIEUX LOCAUX SPÉCIFIQUES",'ETPT A-JUST'!2:2,0)),
 INDEX( 'ETPT A-JUST'!$A:$ZZ,,MATCH("Fonction recodée",'ETPT A-JUST'!2:2,0)),"Fonctionnaire A-B-CBUR placé SUB",

</xml_diff>